<commit_message>
chore(data): batch update intraday vendas - 12:00:02
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -559,17 +559,17 @@
         <v>46217</v>
       </c>
       <c r="B7" t="n">
-        <v>1063</v>
+        <v>610</v>
       </c>
       <c r="C7" t="n">
         <v>8888</v>
       </c>
       <c r="D7" t="n">
-        <v>1251.14</v>
+        <v>590.08</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -578,17 +578,17 @@
         <v>46217</v>
       </c>
       <c r="B8" t="n">
-        <v>325</v>
+        <v>1063</v>
       </c>
       <c r="C8" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D8" t="n">
-        <v>868.83</v>
+        <v>1251.14</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -597,17 +597,17 @@
         <v>46217</v>
       </c>
       <c r="B9" t="n">
-        <v>610</v>
+        <v>325</v>
       </c>
       <c r="C9" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D9" t="n">
-        <v>235.34</v>
+        <v>868.83</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -616,17 +616,17 @@
         <v>46217</v>
       </c>
       <c r="B10" t="n">
-        <v>40</v>
+        <v>610</v>
       </c>
       <c r="C10" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D10" t="n">
-        <v>325.04</v>
+        <v>235.34</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -635,17 +635,17 @@
         <v>46217</v>
       </c>
       <c r="B11" t="n">
-        <v>1117</v>
+        <v>40</v>
       </c>
       <c r="C11" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D11" t="n">
-        <v>349.47</v>
+        <v>325.04</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -654,17 +654,17 @@
         <v>46217</v>
       </c>
       <c r="B12" t="n">
-        <v>949</v>
+        <v>1117</v>
       </c>
       <c r="C12" t="n">
-        <v>998</v>
+        <v>8888</v>
       </c>
       <c r="D12" t="n">
-        <v>129.85</v>
+        <v>349.47</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -673,17 +673,17 @@
         <v>46217</v>
       </c>
       <c r="B13" t="n">
-        <v>2250</v>
+        <v>949</v>
       </c>
       <c r="C13" t="n">
-        <v>8888</v>
+        <v>998</v>
       </c>
       <c r="D13" t="n">
-        <v>2693.99</v>
+        <v>129.85</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -692,17 +692,17 @@
         <v>46217</v>
       </c>
       <c r="B14" t="n">
-        <v>2663</v>
+        <v>2250</v>
       </c>
       <c r="C14" t="n">
         <v>8888</v>
       </c>
       <c r="D14" t="n">
-        <v>2146.08</v>
+        <v>3180.11</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -711,17 +711,17 @@
         <v>46217</v>
       </c>
       <c r="B15" t="n">
-        <v>664</v>
+        <v>2663</v>
       </c>
       <c r="C15" t="n">
         <v>8888</v>
       </c>
       <c r="D15" t="n">
-        <v>350.72</v>
+        <v>2146.08</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -730,17 +730,17 @@
         <v>46217</v>
       </c>
       <c r="B16" t="n">
-        <v>1063</v>
+        <v>664</v>
       </c>
       <c r="C16" t="n">
         <v>8888</v>
       </c>
       <c r="D16" t="n">
-        <v>1902.46</v>
+        <v>350.72</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -749,17 +749,17 @@
         <v>46217</v>
       </c>
       <c r="B17" t="n">
-        <v>949</v>
+        <v>1063</v>
       </c>
       <c r="C17" t="n">
-        <v>1134</v>
+        <v>8888</v>
       </c>
       <c r="D17" t="n">
-        <v>327.6</v>
+        <v>1902.46</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
         <v>46217</v>
       </c>
       <c r="B18" t="n">
-        <v>326</v>
+        <v>949</v>
       </c>
       <c r="C18" t="n">
-        <v>8888</v>
+        <v>1134</v>
       </c>
       <c r="D18" t="n">
-        <v>116.94</v>
+        <v>327.6</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -787,17 +787,17 @@
         <v>46217</v>
       </c>
       <c r="B19" t="n">
-        <v>1116</v>
+        <v>326</v>
       </c>
       <c r="C19" t="n">
         <v>8888</v>
       </c>
       <c r="D19" t="n">
-        <v>971.6</v>
+        <v>116.94</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -806,17 +806,17 @@
         <v>46217</v>
       </c>
       <c r="B20" t="n">
-        <v>1983</v>
+        <v>1116</v>
       </c>
       <c r="C20" t="n">
         <v>8888</v>
       </c>
       <c r="D20" t="n">
-        <v>412.16</v>
+        <v>971.6</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -825,17 +825,17 @@
         <v>46217</v>
       </c>
       <c r="B21" t="n">
-        <v>451</v>
+        <v>1983</v>
       </c>
       <c r="C21" t="n">
         <v>8888</v>
       </c>
       <c r="D21" t="n">
-        <v>2583.46</v>
+        <v>412.16</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -844,17 +844,17 @@
         <v>46217</v>
       </c>
       <c r="B22" t="n">
-        <v>325</v>
+        <v>451</v>
       </c>
       <c r="C22" t="n">
         <v>8888</v>
       </c>
       <c r="D22" t="n">
-        <v>459.43</v>
+        <v>2583.46</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -863,17 +863,17 @@
         <v>46217</v>
       </c>
       <c r="B23" t="n">
-        <v>1063</v>
+        <v>325</v>
       </c>
       <c r="C23" t="n">
         <v>8888</v>
       </c>
       <c r="D23" t="n">
-        <v>352.87</v>
+        <v>459.43</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -882,13 +882,13 @@
         <v>46217</v>
       </c>
       <c r="B24" t="n">
-        <v>629</v>
+        <v>1063</v>
       </c>
       <c r="C24" t="n">
         <v>8888</v>
       </c>
       <c r="D24" t="n">
-        <v>277.36</v>
+        <v>352.87</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -907,11 +907,11 @@
         <v>8888</v>
       </c>
       <c r="D25" t="n">
-        <v>2049.78</v>
+        <v>277.36</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
         <v>46217</v>
       </c>
       <c r="B26" t="n">
-        <v>949</v>
+        <v>629</v>
       </c>
       <c r="C26" t="n">
-        <v>1762</v>
+        <v>8888</v>
       </c>
       <c r="D26" t="n">
-        <v>325.65</v>
+        <v>2049.78</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -939,17 +939,17 @@
         <v>46217</v>
       </c>
       <c r="B27" t="n">
-        <v>2463</v>
+        <v>949</v>
       </c>
       <c r="C27" t="n">
-        <v>8888</v>
+        <v>1762</v>
       </c>
       <c r="D27" t="n">
-        <v>8336.43</v>
+        <v>325.65</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -958,17 +958,17 @@
         <v>46217</v>
       </c>
       <c r="B28" t="n">
-        <v>451</v>
+        <v>2463</v>
       </c>
       <c r="C28" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D28" t="n">
-        <v>327.28</v>
+        <v>8336.43</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -977,17 +977,17 @@
         <v>46217</v>
       </c>
       <c r="B29" t="n">
-        <v>610</v>
+        <v>451</v>
       </c>
       <c r="C29" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D29" t="n">
-        <v>335.61</v>
+        <v>327.28</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -996,17 +996,17 @@
         <v>46217</v>
       </c>
       <c r="B30" t="n">
-        <v>341</v>
+        <v>610</v>
       </c>
       <c r="C30" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D30" t="n">
-        <v>366.88</v>
+        <v>335.61</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1015,17 +1015,17 @@
         <v>46217</v>
       </c>
       <c r="B31" t="n">
-        <v>1064</v>
+        <v>341</v>
       </c>
       <c r="C31" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D31" t="n">
-        <v>692.0599999999999</v>
+        <v>366.88</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1034,13 +1034,13 @@
         <v>46217</v>
       </c>
       <c r="B32" t="n">
-        <v>663</v>
+        <v>1064</v>
       </c>
       <c r="C32" t="n">
         <v>8888</v>
       </c>
       <c r="D32" t="n">
-        <v>824.5599999999999</v>
+        <v>692.0599999999999</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1053,17 +1053,17 @@
         <v>46217</v>
       </c>
       <c r="B33" t="n">
-        <v>1064</v>
+        <v>663</v>
       </c>
       <c r="C33" t="n">
         <v>8888</v>
       </c>
       <c r="D33" t="n">
-        <v>2383.39</v>
+        <v>824.5599999999999</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1072,13 +1072,13 @@
         <v>46217</v>
       </c>
       <c r="B34" t="n">
-        <v>451</v>
+        <v>1064</v>
       </c>
       <c r="C34" t="n">
         <v>8888</v>
       </c>
       <c r="D34" t="n">
-        <v>1371.26</v>
+        <v>2383.39</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1091,17 +1091,17 @@
         <v>46217</v>
       </c>
       <c r="B35" t="n">
-        <v>40</v>
+        <v>451</v>
       </c>
       <c r="C35" t="n">
         <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>488.35</v>
+        <v>1371.26</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1110,17 @@
         <v>46217</v>
       </c>
       <c r="B36" t="n">
-        <v>530</v>
+        <v>40</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>180.08</v>
+        <v>1093.47</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1129,13 +1129,13 @@
         <v>46217</v>
       </c>
       <c r="B37" t="n">
-        <v>559</v>
+        <v>530</v>
       </c>
       <c r="C37" t="n">
         <v>8888</v>
       </c>
       <c r="D37" t="n">
-        <v>512.59</v>
+        <v>180.08</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1148,13 +1148,13 @@
         <v>46217</v>
       </c>
       <c r="B38" t="n">
-        <v>1937</v>
+        <v>559</v>
       </c>
       <c r="C38" t="n">
         <v>8888</v>
       </c>
       <c r="D38" t="n">
-        <v>937.47</v>
+        <v>512.59</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1167,17 +1167,17 @@
         <v>46217</v>
       </c>
       <c r="B39" t="n">
-        <v>131</v>
+        <v>89</v>
       </c>
       <c r="C39" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D39" t="n">
-        <v>211.41</v>
+        <v>1506.42</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1186,17 +1186,17 @@
         <v>46217</v>
       </c>
       <c r="B40" t="n">
-        <v>2250</v>
+        <v>1937</v>
       </c>
       <c r="C40" t="n">
         <v>8888</v>
       </c>
       <c r="D40" t="n">
-        <v>1943.54</v>
+        <v>937.47</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1205,17 +1205,17 @@
         <v>46217</v>
       </c>
       <c r="B41" t="n">
-        <v>89</v>
+        <v>131</v>
       </c>
       <c r="C41" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D41" t="n">
-        <v>573.46</v>
+        <v>211.41</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1224,17 +1224,17 @@
         <v>46217</v>
       </c>
       <c r="B42" t="n">
-        <v>1299</v>
+        <v>2250</v>
       </c>
       <c r="C42" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D42" t="n">
-        <v>262.02</v>
+        <v>1943.54</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1243,17 +1243,17 @@
         <v>46217</v>
       </c>
       <c r="B43" t="n">
-        <v>131</v>
+        <v>1299</v>
       </c>
       <c r="C43" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D43" t="n">
-        <v>609.86</v>
+        <v>262.02</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1262,17 +1262,17 @@
         <v>46217</v>
       </c>
       <c r="B44" t="n">
-        <v>40</v>
+        <v>131</v>
       </c>
       <c r="C44" t="n">
         <v>8888</v>
       </c>
       <c r="D44" t="n">
-        <v>733.37</v>
+        <v>609.86</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1281,13 +1281,13 @@
         <v>46217</v>
       </c>
       <c r="B45" t="n">
-        <v>559</v>
+        <v>40</v>
       </c>
       <c r="C45" t="n">
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>1562.5</v>
+        <v>733.37</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1300,13 +1300,13 @@
         <v>46217</v>
       </c>
       <c r="B46" t="n">
-        <v>2550</v>
+        <v>40</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>321.05</v>
+        <v>799.86</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1319,17 +1319,17 @@
         <v>46217</v>
       </c>
       <c r="B47" t="n">
-        <v>2250</v>
+        <v>2651</v>
       </c>
       <c r="C47" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D47" t="n">
-        <v>1512.17</v>
+        <v>316.61</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1338,13 +1338,13 @@
         <v>46217</v>
       </c>
       <c r="B48" t="n">
-        <v>1465</v>
+        <v>559</v>
       </c>
       <c r="C48" t="n">
         <v>8888</v>
       </c>
       <c r="D48" t="n">
-        <v>8550.709999999999</v>
+        <v>1562.5</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1357,15 +1357,72 @@
         <v>46217</v>
       </c>
       <c r="B49" t="n">
+        <v>2550</v>
+      </c>
+      <c r="C49" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D49" t="n">
+        <v>321.05</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B50" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C50" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D50" t="n">
+        <v>1512.17</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B51" t="n">
+        <v>1465</v>
+      </c>
+      <c r="C51" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D51" t="n">
+        <v>8550.709999999999</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B52" t="n">
         <v>483</v>
       </c>
-      <c r="C49" t="n">
-        <v>8888</v>
-      </c>
-      <c r="D49" t="n">
+      <c r="C52" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D52" t="n">
         <v>720.66</v>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>FORÇA DE VENDAS</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 13:04:43
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,17 +464,17 @@
         <v>46217</v>
       </c>
       <c r="B2" t="n">
-        <v>42</v>
+        <v>1756</v>
       </c>
       <c r="C2" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D2" t="n">
-        <v>22505.79</v>
+        <v>556.23</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -483,17 +483,17 @@
         <v>46217</v>
       </c>
       <c r="B3" t="n">
-        <v>1102</v>
+        <v>42</v>
       </c>
       <c r="C3" t="n">
         <v>8888</v>
       </c>
       <c r="D3" t="n">
-        <v>1199.81</v>
+        <v>22505.79</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -502,13 +502,13 @@
         <v>46217</v>
       </c>
       <c r="B4" t="n">
-        <v>89</v>
+        <v>2109</v>
       </c>
       <c r="C4" t="n">
         <v>8888</v>
       </c>
       <c r="D4" t="n">
-        <v>4572.01</v>
+        <v>4813.6</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -521,13 +521,13 @@
         <v>46217</v>
       </c>
       <c r="B5" t="n">
-        <v>949</v>
+        <v>2015</v>
       </c>
       <c r="C5" t="n">
-        <v>1258</v>
+        <v>2571</v>
       </c>
       <c r="D5" t="n">
-        <v>196.87</v>
+        <v>679.9</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -540,17 +540,17 @@
         <v>46217</v>
       </c>
       <c r="B6" t="n">
-        <v>285</v>
+        <v>1293</v>
       </c>
       <c r="C6" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D6" t="n">
-        <v>1081.17</v>
+        <v>1337.87</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -559,17 +559,17 @@
         <v>46217</v>
       </c>
       <c r="B7" t="n">
-        <v>610</v>
+        <v>1102</v>
       </c>
       <c r="C7" t="n">
         <v>8888</v>
       </c>
       <c r="D7" t="n">
-        <v>590.08</v>
+        <v>1199.81</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -578,17 +578,17 @@
         <v>46217</v>
       </c>
       <c r="B8" t="n">
-        <v>1063</v>
+        <v>89</v>
       </c>
       <c r="C8" t="n">
         <v>8888</v>
       </c>
       <c r="D8" t="n">
-        <v>1251.14</v>
+        <v>4572.01</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -597,17 +597,17 @@
         <v>46217</v>
       </c>
       <c r="B9" t="n">
-        <v>325</v>
+        <v>2768</v>
       </c>
       <c r="C9" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D9" t="n">
-        <v>868.83</v>
+        <v>3436.6</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -616,17 +616,17 @@
         <v>46217</v>
       </c>
       <c r="B10" t="n">
-        <v>610</v>
+        <v>949</v>
       </c>
       <c r="C10" t="n">
-        <v>8888</v>
+        <v>1258</v>
       </c>
       <c r="D10" t="n">
-        <v>235.34</v>
+        <v>196.87</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -635,17 +635,17 @@
         <v>46217</v>
       </c>
       <c r="B11" t="n">
-        <v>40</v>
+        <v>1756</v>
       </c>
       <c r="C11" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D11" t="n">
-        <v>325.04</v>
+        <v>1799.7</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -654,17 +654,17 @@
         <v>46217</v>
       </c>
       <c r="B12" t="n">
-        <v>1117</v>
+        <v>285</v>
       </c>
       <c r="C12" t="n">
         <v>8888</v>
       </c>
       <c r="D12" t="n">
-        <v>349.47</v>
+        <v>1081.17</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -673,17 +673,17 @@
         <v>46217</v>
       </c>
       <c r="B13" t="n">
-        <v>949</v>
+        <v>610</v>
       </c>
       <c r="C13" t="n">
-        <v>998</v>
+        <v>8888</v>
       </c>
       <c r="D13" t="n">
-        <v>129.85</v>
+        <v>590.08</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -692,17 +692,17 @@
         <v>46217</v>
       </c>
       <c r="B14" t="n">
-        <v>2250</v>
+        <v>2755</v>
       </c>
       <c r="C14" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D14" t="n">
-        <v>3180.11</v>
+        <v>1133.17</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -711,17 +711,17 @@
         <v>46217</v>
       </c>
       <c r="B15" t="n">
-        <v>2663</v>
+        <v>2767</v>
       </c>
       <c r="C15" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D15" t="n">
-        <v>2146.08</v>
+        <v>5000.2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -730,13 +730,13 @@
         <v>46217</v>
       </c>
       <c r="B16" t="n">
-        <v>664</v>
+        <v>2767</v>
       </c>
       <c r="C16" t="n">
         <v>8888</v>
       </c>
       <c r="D16" t="n">
-        <v>350.72</v>
+        <v>1175.73</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -755,11 +755,11 @@
         <v>8888</v>
       </c>
       <c r="D17" t="n">
-        <v>1902.46</v>
+        <v>1251.14</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -768,13 +768,13 @@
         <v>46217</v>
       </c>
       <c r="B18" t="n">
-        <v>949</v>
+        <v>325</v>
       </c>
       <c r="C18" t="n">
-        <v>1134</v>
+        <v>58</v>
       </c>
       <c r="D18" t="n">
-        <v>327.6</v>
+        <v>868.83</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -787,17 +787,17 @@
         <v>46217</v>
       </c>
       <c r="B19" t="n">
-        <v>326</v>
+        <v>610</v>
       </c>
       <c r="C19" t="n">
         <v>8888</v>
       </c>
       <c r="D19" t="n">
-        <v>116.94</v>
+        <v>235.34</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -806,17 +806,17 @@
         <v>46217</v>
       </c>
       <c r="B20" t="n">
-        <v>1116</v>
+        <v>1906</v>
       </c>
       <c r="C20" t="n">
         <v>8888</v>
       </c>
       <c r="D20" t="n">
-        <v>971.6</v>
+        <v>889.22</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -825,17 +825,17 @@
         <v>46217</v>
       </c>
       <c r="B21" t="n">
-        <v>1983</v>
+        <v>40</v>
       </c>
       <c r="C21" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D21" t="n">
-        <v>412.16</v>
+        <v>325.04</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -844,17 +844,17 @@
         <v>46217</v>
       </c>
       <c r="B22" t="n">
-        <v>451</v>
+        <v>1117</v>
       </c>
       <c r="C22" t="n">
         <v>8888</v>
       </c>
       <c r="D22" t="n">
-        <v>2583.46</v>
+        <v>349.47</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -863,17 +863,17 @@
         <v>46217</v>
       </c>
       <c r="B23" t="n">
-        <v>325</v>
+        <v>949</v>
       </c>
       <c r="C23" t="n">
-        <v>8888</v>
+        <v>998</v>
       </c>
       <c r="D23" t="n">
-        <v>459.43</v>
+        <v>129.85</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -882,13 +882,13 @@
         <v>46217</v>
       </c>
       <c r="B24" t="n">
-        <v>1063</v>
+        <v>2250</v>
       </c>
       <c r="C24" t="n">
         <v>8888</v>
       </c>
       <c r="D24" t="n">
-        <v>352.87</v>
+        <v>3180.11</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -901,17 +901,17 @@
         <v>46217</v>
       </c>
       <c r="B25" t="n">
-        <v>629</v>
+        <v>2507</v>
       </c>
       <c r="C25" t="n">
         <v>8888</v>
       </c>
       <c r="D25" t="n">
-        <v>277.36</v>
+        <v>4167.12</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
         <v>46217</v>
       </c>
       <c r="B26" t="n">
-        <v>629</v>
+        <v>664</v>
       </c>
       <c r="C26" t="n">
         <v>8888</v>
       </c>
       <c r="D26" t="n">
-        <v>2049.78</v>
+        <v>3523.8</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -939,13 +939,13 @@
         <v>46217</v>
       </c>
       <c r="B27" t="n">
-        <v>949</v>
+        <v>1906</v>
       </c>
       <c r="C27" t="n">
-        <v>1762</v>
+        <v>1954</v>
       </c>
       <c r="D27" t="n">
-        <v>325.65</v>
+        <v>1445.21</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -958,17 +958,17 @@
         <v>46217</v>
       </c>
       <c r="B28" t="n">
-        <v>2463</v>
+        <v>1075</v>
       </c>
       <c r="C28" t="n">
         <v>8888</v>
       </c>
       <c r="D28" t="n">
-        <v>8336.43</v>
+        <v>470.95</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -977,13 +977,13 @@
         <v>46217</v>
       </c>
       <c r="B29" t="n">
-        <v>451</v>
+        <v>2696</v>
       </c>
       <c r="C29" t="n">
-        <v>3403</v>
+        <v>1312</v>
       </c>
       <c r="D29" t="n">
-        <v>327.28</v>
+        <v>677.76</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -996,17 +996,17 @@
         <v>46217</v>
       </c>
       <c r="B30" t="n">
-        <v>610</v>
+        <v>360</v>
       </c>
       <c r="C30" t="n">
-        <v>8888</v>
+        <v>546</v>
       </c>
       <c r="D30" t="n">
-        <v>335.61</v>
+        <v>4515.36</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1015,17 +1015,17 @@
         <v>46217</v>
       </c>
       <c r="B31" t="n">
-        <v>341</v>
+        <v>1293</v>
       </c>
       <c r="C31" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D31" t="n">
-        <v>366.88</v>
+        <v>381.82</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1034,17 +1034,17 @@
         <v>46217</v>
       </c>
       <c r="B32" t="n">
-        <v>1064</v>
+        <v>2663</v>
       </c>
       <c r="C32" t="n">
         <v>8888</v>
       </c>
       <c r="D32" t="n">
-        <v>692.0599999999999</v>
+        <v>2146.08</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1053,13 +1053,13 @@
         <v>46217</v>
       </c>
       <c r="B33" t="n">
-        <v>663</v>
+        <v>675</v>
       </c>
       <c r="C33" t="n">
         <v>8888</v>
       </c>
       <c r="D33" t="n">
-        <v>824.5599999999999</v>
+        <v>289.67</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1072,13 +1072,13 @@
         <v>46217</v>
       </c>
       <c r="B34" t="n">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="C34" t="n">
         <v>8888</v>
       </c>
       <c r="D34" t="n">
-        <v>2383.39</v>
+        <v>1902.46</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1091,17 +1091,17 @@
         <v>46217</v>
       </c>
       <c r="B35" t="n">
-        <v>451</v>
+        <v>1392</v>
       </c>
       <c r="C35" t="n">
         <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>1371.26</v>
+        <v>814.61</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1110,17 @@
         <v>46217</v>
       </c>
       <c r="B36" t="n">
-        <v>40</v>
+        <v>360</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>1093.47</v>
+        <v>749.13</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1129,17 @@
         <v>46217</v>
       </c>
       <c r="B37" t="n">
-        <v>530</v>
+        <v>2491</v>
       </c>
       <c r="C37" t="n">
         <v>8888</v>
       </c>
       <c r="D37" t="n">
-        <v>180.08</v>
+        <v>398.66</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1148,17 +1148,17 @@
         <v>46217</v>
       </c>
       <c r="B38" t="n">
-        <v>559</v>
+        <v>949</v>
       </c>
       <c r="C38" t="n">
-        <v>8888</v>
+        <v>1134</v>
       </c>
       <c r="D38" t="n">
-        <v>512.59</v>
+        <v>327.6</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1167,13 +1167,13 @@
         <v>46217</v>
       </c>
       <c r="B39" t="n">
-        <v>89</v>
+        <v>326</v>
       </c>
       <c r="C39" t="n">
         <v>8888</v>
       </c>
       <c r="D39" t="n">
-        <v>1506.42</v>
+        <v>212.63</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1186,13 +1186,13 @@
         <v>46217</v>
       </c>
       <c r="B40" t="n">
-        <v>1937</v>
+        <v>1116</v>
       </c>
       <c r="C40" t="n">
         <v>8888</v>
       </c>
       <c r="D40" t="n">
-        <v>937.47</v>
+        <v>971.6</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1205,17 +1205,17 @@
         <v>46217</v>
       </c>
       <c r="B41" t="n">
-        <v>131</v>
+        <v>325</v>
       </c>
       <c r="C41" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D41" t="n">
-        <v>211.41</v>
+        <v>538.37</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1224,17 +1224,17 @@
         <v>46217</v>
       </c>
       <c r="B42" t="n">
-        <v>2250</v>
+        <v>1293</v>
       </c>
       <c r="C42" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D42" t="n">
-        <v>1943.54</v>
+        <v>3534.85</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1243,17 +1243,17 @@
         <v>46217</v>
       </c>
       <c r="B43" t="n">
-        <v>1299</v>
+        <v>1983</v>
       </c>
       <c r="C43" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D43" t="n">
-        <v>262.02</v>
+        <v>412.16</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1262,13 +1262,13 @@
         <v>46217</v>
       </c>
       <c r="B44" t="n">
-        <v>131</v>
+        <v>451</v>
       </c>
       <c r="C44" t="n">
         <v>8888</v>
       </c>
       <c r="D44" t="n">
-        <v>609.86</v>
+        <v>2583.46</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1281,13 +1281,13 @@
         <v>46217</v>
       </c>
       <c r="B45" t="n">
-        <v>40</v>
+        <v>2767</v>
       </c>
       <c r="C45" t="n">
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>733.37</v>
+        <v>596.88</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1300,13 +1300,13 @@
         <v>46217</v>
       </c>
       <c r="B46" t="n">
-        <v>40</v>
+        <v>1063</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>799.86</v>
+        <v>352.87</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1319,17 +1319,17 @@
         <v>46217</v>
       </c>
       <c r="B47" t="n">
-        <v>2651</v>
+        <v>58</v>
       </c>
       <c r="C47" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D47" t="n">
-        <v>316.61</v>
+        <v>2637.19</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1338,17 +1338,17 @@
         <v>46217</v>
       </c>
       <c r="B48" t="n">
-        <v>559</v>
+        <v>2211</v>
       </c>
       <c r="C48" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D48" t="n">
-        <v>1562.5</v>
+        <v>967.05</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1357,13 +1357,13 @@
         <v>46217</v>
       </c>
       <c r="B49" t="n">
-        <v>2550</v>
+        <v>629</v>
       </c>
       <c r="C49" t="n">
         <v>8888</v>
       </c>
       <c r="D49" t="n">
-        <v>321.05</v>
+        <v>277.36</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1376,13 +1376,13 @@
         <v>46217</v>
       </c>
       <c r="B50" t="n">
-        <v>2250</v>
+        <v>629</v>
       </c>
       <c r="C50" t="n">
         <v>8888</v>
       </c>
       <c r="D50" t="n">
-        <v>1512.17</v>
+        <v>2049.78</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1395,17 +1395,17 @@
         <v>46217</v>
       </c>
       <c r="B51" t="n">
-        <v>1465</v>
+        <v>949</v>
       </c>
       <c r="C51" t="n">
-        <v>8888</v>
+        <v>1762</v>
       </c>
       <c r="D51" t="n">
-        <v>8550.709999999999</v>
+        <v>325.65</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1414,15 +1414,1231 @@
         <v>46217</v>
       </c>
       <c r="B52" t="n">
+        <v>2463</v>
+      </c>
+      <c r="C52" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D52" t="n">
+        <v>8336.43</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B53" t="n">
+        <v>1064</v>
+      </c>
+      <c r="C53" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1513.21</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B54" t="n">
+        <v>1478</v>
+      </c>
+      <c r="C54" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D54" t="n">
+        <v>1294.76</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B55" t="n">
+        <v>358</v>
+      </c>
+      <c r="C55" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D55" t="n">
+        <v>1918.33</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B56" t="n">
+        <v>2107</v>
+      </c>
+      <c r="C56" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D56" t="n">
+        <v>2745.11</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B57" t="n">
+        <v>675</v>
+      </c>
+      <c r="C57" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D57" t="n">
+        <v>275.17</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B58" t="n">
+        <v>451</v>
+      </c>
+      <c r="C58" t="n">
+        <v>3403</v>
+      </c>
+      <c r="D58" t="n">
+        <v>327.28</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B59" t="n">
+        <v>2571</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1312</v>
+      </c>
+      <c r="D59" t="n">
+        <v>2202.75</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B60" t="n">
+        <v>610</v>
+      </c>
+      <c r="C60" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D60" t="n">
+        <v>335.61</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B61" t="n">
+        <v>1108</v>
+      </c>
+      <c r="C61" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D61" t="n">
+        <v>508.54</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B62" t="n">
+        <v>341</v>
+      </c>
+      <c r="C62" t="n">
+        <v>58</v>
+      </c>
+      <c r="D62" t="n">
+        <v>366.88</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B63" t="n">
+        <v>1653</v>
+      </c>
+      <c r="C63" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D63" t="n">
+        <v>4383.69</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B64" t="n">
+        <v>663</v>
+      </c>
+      <c r="C64" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D64" t="n">
+        <v>824.5599999999999</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B65" t="n">
+        <v>58</v>
+      </c>
+      <c r="C65" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D65" t="n">
+        <v>660.1</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B66" t="n">
+        <v>429</v>
+      </c>
+      <c r="C66" t="n">
+        <v>2571</v>
+      </c>
+      <c r="D66" t="n">
+        <v>667.12</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B67" t="n">
         <v>483</v>
       </c>
-      <c r="C52" t="n">
-        <v>8888</v>
-      </c>
-      <c r="D52" t="n">
+      <c r="C67" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D67" t="n">
+        <v>938.34</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B68" t="n">
+        <v>2709</v>
+      </c>
+      <c r="C68" t="n">
+        <v>2220</v>
+      </c>
+      <c r="D68" t="n">
+        <v>1663.5</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B69" t="n">
+        <v>1937</v>
+      </c>
+      <c r="C69" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D69" t="n">
+        <v>1332.89</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B70" t="n">
+        <v>429</v>
+      </c>
+      <c r="C70" t="n">
+        <v>1281</v>
+      </c>
+      <c r="D70" t="n">
+        <v>1333.52</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B71" t="n">
+        <v>2211</v>
+      </c>
+      <c r="C71" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D71" t="n">
+        <v>797.61</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B72" t="n">
+        <v>1064</v>
+      </c>
+      <c r="C72" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D72" t="n">
+        <v>2383.39</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B73" t="n">
+        <v>451</v>
+      </c>
+      <c r="C73" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D73" t="n">
+        <v>1371.26</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B74" t="n">
+        <v>40</v>
+      </c>
+      <c r="C74" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D74" t="n">
+        <v>1093.47</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B75" t="n">
+        <v>360</v>
+      </c>
+      <c r="C75" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D75" t="n">
+        <v>7017.48</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B76" t="n">
+        <v>530</v>
+      </c>
+      <c r="C76" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D76" t="n">
+        <v>180.08</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B77" t="n">
+        <v>1137</v>
+      </c>
+      <c r="C77" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D77" t="n">
+        <v>2833.69</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B78" t="n">
+        <v>1293</v>
+      </c>
+      <c r="C78" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D78" t="n">
+        <v>3201.32</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B79" t="n">
+        <v>1293</v>
+      </c>
+      <c r="C79" t="n">
+        <v>601</v>
+      </c>
+      <c r="D79" t="n">
+        <v>456.47</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B80" t="n">
+        <v>2118</v>
+      </c>
+      <c r="C80" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D80" t="n">
+        <v>311.54</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B81" t="n">
+        <v>559</v>
+      </c>
+      <c r="C81" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D81" t="n">
+        <v>512.59</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B82" t="n">
+        <v>89</v>
+      </c>
+      <c r="C82" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D82" t="n">
+        <v>1506.42</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B83" t="n">
+        <v>131</v>
+      </c>
+      <c r="C83" t="n">
+        <v>27</v>
+      </c>
+      <c r="D83" t="n">
+        <v>211.41</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B84" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C84" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D84" t="n">
+        <v>1943.54</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B85" t="n">
+        <v>1299</v>
+      </c>
+      <c r="C85" t="n">
+        <v>27</v>
+      </c>
+      <c r="D85" t="n">
+        <v>262.02</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B86" t="n">
+        <v>131</v>
+      </c>
+      <c r="C86" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D86" t="n">
+        <v>609.86</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B87" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C87" t="n">
+        <v>58</v>
+      </c>
+      <c r="D87" t="n">
+        <v>648.71</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B88" t="n">
+        <v>40</v>
+      </c>
+      <c r="C88" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D88" t="n">
+        <v>733.37</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B89" t="n">
+        <v>40</v>
+      </c>
+      <c r="C89" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D89" t="n">
+        <v>2529.31</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B90" t="n">
+        <v>626</v>
+      </c>
+      <c r="C90" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D90" t="n">
+        <v>13218.02</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B91" t="n">
+        <v>363</v>
+      </c>
+      <c r="C91" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D91" t="n">
+        <v>739.17</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B92" t="n">
+        <v>675</v>
+      </c>
+      <c r="C92" t="n">
+        <v>1898</v>
+      </c>
+      <c r="D92" t="n">
+        <v>107.13</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B93" t="n">
+        <v>636</v>
+      </c>
+      <c r="C93" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D93" t="n">
+        <v>5631.89</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B94" t="n">
+        <v>1075</v>
+      </c>
+      <c r="C94" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D94" t="n">
+        <v>421.29</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B95" t="n">
+        <v>2245</v>
+      </c>
+      <c r="C95" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D95" t="n">
+        <v>883.75</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B96" t="n">
+        <v>477</v>
+      </c>
+      <c r="C96" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D96" t="n">
+        <v>994.15</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B97" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C97" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D97" t="n">
+        <v>2931.07</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B98" t="n">
+        <v>2118</v>
+      </c>
+      <c r="C98" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D98" t="n">
+        <v>2646.39</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B99" t="n">
+        <v>2680</v>
+      </c>
+      <c r="C99" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D99" t="n">
+        <v>824.67</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B100" t="n">
+        <v>1653</v>
+      </c>
+      <c r="C100" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D100" t="n">
+        <v>2848.57</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B101" t="n">
+        <v>629</v>
+      </c>
+      <c r="C101" t="n">
+        <v>675</v>
+      </c>
+      <c r="D101" t="n">
+        <v>267.79</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B102" t="n">
+        <v>559</v>
+      </c>
+      <c r="C102" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D102" t="n">
+        <v>1562.5</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B103" t="n">
+        <v>1465</v>
+      </c>
+      <c r="C103" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D103" t="n">
+        <v>9346.120000000001</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B104" t="n">
+        <v>2550</v>
+      </c>
+      <c r="C104" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D104" t="n">
+        <v>321.05</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B105" t="n">
+        <v>1756</v>
+      </c>
+      <c r="C105" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D105" t="n">
+        <v>2445</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B106" t="n">
+        <v>363</v>
+      </c>
+      <c r="C106" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D106" t="n">
+        <v>649.08</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B107" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C107" t="n">
+        <v>874</v>
+      </c>
+      <c r="D107" t="n">
+        <v>1183.42</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B108" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C108" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D108" t="n">
+        <v>1512.17</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B109" t="n">
+        <v>2681</v>
+      </c>
+      <c r="C109" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D109" t="n">
+        <v>2775.8</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B110" t="n">
+        <v>535</v>
+      </c>
+      <c r="C110" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D110" t="n">
+        <v>2806.71</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B111" t="n">
+        <v>2330</v>
+      </c>
+      <c r="C111" t="n">
+        <v>1954</v>
+      </c>
+      <c r="D111" t="n">
+        <v>1923.09</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B112" t="n">
+        <v>363</v>
+      </c>
+      <c r="C112" t="n">
+        <v>1898</v>
+      </c>
+      <c r="D112" t="n">
+        <v>1058.27</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B113" t="n">
+        <v>2709</v>
+      </c>
+      <c r="C113" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D113" t="n">
+        <v>1667.47</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B114" t="n">
+        <v>1137</v>
+      </c>
+      <c r="C114" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D114" t="n">
+        <v>3185.1</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B115" t="n">
+        <v>2251</v>
+      </c>
+      <c r="C115" t="n">
+        <v>3403</v>
+      </c>
+      <c r="D115" t="n">
+        <v>510.18</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B116" t="n">
+        <v>483</v>
+      </c>
+      <c r="C116" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D116" t="n">
         <v>720.66</v>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E116" t="inlineStr">
         <is>
           <t>FORÇA DE VENDAS</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 13:30:03
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E116"/>
+  <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,7 +489,7 @@
         <v>8888</v>
       </c>
       <c r="D3" t="n">
-        <v>22505.79</v>
+        <v>24542.62</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -521,17 +521,17 @@
         <v>46217</v>
       </c>
       <c r="B5" t="n">
-        <v>2015</v>
+        <v>1993</v>
       </c>
       <c r="C5" t="n">
-        <v>2571</v>
+        <v>8888</v>
       </c>
       <c r="D5" t="n">
-        <v>679.9</v>
+        <v>1785.44</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -540,17 +540,17 @@
         <v>46217</v>
       </c>
       <c r="B6" t="n">
-        <v>1293</v>
+        <v>1102</v>
       </c>
       <c r="C6" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D6" t="n">
-        <v>1337.87</v>
+        <v>1264.43</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -559,17 +559,17 @@
         <v>46217</v>
       </c>
       <c r="B7" t="n">
-        <v>1102</v>
+        <v>2015</v>
       </c>
       <c r="C7" t="n">
-        <v>8888</v>
+        <v>2571</v>
       </c>
       <c r="D7" t="n">
-        <v>1199.81</v>
+        <v>679.9</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -578,17 +578,17 @@
         <v>46217</v>
       </c>
       <c r="B8" t="n">
-        <v>89</v>
+        <v>1293</v>
       </c>
       <c r="C8" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D8" t="n">
-        <v>4572.01</v>
+        <v>1337.87</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -597,13 +597,13 @@
         <v>46217</v>
       </c>
       <c r="B9" t="n">
-        <v>2768</v>
+        <v>89</v>
       </c>
       <c r="C9" t="n">
         <v>8888</v>
       </c>
       <c r="D9" t="n">
-        <v>3436.6</v>
+        <v>4572.01</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -616,17 +616,17 @@
         <v>46217</v>
       </c>
       <c r="B10" t="n">
-        <v>949</v>
+        <v>2768</v>
       </c>
       <c r="C10" t="n">
-        <v>1258</v>
+        <v>8888</v>
       </c>
       <c r="D10" t="n">
-        <v>196.87</v>
+        <v>3436.6</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -635,17 +635,17 @@
         <v>46217</v>
       </c>
       <c r="B11" t="n">
-        <v>1756</v>
+        <v>949</v>
       </c>
       <c r="C11" t="n">
-        <v>8888</v>
+        <v>1258</v>
       </c>
       <c r="D11" t="n">
-        <v>1799.7</v>
+        <v>196.87</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -654,17 +654,17 @@
         <v>46217</v>
       </c>
       <c r="B12" t="n">
-        <v>285</v>
+        <v>1756</v>
       </c>
       <c r="C12" t="n">
         <v>8888</v>
       </c>
       <c r="D12" t="n">
-        <v>1081.17</v>
+        <v>1799.7</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -673,13 +673,13 @@
         <v>46217</v>
       </c>
       <c r="B13" t="n">
-        <v>610</v>
+        <v>285</v>
       </c>
       <c r="C13" t="n">
         <v>8888</v>
       </c>
       <c r="D13" t="n">
-        <v>590.08</v>
+        <v>1081.17</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -692,17 +692,17 @@
         <v>46217</v>
       </c>
       <c r="B14" t="n">
-        <v>2755</v>
+        <v>610</v>
       </c>
       <c r="C14" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D14" t="n">
-        <v>1133.17</v>
+        <v>590.08</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -711,17 +711,17 @@
         <v>46217</v>
       </c>
       <c r="B15" t="n">
-        <v>2767</v>
+        <v>619</v>
       </c>
       <c r="C15" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D15" t="n">
-        <v>5000.2</v>
+        <v>236.34</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -730,17 +730,17 @@
         <v>46217</v>
       </c>
       <c r="B16" t="n">
-        <v>2767</v>
+        <v>2755</v>
       </c>
       <c r="C16" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D16" t="n">
-        <v>1175.73</v>
+        <v>1133.17</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -749,17 +749,17 @@
         <v>46217</v>
       </c>
       <c r="B17" t="n">
-        <v>1063</v>
+        <v>2767</v>
       </c>
       <c r="C17" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D17" t="n">
-        <v>1251.14</v>
+        <v>5000.2</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
         <v>46217</v>
       </c>
       <c r="B18" t="n">
-        <v>325</v>
+        <v>559</v>
       </c>
       <c r="C18" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D18" t="n">
-        <v>868.83</v>
+        <v>517.0700000000001</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -787,17 +787,17 @@
         <v>46217</v>
       </c>
       <c r="B19" t="n">
-        <v>610</v>
+        <v>2767</v>
       </c>
       <c r="C19" t="n">
         <v>8888</v>
       </c>
       <c r="D19" t="n">
-        <v>235.34</v>
+        <v>1175.73</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -806,17 +806,17 @@
         <v>46217</v>
       </c>
       <c r="B20" t="n">
-        <v>1906</v>
+        <v>1063</v>
       </c>
       <c r="C20" t="n">
         <v>8888</v>
       </c>
       <c r="D20" t="n">
-        <v>889.22</v>
+        <v>1251.14</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -825,13 +825,13 @@
         <v>46217</v>
       </c>
       <c r="B21" t="n">
-        <v>40</v>
+        <v>325</v>
       </c>
       <c r="C21" t="n">
         <v>58</v>
       </c>
       <c r="D21" t="n">
-        <v>325.04</v>
+        <v>868.83</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -844,17 +844,17 @@
         <v>46217</v>
       </c>
       <c r="B22" t="n">
-        <v>1117</v>
+        <v>610</v>
       </c>
       <c r="C22" t="n">
         <v>8888</v>
       </c>
       <c r="D22" t="n">
-        <v>349.47</v>
+        <v>235.34</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -863,17 +863,17 @@
         <v>46217</v>
       </c>
       <c r="B23" t="n">
-        <v>949</v>
+        <v>1906</v>
       </c>
       <c r="C23" t="n">
-        <v>998</v>
+        <v>8888</v>
       </c>
       <c r="D23" t="n">
-        <v>129.85</v>
+        <v>889.22</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -882,13 +882,13 @@
         <v>46217</v>
       </c>
       <c r="B24" t="n">
-        <v>2250</v>
+        <v>424</v>
       </c>
       <c r="C24" t="n">
         <v>8888</v>
       </c>
       <c r="D24" t="n">
-        <v>3180.11</v>
+        <v>2575.64</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -901,17 +901,17 @@
         <v>46217</v>
       </c>
       <c r="B25" t="n">
-        <v>2507</v>
+        <v>40</v>
       </c>
       <c r="C25" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D25" t="n">
-        <v>4167.12</v>
+        <v>325.04</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
         <v>46217</v>
       </c>
       <c r="B26" t="n">
-        <v>664</v>
+        <v>1117</v>
       </c>
       <c r="C26" t="n">
         <v>8888</v>
       </c>
       <c r="D26" t="n">
-        <v>3523.8</v>
+        <v>349.47</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -939,13 +939,13 @@
         <v>46217</v>
       </c>
       <c r="B27" t="n">
-        <v>1906</v>
+        <v>949</v>
       </c>
       <c r="C27" t="n">
-        <v>1954</v>
+        <v>998</v>
       </c>
       <c r="D27" t="n">
-        <v>1445.21</v>
+        <v>129.85</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -958,17 +958,17 @@
         <v>46217</v>
       </c>
       <c r="B28" t="n">
-        <v>1075</v>
+        <v>2250</v>
       </c>
       <c r="C28" t="n">
         <v>8888</v>
       </c>
       <c r="D28" t="n">
-        <v>470.95</v>
+        <v>3627.44</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -977,17 +977,17 @@
         <v>46217</v>
       </c>
       <c r="B29" t="n">
-        <v>2696</v>
+        <v>2507</v>
       </c>
       <c r="C29" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D29" t="n">
-        <v>677.76</v>
+        <v>4167.12</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -996,17 +996,17 @@
         <v>46217</v>
       </c>
       <c r="B30" t="n">
-        <v>360</v>
+        <v>664</v>
       </c>
       <c r="C30" t="n">
-        <v>546</v>
+        <v>8888</v>
       </c>
       <c r="D30" t="n">
-        <v>4515.36</v>
+        <v>3523.8</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1015,17 +1015,17 @@
         <v>46217</v>
       </c>
       <c r="B31" t="n">
-        <v>1293</v>
+        <v>1906</v>
       </c>
       <c r="C31" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D31" t="n">
-        <v>381.82</v>
+        <v>1445.21</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1034,13 +1034,13 @@
         <v>46217</v>
       </c>
       <c r="B32" t="n">
-        <v>2663</v>
+        <v>1075</v>
       </c>
       <c r="C32" t="n">
         <v>8888</v>
       </c>
       <c r="D32" t="n">
-        <v>2146.08</v>
+        <v>470.95</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1053,17 +1053,17 @@
         <v>46217</v>
       </c>
       <c r="B33" t="n">
-        <v>675</v>
+        <v>2696</v>
       </c>
       <c r="C33" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D33" t="n">
-        <v>289.67</v>
+        <v>677.76</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1072,17 +1072,17 @@
         <v>46217</v>
       </c>
       <c r="B34" t="n">
-        <v>1063</v>
+        <v>360</v>
       </c>
       <c r="C34" t="n">
-        <v>8888</v>
+        <v>546</v>
       </c>
       <c r="D34" t="n">
-        <v>1902.46</v>
+        <v>4515.36</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1091,13 +1091,13 @@
         <v>46217</v>
       </c>
       <c r="B35" t="n">
-        <v>1392</v>
+        <v>1293</v>
       </c>
       <c r="C35" t="n">
         <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>814.61</v>
+        <v>381.82</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1110,17 +1110,17 @@
         <v>46217</v>
       </c>
       <c r="B36" t="n">
-        <v>360</v>
+        <v>2663</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>749.13</v>
+        <v>2146.08</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1129,17 @@
         <v>46217</v>
       </c>
       <c r="B37" t="n">
-        <v>2491</v>
+        <v>675</v>
       </c>
       <c r="C37" t="n">
         <v>8888</v>
       </c>
       <c r="D37" t="n">
-        <v>398.66</v>
+        <v>289.67</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1148,17 +1148,17 @@
         <v>46217</v>
       </c>
       <c r="B38" t="n">
-        <v>949</v>
+        <v>1063</v>
       </c>
       <c r="C38" t="n">
-        <v>1134</v>
+        <v>8888</v>
       </c>
       <c r="D38" t="n">
-        <v>327.6</v>
+        <v>1902.46</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1167,13 +1167,13 @@
         <v>46217</v>
       </c>
       <c r="B39" t="n">
-        <v>326</v>
+        <v>1392</v>
       </c>
       <c r="C39" t="n">
         <v>8888</v>
       </c>
       <c r="D39" t="n">
-        <v>212.63</v>
+        <v>814.61</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1186,13 +1186,13 @@
         <v>46217</v>
       </c>
       <c r="B40" t="n">
-        <v>1116</v>
+        <v>360</v>
       </c>
       <c r="C40" t="n">
         <v>8888</v>
       </c>
       <c r="D40" t="n">
-        <v>971.6</v>
+        <v>749.13</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1205,17 +1205,17 @@
         <v>46217</v>
       </c>
       <c r="B41" t="n">
-        <v>325</v>
+        <v>2491</v>
       </c>
       <c r="C41" t="n">
         <v>8888</v>
       </c>
       <c r="D41" t="n">
-        <v>538.37</v>
+        <v>398.66</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1224,13 +1224,13 @@
         <v>46217</v>
       </c>
       <c r="B42" t="n">
-        <v>1293</v>
+        <v>949</v>
       </c>
       <c r="C42" t="n">
-        <v>1898</v>
+        <v>1134</v>
       </c>
       <c r="D42" t="n">
-        <v>3534.85</v>
+        <v>327.6</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1243,13 +1243,13 @@
         <v>46217</v>
       </c>
       <c r="B43" t="n">
-        <v>1983</v>
+        <v>326</v>
       </c>
       <c r="C43" t="n">
         <v>8888</v>
       </c>
       <c r="D43" t="n">
-        <v>412.16</v>
+        <v>212.63</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1262,17 +1262,17 @@
         <v>46217</v>
       </c>
       <c r="B44" t="n">
-        <v>451</v>
+        <v>131</v>
       </c>
       <c r="C44" t="n">
         <v>8888</v>
       </c>
       <c r="D44" t="n">
-        <v>2583.46</v>
+        <v>360.06</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1281,13 +1281,13 @@
         <v>46217</v>
       </c>
       <c r="B45" t="n">
-        <v>2767</v>
+        <v>2279</v>
       </c>
       <c r="C45" t="n">
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>596.88</v>
+        <v>1034.25</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1300,13 +1300,13 @@
         <v>46217</v>
       </c>
       <c r="B46" t="n">
-        <v>1063</v>
+        <v>1116</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>352.87</v>
+        <v>971.6</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1319,17 +1319,17 @@
         <v>46217</v>
       </c>
       <c r="B47" t="n">
-        <v>58</v>
+        <v>131</v>
       </c>
       <c r="C47" t="n">
         <v>8888</v>
       </c>
       <c r="D47" t="n">
-        <v>2637.19</v>
+        <v>1528.41</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1338,17 +1338,17 @@
         <v>46217</v>
       </c>
       <c r="B48" t="n">
-        <v>2211</v>
+        <v>325</v>
       </c>
       <c r="C48" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D48" t="n">
-        <v>967.05</v>
+        <v>538.37</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1357,17 +1357,17 @@
         <v>46217</v>
       </c>
       <c r="B49" t="n">
-        <v>629</v>
+        <v>1293</v>
       </c>
       <c r="C49" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D49" t="n">
-        <v>277.36</v>
+        <v>3534.85</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1376,17 +1376,17 @@
         <v>46217</v>
       </c>
       <c r="B50" t="n">
-        <v>629</v>
+        <v>1983</v>
       </c>
       <c r="C50" t="n">
         <v>8888</v>
       </c>
       <c r="D50" t="n">
-        <v>2049.78</v>
+        <v>412.16</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1395,17 +1395,17 @@
         <v>46217</v>
       </c>
       <c r="B51" t="n">
-        <v>949</v>
+        <v>451</v>
       </c>
       <c r="C51" t="n">
-        <v>1762</v>
+        <v>8888</v>
       </c>
       <c r="D51" t="n">
-        <v>325.65</v>
+        <v>2583.46</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
         <v>46217</v>
       </c>
       <c r="B52" t="n">
-        <v>2463</v>
+        <v>2767</v>
       </c>
       <c r="C52" t="n">
         <v>8888</v>
       </c>
       <c r="D52" t="n">
-        <v>8336.43</v>
+        <v>596.88</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1433,13 +1433,13 @@
         <v>46217</v>
       </c>
       <c r="B53" t="n">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="C53" t="n">
         <v>8888</v>
       </c>
       <c r="D53" t="n">
-        <v>1513.21</v>
+        <v>352.87</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1452,13 +1452,13 @@
         <v>46217</v>
       </c>
       <c r="B54" t="n">
-        <v>1478</v>
+        <v>629</v>
       </c>
       <c r="C54" t="n">
         <v>8888</v>
       </c>
       <c r="D54" t="n">
-        <v>1294.76</v>
+        <v>559.15</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1471,17 +1471,17 @@
         <v>46217</v>
       </c>
       <c r="B55" t="n">
-        <v>358</v>
+        <v>58</v>
       </c>
       <c r="C55" t="n">
         <v>8888</v>
       </c>
       <c r="D55" t="n">
-        <v>1918.33</v>
+        <v>2637.19</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1490,17 +1490,17 @@
         <v>46217</v>
       </c>
       <c r="B56" t="n">
-        <v>2107</v>
+        <v>2211</v>
       </c>
       <c r="C56" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D56" t="n">
-        <v>2745.11</v>
+        <v>967.05</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1509,13 +1509,13 @@
         <v>46217</v>
       </c>
       <c r="B57" t="n">
-        <v>675</v>
+        <v>629</v>
       </c>
       <c r="C57" t="n">
         <v>8888</v>
       </c>
       <c r="D57" t="n">
-        <v>275.17</v>
+        <v>2049.78</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1528,13 +1528,13 @@
         <v>46217</v>
       </c>
       <c r="B58" t="n">
-        <v>451</v>
+        <v>949</v>
       </c>
       <c r="C58" t="n">
-        <v>3403</v>
+        <v>1762</v>
       </c>
       <c r="D58" t="n">
-        <v>327.28</v>
+        <v>325.65</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1547,17 +1547,17 @@
         <v>46217</v>
       </c>
       <c r="B59" t="n">
-        <v>2571</v>
+        <v>2463</v>
       </c>
       <c r="C59" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D59" t="n">
-        <v>2202.75</v>
+        <v>8336.43</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1566,17 +1566,17 @@
         <v>46217</v>
       </c>
       <c r="B60" t="n">
-        <v>610</v>
+        <v>1064</v>
       </c>
       <c r="C60" t="n">
         <v>8888</v>
       </c>
       <c r="D60" t="n">
-        <v>335.61</v>
+        <v>1513.21</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1585,17 +1585,17 @@
         <v>46217</v>
       </c>
       <c r="B61" t="n">
-        <v>1108</v>
+        <v>1478</v>
       </c>
       <c r="C61" t="n">
         <v>8888</v>
       </c>
       <c r="D61" t="n">
-        <v>508.54</v>
+        <v>1294.76</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1604,17 +1604,17 @@
         <v>46217</v>
       </c>
       <c r="B62" t="n">
-        <v>341</v>
+        <v>358</v>
       </c>
       <c r="C62" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D62" t="n">
-        <v>366.88</v>
+        <v>1918.33</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1623,17 +1623,17 @@
         <v>46217</v>
       </c>
       <c r="B63" t="n">
-        <v>1653</v>
+        <v>2107</v>
       </c>
       <c r="C63" t="n">
         <v>8888</v>
       </c>
       <c r="D63" t="n">
-        <v>4383.69</v>
+        <v>2745.11</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1642,17 +1642,17 @@
         <v>46217</v>
       </c>
       <c r="B64" t="n">
-        <v>663</v>
+        <v>675</v>
       </c>
       <c r="C64" t="n">
         <v>8888</v>
       </c>
       <c r="D64" t="n">
-        <v>824.5599999999999</v>
+        <v>275.17</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1661,17 +1661,17 @@
         <v>46217</v>
       </c>
       <c r="B65" t="n">
-        <v>58</v>
+        <v>2279</v>
       </c>
       <c r="C65" t="n">
         <v>8888</v>
       </c>
       <c r="D65" t="n">
-        <v>660.1</v>
+        <v>1165.17</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1680,13 +1680,13 @@
         <v>46217</v>
       </c>
       <c r="B66" t="n">
-        <v>429</v>
+        <v>451</v>
       </c>
       <c r="C66" t="n">
-        <v>2571</v>
+        <v>3403</v>
       </c>
       <c r="D66" t="n">
-        <v>667.12</v>
+        <v>327.28</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1699,17 +1699,17 @@
         <v>46217</v>
       </c>
       <c r="B67" t="n">
-        <v>483</v>
+        <v>2571</v>
       </c>
       <c r="C67" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D67" t="n">
-        <v>938.34</v>
+        <v>2202.75</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1718,17 +1718,17 @@
         <v>46217</v>
       </c>
       <c r="B68" t="n">
-        <v>2709</v>
+        <v>610</v>
       </c>
       <c r="C68" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D68" t="n">
-        <v>1663.5</v>
+        <v>335.61</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1737,17 +1737,17 @@
         <v>46217</v>
       </c>
       <c r="B69" t="n">
-        <v>1937</v>
+        <v>1108</v>
       </c>
       <c r="C69" t="n">
         <v>8888</v>
       </c>
       <c r="D69" t="n">
-        <v>1332.89</v>
+        <v>508.54</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1756,13 +1756,13 @@
         <v>46217</v>
       </c>
       <c r="B70" t="n">
-        <v>429</v>
+        <v>341</v>
       </c>
       <c r="C70" t="n">
-        <v>1281</v>
+        <v>58</v>
       </c>
       <c r="D70" t="n">
-        <v>1333.52</v>
+        <v>366.88</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -1775,17 +1775,17 @@
         <v>46217</v>
       </c>
       <c r="B71" t="n">
-        <v>2211</v>
+        <v>1653</v>
       </c>
       <c r="C71" t="n">
         <v>8888</v>
       </c>
       <c r="D71" t="n">
-        <v>797.61</v>
+        <v>4383.69</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1794,13 +1794,13 @@
         <v>46217</v>
       </c>
       <c r="B72" t="n">
-        <v>1064</v>
+        <v>619</v>
       </c>
       <c r="C72" t="n">
         <v>8888</v>
       </c>
       <c r="D72" t="n">
-        <v>2383.39</v>
+        <v>779.87</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -1813,17 +1813,17 @@
         <v>46217</v>
       </c>
       <c r="B73" t="n">
-        <v>451</v>
+        <v>663</v>
       </c>
       <c r="C73" t="n">
         <v>8888</v>
       </c>
       <c r="D73" t="n">
-        <v>1371.26</v>
+        <v>824.5599999999999</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1832,17 +1832,17 @@
         <v>46217</v>
       </c>
       <c r="B74" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="C74" t="n">
         <v>8888</v>
       </c>
       <c r="D74" t="n">
-        <v>1093.47</v>
+        <v>660.1</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1851,17 +1851,17 @@
         <v>46217</v>
       </c>
       <c r="B75" t="n">
-        <v>360</v>
+        <v>429</v>
       </c>
       <c r="C75" t="n">
-        <v>8888</v>
+        <v>2571</v>
       </c>
       <c r="D75" t="n">
-        <v>7017.48</v>
+        <v>667.12</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1870,13 +1870,13 @@
         <v>46217</v>
       </c>
       <c r="B76" t="n">
-        <v>530</v>
+        <v>483</v>
       </c>
       <c r="C76" t="n">
         <v>8888</v>
       </c>
       <c r="D76" t="n">
-        <v>180.08</v>
+        <v>1290.28</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -1889,17 +1889,17 @@
         <v>46217</v>
       </c>
       <c r="B77" t="n">
-        <v>1137</v>
+        <v>2709</v>
       </c>
       <c r="C77" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D77" t="n">
-        <v>2833.69</v>
+        <v>1663.5</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1908,17 +1908,17 @@
         <v>46217</v>
       </c>
       <c r="B78" t="n">
-        <v>1293</v>
+        <v>1937</v>
       </c>
       <c r="C78" t="n">
         <v>8888</v>
       </c>
       <c r="D78" t="n">
-        <v>3201.32</v>
+        <v>1332.89</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1927,13 +1927,13 @@
         <v>46217</v>
       </c>
       <c r="B79" t="n">
-        <v>1293</v>
+        <v>429</v>
       </c>
       <c r="C79" t="n">
-        <v>601</v>
+        <v>1281</v>
       </c>
       <c r="D79" t="n">
-        <v>456.47</v>
+        <v>1333.52</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -1946,17 +1946,17 @@
         <v>46217</v>
       </c>
       <c r="B80" t="n">
-        <v>2118</v>
+        <v>2211</v>
       </c>
       <c r="C80" t="n">
         <v>8888</v>
       </c>
       <c r="D80" t="n">
-        <v>311.54</v>
+        <v>797.61</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1965,13 +1965,13 @@
         <v>46217</v>
       </c>
       <c r="B81" t="n">
-        <v>559</v>
+        <v>131</v>
       </c>
       <c r="C81" t="n">
         <v>8888</v>
       </c>
       <c r="D81" t="n">
-        <v>512.59</v>
+        <v>2340.29</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -1984,17 +1984,17 @@
         <v>46217</v>
       </c>
       <c r="B82" t="n">
-        <v>89</v>
+        <v>131</v>
       </c>
       <c r="C82" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D82" t="n">
-        <v>1506.42</v>
+        <v>669.39</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2003,17 +2003,17 @@
         <v>46217</v>
       </c>
       <c r="B83" t="n">
-        <v>131</v>
+        <v>1064</v>
       </c>
       <c r="C83" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D83" t="n">
-        <v>211.41</v>
+        <v>2383.39</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2022,17 +2022,17 @@
         <v>46217</v>
       </c>
       <c r="B84" t="n">
-        <v>2250</v>
+        <v>2251</v>
       </c>
       <c r="C84" t="n">
         <v>8888</v>
       </c>
       <c r="D84" t="n">
-        <v>1943.54</v>
+        <v>797.58</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2041,17 +2041,17 @@
         <v>46217</v>
       </c>
       <c r="B85" t="n">
-        <v>1299</v>
+        <v>451</v>
       </c>
       <c r="C85" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D85" t="n">
-        <v>262.02</v>
+        <v>1371.26</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2060,17 +2060,17 @@
         <v>46217</v>
       </c>
       <c r="B86" t="n">
-        <v>131</v>
+        <v>40</v>
       </c>
       <c r="C86" t="n">
         <v>8888</v>
       </c>
       <c r="D86" t="n">
-        <v>609.86</v>
+        <v>1093.47</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2079,17 +2079,17 @@
         <v>46217</v>
       </c>
       <c r="B87" t="n">
-        <v>2651</v>
+        <v>360</v>
       </c>
       <c r="C87" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D87" t="n">
-        <v>648.71</v>
+        <v>7017.48</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2098,17 +2098,17 @@
         <v>46217</v>
       </c>
       <c r="B88" t="n">
-        <v>40</v>
+        <v>530</v>
       </c>
       <c r="C88" t="n">
         <v>8888</v>
       </c>
       <c r="D88" t="n">
-        <v>733.37</v>
+        <v>180.08</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2117,17 +2117,17 @@
         <v>46217</v>
       </c>
       <c r="B89" t="n">
-        <v>40</v>
+        <v>1137</v>
       </c>
       <c r="C89" t="n">
         <v>8888</v>
       </c>
       <c r="D89" t="n">
-        <v>2529.31</v>
+        <v>2833.69</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2136,17 +2136,17 @@
         <v>46217</v>
       </c>
       <c r="B90" t="n">
-        <v>626</v>
+        <v>1293</v>
       </c>
       <c r="C90" t="n">
         <v>8888</v>
       </c>
       <c r="D90" t="n">
-        <v>13218.02</v>
+        <v>3201.32</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2155,17 +2155,17 @@
         <v>46217</v>
       </c>
       <c r="B91" t="n">
-        <v>363</v>
+        <v>1293</v>
       </c>
       <c r="C91" t="n">
-        <v>8888</v>
+        <v>601</v>
       </c>
       <c r="D91" t="n">
-        <v>739.17</v>
+        <v>456.47</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2174,17 +2174,17 @@
         <v>46217</v>
       </c>
       <c r="B92" t="n">
-        <v>675</v>
+        <v>2118</v>
       </c>
       <c r="C92" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D92" t="n">
-        <v>107.13</v>
+        <v>311.54</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2193,17 +2193,17 @@
         <v>46217</v>
       </c>
       <c r="B93" t="n">
-        <v>636</v>
+        <v>424</v>
       </c>
       <c r="C93" t="n">
         <v>8888</v>
       </c>
       <c r="D93" t="n">
-        <v>5631.89</v>
+        <v>349.68</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2212,13 +2212,13 @@
         <v>46217</v>
       </c>
       <c r="B94" t="n">
-        <v>1075</v>
+        <v>559</v>
       </c>
       <c r="C94" t="n">
         <v>8888</v>
       </c>
       <c r="D94" t="n">
-        <v>421.29</v>
+        <v>1064.63</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2231,17 +2231,17 @@
         <v>46217</v>
       </c>
       <c r="B95" t="n">
-        <v>2245</v>
+        <v>89</v>
       </c>
       <c r="C95" t="n">
         <v>8888</v>
       </c>
       <c r="D95" t="n">
-        <v>883.75</v>
+        <v>1506.42</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2250,17 +2250,17 @@
         <v>46217</v>
       </c>
       <c r="B96" t="n">
-        <v>477</v>
+        <v>2250</v>
       </c>
       <c r="C96" t="n">
         <v>8888</v>
       </c>
       <c r="D96" t="n">
-        <v>994.15</v>
+        <v>1943.54</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2269,17 +2269,17 @@
         <v>46217</v>
       </c>
       <c r="B97" t="n">
-        <v>2015</v>
+        <v>1299</v>
       </c>
       <c r="C97" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D97" t="n">
-        <v>2931.07</v>
+        <v>262.02</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2288,17 +2288,17 @@
         <v>46217</v>
       </c>
       <c r="B98" t="n">
-        <v>2118</v>
+        <v>2651</v>
       </c>
       <c r="C98" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D98" t="n">
-        <v>2646.39</v>
+        <v>648.71</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2307,13 +2307,13 @@
         <v>46217</v>
       </c>
       <c r="B99" t="n">
-        <v>2680</v>
+        <v>40</v>
       </c>
       <c r="C99" t="n">
         <v>8888</v>
       </c>
       <c r="D99" t="n">
-        <v>824.67</v>
+        <v>733.37</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2326,17 +2326,17 @@
         <v>46217</v>
       </c>
       <c r="B100" t="n">
-        <v>1653</v>
+        <v>40</v>
       </c>
       <c r="C100" t="n">
         <v>8888</v>
       </c>
       <c r="D100" t="n">
-        <v>2848.57</v>
+        <v>2529.31</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2345,17 +2345,17 @@
         <v>46217</v>
       </c>
       <c r="B101" t="n">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="C101" t="n">
-        <v>675</v>
+        <v>8888</v>
       </c>
       <c r="D101" t="n">
-        <v>267.79</v>
+        <v>13218.02</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2364,17 +2364,17 @@
         <v>46217</v>
       </c>
       <c r="B102" t="n">
-        <v>559</v>
+        <v>363</v>
       </c>
       <c r="C102" t="n">
         <v>8888</v>
       </c>
       <c r="D102" t="n">
-        <v>1562.5</v>
+        <v>739.17</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2383,17 +2383,17 @@
         <v>46217</v>
       </c>
       <c r="B103" t="n">
-        <v>1465</v>
+        <v>675</v>
       </c>
       <c r="C103" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D103" t="n">
-        <v>9346.120000000001</v>
+        <v>107.13</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2402,17 +2402,17 @@
         <v>46217</v>
       </c>
       <c r="B104" t="n">
-        <v>2550</v>
+        <v>636</v>
       </c>
       <c r="C104" t="n">
         <v>8888</v>
       </c>
       <c r="D104" t="n">
-        <v>321.05</v>
+        <v>5631.89</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2421,13 +2421,13 @@
         <v>46217</v>
       </c>
       <c r="B105" t="n">
-        <v>1756</v>
+        <v>1075</v>
       </c>
       <c r="C105" t="n">
         <v>8888</v>
       </c>
       <c r="D105" t="n">
-        <v>2445</v>
+        <v>1331.89</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2440,17 +2440,17 @@
         <v>46217</v>
       </c>
       <c r="B106" t="n">
-        <v>363</v>
+        <v>2245</v>
       </c>
       <c r="C106" t="n">
         <v>8888</v>
       </c>
       <c r="D106" t="n">
-        <v>649.08</v>
+        <v>883.75</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2459,17 +2459,17 @@
         <v>46217</v>
       </c>
       <c r="B107" t="n">
-        <v>2698</v>
+        <v>477</v>
       </c>
       <c r="C107" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D107" t="n">
-        <v>1183.42</v>
+        <v>994.15</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2478,13 +2478,13 @@
         <v>46217</v>
       </c>
       <c r="B108" t="n">
-        <v>2250</v>
+        <v>2015</v>
       </c>
       <c r="C108" t="n">
         <v>8888</v>
       </c>
       <c r="D108" t="n">
-        <v>1512.17</v>
+        <v>2931.07</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -2497,17 +2497,17 @@
         <v>46217</v>
       </c>
       <c r="B109" t="n">
-        <v>2681</v>
+        <v>1064</v>
       </c>
       <c r="C109" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D109" t="n">
-        <v>2775.8</v>
+        <v>451.38</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2516,17 +2516,17 @@
         <v>46217</v>
       </c>
       <c r="B110" t="n">
-        <v>535</v>
+        <v>1983</v>
       </c>
       <c r="C110" t="n">
         <v>8888</v>
       </c>
       <c r="D110" t="n">
-        <v>2806.71</v>
+        <v>680.42</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2535,17 +2535,17 @@
         <v>46217</v>
       </c>
       <c r="B111" t="n">
-        <v>2330</v>
+        <v>2118</v>
       </c>
       <c r="C111" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D111" t="n">
-        <v>1923.09</v>
+        <v>2646.39</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2554,17 +2554,17 @@
         <v>46217</v>
       </c>
       <c r="B112" t="n">
-        <v>363</v>
+        <v>2680</v>
       </c>
       <c r="C112" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D112" t="n">
-        <v>1058.27</v>
+        <v>824.67</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2573,13 +2573,13 @@
         <v>46217</v>
       </c>
       <c r="B113" t="n">
-        <v>2709</v>
+        <v>1653</v>
       </c>
       <c r="C113" t="n">
         <v>8888</v>
       </c>
       <c r="D113" t="n">
-        <v>1667.47</v>
+        <v>2848.57</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -2592,17 +2592,17 @@
         <v>46217</v>
       </c>
       <c r="B114" t="n">
-        <v>1137</v>
+        <v>629</v>
       </c>
       <c r="C114" t="n">
-        <v>8888</v>
+        <v>675</v>
       </c>
       <c r="D114" t="n">
-        <v>3185.1</v>
+        <v>267.79</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2611,17 +2611,17 @@
         <v>46217</v>
       </c>
       <c r="B115" t="n">
-        <v>2251</v>
+        <v>559</v>
       </c>
       <c r="C115" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D115" t="n">
-        <v>510.18</v>
+        <v>1562.5</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2630,17 +2630,264 @@
         <v>46217</v>
       </c>
       <c r="B116" t="n">
+        <v>1465</v>
+      </c>
+      <c r="C116" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D116" t="n">
+        <v>9346.120000000001</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B117" t="n">
+        <v>2550</v>
+      </c>
+      <c r="C117" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D117" t="n">
+        <v>321.05</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B118" t="n">
+        <v>1756</v>
+      </c>
+      <c r="C118" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D118" t="n">
+        <v>2445</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B119" t="n">
+        <v>363</v>
+      </c>
+      <c r="C119" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D119" t="n">
+        <v>649.08</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B120" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C120" t="n">
+        <v>874</v>
+      </c>
+      <c r="D120" t="n">
+        <v>1183.42</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B121" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C121" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D121" t="n">
+        <v>1512.17</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B122" t="n">
+        <v>2681</v>
+      </c>
+      <c r="C122" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D122" t="n">
+        <v>2775.8</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B123" t="n">
+        <v>535</v>
+      </c>
+      <c r="C123" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D123" t="n">
+        <v>2806.71</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B124" t="n">
         <v>483</v>
       </c>
-      <c r="C116" t="n">
-        <v>8888</v>
-      </c>
-      <c r="D116" t="n">
-        <v>720.66</v>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>FORÇA DE VENDAS</t>
+      <c r="C124" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D124" t="n">
+        <v>2100.84</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B125" t="n">
+        <v>2330</v>
+      </c>
+      <c r="C125" t="n">
+        <v>1954</v>
+      </c>
+      <c r="D125" t="n">
+        <v>1923.09</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B126" t="n">
+        <v>363</v>
+      </c>
+      <c r="C126" t="n">
+        <v>1898</v>
+      </c>
+      <c r="D126" t="n">
+        <v>1058.27</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B127" t="n">
+        <v>2709</v>
+      </c>
+      <c r="C127" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D127" t="n">
+        <v>1667.47</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B128" t="n">
+        <v>1137</v>
+      </c>
+      <c r="C128" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D128" t="n">
+        <v>3185.1</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B129" t="n">
+        <v>2251</v>
+      </c>
+      <c r="C129" t="n">
+        <v>3403</v>
+      </c>
+      <c r="D129" t="n">
+        <v>510.18</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 14:00:04
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E129"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -603,7 +603,7 @@
         <v>8888</v>
       </c>
       <c r="D9" t="n">
-        <v>4572.01</v>
+        <v>5652.15</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -679,7 +679,7 @@
         <v>8888</v>
       </c>
       <c r="D13" t="n">
-        <v>1081.17</v>
+        <v>2593.28</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1091,17 +1091,17 @@
         <v>46217</v>
       </c>
       <c r="B35" t="n">
-        <v>1293</v>
+        <v>2651</v>
       </c>
       <c r="C35" t="n">
         <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>381.82</v>
+        <v>638.64</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1110,17 @@
         <v>46217</v>
       </c>
       <c r="B36" t="n">
-        <v>2663</v>
+        <v>1293</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>2146.08</v>
+        <v>381.82</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1129,17 @@
         <v>46217</v>
       </c>
       <c r="B37" t="n">
-        <v>675</v>
+        <v>2663</v>
       </c>
       <c r="C37" t="n">
         <v>8888</v>
       </c>
       <c r="D37" t="n">
-        <v>289.67</v>
+        <v>2146.08</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1148,17 +1148,17 @@
         <v>46217</v>
       </c>
       <c r="B38" t="n">
-        <v>1063</v>
+        <v>675</v>
       </c>
       <c r="C38" t="n">
         <v>8888</v>
       </c>
       <c r="D38" t="n">
-        <v>1902.46</v>
+        <v>289.67</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1167,17 +1167,17 @@
         <v>46217</v>
       </c>
       <c r="B39" t="n">
-        <v>1392</v>
+        <v>1063</v>
       </c>
       <c r="C39" t="n">
         <v>8888</v>
       </c>
       <c r="D39" t="n">
-        <v>814.61</v>
+        <v>1902.46</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1186,17 +1186,17 @@
         <v>46217</v>
       </c>
       <c r="B40" t="n">
-        <v>360</v>
+        <v>1392</v>
       </c>
       <c r="C40" t="n">
         <v>8888</v>
       </c>
       <c r="D40" t="n">
-        <v>749.13</v>
+        <v>814.61</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1205,17 +1205,17 @@
         <v>46217</v>
       </c>
       <c r="B41" t="n">
-        <v>2491</v>
+        <v>360</v>
       </c>
       <c r="C41" t="n">
         <v>8888</v>
       </c>
       <c r="D41" t="n">
-        <v>398.66</v>
+        <v>749.13</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1224,17 +1224,17 @@
         <v>46217</v>
       </c>
       <c r="B42" t="n">
-        <v>949</v>
+        <v>2491</v>
       </c>
       <c r="C42" t="n">
-        <v>1134</v>
+        <v>8888</v>
       </c>
       <c r="D42" t="n">
-        <v>327.6</v>
+        <v>398.66</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1243,17 +1243,17 @@
         <v>46217</v>
       </c>
       <c r="B43" t="n">
-        <v>326</v>
+        <v>949</v>
       </c>
       <c r="C43" t="n">
-        <v>8888</v>
+        <v>1134</v>
       </c>
       <c r="D43" t="n">
-        <v>212.63</v>
+        <v>327.6</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1262,13 +1262,13 @@
         <v>46217</v>
       </c>
       <c r="B44" t="n">
-        <v>131</v>
+        <v>326</v>
       </c>
       <c r="C44" t="n">
         <v>8888</v>
       </c>
       <c r="D44" t="n">
-        <v>360.06</v>
+        <v>212.63</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1281,17 +1281,17 @@
         <v>46217</v>
       </c>
       <c r="B45" t="n">
-        <v>2279</v>
+        <v>325</v>
       </c>
       <c r="C45" t="n">
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>1034.25</v>
+        <v>584.27</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1300,17 +1300,17 @@
         <v>46217</v>
       </c>
       <c r="B46" t="n">
-        <v>1116</v>
+        <v>131</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>971.6</v>
+        <v>360.06</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1319,13 +1319,13 @@
         <v>46217</v>
       </c>
       <c r="B47" t="n">
-        <v>131</v>
+        <v>2279</v>
       </c>
       <c r="C47" t="n">
         <v>8888</v>
       </c>
       <c r="D47" t="n">
-        <v>1528.41</v>
+        <v>1034.25</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1338,17 +1338,17 @@
         <v>46217</v>
       </c>
       <c r="B48" t="n">
-        <v>325</v>
+        <v>1116</v>
       </c>
       <c r="C48" t="n">
         <v>8888</v>
       </c>
       <c r="D48" t="n">
-        <v>538.37</v>
+        <v>1293.89</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1357,17 +1357,17 @@
         <v>46217</v>
       </c>
       <c r="B49" t="n">
-        <v>1293</v>
+        <v>131</v>
       </c>
       <c r="C49" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D49" t="n">
-        <v>3534.85</v>
+        <v>1528.41</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1376,17 +1376,17 @@
         <v>46217</v>
       </c>
       <c r="B50" t="n">
-        <v>1983</v>
+        <v>1293</v>
       </c>
       <c r="C50" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D50" t="n">
-        <v>412.16</v>
+        <v>3534.85</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1395,17 +1395,17 @@
         <v>46217</v>
       </c>
       <c r="B51" t="n">
-        <v>451</v>
+        <v>1983</v>
       </c>
       <c r="C51" t="n">
         <v>8888</v>
       </c>
       <c r="D51" t="n">
-        <v>2583.46</v>
+        <v>412.16</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
         <v>46217</v>
       </c>
       <c r="B52" t="n">
-        <v>2767</v>
+        <v>451</v>
       </c>
       <c r="C52" t="n">
         <v>8888</v>
       </c>
       <c r="D52" t="n">
-        <v>596.88</v>
+        <v>2583.46</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1433,17 +1433,17 @@
         <v>46217</v>
       </c>
       <c r="B53" t="n">
-        <v>1063</v>
+        <v>2767</v>
       </c>
       <c r="C53" t="n">
         <v>8888</v>
       </c>
       <c r="D53" t="n">
-        <v>352.87</v>
+        <v>596.88</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1452,13 +1452,13 @@
         <v>46217</v>
       </c>
       <c r="B54" t="n">
-        <v>629</v>
+        <v>1063</v>
       </c>
       <c r="C54" t="n">
         <v>8888</v>
       </c>
       <c r="D54" t="n">
-        <v>559.15</v>
+        <v>352.87</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1471,17 +1471,17 @@
         <v>46217</v>
       </c>
       <c r="B55" t="n">
-        <v>58</v>
+        <v>629</v>
       </c>
       <c r="C55" t="n">
         <v>8888</v>
       </c>
       <c r="D55" t="n">
-        <v>2637.19</v>
+        <v>559.15</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1490,17 +1490,17 @@
         <v>46217</v>
       </c>
       <c r="B56" t="n">
-        <v>2211</v>
+        <v>58</v>
       </c>
       <c r="C56" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D56" t="n">
-        <v>967.05</v>
+        <v>2637.19</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1509,17 +1509,17 @@
         <v>46217</v>
       </c>
       <c r="B57" t="n">
-        <v>629</v>
+        <v>2211</v>
       </c>
       <c r="C57" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D57" t="n">
-        <v>2049.78</v>
+        <v>967.05</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1528,17 +1528,17 @@
         <v>46217</v>
       </c>
       <c r="B58" t="n">
-        <v>949</v>
+        <v>1117</v>
       </c>
       <c r="C58" t="n">
-        <v>1762</v>
+        <v>8888</v>
       </c>
       <c r="D58" t="n">
-        <v>325.65</v>
+        <v>581.51</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1547,17 +1547,17 @@
         <v>46217</v>
       </c>
       <c r="B59" t="n">
-        <v>2463</v>
+        <v>629</v>
       </c>
       <c r="C59" t="n">
         <v>8888</v>
       </c>
       <c r="D59" t="n">
-        <v>8336.43</v>
+        <v>2049.78</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1566,17 +1566,17 @@
         <v>46217</v>
       </c>
       <c r="B60" t="n">
-        <v>1064</v>
+        <v>949</v>
       </c>
       <c r="C60" t="n">
-        <v>8888</v>
+        <v>1762</v>
       </c>
       <c r="D60" t="n">
-        <v>1513.21</v>
+        <v>325.65</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1585,17 +1585,17 @@
         <v>46217</v>
       </c>
       <c r="B61" t="n">
-        <v>1478</v>
+        <v>2463</v>
       </c>
       <c r="C61" t="n">
         <v>8888</v>
       </c>
       <c r="D61" t="n">
-        <v>1294.76</v>
+        <v>8336.43</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1604,13 +1604,13 @@
         <v>46217</v>
       </c>
       <c r="B62" t="n">
-        <v>358</v>
+        <v>1064</v>
       </c>
       <c r="C62" t="n">
         <v>8888</v>
       </c>
       <c r="D62" t="n">
-        <v>1918.33</v>
+        <v>1513.21</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1623,17 +1623,17 @@
         <v>46217</v>
       </c>
       <c r="B63" t="n">
-        <v>2107</v>
+        <v>1478</v>
       </c>
       <c r="C63" t="n">
         <v>8888</v>
       </c>
       <c r="D63" t="n">
-        <v>2745.11</v>
+        <v>1294.76</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1642,17 +1642,17 @@
         <v>46217</v>
       </c>
       <c r="B64" t="n">
-        <v>675</v>
+        <v>358</v>
       </c>
       <c r="C64" t="n">
         <v>8888</v>
       </c>
       <c r="D64" t="n">
-        <v>275.17</v>
+        <v>1918.33</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1661,17 +1661,17 @@
         <v>46217</v>
       </c>
       <c r="B65" t="n">
-        <v>2279</v>
+        <v>2107</v>
       </c>
       <c r="C65" t="n">
         <v>8888</v>
       </c>
       <c r="D65" t="n">
-        <v>1165.17</v>
+        <v>2745.11</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1680,17 +1680,17 @@
         <v>46217</v>
       </c>
       <c r="B66" t="n">
-        <v>451</v>
+        <v>675</v>
       </c>
       <c r="C66" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D66" t="n">
-        <v>327.28</v>
+        <v>275.17</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1699,17 +1699,17 @@
         <v>46217</v>
       </c>
       <c r="B67" t="n">
-        <v>2571</v>
+        <v>2279</v>
       </c>
       <c r="C67" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D67" t="n">
-        <v>2202.75</v>
+        <v>1165.17</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1718,17 +1718,17 @@
         <v>46217</v>
       </c>
       <c r="B68" t="n">
-        <v>610</v>
+        <v>451</v>
       </c>
       <c r="C68" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D68" t="n">
-        <v>335.61</v>
+        <v>327.28</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1737,17 +1737,17 @@
         <v>46217</v>
       </c>
       <c r="B69" t="n">
-        <v>1108</v>
+        <v>2571</v>
       </c>
       <c r="C69" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D69" t="n">
-        <v>508.54</v>
+        <v>2202.75</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1756,17 +1756,17 @@
         <v>46217</v>
       </c>
       <c r="B70" t="n">
-        <v>341</v>
+        <v>610</v>
       </c>
       <c r="C70" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D70" t="n">
-        <v>366.88</v>
+        <v>335.61</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1775,17 @@
         <v>46217</v>
       </c>
       <c r="B71" t="n">
-        <v>1653</v>
+        <v>1108</v>
       </c>
       <c r="C71" t="n">
         <v>8888</v>
       </c>
       <c r="D71" t="n">
-        <v>4383.69</v>
+        <v>508.54</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1794,17 +1794,17 @@
         <v>46217</v>
       </c>
       <c r="B72" t="n">
-        <v>619</v>
+        <v>341</v>
       </c>
       <c r="C72" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D72" t="n">
-        <v>779.87</v>
+        <v>366.88</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1813,13 +1813,13 @@
         <v>46217</v>
       </c>
       <c r="B73" t="n">
-        <v>663</v>
+        <v>1653</v>
       </c>
       <c r="C73" t="n">
         <v>8888</v>
       </c>
       <c r="D73" t="n">
-        <v>824.5599999999999</v>
+        <v>4383.69</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -1832,13 +1832,13 @@
         <v>46217</v>
       </c>
       <c r="B74" t="n">
-        <v>58</v>
+        <v>619</v>
       </c>
       <c r="C74" t="n">
         <v>8888</v>
       </c>
       <c r="D74" t="n">
-        <v>660.1</v>
+        <v>779.87</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -1851,17 +1851,17 @@
         <v>46217</v>
       </c>
       <c r="B75" t="n">
-        <v>429</v>
+        <v>663</v>
       </c>
       <c r="C75" t="n">
-        <v>2571</v>
+        <v>8888</v>
       </c>
       <c r="D75" t="n">
-        <v>667.12</v>
+        <v>824.5599999999999</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1870,17 +1870,17 @@
         <v>46217</v>
       </c>
       <c r="B76" t="n">
-        <v>483</v>
+        <v>58</v>
       </c>
       <c r="C76" t="n">
         <v>8888</v>
       </c>
       <c r="D76" t="n">
-        <v>1290.28</v>
+        <v>660.1</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1889,13 +1889,13 @@
         <v>46217</v>
       </c>
       <c r="B77" t="n">
-        <v>2709</v>
+        <v>429</v>
       </c>
       <c r="C77" t="n">
-        <v>2220</v>
+        <v>2571</v>
       </c>
       <c r="D77" t="n">
-        <v>1663.5</v>
+        <v>667.12</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -1908,13 +1908,13 @@
         <v>46217</v>
       </c>
       <c r="B78" t="n">
-        <v>1937</v>
+        <v>483</v>
       </c>
       <c r="C78" t="n">
         <v>8888</v>
       </c>
       <c r="D78" t="n">
-        <v>1332.89</v>
+        <v>1290.28</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -1927,13 +1927,13 @@
         <v>46217</v>
       </c>
       <c r="B79" t="n">
-        <v>429</v>
+        <v>2709</v>
       </c>
       <c r="C79" t="n">
-        <v>1281</v>
+        <v>2220</v>
       </c>
       <c r="D79" t="n">
-        <v>1333.52</v>
+        <v>1663.5</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -1946,17 +1946,17 @@
         <v>46217</v>
       </c>
       <c r="B80" t="n">
-        <v>2211</v>
+        <v>1937</v>
       </c>
       <c r="C80" t="n">
         <v>8888</v>
       </c>
       <c r="D80" t="n">
-        <v>797.61</v>
+        <v>1332.89</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1965,17 +1965,17 @@
         <v>46217</v>
       </c>
       <c r="B81" t="n">
-        <v>131</v>
+        <v>429</v>
       </c>
       <c r="C81" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D81" t="n">
-        <v>2340.29</v>
+        <v>1333.52</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1984,17 +1984,17 @@
         <v>46217</v>
       </c>
       <c r="B82" t="n">
-        <v>131</v>
+        <v>2211</v>
       </c>
       <c r="C82" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D82" t="n">
-        <v>669.39</v>
+        <v>797.61</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2003,17 +2003,17 @@
         <v>46217</v>
       </c>
       <c r="B83" t="n">
-        <v>1064</v>
+        <v>131</v>
       </c>
       <c r="C83" t="n">
         <v>8888</v>
       </c>
       <c r="D83" t="n">
-        <v>2383.39</v>
+        <v>2340.29</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2022,17 +2022,17 @@
         <v>46217</v>
       </c>
       <c r="B84" t="n">
-        <v>2251</v>
+        <v>131</v>
       </c>
       <c r="C84" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D84" t="n">
-        <v>797.58</v>
+        <v>669.39</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2041,13 +2041,13 @@
         <v>46217</v>
       </c>
       <c r="B85" t="n">
-        <v>451</v>
+        <v>1064</v>
       </c>
       <c r="C85" t="n">
         <v>8888</v>
       </c>
       <c r="D85" t="n">
-        <v>1371.26</v>
+        <v>2383.39</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2060,17 +2060,17 @@
         <v>46217</v>
       </c>
       <c r="B86" t="n">
-        <v>40</v>
+        <v>2251</v>
       </c>
       <c r="C86" t="n">
         <v>8888</v>
       </c>
       <c r="D86" t="n">
-        <v>1093.47</v>
+        <v>797.58</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2079,13 +2079,13 @@
         <v>46217</v>
       </c>
       <c r="B87" t="n">
-        <v>360</v>
+        <v>451</v>
       </c>
       <c r="C87" t="n">
         <v>8888</v>
       </c>
       <c r="D87" t="n">
-        <v>7017.48</v>
+        <v>1371.26</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2098,17 +2098,17 @@
         <v>46217</v>
       </c>
       <c r="B88" t="n">
-        <v>530</v>
+        <v>40</v>
       </c>
       <c r="C88" t="n">
         <v>8888</v>
       </c>
       <c r="D88" t="n">
-        <v>180.08</v>
+        <v>1093.47</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2117,17 +2117,17 @@
         <v>46217</v>
       </c>
       <c r="B89" t="n">
-        <v>1137</v>
+        <v>360</v>
       </c>
       <c r="C89" t="n">
         <v>8888</v>
       </c>
       <c r="D89" t="n">
-        <v>2833.69</v>
+        <v>7017.48</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2136,17 +2136,17 @@
         <v>46217</v>
       </c>
       <c r="B90" t="n">
-        <v>1293</v>
+        <v>530</v>
       </c>
       <c r="C90" t="n">
         <v>8888</v>
       </c>
       <c r="D90" t="n">
-        <v>3201.32</v>
+        <v>180.08</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2155,17 +2155,17 @@
         <v>46217</v>
       </c>
       <c r="B91" t="n">
-        <v>1293</v>
+        <v>1137</v>
       </c>
       <c r="C91" t="n">
-        <v>601</v>
+        <v>8888</v>
       </c>
       <c r="D91" t="n">
-        <v>456.47</v>
+        <v>2833.69</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2174,17 +2174,17 @@
         <v>46217</v>
       </c>
       <c r="B92" t="n">
-        <v>2118</v>
+        <v>1293</v>
       </c>
       <c r="C92" t="n">
         <v>8888</v>
       </c>
       <c r="D92" t="n">
-        <v>311.54</v>
+        <v>3201.32</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2193,17 +2193,17 @@
         <v>46217</v>
       </c>
       <c r="B93" t="n">
-        <v>424</v>
+        <v>1293</v>
       </c>
       <c r="C93" t="n">
-        <v>8888</v>
+        <v>601</v>
       </c>
       <c r="D93" t="n">
-        <v>349.68</v>
+        <v>456.47</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2212,17 +2212,17 @@
         <v>46217</v>
       </c>
       <c r="B94" t="n">
-        <v>559</v>
+        <v>2118</v>
       </c>
       <c r="C94" t="n">
         <v>8888</v>
       </c>
       <c r="D94" t="n">
-        <v>1064.63</v>
+        <v>311.54</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2231,13 +2231,13 @@
         <v>46217</v>
       </c>
       <c r="B95" t="n">
-        <v>89</v>
+        <v>424</v>
       </c>
       <c r="C95" t="n">
         <v>8888</v>
       </c>
       <c r="D95" t="n">
-        <v>1506.42</v>
+        <v>349.68</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2250,17 +2250,17 @@
         <v>46217</v>
       </c>
       <c r="B96" t="n">
-        <v>2250</v>
+        <v>559</v>
       </c>
       <c r="C96" t="n">
         <v>8888</v>
       </c>
       <c r="D96" t="n">
-        <v>1943.54</v>
+        <v>1064.63</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2269,17 +2269,17 @@
         <v>46217</v>
       </c>
       <c r="B97" t="n">
-        <v>1299</v>
+        <v>89</v>
       </c>
       <c r="C97" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D97" t="n">
-        <v>262.02</v>
+        <v>1506.42</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2288,17 +2288,17 @@
         <v>46217</v>
       </c>
       <c r="B98" t="n">
-        <v>2651</v>
+        <v>2250</v>
       </c>
       <c r="C98" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D98" t="n">
-        <v>648.71</v>
+        <v>1943.54</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2307,17 +2307,17 @@
         <v>46217</v>
       </c>
       <c r="B99" t="n">
-        <v>40</v>
+        <v>1299</v>
       </c>
       <c r="C99" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D99" t="n">
-        <v>733.37</v>
+        <v>262.02</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2326,17 +2326,17 @@
         <v>46217</v>
       </c>
       <c r="B100" t="n">
-        <v>40</v>
+        <v>2651</v>
       </c>
       <c r="C100" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D100" t="n">
-        <v>2529.31</v>
+        <v>648.71</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2345,17 +2345,17 @@
         <v>46217</v>
       </c>
       <c r="B101" t="n">
-        <v>626</v>
+        <v>40</v>
       </c>
       <c r="C101" t="n">
         <v>8888</v>
       </c>
       <c r="D101" t="n">
-        <v>13218.02</v>
+        <v>3583.39</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2364,13 +2364,13 @@
         <v>46217</v>
       </c>
       <c r="B102" t="n">
-        <v>363</v>
+        <v>40</v>
       </c>
       <c r="C102" t="n">
         <v>8888</v>
       </c>
       <c r="D102" t="n">
-        <v>739.17</v>
+        <v>2529.31</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2383,17 +2383,17 @@
         <v>46217</v>
       </c>
       <c r="B103" t="n">
-        <v>675</v>
+        <v>626</v>
       </c>
       <c r="C103" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D103" t="n">
-        <v>107.13</v>
+        <v>13218.02</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2402,17 +2402,17 @@
         <v>46217</v>
       </c>
       <c r="B104" t="n">
-        <v>636</v>
+        <v>363</v>
       </c>
       <c r="C104" t="n">
         <v>8888</v>
       </c>
       <c r="D104" t="n">
-        <v>5631.89</v>
+        <v>739.17</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2421,17 +2421,17 @@
         <v>46217</v>
       </c>
       <c r="B105" t="n">
-        <v>1075</v>
+        <v>675</v>
       </c>
       <c r="C105" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D105" t="n">
-        <v>1331.89</v>
+        <v>107.13</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2440,17 +2440,17 @@
         <v>46217</v>
       </c>
       <c r="B106" t="n">
-        <v>2245</v>
+        <v>636</v>
       </c>
       <c r="C106" t="n">
         <v>8888</v>
       </c>
       <c r="D106" t="n">
-        <v>883.75</v>
+        <v>5631.89</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2459,13 +2459,13 @@
         <v>46217</v>
       </c>
       <c r="B107" t="n">
-        <v>477</v>
+        <v>1075</v>
       </c>
       <c r="C107" t="n">
         <v>8888</v>
       </c>
       <c r="D107" t="n">
-        <v>994.15</v>
+        <v>1331.89</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -2478,17 +2478,17 @@
         <v>46217</v>
       </c>
       <c r="B108" t="n">
-        <v>2015</v>
+        <v>2245</v>
       </c>
       <c r="C108" t="n">
         <v>8888</v>
       </c>
       <c r="D108" t="n">
-        <v>2931.07</v>
+        <v>883.75</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2497,17 +2497,17 @@
         <v>46217</v>
       </c>
       <c r="B109" t="n">
-        <v>1064</v>
+        <v>477</v>
       </c>
       <c r="C109" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D109" t="n">
-        <v>451.38</v>
+        <v>994.15</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2516,17 +2516,17 @@
         <v>46217</v>
       </c>
       <c r="B110" t="n">
-        <v>1983</v>
+        <v>2015</v>
       </c>
       <c r="C110" t="n">
         <v>8888</v>
       </c>
       <c r="D110" t="n">
-        <v>680.42</v>
+        <v>2931.07</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2535,17 +2535,17 @@
         <v>46217</v>
       </c>
       <c r="B111" t="n">
-        <v>2118</v>
+        <v>1064</v>
       </c>
       <c r="C111" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D111" t="n">
-        <v>2646.39</v>
+        <v>451.38</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2554,17 +2554,17 @@
         <v>46217</v>
       </c>
       <c r="B112" t="n">
-        <v>2680</v>
+        <v>1983</v>
       </c>
       <c r="C112" t="n">
         <v>8888</v>
       </c>
       <c r="D112" t="n">
-        <v>824.67</v>
+        <v>1246.33</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2573,13 +2573,13 @@
         <v>46217</v>
       </c>
       <c r="B113" t="n">
-        <v>1653</v>
+        <v>2118</v>
       </c>
       <c r="C113" t="n">
         <v>8888</v>
       </c>
       <c r="D113" t="n">
-        <v>2848.57</v>
+        <v>2646.39</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -2592,17 +2592,17 @@
         <v>46217</v>
       </c>
       <c r="B114" t="n">
-        <v>629</v>
+        <v>2680</v>
       </c>
       <c r="C114" t="n">
-        <v>675</v>
+        <v>8888</v>
       </c>
       <c r="D114" t="n">
-        <v>267.79</v>
+        <v>824.67</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2611,13 +2611,13 @@
         <v>46217</v>
       </c>
       <c r="B115" t="n">
-        <v>559</v>
+        <v>1653</v>
       </c>
       <c r="C115" t="n">
         <v>8888</v>
       </c>
       <c r="D115" t="n">
-        <v>1562.5</v>
+        <v>2848.57</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -2630,17 +2630,17 @@
         <v>46217</v>
       </c>
       <c r="B116" t="n">
-        <v>1465</v>
+        <v>629</v>
       </c>
       <c r="C116" t="n">
-        <v>8888</v>
+        <v>675</v>
       </c>
       <c r="D116" t="n">
-        <v>9346.120000000001</v>
+        <v>267.79</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2649,17 +2649,17 @@
         <v>46217</v>
       </c>
       <c r="B117" t="n">
-        <v>2550</v>
+        <v>559</v>
       </c>
       <c r="C117" t="n">
         <v>8888</v>
       </c>
       <c r="D117" t="n">
-        <v>321.05</v>
+        <v>1562.5</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2668,17 +2668,17 @@
         <v>46217</v>
       </c>
       <c r="B118" t="n">
-        <v>1756</v>
+        <v>1465</v>
       </c>
       <c r="C118" t="n">
         <v>8888</v>
       </c>
       <c r="D118" t="n">
-        <v>2445</v>
+        <v>9346.120000000001</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2687,17 +2687,17 @@
         <v>46217</v>
       </c>
       <c r="B119" t="n">
-        <v>363</v>
+        <v>2550</v>
       </c>
       <c r="C119" t="n">
         <v>8888</v>
       </c>
       <c r="D119" t="n">
-        <v>649.08</v>
+        <v>321.05</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2706,17 +2706,17 @@
         <v>46217</v>
       </c>
       <c r="B120" t="n">
-        <v>2698</v>
+        <v>1756</v>
       </c>
       <c r="C120" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D120" t="n">
-        <v>1183.42</v>
+        <v>2445</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2725,13 +2725,13 @@
         <v>46217</v>
       </c>
       <c r="B121" t="n">
-        <v>2250</v>
+        <v>363</v>
       </c>
       <c r="C121" t="n">
         <v>8888</v>
       </c>
       <c r="D121" t="n">
-        <v>1512.17</v>
+        <v>649.08</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -2744,17 +2744,17 @@
         <v>46217</v>
       </c>
       <c r="B122" t="n">
-        <v>2681</v>
+        <v>2698</v>
       </c>
       <c r="C122" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D122" t="n">
-        <v>2775.8</v>
+        <v>1183.42</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2763,13 +2763,13 @@
         <v>46217</v>
       </c>
       <c r="B123" t="n">
-        <v>535</v>
+        <v>2250</v>
       </c>
       <c r="C123" t="n">
         <v>8888</v>
       </c>
       <c r="D123" t="n">
-        <v>2806.71</v>
+        <v>1512.17</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -2782,17 +2782,17 @@
         <v>46217</v>
       </c>
       <c r="B124" t="n">
-        <v>483</v>
+        <v>2681</v>
       </c>
       <c r="C124" t="n">
         <v>8888</v>
       </c>
       <c r="D124" t="n">
-        <v>2100.84</v>
+        <v>2775.8</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2801,17 +2801,17 @@
         <v>46217</v>
       </c>
       <c r="B125" t="n">
-        <v>2330</v>
+        <v>535</v>
       </c>
       <c r="C125" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D125" t="n">
-        <v>1923.09</v>
+        <v>2806.71</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2820,17 +2820,17 @@
         <v>46217</v>
       </c>
       <c r="B126" t="n">
-        <v>363</v>
+        <v>483</v>
       </c>
       <c r="C126" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D126" t="n">
-        <v>1058.27</v>
+        <v>2100.84</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2839,17 +2839,17 @@
         <v>46217</v>
       </c>
       <c r="B127" t="n">
-        <v>2709</v>
+        <v>2330</v>
       </c>
       <c r="C127" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D127" t="n">
-        <v>1667.47</v>
+        <v>1923.09</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2858,17 +2858,17 @@
         <v>46217</v>
       </c>
       <c r="B128" t="n">
-        <v>1137</v>
+        <v>363</v>
       </c>
       <c r="C128" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D128" t="n">
-        <v>3185.1</v>
+        <v>1058.27</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2877,15 +2877,53 @@
         <v>46217</v>
       </c>
       <c r="B129" t="n">
+        <v>2709</v>
+      </c>
+      <c r="C129" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D129" t="n">
+        <v>1667.47</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B130" t="n">
+        <v>1137</v>
+      </c>
+      <c r="C130" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D130" t="n">
+        <v>3185.1</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B131" t="n">
         <v>2251</v>
       </c>
-      <c r="C129" t="n">
+      <c r="C131" t="n">
         <v>3403</v>
       </c>
-      <c r="D129" t="n">
+      <c r="D131" t="n">
         <v>510.18</v>
       </c>
-      <c r="E129" t="inlineStr">
+      <c r="E131" t="inlineStr">
         <is>
           <t>TELEMARKETING</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 14:30:03
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E131"/>
+  <dimension ref="A1:E152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -502,17 +502,17 @@
         <v>46217</v>
       </c>
       <c r="B4" t="n">
-        <v>2109</v>
+        <v>1653</v>
       </c>
       <c r="C4" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D4" t="n">
-        <v>4813.6</v>
+        <v>4524.08</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -521,17 +521,17 @@
         <v>46217</v>
       </c>
       <c r="B5" t="n">
-        <v>1993</v>
+        <v>2109</v>
       </c>
       <c r="C5" t="n">
         <v>8888</v>
       </c>
       <c r="D5" t="n">
-        <v>1785.44</v>
+        <v>4813.6</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -540,17 +540,17 @@
         <v>46217</v>
       </c>
       <c r="B6" t="n">
-        <v>1102</v>
+        <v>2015</v>
       </c>
       <c r="C6" t="n">
-        <v>8888</v>
+        <v>2571</v>
       </c>
       <c r="D6" t="n">
-        <v>1264.43</v>
+        <v>1790.54</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -559,17 +559,17 @@
         <v>46217</v>
       </c>
       <c r="B7" t="n">
-        <v>2015</v>
+        <v>1993</v>
       </c>
       <c r="C7" t="n">
-        <v>2571</v>
+        <v>8888</v>
       </c>
       <c r="D7" t="n">
-        <v>679.9</v>
+        <v>1785.44</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -578,17 +578,17 @@
         <v>46217</v>
       </c>
       <c r="B8" t="n">
-        <v>1293</v>
+        <v>1102</v>
       </c>
       <c r="C8" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D8" t="n">
-        <v>1337.87</v>
+        <v>2432.31</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -597,17 +597,17 @@
         <v>46217</v>
       </c>
       <c r="B9" t="n">
-        <v>89</v>
+        <v>1293</v>
       </c>
       <c r="C9" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D9" t="n">
-        <v>5652.15</v>
+        <v>1337.87</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -616,13 +616,13 @@
         <v>46217</v>
       </c>
       <c r="B10" t="n">
-        <v>2768</v>
+        <v>1254</v>
       </c>
       <c r="C10" t="n">
         <v>8888</v>
       </c>
       <c r="D10" t="n">
-        <v>3436.6</v>
+        <v>428.16</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -635,13 +635,13 @@
         <v>46217</v>
       </c>
       <c r="B11" t="n">
-        <v>949</v>
+        <v>2726</v>
       </c>
       <c r="C11" t="n">
-        <v>1258</v>
+        <v>1929</v>
       </c>
       <c r="D11" t="n">
-        <v>196.87</v>
+        <v>640.1799999999999</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -654,13 +654,13 @@
         <v>46217</v>
       </c>
       <c r="B12" t="n">
-        <v>1756</v>
+        <v>89</v>
       </c>
       <c r="C12" t="n">
         <v>8888</v>
       </c>
       <c r="D12" t="n">
-        <v>1799.7</v>
+        <v>5652.15</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -673,17 +673,17 @@
         <v>46217</v>
       </c>
       <c r="B13" t="n">
-        <v>285</v>
+        <v>2768</v>
       </c>
       <c r="C13" t="n">
         <v>8888</v>
       </c>
       <c r="D13" t="n">
-        <v>2593.28</v>
+        <v>3436.6</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -692,17 +692,17 @@
         <v>46217</v>
       </c>
       <c r="B14" t="n">
-        <v>610</v>
+        <v>1890</v>
       </c>
       <c r="C14" t="n">
-        <v>8888</v>
+        <v>3449</v>
       </c>
       <c r="D14" t="n">
-        <v>590.08</v>
+        <v>589.0599999999999</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -711,13 +711,13 @@
         <v>46217</v>
       </c>
       <c r="B15" t="n">
-        <v>619</v>
+        <v>2641</v>
       </c>
       <c r="C15" t="n">
         <v>8888</v>
       </c>
       <c r="D15" t="n">
-        <v>236.34</v>
+        <v>607.79</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -730,13 +730,13 @@
         <v>46217</v>
       </c>
       <c r="B16" t="n">
-        <v>2755</v>
+        <v>949</v>
       </c>
       <c r="C16" t="n">
-        <v>2220</v>
+        <v>1258</v>
       </c>
       <c r="D16" t="n">
-        <v>1133.17</v>
+        <v>196.87</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -749,17 +749,17 @@
         <v>46217</v>
       </c>
       <c r="B17" t="n">
-        <v>2767</v>
+        <v>1756</v>
       </c>
       <c r="C17" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D17" t="n">
-        <v>5000.2</v>
+        <v>1799.7</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
         <v>46217</v>
       </c>
       <c r="B18" t="n">
-        <v>559</v>
+        <v>285</v>
       </c>
       <c r="C18" t="n">
         <v>8888</v>
       </c>
       <c r="D18" t="n">
-        <v>517.0700000000001</v>
+        <v>2593.28</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -787,13 +787,13 @@
         <v>46217</v>
       </c>
       <c r="B19" t="n">
-        <v>2767</v>
+        <v>610</v>
       </c>
       <c r="C19" t="n">
         <v>8888</v>
       </c>
       <c r="D19" t="n">
-        <v>1175.73</v>
+        <v>590.08</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -806,17 +806,17 @@
         <v>46217</v>
       </c>
       <c r="B20" t="n">
-        <v>1063</v>
+        <v>1906</v>
       </c>
       <c r="C20" t="n">
         <v>8888</v>
       </c>
       <c r="D20" t="n">
-        <v>1251.14</v>
+        <v>1580.84</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -825,17 +825,17 @@
         <v>46217</v>
       </c>
       <c r="B21" t="n">
-        <v>325</v>
+        <v>619</v>
       </c>
       <c r="C21" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D21" t="n">
-        <v>868.83</v>
+        <v>236.34</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -844,17 +844,17 @@
         <v>46217</v>
       </c>
       <c r="B22" t="n">
-        <v>610</v>
+        <v>2755</v>
       </c>
       <c r="C22" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D22" t="n">
-        <v>235.34</v>
+        <v>1133.17</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -863,17 +863,17 @@
         <v>46217</v>
       </c>
       <c r="B23" t="n">
-        <v>1906</v>
+        <v>2767</v>
       </c>
       <c r="C23" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D23" t="n">
-        <v>889.22</v>
+        <v>5000.2</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -882,17 +882,17 @@
         <v>46217</v>
       </c>
       <c r="B24" t="n">
-        <v>424</v>
+        <v>559</v>
       </c>
       <c r="C24" t="n">
         <v>8888</v>
       </c>
       <c r="D24" t="n">
-        <v>2575.64</v>
+        <v>1200.99</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -901,17 +901,17 @@
         <v>46217</v>
       </c>
       <c r="B25" t="n">
-        <v>40</v>
+        <v>2767</v>
       </c>
       <c r="C25" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D25" t="n">
-        <v>325.04</v>
+        <v>1175.73</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -920,13 +920,13 @@
         <v>46217</v>
       </c>
       <c r="B26" t="n">
-        <v>1117</v>
+        <v>1063</v>
       </c>
       <c r="C26" t="n">
         <v>8888</v>
       </c>
       <c r="D26" t="n">
-        <v>349.47</v>
+        <v>1251.14</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -939,13 +939,13 @@
         <v>46217</v>
       </c>
       <c r="B27" t="n">
-        <v>949</v>
+        <v>325</v>
       </c>
       <c r="C27" t="n">
-        <v>998</v>
+        <v>58</v>
       </c>
       <c r="D27" t="n">
-        <v>129.85</v>
+        <v>868.83</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -958,17 +958,17 @@
         <v>46217</v>
       </c>
       <c r="B28" t="n">
-        <v>2250</v>
+        <v>2660</v>
       </c>
       <c r="C28" t="n">
         <v>8888</v>
       </c>
       <c r="D28" t="n">
-        <v>3627.44</v>
+        <v>281.24</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -977,13 +977,13 @@
         <v>46217</v>
       </c>
       <c r="B29" t="n">
-        <v>2507</v>
+        <v>610</v>
       </c>
       <c r="C29" t="n">
         <v>8888</v>
       </c>
       <c r="D29" t="n">
-        <v>4167.12</v>
+        <v>235.34</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -996,13 +996,13 @@
         <v>46217</v>
       </c>
       <c r="B30" t="n">
-        <v>664</v>
+        <v>424</v>
       </c>
       <c r="C30" t="n">
         <v>8888</v>
       </c>
       <c r="D30" t="n">
-        <v>3523.8</v>
+        <v>3214.29</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1015,13 +1015,13 @@
         <v>46217</v>
       </c>
       <c r="B31" t="n">
-        <v>1906</v>
+        <v>40</v>
       </c>
       <c r="C31" t="n">
-        <v>1954</v>
+        <v>58</v>
       </c>
       <c r="D31" t="n">
-        <v>1445.21</v>
+        <v>325.04</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1034,17 +1034,17 @@
         <v>46217</v>
       </c>
       <c r="B32" t="n">
-        <v>1075</v>
+        <v>1117</v>
       </c>
       <c r="C32" t="n">
         <v>8888</v>
       </c>
       <c r="D32" t="n">
-        <v>470.95</v>
+        <v>349.47</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1053,13 +1053,13 @@
         <v>46217</v>
       </c>
       <c r="B33" t="n">
-        <v>2696</v>
+        <v>949</v>
       </c>
       <c r="C33" t="n">
-        <v>1312</v>
+        <v>998</v>
       </c>
       <c r="D33" t="n">
-        <v>677.76</v>
+        <v>129.85</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1072,17 +1072,17 @@
         <v>46217</v>
       </c>
       <c r="B34" t="n">
-        <v>360</v>
+        <v>2250</v>
       </c>
       <c r="C34" t="n">
-        <v>546</v>
+        <v>8888</v>
       </c>
       <c r="D34" t="n">
-        <v>4515.36</v>
+        <v>3627.44</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1091,17 +1091,17 @@
         <v>46217</v>
       </c>
       <c r="B35" t="n">
-        <v>2651</v>
+        <v>2507</v>
       </c>
       <c r="C35" t="n">
         <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>638.64</v>
+        <v>4167.12</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1110,17 @@
         <v>46217</v>
       </c>
       <c r="B36" t="n">
-        <v>1293</v>
+        <v>664</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>381.82</v>
+        <v>3523.8</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1129,17 @@
         <v>46217</v>
       </c>
       <c r="B37" t="n">
-        <v>2663</v>
+        <v>1906</v>
       </c>
       <c r="C37" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D37" t="n">
-        <v>2146.08</v>
+        <v>1445.21</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1148,17 +1148,17 @@
         <v>46217</v>
       </c>
       <c r="B38" t="n">
-        <v>675</v>
+        <v>1075</v>
       </c>
       <c r="C38" t="n">
         <v>8888</v>
       </c>
       <c r="D38" t="n">
-        <v>289.67</v>
+        <v>470.95</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1167,17 +1167,17 @@
         <v>46217</v>
       </c>
       <c r="B39" t="n">
-        <v>1063</v>
+        <v>2696</v>
       </c>
       <c r="C39" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D39" t="n">
-        <v>1902.46</v>
+        <v>677.76</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1186,17 +1186,17 @@
         <v>46217</v>
       </c>
       <c r="B40" t="n">
-        <v>1392</v>
+        <v>360</v>
       </c>
       <c r="C40" t="n">
-        <v>8888</v>
+        <v>546</v>
       </c>
       <c r="D40" t="n">
-        <v>814.61</v>
+        <v>5188.86</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1205,17 +1205,17 @@
         <v>46217</v>
       </c>
       <c r="B41" t="n">
-        <v>360</v>
+        <v>2491</v>
       </c>
       <c r="C41" t="n">
         <v>8888</v>
       </c>
       <c r="D41" t="n">
-        <v>749.13</v>
+        <v>2031.53</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1224,17 +1224,17 @@
         <v>46217</v>
       </c>
       <c r="B42" t="n">
-        <v>2491</v>
+        <v>2651</v>
       </c>
       <c r="C42" t="n">
         <v>8888</v>
       </c>
       <c r="D42" t="n">
-        <v>398.66</v>
+        <v>638.64</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1243,17 +1243,17 @@
         <v>46217</v>
       </c>
       <c r="B43" t="n">
-        <v>949</v>
+        <v>1293</v>
       </c>
       <c r="C43" t="n">
-        <v>1134</v>
+        <v>8888</v>
       </c>
       <c r="D43" t="n">
-        <v>327.6</v>
+        <v>381.82</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1262,17 +1262,17 @@
         <v>46217</v>
       </c>
       <c r="B44" t="n">
-        <v>326</v>
+        <v>2663</v>
       </c>
       <c r="C44" t="n">
         <v>8888</v>
       </c>
       <c r="D44" t="n">
-        <v>212.63</v>
+        <v>2146.08</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1281,17 +1281,17 @@
         <v>46217</v>
       </c>
       <c r="B45" t="n">
-        <v>325</v>
+        <v>525</v>
       </c>
       <c r="C45" t="n">
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>584.27</v>
+        <v>639.9</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1300,17 +1300,17 @@
         <v>46217</v>
       </c>
       <c r="B46" t="n">
-        <v>131</v>
+        <v>2711</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>360.06</v>
+        <v>750.3200000000001</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1319,17 +1319,17 @@
         <v>46217</v>
       </c>
       <c r="B47" t="n">
-        <v>2279</v>
+        <v>675</v>
       </c>
       <c r="C47" t="n">
         <v>8888</v>
       </c>
       <c r="D47" t="n">
-        <v>1034.25</v>
+        <v>289.67</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1338,17 +1338,17 @@
         <v>46217</v>
       </c>
       <c r="B48" t="n">
-        <v>1116</v>
+        <v>1063</v>
       </c>
       <c r="C48" t="n">
         <v>8888</v>
       </c>
       <c r="D48" t="n">
-        <v>1293.89</v>
+        <v>1902.46</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1357,17 +1357,17 @@
         <v>46217</v>
       </c>
       <c r="B49" t="n">
-        <v>131</v>
+        <v>1392</v>
       </c>
       <c r="C49" t="n">
         <v>8888</v>
       </c>
       <c r="D49" t="n">
-        <v>1528.41</v>
+        <v>814.61</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1376,17 +1376,17 @@
         <v>46217</v>
       </c>
       <c r="B50" t="n">
-        <v>1293</v>
+        <v>360</v>
       </c>
       <c r="C50" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D50" t="n">
-        <v>3534.85</v>
+        <v>749.13</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1395,17 +1395,17 @@
         <v>46217</v>
       </c>
       <c r="B51" t="n">
-        <v>1983</v>
+        <v>949</v>
       </c>
       <c r="C51" t="n">
-        <v>8888</v>
+        <v>1134</v>
       </c>
       <c r="D51" t="n">
-        <v>412.16</v>
+        <v>327.6</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
         <v>46217</v>
       </c>
       <c r="B52" t="n">
-        <v>451</v>
+        <v>326</v>
       </c>
       <c r="C52" t="n">
         <v>8888</v>
       </c>
       <c r="D52" t="n">
-        <v>2583.46</v>
+        <v>212.63</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1433,17 +1433,17 @@
         <v>46217</v>
       </c>
       <c r="B53" t="n">
-        <v>2767</v>
+        <v>325</v>
       </c>
       <c r="C53" t="n">
         <v>8888</v>
       </c>
       <c r="D53" t="n">
-        <v>596.88</v>
+        <v>616.95</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1452,17 +1452,17 @@
         <v>46217</v>
       </c>
       <c r="B54" t="n">
-        <v>1063</v>
+        <v>131</v>
       </c>
       <c r="C54" t="n">
         <v>8888</v>
       </c>
       <c r="D54" t="n">
-        <v>352.87</v>
+        <v>360.06</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1471,17 +1471,17 @@
         <v>46217</v>
       </c>
       <c r="B55" t="n">
-        <v>629</v>
+        <v>2697</v>
       </c>
       <c r="C55" t="n">
         <v>8888</v>
       </c>
       <c r="D55" t="n">
-        <v>559.15</v>
+        <v>420.48</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1490,17 +1490,17 @@
         <v>46217</v>
       </c>
       <c r="B56" t="n">
-        <v>58</v>
+        <v>2279</v>
       </c>
       <c r="C56" t="n">
         <v>8888</v>
       </c>
       <c r="D56" t="n">
-        <v>2637.19</v>
+        <v>1034.25</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1509,17 +1509,17 @@
         <v>46217</v>
       </c>
       <c r="B57" t="n">
-        <v>2211</v>
+        <v>1116</v>
       </c>
       <c r="C57" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D57" t="n">
-        <v>967.05</v>
+        <v>1293.89</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1528,17 +1528,17 @@
         <v>46217</v>
       </c>
       <c r="B58" t="n">
-        <v>1117</v>
+        <v>131</v>
       </c>
       <c r="C58" t="n">
         <v>8888</v>
       </c>
       <c r="D58" t="n">
-        <v>581.51</v>
+        <v>1528.41</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1547,17 +1547,17 @@
         <v>46217</v>
       </c>
       <c r="B59" t="n">
-        <v>629</v>
+        <v>1293</v>
       </c>
       <c r="C59" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D59" t="n">
-        <v>2049.78</v>
+        <v>3534.85</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1566,17 +1566,17 @@
         <v>46217</v>
       </c>
       <c r="B60" t="n">
-        <v>949</v>
+        <v>451</v>
       </c>
       <c r="C60" t="n">
-        <v>1762</v>
+        <v>8888</v>
       </c>
       <c r="D60" t="n">
-        <v>325.65</v>
+        <v>2583.46</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1585,13 +1585,13 @@
         <v>46217</v>
       </c>
       <c r="B61" t="n">
-        <v>2463</v>
+        <v>1983</v>
       </c>
       <c r="C61" t="n">
         <v>8888</v>
       </c>
       <c r="D61" t="n">
-        <v>8336.43</v>
+        <v>412.16</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1604,17 +1604,17 @@
         <v>46217</v>
       </c>
       <c r="B62" t="n">
-        <v>1064</v>
+        <v>2767</v>
       </c>
       <c r="C62" t="n">
         <v>8888</v>
       </c>
       <c r="D62" t="n">
-        <v>1513.21</v>
+        <v>596.88</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1623,17 +1623,17 @@
         <v>46217</v>
       </c>
       <c r="B63" t="n">
-        <v>1478</v>
+        <v>2697</v>
       </c>
       <c r="C63" t="n">
         <v>8888</v>
       </c>
       <c r="D63" t="n">
-        <v>1294.76</v>
+        <v>2055.26</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1642,13 +1642,13 @@
         <v>46217</v>
       </c>
       <c r="B64" t="n">
-        <v>358</v>
+        <v>569</v>
       </c>
       <c r="C64" t="n">
         <v>8888</v>
       </c>
       <c r="D64" t="n">
-        <v>1918.33</v>
+        <v>2291.64</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1661,17 +1661,17 @@
         <v>46217</v>
       </c>
       <c r="B65" t="n">
-        <v>2107</v>
+        <v>1063</v>
       </c>
       <c r="C65" t="n">
         <v>8888</v>
       </c>
       <c r="D65" t="n">
-        <v>2745.11</v>
+        <v>352.87</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1680,13 +1680,13 @@
         <v>46217</v>
       </c>
       <c r="B66" t="n">
-        <v>675</v>
+        <v>2687</v>
       </c>
       <c r="C66" t="n">
         <v>8888</v>
       </c>
       <c r="D66" t="n">
-        <v>275.17</v>
+        <v>1760.22</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1699,13 +1699,13 @@
         <v>46217</v>
       </c>
       <c r="B67" t="n">
-        <v>2279</v>
+        <v>629</v>
       </c>
       <c r="C67" t="n">
         <v>8888</v>
       </c>
       <c r="D67" t="n">
-        <v>1165.17</v>
+        <v>559.15</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1718,13 +1718,13 @@
         <v>46217</v>
       </c>
       <c r="B68" t="n">
-        <v>451</v>
+        <v>1890</v>
       </c>
       <c r="C68" t="n">
-        <v>3403</v>
+        <v>1953</v>
       </c>
       <c r="D68" t="n">
-        <v>327.28</v>
+        <v>697.04</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1737,17 +1737,17 @@
         <v>46217</v>
       </c>
       <c r="B69" t="n">
-        <v>2571</v>
+        <v>58</v>
       </c>
       <c r="C69" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D69" t="n">
-        <v>2202.75</v>
+        <v>2637.19</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1756,17 +1756,17 @@
         <v>46217</v>
       </c>
       <c r="B70" t="n">
-        <v>610</v>
+        <v>2211</v>
       </c>
       <c r="C70" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D70" t="n">
-        <v>335.61</v>
+        <v>967.05</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1775,17 @@
         <v>46217</v>
       </c>
       <c r="B71" t="n">
-        <v>1108</v>
+        <v>1117</v>
       </c>
       <c r="C71" t="n">
         <v>8888</v>
       </c>
       <c r="D71" t="n">
-        <v>508.54</v>
+        <v>581.51</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1794,17 +1794,17 @@
         <v>46217</v>
       </c>
       <c r="B72" t="n">
-        <v>341</v>
+        <v>629</v>
       </c>
       <c r="C72" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D72" t="n">
-        <v>366.88</v>
+        <v>2049.78</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1813,17 +1813,17 @@
         <v>46217</v>
       </c>
       <c r="B73" t="n">
-        <v>1653</v>
+        <v>949</v>
       </c>
       <c r="C73" t="n">
-        <v>8888</v>
+        <v>1762</v>
       </c>
       <c r="D73" t="n">
-        <v>4383.69</v>
+        <v>325.65</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1832,17 +1832,17 @@
         <v>46217</v>
       </c>
       <c r="B74" t="n">
-        <v>619</v>
+        <v>2463</v>
       </c>
       <c r="C74" t="n">
         <v>8888</v>
       </c>
       <c r="D74" t="n">
-        <v>779.87</v>
+        <v>8336.43</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1851,13 +1851,13 @@
         <v>46217</v>
       </c>
       <c r="B75" t="n">
-        <v>663</v>
+        <v>1064</v>
       </c>
       <c r="C75" t="n">
         <v>8888</v>
       </c>
       <c r="D75" t="n">
-        <v>824.5599999999999</v>
+        <v>1513.21</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -1870,17 +1870,17 @@
         <v>46217</v>
       </c>
       <c r="B76" t="n">
-        <v>58</v>
+        <v>1478</v>
       </c>
       <c r="C76" t="n">
         <v>8888</v>
       </c>
       <c r="D76" t="n">
-        <v>660.1</v>
+        <v>1294.76</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1889,17 +1889,17 @@
         <v>46217</v>
       </c>
       <c r="B77" t="n">
-        <v>429</v>
+        <v>358</v>
       </c>
       <c r="C77" t="n">
-        <v>2571</v>
+        <v>8888</v>
       </c>
       <c r="D77" t="n">
-        <v>667.12</v>
+        <v>1918.33</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1908,17 +1908,17 @@
         <v>46217</v>
       </c>
       <c r="B78" t="n">
-        <v>483</v>
+        <v>2107</v>
       </c>
       <c r="C78" t="n">
         <v>8888</v>
       </c>
       <c r="D78" t="n">
-        <v>1290.28</v>
+        <v>2745.11</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1927,17 +1927,17 @@
         <v>46217</v>
       </c>
       <c r="B79" t="n">
-        <v>2709</v>
+        <v>675</v>
       </c>
       <c r="C79" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D79" t="n">
-        <v>1663.5</v>
+        <v>275.17</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1946,13 +1946,13 @@
         <v>46217</v>
       </c>
       <c r="B80" t="n">
-        <v>1937</v>
+        <v>2279</v>
       </c>
       <c r="C80" t="n">
         <v>8888</v>
       </c>
       <c r="D80" t="n">
-        <v>1332.89</v>
+        <v>1165.17</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -1965,13 +1965,13 @@
         <v>46217</v>
       </c>
       <c r="B81" t="n">
-        <v>429</v>
+        <v>451</v>
       </c>
       <c r="C81" t="n">
-        <v>1281</v>
+        <v>3403</v>
       </c>
       <c r="D81" t="n">
-        <v>1333.52</v>
+        <v>327.28</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -1984,17 +1984,17 @@
         <v>46217</v>
       </c>
       <c r="B82" t="n">
-        <v>2211</v>
+        <v>2571</v>
       </c>
       <c r="C82" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D82" t="n">
-        <v>797.61</v>
+        <v>2202.75</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2003,17 +2003,17 @@
         <v>46217</v>
       </c>
       <c r="B83" t="n">
-        <v>131</v>
+        <v>610</v>
       </c>
       <c r="C83" t="n">
         <v>8888</v>
       </c>
       <c r="D83" t="n">
-        <v>2340.29</v>
+        <v>335.61</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2022,17 +2022,17 @@
         <v>46217</v>
       </c>
       <c r="B84" t="n">
-        <v>131</v>
+        <v>1108</v>
       </c>
       <c r="C84" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D84" t="n">
-        <v>669.39</v>
+        <v>508.54</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2041,17 +2041,17 @@
         <v>46217</v>
       </c>
       <c r="B85" t="n">
-        <v>1064</v>
+        <v>341</v>
       </c>
       <c r="C85" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D85" t="n">
-        <v>2383.39</v>
+        <v>366.88</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2060,17 +2060,17 @@
         <v>46217</v>
       </c>
       <c r="B86" t="n">
-        <v>2251</v>
+        <v>1653</v>
       </c>
       <c r="C86" t="n">
         <v>8888</v>
       </c>
       <c r="D86" t="n">
-        <v>797.58</v>
+        <v>4383.69</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2079,13 +2079,13 @@
         <v>46217</v>
       </c>
       <c r="B87" t="n">
-        <v>451</v>
+        <v>619</v>
       </c>
       <c r="C87" t="n">
         <v>8888</v>
       </c>
       <c r="D87" t="n">
-        <v>1371.26</v>
+        <v>1557.5</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2098,17 +2098,17 @@
         <v>46217</v>
       </c>
       <c r="B88" t="n">
-        <v>40</v>
+        <v>663</v>
       </c>
       <c r="C88" t="n">
         <v>8888</v>
       </c>
       <c r="D88" t="n">
-        <v>1093.47</v>
+        <v>824.5599999999999</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2117,13 +2117,13 @@
         <v>46217</v>
       </c>
       <c r="B89" t="n">
-        <v>360</v>
+        <v>58</v>
       </c>
       <c r="C89" t="n">
         <v>8888</v>
       </c>
       <c r="D89" t="n">
-        <v>7017.48</v>
+        <v>660.1</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2136,17 +2136,17 @@
         <v>46217</v>
       </c>
       <c r="B90" t="n">
-        <v>530</v>
+        <v>429</v>
       </c>
       <c r="C90" t="n">
-        <v>8888</v>
+        <v>2571</v>
       </c>
       <c r="D90" t="n">
-        <v>180.08</v>
+        <v>667.12</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2155,17 +2155,17 @@
         <v>46217</v>
       </c>
       <c r="B91" t="n">
-        <v>1137</v>
+        <v>2641</v>
       </c>
       <c r="C91" t="n">
         <v>8888</v>
       </c>
       <c r="D91" t="n">
-        <v>2833.69</v>
+        <v>252.41</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
         <v>8888</v>
       </c>
       <c r="D92" t="n">
-        <v>3201.32</v>
+        <v>8102.01</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2193,17 +2193,17 @@
         <v>46217</v>
       </c>
       <c r="B93" t="n">
-        <v>1293</v>
+        <v>483</v>
       </c>
       <c r="C93" t="n">
-        <v>601</v>
+        <v>8888</v>
       </c>
       <c r="D93" t="n">
-        <v>456.47</v>
+        <v>1290.28</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2212,17 +2212,17 @@
         <v>46217</v>
       </c>
       <c r="B94" t="n">
-        <v>2118</v>
+        <v>2308</v>
       </c>
       <c r="C94" t="n">
-        <v>8888</v>
+        <v>546</v>
       </c>
       <c r="D94" t="n">
-        <v>311.54</v>
+        <v>1292.23</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2231,17 +2231,17 @@
         <v>46217</v>
       </c>
       <c r="B95" t="n">
-        <v>424</v>
+        <v>2709</v>
       </c>
       <c r="C95" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D95" t="n">
-        <v>349.68</v>
+        <v>1663.5</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2250,13 +2250,13 @@
         <v>46217</v>
       </c>
       <c r="B96" t="n">
-        <v>559</v>
+        <v>1937</v>
       </c>
       <c r="C96" t="n">
         <v>8888</v>
       </c>
       <c r="D96" t="n">
-        <v>1064.63</v>
+        <v>1332.89</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2269,17 +2269,17 @@
         <v>46217</v>
       </c>
       <c r="B97" t="n">
-        <v>89</v>
+        <v>429</v>
       </c>
       <c r="C97" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D97" t="n">
-        <v>1506.42</v>
+        <v>2195.97</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2288,17 +2288,17 @@
         <v>46217</v>
       </c>
       <c r="B98" t="n">
-        <v>2250</v>
+        <v>2211</v>
       </c>
       <c r="C98" t="n">
         <v>8888</v>
       </c>
       <c r="D98" t="n">
-        <v>1943.54</v>
+        <v>797.61</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2307,17 +2307,17 @@
         <v>46217</v>
       </c>
       <c r="B99" t="n">
-        <v>1299</v>
+        <v>360</v>
       </c>
       <c r="C99" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D99" t="n">
-        <v>262.02</v>
+        <v>13118.46</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2326,17 +2326,17 @@
         <v>46217</v>
       </c>
       <c r="B100" t="n">
-        <v>2651</v>
+        <v>131</v>
       </c>
       <c r="C100" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D100" t="n">
-        <v>648.71</v>
+        <v>2340.29</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2345,17 +2345,17 @@
         <v>46217</v>
       </c>
       <c r="B101" t="n">
-        <v>40</v>
+        <v>131</v>
       </c>
       <c r="C101" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D101" t="n">
-        <v>3583.39</v>
+        <v>669.39</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2364,17 +2364,17 @@
         <v>46217</v>
       </c>
       <c r="B102" t="n">
-        <v>40</v>
+        <v>1064</v>
       </c>
       <c r="C102" t="n">
         <v>8888</v>
       </c>
       <c r="D102" t="n">
-        <v>2529.31</v>
+        <v>103288.88</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2383,17 +2383,17 @@
         <v>46217</v>
       </c>
       <c r="B103" t="n">
-        <v>626</v>
+        <v>2251</v>
       </c>
       <c r="C103" t="n">
         <v>8888</v>
       </c>
       <c r="D103" t="n">
-        <v>13218.02</v>
+        <v>797.58</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2402,17 +2402,17 @@
         <v>46217</v>
       </c>
       <c r="B104" t="n">
-        <v>363</v>
+        <v>451</v>
       </c>
       <c r="C104" t="n">
         <v>8888</v>
       </c>
       <c r="D104" t="n">
-        <v>739.17</v>
+        <v>1371.26</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2421,17 +2421,17 @@
         <v>46217</v>
       </c>
       <c r="B105" t="n">
-        <v>675</v>
+        <v>40</v>
       </c>
       <c r="C105" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D105" t="n">
-        <v>107.13</v>
+        <v>1093.47</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2440,17 +2440,17 @@
         <v>46217</v>
       </c>
       <c r="B106" t="n">
-        <v>636</v>
+        <v>530</v>
       </c>
       <c r="C106" t="n">
         <v>8888</v>
       </c>
       <c r="D106" t="n">
-        <v>5631.89</v>
+        <v>180.08</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2459,17 +2459,17 @@
         <v>46217</v>
       </c>
       <c r="B107" t="n">
-        <v>1075</v>
+        <v>1137</v>
       </c>
       <c r="C107" t="n">
         <v>8888</v>
       </c>
       <c r="D107" t="n">
-        <v>1331.89</v>
+        <v>2833.69</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2478,17 +2478,17 @@
         <v>46217</v>
       </c>
       <c r="B108" t="n">
-        <v>2245</v>
+        <v>1293</v>
       </c>
       <c r="C108" t="n">
-        <v>8888</v>
+        <v>601</v>
       </c>
       <c r="D108" t="n">
-        <v>883.75</v>
+        <v>456.47</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2497,17 +2497,17 @@
         <v>46217</v>
       </c>
       <c r="B109" t="n">
-        <v>477</v>
+        <v>2118</v>
       </c>
       <c r="C109" t="n">
         <v>8888</v>
       </c>
       <c r="D109" t="n">
-        <v>994.15</v>
+        <v>311.54</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2516,17 +2516,17 @@
         <v>46217</v>
       </c>
       <c r="B110" t="n">
-        <v>2015</v>
+        <v>424</v>
       </c>
       <c r="C110" t="n">
         <v>8888</v>
       </c>
       <c r="D110" t="n">
-        <v>2931.07</v>
+        <v>349.68</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2535,13 +2535,13 @@
         <v>46217</v>
       </c>
       <c r="B111" t="n">
-        <v>1064</v>
+        <v>1299</v>
       </c>
       <c r="C111" t="n">
         <v>27</v>
       </c>
       <c r="D111" t="n">
-        <v>451.38</v>
+        <v>1425.22</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -2554,13 +2554,13 @@
         <v>46217</v>
       </c>
       <c r="B112" t="n">
-        <v>1983</v>
+        <v>559</v>
       </c>
       <c r="C112" t="n">
         <v>8888</v>
       </c>
       <c r="D112" t="n">
-        <v>1246.33</v>
+        <v>1064.63</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -2573,17 +2573,17 @@
         <v>46217</v>
       </c>
       <c r="B113" t="n">
-        <v>2118</v>
+        <v>89</v>
       </c>
       <c r="C113" t="n">
         <v>8888</v>
       </c>
       <c r="D113" t="n">
-        <v>2646.39</v>
+        <v>1506.42</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2592,17 +2592,17 @@
         <v>46217</v>
       </c>
       <c r="B114" t="n">
-        <v>2680</v>
+        <v>2250</v>
       </c>
       <c r="C114" t="n">
         <v>8888</v>
       </c>
       <c r="D114" t="n">
-        <v>824.67</v>
+        <v>1943.54</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2611,13 +2611,13 @@
         <v>46217</v>
       </c>
       <c r="B115" t="n">
-        <v>1653</v>
+        <v>767</v>
       </c>
       <c r="C115" t="n">
         <v>8888</v>
       </c>
       <c r="D115" t="n">
-        <v>2848.57</v>
+        <v>472.62</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -2630,13 +2630,13 @@
         <v>46217</v>
       </c>
       <c r="B116" t="n">
-        <v>629</v>
+        <v>2651</v>
       </c>
       <c r="C116" t="n">
-        <v>675</v>
+        <v>58</v>
       </c>
       <c r="D116" t="n">
-        <v>267.79</v>
+        <v>648.71</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -2649,17 +2649,17 @@
         <v>46217</v>
       </c>
       <c r="B117" t="n">
-        <v>559</v>
+        <v>2114</v>
       </c>
       <c r="C117" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D117" t="n">
-        <v>1562.5</v>
+        <v>879.03</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2668,13 +2668,13 @@
         <v>46217</v>
       </c>
       <c r="B118" t="n">
-        <v>1465</v>
+        <v>40</v>
       </c>
       <c r="C118" t="n">
         <v>8888</v>
       </c>
       <c r="D118" t="n">
-        <v>9346.120000000001</v>
+        <v>3583.39</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -2687,13 +2687,13 @@
         <v>46217</v>
       </c>
       <c r="B119" t="n">
-        <v>2550</v>
+        <v>40</v>
       </c>
       <c r="C119" t="n">
         <v>8888</v>
       </c>
       <c r="D119" t="n">
-        <v>321.05</v>
+        <v>2529.31</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -2706,13 +2706,13 @@
         <v>46217</v>
       </c>
       <c r="B120" t="n">
-        <v>1756</v>
+        <v>626</v>
       </c>
       <c r="C120" t="n">
         <v>8888</v>
       </c>
       <c r="D120" t="n">
-        <v>2445</v>
+        <v>13218.02</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -2731,11 +2731,11 @@
         <v>8888</v>
       </c>
       <c r="D121" t="n">
-        <v>649.08</v>
+        <v>739.17</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2744,13 +2744,13 @@
         <v>46217</v>
       </c>
       <c r="B122" t="n">
-        <v>2698</v>
+        <v>675</v>
       </c>
       <c r="C122" t="n">
-        <v>874</v>
+        <v>1898</v>
       </c>
       <c r="D122" t="n">
-        <v>1183.42</v>
+        <v>107.13</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -2763,13 +2763,13 @@
         <v>46217</v>
       </c>
       <c r="B123" t="n">
-        <v>2250</v>
+        <v>636</v>
       </c>
       <c r="C123" t="n">
         <v>8888</v>
       </c>
       <c r="D123" t="n">
-        <v>1512.17</v>
+        <v>5631.89</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -2782,13 +2782,13 @@
         <v>46217</v>
       </c>
       <c r="B124" t="n">
-        <v>2681</v>
+        <v>1075</v>
       </c>
       <c r="C124" t="n">
         <v>8888</v>
       </c>
       <c r="D124" t="n">
-        <v>2775.8</v>
+        <v>1331.89</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -2801,17 +2801,17 @@
         <v>46217</v>
       </c>
       <c r="B125" t="n">
-        <v>535</v>
+        <v>2245</v>
       </c>
       <c r="C125" t="n">
         <v>8888</v>
       </c>
       <c r="D125" t="n">
-        <v>2806.71</v>
+        <v>883.75</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2820,17 +2820,17 @@
         <v>46217</v>
       </c>
       <c r="B126" t="n">
-        <v>483</v>
+        <v>477</v>
       </c>
       <c r="C126" t="n">
         <v>8888</v>
       </c>
       <c r="D126" t="n">
-        <v>2100.84</v>
+        <v>994.15</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2839,17 +2839,17 @@
         <v>46217</v>
       </c>
       <c r="B127" t="n">
-        <v>2330</v>
+        <v>2015</v>
       </c>
       <c r="C127" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D127" t="n">
-        <v>1923.09</v>
+        <v>2931.07</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2858,17 +2858,17 @@
         <v>46217</v>
       </c>
       <c r="B128" t="n">
-        <v>363</v>
+        <v>1653</v>
       </c>
       <c r="C128" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D128" t="n">
-        <v>1058.27</v>
+        <v>4115.53</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2877,17 +2877,17 @@
         <v>46217</v>
       </c>
       <c r="B129" t="n">
-        <v>2709</v>
+        <v>1064</v>
       </c>
       <c r="C129" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D129" t="n">
-        <v>1667.47</v>
+        <v>451.38</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2896,17 +2896,17 @@
         <v>46217</v>
       </c>
       <c r="B130" t="n">
-        <v>1137</v>
+        <v>1983</v>
       </c>
       <c r="C130" t="n">
         <v>8888</v>
       </c>
       <c r="D130" t="n">
-        <v>3185.1</v>
+        <v>1246.33</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2915,15 +2915,414 @@
         <v>46217</v>
       </c>
       <c r="B131" t="n">
+        <v>2118</v>
+      </c>
+      <c r="C131" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D131" t="n">
+        <v>2646.39</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B132" t="n">
+        <v>2680</v>
+      </c>
+      <c r="C132" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D132" t="n">
+        <v>824.67</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B133" t="n">
+        <v>2637</v>
+      </c>
+      <c r="C133" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D133" t="n">
+        <v>1302.18</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B134" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C134" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D134" t="n">
+        <v>699.05</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B135" t="n">
+        <v>629</v>
+      </c>
+      <c r="C135" t="n">
+        <v>675</v>
+      </c>
+      <c r="D135" t="n">
+        <v>267.79</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B136" t="n">
+        <v>559</v>
+      </c>
+      <c r="C136" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D136" t="n">
+        <v>1562.5</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B137" t="n">
+        <v>1465</v>
+      </c>
+      <c r="C137" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D137" t="n">
+        <v>9346.120000000001</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B138" t="n">
+        <v>2550</v>
+      </c>
+      <c r="C138" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D138" t="n">
+        <v>321.05</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B139" t="n">
+        <v>1756</v>
+      </c>
+      <c r="C139" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D139" t="n">
+        <v>2445</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B140" t="n">
+        <v>363</v>
+      </c>
+      <c r="C140" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D140" t="n">
+        <v>2517.01</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B141" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C141" t="n">
+        <v>874</v>
+      </c>
+      <c r="D141" t="n">
+        <v>1183.42</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B142" t="n">
+        <v>535</v>
+      </c>
+      <c r="C142" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D142" t="n">
+        <v>5293.96</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B143" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C143" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D143" t="n">
+        <v>1512.17</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B144" t="n">
+        <v>2681</v>
+      </c>
+      <c r="C144" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D144" t="n">
+        <v>2775.8</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B145" t="n">
+        <v>363</v>
+      </c>
+      <c r="C145" t="n">
+        <v>1898</v>
+      </c>
+      <c r="D145" t="n">
+        <v>3635.16</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B146" t="n">
+        <v>483</v>
+      </c>
+      <c r="C146" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D146" t="n">
+        <v>2527.71</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B147" t="n">
+        <v>2607</v>
+      </c>
+      <c r="C147" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D147" t="n">
+        <v>1075.36</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B148" t="n">
+        <v>2330</v>
+      </c>
+      <c r="C148" t="n">
+        <v>1954</v>
+      </c>
+      <c r="D148" t="n">
+        <v>1923.09</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B149" t="n">
+        <v>2709</v>
+      </c>
+      <c r="C149" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D149" t="n">
+        <v>1667.47</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B150" t="n">
+        <v>374</v>
+      </c>
+      <c r="C150" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D150" t="n">
+        <v>1150.97</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B151" t="n">
+        <v>1137</v>
+      </c>
+      <c r="C151" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D151" t="n">
+        <v>4413.34</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B152" t="n">
         <v>2251</v>
       </c>
-      <c r="C131" t="n">
+      <c r="C152" t="n">
         <v>3403</v>
       </c>
-      <c r="D131" t="n">
+      <c r="D152" t="n">
         <v>510.18</v>
       </c>
-      <c r="E131" t="inlineStr">
+      <c r="E152" t="inlineStr">
         <is>
           <t>TELEMARKETING</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 15:00:03
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E152"/>
+  <dimension ref="A1:E166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,17 +464,17 @@
         <v>46217</v>
       </c>
       <c r="B2" t="n">
-        <v>1756</v>
+        <v>42</v>
       </c>
       <c r="C2" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D2" t="n">
-        <v>556.23</v>
+        <v>26575.79</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -483,17 +483,17 @@
         <v>46217</v>
       </c>
       <c r="B3" t="n">
-        <v>42</v>
+        <v>1756</v>
       </c>
       <c r="C3" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D3" t="n">
-        <v>24542.62</v>
+        <v>556.23</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -502,17 +502,17 @@
         <v>46217</v>
       </c>
       <c r="B4" t="n">
-        <v>1653</v>
+        <v>1254</v>
       </c>
       <c r="C4" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D4" t="n">
-        <v>4524.08</v>
+        <v>1508.08</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -521,17 +521,17 @@
         <v>46217</v>
       </c>
       <c r="B5" t="n">
-        <v>2109</v>
+        <v>1653</v>
       </c>
       <c r="C5" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D5" t="n">
-        <v>4813.6</v>
+        <v>4524.08</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -540,17 +540,17 @@
         <v>46217</v>
       </c>
       <c r="B6" t="n">
-        <v>2015</v>
+        <v>2109</v>
       </c>
       <c r="C6" t="n">
-        <v>2571</v>
+        <v>8888</v>
       </c>
       <c r="D6" t="n">
-        <v>1790.54</v>
+        <v>4813.6</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -559,17 +559,17 @@
         <v>46217</v>
       </c>
       <c r="B7" t="n">
-        <v>1993</v>
+        <v>2015</v>
       </c>
       <c r="C7" t="n">
-        <v>8888</v>
+        <v>2571</v>
       </c>
       <c r="D7" t="n">
-        <v>1785.44</v>
+        <v>2593.26</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -578,17 +578,17 @@
         <v>46217</v>
       </c>
       <c r="B8" t="n">
-        <v>1102</v>
+        <v>1993</v>
       </c>
       <c r="C8" t="n">
         <v>8888</v>
       </c>
       <c r="D8" t="n">
-        <v>2432.31</v>
+        <v>1785.44</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -597,17 +597,17 @@
         <v>46217</v>
       </c>
       <c r="B9" t="n">
-        <v>1293</v>
+        <v>1102</v>
       </c>
       <c r="C9" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D9" t="n">
-        <v>1337.87</v>
+        <v>2432.31</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -616,17 +616,17 @@
         <v>46217</v>
       </c>
       <c r="B10" t="n">
-        <v>1254</v>
+        <v>1293</v>
       </c>
       <c r="C10" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D10" t="n">
-        <v>428.16</v>
+        <v>1337.87</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -635,17 +635,17 @@
         <v>46217</v>
       </c>
       <c r="B11" t="n">
-        <v>2726</v>
+        <v>2768</v>
       </c>
       <c r="C11" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D11" t="n">
-        <v>640.1799999999999</v>
+        <v>4890.12</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -654,17 +654,17 @@
         <v>46217</v>
       </c>
       <c r="B12" t="n">
-        <v>89</v>
+        <v>2726</v>
       </c>
       <c r="C12" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D12" t="n">
-        <v>5652.15</v>
+        <v>640.1799999999999</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -673,13 +673,13 @@
         <v>46217</v>
       </c>
       <c r="B13" t="n">
-        <v>2768</v>
+        <v>89</v>
       </c>
       <c r="C13" t="n">
         <v>8888</v>
       </c>
       <c r="D13" t="n">
-        <v>3436.6</v>
+        <v>5652.15</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -749,17 +749,17 @@
         <v>46217</v>
       </c>
       <c r="B17" t="n">
-        <v>1756</v>
+        <v>353</v>
       </c>
       <c r="C17" t="n">
         <v>8888</v>
       </c>
       <c r="D17" t="n">
-        <v>1799.7</v>
+        <v>2121.12</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
         <v>46217</v>
       </c>
       <c r="B18" t="n">
-        <v>285</v>
+        <v>1756</v>
       </c>
       <c r="C18" t="n">
         <v>8888</v>
       </c>
       <c r="D18" t="n">
-        <v>2593.28</v>
+        <v>1799.7</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -787,13 +787,13 @@
         <v>46217</v>
       </c>
       <c r="B19" t="n">
-        <v>610</v>
+        <v>285</v>
       </c>
       <c r="C19" t="n">
         <v>8888</v>
       </c>
       <c r="D19" t="n">
-        <v>590.08</v>
+        <v>3092.58</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -806,17 +806,17 @@
         <v>46217</v>
       </c>
       <c r="B20" t="n">
-        <v>1906</v>
+        <v>610</v>
       </c>
       <c r="C20" t="n">
         <v>8888</v>
       </c>
       <c r="D20" t="n">
-        <v>1580.84</v>
+        <v>590.08</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -825,17 +825,17 @@
         <v>46217</v>
       </c>
       <c r="B21" t="n">
-        <v>619</v>
+        <v>1906</v>
       </c>
       <c r="C21" t="n">
         <v>8888</v>
       </c>
       <c r="D21" t="n">
-        <v>236.34</v>
+        <v>2437.98</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -844,17 +844,17 @@
         <v>46217</v>
       </c>
       <c r="B22" t="n">
-        <v>2755</v>
+        <v>619</v>
       </c>
       <c r="C22" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D22" t="n">
-        <v>1133.17</v>
+        <v>236.34</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -863,13 +863,13 @@
         <v>46217</v>
       </c>
       <c r="B23" t="n">
-        <v>2767</v>
+        <v>2755</v>
       </c>
       <c r="C23" t="n">
-        <v>1898</v>
+        <v>2220</v>
       </c>
       <c r="D23" t="n">
-        <v>5000.2</v>
+        <v>1133.17</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -882,17 +882,17 @@
         <v>46217</v>
       </c>
       <c r="B24" t="n">
-        <v>559</v>
+        <v>2767</v>
       </c>
       <c r="C24" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D24" t="n">
-        <v>1200.99</v>
+        <v>5000.2</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -901,17 +901,17 @@
         <v>46217</v>
       </c>
       <c r="B25" t="n">
-        <v>2767</v>
+        <v>559</v>
       </c>
       <c r="C25" t="n">
         <v>8888</v>
       </c>
       <c r="D25" t="n">
-        <v>1175.73</v>
+        <v>1200.99</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
         <v>46217</v>
       </c>
       <c r="B26" t="n">
-        <v>1063</v>
+        <v>2767</v>
       </c>
       <c r="C26" t="n">
         <v>8888</v>
       </c>
       <c r="D26" t="n">
-        <v>1251.14</v>
+        <v>1175.73</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -939,17 +939,17 @@
         <v>46217</v>
       </c>
       <c r="B27" t="n">
-        <v>325</v>
+        <v>1063</v>
       </c>
       <c r="C27" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D27" t="n">
-        <v>868.83</v>
+        <v>1251.14</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -958,17 +958,17 @@
         <v>46217</v>
       </c>
       <c r="B28" t="n">
-        <v>2660</v>
+        <v>325</v>
       </c>
       <c r="C28" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D28" t="n">
-        <v>281.24</v>
+        <v>868.83</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -977,13 +977,13 @@
         <v>46217</v>
       </c>
       <c r="B29" t="n">
-        <v>610</v>
+        <v>2660</v>
       </c>
       <c r="C29" t="n">
         <v>8888</v>
       </c>
       <c r="D29" t="n">
-        <v>235.34</v>
+        <v>281.24</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -996,17 +996,17 @@
         <v>46217</v>
       </c>
       <c r="B30" t="n">
-        <v>424</v>
+        <v>610</v>
       </c>
       <c r="C30" t="n">
         <v>8888</v>
       </c>
       <c r="D30" t="n">
-        <v>3214.29</v>
+        <v>235.34</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1015,17 +1015,17 @@
         <v>46217</v>
       </c>
       <c r="B31" t="n">
-        <v>40</v>
+        <v>424</v>
       </c>
       <c r="C31" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D31" t="n">
-        <v>325.04</v>
+        <v>3214.29</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1034,17 +1034,17 @@
         <v>46217</v>
       </c>
       <c r="B32" t="n">
-        <v>1117</v>
+        <v>40</v>
       </c>
       <c r="C32" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D32" t="n">
-        <v>349.47</v>
+        <v>325.04</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1053,17 +1053,17 @@
         <v>46217</v>
       </c>
       <c r="B33" t="n">
-        <v>949</v>
+        <v>1117</v>
       </c>
       <c r="C33" t="n">
-        <v>998</v>
+        <v>8888</v>
       </c>
       <c r="D33" t="n">
-        <v>129.85</v>
+        <v>349.47</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1072,17 +1072,17 @@
         <v>46217</v>
       </c>
       <c r="B34" t="n">
-        <v>2250</v>
+        <v>949</v>
       </c>
       <c r="C34" t="n">
-        <v>8888</v>
+        <v>998</v>
       </c>
       <c r="D34" t="n">
-        <v>3627.44</v>
+        <v>129.85</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1091,13 +1091,13 @@
         <v>46217</v>
       </c>
       <c r="B35" t="n">
-        <v>2507</v>
+        <v>1853</v>
       </c>
       <c r="C35" t="n">
         <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>4167.12</v>
+        <v>522.4</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1110,13 +1110,13 @@
         <v>46217</v>
       </c>
       <c r="B36" t="n">
-        <v>664</v>
+        <v>2250</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>3523.8</v>
+        <v>4131.57</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1129,17 +1129,17 @@
         <v>46217</v>
       </c>
       <c r="B37" t="n">
-        <v>1906</v>
+        <v>2507</v>
       </c>
       <c r="C37" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D37" t="n">
-        <v>1445.21</v>
+        <v>4167.12</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1148,17 +1148,17 @@
         <v>46217</v>
       </c>
       <c r="B38" t="n">
-        <v>1075</v>
+        <v>664</v>
       </c>
       <c r="C38" t="n">
         <v>8888</v>
       </c>
       <c r="D38" t="n">
-        <v>470.95</v>
+        <v>3815.91</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1167,17 +1167,17 @@
         <v>46217</v>
       </c>
       <c r="B39" t="n">
-        <v>2696</v>
+        <v>1075</v>
       </c>
       <c r="C39" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D39" t="n">
-        <v>677.76</v>
+        <v>1013.2</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1186,13 +1186,13 @@
         <v>46217</v>
       </c>
       <c r="B40" t="n">
-        <v>360</v>
+        <v>1906</v>
       </c>
       <c r="C40" t="n">
-        <v>546</v>
+        <v>1954</v>
       </c>
       <c r="D40" t="n">
-        <v>5188.86</v>
+        <v>1445.21</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1205,17 +1205,17 @@
         <v>46217</v>
       </c>
       <c r="B41" t="n">
-        <v>2491</v>
+        <v>2696</v>
       </c>
       <c r="C41" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D41" t="n">
-        <v>2031.53</v>
+        <v>677.76</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1224,17 +1224,17 @@
         <v>46217</v>
       </c>
       <c r="B42" t="n">
-        <v>2651</v>
+        <v>360</v>
       </c>
       <c r="C42" t="n">
-        <v>8888</v>
+        <v>546</v>
       </c>
       <c r="D42" t="n">
-        <v>638.64</v>
+        <v>5741.5</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1243,17 +1243,17 @@
         <v>46217</v>
       </c>
       <c r="B43" t="n">
-        <v>1293</v>
+        <v>2491</v>
       </c>
       <c r="C43" t="n">
         <v>8888</v>
       </c>
       <c r="D43" t="n">
-        <v>381.82</v>
+        <v>2031.53</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1262,17 +1262,17 @@
         <v>46217</v>
       </c>
       <c r="B44" t="n">
-        <v>2663</v>
+        <v>2651</v>
       </c>
       <c r="C44" t="n">
         <v>8888</v>
       </c>
       <c r="D44" t="n">
-        <v>2146.08</v>
+        <v>638.64</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1281,17 +1281,17 @@
         <v>46217</v>
       </c>
       <c r="B45" t="n">
-        <v>525</v>
+        <v>2695</v>
       </c>
       <c r="C45" t="n">
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>639.9</v>
+        <v>532.53</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1300,17 +1300,17 @@
         <v>46217</v>
       </c>
       <c r="B46" t="n">
-        <v>2711</v>
+        <v>1293</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>750.3200000000001</v>
+        <v>381.82</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1319,17 +1319,17 @@
         <v>46217</v>
       </c>
       <c r="B47" t="n">
-        <v>675</v>
+        <v>2663</v>
       </c>
       <c r="C47" t="n">
         <v>8888</v>
       </c>
       <c r="D47" t="n">
-        <v>289.67</v>
+        <v>2146.08</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1338,13 +1338,13 @@
         <v>46217</v>
       </c>
       <c r="B48" t="n">
-        <v>1063</v>
+        <v>525</v>
       </c>
       <c r="C48" t="n">
         <v>8888</v>
       </c>
       <c r="D48" t="n">
-        <v>1902.46</v>
+        <v>1240.79</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1357,17 +1357,17 @@
         <v>46217</v>
       </c>
       <c r="B49" t="n">
-        <v>1392</v>
+        <v>2711</v>
       </c>
       <c r="C49" t="n">
         <v>8888</v>
       </c>
       <c r="D49" t="n">
-        <v>814.61</v>
+        <v>1953.5</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1376,13 +1376,13 @@
         <v>46217</v>
       </c>
       <c r="B50" t="n">
-        <v>360</v>
+        <v>675</v>
       </c>
       <c r="C50" t="n">
         <v>8888</v>
       </c>
       <c r="D50" t="n">
-        <v>749.13</v>
+        <v>289.67</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1395,17 +1395,17 @@
         <v>46217</v>
       </c>
       <c r="B51" t="n">
-        <v>949</v>
+        <v>1063</v>
       </c>
       <c r="C51" t="n">
-        <v>1134</v>
+        <v>8888</v>
       </c>
       <c r="D51" t="n">
-        <v>327.6</v>
+        <v>1902.46</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1414,13 +1414,13 @@
         <v>46217</v>
       </c>
       <c r="B52" t="n">
-        <v>326</v>
+        <v>1392</v>
       </c>
       <c r="C52" t="n">
         <v>8888</v>
       </c>
       <c r="D52" t="n">
-        <v>212.63</v>
+        <v>814.61</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1433,17 +1433,17 @@
         <v>46217</v>
       </c>
       <c r="B53" t="n">
-        <v>325</v>
+        <v>360</v>
       </c>
       <c r="C53" t="n">
         <v>8888</v>
       </c>
       <c r="D53" t="n">
-        <v>616.95</v>
+        <v>749.13</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1452,17 +1452,17 @@
         <v>46217</v>
       </c>
       <c r="B54" t="n">
-        <v>131</v>
+        <v>949</v>
       </c>
       <c r="C54" t="n">
-        <v>8888</v>
+        <v>1134</v>
       </c>
       <c r="D54" t="n">
-        <v>360.06</v>
+        <v>327.6</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1471,13 +1471,13 @@
         <v>46217</v>
       </c>
       <c r="B55" t="n">
-        <v>2697</v>
+        <v>326</v>
       </c>
       <c r="C55" t="n">
         <v>8888</v>
       </c>
       <c r="D55" t="n">
-        <v>420.48</v>
+        <v>212.63</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1490,17 +1490,17 @@
         <v>46217</v>
       </c>
       <c r="B56" t="n">
-        <v>2279</v>
+        <v>325</v>
       </c>
       <c r="C56" t="n">
         <v>8888</v>
       </c>
       <c r="D56" t="n">
-        <v>1034.25</v>
+        <v>616.95</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1509,17 +1509,17 @@
         <v>46217</v>
       </c>
       <c r="B57" t="n">
-        <v>1116</v>
+        <v>131</v>
       </c>
       <c r="C57" t="n">
         <v>8888</v>
       </c>
       <c r="D57" t="n">
-        <v>1293.89</v>
+        <v>1969.93</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1528,17 +1528,17 @@
         <v>46217</v>
       </c>
       <c r="B58" t="n">
-        <v>131</v>
+        <v>2697</v>
       </c>
       <c r="C58" t="n">
         <v>8888</v>
       </c>
       <c r="D58" t="n">
-        <v>1528.41</v>
+        <v>420.48</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1547,17 +1547,17 @@
         <v>46217</v>
       </c>
       <c r="B59" t="n">
-        <v>1293</v>
+        <v>2279</v>
       </c>
       <c r="C59" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D59" t="n">
-        <v>3534.85</v>
+        <v>1034.25</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1566,13 +1566,13 @@
         <v>46217</v>
       </c>
       <c r="B60" t="n">
-        <v>451</v>
+        <v>1116</v>
       </c>
       <c r="C60" t="n">
         <v>8888</v>
       </c>
       <c r="D60" t="n">
-        <v>2583.46</v>
+        <v>1293.89</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1585,17 +1585,17 @@
         <v>46217</v>
       </c>
       <c r="B61" t="n">
-        <v>1983</v>
+        <v>131</v>
       </c>
       <c r="C61" t="n">
         <v>8888</v>
       </c>
       <c r="D61" t="n">
-        <v>412.16</v>
+        <v>5470.1</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1604,17 +1604,17 @@
         <v>46217</v>
       </c>
       <c r="B62" t="n">
-        <v>2767</v>
+        <v>1293</v>
       </c>
       <c r="C62" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D62" t="n">
-        <v>596.88</v>
+        <v>5154.68</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1623,13 +1623,13 @@
         <v>46217</v>
       </c>
       <c r="B63" t="n">
-        <v>2697</v>
+        <v>1937</v>
       </c>
       <c r="C63" t="n">
         <v>8888</v>
       </c>
       <c r="D63" t="n">
-        <v>2055.26</v>
+        <v>692.86</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1642,17 +1642,17 @@
         <v>46217</v>
       </c>
       <c r="B64" t="n">
-        <v>569</v>
+        <v>1983</v>
       </c>
       <c r="C64" t="n">
         <v>8888</v>
       </c>
       <c r="D64" t="n">
-        <v>2291.64</v>
+        <v>412.16</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1661,13 +1661,13 @@
         <v>46217</v>
       </c>
       <c r="B65" t="n">
-        <v>1063</v>
+        <v>451</v>
       </c>
       <c r="C65" t="n">
         <v>8888</v>
       </c>
       <c r="D65" t="n">
-        <v>352.87</v>
+        <v>2583.46</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1680,13 +1680,13 @@
         <v>46217</v>
       </c>
       <c r="B66" t="n">
-        <v>2687</v>
+        <v>2767</v>
       </c>
       <c r="C66" t="n">
         <v>8888</v>
       </c>
       <c r="D66" t="n">
-        <v>1760.22</v>
+        <v>596.88</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1699,17 +1699,17 @@
         <v>46217</v>
       </c>
       <c r="B67" t="n">
-        <v>629</v>
+        <v>2697</v>
       </c>
       <c r="C67" t="n">
         <v>8888</v>
       </c>
       <c r="D67" t="n">
-        <v>559.15</v>
+        <v>2880.19</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1718,17 +1718,17 @@
         <v>46217</v>
       </c>
       <c r="B68" t="n">
-        <v>1890</v>
+        <v>569</v>
       </c>
       <c r="C68" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D68" t="n">
-        <v>697.04</v>
+        <v>2291.64</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1737,17 +1737,17 @@
         <v>46217</v>
       </c>
       <c r="B69" t="n">
-        <v>58</v>
+        <v>2211</v>
       </c>
       <c r="C69" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D69" t="n">
-        <v>2637.19</v>
+        <v>1833.56</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1756,17 +1756,17 @@
         <v>46217</v>
       </c>
       <c r="B70" t="n">
-        <v>2211</v>
+        <v>1063</v>
       </c>
       <c r="C70" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D70" t="n">
-        <v>967.05</v>
+        <v>352.87</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1775,17 @@
         <v>46217</v>
       </c>
       <c r="B71" t="n">
-        <v>1117</v>
+        <v>2687</v>
       </c>
       <c r="C71" t="n">
         <v>8888</v>
       </c>
       <c r="D71" t="n">
-        <v>581.51</v>
+        <v>1760.22</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1800,11 +1800,11 @@
         <v>8888</v>
       </c>
       <c r="D72" t="n">
-        <v>2049.78</v>
+        <v>559.15</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1813,13 +1813,13 @@
         <v>46217</v>
       </c>
       <c r="B73" t="n">
-        <v>949</v>
+        <v>1890</v>
       </c>
       <c r="C73" t="n">
-        <v>1762</v>
+        <v>1953</v>
       </c>
       <c r="D73" t="n">
-        <v>325.65</v>
+        <v>1122</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -1832,17 +1832,17 @@
         <v>46217</v>
       </c>
       <c r="B74" t="n">
-        <v>2463</v>
+        <v>1289</v>
       </c>
       <c r="C74" t="n">
         <v>8888</v>
       </c>
       <c r="D74" t="n">
-        <v>8336.43</v>
+        <v>1214.09</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1851,17 +1851,17 @@
         <v>46217</v>
       </c>
       <c r="B75" t="n">
-        <v>1064</v>
+        <v>2107</v>
       </c>
       <c r="C75" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D75" t="n">
-        <v>1513.21</v>
+        <v>2000.86</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1870,17 +1870,17 @@
         <v>46217</v>
       </c>
       <c r="B76" t="n">
-        <v>1478</v>
+        <v>1116</v>
       </c>
       <c r="C76" t="n">
         <v>8888</v>
       </c>
       <c r="D76" t="n">
-        <v>1294.76</v>
+        <v>1065.24</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1889,17 +1889,17 @@
         <v>46217</v>
       </c>
       <c r="B77" t="n">
-        <v>358</v>
+        <v>58</v>
       </c>
       <c r="C77" t="n">
         <v>8888</v>
       </c>
       <c r="D77" t="n">
-        <v>1918.33</v>
+        <v>2637.19</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1908,17 +1908,17 @@
         <v>46217</v>
       </c>
       <c r="B78" t="n">
-        <v>2107</v>
+        <v>1117</v>
       </c>
       <c r="C78" t="n">
         <v>8888</v>
       </c>
       <c r="D78" t="n">
-        <v>2745.11</v>
+        <v>581.51</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1927,13 +1927,13 @@
         <v>46217</v>
       </c>
       <c r="B79" t="n">
-        <v>675</v>
+        <v>58</v>
       </c>
       <c r="C79" t="n">
         <v>8888</v>
       </c>
       <c r="D79" t="n">
-        <v>275.17</v>
+        <v>1411.43</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -1946,17 +1946,17 @@
         <v>46217</v>
       </c>
       <c r="B80" t="n">
-        <v>2279</v>
+        <v>629</v>
       </c>
       <c r="C80" t="n">
         <v>8888</v>
       </c>
       <c r="D80" t="n">
-        <v>1165.17</v>
+        <v>2049.78</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1965,13 +1965,13 @@
         <v>46217</v>
       </c>
       <c r="B81" t="n">
-        <v>451</v>
+        <v>949</v>
       </c>
       <c r="C81" t="n">
-        <v>3403</v>
+        <v>1762</v>
       </c>
       <c r="D81" t="n">
-        <v>327.28</v>
+        <v>325.65</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -1984,17 +1984,17 @@
         <v>46217</v>
       </c>
       <c r="B82" t="n">
-        <v>2571</v>
+        <v>2463</v>
       </c>
       <c r="C82" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D82" t="n">
-        <v>2202.75</v>
+        <v>8336.43</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2003,17 +2003,17 @@
         <v>46217</v>
       </c>
       <c r="B83" t="n">
-        <v>610</v>
+        <v>1064</v>
       </c>
       <c r="C83" t="n">
         <v>8888</v>
       </c>
       <c r="D83" t="n">
-        <v>335.61</v>
+        <v>1513.21</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2022,17 +2022,17 @@
         <v>46217</v>
       </c>
       <c r="B84" t="n">
-        <v>1108</v>
+        <v>1478</v>
       </c>
       <c r="C84" t="n">
         <v>8888</v>
       </c>
       <c r="D84" t="n">
-        <v>508.54</v>
+        <v>2261.67</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2041,17 +2041,17 @@
         <v>46217</v>
       </c>
       <c r="B85" t="n">
-        <v>341</v>
+        <v>358</v>
       </c>
       <c r="C85" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D85" t="n">
-        <v>366.88</v>
+        <v>1918.33</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2060,17 +2060,17 @@
         <v>46217</v>
       </c>
       <c r="B86" t="n">
-        <v>1653</v>
+        <v>2107</v>
       </c>
       <c r="C86" t="n">
         <v>8888</v>
       </c>
       <c r="D86" t="n">
-        <v>4383.69</v>
+        <v>2745.11</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2079,13 +2079,13 @@
         <v>46217</v>
       </c>
       <c r="B87" t="n">
-        <v>619</v>
+        <v>675</v>
       </c>
       <c r="C87" t="n">
         <v>8888</v>
       </c>
       <c r="D87" t="n">
-        <v>1557.5</v>
+        <v>678.88</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2098,13 +2098,13 @@
         <v>46217</v>
       </c>
       <c r="B88" t="n">
-        <v>663</v>
+        <v>2279</v>
       </c>
       <c r="C88" t="n">
         <v>8888</v>
       </c>
       <c r="D88" t="n">
-        <v>824.5599999999999</v>
+        <v>1165.17</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2117,17 +2117,17 @@
         <v>46217</v>
       </c>
       <c r="B89" t="n">
-        <v>58</v>
+        <v>451</v>
       </c>
       <c r="C89" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D89" t="n">
-        <v>660.1</v>
+        <v>327.28</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2136,13 +2136,13 @@
         <v>46217</v>
       </c>
       <c r="B90" t="n">
-        <v>429</v>
+        <v>2571</v>
       </c>
       <c r="C90" t="n">
-        <v>2571</v>
+        <v>1312</v>
       </c>
       <c r="D90" t="n">
-        <v>667.12</v>
+        <v>2202.75</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2155,13 +2155,13 @@
         <v>46217</v>
       </c>
       <c r="B91" t="n">
-        <v>2641</v>
+        <v>2782</v>
       </c>
       <c r="C91" t="n">
         <v>8888</v>
       </c>
       <c r="D91" t="n">
-        <v>252.41</v>
+        <v>753.8</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2174,17 +2174,17 @@
         <v>46217</v>
       </c>
       <c r="B92" t="n">
-        <v>1293</v>
+        <v>610</v>
       </c>
       <c r="C92" t="n">
         <v>8888</v>
       </c>
       <c r="D92" t="n">
-        <v>8102.01</v>
+        <v>335.61</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2193,17 +2193,17 @@
         <v>46217</v>
       </c>
       <c r="B93" t="n">
-        <v>483</v>
+        <v>2245</v>
       </c>
       <c r="C93" t="n">
         <v>8888</v>
       </c>
       <c r="D93" t="n">
-        <v>1290.28</v>
+        <v>355.88</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2212,17 +2212,17 @@
         <v>46217</v>
       </c>
       <c r="B94" t="n">
-        <v>2308</v>
+        <v>1108</v>
       </c>
       <c r="C94" t="n">
-        <v>546</v>
+        <v>8888</v>
       </c>
       <c r="D94" t="n">
-        <v>1292.23</v>
+        <v>508.54</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2231,13 +2231,13 @@
         <v>46217</v>
       </c>
       <c r="B95" t="n">
-        <v>2709</v>
+        <v>341</v>
       </c>
       <c r="C95" t="n">
-        <v>2220</v>
+        <v>58</v>
       </c>
       <c r="D95" t="n">
-        <v>1663.5</v>
+        <v>366.88</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2250,13 +2250,13 @@
         <v>46217</v>
       </c>
       <c r="B96" t="n">
-        <v>1937</v>
+        <v>1653</v>
       </c>
       <c r="C96" t="n">
         <v>8888</v>
       </c>
       <c r="D96" t="n">
-        <v>1332.89</v>
+        <v>4383.69</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2269,17 +2269,17 @@
         <v>46217</v>
       </c>
       <c r="B97" t="n">
-        <v>429</v>
+        <v>619</v>
       </c>
       <c r="C97" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D97" t="n">
-        <v>2195.97</v>
+        <v>1557.5</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2288,17 +2288,17 @@
         <v>46217</v>
       </c>
       <c r="B98" t="n">
-        <v>2211</v>
+        <v>663</v>
       </c>
       <c r="C98" t="n">
         <v>8888</v>
       </c>
       <c r="D98" t="n">
-        <v>797.61</v>
+        <v>824.5599999999999</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2307,17 +2307,17 @@
         <v>46217</v>
       </c>
       <c r="B99" t="n">
-        <v>360</v>
+        <v>429</v>
       </c>
       <c r="C99" t="n">
-        <v>8888</v>
+        <v>2571</v>
       </c>
       <c r="D99" t="n">
-        <v>13118.46</v>
+        <v>667.12</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2326,17 +2326,17 @@
         <v>46217</v>
       </c>
       <c r="B100" t="n">
-        <v>131</v>
+        <v>2641</v>
       </c>
       <c r="C100" t="n">
         <v>8888</v>
       </c>
       <c r="D100" t="n">
-        <v>2340.29</v>
+        <v>252.41</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2345,17 +2345,17 @@
         <v>46217</v>
       </c>
       <c r="B101" t="n">
-        <v>131</v>
+        <v>1293</v>
       </c>
       <c r="C101" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D101" t="n">
-        <v>669.39</v>
+        <v>8102.01</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2364,17 +2364,17 @@
         <v>46217</v>
       </c>
       <c r="B102" t="n">
-        <v>1064</v>
+        <v>1465</v>
       </c>
       <c r="C102" t="n">
         <v>8888</v>
       </c>
       <c r="D102" t="n">
-        <v>103288.88</v>
+        <v>814.65</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2383,17 +2383,17 @@
         <v>46217</v>
       </c>
       <c r="B103" t="n">
-        <v>2251</v>
+        <v>483</v>
       </c>
       <c r="C103" t="n">
         <v>8888</v>
       </c>
       <c r="D103" t="n">
-        <v>797.58</v>
+        <v>1290.28</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2402,13 +2402,13 @@
         <v>46217</v>
       </c>
       <c r="B104" t="n">
-        <v>451</v>
+        <v>1064</v>
       </c>
       <c r="C104" t="n">
         <v>8888</v>
       </c>
       <c r="D104" t="n">
-        <v>1371.26</v>
+        <v>104632.21</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2421,17 +2421,17 @@
         <v>46217</v>
       </c>
       <c r="B105" t="n">
-        <v>40</v>
+        <v>131</v>
       </c>
       <c r="C105" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D105" t="n">
-        <v>1093.47</v>
+        <v>876.48</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2440,17 +2440,17 @@
         <v>46217</v>
       </c>
       <c r="B106" t="n">
-        <v>530</v>
+        <v>663</v>
       </c>
       <c r="C106" t="n">
         <v>8888</v>
       </c>
       <c r="D106" t="n">
-        <v>180.08</v>
+        <v>979.4</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2459,17 +2459,17 @@
         <v>46217</v>
       </c>
       <c r="B107" t="n">
-        <v>1137</v>
+        <v>131</v>
       </c>
       <c r="C107" t="n">
         <v>8888</v>
       </c>
       <c r="D107" t="n">
-        <v>2833.69</v>
+        <v>4787.28</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2478,13 +2478,13 @@
         <v>46217</v>
       </c>
       <c r="B108" t="n">
-        <v>1293</v>
+        <v>2308</v>
       </c>
       <c r="C108" t="n">
-        <v>601</v>
+        <v>546</v>
       </c>
       <c r="D108" t="n">
-        <v>456.47</v>
+        <v>1292.23</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -2497,17 +2497,17 @@
         <v>46217</v>
       </c>
       <c r="B109" t="n">
-        <v>2118</v>
+        <v>2709</v>
       </c>
       <c r="C109" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D109" t="n">
-        <v>311.54</v>
+        <v>1663.5</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2516,17 +2516,17 @@
         <v>46217</v>
       </c>
       <c r="B110" t="n">
-        <v>424</v>
+        <v>1937</v>
       </c>
       <c r="C110" t="n">
         <v>8888</v>
       </c>
       <c r="D110" t="n">
-        <v>349.68</v>
+        <v>1492.4</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2535,13 +2535,13 @@
         <v>46217</v>
       </c>
       <c r="B111" t="n">
-        <v>1299</v>
+        <v>429</v>
       </c>
       <c r="C111" t="n">
-        <v>27</v>
+        <v>1281</v>
       </c>
       <c r="D111" t="n">
-        <v>1425.22</v>
+        <v>2195.97</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -2554,17 +2554,17 @@
         <v>46217</v>
       </c>
       <c r="B112" t="n">
-        <v>559</v>
+        <v>2211</v>
       </c>
       <c r="C112" t="n">
         <v>8888</v>
       </c>
       <c r="D112" t="n">
-        <v>1064.63</v>
+        <v>797.61</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2573,17 +2573,17 @@
         <v>46217</v>
       </c>
       <c r="B113" t="n">
-        <v>89</v>
+        <v>360</v>
       </c>
       <c r="C113" t="n">
         <v>8888</v>
       </c>
       <c r="D113" t="n">
-        <v>1506.42</v>
+        <v>13786.36</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2592,17 +2592,17 @@
         <v>46217</v>
       </c>
       <c r="B114" t="n">
-        <v>2250</v>
+        <v>2251</v>
       </c>
       <c r="C114" t="n">
         <v>8888</v>
       </c>
       <c r="D114" t="n">
-        <v>1943.54</v>
+        <v>797.58</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2611,13 +2611,13 @@
         <v>46217</v>
       </c>
       <c r="B115" t="n">
-        <v>767</v>
+        <v>451</v>
       </c>
       <c r="C115" t="n">
         <v>8888</v>
       </c>
       <c r="D115" t="n">
-        <v>472.62</v>
+        <v>1371.26</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -2630,17 +2630,17 @@
         <v>46217</v>
       </c>
       <c r="B116" t="n">
-        <v>2651</v>
+        <v>40</v>
       </c>
       <c r="C116" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D116" t="n">
-        <v>648.71</v>
+        <v>1093.47</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2649,17 +2649,17 @@
         <v>46217</v>
       </c>
       <c r="B117" t="n">
-        <v>2114</v>
+        <v>530</v>
       </c>
       <c r="C117" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D117" t="n">
-        <v>879.03</v>
+        <v>180.08</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2668,17 +2668,17 @@
         <v>46217</v>
       </c>
       <c r="B118" t="n">
-        <v>40</v>
+        <v>1137</v>
       </c>
       <c r="C118" t="n">
         <v>8888</v>
       </c>
       <c r="D118" t="n">
-        <v>3583.39</v>
+        <v>2833.69</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2687,17 +2687,17 @@
         <v>46217</v>
       </c>
       <c r="B119" t="n">
-        <v>40</v>
+        <v>1293</v>
       </c>
       <c r="C119" t="n">
-        <v>8888</v>
+        <v>601</v>
       </c>
       <c r="D119" t="n">
-        <v>2529.31</v>
+        <v>456.47</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2706,17 +2706,17 @@
         <v>46217</v>
       </c>
       <c r="B120" t="n">
-        <v>626</v>
+        <v>2118</v>
       </c>
       <c r="C120" t="n">
         <v>8888</v>
       </c>
       <c r="D120" t="n">
-        <v>13218.02</v>
+        <v>311.54</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2725,17 +2725,17 @@
         <v>46217</v>
       </c>
       <c r="B121" t="n">
-        <v>363</v>
+        <v>424</v>
       </c>
       <c r="C121" t="n">
         <v>8888</v>
       </c>
       <c r="D121" t="n">
-        <v>739.17</v>
+        <v>349.68</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2744,13 +2744,13 @@
         <v>46217</v>
       </c>
       <c r="B122" t="n">
-        <v>675</v>
+        <v>1299</v>
       </c>
       <c r="C122" t="n">
-        <v>1898</v>
+        <v>27</v>
       </c>
       <c r="D122" t="n">
-        <v>107.13</v>
+        <v>3625.32</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -2763,17 +2763,17 @@
         <v>46217</v>
       </c>
       <c r="B123" t="n">
-        <v>636</v>
+        <v>559</v>
       </c>
       <c r="C123" t="n">
         <v>8888</v>
       </c>
       <c r="D123" t="n">
-        <v>5631.89</v>
+        <v>1064.63</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2782,17 +2782,17 @@
         <v>46217</v>
       </c>
       <c r="B124" t="n">
-        <v>1075</v>
+        <v>89</v>
       </c>
       <c r="C124" t="n">
         <v>8888</v>
       </c>
       <c r="D124" t="n">
-        <v>1331.89</v>
+        <v>1506.42</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2801,17 +2801,17 @@
         <v>46217</v>
       </c>
       <c r="B125" t="n">
-        <v>2245</v>
+        <v>2250</v>
       </c>
       <c r="C125" t="n">
         <v>8888</v>
       </c>
       <c r="D125" t="n">
-        <v>883.75</v>
+        <v>1943.54</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2820,17 +2820,17 @@
         <v>46217</v>
       </c>
       <c r="B126" t="n">
-        <v>477</v>
+        <v>767</v>
       </c>
       <c r="C126" t="n">
         <v>8888</v>
       </c>
       <c r="D126" t="n">
-        <v>994.15</v>
+        <v>472.62</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2839,17 +2839,17 @@
         <v>46217</v>
       </c>
       <c r="B127" t="n">
-        <v>2015</v>
+        <v>2651</v>
       </c>
       <c r="C127" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D127" t="n">
-        <v>2931.07</v>
+        <v>648.71</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2858,17 +2858,17 @@
         <v>46217</v>
       </c>
       <c r="B128" t="n">
-        <v>1653</v>
+        <v>2114</v>
       </c>
       <c r="C128" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D128" t="n">
-        <v>4115.53</v>
+        <v>879.03</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2877,17 +2877,17 @@
         <v>46217</v>
       </c>
       <c r="B129" t="n">
-        <v>1064</v>
+        <v>40</v>
       </c>
       <c r="C129" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D129" t="n">
-        <v>451.38</v>
+        <v>3583.39</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2896,13 +2896,13 @@
         <v>46217</v>
       </c>
       <c r="B130" t="n">
-        <v>1983</v>
+        <v>40</v>
       </c>
       <c r="C130" t="n">
         <v>8888</v>
       </c>
       <c r="D130" t="n">
-        <v>1246.33</v>
+        <v>2529.31</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -2915,17 +2915,17 @@
         <v>46217</v>
       </c>
       <c r="B131" t="n">
-        <v>2118</v>
+        <v>626</v>
       </c>
       <c r="C131" t="n">
         <v>8888</v>
       </c>
       <c r="D131" t="n">
-        <v>2646.39</v>
+        <v>13218.02</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2934,17 +2934,17 @@
         <v>46217</v>
       </c>
       <c r="B132" t="n">
-        <v>2680</v>
+        <v>363</v>
       </c>
       <c r="C132" t="n">
         <v>8888</v>
       </c>
       <c r="D132" t="n">
-        <v>824.67</v>
+        <v>739.17</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2953,17 +2953,17 @@
         <v>46217</v>
       </c>
       <c r="B133" t="n">
-        <v>2637</v>
+        <v>675</v>
       </c>
       <c r="C133" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D133" t="n">
-        <v>1302.18</v>
+        <v>107.13</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2972,17 +2972,17 @@
         <v>46217</v>
       </c>
       <c r="B134" t="n">
-        <v>2026</v>
+        <v>636</v>
       </c>
       <c r="C134" t="n">
         <v>8888</v>
       </c>
       <c r="D134" t="n">
-        <v>699.05</v>
+        <v>5631.89</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2991,17 +2991,17 @@
         <v>46217</v>
       </c>
       <c r="B135" t="n">
-        <v>629</v>
+        <v>1075</v>
       </c>
       <c r="C135" t="n">
-        <v>675</v>
+        <v>8888</v>
       </c>
       <c r="D135" t="n">
-        <v>267.79</v>
+        <v>1331.89</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3010,17 +3010,17 @@
         <v>46217</v>
       </c>
       <c r="B136" t="n">
-        <v>559</v>
+        <v>2245</v>
       </c>
       <c r="C136" t="n">
         <v>8888</v>
       </c>
       <c r="D136" t="n">
-        <v>1562.5</v>
+        <v>883.75</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3029,17 +3029,17 @@
         <v>46217</v>
       </c>
       <c r="B137" t="n">
-        <v>1465</v>
+        <v>477</v>
       </c>
       <c r="C137" t="n">
         <v>8888</v>
       </c>
       <c r="D137" t="n">
-        <v>9346.120000000001</v>
+        <v>994.15</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3048,17 +3048,17 @@
         <v>46217</v>
       </c>
       <c r="B138" t="n">
-        <v>2550</v>
+        <v>2015</v>
       </c>
       <c r="C138" t="n">
         <v>8888</v>
       </c>
       <c r="D138" t="n">
-        <v>321.05</v>
+        <v>2931.07</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3067,17 +3067,17 @@
         <v>46217</v>
       </c>
       <c r="B139" t="n">
-        <v>1756</v>
+        <v>1653</v>
       </c>
       <c r="C139" t="n">
         <v>8888</v>
       </c>
       <c r="D139" t="n">
-        <v>2445</v>
+        <v>4115.53</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3086,17 +3086,17 @@
         <v>46217</v>
       </c>
       <c r="B140" t="n">
-        <v>363</v>
+        <v>1064</v>
       </c>
       <c r="C140" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D140" t="n">
-        <v>2517.01</v>
+        <v>1052.68</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3105,17 +3105,17 @@
         <v>46217</v>
       </c>
       <c r="B141" t="n">
-        <v>2698</v>
+        <v>1983</v>
       </c>
       <c r="C141" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D141" t="n">
-        <v>1183.42</v>
+        <v>1246.33</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3124,13 +3124,13 @@
         <v>46217</v>
       </c>
       <c r="B142" t="n">
-        <v>535</v>
+        <v>2118</v>
       </c>
       <c r="C142" t="n">
         <v>8888</v>
       </c>
       <c r="D142" t="n">
-        <v>5293.96</v>
+        <v>4886.49</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3143,13 +3143,13 @@
         <v>46217</v>
       </c>
       <c r="B143" t="n">
-        <v>2250</v>
+        <v>2680</v>
       </c>
       <c r="C143" t="n">
         <v>8888</v>
       </c>
       <c r="D143" t="n">
-        <v>1512.17</v>
+        <v>2285.31</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3162,17 +3162,17 @@
         <v>46217</v>
       </c>
       <c r="B144" t="n">
-        <v>2681</v>
+        <v>2637</v>
       </c>
       <c r="C144" t="n">
         <v>8888</v>
       </c>
       <c r="D144" t="n">
-        <v>2775.8</v>
+        <v>1302.18</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3181,17 +3181,17 @@
         <v>46217</v>
       </c>
       <c r="B145" t="n">
-        <v>363</v>
+        <v>1632</v>
       </c>
       <c r="C145" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D145" t="n">
-        <v>3635.16</v>
+        <v>689.76</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3200,17 +3200,17 @@
         <v>46217</v>
       </c>
       <c r="B146" t="n">
-        <v>483</v>
+        <v>1299</v>
       </c>
       <c r="C146" t="n">
-        <v>8888</v>
+        <v>2522</v>
       </c>
       <c r="D146" t="n">
-        <v>2527.71</v>
+        <v>3319.01</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3219,17 +3219,17 @@
         <v>46217</v>
       </c>
       <c r="B147" t="n">
-        <v>2607</v>
+        <v>2026</v>
       </c>
       <c r="C147" t="n">
         <v>8888</v>
       </c>
       <c r="D147" t="n">
-        <v>1075.36</v>
+        <v>699.05</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3238,17 +3238,17 @@
         <v>46217</v>
       </c>
       <c r="B148" t="n">
-        <v>2330</v>
+        <v>664</v>
       </c>
       <c r="C148" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D148" t="n">
-        <v>1923.09</v>
+        <v>440.92</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3257,17 +3257,17 @@
         <v>46217</v>
       </c>
       <c r="B149" t="n">
-        <v>2709</v>
+        <v>629</v>
       </c>
       <c r="C149" t="n">
-        <v>8888</v>
+        <v>675</v>
       </c>
       <c r="D149" t="n">
-        <v>1667.47</v>
+        <v>267.79</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3276,17 +3276,17 @@
         <v>46217</v>
       </c>
       <c r="B150" t="n">
-        <v>374</v>
+        <v>559</v>
       </c>
       <c r="C150" t="n">
         <v>8888</v>
       </c>
       <c r="D150" t="n">
-        <v>1150.97</v>
+        <v>1562.5</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3295,13 +3295,13 @@
         <v>46217</v>
       </c>
       <c r="B151" t="n">
-        <v>1137</v>
+        <v>1465</v>
       </c>
       <c r="C151" t="n">
         <v>8888</v>
       </c>
       <c r="D151" t="n">
-        <v>4413.34</v>
+        <v>10920.6</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -3314,15 +3314,281 @@
         <v>46217</v>
       </c>
       <c r="B152" t="n">
+        <v>2550</v>
+      </c>
+      <c r="C152" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D152" t="n">
+        <v>321.05</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B153" t="n">
+        <v>1756</v>
+      </c>
+      <c r="C153" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D153" t="n">
+        <v>2445</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B154" t="n">
+        <v>363</v>
+      </c>
+      <c r="C154" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D154" t="n">
+        <v>2517.01</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B155" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C155" t="n">
+        <v>874</v>
+      </c>
+      <c r="D155" t="n">
+        <v>1183.42</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B156" t="n">
+        <v>535</v>
+      </c>
+      <c r="C156" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D156" t="n">
+        <v>5293.96</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B157" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C157" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D157" t="n">
+        <v>2650.33</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B158" t="n">
+        <v>2681</v>
+      </c>
+      <c r="C158" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D158" t="n">
+        <v>2775.8</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B159" t="n">
+        <v>363</v>
+      </c>
+      <c r="C159" t="n">
+        <v>1898</v>
+      </c>
+      <c r="D159" t="n">
+        <v>3635.16</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B160" t="n">
+        <v>483</v>
+      </c>
+      <c r="C160" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D160" t="n">
+        <v>2527.71</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B161" t="n">
+        <v>2607</v>
+      </c>
+      <c r="C161" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D161" t="n">
+        <v>1075.36</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B162" t="n">
+        <v>2330</v>
+      </c>
+      <c r="C162" t="n">
+        <v>1954</v>
+      </c>
+      <c r="D162" t="n">
+        <v>1923.09</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B163" t="n">
+        <v>2709</v>
+      </c>
+      <c r="C163" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D163" t="n">
+        <v>1667.47</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B164" t="n">
+        <v>374</v>
+      </c>
+      <c r="C164" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D164" t="n">
+        <v>1150.97</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B165" t="n">
+        <v>1137</v>
+      </c>
+      <c r="C165" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D165" t="n">
+        <v>4413.34</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B166" t="n">
         <v>2251</v>
       </c>
-      <c r="C152" t="n">
+      <c r="C166" t="n">
         <v>3403</v>
       </c>
-      <c r="D152" t="n">
+      <c r="D166" t="n">
         <v>510.18</v>
       </c>
-      <c r="E152" t="inlineStr">
+      <c r="E166" t="inlineStr">
         <is>
           <t>TELEMARKETING</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 15:30:49
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E166"/>
+  <dimension ref="A1:E192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,13 +521,13 @@
         <v>46217</v>
       </c>
       <c r="B5" t="n">
-        <v>1653</v>
+        <v>6</v>
       </c>
       <c r="C5" t="n">
-        <v>1281</v>
+        <v>1533</v>
       </c>
       <c r="D5" t="n">
-        <v>4524.08</v>
+        <v>1154.58</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -540,13 +540,13 @@
         <v>46217</v>
       </c>
       <c r="B6" t="n">
-        <v>2109</v>
+        <v>1298</v>
       </c>
       <c r="C6" t="n">
         <v>8888</v>
       </c>
       <c r="D6" t="n">
-        <v>4813.6</v>
+        <v>6359.39</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -559,17 +559,17 @@
         <v>46217</v>
       </c>
       <c r="B7" t="n">
-        <v>2015</v>
+        <v>415</v>
       </c>
       <c r="C7" t="n">
-        <v>2571</v>
+        <v>8888</v>
       </c>
       <c r="D7" t="n">
-        <v>2593.26</v>
+        <v>10705.35</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -578,17 +578,17 @@
         <v>46217</v>
       </c>
       <c r="B8" t="n">
-        <v>1993</v>
+        <v>1653</v>
       </c>
       <c r="C8" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D8" t="n">
-        <v>1785.44</v>
+        <v>4524.08</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -597,13 +597,13 @@
         <v>46217</v>
       </c>
       <c r="B9" t="n">
-        <v>1102</v>
+        <v>2109</v>
       </c>
       <c r="C9" t="n">
         <v>8888</v>
       </c>
       <c r="D9" t="n">
-        <v>2432.31</v>
+        <v>4813.6</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -616,13 +616,13 @@
         <v>46217</v>
       </c>
       <c r="B10" t="n">
-        <v>1293</v>
+        <v>2015</v>
       </c>
       <c r="C10" t="n">
-        <v>1281</v>
+        <v>2571</v>
       </c>
       <c r="D10" t="n">
-        <v>1337.87</v>
+        <v>2593.26</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -635,17 +635,17 @@
         <v>46217</v>
       </c>
       <c r="B11" t="n">
-        <v>2768</v>
+        <v>1993</v>
       </c>
       <c r="C11" t="n">
         <v>8888</v>
       </c>
       <c r="D11" t="n">
-        <v>4890.12</v>
+        <v>1785.44</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -654,17 +654,17 @@
         <v>46217</v>
       </c>
       <c r="B12" t="n">
-        <v>2726</v>
+        <v>1102</v>
       </c>
       <c r="C12" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D12" t="n">
-        <v>640.1799999999999</v>
+        <v>3129.4</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -673,17 +673,17 @@
         <v>46217</v>
       </c>
       <c r="B13" t="n">
-        <v>89</v>
+        <v>1293</v>
       </c>
       <c r="C13" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D13" t="n">
-        <v>5652.15</v>
+        <v>1337.87</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -692,17 +692,17 @@
         <v>46217</v>
       </c>
       <c r="B14" t="n">
-        <v>1890</v>
+        <v>2657</v>
       </c>
       <c r="C14" t="n">
-        <v>3449</v>
+        <v>8888</v>
       </c>
       <c r="D14" t="n">
-        <v>589.0599999999999</v>
+        <v>877.0700000000001</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -711,17 +711,17 @@
         <v>46217</v>
       </c>
       <c r="B15" t="n">
-        <v>2641</v>
+        <v>2768</v>
       </c>
       <c r="C15" t="n">
         <v>8888</v>
       </c>
       <c r="D15" t="n">
-        <v>607.79</v>
+        <v>4890.12</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -730,17 +730,17 @@
         <v>46217</v>
       </c>
       <c r="B16" t="n">
-        <v>949</v>
+        <v>2686</v>
       </c>
       <c r="C16" t="n">
-        <v>1258</v>
+        <v>8888</v>
       </c>
       <c r="D16" t="n">
-        <v>196.87</v>
+        <v>422.71</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -749,17 +749,17 @@
         <v>46217</v>
       </c>
       <c r="B17" t="n">
-        <v>353</v>
+        <v>1890</v>
       </c>
       <c r="C17" t="n">
-        <v>8888</v>
+        <v>3449</v>
       </c>
       <c r="D17" t="n">
-        <v>2121.12</v>
+        <v>809.78</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
         <v>46217</v>
       </c>
       <c r="B18" t="n">
-        <v>1756</v>
+        <v>2726</v>
       </c>
       <c r="C18" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D18" t="n">
-        <v>1799.7</v>
+        <v>640.1799999999999</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -787,17 +787,17 @@
         <v>46217</v>
       </c>
       <c r="B19" t="n">
-        <v>285</v>
+        <v>89</v>
       </c>
       <c r="C19" t="n">
         <v>8888</v>
       </c>
       <c r="D19" t="n">
-        <v>3092.58</v>
+        <v>5652.15</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -806,13 +806,13 @@
         <v>46217</v>
       </c>
       <c r="B20" t="n">
-        <v>610</v>
+        <v>2641</v>
       </c>
       <c r="C20" t="n">
         <v>8888</v>
       </c>
       <c r="D20" t="n">
-        <v>590.08</v>
+        <v>607.79</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -825,17 +825,17 @@
         <v>46217</v>
       </c>
       <c r="B21" t="n">
-        <v>1906</v>
+        <v>949</v>
       </c>
       <c r="C21" t="n">
-        <v>8888</v>
+        <v>1258</v>
       </c>
       <c r="D21" t="n">
-        <v>2437.98</v>
+        <v>196.87</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -844,17 +844,17 @@
         <v>46217</v>
       </c>
       <c r="B22" t="n">
-        <v>619</v>
+        <v>353</v>
       </c>
       <c r="C22" t="n">
         <v>8888</v>
       </c>
       <c r="D22" t="n">
-        <v>236.34</v>
+        <v>2121.12</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -863,17 +863,17 @@
         <v>46217</v>
       </c>
       <c r="B23" t="n">
-        <v>2755</v>
+        <v>1756</v>
       </c>
       <c r="C23" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D23" t="n">
-        <v>1133.17</v>
+        <v>1799.7</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -882,17 +882,17 @@
         <v>46217</v>
       </c>
       <c r="B24" t="n">
-        <v>2767</v>
+        <v>285</v>
       </c>
       <c r="C24" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D24" t="n">
-        <v>5000.2</v>
+        <v>3092.58</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -901,17 +901,17 @@
         <v>46217</v>
       </c>
       <c r="B25" t="n">
-        <v>559</v>
+        <v>1906</v>
       </c>
       <c r="C25" t="n">
         <v>8888</v>
       </c>
       <c r="D25" t="n">
-        <v>1200.99</v>
+        <v>3142.54</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
         <v>46217</v>
       </c>
       <c r="B26" t="n">
-        <v>2767</v>
+        <v>1308</v>
       </c>
       <c r="C26" t="n">
         <v>8888</v>
       </c>
       <c r="D26" t="n">
-        <v>1175.73</v>
+        <v>3127.35</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -939,17 +939,17 @@
         <v>46217</v>
       </c>
       <c r="B27" t="n">
-        <v>1063</v>
+        <v>610</v>
       </c>
       <c r="C27" t="n">
         <v>8888</v>
       </c>
       <c r="D27" t="n">
-        <v>1251.14</v>
+        <v>590.08</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -958,17 +958,17 @@
         <v>46217</v>
       </c>
       <c r="B28" t="n">
-        <v>325</v>
+        <v>619</v>
       </c>
       <c r="C28" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D28" t="n">
-        <v>868.83</v>
+        <v>236.34</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -977,17 +977,17 @@
         <v>46217</v>
       </c>
       <c r="B29" t="n">
-        <v>2660</v>
+        <v>2755</v>
       </c>
       <c r="C29" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D29" t="n">
-        <v>281.24</v>
+        <v>1133.17</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -996,17 +996,17 @@
         <v>46217</v>
       </c>
       <c r="B30" t="n">
-        <v>610</v>
+        <v>2767</v>
       </c>
       <c r="C30" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D30" t="n">
-        <v>235.34</v>
+        <v>5000.2</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1015,17 +1015,17 @@
         <v>46217</v>
       </c>
       <c r="B31" t="n">
-        <v>424</v>
+        <v>559</v>
       </c>
       <c r="C31" t="n">
         <v>8888</v>
       </c>
       <c r="D31" t="n">
-        <v>3214.29</v>
+        <v>1200.99</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1034,17 +1034,17 @@
         <v>46217</v>
       </c>
       <c r="B32" t="n">
-        <v>40</v>
+        <v>358</v>
       </c>
       <c r="C32" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D32" t="n">
-        <v>325.04</v>
+        <v>1301.77</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1053,17 +1053,17 @@
         <v>46217</v>
       </c>
       <c r="B33" t="n">
-        <v>1117</v>
+        <v>609</v>
       </c>
       <c r="C33" t="n">
         <v>8888</v>
       </c>
       <c r="D33" t="n">
-        <v>349.47</v>
+        <v>962.08</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1072,17 +1072,17 @@
         <v>46217</v>
       </c>
       <c r="B34" t="n">
-        <v>949</v>
+        <v>2507</v>
       </c>
       <c r="C34" t="n">
-        <v>998</v>
+        <v>8888</v>
       </c>
       <c r="D34" t="n">
-        <v>129.85</v>
+        <v>448.36</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1091,17 +1091,17 @@
         <v>46217</v>
       </c>
       <c r="B35" t="n">
-        <v>1853</v>
+        <v>2767</v>
       </c>
       <c r="C35" t="n">
         <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>522.4</v>
+        <v>1175.73</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1110,17 @@
         <v>46217</v>
       </c>
       <c r="B36" t="n">
-        <v>2250</v>
+        <v>1063</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>4131.57</v>
+        <v>1251.14</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1129,17 @@
         <v>46217</v>
       </c>
       <c r="B37" t="n">
-        <v>2507</v>
+        <v>325</v>
       </c>
       <c r="C37" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D37" t="n">
-        <v>4167.12</v>
+        <v>868.83</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1148,17 +1148,17 @@
         <v>46217</v>
       </c>
       <c r="B38" t="n">
-        <v>664</v>
+        <v>2660</v>
       </c>
       <c r="C38" t="n">
         <v>8888</v>
       </c>
       <c r="D38" t="n">
-        <v>3815.91</v>
+        <v>281.24</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1167,13 +1167,13 @@
         <v>46217</v>
       </c>
       <c r="B39" t="n">
-        <v>1075</v>
+        <v>610</v>
       </c>
       <c r="C39" t="n">
         <v>8888</v>
       </c>
       <c r="D39" t="n">
-        <v>1013.2</v>
+        <v>235.34</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1186,17 +1186,17 @@
         <v>46217</v>
       </c>
       <c r="B40" t="n">
-        <v>1906</v>
+        <v>424</v>
       </c>
       <c r="C40" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D40" t="n">
-        <v>1445.21</v>
+        <v>3214.29</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
         <v>46217</v>
       </c>
       <c r="B41" t="n">
-        <v>2696</v>
+        <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>1312</v>
+        <v>58</v>
       </c>
       <c r="D41" t="n">
-        <v>677.76</v>
+        <v>325.04</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1224,17 +1224,17 @@
         <v>46217</v>
       </c>
       <c r="B42" t="n">
-        <v>360</v>
+        <v>1117</v>
       </c>
       <c r="C42" t="n">
-        <v>546</v>
+        <v>8888</v>
       </c>
       <c r="D42" t="n">
-        <v>5741.5</v>
+        <v>349.47</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1243,17 +1243,17 @@
         <v>46217</v>
       </c>
       <c r="B43" t="n">
-        <v>2491</v>
+        <v>949</v>
       </c>
       <c r="C43" t="n">
-        <v>8888</v>
+        <v>998</v>
       </c>
       <c r="D43" t="n">
-        <v>2031.53</v>
+        <v>129.85</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1262,17 +1262,17 @@
         <v>46217</v>
       </c>
       <c r="B44" t="n">
-        <v>2651</v>
+        <v>1853</v>
       </c>
       <c r="C44" t="n">
         <v>8888</v>
       </c>
       <c r="D44" t="n">
-        <v>638.64</v>
+        <v>522.4</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1281,13 +1281,13 @@
         <v>46217</v>
       </c>
       <c r="B45" t="n">
-        <v>2695</v>
+        <v>2250</v>
       </c>
       <c r="C45" t="n">
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>532.53</v>
+        <v>4131.57</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1300,17 +1300,17 @@
         <v>46217</v>
       </c>
       <c r="B46" t="n">
-        <v>1293</v>
+        <v>2507</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>381.82</v>
+        <v>4167.12</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1319,17 +1319,17 @@
         <v>46217</v>
       </c>
       <c r="B47" t="n">
-        <v>2663</v>
+        <v>664</v>
       </c>
       <c r="C47" t="n">
         <v>8888</v>
       </c>
       <c r="D47" t="n">
-        <v>2146.08</v>
+        <v>3815.91</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1338,13 +1338,13 @@
         <v>46217</v>
       </c>
       <c r="B48" t="n">
-        <v>525</v>
+        <v>1075</v>
       </c>
       <c r="C48" t="n">
         <v>8888</v>
       </c>
       <c r="D48" t="n">
-        <v>1240.79</v>
+        <v>1013.2</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1357,17 +1357,17 @@
         <v>46217</v>
       </c>
       <c r="B49" t="n">
-        <v>2711</v>
+        <v>1906</v>
       </c>
       <c r="C49" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D49" t="n">
-        <v>1953.5</v>
+        <v>1445.21</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1376,17 +1376,17 @@
         <v>46217</v>
       </c>
       <c r="B50" t="n">
-        <v>675</v>
+        <v>595</v>
       </c>
       <c r="C50" t="n">
-        <v>8888</v>
+        <v>691</v>
       </c>
       <c r="D50" t="n">
-        <v>289.67</v>
+        <v>314.52</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1395,17 +1395,17 @@
         <v>46217</v>
       </c>
       <c r="B51" t="n">
-        <v>1063</v>
+        <v>2696</v>
       </c>
       <c r="C51" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D51" t="n">
-        <v>1902.46</v>
+        <v>677.76</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1414,13 +1414,13 @@
         <v>46217</v>
       </c>
       <c r="B52" t="n">
-        <v>1392</v>
+        <v>525</v>
       </c>
       <c r="C52" t="n">
         <v>8888</v>
       </c>
       <c r="D52" t="n">
-        <v>814.61</v>
+        <v>490.08</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1433,17 +1433,17 @@
         <v>46217</v>
       </c>
       <c r="B53" t="n">
-        <v>360</v>
+        <v>2491</v>
       </c>
       <c r="C53" t="n">
         <v>8888</v>
       </c>
       <c r="D53" t="n">
-        <v>749.13</v>
+        <v>2909.58</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1452,13 +1452,13 @@
         <v>46217</v>
       </c>
       <c r="B54" t="n">
-        <v>949</v>
+        <v>360</v>
       </c>
       <c r="C54" t="n">
-        <v>1134</v>
+        <v>546</v>
       </c>
       <c r="D54" t="n">
-        <v>327.6</v>
+        <v>6094.25</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1471,17 +1471,17 @@
         <v>46217</v>
       </c>
       <c r="B55" t="n">
-        <v>326</v>
+        <v>2651</v>
       </c>
       <c r="C55" t="n">
         <v>8888</v>
       </c>
       <c r="D55" t="n">
-        <v>212.63</v>
+        <v>638.64</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1490,17 +1490,17 @@
         <v>46217</v>
       </c>
       <c r="B56" t="n">
-        <v>325</v>
+        <v>2695</v>
       </c>
       <c r="C56" t="n">
         <v>8888</v>
       </c>
       <c r="D56" t="n">
-        <v>616.95</v>
+        <v>532.53</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1509,13 +1509,13 @@
         <v>46217</v>
       </c>
       <c r="B57" t="n">
-        <v>131</v>
+        <v>1293</v>
       </c>
       <c r="C57" t="n">
         <v>8888</v>
       </c>
       <c r="D57" t="n">
-        <v>1969.93</v>
+        <v>381.82</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1528,17 +1528,17 @@
         <v>46217</v>
       </c>
       <c r="B58" t="n">
-        <v>2697</v>
+        <v>2663</v>
       </c>
       <c r="C58" t="n">
         <v>8888</v>
       </c>
       <c r="D58" t="n">
-        <v>420.48</v>
+        <v>2146.08</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1547,13 +1547,13 @@
         <v>46217</v>
       </c>
       <c r="B59" t="n">
-        <v>2279</v>
+        <v>525</v>
       </c>
       <c r="C59" t="n">
         <v>8888</v>
       </c>
       <c r="D59" t="n">
-        <v>1034.25</v>
+        <v>1240.79</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1566,17 +1566,17 @@
         <v>46217</v>
       </c>
       <c r="B60" t="n">
-        <v>1116</v>
+        <v>2711</v>
       </c>
       <c r="C60" t="n">
         <v>8888</v>
       </c>
       <c r="D60" t="n">
-        <v>1293.89</v>
+        <v>2193.56</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1585,13 +1585,13 @@
         <v>46217</v>
       </c>
       <c r="B61" t="n">
-        <v>131</v>
+        <v>1317</v>
       </c>
       <c r="C61" t="n">
         <v>8888</v>
       </c>
       <c r="D61" t="n">
-        <v>5470.1</v>
+        <v>787.51</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1604,17 +1604,17 @@
         <v>46217</v>
       </c>
       <c r="B62" t="n">
-        <v>1293</v>
+        <v>675</v>
       </c>
       <c r="C62" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D62" t="n">
-        <v>5154.68</v>
+        <v>289.67</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1623,13 +1623,13 @@
         <v>46217</v>
       </c>
       <c r="B63" t="n">
-        <v>1937</v>
+        <v>1063</v>
       </c>
       <c r="C63" t="n">
         <v>8888</v>
       </c>
       <c r="D63" t="n">
-        <v>692.86</v>
+        <v>1902.46</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1642,17 +1642,17 @@
         <v>46217</v>
       </c>
       <c r="B64" t="n">
-        <v>1983</v>
+        <v>1658</v>
       </c>
       <c r="C64" t="n">
         <v>8888</v>
       </c>
       <c r="D64" t="n">
-        <v>412.16</v>
+        <v>1357.94</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1661,17 +1661,17 @@
         <v>46217</v>
       </c>
       <c r="B65" t="n">
-        <v>451</v>
+        <v>1392</v>
       </c>
       <c r="C65" t="n">
         <v>8888</v>
       </c>
       <c r="D65" t="n">
-        <v>2583.46</v>
+        <v>814.61</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1680,17 +1680,17 @@
         <v>46217</v>
       </c>
       <c r="B66" t="n">
-        <v>2767</v>
+        <v>360</v>
       </c>
       <c r="C66" t="n">
         <v>8888</v>
       </c>
       <c r="D66" t="n">
-        <v>596.88</v>
+        <v>749.13</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1699,17 +1699,17 @@
         <v>46217</v>
       </c>
       <c r="B67" t="n">
-        <v>2697</v>
+        <v>949</v>
       </c>
       <c r="C67" t="n">
-        <v>8888</v>
+        <v>1134</v>
       </c>
       <c r="D67" t="n">
-        <v>2880.19</v>
+        <v>327.6</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1718,13 +1718,13 @@
         <v>46217</v>
       </c>
       <c r="B68" t="n">
-        <v>569</v>
+        <v>2133</v>
       </c>
       <c r="C68" t="n">
         <v>8888</v>
       </c>
       <c r="D68" t="n">
-        <v>2291.64</v>
+        <v>66030.34</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1737,17 +1737,17 @@
         <v>46217</v>
       </c>
       <c r="B69" t="n">
-        <v>2211</v>
+        <v>326</v>
       </c>
       <c r="C69" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D69" t="n">
-        <v>1833.56</v>
+        <v>360.45</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1756,17 +1756,17 @@
         <v>46217</v>
       </c>
       <c r="B70" t="n">
-        <v>1063</v>
+        <v>325</v>
       </c>
       <c r="C70" t="n">
         <v>8888</v>
       </c>
       <c r="D70" t="n">
-        <v>352.87</v>
+        <v>774.73</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1775,17 @@
         <v>46217</v>
       </c>
       <c r="B71" t="n">
-        <v>2687</v>
+        <v>1293</v>
       </c>
       <c r="C71" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D71" t="n">
-        <v>1760.22</v>
+        <v>8365.559999999999</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1794,17 +1794,17 @@
         <v>46217</v>
       </c>
       <c r="B72" t="n">
-        <v>629</v>
+        <v>131</v>
       </c>
       <c r="C72" t="n">
         <v>8888</v>
       </c>
       <c r="D72" t="n">
-        <v>559.15</v>
+        <v>1969.93</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1813,17 +1813,17 @@
         <v>46217</v>
       </c>
       <c r="B73" t="n">
-        <v>1890</v>
+        <v>2697</v>
       </c>
       <c r="C73" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D73" t="n">
-        <v>1122</v>
+        <v>420.48</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1832,13 +1832,13 @@
         <v>46217</v>
       </c>
       <c r="B74" t="n">
-        <v>1289</v>
+        <v>2279</v>
       </c>
       <c r="C74" t="n">
         <v>8888</v>
       </c>
       <c r="D74" t="n">
-        <v>1214.09</v>
+        <v>1034.25</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -1851,17 +1851,17 @@
         <v>46217</v>
       </c>
       <c r="B75" t="n">
-        <v>2107</v>
+        <v>1116</v>
       </c>
       <c r="C75" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D75" t="n">
-        <v>2000.86</v>
+        <v>1293.89</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1870,13 +1870,13 @@
         <v>46217</v>
       </c>
       <c r="B76" t="n">
-        <v>1116</v>
+        <v>131</v>
       </c>
       <c r="C76" t="n">
         <v>8888</v>
       </c>
       <c r="D76" t="n">
-        <v>1065.24</v>
+        <v>5470.1</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -1889,17 +1889,17 @@
         <v>46217</v>
       </c>
       <c r="B77" t="n">
-        <v>58</v>
+        <v>1937</v>
       </c>
       <c r="C77" t="n">
         <v>8888</v>
       </c>
       <c r="D77" t="n">
-        <v>2637.19</v>
+        <v>692.86</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1908,17 +1908,17 @@
         <v>46217</v>
       </c>
       <c r="B78" t="n">
-        <v>1117</v>
+        <v>1983</v>
       </c>
       <c r="C78" t="n">
         <v>8888</v>
       </c>
       <c r="D78" t="n">
-        <v>581.51</v>
+        <v>412.16</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1927,17 +1927,17 @@
         <v>46217</v>
       </c>
       <c r="B79" t="n">
-        <v>58</v>
+        <v>451</v>
       </c>
       <c r="C79" t="n">
         <v>8888</v>
       </c>
       <c r="D79" t="n">
-        <v>1411.43</v>
+        <v>2583.46</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1946,13 +1946,13 @@
         <v>46217</v>
       </c>
       <c r="B80" t="n">
-        <v>629</v>
+        <v>2767</v>
       </c>
       <c r="C80" t="n">
         <v>8888</v>
       </c>
       <c r="D80" t="n">
-        <v>2049.78</v>
+        <v>920.85</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -1965,17 +1965,17 @@
         <v>46217</v>
       </c>
       <c r="B81" t="n">
-        <v>949</v>
+        <v>2697</v>
       </c>
       <c r="C81" t="n">
-        <v>1762</v>
+        <v>8888</v>
       </c>
       <c r="D81" t="n">
-        <v>325.65</v>
+        <v>2880.19</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1984,17 +1984,17 @@
         <v>46217</v>
       </c>
       <c r="B82" t="n">
-        <v>2463</v>
+        <v>569</v>
       </c>
       <c r="C82" t="n">
         <v>8888</v>
       </c>
       <c r="D82" t="n">
-        <v>8336.43</v>
+        <v>2291.64</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2003,17 +2003,17 @@
         <v>46217</v>
       </c>
       <c r="B83" t="n">
-        <v>1064</v>
+        <v>2211</v>
       </c>
       <c r="C83" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D83" t="n">
-        <v>1513.21</v>
+        <v>1833.56</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2022,13 +2022,13 @@
         <v>46217</v>
       </c>
       <c r="B84" t="n">
-        <v>1478</v>
+        <v>1063</v>
       </c>
       <c r="C84" t="n">
         <v>8888</v>
       </c>
       <c r="D84" t="n">
-        <v>2261.67</v>
+        <v>352.87</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2041,17 +2041,17 @@
         <v>46217</v>
       </c>
       <c r="B85" t="n">
-        <v>358</v>
+        <v>2687</v>
       </c>
       <c r="C85" t="n">
         <v>8888</v>
       </c>
       <c r="D85" t="n">
-        <v>1918.33</v>
+        <v>1760.22</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2060,17 +2060,17 @@
         <v>46217</v>
       </c>
       <c r="B86" t="n">
-        <v>2107</v>
+        <v>629</v>
       </c>
       <c r="C86" t="n">
         <v>8888</v>
       </c>
       <c r="D86" t="n">
-        <v>2745.11</v>
+        <v>559.15</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2079,17 +2079,17 @@
         <v>46217</v>
       </c>
       <c r="B87" t="n">
-        <v>675</v>
+        <v>1890</v>
       </c>
       <c r="C87" t="n">
-        <v>8888</v>
+        <v>1953</v>
       </c>
       <c r="D87" t="n">
-        <v>678.88</v>
+        <v>1122</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2098,17 +2098,17 @@
         <v>46217</v>
       </c>
       <c r="B88" t="n">
-        <v>2279</v>
+        <v>1289</v>
       </c>
       <c r="C88" t="n">
         <v>8888</v>
       </c>
       <c r="D88" t="n">
-        <v>1165.17</v>
+        <v>1214.09</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2117,13 +2117,13 @@
         <v>46217</v>
       </c>
       <c r="B89" t="n">
-        <v>451</v>
+        <v>2107</v>
       </c>
       <c r="C89" t="n">
-        <v>3403</v>
+        <v>1954</v>
       </c>
       <c r="D89" t="n">
-        <v>327.28</v>
+        <v>2000.86</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2136,17 +2136,17 @@
         <v>46217</v>
       </c>
       <c r="B90" t="n">
-        <v>2571</v>
+        <v>1116</v>
       </c>
       <c r="C90" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D90" t="n">
-        <v>2202.75</v>
+        <v>1065.24</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2155,17 +2155,17 @@
         <v>46217</v>
       </c>
       <c r="B91" t="n">
-        <v>2782</v>
+        <v>58</v>
       </c>
       <c r="C91" t="n">
         <v>8888</v>
       </c>
       <c r="D91" t="n">
-        <v>753.8</v>
+        <v>2637.19</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2174,17 +2174,17 @@
         <v>46217</v>
       </c>
       <c r="B92" t="n">
-        <v>610</v>
+        <v>1117</v>
       </c>
       <c r="C92" t="n">
         <v>8888</v>
       </c>
       <c r="D92" t="n">
-        <v>335.61</v>
+        <v>581.51</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2193,13 +2193,13 @@
         <v>46217</v>
       </c>
       <c r="B93" t="n">
-        <v>2245</v>
+        <v>58</v>
       </c>
       <c r="C93" t="n">
         <v>8888</v>
       </c>
       <c r="D93" t="n">
-        <v>355.88</v>
+        <v>1411.43</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2212,17 +2212,17 @@
         <v>46217</v>
       </c>
       <c r="B94" t="n">
-        <v>1108</v>
+        <v>629</v>
       </c>
       <c r="C94" t="n">
         <v>8888</v>
       </c>
       <c r="D94" t="n">
-        <v>508.54</v>
+        <v>2049.78</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2231,17 +2231,17 @@
         <v>46217</v>
       </c>
       <c r="B95" t="n">
-        <v>341</v>
+        <v>595</v>
       </c>
       <c r="C95" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D95" t="n">
-        <v>366.88</v>
+        <v>3191</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2250,17 +2250,17 @@
         <v>46217</v>
       </c>
       <c r="B96" t="n">
-        <v>1653</v>
+        <v>949</v>
       </c>
       <c r="C96" t="n">
-        <v>8888</v>
+        <v>1762</v>
       </c>
       <c r="D96" t="n">
-        <v>4383.69</v>
+        <v>325.65</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2269,17 +2269,17 @@
         <v>46217</v>
       </c>
       <c r="B97" t="n">
-        <v>619</v>
+        <v>2463</v>
       </c>
       <c r="C97" t="n">
         <v>8888</v>
       </c>
       <c r="D97" t="n">
-        <v>1557.5</v>
+        <v>8336.43</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2288,13 +2288,13 @@
         <v>46217</v>
       </c>
       <c r="B98" t="n">
-        <v>663</v>
+        <v>1064</v>
       </c>
       <c r="C98" t="n">
         <v>8888</v>
       </c>
       <c r="D98" t="n">
-        <v>824.5599999999999</v>
+        <v>1513.21</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2307,17 +2307,17 @@
         <v>46217</v>
       </c>
       <c r="B99" t="n">
-        <v>429</v>
+        <v>1478</v>
       </c>
       <c r="C99" t="n">
-        <v>2571</v>
+        <v>8888</v>
       </c>
       <c r="D99" t="n">
-        <v>667.12</v>
+        <v>2261.67</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2326,17 +2326,17 @@
         <v>46217</v>
       </c>
       <c r="B100" t="n">
-        <v>2641</v>
+        <v>358</v>
       </c>
       <c r="C100" t="n">
         <v>8888</v>
       </c>
       <c r="D100" t="n">
-        <v>252.41</v>
+        <v>1918.33</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2345,13 +2345,13 @@
         <v>46217</v>
       </c>
       <c r="B101" t="n">
-        <v>1293</v>
+        <v>2107</v>
       </c>
       <c r="C101" t="n">
         <v>8888</v>
       </c>
       <c r="D101" t="n">
-        <v>8102.01</v>
+        <v>2745.11</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2364,17 +2364,17 @@
         <v>46217</v>
       </c>
       <c r="B102" t="n">
-        <v>1465</v>
+        <v>675</v>
       </c>
       <c r="C102" t="n">
         <v>8888</v>
       </c>
       <c r="D102" t="n">
-        <v>814.65</v>
+        <v>678.88</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2383,13 +2383,13 @@
         <v>46217</v>
       </c>
       <c r="B103" t="n">
-        <v>483</v>
+        <v>2279</v>
       </c>
       <c r="C103" t="n">
         <v>8888</v>
       </c>
       <c r="D103" t="n">
-        <v>1290.28</v>
+        <v>1165.17</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2402,17 +2402,17 @@
         <v>46217</v>
       </c>
       <c r="B104" t="n">
-        <v>1064</v>
+        <v>451</v>
       </c>
       <c r="C104" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D104" t="n">
-        <v>104632.21</v>
+        <v>327.28</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2421,13 +2421,13 @@
         <v>46217</v>
       </c>
       <c r="B105" t="n">
-        <v>131</v>
+        <v>2571</v>
       </c>
       <c r="C105" t="n">
-        <v>27</v>
+        <v>1312</v>
       </c>
       <c r="D105" t="n">
-        <v>876.48</v>
+        <v>2202.75</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2440,17 +2440,17 @@
         <v>46217</v>
       </c>
       <c r="B106" t="n">
-        <v>663</v>
+        <v>2782</v>
       </c>
       <c r="C106" t="n">
         <v>8888</v>
       </c>
       <c r="D106" t="n">
-        <v>979.4</v>
+        <v>753.8</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2459,17 +2459,17 @@
         <v>46217</v>
       </c>
       <c r="B107" t="n">
-        <v>131</v>
+        <v>610</v>
       </c>
       <c r="C107" t="n">
         <v>8888</v>
       </c>
       <c r="D107" t="n">
-        <v>4787.28</v>
+        <v>335.61</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2478,17 +2478,17 @@
         <v>46217</v>
       </c>
       <c r="B108" t="n">
-        <v>2308</v>
+        <v>2245</v>
       </c>
       <c r="C108" t="n">
-        <v>546</v>
+        <v>8888</v>
       </c>
       <c r="D108" t="n">
-        <v>1292.23</v>
+        <v>355.88</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2497,17 +2497,17 @@
         <v>46217</v>
       </c>
       <c r="B109" t="n">
-        <v>2709</v>
+        <v>1108</v>
       </c>
       <c r="C109" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D109" t="n">
-        <v>1663.5</v>
+        <v>508.54</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2516,17 +2516,17 @@
         <v>46217</v>
       </c>
       <c r="B110" t="n">
-        <v>1937</v>
+        <v>341</v>
       </c>
       <c r="C110" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D110" t="n">
-        <v>1492.4</v>
+        <v>366.88</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2535,13 +2535,13 @@
         <v>46217</v>
       </c>
       <c r="B111" t="n">
-        <v>429</v>
+        <v>525</v>
       </c>
       <c r="C111" t="n">
-        <v>1281</v>
+        <v>1087</v>
       </c>
       <c r="D111" t="n">
-        <v>2195.97</v>
+        <v>1830.26</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -2554,17 +2554,17 @@
         <v>46217</v>
       </c>
       <c r="B112" t="n">
-        <v>2211</v>
+        <v>1653</v>
       </c>
       <c r="C112" t="n">
         <v>8888</v>
       </c>
       <c r="D112" t="n">
-        <v>797.61</v>
+        <v>4383.69</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2573,13 +2573,13 @@
         <v>46217</v>
       </c>
       <c r="B113" t="n">
-        <v>360</v>
+        <v>619</v>
       </c>
       <c r="C113" t="n">
         <v>8888</v>
       </c>
       <c r="D113" t="n">
-        <v>13786.36</v>
+        <v>1557.5</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -2592,17 +2592,17 @@
         <v>46217</v>
       </c>
       <c r="B114" t="n">
-        <v>2251</v>
+        <v>1518</v>
       </c>
       <c r="C114" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D114" t="n">
-        <v>797.58</v>
+        <v>479.84</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2611,17 +2611,17 @@
         <v>46217</v>
       </c>
       <c r="B115" t="n">
-        <v>451</v>
+        <v>663</v>
       </c>
       <c r="C115" t="n">
         <v>8888</v>
       </c>
       <c r="D115" t="n">
-        <v>1371.26</v>
+        <v>824.5599999999999</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2630,17 +2630,17 @@
         <v>46217</v>
       </c>
       <c r="B116" t="n">
-        <v>40</v>
+        <v>2089</v>
       </c>
       <c r="C116" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D116" t="n">
-        <v>1093.47</v>
+        <v>822.05</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2649,17 +2649,17 @@
         <v>46217</v>
       </c>
       <c r="B117" t="n">
-        <v>530</v>
+        <v>2133</v>
       </c>
       <c r="C117" t="n">
-        <v>8888</v>
+        <v>691</v>
       </c>
       <c r="D117" t="n">
-        <v>180.08</v>
+        <v>1414.98</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2668,17 +2668,17 @@
         <v>46217</v>
       </c>
       <c r="B118" t="n">
-        <v>1137</v>
+        <v>429</v>
       </c>
       <c r="C118" t="n">
-        <v>8888</v>
+        <v>2571</v>
       </c>
       <c r="D118" t="n">
-        <v>2833.69</v>
+        <v>667.12</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2687,17 +2687,17 @@
         <v>46217</v>
       </c>
       <c r="B119" t="n">
-        <v>1293</v>
+        <v>2641</v>
       </c>
       <c r="C119" t="n">
-        <v>601</v>
+        <v>8888</v>
       </c>
       <c r="D119" t="n">
-        <v>456.47</v>
+        <v>252.41</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2706,17 +2706,17 @@
         <v>46217</v>
       </c>
       <c r="B120" t="n">
-        <v>2118</v>
+        <v>1293</v>
       </c>
       <c r="C120" t="n">
         <v>8888</v>
       </c>
       <c r="D120" t="n">
-        <v>311.54</v>
+        <v>8102.01</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2725,17 +2725,17 @@
         <v>46217</v>
       </c>
       <c r="B121" t="n">
-        <v>424</v>
+        <v>1465</v>
       </c>
       <c r="C121" t="n">
         <v>8888</v>
       </c>
       <c r="D121" t="n">
-        <v>349.68</v>
+        <v>814.65</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2744,17 +2744,17 @@
         <v>46217</v>
       </c>
       <c r="B122" t="n">
-        <v>1299</v>
+        <v>483</v>
       </c>
       <c r="C122" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D122" t="n">
-        <v>3625.32</v>
+        <v>1980.79</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2763,17 +2763,17 @@
         <v>46217</v>
       </c>
       <c r="B123" t="n">
-        <v>559</v>
+        <v>1064</v>
       </c>
       <c r="C123" t="n">
         <v>8888</v>
       </c>
       <c r="D123" t="n">
-        <v>1064.63</v>
+        <v>104632.21</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2782,17 +2782,17 @@
         <v>46217</v>
       </c>
       <c r="B124" t="n">
-        <v>89</v>
+        <v>131</v>
       </c>
       <c r="C124" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D124" t="n">
-        <v>1506.42</v>
+        <v>876.48</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2801,13 +2801,13 @@
         <v>46217</v>
       </c>
       <c r="B125" t="n">
-        <v>2250</v>
+        <v>663</v>
       </c>
       <c r="C125" t="n">
         <v>8888</v>
       </c>
       <c r="D125" t="n">
-        <v>1943.54</v>
+        <v>1769.59</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -2820,17 +2820,17 @@
         <v>46217</v>
       </c>
       <c r="B126" t="n">
-        <v>767</v>
+        <v>131</v>
       </c>
       <c r="C126" t="n">
         <v>8888</v>
       </c>
       <c r="D126" t="n">
-        <v>472.62</v>
+        <v>4787.28</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2839,13 +2839,13 @@
         <v>46217</v>
       </c>
       <c r="B127" t="n">
-        <v>2651</v>
+        <v>2308</v>
       </c>
       <c r="C127" t="n">
-        <v>58</v>
+        <v>546</v>
       </c>
       <c r="D127" t="n">
-        <v>648.71</v>
+        <v>1292.23</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -2858,13 +2858,13 @@
         <v>46217</v>
       </c>
       <c r="B128" t="n">
-        <v>2114</v>
+        <v>2709</v>
       </c>
       <c r="C128" t="n">
-        <v>1954</v>
+        <v>2220</v>
       </c>
       <c r="D128" t="n">
-        <v>879.03</v>
+        <v>1663.5</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -2877,17 +2877,17 @@
         <v>46217</v>
       </c>
       <c r="B129" t="n">
-        <v>40</v>
+        <v>1937</v>
       </c>
       <c r="C129" t="n">
         <v>8888</v>
       </c>
       <c r="D129" t="n">
-        <v>3583.39</v>
+        <v>1492.4</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2896,17 +2896,17 @@
         <v>46217</v>
       </c>
       <c r="B130" t="n">
-        <v>40</v>
+        <v>429</v>
       </c>
       <c r="C130" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D130" t="n">
-        <v>2529.31</v>
+        <v>2195.97</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2915,17 +2915,17 @@
         <v>46217</v>
       </c>
       <c r="B131" t="n">
-        <v>626</v>
+        <v>2211</v>
       </c>
       <c r="C131" t="n">
         <v>8888</v>
       </c>
       <c r="D131" t="n">
-        <v>13218.02</v>
+        <v>1563.28</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2934,17 +2934,17 @@
         <v>46217</v>
       </c>
       <c r="B132" t="n">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C132" t="n">
         <v>8888</v>
       </c>
       <c r="D132" t="n">
-        <v>739.17</v>
+        <v>15052.63</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2953,17 +2953,17 @@
         <v>46217</v>
       </c>
       <c r="B133" t="n">
-        <v>675</v>
+        <v>2251</v>
       </c>
       <c r="C133" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D133" t="n">
-        <v>107.13</v>
+        <v>797.58</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2972,13 +2972,13 @@
         <v>46217</v>
       </c>
       <c r="B134" t="n">
-        <v>636</v>
+        <v>451</v>
       </c>
       <c r="C134" t="n">
         <v>8888</v>
       </c>
       <c r="D134" t="n">
-        <v>5631.89</v>
+        <v>1371.26</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -2991,17 +2991,17 @@
         <v>46217</v>
       </c>
       <c r="B135" t="n">
-        <v>1075</v>
+        <v>40</v>
       </c>
       <c r="C135" t="n">
         <v>8888</v>
       </c>
       <c r="D135" t="n">
-        <v>1331.89</v>
+        <v>1093.47</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3010,13 +3010,13 @@
         <v>46217</v>
       </c>
       <c r="B136" t="n">
-        <v>2245</v>
+        <v>530</v>
       </c>
       <c r="C136" t="n">
         <v>8888</v>
       </c>
       <c r="D136" t="n">
-        <v>883.75</v>
+        <v>180.08</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3029,17 +3029,17 @@
         <v>46217</v>
       </c>
       <c r="B137" t="n">
-        <v>477</v>
+        <v>1137</v>
       </c>
       <c r="C137" t="n">
         <v>8888</v>
       </c>
       <c r="D137" t="n">
-        <v>994.15</v>
+        <v>3528.55</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3048,17 +3048,17 @@
         <v>46217</v>
       </c>
       <c r="B138" t="n">
-        <v>2015</v>
+        <v>1293</v>
       </c>
       <c r="C138" t="n">
-        <v>8888</v>
+        <v>601</v>
       </c>
       <c r="D138" t="n">
-        <v>2931.07</v>
+        <v>456.47</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3067,17 +3067,17 @@
         <v>46217</v>
       </c>
       <c r="B139" t="n">
-        <v>1653</v>
+        <v>2118</v>
       </c>
       <c r="C139" t="n">
         <v>8888</v>
       </c>
       <c r="D139" t="n">
-        <v>4115.53</v>
+        <v>311.54</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3086,17 +3086,17 @@
         <v>46217</v>
       </c>
       <c r="B140" t="n">
-        <v>1064</v>
+        <v>424</v>
       </c>
       <c r="C140" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D140" t="n">
-        <v>1052.68</v>
+        <v>349.68</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3105,17 +3105,17 @@
         <v>46217</v>
       </c>
       <c r="B141" t="n">
-        <v>1983</v>
+        <v>1299</v>
       </c>
       <c r="C141" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D141" t="n">
-        <v>1246.33</v>
+        <v>3625.32</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3124,17 +3124,17 @@
         <v>46217</v>
       </c>
       <c r="B142" t="n">
-        <v>2118</v>
+        <v>559</v>
       </c>
       <c r="C142" t="n">
         <v>8888</v>
       </c>
       <c r="D142" t="n">
-        <v>4886.49</v>
+        <v>1064.63</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3143,17 +3143,17 @@
         <v>46217</v>
       </c>
       <c r="B143" t="n">
-        <v>2680</v>
+        <v>89</v>
       </c>
       <c r="C143" t="n">
         <v>8888</v>
       </c>
       <c r="D143" t="n">
-        <v>2285.31</v>
+        <v>1506.42</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3162,17 +3162,17 @@
         <v>46217</v>
       </c>
       <c r="B144" t="n">
-        <v>2637</v>
+        <v>2250</v>
       </c>
       <c r="C144" t="n">
         <v>8888</v>
       </c>
       <c r="D144" t="n">
-        <v>1302.18</v>
+        <v>1943.54</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3181,13 +3181,13 @@
         <v>46217</v>
       </c>
       <c r="B145" t="n">
-        <v>1632</v>
+        <v>767</v>
       </c>
       <c r="C145" t="n">
         <v>8888</v>
       </c>
       <c r="D145" t="n">
-        <v>689.76</v>
+        <v>472.62</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3200,13 +3200,13 @@
         <v>46217</v>
       </c>
       <c r="B146" t="n">
-        <v>1299</v>
+        <v>2651</v>
       </c>
       <c r="C146" t="n">
-        <v>2522</v>
+        <v>58</v>
       </c>
       <c r="D146" t="n">
-        <v>3319.01</v>
+        <v>648.71</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3219,17 +3219,17 @@
         <v>46217</v>
       </c>
       <c r="B147" t="n">
-        <v>2026</v>
+        <v>2114</v>
       </c>
       <c r="C147" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D147" t="n">
-        <v>699.05</v>
+        <v>879.03</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3238,13 +3238,13 @@
         <v>46217</v>
       </c>
       <c r="B148" t="n">
-        <v>664</v>
+        <v>40</v>
       </c>
       <c r="C148" t="n">
         <v>8888</v>
       </c>
       <c r="D148" t="n">
-        <v>440.92</v>
+        <v>3583.39</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -3257,17 +3257,17 @@
         <v>46217</v>
       </c>
       <c r="B149" t="n">
-        <v>629</v>
+        <v>40</v>
       </c>
       <c r="C149" t="n">
-        <v>675</v>
+        <v>8888</v>
       </c>
       <c r="D149" t="n">
-        <v>267.79</v>
+        <v>2529.31</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3276,17 +3276,17 @@
         <v>46217</v>
       </c>
       <c r="B150" t="n">
-        <v>559</v>
+        <v>626</v>
       </c>
       <c r="C150" t="n">
         <v>8888</v>
       </c>
       <c r="D150" t="n">
-        <v>1562.5</v>
+        <v>18654.36</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3295,17 +3295,17 @@
         <v>46217</v>
       </c>
       <c r="B151" t="n">
-        <v>1465</v>
+        <v>363</v>
       </c>
       <c r="C151" t="n">
         <v>8888</v>
       </c>
       <c r="D151" t="n">
-        <v>10920.6</v>
+        <v>739.17</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3314,17 +3314,17 @@
         <v>46217</v>
       </c>
       <c r="B152" t="n">
-        <v>2550</v>
+        <v>675</v>
       </c>
       <c r="C152" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D152" t="n">
-        <v>321.05</v>
+        <v>107.13</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3333,17 +3333,17 @@
         <v>46217</v>
       </c>
       <c r="B153" t="n">
-        <v>1756</v>
+        <v>636</v>
       </c>
       <c r="C153" t="n">
         <v>8888</v>
       </c>
       <c r="D153" t="n">
-        <v>2445</v>
+        <v>7476.56</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3352,17 +3352,17 @@
         <v>46217</v>
       </c>
       <c r="B154" t="n">
-        <v>363</v>
+        <v>1075</v>
       </c>
       <c r="C154" t="n">
         <v>8888</v>
       </c>
       <c r="D154" t="n">
-        <v>2517.01</v>
+        <v>1331.89</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3371,17 +3371,17 @@
         <v>46217</v>
       </c>
       <c r="B155" t="n">
-        <v>2698</v>
+        <v>2245</v>
       </c>
       <c r="C155" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D155" t="n">
-        <v>1183.42</v>
+        <v>883.75</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3390,17 +3390,17 @@
         <v>46217</v>
       </c>
       <c r="B156" t="n">
-        <v>535</v>
+        <v>477</v>
       </c>
       <c r="C156" t="n">
         <v>8888</v>
       </c>
       <c r="D156" t="n">
-        <v>5293.96</v>
+        <v>994.15</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3409,13 +3409,13 @@
         <v>46217</v>
       </c>
       <c r="B157" t="n">
-        <v>2250</v>
+        <v>2015</v>
       </c>
       <c r="C157" t="n">
         <v>8888</v>
       </c>
       <c r="D157" t="n">
-        <v>2650.33</v>
+        <v>3243.05</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -3428,17 +3428,17 @@
         <v>46217</v>
       </c>
       <c r="B158" t="n">
-        <v>2681</v>
+        <v>1996</v>
       </c>
       <c r="C158" t="n">
-        <v>8888</v>
+        <v>691</v>
       </c>
       <c r="D158" t="n">
-        <v>2775.8</v>
+        <v>500.79</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3447,17 +3447,17 @@
         <v>46217</v>
       </c>
       <c r="B159" t="n">
-        <v>363</v>
+        <v>1653</v>
       </c>
       <c r="C159" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D159" t="n">
-        <v>3635.16</v>
+        <v>4115.53</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3466,17 +3466,17 @@
         <v>46217</v>
       </c>
       <c r="B160" t="n">
-        <v>483</v>
+        <v>1064</v>
       </c>
       <c r="C160" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D160" t="n">
-        <v>2527.71</v>
+        <v>1052.68</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3485,17 +3485,17 @@
         <v>46217</v>
       </c>
       <c r="B161" t="n">
-        <v>2607</v>
+        <v>1983</v>
       </c>
       <c r="C161" t="n">
         <v>8888</v>
       </c>
       <c r="D161" t="n">
-        <v>1075.36</v>
+        <v>1246.33</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3504,17 +3504,17 @@
         <v>46217</v>
       </c>
       <c r="B162" t="n">
-        <v>2330</v>
+        <v>2118</v>
       </c>
       <c r="C162" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D162" t="n">
-        <v>1923.09</v>
+        <v>4886.49</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3523,13 +3523,13 @@
         <v>46217</v>
       </c>
       <c r="B163" t="n">
-        <v>2709</v>
+        <v>2680</v>
       </c>
       <c r="C163" t="n">
         <v>8888</v>
       </c>
       <c r="D163" t="n">
-        <v>1667.47</v>
+        <v>2285.31</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -3542,17 +3542,17 @@
         <v>46217</v>
       </c>
       <c r="B164" t="n">
-        <v>374</v>
+        <v>2637</v>
       </c>
       <c r="C164" t="n">
         <v>8888</v>
       </c>
       <c r="D164" t="n">
-        <v>1150.97</v>
+        <v>1302.18</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3561,13 +3561,13 @@
         <v>46217</v>
       </c>
       <c r="B165" t="n">
-        <v>1137</v>
+        <v>1632</v>
       </c>
       <c r="C165" t="n">
         <v>8888</v>
       </c>
       <c r="D165" t="n">
-        <v>4413.34</v>
+        <v>689.76</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -3580,15 +3580,509 @@
         <v>46217</v>
       </c>
       <c r="B166" t="n">
+        <v>1299</v>
+      </c>
+      <c r="C166" t="n">
+        <v>2522</v>
+      </c>
+      <c r="D166" t="n">
+        <v>3319.01</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B167" t="n">
+        <v>2727</v>
+      </c>
+      <c r="C167" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D167" t="n">
+        <v>548.33</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B168" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C168" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D168" t="n">
+        <v>699.05</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B169" t="n">
+        <v>664</v>
+      </c>
+      <c r="C169" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D169" t="n">
+        <v>440.92</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B170" t="n">
+        <v>629</v>
+      </c>
+      <c r="C170" t="n">
+        <v>675</v>
+      </c>
+      <c r="D170" t="n">
+        <v>267.79</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B171" t="n">
+        <v>559</v>
+      </c>
+      <c r="C171" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D171" t="n">
+        <v>1562.5</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B172" t="n">
+        <v>1465</v>
+      </c>
+      <c r="C172" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D172" t="n">
+        <v>10920.6</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B173" t="n">
+        <v>2550</v>
+      </c>
+      <c r="C173" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D173" t="n">
+        <v>321.05</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B174" t="n">
+        <v>1756</v>
+      </c>
+      <c r="C174" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D174" t="n">
+        <v>2445</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B175" t="n">
+        <v>890</v>
+      </c>
+      <c r="C175" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D175" t="n">
+        <v>4287.14</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B176" t="n">
+        <v>363</v>
+      </c>
+      <c r="C176" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D176" t="n">
+        <v>2517.01</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B177" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C177" t="n">
+        <v>874</v>
+      </c>
+      <c r="D177" t="n">
+        <v>1183.42</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B178" t="n">
+        <v>535</v>
+      </c>
+      <c r="C178" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D178" t="n">
+        <v>5293.96</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B179" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C179" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D179" t="n">
+        <v>2650.33</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B180" t="n">
+        <v>2681</v>
+      </c>
+      <c r="C180" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D180" t="n">
+        <v>2853.99</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B181" t="n">
+        <v>132</v>
+      </c>
+      <c r="C181" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D181" t="n">
+        <v>2623.22</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B182" t="n">
+        <v>2442</v>
+      </c>
+      <c r="C182" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D182" t="n">
+        <v>2822.22</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B183" t="n">
+        <v>363</v>
+      </c>
+      <c r="C183" t="n">
+        <v>1898</v>
+      </c>
+      <c r="D183" t="n">
+        <v>3635.16</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B184" t="n">
+        <v>483</v>
+      </c>
+      <c r="C184" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D184" t="n">
+        <v>2527.71</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B185" t="n">
+        <v>2607</v>
+      </c>
+      <c r="C185" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D185" t="n">
+        <v>1075.36</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B186" t="n">
+        <v>2330</v>
+      </c>
+      <c r="C186" t="n">
+        <v>1954</v>
+      </c>
+      <c r="D186" t="n">
+        <v>1923.09</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B187" t="n">
+        <v>2472</v>
+      </c>
+      <c r="C187" t="n">
+        <v>2853</v>
+      </c>
+      <c r="D187" t="n">
+        <v>824.0599999999999</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B188" t="n">
+        <v>1384</v>
+      </c>
+      <c r="C188" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D188" t="n">
+        <v>585.27</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B189" t="n">
+        <v>2709</v>
+      </c>
+      <c r="C189" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D189" t="n">
+        <v>1667.47</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B190" t="n">
+        <v>374</v>
+      </c>
+      <c r="C190" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D190" t="n">
+        <v>1150.97</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B191" t="n">
+        <v>1137</v>
+      </c>
+      <c r="C191" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D191" t="n">
+        <v>4413.34</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B192" t="n">
         <v>2251</v>
       </c>
-      <c r="C166" t="n">
+      <c r="C192" t="n">
         <v>3403</v>
       </c>
-      <c r="D166" t="n">
+      <c r="D192" t="n">
         <v>510.18</v>
       </c>
-      <c r="E166" t="inlineStr">
+      <c r="E192" t="inlineStr">
         <is>
           <t>TELEMARKETING</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 16:00:03
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E192"/>
+  <dimension ref="A1:E245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,7 +489,7 @@
         <v>27</v>
       </c>
       <c r="D3" t="n">
-        <v>556.23</v>
+        <v>2389.55</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -546,7 +546,7 @@
         <v>8888</v>
       </c>
       <c r="D6" t="n">
-        <v>6359.39</v>
+        <v>13194.04</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -597,17 +597,17 @@
         <v>46217</v>
       </c>
       <c r="B9" t="n">
-        <v>2109</v>
+        <v>1064</v>
       </c>
       <c r="C9" t="n">
         <v>8888</v>
       </c>
       <c r="D9" t="n">
-        <v>4813.6</v>
+        <v>823.42</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -616,17 +616,17 @@
         <v>46217</v>
       </c>
       <c r="B10" t="n">
-        <v>2015</v>
+        <v>1381</v>
       </c>
       <c r="C10" t="n">
-        <v>2571</v>
+        <v>8888</v>
       </c>
       <c r="D10" t="n">
-        <v>2593.26</v>
+        <v>2196.92</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -635,17 +635,17 @@
         <v>46217</v>
       </c>
       <c r="B11" t="n">
-        <v>1993</v>
+        <v>703</v>
       </c>
       <c r="C11" t="n">
         <v>8888</v>
       </c>
       <c r="D11" t="n">
-        <v>1785.44</v>
+        <v>11161.25</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -654,13 +654,13 @@
         <v>46217</v>
       </c>
       <c r="B12" t="n">
-        <v>1102</v>
+        <v>2109</v>
       </c>
       <c r="C12" t="n">
         <v>8888</v>
       </c>
       <c r="D12" t="n">
-        <v>3129.4</v>
+        <v>4813.6</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -673,13 +673,13 @@
         <v>46217</v>
       </c>
       <c r="B13" t="n">
-        <v>1293</v>
+        <v>2015</v>
       </c>
       <c r="C13" t="n">
-        <v>1281</v>
+        <v>2571</v>
       </c>
       <c r="D13" t="n">
-        <v>1337.87</v>
+        <v>2593.26</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -692,17 +692,17 @@
         <v>46217</v>
       </c>
       <c r="B14" t="n">
-        <v>2657</v>
+        <v>1993</v>
       </c>
       <c r="C14" t="n">
         <v>8888</v>
       </c>
       <c r="D14" t="n">
-        <v>877.0700000000001</v>
+        <v>1785.44</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -711,13 +711,13 @@
         <v>46217</v>
       </c>
       <c r="B15" t="n">
-        <v>2768</v>
+        <v>1102</v>
       </c>
       <c r="C15" t="n">
         <v>8888</v>
       </c>
       <c r="D15" t="n">
-        <v>4890.12</v>
+        <v>3406.59</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -730,17 +730,17 @@
         <v>46217</v>
       </c>
       <c r="B16" t="n">
-        <v>2686</v>
+        <v>1937</v>
       </c>
       <c r="C16" t="n">
         <v>8888</v>
       </c>
       <c r="D16" t="n">
-        <v>422.71</v>
+        <v>3337.21</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -749,13 +749,13 @@
         <v>46217</v>
       </c>
       <c r="B17" t="n">
-        <v>1890</v>
+        <v>1293</v>
       </c>
       <c r="C17" t="n">
-        <v>3449</v>
+        <v>1281</v>
       </c>
       <c r="D17" t="n">
-        <v>809.78</v>
+        <v>1337.87</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -768,17 +768,17 @@
         <v>46217</v>
       </c>
       <c r="B18" t="n">
-        <v>2726</v>
+        <v>2657</v>
       </c>
       <c r="C18" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D18" t="n">
-        <v>640.1799999999999</v>
+        <v>877.0700000000001</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -787,13 +787,13 @@
         <v>46217</v>
       </c>
       <c r="B19" t="n">
-        <v>89</v>
+        <v>2768</v>
       </c>
       <c r="C19" t="n">
         <v>8888</v>
       </c>
       <c r="D19" t="n">
-        <v>5652.15</v>
+        <v>4890.12</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -806,17 +806,17 @@
         <v>46217</v>
       </c>
       <c r="B20" t="n">
-        <v>2641</v>
+        <v>2686</v>
       </c>
       <c r="C20" t="n">
         <v>8888</v>
       </c>
       <c r="D20" t="n">
-        <v>607.79</v>
+        <v>422.71</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -825,13 +825,13 @@
         <v>46217</v>
       </c>
       <c r="B21" t="n">
-        <v>949</v>
+        <v>1890</v>
       </c>
       <c r="C21" t="n">
-        <v>1258</v>
+        <v>3449</v>
       </c>
       <c r="D21" t="n">
-        <v>196.87</v>
+        <v>1575.78</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -844,17 +844,17 @@
         <v>46217</v>
       </c>
       <c r="B22" t="n">
-        <v>353</v>
+        <v>33</v>
       </c>
       <c r="C22" t="n">
         <v>8888</v>
       </c>
       <c r="D22" t="n">
-        <v>2121.12</v>
+        <v>1041.47</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -863,17 +863,17 @@
         <v>46217</v>
       </c>
       <c r="B23" t="n">
-        <v>1756</v>
+        <v>2726</v>
       </c>
       <c r="C23" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D23" t="n">
-        <v>1799.7</v>
+        <v>640.1799999999999</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -882,17 +882,17 @@
         <v>46217</v>
       </c>
       <c r="B24" t="n">
-        <v>285</v>
+        <v>89</v>
       </c>
       <c r="C24" t="n">
         <v>8888</v>
       </c>
       <c r="D24" t="n">
-        <v>3092.58</v>
+        <v>5652.15</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -901,17 +901,17 @@
         <v>46217</v>
       </c>
       <c r="B25" t="n">
-        <v>1906</v>
+        <v>2178</v>
       </c>
       <c r="C25" t="n">
-        <v>8888</v>
+        <v>738</v>
       </c>
       <c r="D25" t="n">
-        <v>3142.54</v>
+        <v>291.83</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
         <v>46217</v>
       </c>
       <c r="B26" t="n">
-        <v>1308</v>
+        <v>2209</v>
       </c>
       <c r="C26" t="n">
-        <v>8888</v>
+        <v>738</v>
       </c>
       <c r="D26" t="n">
-        <v>3127.35</v>
+        <v>2043.28</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -939,17 +939,17 @@
         <v>46217</v>
       </c>
       <c r="B27" t="n">
-        <v>610</v>
+        <v>429</v>
       </c>
       <c r="C27" t="n">
         <v>8888</v>
       </c>
       <c r="D27" t="n">
-        <v>590.08</v>
+        <v>3775.81</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -958,13 +958,13 @@
         <v>46217</v>
       </c>
       <c r="B28" t="n">
-        <v>619</v>
+        <v>2641</v>
       </c>
       <c r="C28" t="n">
         <v>8888</v>
       </c>
       <c r="D28" t="n">
-        <v>236.34</v>
+        <v>607.79</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -977,13 +977,13 @@
         <v>46217</v>
       </c>
       <c r="B29" t="n">
-        <v>2755</v>
+        <v>949</v>
       </c>
       <c r="C29" t="n">
-        <v>2220</v>
+        <v>1258</v>
       </c>
       <c r="D29" t="n">
-        <v>1133.17</v>
+        <v>196.87</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -996,17 +996,17 @@
         <v>46217</v>
       </c>
       <c r="B30" t="n">
-        <v>2767</v>
+        <v>353</v>
       </c>
       <c r="C30" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D30" t="n">
-        <v>5000.2</v>
+        <v>2121.12</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1015,17 +1015,17 @@
         <v>46217</v>
       </c>
       <c r="B31" t="n">
-        <v>559</v>
+        <v>1756</v>
       </c>
       <c r="C31" t="n">
         <v>8888</v>
       </c>
       <c r="D31" t="n">
-        <v>1200.99</v>
+        <v>1799.7</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1034,17 +1034,17 @@
         <v>46217</v>
       </c>
       <c r="B32" t="n">
-        <v>358</v>
+        <v>285</v>
       </c>
       <c r="C32" t="n">
         <v>8888</v>
       </c>
       <c r="D32" t="n">
-        <v>1301.77</v>
+        <v>3937.9</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1053,13 +1053,13 @@
         <v>46217</v>
       </c>
       <c r="B33" t="n">
-        <v>609</v>
+        <v>1906</v>
       </c>
       <c r="C33" t="n">
         <v>8888</v>
       </c>
       <c r="D33" t="n">
-        <v>962.08</v>
+        <v>3142.54</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1072,17 +1072,17 @@
         <v>46217</v>
       </c>
       <c r="B34" t="n">
-        <v>2507</v>
+        <v>1308</v>
       </c>
       <c r="C34" t="n">
         <v>8888</v>
       </c>
       <c r="D34" t="n">
-        <v>448.36</v>
+        <v>3127.35</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1091,13 +1091,13 @@
         <v>46217</v>
       </c>
       <c r="B35" t="n">
-        <v>2767</v>
+        <v>610</v>
       </c>
       <c r="C35" t="n">
         <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>1175.73</v>
+        <v>590.08</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1110,17 +1110,17 @@
         <v>46217</v>
       </c>
       <c r="B36" t="n">
-        <v>1063</v>
+        <v>619</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>1251.14</v>
+        <v>236.34</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1129,17 @@
         <v>46217</v>
       </c>
       <c r="B37" t="n">
-        <v>325</v>
+        <v>1324</v>
       </c>
       <c r="C37" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D37" t="n">
-        <v>868.83</v>
+        <v>2603.19</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1148,17 +1148,17 @@
         <v>46217</v>
       </c>
       <c r="B38" t="n">
-        <v>2660</v>
+        <v>483</v>
       </c>
       <c r="C38" t="n">
         <v>8888</v>
       </c>
       <c r="D38" t="n">
-        <v>281.24</v>
+        <v>461.28</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1167,17 +1167,17 @@
         <v>46217</v>
       </c>
       <c r="B39" t="n">
-        <v>610</v>
+        <v>1117</v>
       </c>
       <c r="C39" t="n">
         <v>8888</v>
       </c>
       <c r="D39" t="n">
-        <v>235.34</v>
+        <v>755.71</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1186,17 +1186,17 @@
         <v>46217</v>
       </c>
       <c r="B40" t="n">
-        <v>424</v>
+        <v>2755</v>
       </c>
       <c r="C40" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D40" t="n">
-        <v>3214.29</v>
+        <v>1133.17</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
         <v>46217</v>
       </c>
       <c r="B41" t="n">
-        <v>40</v>
+        <v>2767</v>
       </c>
       <c r="C41" t="n">
-        <v>58</v>
+        <v>1898</v>
       </c>
       <c r="D41" t="n">
-        <v>325.04</v>
+        <v>5000.2</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1224,13 +1224,13 @@
         <v>46217</v>
       </c>
       <c r="B42" t="n">
-        <v>1117</v>
+        <v>559</v>
       </c>
       <c r="C42" t="n">
         <v>8888</v>
       </c>
       <c r="D42" t="n">
-        <v>349.47</v>
+        <v>1516.25</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1243,17 +1243,17 @@
         <v>46217</v>
       </c>
       <c r="B43" t="n">
-        <v>949</v>
+        <v>1277</v>
       </c>
       <c r="C43" t="n">
-        <v>998</v>
+        <v>8888</v>
       </c>
       <c r="D43" t="n">
-        <v>129.85</v>
+        <v>574.7</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1262,13 +1262,13 @@
         <v>46217</v>
       </c>
       <c r="B44" t="n">
-        <v>1853</v>
+        <v>358</v>
       </c>
       <c r="C44" t="n">
         <v>8888</v>
       </c>
       <c r="D44" t="n">
-        <v>522.4</v>
+        <v>1301.77</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1281,17 +1281,17 @@
         <v>46217</v>
       </c>
       <c r="B45" t="n">
-        <v>2250</v>
+        <v>1993</v>
       </c>
       <c r="C45" t="n">
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>4131.57</v>
+        <v>5280</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1300,13 +1300,13 @@
         <v>46217</v>
       </c>
       <c r="B46" t="n">
-        <v>2507</v>
+        <v>609</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>4167.12</v>
+        <v>962.08</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1319,17 +1319,17 @@
         <v>46217</v>
       </c>
       <c r="B47" t="n">
-        <v>664</v>
+        <v>2507</v>
       </c>
       <c r="C47" t="n">
         <v>8888</v>
       </c>
       <c r="D47" t="n">
-        <v>3815.91</v>
+        <v>448.36</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1338,17 +1338,17 @@
         <v>46217</v>
       </c>
       <c r="B48" t="n">
-        <v>1075</v>
+        <v>2767</v>
       </c>
       <c r="C48" t="n">
         <v>8888</v>
       </c>
       <c r="D48" t="n">
-        <v>1013.2</v>
+        <v>1175.73</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1357,17 +1357,17 @@
         <v>46217</v>
       </c>
       <c r="B49" t="n">
-        <v>1906</v>
+        <v>1063</v>
       </c>
       <c r="C49" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D49" t="n">
-        <v>1445.21</v>
+        <v>1251.14</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1376,13 +1376,13 @@
         <v>46217</v>
       </c>
       <c r="B50" t="n">
-        <v>595</v>
+        <v>325</v>
       </c>
       <c r="C50" t="n">
-        <v>691</v>
+        <v>58</v>
       </c>
       <c r="D50" t="n">
-        <v>314.52</v>
+        <v>868.83</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1395,17 +1395,17 @@
         <v>46217</v>
       </c>
       <c r="B51" t="n">
-        <v>2696</v>
+        <v>2660</v>
       </c>
       <c r="C51" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D51" t="n">
-        <v>677.76</v>
+        <v>281.24</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
         <v>46217</v>
       </c>
       <c r="B52" t="n">
-        <v>525</v>
+        <v>610</v>
       </c>
       <c r="C52" t="n">
         <v>8888</v>
       </c>
       <c r="D52" t="n">
-        <v>490.08</v>
+        <v>235.34</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1433,17 +1433,17 @@
         <v>46217</v>
       </c>
       <c r="B53" t="n">
-        <v>2491</v>
+        <v>424</v>
       </c>
       <c r="C53" t="n">
         <v>8888</v>
       </c>
       <c r="D53" t="n">
-        <v>2909.58</v>
+        <v>3214.29</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1452,17 +1452,17 @@
         <v>46217</v>
       </c>
       <c r="B54" t="n">
-        <v>360</v>
+        <v>664</v>
       </c>
       <c r="C54" t="n">
-        <v>546</v>
+        <v>8888</v>
       </c>
       <c r="D54" t="n">
-        <v>6094.25</v>
+        <v>364.07</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1471,17 +1471,17 @@
         <v>46217</v>
       </c>
       <c r="B55" t="n">
-        <v>2651</v>
+        <v>2279</v>
       </c>
       <c r="C55" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D55" t="n">
-        <v>638.64</v>
+        <v>448.78</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1490,17 +1490,17 @@
         <v>46217</v>
       </c>
       <c r="B56" t="n">
-        <v>2695</v>
+        <v>40</v>
       </c>
       <c r="C56" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D56" t="n">
-        <v>532.53</v>
+        <v>325.04</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1509,17 +1509,17 @@
         <v>46217</v>
       </c>
       <c r="B57" t="n">
-        <v>1293</v>
+        <v>2069</v>
       </c>
       <c r="C57" t="n">
         <v>8888</v>
       </c>
       <c r="D57" t="n">
-        <v>381.82</v>
+        <v>176.8</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1528,17 +1528,17 @@
         <v>46217</v>
       </c>
       <c r="B58" t="n">
-        <v>2663</v>
+        <v>522</v>
       </c>
       <c r="C58" t="n">
         <v>8888</v>
       </c>
       <c r="D58" t="n">
-        <v>2146.08</v>
+        <v>151.86</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1547,17 +1547,17 @@
         <v>46217</v>
       </c>
       <c r="B59" t="n">
-        <v>525</v>
+        <v>1304</v>
       </c>
       <c r="C59" t="n">
-        <v>8888</v>
+        <v>213</v>
       </c>
       <c r="D59" t="n">
-        <v>1240.79</v>
+        <v>297.1</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1566,13 +1566,13 @@
         <v>46217</v>
       </c>
       <c r="B60" t="n">
-        <v>2711</v>
+        <v>1869</v>
       </c>
       <c r="C60" t="n">
         <v>8888</v>
       </c>
       <c r="D60" t="n">
-        <v>2193.56</v>
+        <v>447.76</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1585,17 +1585,17 @@
         <v>46217</v>
       </c>
       <c r="B61" t="n">
-        <v>1317</v>
+        <v>949</v>
       </c>
       <c r="C61" t="n">
-        <v>8888</v>
+        <v>998</v>
       </c>
       <c r="D61" t="n">
-        <v>787.51</v>
+        <v>129.85</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1604,17 +1604,17 @@
         <v>46217</v>
       </c>
       <c r="B62" t="n">
-        <v>675</v>
+        <v>1853</v>
       </c>
       <c r="C62" t="n">
         <v>8888</v>
       </c>
       <c r="D62" t="n">
-        <v>289.67</v>
+        <v>522.4</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1623,17 +1623,17 @@
         <v>46217</v>
       </c>
       <c r="B63" t="n">
-        <v>1063</v>
+        <v>2250</v>
       </c>
       <c r="C63" t="n">
         <v>8888</v>
       </c>
       <c r="D63" t="n">
-        <v>1902.46</v>
+        <v>4131.57</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1642,13 +1642,13 @@
         <v>46217</v>
       </c>
       <c r="B64" t="n">
-        <v>1658</v>
+        <v>2507</v>
       </c>
       <c r="C64" t="n">
         <v>8888</v>
       </c>
       <c r="D64" t="n">
-        <v>1357.94</v>
+        <v>4167.12</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1661,17 +1661,17 @@
         <v>46217</v>
       </c>
       <c r="B65" t="n">
-        <v>1392</v>
+        <v>664</v>
       </c>
       <c r="C65" t="n">
         <v>8888</v>
       </c>
       <c r="D65" t="n">
-        <v>814.61</v>
+        <v>4099.16</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1680,17 +1680,17 @@
         <v>46217</v>
       </c>
       <c r="B66" t="n">
-        <v>360</v>
+        <v>1075</v>
       </c>
       <c r="C66" t="n">
         <v>8888</v>
       </c>
       <c r="D66" t="n">
-        <v>749.13</v>
+        <v>1743.47</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1699,13 +1699,13 @@
         <v>46217</v>
       </c>
       <c r="B67" t="n">
-        <v>949</v>
+        <v>1324</v>
       </c>
       <c r="C67" t="n">
-        <v>1134</v>
+        <v>738</v>
       </c>
       <c r="D67" t="n">
-        <v>327.6</v>
+        <v>4548.42</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1718,17 +1718,17 @@
         <v>46217</v>
       </c>
       <c r="B68" t="n">
-        <v>2133</v>
+        <v>1906</v>
       </c>
       <c r="C68" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D68" t="n">
-        <v>66030.34</v>
+        <v>1445.21</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1737,17 +1737,17 @@
         <v>46217</v>
       </c>
       <c r="B69" t="n">
-        <v>326</v>
+        <v>595</v>
       </c>
       <c r="C69" t="n">
-        <v>8888</v>
+        <v>691</v>
       </c>
       <c r="D69" t="n">
-        <v>360.45</v>
+        <v>314.52</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1756,17 +1756,17 @@
         <v>46217</v>
       </c>
       <c r="B70" t="n">
-        <v>325</v>
+        <v>2696</v>
       </c>
       <c r="C70" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D70" t="n">
-        <v>774.73</v>
+        <v>677.76</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1775,17 @@
         <v>46217</v>
       </c>
       <c r="B71" t="n">
-        <v>1293</v>
+        <v>525</v>
       </c>
       <c r="C71" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D71" t="n">
-        <v>8365.559999999999</v>
+        <v>490.08</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1794,17 +1794,17 @@
         <v>46217</v>
       </c>
       <c r="B72" t="n">
-        <v>131</v>
+        <v>2491</v>
       </c>
       <c r="C72" t="n">
         <v>8888</v>
       </c>
       <c r="D72" t="n">
-        <v>1969.93</v>
+        <v>2909.58</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1813,17 +1813,17 @@
         <v>46217</v>
       </c>
       <c r="B73" t="n">
-        <v>2697</v>
+        <v>360</v>
       </c>
       <c r="C73" t="n">
-        <v>8888</v>
+        <v>546</v>
       </c>
       <c r="D73" t="n">
-        <v>420.48</v>
+        <v>7463.12</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1832,17 +1832,17 @@
         <v>46217</v>
       </c>
       <c r="B74" t="n">
-        <v>2279</v>
+        <v>2651</v>
       </c>
       <c r="C74" t="n">
         <v>8888</v>
       </c>
       <c r="D74" t="n">
-        <v>1034.25</v>
+        <v>638.64</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1851,17 +1851,17 @@
         <v>46217</v>
       </c>
       <c r="B75" t="n">
-        <v>1116</v>
+        <v>525</v>
       </c>
       <c r="C75" t="n">
         <v>8888</v>
       </c>
       <c r="D75" t="n">
-        <v>1293.89</v>
+        <v>4351.19</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1870,13 +1870,13 @@
         <v>46217</v>
       </c>
       <c r="B76" t="n">
-        <v>131</v>
+        <v>2124</v>
       </c>
       <c r="C76" t="n">
         <v>8888</v>
       </c>
       <c r="D76" t="n">
-        <v>5470.1</v>
+        <v>3875.99</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -1889,17 +1889,17 @@
         <v>46217</v>
       </c>
       <c r="B77" t="n">
-        <v>1937</v>
+        <v>2695</v>
       </c>
       <c r="C77" t="n">
         <v>8888</v>
       </c>
       <c r="D77" t="n">
-        <v>692.86</v>
+        <v>1244.27</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1908,13 +1908,13 @@
         <v>46217</v>
       </c>
       <c r="B78" t="n">
-        <v>1983</v>
+        <v>1293</v>
       </c>
       <c r="C78" t="n">
         <v>8888</v>
       </c>
       <c r="D78" t="n">
-        <v>412.16</v>
+        <v>381.82</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -1927,17 +1927,17 @@
         <v>46217</v>
       </c>
       <c r="B79" t="n">
-        <v>451</v>
+        <v>2363</v>
       </c>
       <c r="C79" t="n">
         <v>8888</v>
       </c>
       <c r="D79" t="n">
-        <v>2583.46</v>
+        <v>2985.2</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1946,13 +1946,13 @@
         <v>46217</v>
       </c>
       <c r="B80" t="n">
-        <v>2767</v>
+        <v>2663</v>
       </c>
       <c r="C80" t="n">
         <v>8888</v>
       </c>
       <c r="D80" t="n">
-        <v>920.85</v>
+        <v>2146.08</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -1965,13 +1965,13 @@
         <v>46217</v>
       </c>
       <c r="B81" t="n">
-        <v>2697</v>
+        <v>2711</v>
       </c>
       <c r="C81" t="n">
         <v>8888</v>
       </c>
       <c r="D81" t="n">
-        <v>2880.19</v>
+        <v>2193.56</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -1984,17 +1984,17 @@
         <v>46217</v>
       </c>
       <c r="B82" t="n">
-        <v>569</v>
+        <v>1317</v>
       </c>
       <c r="C82" t="n">
         <v>8888</v>
       </c>
       <c r="D82" t="n">
-        <v>2291.64</v>
+        <v>787.51</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2003,17 +2003,17 @@
         <v>46217</v>
       </c>
       <c r="B83" t="n">
-        <v>2211</v>
+        <v>675</v>
       </c>
       <c r="C83" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D83" t="n">
-        <v>1833.56</v>
+        <v>289.67</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2028,11 +2028,11 @@
         <v>8888</v>
       </c>
       <c r="D84" t="n">
-        <v>352.87</v>
+        <v>1902.46</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2041,13 +2041,13 @@
         <v>46217</v>
       </c>
       <c r="B85" t="n">
-        <v>2687</v>
+        <v>1658</v>
       </c>
       <c r="C85" t="n">
         <v>8888</v>
       </c>
       <c r="D85" t="n">
-        <v>1760.22</v>
+        <v>1357.94</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2060,17 +2060,17 @@
         <v>46217</v>
       </c>
       <c r="B86" t="n">
-        <v>629</v>
+        <v>1392</v>
       </c>
       <c r="C86" t="n">
         <v>8888</v>
       </c>
       <c r="D86" t="n">
-        <v>559.15</v>
+        <v>814.61</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2079,17 +2079,17 @@
         <v>46217</v>
       </c>
       <c r="B87" t="n">
-        <v>1890</v>
+        <v>360</v>
       </c>
       <c r="C87" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D87" t="n">
-        <v>1122</v>
+        <v>749.13</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2098,17 +2098,17 @@
         <v>46217</v>
       </c>
       <c r="B88" t="n">
-        <v>1289</v>
+        <v>1324</v>
       </c>
       <c r="C88" t="n">
         <v>8888</v>
       </c>
       <c r="D88" t="n">
-        <v>1214.09</v>
+        <v>327.19</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2117,17 +2117,17 @@
         <v>46217</v>
       </c>
       <c r="B89" t="n">
-        <v>2107</v>
+        <v>525</v>
       </c>
       <c r="C89" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D89" t="n">
-        <v>2000.86</v>
+        <v>643.3</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2136,17 +2136,17 @@
         <v>46217</v>
       </c>
       <c r="B90" t="n">
-        <v>1116</v>
+        <v>949</v>
       </c>
       <c r="C90" t="n">
-        <v>8888</v>
+        <v>1134</v>
       </c>
       <c r="D90" t="n">
-        <v>1065.24</v>
+        <v>327.6</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2155,17 +2155,17 @@
         <v>46217</v>
       </c>
       <c r="B91" t="n">
-        <v>58</v>
+        <v>2133</v>
       </c>
       <c r="C91" t="n">
         <v>8888</v>
       </c>
       <c r="D91" t="n">
-        <v>2637.19</v>
+        <v>66030.34</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2174,17 +2174,17 @@
         <v>46217</v>
       </c>
       <c r="B92" t="n">
-        <v>1117</v>
+        <v>326</v>
       </c>
       <c r="C92" t="n">
         <v>8888</v>
       </c>
       <c r="D92" t="n">
-        <v>581.51</v>
+        <v>695.99</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2193,17 +2193,17 @@
         <v>46217</v>
       </c>
       <c r="B93" t="n">
-        <v>58</v>
+        <v>325</v>
       </c>
       <c r="C93" t="n">
         <v>8888</v>
       </c>
       <c r="D93" t="n">
-        <v>1411.43</v>
+        <v>774.73</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2212,17 +2212,17 @@
         <v>46217</v>
       </c>
       <c r="B94" t="n">
-        <v>629</v>
+        <v>1293</v>
       </c>
       <c r="C94" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D94" t="n">
-        <v>2049.78</v>
+        <v>8365.559999999999</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2231,17 +2231,17 @@
         <v>46217</v>
       </c>
       <c r="B95" t="n">
-        <v>595</v>
+        <v>131</v>
       </c>
       <c r="C95" t="n">
         <v>8888</v>
       </c>
       <c r="D95" t="n">
-        <v>3191</v>
+        <v>1969.93</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2250,17 +2250,17 @@
         <v>46217</v>
       </c>
       <c r="B96" t="n">
-        <v>949</v>
+        <v>2697</v>
       </c>
       <c r="C96" t="n">
-        <v>1762</v>
+        <v>8888</v>
       </c>
       <c r="D96" t="n">
-        <v>325.65</v>
+        <v>420.48</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2269,17 +2269,17 @@
         <v>46217</v>
       </c>
       <c r="B97" t="n">
-        <v>2463</v>
+        <v>2279</v>
       </c>
       <c r="C97" t="n">
         <v>8888</v>
       </c>
       <c r="D97" t="n">
-        <v>8336.43</v>
+        <v>1034.25</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2288,17 +2288,17 @@
         <v>46217</v>
       </c>
       <c r="B98" t="n">
-        <v>1064</v>
+        <v>1340</v>
       </c>
       <c r="C98" t="n">
         <v>8888</v>
       </c>
       <c r="D98" t="n">
-        <v>1513.21</v>
+        <v>3037.55</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2307,17 +2307,17 @@
         <v>46217</v>
       </c>
       <c r="B99" t="n">
-        <v>1478</v>
+        <v>2641</v>
       </c>
       <c r="C99" t="n">
         <v>8888</v>
       </c>
       <c r="D99" t="n">
-        <v>2261.67</v>
+        <v>557.52</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2326,13 +2326,13 @@
         <v>46217</v>
       </c>
       <c r="B100" t="n">
-        <v>358</v>
+        <v>1116</v>
       </c>
       <c r="C100" t="n">
         <v>8888</v>
       </c>
       <c r="D100" t="n">
-        <v>1918.33</v>
+        <v>1293.89</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2345,13 +2345,13 @@
         <v>46217</v>
       </c>
       <c r="B101" t="n">
-        <v>2107</v>
+        <v>2178</v>
       </c>
       <c r="C101" t="n">
         <v>8888</v>
       </c>
       <c r="D101" t="n">
-        <v>2745.11</v>
+        <v>5333.4</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2364,17 +2364,17 @@
         <v>46217</v>
       </c>
       <c r="B102" t="n">
-        <v>675</v>
+        <v>1756</v>
       </c>
       <c r="C102" t="n">
         <v>8888</v>
       </c>
       <c r="D102" t="n">
-        <v>678.88</v>
+        <v>742.23</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2383,17 +2383,17 @@
         <v>46217</v>
       </c>
       <c r="B103" t="n">
-        <v>2279</v>
+        <v>131</v>
       </c>
       <c r="C103" t="n">
         <v>8888</v>
       </c>
       <c r="D103" t="n">
-        <v>1165.17</v>
+        <v>5470.1</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2402,17 +2402,17 @@
         <v>46217</v>
       </c>
       <c r="B104" t="n">
-        <v>451</v>
+        <v>2081</v>
       </c>
       <c r="C104" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D104" t="n">
-        <v>327.28</v>
+        <v>1022.42</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2421,13 +2421,13 @@
         <v>46217</v>
       </c>
       <c r="B105" t="n">
-        <v>2571</v>
+        <v>1374</v>
       </c>
       <c r="C105" t="n">
-        <v>1312</v>
+        <v>2845</v>
       </c>
       <c r="D105" t="n">
-        <v>2202.75</v>
+        <v>625.77</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2440,17 +2440,17 @@
         <v>46217</v>
       </c>
       <c r="B106" t="n">
-        <v>2782</v>
+        <v>58</v>
       </c>
       <c r="C106" t="n">
         <v>8888</v>
       </c>
       <c r="D106" t="n">
-        <v>753.8</v>
+        <v>3050.12</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2459,17 +2459,17 @@
         <v>46217</v>
       </c>
       <c r="B107" t="n">
-        <v>610</v>
+        <v>1937</v>
       </c>
       <c r="C107" t="n">
         <v>8888</v>
       </c>
       <c r="D107" t="n">
-        <v>335.61</v>
+        <v>2199.57</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2478,17 +2478,17 @@
         <v>46217</v>
       </c>
       <c r="B108" t="n">
-        <v>2245</v>
+        <v>1983</v>
       </c>
       <c r="C108" t="n">
         <v>8888</v>
       </c>
       <c r="D108" t="n">
-        <v>355.88</v>
+        <v>412.16</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2497,17 +2497,17 @@
         <v>46217</v>
       </c>
       <c r="B109" t="n">
-        <v>1108</v>
+        <v>451</v>
       </c>
       <c r="C109" t="n">
         <v>8888</v>
       </c>
       <c r="D109" t="n">
-        <v>508.54</v>
+        <v>2583.46</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2516,13 +2516,13 @@
         <v>46217</v>
       </c>
       <c r="B110" t="n">
-        <v>341</v>
+        <v>1102</v>
       </c>
       <c r="C110" t="n">
-        <v>58</v>
+        <v>13148</v>
       </c>
       <c r="D110" t="n">
-        <v>366.88</v>
+        <v>1346.4</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -2535,17 +2535,17 @@
         <v>46217</v>
       </c>
       <c r="B111" t="n">
-        <v>525</v>
+        <v>2767</v>
       </c>
       <c r="C111" t="n">
-        <v>1087</v>
+        <v>8888</v>
       </c>
       <c r="D111" t="n">
-        <v>1830.26</v>
+        <v>920.85</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2554,17 +2554,17 @@
         <v>46217</v>
       </c>
       <c r="B112" t="n">
-        <v>1653</v>
+        <v>2697</v>
       </c>
       <c r="C112" t="n">
         <v>8888</v>
       </c>
       <c r="D112" t="n">
-        <v>4383.69</v>
+        <v>2880.19</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2573,17 +2573,17 @@
         <v>46217</v>
       </c>
       <c r="B113" t="n">
-        <v>619</v>
+        <v>569</v>
       </c>
       <c r="C113" t="n">
         <v>8888</v>
       </c>
       <c r="D113" t="n">
-        <v>1557.5</v>
+        <v>3002.06</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2592,13 +2592,13 @@
         <v>46217</v>
       </c>
       <c r="B114" t="n">
-        <v>1518</v>
+        <v>2211</v>
       </c>
       <c r="C114" t="n">
-        <v>1533</v>
+        <v>874</v>
       </c>
       <c r="D114" t="n">
-        <v>479.84</v>
+        <v>1833.56</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -2611,13 +2611,13 @@
         <v>46217</v>
       </c>
       <c r="B115" t="n">
-        <v>663</v>
+        <v>1063</v>
       </c>
       <c r="C115" t="n">
         <v>8888</v>
       </c>
       <c r="D115" t="n">
-        <v>824.5599999999999</v>
+        <v>352.87</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -2630,17 +2630,17 @@
         <v>46217</v>
       </c>
       <c r="B116" t="n">
-        <v>2089</v>
+        <v>2687</v>
       </c>
       <c r="C116" t="n">
-        <v>1533</v>
+        <v>8888</v>
       </c>
       <c r="D116" t="n">
-        <v>822.05</v>
+        <v>1760.22</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2649,17 +2649,17 @@
         <v>46217</v>
       </c>
       <c r="B117" t="n">
-        <v>2133</v>
+        <v>629</v>
       </c>
       <c r="C117" t="n">
-        <v>691</v>
+        <v>8888</v>
       </c>
       <c r="D117" t="n">
-        <v>1414.98</v>
+        <v>559.15</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2668,17 +2668,17 @@
         <v>46217</v>
       </c>
       <c r="B118" t="n">
-        <v>429</v>
+        <v>1117</v>
       </c>
       <c r="C118" t="n">
-        <v>2571</v>
+        <v>8888</v>
       </c>
       <c r="D118" t="n">
-        <v>667.12</v>
+        <v>1988.42</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2687,17 +2687,17 @@
         <v>46217</v>
       </c>
       <c r="B119" t="n">
-        <v>2641</v>
+        <v>1890</v>
       </c>
       <c r="C119" t="n">
-        <v>8888</v>
+        <v>1953</v>
       </c>
       <c r="D119" t="n">
-        <v>252.41</v>
+        <v>1122</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2706,13 +2706,13 @@
         <v>46217</v>
       </c>
       <c r="B120" t="n">
-        <v>1293</v>
+        <v>1289</v>
       </c>
       <c r="C120" t="n">
         <v>8888</v>
       </c>
       <c r="D120" t="n">
-        <v>8102.01</v>
+        <v>1214.09</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -2725,17 +2725,17 @@
         <v>46217</v>
       </c>
       <c r="B121" t="n">
-        <v>1465</v>
+        <v>2363</v>
       </c>
       <c r="C121" t="n">
         <v>8888</v>
       </c>
       <c r="D121" t="n">
-        <v>814.65</v>
+        <v>301.92</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2744,17 +2744,17 @@
         <v>46217</v>
       </c>
       <c r="B122" t="n">
-        <v>483</v>
+        <v>1075</v>
       </c>
       <c r="C122" t="n">
         <v>8888</v>
       </c>
       <c r="D122" t="n">
-        <v>1980.79</v>
+        <v>1845.09</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2763,17 +2763,17 @@
         <v>46217</v>
       </c>
       <c r="B123" t="n">
-        <v>1064</v>
+        <v>2107</v>
       </c>
       <c r="C123" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D123" t="n">
-        <v>104632.21</v>
+        <v>2000.86</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2782,17 +2782,17 @@
         <v>46217</v>
       </c>
       <c r="B124" t="n">
-        <v>131</v>
+        <v>1116</v>
       </c>
       <c r="C124" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D124" t="n">
-        <v>876.48</v>
+        <v>1065.24</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2801,17 +2801,17 @@
         <v>46217</v>
       </c>
       <c r="B125" t="n">
-        <v>663</v>
+        <v>2190</v>
       </c>
       <c r="C125" t="n">
         <v>8888</v>
       </c>
       <c r="D125" t="n">
-        <v>1769.59</v>
+        <v>2781.91</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2820,17 +2820,17 @@
         <v>46217</v>
       </c>
       <c r="B126" t="n">
-        <v>131</v>
+        <v>559</v>
       </c>
       <c r="C126" t="n">
-        <v>8888</v>
+        <v>3009</v>
       </c>
       <c r="D126" t="n">
-        <v>4787.28</v>
+        <v>1194.24</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2839,17 +2839,17 @@
         <v>46217</v>
       </c>
       <c r="B127" t="n">
-        <v>2308</v>
+        <v>1278</v>
       </c>
       <c r="C127" t="n">
-        <v>546</v>
+        <v>8888</v>
       </c>
       <c r="D127" t="n">
-        <v>1292.23</v>
+        <v>508.07</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2858,17 +2858,17 @@
         <v>46217</v>
       </c>
       <c r="B128" t="n">
-        <v>2709</v>
+        <v>58</v>
       </c>
       <c r="C128" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D128" t="n">
-        <v>1663.5</v>
+        <v>1411.43</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2877,17 +2877,17 @@
         <v>46217</v>
       </c>
       <c r="B129" t="n">
-        <v>1937</v>
+        <v>629</v>
       </c>
       <c r="C129" t="n">
         <v>8888</v>
       </c>
       <c r="D129" t="n">
-        <v>1492.4</v>
+        <v>2049.78</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2896,17 +2896,17 @@
         <v>46217</v>
       </c>
       <c r="B130" t="n">
-        <v>429</v>
+        <v>595</v>
       </c>
       <c r="C130" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D130" t="n">
-        <v>2195.97</v>
+        <v>3191</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2915,17 +2915,17 @@
         <v>46217</v>
       </c>
       <c r="B131" t="n">
-        <v>2211</v>
+        <v>949</v>
       </c>
       <c r="C131" t="n">
-        <v>8888</v>
+        <v>1762</v>
       </c>
       <c r="D131" t="n">
-        <v>1563.28</v>
+        <v>325.65</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2934,17 +2934,17 @@
         <v>46217</v>
       </c>
       <c r="B132" t="n">
-        <v>360</v>
+        <v>2463</v>
       </c>
       <c r="C132" t="n">
         <v>8888</v>
       </c>
       <c r="D132" t="n">
-        <v>15052.63</v>
+        <v>8336.43</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2953,17 +2953,17 @@
         <v>46217</v>
       </c>
       <c r="B133" t="n">
-        <v>2251</v>
+        <v>1064</v>
       </c>
       <c r="C133" t="n">
         <v>8888</v>
       </c>
       <c r="D133" t="n">
-        <v>797.58</v>
+        <v>1513.21</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2972,17 +2972,17 @@
         <v>46217</v>
       </c>
       <c r="B134" t="n">
-        <v>451</v>
+        <v>1478</v>
       </c>
       <c r="C134" t="n">
         <v>8888</v>
       </c>
       <c r="D134" t="n">
-        <v>1371.26</v>
+        <v>4067.5</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2991,17 +2991,17 @@
         <v>46217</v>
       </c>
       <c r="B135" t="n">
-        <v>40</v>
+        <v>438</v>
       </c>
       <c r="C135" t="n">
-        <v>8888</v>
+        <v>2845</v>
       </c>
       <c r="D135" t="n">
-        <v>1093.47</v>
+        <v>826.76</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3010,17 +3010,17 @@
         <v>46217</v>
       </c>
       <c r="B136" t="n">
-        <v>530</v>
+        <v>2539</v>
       </c>
       <c r="C136" t="n">
-        <v>8888</v>
+        <v>3009</v>
       </c>
       <c r="D136" t="n">
-        <v>180.08</v>
+        <v>1479.56</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3029,17 +3029,17 @@
         <v>46217</v>
       </c>
       <c r="B137" t="n">
-        <v>1137</v>
+        <v>358</v>
       </c>
       <c r="C137" t="n">
         <v>8888</v>
       </c>
       <c r="D137" t="n">
-        <v>3528.55</v>
+        <v>1918.33</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3048,17 +3048,17 @@
         <v>46217</v>
       </c>
       <c r="B138" t="n">
-        <v>1293</v>
+        <v>2107</v>
       </c>
       <c r="C138" t="n">
-        <v>601</v>
+        <v>8888</v>
       </c>
       <c r="D138" t="n">
-        <v>456.47</v>
+        <v>4459.75</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3067,17 +3067,17 @@
         <v>46217</v>
       </c>
       <c r="B139" t="n">
-        <v>2118</v>
+        <v>675</v>
       </c>
       <c r="C139" t="n">
         <v>8888</v>
       </c>
       <c r="D139" t="n">
-        <v>311.54</v>
+        <v>1559.23</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3086,17 +3086,17 @@
         <v>46217</v>
       </c>
       <c r="B140" t="n">
-        <v>424</v>
+        <v>2279</v>
       </c>
       <c r="C140" t="n">
         <v>8888</v>
       </c>
       <c r="D140" t="n">
-        <v>349.68</v>
+        <v>1165.17</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3105,13 +3105,13 @@
         <v>46217</v>
       </c>
       <c r="B141" t="n">
-        <v>1299</v>
+        <v>2727</v>
       </c>
       <c r="C141" t="n">
-        <v>27</v>
+        <v>3179</v>
       </c>
       <c r="D141" t="n">
-        <v>3625.32</v>
+        <v>514.7</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3124,17 +3124,17 @@
         <v>46217</v>
       </c>
       <c r="B142" t="n">
-        <v>559</v>
+        <v>451</v>
       </c>
       <c r="C142" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D142" t="n">
-        <v>1064.63</v>
+        <v>327.28</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3143,17 +3143,17 @@
         <v>46217</v>
       </c>
       <c r="B143" t="n">
-        <v>89</v>
+        <v>535</v>
       </c>
       <c r="C143" t="n">
         <v>8888</v>
       </c>
       <c r="D143" t="n">
-        <v>1506.42</v>
+        <v>1369.04</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3162,17 +3162,17 @@
         <v>46217</v>
       </c>
       <c r="B144" t="n">
-        <v>2250</v>
+        <v>2571</v>
       </c>
       <c r="C144" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D144" t="n">
-        <v>1943.54</v>
+        <v>2202.75</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3181,13 +3181,13 @@
         <v>46217</v>
       </c>
       <c r="B145" t="n">
-        <v>767</v>
+        <v>2782</v>
       </c>
       <c r="C145" t="n">
         <v>8888</v>
       </c>
       <c r="D145" t="n">
-        <v>472.62</v>
+        <v>753.8</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3200,17 +3200,17 @@
         <v>46217</v>
       </c>
       <c r="B146" t="n">
-        <v>2651</v>
+        <v>610</v>
       </c>
       <c r="C146" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D146" t="n">
-        <v>648.71</v>
+        <v>335.61</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3219,17 +3219,17 @@
         <v>46217</v>
       </c>
       <c r="B147" t="n">
-        <v>2114</v>
+        <v>2245</v>
       </c>
       <c r="C147" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D147" t="n">
-        <v>879.03</v>
+        <v>355.88</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3238,13 +3238,13 @@
         <v>46217</v>
       </c>
       <c r="B148" t="n">
-        <v>40</v>
+        <v>619</v>
       </c>
       <c r="C148" t="n">
         <v>8888</v>
       </c>
       <c r="D148" t="n">
-        <v>3583.39</v>
+        <v>3019.73</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -3257,17 +3257,17 @@
         <v>46217</v>
       </c>
       <c r="B149" t="n">
-        <v>40</v>
+        <v>1108</v>
       </c>
       <c r="C149" t="n">
         <v>8888</v>
       </c>
       <c r="D149" t="n">
-        <v>2529.31</v>
+        <v>508.54</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3276,17 +3276,17 @@
         <v>46217</v>
       </c>
       <c r="B150" t="n">
-        <v>626</v>
+        <v>341</v>
       </c>
       <c r="C150" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D150" t="n">
-        <v>18654.36</v>
+        <v>366.88</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3295,17 +3295,17 @@
         <v>46217</v>
       </c>
       <c r="B151" t="n">
-        <v>363</v>
+        <v>525</v>
       </c>
       <c r="C151" t="n">
-        <v>8888</v>
+        <v>1087</v>
       </c>
       <c r="D151" t="n">
-        <v>739.17</v>
+        <v>1830.26</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3314,13 +3314,13 @@
         <v>46217</v>
       </c>
       <c r="B152" t="n">
-        <v>675</v>
+        <v>1344</v>
       </c>
       <c r="C152" t="n">
-        <v>1898</v>
+        <v>2845</v>
       </c>
       <c r="D152" t="n">
-        <v>107.13</v>
+        <v>394.8</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -3333,17 +3333,17 @@
         <v>46217</v>
       </c>
       <c r="B153" t="n">
-        <v>636</v>
+        <v>1653</v>
       </c>
       <c r="C153" t="n">
         <v>8888</v>
       </c>
       <c r="D153" t="n">
-        <v>7476.56</v>
+        <v>4383.69</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3352,17 +3352,17 @@
         <v>46217</v>
       </c>
       <c r="B154" t="n">
-        <v>1075</v>
+        <v>1518</v>
       </c>
       <c r="C154" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D154" t="n">
-        <v>1331.89</v>
+        <v>479.84</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3371,13 +3371,13 @@
         <v>46217</v>
       </c>
       <c r="B155" t="n">
-        <v>2245</v>
+        <v>663</v>
       </c>
       <c r="C155" t="n">
         <v>8888</v>
       </c>
       <c r="D155" t="n">
-        <v>883.75</v>
+        <v>824.5599999999999</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -3390,13 +3390,13 @@
         <v>46217</v>
       </c>
       <c r="B156" t="n">
-        <v>477</v>
+        <v>1278</v>
       </c>
       <c r="C156" t="n">
         <v>8888</v>
       </c>
       <c r="D156" t="n">
-        <v>994.15</v>
+        <v>1267.68</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -3409,17 +3409,17 @@
         <v>46217</v>
       </c>
       <c r="B157" t="n">
-        <v>2015</v>
+        <v>2089</v>
       </c>
       <c r="C157" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D157" t="n">
-        <v>3243.05</v>
+        <v>822.05</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3428,13 +3428,13 @@
         <v>46217</v>
       </c>
       <c r="B158" t="n">
-        <v>1996</v>
+        <v>2133</v>
       </c>
       <c r="C158" t="n">
         <v>691</v>
       </c>
       <c r="D158" t="n">
-        <v>500.79</v>
+        <v>1414.98</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -3447,17 +3447,17 @@
         <v>46217</v>
       </c>
       <c r="B159" t="n">
-        <v>1653</v>
+        <v>429</v>
       </c>
       <c r="C159" t="n">
-        <v>8888</v>
+        <v>2571</v>
       </c>
       <c r="D159" t="n">
-        <v>4115.53</v>
+        <v>667.12</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3466,17 +3466,17 @@
         <v>46217</v>
       </c>
       <c r="B160" t="n">
-        <v>1064</v>
+        <v>2641</v>
       </c>
       <c r="C160" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D160" t="n">
-        <v>1052.68</v>
+        <v>252.41</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3485,17 +3485,17 @@
         <v>46217</v>
       </c>
       <c r="B161" t="n">
-        <v>1983</v>
+        <v>351</v>
       </c>
       <c r="C161" t="n">
-        <v>8888</v>
+        <v>3009</v>
       </c>
       <c r="D161" t="n">
-        <v>1246.33</v>
+        <v>1007.64</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3504,17 +3504,17 @@
         <v>46217</v>
       </c>
       <c r="B162" t="n">
-        <v>2118</v>
+        <v>1137</v>
       </c>
       <c r="C162" t="n">
         <v>8888</v>
       </c>
       <c r="D162" t="n">
-        <v>4886.49</v>
+        <v>5032.13</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3523,13 +3523,13 @@
         <v>46217</v>
       </c>
       <c r="B163" t="n">
-        <v>2680</v>
+        <v>1293</v>
       </c>
       <c r="C163" t="n">
         <v>8888</v>
       </c>
       <c r="D163" t="n">
-        <v>2285.31</v>
+        <v>8102.01</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -3542,17 +3542,17 @@
         <v>46217</v>
       </c>
       <c r="B164" t="n">
-        <v>2637</v>
+        <v>1465</v>
       </c>
       <c r="C164" t="n">
         <v>8888</v>
       </c>
       <c r="D164" t="n">
-        <v>1302.18</v>
+        <v>1609</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3561,17 +3561,17 @@
         <v>46217</v>
       </c>
       <c r="B165" t="n">
-        <v>1632</v>
+        <v>483</v>
       </c>
       <c r="C165" t="n">
         <v>8888</v>
       </c>
       <c r="D165" t="n">
-        <v>689.76</v>
+        <v>2444.39</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3580,17 +3580,17 @@
         <v>46217</v>
       </c>
       <c r="B166" t="n">
-        <v>1299</v>
+        <v>1064</v>
       </c>
       <c r="C166" t="n">
-        <v>2522</v>
+        <v>8888</v>
       </c>
       <c r="D166" t="n">
-        <v>3319.01</v>
+        <v>104632.21</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3599,17 +3599,17 @@
         <v>46217</v>
       </c>
       <c r="B167" t="n">
-        <v>2727</v>
+        <v>131</v>
       </c>
       <c r="C167" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D167" t="n">
-        <v>548.33</v>
+        <v>876.48</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3618,17 +3618,17 @@
         <v>46217</v>
       </c>
       <c r="B168" t="n">
-        <v>2026</v>
+        <v>663</v>
       </c>
       <c r="C168" t="n">
         <v>8888</v>
       </c>
       <c r="D168" t="n">
-        <v>699.05</v>
+        <v>1769.59</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3637,17 +3637,17 @@
         <v>46217</v>
       </c>
       <c r="B169" t="n">
-        <v>664</v>
+        <v>131</v>
       </c>
       <c r="C169" t="n">
         <v>8888</v>
       </c>
       <c r="D169" t="n">
-        <v>440.92</v>
+        <v>4787.28</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3656,13 +3656,13 @@
         <v>46217</v>
       </c>
       <c r="B170" t="n">
-        <v>629</v>
+        <v>2308</v>
       </c>
       <c r="C170" t="n">
-        <v>675</v>
+        <v>546</v>
       </c>
       <c r="D170" t="n">
-        <v>267.79</v>
+        <v>1292.23</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -3675,17 +3675,17 @@
         <v>46217</v>
       </c>
       <c r="B171" t="n">
-        <v>559</v>
+        <v>2709</v>
       </c>
       <c r="C171" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D171" t="n">
-        <v>1562.5</v>
+        <v>1663.5</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3694,17 +3694,17 @@
         <v>46217</v>
       </c>
       <c r="B172" t="n">
-        <v>1465</v>
+        <v>1937</v>
       </c>
       <c r="C172" t="n">
         <v>8888</v>
       </c>
       <c r="D172" t="n">
-        <v>10920.6</v>
+        <v>1492.4</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3713,17 +3713,17 @@
         <v>46217</v>
       </c>
       <c r="B173" t="n">
-        <v>2550</v>
+        <v>429</v>
       </c>
       <c r="C173" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D173" t="n">
-        <v>321.05</v>
+        <v>2195.97</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3732,17 +3732,17 @@
         <v>46217</v>
       </c>
       <c r="B174" t="n">
-        <v>1756</v>
+        <v>2211</v>
       </c>
       <c r="C174" t="n">
         <v>8888</v>
       </c>
       <c r="D174" t="n">
-        <v>2445</v>
+        <v>8568.99</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3751,17 +3751,17 @@
         <v>46217</v>
       </c>
       <c r="B175" t="n">
-        <v>890</v>
+        <v>360</v>
       </c>
       <c r="C175" t="n">
         <v>8888</v>
       </c>
       <c r="D175" t="n">
-        <v>4287.14</v>
+        <v>15052.63</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3770,13 +3770,13 @@
         <v>46217</v>
       </c>
       <c r="B176" t="n">
-        <v>363</v>
+        <v>2251</v>
       </c>
       <c r="C176" t="n">
         <v>8888</v>
       </c>
       <c r="D176" t="n">
-        <v>2517.01</v>
+        <v>797.58</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -3789,17 +3789,17 @@
         <v>46217</v>
       </c>
       <c r="B177" t="n">
-        <v>2698</v>
+        <v>451</v>
       </c>
       <c r="C177" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D177" t="n">
-        <v>1183.42</v>
+        <v>1371.26</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3808,17 +3808,17 @@
         <v>46217</v>
       </c>
       <c r="B178" t="n">
-        <v>535</v>
+        <v>40</v>
       </c>
       <c r="C178" t="n">
         <v>8888</v>
       </c>
       <c r="D178" t="n">
-        <v>5293.96</v>
+        <v>1093.47</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3827,17 +3827,17 @@
         <v>46217</v>
       </c>
       <c r="B179" t="n">
-        <v>2250</v>
+        <v>530</v>
       </c>
       <c r="C179" t="n">
         <v>8888</v>
       </c>
       <c r="D179" t="n">
-        <v>2650.33</v>
+        <v>180.08</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3846,17 +3846,17 @@
         <v>46217</v>
       </c>
       <c r="B180" t="n">
-        <v>2681</v>
+        <v>1327</v>
       </c>
       <c r="C180" t="n">
-        <v>8888</v>
+        <v>3009</v>
       </c>
       <c r="D180" t="n">
-        <v>2853.99</v>
+        <v>946.8</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3865,17 +3865,17 @@
         <v>46217</v>
       </c>
       <c r="B181" t="n">
-        <v>132</v>
+        <v>1293</v>
       </c>
       <c r="C181" t="n">
-        <v>8888</v>
+        <v>601</v>
       </c>
       <c r="D181" t="n">
-        <v>2623.22</v>
+        <v>456.47</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3884,17 +3884,17 @@
         <v>46217</v>
       </c>
       <c r="B182" t="n">
-        <v>2442</v>
+        <v>424</v>
       </c>
       <c r="C182" t="n">
         <v>8888</v>
       </c>
       <c r="D182" t="n">
-        <v>2822.22</v>
+        <v>1758.85</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3903,17 +3903,17 @@
         <v>46217</v>
       </c>
       <c r="B183" t="n">
-        <v>363</v>
+        <v>2118</v>
       </c>
       <c r="C183" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D183" t="n">
-        <v>3635.16</v>
+        <v>311.54</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3922,17 +3922,17 @@
         <v>46217</v>
       </c>
       <c r="B184" t="n">
-        <v>483</v>
+        <v>2251</v>
       </c>
       <c r="C184" t="n">
         <v>8888</v>
       </c>
       <c r="D184" t="n">
-        <v>2527.71</v>
+        <v>603.66</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3941,17 +3941,17 @@
         <v>46217</v>
       </c>
       <c r="B185" t="n">
-        <v>2607</v>
+        <v>1478</v>
       </c>
       <c r="C185" t="n">
-        <v>8888</v>
+        <v>675</v>
       </c>
       <c r="D185" t="n">
-        <v>1075.36</v>
+        <v>945.74</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3960,13 +3960,13 @@
         <v>46217</v>
       </c>
       <c r="B186" t="n">
-        <v>2330</v>
+        <v>1299</v>
       </c>
       <c r="C186" t="n">
-        <v>1954</v>
+        <v>27</v>
       </c>
       <c r="D186" t="n">
-        <v>1923.09</v>
+        <v>3625.32</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -3979,17 +3979,17 @@
         <v>46217</v>
       </c>
       <c r="B187" t="n">
-        <v>2472</v>
+        <v>559</v>
       </c>
       <c r="C187" t="n">
-        <v>2853</v>
+        <v>8888</v>
       </c>
       <c r="D187" t="n">
-        <v>824.0599999999999</v>
+        <v>1064.63</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3998,17 +3998,17 @@
         <v>46217</v>
       </c>
       <c r="B188" t="n">
-        <v>1384</v>
+        <v>89</v>
       </c>
       <c r="C188" t="n">
         <v>8888</v>
       </c>
       <c r="D188" t="n">
-        <v>585.27</v>
+        <v>1506.42</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4017,17 +4017,17 @@
         <v>46217</v>
       </c>
       <c r="B189" t="n">
-        <v>2709</v>
+        <v>2250</v>
       </c>
       <c r="C189" t="n">
         <v>8888</v>
       </c>
       <c r="D189" t="n">
-        <v>1667.47</v>
+        <v>1943.54</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4036,17 +4036,17 @@
         <v>46217</v>
       </c>
       <c r="B190" t="n">
-        <v>374</v>
+        <v>1327</v>
       </c>
       <c r="C190" t="n">
         <v>8888</v>
       </c>
       <c r="D190" t="n">
-        <v>1150.97</v>
+        <v>319.23</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4055,17 +4055,17 @@
         <v>46217</v>
       </c>
       <c r="B191" t="n">
-        <v>1137</v>
+        <v>326</v>
       </c>
       <c r="C191" t="n">
         <v>8888</v>
       </c>
       <c r="D191" t="n">
-        <v>4413.34</v>
+        <v>151.86</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4074,17 +4074,1024 @@
         <v>46217</v>
       </c>
       <c r="B192" t="n">
+        <v>1372</v>
+      </c>
+      <c r="C192" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D192" t="n">
+        <v>1088.02</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B193" t="n">
+        <v>767</v>
+      </c>
+      <c r="C193" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D193" t="n">
+        <v>472.62</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B194" t="n">
+        <v>626</v>
+      </c>
+      <c r="C194" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D194" t="n">
+        <v>24505.65</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B195" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C195" t="n">
+        <v>58</v>
+      </c>
+      <c r="D195" t="n">
+        <v>648.71</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B196" t="n">
+        <v>2114</v>
+      </c>
+      <c r="C196" t="n">
+        <v>1954</v>
+      </c>
+      <c r="D196" t="n">
+        <v>879.03</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B197" t="n">
+        <v>40</v>
+      </c>
+      <c r="C197" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D197" t="n">
+        <v>3583.39</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B198" t="n">
+        <v>40</v>
+      </c>
+      <c r="C198" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D198" t="n">
+        <v>2529.31</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B199" t="n">
+        <v>363</v>
+      </c>
+      <c r="C199" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D199" t="n">
+        <v>739.17</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B200" t="n">
+        <v>675</v>
+      </c>
+      <c r="C200" t="n">
+        <v>1898</v>
+      </c>
+      <c r="D200" t="n">
+        <v>107.13</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B201" t="n">
+        <v>636</v>
+      </c>
+      <c r="C201" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D201" t="n">
+        <v>7476.56</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B202" t="n">
+        <v>1075</v>
+      </c>
+      <c r="C202" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D202" t="n">
+        <v>1331.89</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B203" t="n">
+        <v>2245</v>
+      </c>
+      <c r="C203" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D203" t="n">
+        <v>883.75</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B204" t="n">
+        <v>477</v>
+      </c>
+      <c r="C204" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D204" t="n">
+        <v>994.15</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B205" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C205" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D205" t="n">
+        <v>3243.05</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B206" t="n">
+        <v>1996</v>
+      </c>
+      <c r="C206" t="n">
+        <v>691</v>
+      </c>
+      <c r="D206" t="n">
+        <v>500.79</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B207" t="n">
+        <v>1653</v>
+      </c>
+      <c r="C207" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D207" t="n">
+        <v>4115.53</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B208" t="n">
+        <v>1064</v>
+      </c>
+      <c r="C208" t="n">
+        <v>27</v>
+      </c>
+      <c r="D208" t="n">
+        <v>1153.23</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B209" t="n">
+        <v>1983</v>
+      </c>
+      <c r="C209" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D209" t="n">
+        <v>1246.33</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B210" t="n">
+        <v>2118</v>
+      </c>
+      <c r="C210" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D210" t="n">
+        <v>5870.04</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B211" t="n">
+        <v>559</v>
+      </c>
+      <c r="C211" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D211" t="n">
+        <v>2189.12</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B212" t="n">
+        <v>2680</v>
+      </c>
+      <c r="C212" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D212" t="n">
+        <v>2285.31</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B213" t="n">
+        <v>2637</v>
+      </c>
+      <c r="C213" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D213" t="n">
+        <v>1302.18</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B214" t="n">
+        <v>1632</v>
+      </c>
+      <c r="C214" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D214" t="n">
+        <v>689.76</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B215" t="n">
+        <v>1299</v>
+      </c>
+      <c r="C215" t="n">
+        <v>2522</v>
+      </c>
+      <c r="D215" t="n">
+        <v>3319.01</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B216" t="n">
+        <v>2727</v>
+      </c>
+      <c r="C216" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D216" t="n">
+        <v>548.33</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B217" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C217" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D217" t="n">
+        <v>699.05</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B218" t="n">
+        <v>664</v>
+      </c>
+      <c r="C218" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D218" t="n">
+        <v>3483.46</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B219" t="n">
+        <v>629</v>
+      </c>
+      <c r="C219" t="n">
+        <v>675</v>
+      </c>
+      <c r="D219" t="n">
+        <v>267.79</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B220" t="n">
+        <v>1465</v>
+      </c>
+      <c r="C220" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D220" t="n">
+        <v>12894.64</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B221" t="n">
+        <v>2550</v>
+      </c>
+      <c r="C221" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D221" t="n">
+        <v>321.05</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B222" t="n">
+        <v>1756</v>
+      </c>
+      <c r="C222" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D222" t="n">
+        <v>2445</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B223" t="n">
+        <v>890</v>
+      </c>
+      <c r="C223" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D223" t="n">
+        <v>4287.14</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B224" t="n">
+        <v>363</v>
+      </c>
+      <c r="C224" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D224" t="n">
+        <v>2517.01</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B225" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C225" t="n">
+        <v>874</v>
+      </c>
+      <c r="D225" t="n">
+        <v>1183.42</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B226" t="n">
+        <v>535</v>
+      </c>
+      <c r="C226" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D226" t="n">
+        <v>5293.96</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B227" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C227" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D227" t="n">
+        <v>2650.33</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B228" t="n">
+        <v>2681</v>
+      </c>
+      <c r="C228" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D228" t="n">
+        <v>2853.99</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B229" t="n">
+        <v>132</v>
+      </c>
+      <c r="C229" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D229" t="n">
+        <v>11123.92</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B230" t="n">
+        <v>2442</v>
+      </c>
+      <c r="C230" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D230" t="n">
+        <v>2822.22</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B231" t="n">
+        <v>363</v>
+      </c>
+      <c r="C231" t="n">
+        <v>1898</v>
+      </c>
+      <c r="D231" t="n">
+        <v>4028</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B232" t="n">
+        <v>483</v>
+      </c>
+      <c r="C232" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D232" t="n">
+        <v>3025.94</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B233" t="n">
+        <v>2279</v>
+      </c>
+      <c r="C233" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D233" t="n">
+        <v>740.38</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B234" t="n">
+        <v>2607</v>
+      </c>
+      <c r="C234" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D234" t="n">
+        <v>1075.36</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B235" t="n">
+        <v>2330</v>
+      </c>
+      <c r="C235" t="n">
+        <v>1954</v>
+      </c>
+      <c r="D235" t="n">
+        <v>1923.09</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B236" t="n">
+        <v>2472</v>
+      </c>
+      <c r="C236" t="n">
+        <v>2853</v>
+      </c>
+      <c r="D236" t="n">
+        <v>824.0599999999999</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B237" t="n">
+        <v>1384</v>
+      </c>
+      <c r="C237" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D237" t="n">
+        <v>585.27</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B238" t="n">
+        <v>2709</v>
+      </c>
+      <c r="C238" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D238" t="n">
+        <v>2210.08</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B239" t="n">
+        <v>619</v>
+      </c>
+      <c r="C239" t="n">
+        <v>1139</v>
+      </c>
+      <c r="D239" t="n">
+        <v>2098.5</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B240" t="n">
+        <v>374</v>
+      </c>
+      <c r="C240" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D240" t="n">
+        <v>1725.89</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B241" t="n">
+        <v>1137</v>
+      </c>
+      <c r="C241" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D241" t="n">
+        <v>4413.34</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B242" t="n">
         <v>2251</v>
       </c>
-      <c r="C192" t="n">
+      <c r="C242" t="n">
         <v>3403</v>
       </c>
-      <c r="D192" t="n">
+      <c r="D242" t="n">
         <v>510.18</v>
       </c>
-      <c r="E192" t="inlineStr">
-        <is>
-          <t>TELEMARKETING</t>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B243" t="n">
+        <v>2728</v>
+      </c>
+      <c r="C243" t="n">
+        <v>977</v>
+      </c>
+      <c r="D243" t="n">
+        <v>2256.87</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B244" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C244" t="n">
+        <v>1533</v>
+      </c>
+      <c r="D244" t="n">
+        <v>620.97</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B245" t="n">
+        <v>1380</v>
+      </c>
+      <c r="C245" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D245" t="n">
+        <v>947.8200000000001</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 08:47:42
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,17 +521,17 @@
         <v>46218</v>
       </c>
       <c r="B5" t="n">
-        <v>438</v>
+        <v>949</v>
       </c>
       <c r="C5" t="n">
-        <v>8888</v>
+        <v>1134</v>
       </c>
       <c r="D5" t="n">
-        <v>220.06</v>
+        <v>30.46</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -540,13 +540,13 @@
         <v>46218</v>
       </c>
       <c r="B6" t="n">
-        <v>451</v>
+        <v>438</v>
       </c>
       <c r="C6" t="n">
         <v>8888</v>
       </c>
       <c r="D6" t="n">
-        <v>368.93</v>
+        <v>220.06</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -559,17 +559,17 @@
         <v>46218</v>
       </c>
       <c r="B7" t="n">
-        <v>89</v>
+        <v>451</v>
       </c>
       <c r="C7" t="n">
-        <v>13148</v>
+        <v>8888</v>
       </c>
       <c r="D7" t="n">
-        <v>993.65</v>
+        <v>368.93</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -578,17 +578,17 @@
         <v>46218</v>
       </c>
       <c r="B8" t="n">
-        <v>1063</v>
+        <v>89</v>
       </c>
       <c r="C8" t="n">
-        <v>8888</v>
+        <v>13148</v>
       </c>
       <c r="D8" t="n">
-        <v>3137.87</v>
+        <v>993.65</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -603,11 +603,11 @@
         <v>8888</v>
       </c>
       <c r="D9" t="n">
-        <v>932.71</v>
+        <v>3137.87</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -616,17 +616,17 @@
         <v>46218</v>
       </c>
       <c r="B10" t="n">
-        <v>1007</v>
+        <v>1063</v>
       </c>
       <c r="C10" t="n">
         <v>8888</v>
       </c>
       <c r="D10" t="n">
-        <v>241.44</v>
+        <v>932.71</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -635,13 +635,13 @@
         <v>46218</v>
       </c>
       <c r="B11" t="n">
-        <v>1380</v>
+        <v>1007</v>
       </c>
       <c r="C11" t="n">
         <v>8888</v>
       </c>
       <c r="D11" t="n">
-        <v>520.2</v>
+        <v>241.44</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -654,17 +654,17 @@
         <v>46218</v>
       </c>
       <c r="B12" t="n">
-        <v>1756</v>
+        <v>1380</v>
       </c>
       <c r="C12" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D12" t="n">
-        <v>741.1799999999999</v>
+        <v>520.2</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -673,17 +673,17 @@
         <v>46218</v>
       </c>
       <c r="B13" t="n">
-        <v>816</v>
+        <v>1756</v>
       </c>
       <c r="C13" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D13" t="n">
-        <v>438.24</v>
+        <v>741.1799999999999</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -692,17 +692,17 @@
         <v>46218</v>
       </c>
       <c r="B14" t="n">
-        <v>953</v>
+        <v>816</v>
       </c>
       <c r="C14" t="n">
         <v>8888</v>
       </c>
       <c r="D14" t="n">
-        <v>926.16</v>
+        <v>438.24</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -711,15 +711,34 @@
         <v>46218</v>
       </c>
       <c r="B15" t="n">
+        <v>953</v>
+      </c>
+      <c r="C15" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D15" t="n">
+        <v>926.16</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B16" t="n">
         <v>1116</v>
       </c>
-      <c r="C15" t="n">
-        <v>8888</v>
-      </c>
-      <c r="D15" t="n">
+      <c r="C16" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D16" t="n">
         <v>2919.53</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>OPERADOR LOGÍSTICO</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 09:30:12
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -744,6 +744,25 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B17" t="n">
+        <v>42</v>
+      </c>
+      <c r="C17" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D17" t="n">
+        <v>79947.14999999999</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 10:30:03
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,17 +464,17 @@
         <v>46218</v>
       </c>
       <c r="B2" t="n">
-        <v>451</v>
+        <v>1075</v>
       </c>
       <c r="C2" t="n">
-        <v>8888</v>
+        <v>675</v>
       </c>
       <c r="D2" t="n">
-        <v>1103.58</v>
+        <v>638.4299999999999</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -483,17 +483,17 @@
         <v>46218</v>
       </c>
       <c r="B3" t="n">
-        <v>1364</v>
+        <v>451</v>
       </c>
       <c r="C3" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D3" t="n">
-        <v>275.01</v>
+        <v>1103.58</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -502,13 +502,13 @@
         <v>46218</v>
       </c>
       <c r="B4" t="n">
-        <v>1075</v>
+        <v>1364</v>
       </c>
       <c r="C4" t="n">
-        <v>675</v>
+        <v>3403</v>
       </c>
       <c r="D4" t="n">
-        <v>233.83</v>
+        <v>275.01</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -540,17 +540,17 @@
         <v>46218</v>
       </c>
       <c r="B6" t="n">
-        <v>438</v>
+        <v>58</v>
       </c>
       <c r="C6" t="n">
         <v>8888</v>
       </c>
       <c r="D6" t="n">
-        <v>220.06</v>
+        <v>499.11</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -559,17 +559,17 @@
         <v>46218</v>
       </c>
       <c r="B7" t="n">
-        <v>451</v>
+        <v>2245</v>
       </c>
       <c r="C7" t="n">
         <v>8888</v>
       </c>
       <c r="D7" t="n">
-        <v>368.93</v>
+        <v>2433.47</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -578,17 +578,17 @@
         <v>46218</v>
       </c>
       <c r="B8" t="n">
-        <v>89</v>
+        <v>438</v>
       </c>
       <c r="C8" t="n">
-        <v>13148</v>
+        <v>8888</v>
       </c>
       <c r="D8" t="n">
-        <v>993.65</v>
+        <v>220.06</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -597,13 +597,13 @@
         <v>46218</v>
       </c>
       <c r="B9" t="n">
-        <v>1063</v>
+        <v>451</v>
       </c>
       <c r="C9" t="n">
         <v>8888</v>
       </c>
       <c r="D9" t="n">
-        <v>3137.87</v>
+        <v>368.93</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -616,13 +616,13 @@
         <v>46218</v>
       </c>
       <c r="B10" t="n">
-        <v>1063</v>
+        <v>1075</v>
       </c>
       <c r="C10" t="n">
         <v>8888</v>
       </c>
       <c r="D10" t="n">
-        <v>932.71</v>
+        <v>1813.45</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -635,17 +635,17 @@
         <v>46218</v>
       </c>
       <c r="B11" t="n">
-        <v>1007</v>
+        <v>89</v>
       </c>
       <c r="C11" t="n">
-        <v>8888</v>
+        <v>13148</v>
       </c>
       <c r="D11" t="n">
-        <v>241.44</v>
+        <v>1883.74</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -654,13 +654,13 @@
         <v>46218</v>
       </c>
       <c r="B12" t="n">
-        <v>1380</v>
+        <v>1063</v>
       </c>
       <c r="C12" t="n">
         <v>8888</v>
       </c>
       <c r="D12" t="n">
-        <v>520.2</v>
+        <v>3576.45</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -673,17 +673,17 @@
         <v>46218</v>
       </c>
       <c r="B13" t="n">
-        <v>1756</v>
+        <v>285</v>
       </c>
       <c r="C13" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D13" t="n">
-        <v>741.1799999999999</v>
+        <v>555.64</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -692,17 +692,17 @@
         <v>46218</v>
       </c>
       <c r="B14" t="n">
-        <v>816</v>
+        <v>1063</v>
       </c>
       <c r="C14" t="n">
         <v>8888</v>
       </c>
       <c r="D14" t="n">
-        <v>438.24</v>
+        <v>932.71</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -711,13 +711,13 @@
         <v>46218</v>
       </c>
       <c r="B15" t="n">
-        <v>953</v>
+        <v>1937</v>
       </c>
       <c r="C15" t="n">
         <v>8888</v>
       </c>
       <c r="D15" t="n">
-        <v>926.16</v>
+        <v>338.93</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -730,17 +730,17 @@
         <v>46218</v>
       </c>
       <c r="B16" t="n">
-        <v>1116</v>
+        <v>1063</v>
       </c>
       <c r="C16" t="n">
         <v>8888</v>
       </c>
       <c r="D16" t="n">
-        <v>2919.53</v>
+        <v>1113.08</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -749,15 +749,205 @@
         <v>46218</v>
       </c>
       <c r="B17" t="n">
+        <v>1007</v>
+      </c>
+      <c r="C17" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D17" t="n">
+        <v>241.44</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B18" t="n">
+        <v>1380</v>
+      </c>
+      <c r="C18" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D18" t="n">
+        <v>520.2</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B19" t="n">
+        <v>285</v>
+      </c>
+      <c r="C19" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D19" t="n">
+        <v>364.44</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B20" t="n">
+        <v>1756</v>
+      </c>
+      <c r="C20" t="n">
+        <v>27</v>
+      </c>
+      <c r="D20" t="n">
+        <v>741.1799999999999</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B21" t="n">
+        <v>816</v>
+      </c>
+      <c r="C21" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D21" t="n">
+        <v>438.24</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B22" t="n">
+        <v>953</v>
+      </c>
+      <c r="C22" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1254.07</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B23" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C23" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D23" t="n">
+        <v>532.91</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B24" t="n">
+        <v>1478</v>
+      </c>
+      <c r="C24" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D24" t="n">
+        <v>251.69</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B25" t="n">
+        <v>131</v>
+      </c>
+      <c r="C25" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D25" t="n">
+        <v>765.99</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B26" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C26" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D26" t="n">
+        <v>2919.53</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B27" t="n">
         <v>42</v>
       </c>
-      <c r="C17" t="n">
-        <v>8888</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="C27" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D27" t="n">
         <v>79947.14999999999</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>OPERADOR LOGÍSTICO</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 11:00:02
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,7 +622,7 @@
         <v>8888</v>
       </c>
       <c r="D10" t="n">
-        <v>1813.45</v>
+        <v>2568.51</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -635,17 +635,17 @@
         <v>46218</v>
       </c>
       <c r="B11" t="n">
-        <v>89</v>
+        <v>483</v>
       </c>
       <c r="C11" t="n">
-        <v>13148</v>
+        <v>8888</v>
       </c>
       <c r="D11" t="n">
-        <v>1883.74</v>
+        <v>2027.7</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -654,17 +654,17 @@
         <v>46218</v>
       </c>
       <c r="B12" t="n">
-        <v>1063</v>
+        <v>89</v>
       </c>
       <c r="C12" t="n">
-        <v>8888</v>
+        <v>13148</v>
       </c>
       <c r="D12" t="n">
-        <v>3576.45</v>
+        <v>1883.74</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -673,17 +673,17 @@
         <v>46218</v>
       </c>
       <c r="B13" t="n">
-        <v>285</v>
+        <v>1063</v>
       </c>
       <c r="C13" t="n">
         <v>8888</v>
       </c>
       <c r="D13" t="n">
-        <v>555.64</v>
+        <v>3576.45</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -692,13 +692,13 @@
         <v>46218</v>
       </c>
       <c r="B14" t="n">
-        <v>1063</v>
+        <v>285</v>
       </c>
       <c r="C14" t="n">
         <v>8888</v>
       </c>
       <c r="D14" t="n">
-        <v>932.71</v>
+        <v>555.64</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -711,13 +711,13 @@
         <v>46218</v>
       </c>
       <c r="B15" t="n">
-        <v>1937</v>
+        <v>1063</v>
       </c>
       <c r="C15" t="n">
         <v>8888</v>
       </c>
       <c r="D15" t="n">
-        <v>338.93</v>
+        <v>932.71</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -730,17 +730,17 @@
         <v>46218</v>
       </c>
       <c r="B16" t="n">
-        <v>1063</v>
+        <v>1937</v>
       </c>
       <c r="C16" t="n">
         <v>8888</v>
       </c>
       <c r="D16" t="n">
-        <v>1113.08</v>
+        <v>338.93</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -749,17 +749,17 @@
         <v>46218</v>
       </c>
       <c r="B17" t="n">
-        <v>1007</v>
+        <v>1063</v>
       </c>
       <c r="C17" t="n">
         <v>8888</v>
       </c>
       <c r="D17" t="n">
-        <v>241.44</v>
+        <v>1113.08</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -768,13 +768,13 @@
         <v>46218</v>
       </c>
       <c r="B18" t="n">
-        <v>1380</v>
+        <v>1007</v>
       </c>
       <c r="C18" t="n">
         <v>8888</v>
       </c>
       <c r="D18" t="n">
-        <v>520.2</v>
+        <v>241.44</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -787,17 +787,17 @@
         <v>46218</v>
       </c>
       <c r="B19" t="n">
-        <v>285</v>
+        <v>1380</v>
       </c>
       <c r="C19" t="n">
         <v>8888</v>
       </c>
       <c r="D19" t="n">
-        <v>364.44</v>
+        <v>520.2</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -806,13 +806,13 @@
         <v>46218</v>
       </c>
       <c r="B20" t="n">
-        <v>1756</v>
+        <v>483</v>
       </c>
       <c r="C20" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="D20" t="n">
-        <v>741.1799999999999</v>
+        <v>2026.73</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -825,17 +825,17 @@
         <v>46218</v>
       </c>
       <c r="B21" t="n">
-        <v>816</v>
+        <v>285</v>
       </c>
       <c r="C21" t="n">
         <v>8888</v>
       </c>
       <c r="D21" t="n">
-        <v>438.24</v>
+        <v>364.44</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -844,17 +844,17 @@
         <v>46218</v>
       </c>
       <c r="B22" t="n">
-        <v>953</v>
+        <v>1756</v>
       </c>
       <c r="C22" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D22" t="n">
-        <v>1254.07</v>
+        <v>741.1799999999999</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -863,13 +863,13 @@
         <v>46218</v>
       </c>
       <c r="B23" t="n">
-        <v>2782</v>
+        <v>629</v>
       </c>
       <c r="C23" t="n">
         <v>8888</v>
       </c>
       <c r="D23" t="n">
-        <v>532.91</v>
+        <v>339.19</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -882,17 +882,17 @@
         <v>46218</v>
       </c>
       <c r="B24" t="n">
-        <v>1478</v>
+        <v>816</v>
       </c>
       <c r="C24" t="n">
         <v>8888</v>
       </c>
       <c r="D24" t="n">
-        <v>251.69</v>
+        <v>438.24</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -901,13 +901,13 @@
         <v>46218</v>
       </c>
       <c r="B25" t="n">
-        <v>131</v>
+        <v>953</v>
       </c>
       <c r="C25" t="n">
         <v>8888</v>
       </c>
       <c r="D25" t="n">
-        <v>765.99</v>
+        <v>1254.07</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -920,17 +920,17 @@
         <v>46218</v>
       </c>
       <c r="B26" t="n">
-        <v>1116</v>
+        <v>131</v>
       </c>
       <c r="C26" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D26" t="n">
-        <v>2919.53</v>
+        <v>91.86</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -939,15 +939,91 @@
         <v>46218</v>
       </c>
       <c r="B27" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C27" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D27" t="n">
+        <v>532.91</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B28" t="n">
+        <v>1478</v>
+      </c>
+      <c r="C28" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D28" t="n">
+        <v>251.69</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B29" t="n">
+        <v>131</v>
+      </c>
+      <c r="C29" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1125.63</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B30" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C30" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D30" t="n">
+        <v>2919.53</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B31" t="n">
         <v>42</v>
       </c>
-      <c r="C27" t="n">
-        <v>8888</v>
-      </c>
-      <c r="D27" t="n">
+      <c r="C31" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D31" t="n">
         <v>79947.14999999999</v>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>OPERADOR LOGÍSTICO</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 11:30:03
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -616,17 +616,17 @@
         <v>46218</v>
       </c>
       <c r="B10" t="n">
-        <v>1075</v>
+        <v>2714</v>
       </c>
       <c r="C10" t="n">
-        <v>8888</v>
+        <v>519</v>
       </c>
       <c r="D10" t="n">
-        <v>2568.51</v>
+        <v>61939.22</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -635,17 +635,17 @@
         <v>46218</v>
       </c>
       <c r="B11" t="n">
-        <v>483</v>
+        <v>1075</v>
       </c>
       <c r="C11" t="n">
         <v>8888</v>
       </c>
       <c r="D11" t="n">
-        <v>2027.7</v>
+        <v>5216.32</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -654,17 +654,17 @@
         <v>46218</v>
       </c>
       <c r="B12" t="n">
-        <v>89</v>
+        <v>483</v>
       </c>
       <c r="C12" t="n">
-        <v>13148</v>
+        <v>8888</v>
       </c>
       <c r="D12" t="n">
-        <v>1883.74</v>
+        <v>2027.7</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -673,17 +673,17 @@
         <v>46218</v>
       </c>
       <c r="B13" t="n">
-        <v>1063</v>
+        <v>89</v>
       </c>
       <c r="C13" t="n">
-        <v>8888</v>
+        <v>13148</v>
       </c>
       <c r="D13" t="n">
-        <v>3576.45</v>
+        <v>1883.74</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -692,17 +692,17 @@
         <v>46218</v>
       </c>
       <c r="B14" t="n">
-        <v>285</v>
+        <v>1063</v>
       </c>
       <c r="C14" t="n">
         <v>8888</v>
       </c>
       <c r="D14" t="n">
-        <v>555.64</v>
+        <v>3576.45</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -711,17 +711,17 @@
         <v>46218</v>
       </c>
       <c r="B15" t="n">
-        <v>1063</v>
+        <v>1299</v>
       </c>
       <c r="C15" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D15" t="n">
-        <v>932.71</v>
+        <v>990.24</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -730,13 +730,13 @@
         <v>46218</v>
       </c>
       <c r="B16" t="n">
-        <v>1937</v>
+        <v>285</v>
       </c>
       <c r="C16" t="n">
         <v>8888</v>
       </c>
       <c r="D16" t="n">
-        <v>338.93</v>
+        <v>555.64</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -755,11 +755,11 @@
         <v>8888</v>
       </c>
       <c r="D17" t="n">
-        <v>1113.08</v>
+        <v>932.71</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -768,13 +768,13 @@
         <v>46218</v>
       </c>
       <c r="B18" t="n">
-        <v>1007</v>
+        <v>1465</v>
       </c>
       <c r="C18" t="n">
         <v>8888</v>
       </c>
       <c r="D18" t="n">
-        <v>241.44</v>
+        <v>2431.47</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -787,17 +787,17 @@
         <v>46218</v>
       </c>
       <c r="B19" t="n">
-        <v>1380</v>
+        <v>1937</v>
       </c>
       <c r="C19" t="n">
         <v>8888</v>
       </c>
       <c r="D19" t="n">
-        <v>520.2</v>
+        <v>833.52</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -806,13 +806,13 @@
         <v>46218</v>
       </c>
       <c r="B20" t="n">
-        <v>483</v>
+        <v>477</v>
       </c>
       <c r="C20" t="n">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="D20" t="n">
-        <v>2026.73</v>
+        <v>736.03</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -825,13 +825,13 @@
         <v>46218</v>
       </c>
       <c r="B21" t="n">
-        <v>285</v>
+        <v>1063</v>
       </c>
       <c r="C21" t="n">
         <v>8888</v>
       </c>
       <c r="D21" t="n">
-        <v>364.44</v>
+        <v>1113.08</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -844,17 +844,17 @@
         <v>46218</v>
       </c>
       <c r="B22" t="n">
-        <v>1756</v>
+        <v>1007</v>
       </c>
       <c r="C22" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D22" t="n">
-        <v>741.1799999999999</v>
+        <v>241.44</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -863,13 +863,13 @@
         <v>46218</v>
       </c>
       <c r="B23" t="n">
-        <v>629</v>
+        <v>1380</v>
       </c>
       <c r="C23" t="n">
         <v>8888</v>
       </c>
       <c r="D23" t="n">
-        <v>339.19</v>
+        <v>520.2</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -882,17 +882,17 @@
         <v>46218</v>
       </c>
       <c r="B24" t="n">
-        <v>816</v>
+        <v>483</v>
       </c>
       <c r="C24" t="n">
-        <v>8888</v>
+        <v>38</v>
       </c>
       <c r="D24" t="n">
-        <v>438.24</v>
+        <v>2026.73</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -901,17 +901,17 @@
         <v>46218</v>
       </c>
       <c r="B25" t="n">
-        <v>953</v>
+        <v>1075</v>
       </c>
       <c r="C25" t="n">
         <v>8888</v>
       </c>
       <c r="D25" t="n">
-        <v>1254.07</v>
+        <v>557.62</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
         <v>46218</v>
       </c>
       <c r="B26" t="n">
-        <v>131</v>
+        <v>285</v>
       </c>
       <c r="C26" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D26" t="n">
-        <v>91.86</v>
+        <v>364.44</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -939,17 +939,17 @@
         <v>46218</v>
       </c>
       <c r="B27" t="n">
-        <v>2782</v>
+        <v>1756</v>
       </c>
       <c r="C27" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D27" t="n">
-        <v>532.91</v>
+        <v>741.1799999999999</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -958,17 +958,17 @@
         <v>46218</v>
       </c>
       <c r="B28" t="n">
-        <v>1478</v>
+        <v>629</v>
       </c>
       <c r="C28" t="n">
         <v>8888</v>
       </c>
       <c r="D28" t="n">
-        <v>251.69</v>
+        <v>339.19</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -977,17 +977,17 @@
         <v>46218</v>
       </c>
       <c r="B29" t="n">
-        <v>131</v>
+        <v>816</v>
       </c>
       <c r="C29" t="n">
         <v>8888</v>
       </c>
       <c r="D29" t="n">
-        <v>1125.63</v>
+        <v>438.24</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -996,13 +996,13 @@
         <v>46218</v>
       </c>
       <c r="B30" t="n">
-        <v>1116</v>
+        <v>953</v>
       </c>
       <c r="C30" t="n">
         <v>8888</v>
       </c>
       <c r="D30" t="n">
-        <v>2919.53</v>
+        <v>1254.07</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1015,15 +1015,129 @@
         <v>46218</v>
       </c>
       <c r="B31" t="n">
+        <v>1465</v>
+      </c>
+      <c r="C31" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1342.74</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B32" t="n">
+        <v>131</v>
+      </c>
+      <c r="C32" t="n">
+        <v>27</v>
+      </c>
+      <c r="D32" t="n">
+        <v>91.86</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B33" t="n">
+        <v>1478</v>
+      </c>
+      <c r="C33" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D33" t="n">
+        <v>459.57</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B34" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C34" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D34" t="n">
+        <v>994.77</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B35" t="n">
+        <v>131</v>
+      </c>
+      <c r="C35" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1125.63</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B36" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C36" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D36" t="n">
+        <v>2919.53</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B37" t="n">
         <v>42</v>
       </c>
-      <c r="C31" t="n">
-        <v>8888</v>
-      </c>
-      <c r="D31" t="n">
+      <c r="C37" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D37" t="n">
         <v>79947.14999999999</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>OPERADOR LOGÍSTICO</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 13:22:24
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,17 +483,17 @@
         <v>46218</v>
       </c>
       <c r="B3" t="n">
-        <v>451</v>
+        <v>1364</v>
       </c>
       <c r="C3" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D3" t="n">
-        <v>1103.58</v>
+        <v>1300.54</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -502,17 +502,17 @@
         <v>46218</v>
       </c>
       <c r="B4" t="n">
-        <v>1364</v>
+        <v>451</v>
       </c>
       <c r="C4" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D4" t="n">
-        <v>275.01</v>
+        <v>1103.58</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -521,17 +521,17 @@
         <v>46218</v>
       </c>
       <c r="B5" t="n">
-        <v>949</v>
+        <v>2651</v>
       </c>
       <c r="C5" t="n">
-        <v>1134</v>
+        <v>8888</v>
       </c>
       <c r="D5" t="n">
-        <v>30.46</v>
+        <v>660.95</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -540,17 +540,17 @@
         <v>46218</v>
       </c>
       <c r="B6" t="n">
-        <v>58</v>
+        <v>2118</v>
       </c>
       <c r="C6" t="n">
         <v>8888</v>
       </c>
       <c r="D6" t="n">
-        <v>499.11</v>
+        <v>452.46</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -559,17 +559,17 @@
         <v>46218</v>
       </c>
       <c r="B7" t="n">
-        <v>2245</v>
+        <v>949</v>
       </c>
       <c r="C7" t="n">
-        <v>8888</v>
+        <v>1134</v>
       </c>
       <c r="D7" t="n">
-        <v>2433.47</v>
+        <v>30.46</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -578,17 +578,17 @@
         <v>46218</v>
       </c>
       <c r="B8" t="n">
-        <v>438</v>
+        <v>58</v>
       </c>
       <c r="C8" t="n">
         <v>8888</v>
       </c>
       <c r="D8" t="n">
-        <v>220.06</v>
+        <v>499.11</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -597,17 +597,17 @@
         <v>46218</v>
       </c>
       <c r="B9" t="n">
-        <v>451</v>
+        <v>2245</v>
       </c>
       <c r="C9" t="n">
         <v>8888</v>
       </c>
       <c r="D9" t="n">
-        <v>368.93</v>
+        <v>2433.47</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -616,17 +616,17 @@
         <v>46218</v>
       </c>
       <c r="B10" t="n">
-        <v>2714</v>
+        <v>535</v>
       </c>
       <c r="C10" t="n">
-        <v>519</v>
+        <v>8888</v>
       </c>
       <c r="D10" t="n">
-        <v>61939.22</v>
+        <v>583.85</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -635,17 +635,17 @@
         <v>46218</v>
       </c>
       <c r="B11" t="n">
-        <v>1075</v>
+        <v>438</v>
       </c>
       <c r="C11" t="n">
         <v>8888</v>
       </c>
       <c r="D11" t="n">
-        <v>5216.32</v>
+        <v>220.06</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -654,17 +654,17 @@
         <v>46218</v>
       </c>
       <c r="B12" t="n">
-        <v>483</v>
+        <v>325</v>
       </c>
       <c r="C12" t="n">
         <v>8888</v>
       </c>
       <c r="D12" t="n">
-        <v>2027.7</v>
+        <v>57.46</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -673,17 +673,17 @@
         <v>46218</v>
       </c>
       <c r="B13" t="n">
-        <v>89</v>
+        <v>451</v>
       </c>
       <c r="C13" t="n">
-        <v>13148</v>
+        <v>8888</v>
       </c>
       <c r="D13" t="n">
-        <v>1883.74</v>
+        <v>368.93</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -692,17 +692,17 @@
         <v>46218</v>
       </c>
       <c r="B14" t="n">
-        <v>1063</v>
+        <v>2714</v>
       </c>
       <c r="C14" t="n">
-        <v>8888</v>
+        <v>519</v>
       </c>
       <c r="D14" t="n">
-        <v>3576.45</v>
+        <v>61939.22</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -711,17 +711,17 @@
         <v>46218</v>
       </c>
       <c r="B15" t="n">
-        <v>1299</v>
+        <v>1075</v>
       </c>
       <c r="C15" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D15" t="n">
-        <v>990.24</v>
+        <v>11607.79</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -730,17 +730,17 @@
         <v>46218</v>
       </c>
       <c r="B16" t="n">
-        <v>285</v>
+        <v>2651</v>
       </c>
       <c r="C16" t="n">
         <v>8888</v>
       </c>
       <c r="D16" t="n">
-        <v>555.64</v>
+        <v>1296.58</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -749,17 +749,17 @@
         <v>46218</v>
       </c>
       <c r="B17" t="n">
-        <v>1063</v>
+        <v>89</v>
       </c>
       <c r="C17" t="n">
-        <v>8888</v>
+        <v>13148</v>
       </c>
       <c r="D17" t="n">
-        <v>932.71</v>
+        <v>1883.74</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
         <v>46218</v>
       </c>
       <c r="B18" t="n">
-        <v>1465</v>
+        <v>629</v>
       </c>
       <c r="C18" t="n">
         <v>8888</v>
       </c>
       <c r="D18" t="n">
-        <v>2431.47</v>
+        <v>553.13</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -787,17 +787,17 @@
         <v>46218</v>
       </c>
       <c r="B19" t="n">
-        <v>1937</v>
+        <v>2211</v>
       </c>
       <c r="C19" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D19" t="n">
-        <v>833.52</v>
+        <v>1526.94</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -806,17 +806,17 @@
         <v>46218</v>
       </c>
       <c r="B20" t="n">
-        <v>477</v>
+        <v>1063</v>
       </c>
       <c r="C20" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D20" t="n">
-        <v>736.03</v>
+        <v>4487.11</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -825,17 +825,17 @@
         <v>46218</v>
       </c>
       <c r="B21" t="n">
-        <v>1063</v>
+        <v>1299</v>
       </c>
       <c r="C21" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D21" t="n">
-        <v>1113.08</v>
+        <v>990.24</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -844,17 +844,17 @@
         <v>46218</v>
       </c>
       <c r="B22" t="n">
-        <v>1007</v>
+        <v>285</v>
       </c>
       <c r="C22" t="n">
         <v>8888</v>
       </c>
       <c r="D22" t="n">
-        <v>241.44</v>
+        <v>555.64</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -863,17 +863,17 @@
         <v>46218</v>
       </c>
       <c r="B23" t="n">
-        <v>1380</v>
+        <v>477</v>
       </c>
       <c r="C23" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D23" t="n">
-        <v>520.2</v>
+        <v>1540.55</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -882,17 +882,17 @@
         <v>46218</v>
       </c>
       <c r="B24" t="n">
-        <v>483</v>
+        <v>1063</v>
       </c>
       <c r="C24" t="n">
-        <v>38</v>
+        <v>8888</v>
       </c>
       <c r="D24" t="n">
-        <v>2026.73</v>
+        <v>2549.86</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -901,13 +901,13 @@
         <v>46218</v>
       </c>
       <c r="B25" t="n">
-        <v>1075</v>
+        <v>1465</v>
       </c>
       <c r="C25" t="n">
         <v>8888</v>
       </c>
       <c r="D25" t="n">
-        <v>557.62</v>
+        <v>2431.47</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -920,13 +920,13 @@
         <v>46218</v>
       </c>
       <c r="B26" t="n">
-        <v>285</v>
+        <v>89</v>
       </c>
       <c r="C26" t="n">
         <v>8888</v>
       </c>
       <c r="D26" t="n">
-        <v>364.44</v>
+        <v>479</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -939,13 +939,13 @@
         <v>46218</v>
       </c>
       <c r="B27" t="n">
-        <v>1756</v>
+        <v>1465</v>
       </c>
       <c r="C27" t="n">
-        <v>27</v>
+        <v>3403</v>
       </c>
       <c r="D27" t="n">
-        <v>741.1799999999999</v>
+        <v>777.2</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -958,17 +958,17 @@
         <v>46218</v>
       </c>
       <c r="B28" t="n">
-        <v>629</v>
+        <v>1937</v>
       </c>
       <c r="C28" t="n">
         <v>8888</v>
       </c>
       <c r="D28" t="n">
-        <v>339.19</v>
+        <v>833.52</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -977,17 +977,17 @@
         <v>46218</v>
       </c>
       <c r="B29" t="n">
-        <v>816</v>
+        <v>1063</v>
       </c>
       <c r="C29" t="n">
         <v>8888</v>
       </c>
       <c r="D29" t="n">
-        <v>438.24</v>
+        <v>1113.08</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -996,13 +996,13 @@
         <v>46218</v>
       </c>
       <c r="B30" t="n">
-        <v>953</v>
+        <v>1293</v>
       </c>
       <c r="C30" t="n">
         <v>8888</v>
       </c>
       <c r="D30" t="n">
-        <v>1254.07</v>
+        <v>386.33</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1015,17 +1015,17 @@
         <v>46218</v>
       </c>
       <c r="B31" t="n">
-        <v>1465</v>
+        <v>2089</v>
       </c>
       <c r="C31" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D31" t="n">
-        <v>1342.74</v>
+        <v>442.44</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1034,17 +1034,17 @@
         <v>46218</v>
       </c>
       <c r="B32" t="n">
-        <v>131</v>
+        <v>1007</v>
       </c>
       <c r="C32" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D32" t="n">
-        <v>91.86</v>
+        <v>241.44</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1053,17 +1053,17 @@
         <v>46218</v>
       </c>
       <c r="B33" t="n">
-        <v>1478</v>
+        <v>1380</v>
       </c>
       <c r="C33" t="n">
         <v>8888</v>
       </c>
       <c r="D33" t="n">
-        <v>459.57</v>
+        <v>520.2</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1072,13 +1072,13 @@
         <v>46218</v>
       </c>
       <c r="B34" t="n">
-        <v>2782</v>
+        <v>1075</v>
       </c>
       <c r="C34" t="n">
         <v>8888</v>
       </c>
       <c r="D34" t="n">
-        <v>994.77</v>
+        <v>2179.03</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1091,17 +1091,17 @@
         <v>46218</v>
       </c>
       <c r="B35" t="n">
-        <v>131</v>
+        <v>2245</v>
       </c>
       <c r="C35" t="n">
         <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>1125.63</v>
+        <v>361.58</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1110,17 @@
         <v>46218</v>
       </c>
       <c r="B36" t="n">
-        <v>1116</v>
+        <v>285</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>2919.53</v>
+        <v>364.44</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1129,378 @@
         <v>46218</v>
       </c>
       <c r="B37" t="n">
+        <v>1756</v>
+      </c>
+      <c r="C37" t="n">
+        <v>27</v>
+      </c>
+      <c r="D37" t="n">
+        <v>741.1799999999999</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B38" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" t="n">
+        <v>58</v>
+      </c>
+      <c r="D38" t="n">
+        <v>363.7</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B39" t="n">
+        <v>1064</v>
+      </c>
+      <c r="C39" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1274.3</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B40" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C40" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D40" t="n">
+        <v>552.15</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B41" t="n">
+        <v>629</v>
+      </c>
+      <c r="C41" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D41" t="n">
+        <v>339.19</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B42" t="n">
+        <v>664</v>
+      </c>
+      <c r="C42" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1595.68</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B43" t="n">
+        <v>816</v>
+      </c>
+      <c r="C43" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D43" t="n">
+        <v>438.24</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B44" t="n">
+        <v>953</v>
+      </c>
+      <c r="C44" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D44" t="n">
+        <v>2618.89</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B45" t="n">
+        <v>1465</v>
+      </c>
+      <c r="C45" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D45" t="n">
+        <v>3504</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B46" t="n">
+        <v>2245</v>
+      </c>
+      <c r="C46" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D46" t="n">
+        <v>427.51</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B47" t="n">
+        <v>131</v>
+      </c>
+      <c r="C47" t="n">
+        <v>27</v>
+      </c>
+      <c r="D47" t="n">
+        <v>91.86</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B48" t="n">
+        <v>451</v>
+      </c>
+      <c r="C48" t="n">
+        <v>3403</v>
+      </c>
+      <c r="D48" t="n">
+        <v>445.58</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B49" t="n">
+        <v>2114</v>
+      </c>
+      <c r="C49" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D49" t="n">
+        <v>641.92</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B50" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C50" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D50" t="n">
+        <v>1786.32</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B51" t="n">
+        <v>1478</v>
+      </c>
+      <c r="C51" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D51" t="n">
+        <v>459.57</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B52" t="n">
+        <v>131</v>
+      </c>
+      <c r="C52" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D52" t="n">
+        <v>1125.63</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B53" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C53" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D53" t="n">
+        <v>2599.69</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B54" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C54" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D54" t="n">
+        <v>2919.53</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B55" t="n">
         <v>42</v>
       </c>
-      <c r="C37" t="n">
-        <v>8888</v>
-      </c>
-      <c r="D37" t="n">
+      <c r="C55" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D55" t="n">
         <v>79947.14999999999</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B56" t="n">
+        <v>2109</v>
+      </c>
+      <c r="C56" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D56" t="n">
+        <v>788.98</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 13:30:04
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1110,17 +1110,17 @@
         <v>46218</v>
       </c>
       <c r="B36" t="n">
-        <v>285</v>
+        <v>452</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>364.44</v>
+        <v>608.78</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1129,17 @@
         <v>46218</v>
       </c>
       <c r="B37" t="n">
-        <v>1756</v>
+        <v>285</v>
       </c>
       <c r="C37" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D37" t="n">
-        <v>741.1799999999999</v>
+        <v>364.44</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1148,13 +1148,13 @@
         <v>46218</v>
       </c>
       <c r="B38" t="n">
-        <v>2651</v>
+        <v>1756</v>
       </c>
       <c r="C38" t="n">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="D38" t="n">
-        <v>363.7</v>
+        <v>741.1799999999999</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1167,17 +1167,17 @@
         <v>46218</v>
       </c>
       <c r="B39" t="n">
-        <v>1064</v>
+        <v>2651</v>
       </c>
       <c r="C39" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D39" t="n">
-        <v>1274.3</v>
+        <v>363.7</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1186,13 +1186,13 @@
         <v>46218</v>
       </c>
       <c r="B40" t="n">
-        <v>2698</v>
+        <v>1064</v>
       </c>
       <c r="C40" t="n">
         <v>8888</v>
       </c>
       <c r="D40" t="n">
-        <v>552.15</v>
+        <v>1274.3</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1205,13 +1205,13 @@
         <v>46218</v>
       </c>
       <c r="B41" t="n">
-        <v>629</v>
+        <v>2698</v>
       </c>
       <c r="C41" t="n">
         <v>8888</v>
       </c>
       <c r="D41" t="n">
-        <v>339.19</v>
+        <v>552.15</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1224,17 +1224,17 @@
         <v>46218</v>
       </c>
       <c r="B42" t="n">
-        <v>664</v>
+        <v>629</v>
       </c>
       <c r="C42" t="n">
         <v>8888</v>
       </c>
       <c r="D42" t="n">
-        <v>1595.68</v>
+        <v>339.19</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1243,17 +1243,17 @@
         <v>46218</v>
       </c>
       <c r="B43" t="n">
-        <v>816</v>
+        <v>664</v>
       </c>
       <c r="C43" t="n">
         <v>8888</v>
       </c>
       <c r="D43" t="n">
-        <v>438.24</v>
+        <v>1595.68</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1262,17 +1262,17 @@
         <v>46218</v>
       </c>
       <c r="B44" t="n">
-        <v>953</v>
+        <v>816</v>
       </c>
       <c r="C44" t="n">
         <v>8888</v>
       </c>
       <c r="D44" t="n">
-        <v>2618.89</v>
+        <v>438.24</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1281,13 +1281,13 @@
         <v>46218</v>
       </c>
       <c r="B45" t="n">
-        <v>1465</v>
+        <v>953</v>
       </c>
       <c r="C45" t="n">
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>3504</v>
+        <v>2618.89</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1300,17 +1300,17 @@
         <v>46218</v>
       </c>
       <c r="B46" t="n">
-        <v>2245</v>
+        <v>1465</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>427.51</v>
+        <v>3504</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1319,17 +1319,17 @@
         <v>46218</v>
       </c>
       <c r="B47" t="n">
-        <v>131</v>
+        <v>2245</v>
       </c>
       <c r="C47" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D47" t="n">
-        <v>91.86</v>
+        <v>427.51</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1338,13 +1338,13 @@
         <v>46218</v>
       </c>
       <c r="B48" t="n">
-        <v>451</v>
+        <v>131</v>
       </c>
       <c r="C48" t="n">
-        <v>3403</v>
+        <v>27</v>
       </c>
       <c r="D48" t="n">
-        <v>445.58</v>
+        <v>91.86</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1357,17 +1357,17 @@
         <v>46218</v>
       </c>
       <c r="B49" t="n">
-        <v>2114</v>
+        <v>451</v>
       </c>
       <c r="C49" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D49" t="n">
-        <v>641.92</v>
+        <v>445.58</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1376,13 +1376,13 @@
         <v>46218</v>
       </c>
       <c r="B50" t="n">
-        <v>2782</v>
+        <v>2114</v>
       </c>
       <c r="C50" t="n">
         <v>8888</v>
       </c>
       <c r="D50" t="n">
-        <v>1786.32</v>
+        <v>641.92</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1395,17 +1395,17 @@
         <v>46218</v>
       </c>
       <c r="B51" t="n">
-        <v>1478</v>
+        <v>2782</v>
       </c>
       <c r="C51" t="n">
         <v>8888</v>
       </c>
       <c r="D51" t="n">
-        <v>459.57</v>
+        <v>1786.32</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1414,13 +1414,13 @@
         <v>46218</v>
       </c>
       <c r="B52" t="n">
-        <v>131</v>
+        <v>1478</v>
       </c>
       <c r="C52" t="n">
         <v>8888</v>
       </c>
       <c r="D52" t="n">
-        <v>1125.63</v>
+        <v>459.57</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1433,17 +1433,17 @@
         <v>46218</v>
       </c>
       <c r="B53" t="n">
-        <v>2015</v>
+        <v>131</v>
       </c>
       <c r="C53" t="n">
         <v>8888</v>
       </c>
       <c r="D53" t="n">
-        <v>2599.69</v>
+        <v>1125.63</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1452,17 +1452,17 @@
         <v>46218</v>
       </c>
       <c r="B54" t="n">
-        <v>1116</v>
+        <v>2015</v>
       </c>
       <c r="C54" t="n">
         <v>8888</v>
       </c>
       <c r="D54" t="n">
-        <v>2919.53</v>
+        <v>2599.69</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1471,13 +1471,13 @@
         <v>46218</v>
       </c>
       <c r="B55" t="n">
-        <v>42</v>
+        <v>1116</v>
       </c>
       <c r="C55" t="n">
         <v>8888</v>
       </c>
       <c r="D55" t="n">
-        <v>79947.14999999999</v>
+        <v>2919.53</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1490,15 +1490,34 @@
         <v>46218</v>
       </c>
       <c r="B56" t="n">
+        <v>42</v>
+      </c>
+      <c r="C56" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D56" t="n">
+        <v>79947.14999999999</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B57" t="n">
         <v>2109</v>
       </c>
-      <c r="C56" t="n">
-        <v>8888</v>
-      </c>
-      <c r="D56" t="n">
+      <c r="C57" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D57" t="n">
         <v>788.98</v>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>FORÇA DE VENDAS</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 14:30:07
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:E137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,17 +483,17 @@
         <v>46218</v>
       </c>
       <c r="B3" t="n">
-        <v>1364</v>
+        <v>664</v>
       </c>
       <c r="C3" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D3" t="n">
-        <v>1300.54</v>
+        <v>463.88</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -502,17 +502,17 @@
         <v>46218</v>
       </c>
       <c r="B4" t="n">
-        <v>451</v>
+        <v>1364</v>
       </c>
       <c r="C4" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D4" t="n">
-        <v>1103.58</v>
+        <v>1300.54</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -521,17 +521,17 @@
         <v>46218</v>
       </c>
       <c r="B5" t="n">
-        <v>131</v>
+        <v>451</v>
       </c>
       <c r="C5" t="n">
         <v>8888</v>
       </c>
       <c r="D5" t="n">
-        <v>1469.86</v>
+        <v>1103.58</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -540,17 +540,17 @@
         <v>46218</v>
       </c>
       <c r="B6" t="n">
-        <v>2651</v>
+        <v>131</v>
       </c>
       <c r="C6" t="n">
         <v>8888</v>
       </c>
       <c r="D6" t="n">
-        <v>660.95</v>
+        <v>1469.86</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -559,13 +559,13 @@
         <v>46218</v>
       </c>
       <c r="B7" t="n">
-        <v>2118</v>
+        <v>2211</v>
       </c>
       <c r="C7" t="n">
         <v>8888</v>
       </c>
       <c r="D7" t="n">
-        <v>452.46</v>
+        <v>2190.93</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -578,17 +578,17 @@
         <v>46218</v>
       </c>
       <c r="B8" t="n">
-        <v>949</v>
+        <v>2660</v>
       </c>
       <c r="C8" t="n">
-        <v>1134</v>
+        <v>8888</v>
       </c>
       <c r="D8" t="n">
-        <v>30.46</v>
+        <v>875.61</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -597,13 +597,13 @@
         <v>46218</v>
       </c>
       <c r="B9" t="n">
-        <v>2499</v>
+        <v>2651</v>
       </c>
       <c r="C9" t="n">
         <v>8888</v>
       </c>
       <c r="D9" t="n">
-        <v>261.63</v>
+        <v>660.95</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -616,13 +616,13 @@
         <v>46218</v>
       </c>
       <c r="B10" t="n">
-        <v>58</v>
+        <v>2197</v>
       </c>
       <c r="C10" t="n">
         <v>8888</v>
       </c>
       <c r="D10" t="n">
-        <v>499.11</v>
+        <v>892.66</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -635,17 +635,17 @@
         <v>46218</v>
       </c>
       <c r="B11" t="n">
-        <v>2245</v>
+        <v>609</v>
       </c>
       <c r="C11" t="n">
-        <v>8888</v>
+        <v>3179</v>
       </c>
       <c r="D11" t="n">
-        <v>2433.47</v>
+        <v>1611.48</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -654,13 +654,13 @@
         <v>46218</v>
       </c>
       <c r="B12" t="n">
-        <v>2383</v>
+        <v>2118</v>
       </c>
       <c r="C12" t="n">
         <v>8888</v>
       </c>
       <c r="D12" t="n">
-        <v>6204.03</v>
+        <v>452.46</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -673,13 +673,13 @@
         <v>46218</v>
       </c>
       <c r="B13" t="n">
-        <v>1117</v>
+        <v>931</v>
       </c>
       <c r="C13" t="n">
-        <v>1139</v>
+        <v>423</v>
       </c>
       <c r="D13" t="n">
-        <v>916.72</v>
+        <v>492.34</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -692,17 +692,17 @@
         <v>46218</v>
       </c>
       <c r="B14" t="n">
-        <v>2279</v>
+        <v>525</v>
       </c>
       <c r="C14" t="n">
         <v>8888</v>
       </c>
       <c r="D14" t="n">
-        <v>712.66</v>
+        <v>408.25</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -711,17 +711,17 @@
         <v>46218</v>
       </c>
       <c r="B15" t="n">
-        <v>535</v>
+        <v>1808</v>
       </c>
       <c r="C15" t="n">
         <v>8888</v>
       </c>
       <c r="D15" t="n">
-        <v>2144.17</v>
+        <v>695.3200000000001</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -730,17 +730,17 @@
         <v>46218</v>
       </c>
       <c r="B16" t="n">
-        <v>535</v>
+        <v>949</v>
       </c>
       <c r="C16" t="n">
-        <v>8888</v>
+        <v>1134</v>
       </c>
       <c r="D16" t="n">
-        <v>1056.19</v>
+        <v>30.46</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -749,17 +749,17 @@
         <v>46218</v>
       </c>
       <c r="B17" t="n">
-        <v>438</v>
+        <v>2499</v>
       </c>
       <c r="C17" t="n">
         <v>8888</v>
       </c>
       <c r="D17" t="n">
-        <v>220.06</v>
+        <v>261.63</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
         <v>46218</v>
       </c>
       <c r="B18" t="n">
-        <v>1293</v>
+        <v>58</v>
       </c>
       <c r="C18" t="n">
         <v>8888</v>
       </c>
       <c r="D18" t="n">
-        <v>1388.12</v>
+        <v>499.11</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -787,17 +787,17 @@
         <v>46218</v>
       </c>
       <c r="B19" t="n">
-        <v>2279</v>
+        <v>2245</v>
       </c>
       <c r="C19" t="n">
         <v>8888</v>
       </c>
       <c r="D19" t="n">
-        <v>2753.96</v>
+        <v>2740.06</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -806,17 +806,17 @@
         <v>46218</v>
       </c>
       <c r="B20" t="n">
-        <v>1137</v>
+        <v>2383</v>
       </c>
       <c r="C20" t="n">
         <v>8888</v>
       </c>
       <c r="D20" t="n">
-        <v>952.95</v>
+        <v>7926.02</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -825,17 +825,17 @@
         <v>46218</v>
       </c>
       <c r="B21" t="n">
-        <v>325</v>
+        <v>1117</v>
       </c>
       <c r="C21" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D21" t="n">
-        <v>57.46</v>
+        <v>916.72</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -844,17 +844,17 @@
         <v>46218</v>
       </c>
       <c r="B22" t="n">
-        <v>451</v>
+        <v>2279</v>
       </c>
       <c r="C22" t="n">
         <v>8888</v>
       </c>
       <c r="D22" t="n">
-        <v>368.93</v>
+        <v>712.66</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -863,17 +863,17 @@
         <v>46218</v>
       </c>
       <c r="B23" t="n">
-        <v>2714</v>
+        <v>535</v>
       </c>
       <c r="C23" t="n">
-        <v>519</v>
+        <v>8888</v>
       </c>
       <c r="D23" t="n">
-        <v>61939.22</v>
+        <v>3228.46</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -882,17 +882,17 @@
         <v>46218</v>
       </c>
       <c r="B24" t="n">
-        <v>483</v>
+        <v>535</v>
       </c>
       <c r="C24" t="n">
         <v>8888</v>
       </c>
       <c r="D24" t="n">
-        <v>2532.06</v>
+        <v>1352.51</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -901,17 +901,17 @@
         <v>46218</v>
       </c>
       <c r="B25" t="n">
-        <v>1075</v>
+        <v>2678</v>
       </c>
       <c r="C25" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D25" t="n">
-        <v>11607.79</v>
+        <v>364.96</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
         <v>46218</v>
       </c>
       <c r="B26" t="n">
-        <v>629</v>
+        <v>438</v>
       </c>
       <c r="C26" t="n">
         <v>8888</v>
       </c>
       <c r="D26" t="n">
-        <v>4569.78</v>
+        <v>220.06</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -939,17 +939,17 @@
         <v>46218</v>
       </c>
       <c r="B27" t="n">
-        <v>1983</v>
+        <v>1293</v>
       </c>
       <c r="C27" t="n">
-        <v>841</v>
+        <v>8888</v>
       </c>
       <c r="D27" t="n">
-        <v>105.6</v>
+        <v>1388.12</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -958,17 +958,17 @@
         <v>46218</v>
       </c>
       <c r="B28" t="n">
-        <v>2651</v>
+        <v>2279</v>
       </c>
       <c r="C28" t="n">
         <v>8888</v>
       </c>
       <c r="D28" t="n">
-        <v>1296.58</v>
+        <v>2753.96</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -977,17 +977,17 @@
         <v>46218</v>
       </c>
       <c r="B29" t="n">
-        <v>89</v>
+        <v>1137</v>
       </c>
       <c r="C29" t="n">
-        <v>13148</v>
+        <v>8888</v>
       </c>
       <c r="D29" t="n">
-        <v>1883.74</v>
+        <v>952.95</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -996,17 +996,17 @@
         <v>46218</v>
       </c>
       <c r="B30" t="n">
-        <v>2211</v>
+        <v>325</v>
       </c>
       <c r="C30" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D30" t="n">
-        <v>1526.94</v>
+        <v>399.62</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1015,17 +1015,17 @@
         <v>46218</v>
       </c>
       <c r="B31" t="n">
-        <v>559</v>
+        <v>664</v>
       </c>
       <c r="C31" t="n">
         <v>8888</v>
       </c>
       <c r="D31" t="n">
-        <v>859.92</v>
+        <v>682.3200000000001</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1034,17 +1034,17 @@
         <v>46218</v>
       </c>
       <c r="B32" t="n">
-        <v>1063</v>
+        <v>945</v>
       </c>
       <c r="C32" t="n">
         <v>8888</v>
       </c>
       <c r="D32" t="n">
-        <v>4487.11</v>
+        <v>365.11</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>PEDIDO ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -1053,17 +1053,17 @@
         <v>46218</v>
       </c>
       <c r="B33" t="n">
-        <v>2279</v>
+        <v>451</v>
       </c>
       <c r="C33" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D33" t="n">
-        <v>652.51</v>
+        <v>368.93</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1072,17 +1072,17 @@
         <v>46218</v>
       </c>
       <c r="B34" t="n">
-        <v>1299</v>
+        <v>1756</v>
       </c>
       <c r="C34" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D34" t="n">
-        <v>990.24</v>
+        <v>824.3200000000001</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1091,17 +1091,17 @@
         <v>46218</v>
       </c>
       <c r="B35" t="n">
-        <v>285</v>
+        <v>2631</v>
       </c>
       <c r="C35" t="n">
-        <v>8888</v>
+        <v>2853</v>
       </c>
       <c r="D35" t="n">
-        <v>3349.8</v>
+        <v>509.88</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1110,17 @@
         <v>46218</v>
       </c>
       <c r="B36" t="n">
-        <v>1983</v>
+        <v>2714</v>
       </c>
       <c r="C36" t="n">
-        <v>8888</v>
+        <v>519</v>
       </c>
       <c r="D36" t="n">
-        <v>2451.28</v>
+        <v>61939.22</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1129,17 @@
         <v>46218</v>
       </c>
       <c r="B37" t="n">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="C37" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D37" t="n">
-        <v>1540.55</v>
+        <v>4920.11</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1148,13 +1148,13 @@
         <v>46218</v>
       </c>
       <c r="B38" t="n">
-        <v>1063</v>
+        <v>1075</v>
       </c>
       <c r="C38" t="n">
         <v>8888</v>
       </c>
       <c r="D38" t="n">
-        <v>2549.86</v>
+        <v>11607.79</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1167,13 +1167,13 @@
         <v>46218</v>
       </c>
       <c r="B39" t="n">
-        <v>424</v>
+        <v>629</v>
       </c>
       <c r="C39" t="n">
         <v>8888</v>
       </c>
       <c r="D39" t="n">
-        <v>1035.17</v>
+        <v>9233.719999999999</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1186,17 +1186,17 @@
         <v>46218</v>
       </c>
       <c r="B40" t="n">
-        <v>675</v>
+        <v>1983</v>
       </c>
       <c r="C40" t="n">
-        <v>8888</v>
+        <v>841</v>
       </c>
       <c r="D40" t="n">
-        <v>616.73</v>
+        <v>105.6</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1205,17 +1205,17 @@
         <v>46218</v>
       </c>
       <c r="B41" t="n">
-        <v>1993</v>
+        <v>1137</v>
       </c>
       <c r="C41" t="n">
         <v>8888</v>
       </c>
       <c r="D41" t="n">
-        <v>362.63</v>
+        <v>3578.51</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1224,17 +1224,17 @@
         <v>46218</v>
       </c>
       <c r="B42" t="n">
-        <v>1465</v>
+        <v>2651</v>
       </c>
       <c r="C42" t="n">
         <v>8888</v>
       </c>
       <c r="D42" t="n">
-        <v>2431.47</v>
+        <v>1296.58</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1243,17 +1243,17 @@
         <v>46218</v>
       </c>
       <c r="B43" t="n">
-        <v>89</v>
+        <v>2709</v>
       </c>
       <c r="C43" t="n">
         <v>8888</v>
       </c>
       <c r="D43" t="n">
-        <v>479</v>
+        <v>547.6900000000001</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1262,13 +1262,13 @@
         <v>46218</v>
       </c>
       <c r="B44" t="n">
-        <v>1465</v>
+        <v>89</v>
       </c>
       <c r="C44" t="n">
-        <v>3403</v>
+        <v>13148</v>
       </c>
       <c r="D44" t="n">
-        <v>777.2</v>
+        <v>1883.74</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1281,17 +1281,17 @@
         <v>46218</v>
       </c>
       <c r="B45" t="n">
-        <v>1937</v>
+        <v>2709</v>
       </c>
       <c r="C45" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D45" t="n">
-        <v>833.52</v>
+        <v>390.19</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1300,13 +1300,13 @@
         <v>46218</v>
       </c>
       <c r="B46" t="n">
-        <v>360</v>
+        <v>2345</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>731.37</v>
+        <v>748.86</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1319,17 +1319,17 @@
         <v>46218</v>
       </c>
       <c r="B47" t="n">
-        <v>1063</v>
+        <v>1308</v>
       </c>
       <c r="C47" t="n">
         <v>8888</v>
       </c>
       <c r="D47" t="n">
-        <v>1113.08</v>
+        <v>276.16</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1338,17 +1338,17 @@
         <v>46218</v>
       </c>
       <c r="B48" t="n">
-        <v>1293</v>
+        <v>2211</v>
       </c>
       <c r="C48" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D48" t="n">
-        <v>386.33</v>
+        <v>1526.94</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1357,17 +1357,17 @@
         <v>46218</v>
       </c>
       <c r="B49" t="n">
-        <v>2089</v>
+        <v>559</v>
       </c>
       <c r="C49" t="n">
-        <v>1533</v>
+        <v>8888</v>
       </c>
       <c r="D49" t="n">
-        <v>442.44</v>
+        <v>859.92</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1376,13 +1376,13 @@
         <v>46218</v>
       </c>
       <c r="B50" t="n">
-        <v>1007</v>
+        <v>1063</v>
       </c>
       <c r="C50" t="n">
         <v>8888</v>
       </c>
       <c r="D50" t="n">
-        <v>241.44</v>
+        <v>4487.11</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1395,17 +1395,17 @@
         <v>46218</v>
       </c>
       <c r="B51" t="n">
-        <v>1380</v>
+        <v>2279</v>
       </c>
       <c r="C51" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D51" t="n">
-        <v>520.2</v>
+        <v>652.51</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
         <v>46218</v>
       </c>
       <c r="B52" t="n">
-        <v>1102</v>
+        <v>1299</v>
       </c>
       <c r="C52" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D52" t="n">
-        <v>349.4</v>
+        <v>1435.52</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1433,17 +1433,17 @@
         <v>46218</v>
       </c>
       <c r="B53" t="n">
-        <v>1075</v>
+        <v>1478</v>
       </c>
       <c r="C53" t="n">
-        <v>8888</v>
+        <v>675</v>
       </c>
       <c r="D53" t="n">
-        <v>2179.03</v>
+        <v>511.84</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1452,17 +1452,17 @@
         <v>46218</v>
       </c>
       <c r="B54" t="n">
-        <v>2245</v>
+        <v>285</v>
       </c>
       <c r="C54" t="n">
         <v>8888</v>
       </c>
       <c r="D54" t="n">
-        <v>361.58</v>
+        <v>3349.8</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1471,17 +1471,17 @@
         <v>46218</v>
       </c>
       <c r="B55" t="n">
-        <v>452</v>
+        <v>1983</v>
       </c>
       <c r="C55" t="n">
         <v>8888</v>
       </c>
       <c r="D55" t="n">
-        <v>608.78</v>
+        <v>2451.28</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1490,17 +1490,17 @@
         <v>46218</v>
       </c>
       <c r="B56" t="n">
-        <v>285</v>
+        <v>477</v>
       </c>
       <c r="C56" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D56" t="n">
-        <v>2090.81</v>
+        <v>1540.55</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1509,17 +1509,17 @@
         <v>46218</v>
       </c>
       <c r="B57" t="n">
-        <v>1102</v>
+        <v>1063</v>
       </c>
       <c r="C57" t="n">
         <v>8888</v>
       </c>
       <c r="D57" t="n">
-        <v>1119.32</v>
+        <v>2549.86</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1528,13 +1528,13 @@
         <v>46218</v>
       </c>
       <c r="B58" t="n">
-        <v>626</v>
+        <v>424</v>
       </c>
       <c r="C58" t="n">
         <v>8888</v>
       </c>
       <c r="D58" t="n">
-        <v>3520.98</v>
+        <v>1035.17</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1547,17 +1547,17 @@
         <v>46218</v>
       </c>
       <c r="B59" t="n">
-        <v>1756</v>
+        <v>675</v>
       </c>
       <c r="C59" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D59" t="n">
-        <v>741.1799999999999</v>
+        <v>616.73</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1566,17 +1566,17 @@
         <v>46218</v>
       </c>
       <c r="B60" t="n">
-        <v>2651</v>
+        <v>1993</v>
       </c>
       <c r="C60" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D60" t="n">
-        <v>363.7</v>
+        <v>362.63</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1585,13 +1585,13 @@
         <v>46218</v>
       </c>
       <c r="B61" t="n">
-        <v>1064</v>
+        <v>1465</v>
       </c>
       <c r="C61" t="n">
         <v>8888</v>
       </c>
       <c r="D61" t="n">
-        <v>1274.3</v>
+        <v>3373.83</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1604,17 +1604,17 @@
         <v>46218</v>
       </c>
       <c r="B62" t="n">
-        <v>2698</v>
+        <v>89</v>
       </c>
       <c r="C62" t="n">
         <v>8888</v>
       </c>
       <c r="D62" t="n">
-        <v>552.15</v>
+        <v>479</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1623,17 +1623,17 @@
         <v>46218</v>
       </c>
       <c r="B63" t="n">
-        <v>629</v>
+        <v>2696</v>
       </c>
       <c r="C63" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D63" t="n">
-        <v>721.25</v>
+        <v>259.97</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1642,17 +1642,17 @@
         <v>46218</v>
       </c>
       <c r="B64" t="n">
-        <v>664</v>
+        <v>360</v>
       </c>
       <c r="C64" t="n">
         <v>8888</v>
       </c>
       <c r="D64" t="n">
-        <v>1595.68</v>
+        <v>2023.17</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1661,17 +1661,17 @@
         <v>46218</v>
       </c>
       <c r="B65" t="n">
-        <v>816</v>
+        <v>1465</v>
       </c>
       <c r="C65" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D65" t="n">
-        <v>438.24</v>
+        <v>777.2</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1680,17 +1680,17 @@
         <v>46218</v>
       </c>
       <c r="B66" t="n">
-        <v>285</v>
+        <v>1937</v>
       </c>
       <c r="C66" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D66" t="n">
-        <v>364.99</v>
+        <v>833.52</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1699,17 +1699,17 @@
         <v>46218</v>
       </c>
       <c r="B67" t="n">
-        <v>2114</v>
+        <v>1293</v>
       </c>
       <c r="C67" t="n">
         <v>8888</v>
       </c>
       <c r="D67" t="n">
-        <v>1682.3</v>
+        <v>1607.2</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1718,17 +1718,17 @@
         <v>46218</v>
       </c>
       <c r="B68" t="n">
-        <v>953</v>
+        <v>630</v>
       </c>
       <c r="C68" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D68" t="n">
-        <v>2618.89</v>
+        <v>1210.85</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1737,17 +1737,17 @@
         <v>46218</v>
       </c>
       <c r="B69" t="n">
-        <v>1102</v>
+        <v>2571</v>
       </c>
       <c r="C69" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D69" t="n">
-        <v>1771.61</v>
+        <v>268.53</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1756,17 +1756,17 @@
         <v>46218</v>
       </c>
       <c r="B70" t="n">
-        <v>619</v>
+        <v>1063</v>
       </c>
       <c r="C70" t="n">
         <v>8888</v>
       </c>
       <c r="D70" t="n">
-        <v>2021.67</v>
+        <v>1113.08</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1775,17 @@
         <v>46218</v>
       </c>
       <c r="B71" t="n">
-        <v>1465</v>
+        <v>1756</v>
       </c>
       <c r="C71" t="n">
         <v>8888</v>
       </c>
       <c r="D71" t="n">
-        <v>3504</v>
+        <v>1357.12</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1794,17 +1794,17 @@
         <v>46218</v>
       </c>
       <c r="B72" t="n">
-        <v>2767</v>
+        <v>569</v>
       </c>
       <c r="C72" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D72" t="n">
-        <v>466.12</v>
+        <v>4504.72</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1813,17 +1813,17 @@
         <v>46218</v>
       </c>
       <c r="B73" t="n">
-        <v>2245</v>
+        <v>2089</v>
       </c>
       <c r="C73" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D73" t="n">
-        <v>427.51</v>
+        <v>442.44</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1832,17 +1832,17 @@
         <v>46218</v>
       </c>
       <c r="B74" t="n">
-        <v>131</v>
+        <v>1007</v>
       </c>
       <c r="C74" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D74" t="n">
-        <v>299.37</v>
+        <v>241.44</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1851,13 +1851,13 @@
         <v>46218</v>
       </c>
       <c r="B75" t="n">
-        <v>1993</v>
+        <v>1380</v>
       </c>
       <c r="C75" t="n">
         <v>8888</v>
       </c>
       <c r="D75" t="n">
-        <v>1864.73</v>
+        <v>520.2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -1870,17 +1870,17 @@
         <v>46218</v>
       </c>
       <c r="B76" t="n">
-        <v>451</v>
+        <v>1102</v>
       </c>
       <c r="C76" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D76" t="n">
-        <v>445.58</v>
+        <v>1137.04</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1889,17 +1889,17 @@
         <v>46218</v>
       </c>
       <c r="B77" t="n">
-        <v>2749</v>
+        <v>1075</v>
       </c>
       <c r="C77" t="n">
         <v>8888</v>
       </c>
       <c r="D77" t="n">
-        <v>1860.64</v>
+        <v>2179.03</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1908,13 +1908,13 @@
         <v>46218</v>
       </c>
       <c r="B78" t="n">
-        <v>1117</v>
+        <v>2245</v>
       </c>
       <c r="C78" t="n">
         <v>8888</v>
       </c>
       <c r="D78" t="n">
-        <v>342.2</v>
+        <v>361.58</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -1927,17 +1927,17 @@
         <v>46218</v>
       </c>
       <c r="B79" t="n">
-        <v>2491</v>
+        <v>2660</v>
       </c>
       <c r="C79" t="n">
         <v>8888</v>
       </c>
       <c r="D79" t="n">
-        <v>650.4299999999999</v>
+        <v>528.4299999999999</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1946,13 +1946,13 @@
         <v>46218</v>
       </c>
       <c r="B80" t="n">
-        <v>2782</v>
+        <v>452</v>
       </c>
       <c r="C80" t="n">
         <v>8888</v>
       </c>
       <c r="D80" t="n">
-        <v>1786.32</v>
+        <v>608.78</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -1965,13 +1965,13 @@
         <v>46218</v>
       </c>
       <c r="B81" t="n">
-        <v>483</v>
+        <v>1293</v>
       </c>
       <c r="C81" t="n">
-        <v>841</v>
+        <v>1281</v>
       </c>
       <c r="D81" t="n">
-        <v>1393.15</v>
+        <v>1780.93</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -1984,17 +1984,17 @@
         <v>46218</v>
       </c>
       <c r="B82" t="n">
-        <v>1478</v>
+        <v>525</v>
       </c>
       <c r="C82" t="n">
         <v>8888</v>
       </c>
       <c r="D82" t="n">
-        <v>459.57</v>
+        <v>4599.72</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2003,13 +2003,13 @@
         <v>46218</v>
       </c>
       <c r="B83" t="n">
-        <v>131</v>
+        <v>609</v>
       </c>
       <c r="C83" t="n">
         <v>8888</v>
       </c>
       <c r="D83" t="n">
-        <v>1369.91</v>
+        <v>886.1</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2022,17 +2022,17 @@
         <v>46218</v>
       </c>
       <c r="B84" t="n">
-        <v>2015</v>
+        <v>619</v>
       </c>
       <c r="C84" t="n">
         <v>8888</v>
       </c>
       <c r="D84" t="n">
-        <v>2599.69</v>
+        <v>2330.47</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2041,17 +2041,17 @@
         <v>46218</v>
       </c>
       <c r="B85" t="n">
-        <v>2109</v>
+        <v>285</v>
       </c>
       <c r="C85" t="n">
         <v>8888</v>
       </c>
       <c r="D85" t="n">
-        <v>2293.78</v>
+        <v>2090.81</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2060,17 +2060,17 @@
         <v>46218</v>
       </c>
       <c r="B86" t="n">
-        <v>1116</v>
+        <v>1102</v>
       </c>
       <c r="C86" t="n">
         <v>8888</v>
       </c>
       <c r="D86" t="n">
-        <v>2919.53</v>
+        <v>1119.32</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2079,17 +2079,17 @@
         <v>46218</v>
       </c>
       <c r="B87" t="n">
-        <v>2250</v>
+        <v>626</v>
       </c>
       <c r="C87" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D87" t="n">
-        <v>1573.32</v>
+        <v>5211.29</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2098,17 +2098,17 @@
         <v>46218</v>
       </c>
       <c r="B88" t="n">
-        <v>42</v>
+        <v>1137</v>
       </c>
       <c r="C88" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D88" t="n">
-        <v>79947.14999999999</v>
+        <v>1370.86</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2117,17 +2117,17 @@
         <v>46218</v>
       </c>
       <c r="B89" t="n">
-        <v>1993</v>
+        <v>1756</v>
       </c>
       <c r="C89" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D89" t="n">
-        <v>456.62</v>
+        <v>5078.1</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2136,15 +2136,908 @@
         <v>46218</v>
       </c>
       <c r="B90" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C90" t="n">
+        <v>58</v>
+      </c>
+      <c r="D90" t="n">
+        <v>363.7</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B91" t="n">
+        <v>360</v>
+      </c>
+      <c r="C91" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D91" t="n">
+        <v>1594.84</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B92" t="n">
+        <v>2582</v>
+      </c>
+      <c r="C92" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D92" t="n">
+        <v>379.33</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B93" t="n">
+        <v>1756</v>
+      </c>
+      <c r="C93" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D93" t="n">
+        <v>1715.26</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B94" t="n">
+        <v>1289</v>
+      </c>
+      <c r="C94" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D94" t="n">
+        <v>2396.98</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B95" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C95" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D95" t="n">
+        <v>315.69</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B96" t="n">
+        <v>1064</v>
+      </c>
+      <c r="C96" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D96" t="n">
+        <v>1274.3</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B97" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C97" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D97" t="n">
+        <v>552.15</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B98" t="n">
         <v>629</v>
       </c>
-      <c r="C90" t="n">
+      <c r="C98" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D98" t="n">
+        <v>721.25</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B99" t="n">
+        <v>2686</v>
+      </c>
+      <c r="C99" t="n">
+        <v>1929</v>
+      </c>
+      <c r="D99" t="n">
+        <v>521.79</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B100" t="n">
+        <v>2584</v>
+      </c>
+      <c r="C100" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D100" t="n">
+        <v>1852.83</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B101" t="n">
+        <v>2641</v>
+      </c>
+      <c r="C101" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D101" t="n">
+        <v>820</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B102" t="n">
+        <v>664</v>
+      </c>
+      <c r="C102" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D102" t="n">
+        <v>1595.68</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B103" t="n">
+        <v>816</v>
+      </c>
+      <c r="C103" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D103" t="n">
+        <v>438.24</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B104" t="n">
+        <v>285</v>
+      </c>
+      <c r="C104" t="n">
+        <v>58</v>
+      </c>
+      <c r="D104" t="n">
+        <v>364.99</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B105" t="n">
+        <v>2114</v>
+      </c>
+      <c r="C105" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D105" t="n">
+        <v>1682.3</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B106" t="n">
+        <v>953</v>
+      </c>
+      <c r="C106" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D106" t="n">
+        <v>2618.89</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B107" t="n">
+        <v>1102</v>
+      </c>
+      <c r="C107" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D107" t="n">
+        <v>2344.41</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B108" t="n">
+        <v>619</v>
+      </c>
+      <c r="C108" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D108" t="n">
+        <v>2021.67</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B109" t="n">
+        <v>1465</v>
+      </c>
+      <c r="C109" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D109" t="n">
+        <v>3504</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B110" t="n">
+        <v>2767</v>
+      </c>
+      <c r="C110" t="n">
+        <v>1898</v>
+      </c>
+      <c r="D110" t="n">
+        <v>466.12</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B111" t="n">
+        <v>2245</v>
+      </c>
+      <c r="C111" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D111" t="n">
+        <v>427.51</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B112" t="n">
+        <v>2657</v>
+      </c>
+      <c r="C112" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D112" t="n">
+        <v>703.6799999999999</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B113" t="n">
+        <v>131</v>
+      </c>
+      <c r="C113" t="n">
+        <v>27</v>
+      </c>
+      <c r="D113" t="n">
+        <v>299.37</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B114" t="n">
+        <v>2692</v>
+      </c>
+      <c r="C114" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D114" t="n">
+        <v>731.28</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B115" t="n">
+        <v>1317</v>
+      </c>
+      <c r="C115" t="n">
+        <v>3179</v>
+      </c>
+      <c r="D115" t="n">
+        <v>991.6799999999999</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B116" t="n">
+        <v>1993</v>
+      </c>
+      <c r="C116" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D116" t="n">
+        <v>2875.39</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B117" t="n">
+        <v>1632</v>
+      </c>
+      <c r="C117" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D117" t="n">
+        <v>564.55</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B118" t="n">
+        <v>1890</v>
+      </c>
+      <c r="C118" t="n">
+        <v>3449</v>
+      </c>
+      <c r="D118" t="n">
+        <v>3063.24</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B119" t="n">
+        <v>451</v>
+      </c>
+      <c r="C119" t="n">
+        <v>3403</v>
+      </c>
+      <c r="D119" t="n">
+        <v>445.58</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B120" t="n">
+        <v>2749</v>
+      </c>
+      <c r="C120" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D120" t="n">
+        <v>1860.64</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B121" t="n">
+        <v>1117</v>
+      </c>
+      <c r="C121" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D121" t="n">
+        <v>342.2</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B122" t="n">
+        <v>1478</v>
+      </c>
+      <c r="C122" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D122" t="n">
+        <v>875.34</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B123" t="n">
+        <v>2491</v>
+      </c>
+      <c r="C123" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D123" t="n">
+        <v>650.4299999999999</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B124" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C124" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D124" t="n">
+        <v>4436.15</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B125" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C125" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D125" t="n">
+        <v>1786.32</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B126" t="n">
+        <v>483</v>
+      </c>
+      <c r="C126" t="n">
+        <v>841</v>
+      </c>
+      <c r="D126" t="n">
+        <v>1393.15</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B127" t="n">
+        <v>2648</v>
+      </c>
+      <c r="C127" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D127" t="n">
+        <v>1873.52</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B128" t="n">
+        <v>131</v>
+      </c>
+      <c r="C128" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D128" t="n">
+        <v>1369.91</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B129" t="n">
+        <v>2109</v>
+      </c>
+      <c r="C129" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D129" t="n">
+        <v>2293.78</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B130" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C130" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D130" t="n">
+        <v>2919.53</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B131" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C131" t="n">
+        <v>27</v>
+      </c>
+      <c r="D131" t="n">
+        <v>1573.32</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B132" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C132" t="n">
+        <v>874</v>
+      </c>
+      <c r="D132" t="n">
+        <v>1230.43</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B133" t="n">
+        <v>42</v>
+      </c>
+      <c r="C133" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D133" t="n">
+        <v>79947.14999999999</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B134" t="n">
+        <v>2716</v>
+      </c>
+      <c r="C134" t="n">
+        <v>1929</v>
+      </c>
+      <c r="D134" t="n">
+        <v>750.4299999999999</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B135" t="n">
+        <v>2716</v>
+      </c>
+      <c r="C135" t="n">
+        <v>977</v>
+      </c>
+      <c r="D135" t="n">
+        <v>729.29</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B136" t="n">
+        <v>1993</v>
+      </c>
+      <c r="C136" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D136" t="n">
+        <v>456.62</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B137" t="n">
+        <v>629</v>
+      </c>
+      <c r="C137" t="n">
         <v>675</v>
       </c>
-      <c r="D90" t="n">
+      <c r="D137" t="n">
         <v>1054.76</v>
       </c>
-      <c r="E90" t="inlineStr">
+      <c r="E137" t="inlineStr">
         <is>
           <t>TELEMARKETING</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 15:00:04
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E137"/>
+  <dimension ref="A1:E189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,17 +464,17 @@
         <v>46218</v>
       </c>
       <c r="B2" t="n">
-        <v>1075</v>
+        <v>326</v>
       </c>
       <c r="C2" t="n">
-        <v>675</v>
+        <v>8888</v>
       </c>
       <c r="D2" t="n">
-        <v>638.4299999999999</v>
+        <v>312.98</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -483,17 +483,17 @@
         <v>46218</v>
       </c>
       <c r="B3" t="n">
-        <v>664</v>
+        <v>1075</v>
       </c>
       <c r="C3" t="n">
-        <v>8888</v>
+        <v>675</v>
       </c>
       <c r="D3" t="n">
-        <v>463.88</v>
+        <v>638.4299999999999</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -502,17 +502,17 @@
         <v>46218</v>
       </c>
       <c r="B4" t="n">
-        <v>1364</v>
+        <v>664</v>
       </c>
       <c r="C4" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D4" t="n">
-        <v>1300.54</v>
+        <v>463.88</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -521,17 +521,17 @@
         <v>46218</v>
       </c>
       <c r="B5" t="n">
-        <v>451</v>
+        <v>1364</v>
       </c>
       <c r="C5" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D5" t="n">
-        <v>1103.58</v>
+        <v>1300.54</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -540,17 +540,17 @@
         <v>46218</v>
       </c>
       <c r="B6" t="n">
-        <v>131</v>
+        <v>451</v>
       </c>
       <c r="C6" t="n">
         <v>8888</v>
       </c>
       <c r="D6" t="n">
-        <v>1469.86</v>
+        <v>1103.58</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -559,13 +559,13 @@
         <v>46218</v>
       </c>
       <c r="B7" t="n">
-        <v>2211</v>
+        <v>131</v>
       </c>
       <c r="C7" t="n">
         <v>8888</v>
       </c>
       <c r="D7" t="n">
-        <v>2190.93</v>
+        <v>7071.12</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -578,17 +578,17 @@
         <v>46218</v>
       </c>
       <c r="B8" t="n">
-        <v>2660</v>
+        <v>2015</v>
       </c>
       <c r="C8" t="n">
-        <v>8888</v>
+        <v>2571</v>
       </c>
       <c r="D8" t="n">
-        <v>875.61</v>
+        <v>714.53</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -597,17 +597,17 @@
         <v>46218</v>
       </c>
       <c r="B9" t="n">
-        <v>2651</v>
+        <v>1289</v>
       </c>
       <c r="C9" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D9" t="n">
-        <v>660.95</v>
+        <v>727.05</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -616,17 +616,17 @@
         <v>46218</v>
       </c>
       <c r="B10" t="n">
-        <v>2197</v>
+        <v>609</v>
       </c>
       <c r="C10" t="n">
-        <v>8888</v>
+        <v>3179</v>
       </c>
       <c r="D10" t="n">
-        <v>892.66</v>
+        <v>2603.16</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -635,17 +635,17 @@
         <v>46218</v>
       </c>
       <c r="B11" t="n">
-        <v>609</v>
+        <v>2211</v>
       </c>
       <c r="C11" t="n">
-        <v>3179</v>
+        <v>8888</v>
       </c>
       <c r="D11" t="n">
-        <v>1611.48</v>
+        <v>2190.93</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -654,13 +654,13 @@
         <v>46218</v>
       </c>
       <c r="B12" t="n">
-        <v>2118</v>
+        <v>2660</v>
       </c>
       <c r="C12" t="n">
         <v>8888</v>
       </c>
       <c r="D12" t="n">
-        <v>452.46</v>
+        <v>875.61</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -673,17 +673,17 @@
         <v>46218</v>
       </c>
       <c r="B13" t="n">
-        <v>931</v>
+        <v>890</v>
       </c>
       <c r="C13" t="n">
-        <v>423</v>
+        <v>8888</v>
       </c>
       <c r="D13" t="n">
-        <v>492.34</v>
+        <v>1051.23</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -692,13 +692,13 @@
         <v>46218</v>
       </c>
       <c r="B14" t="n">
-        <v>525</v>
+        <v>2190</v>
       </c>
       <c r="C14" t="n">
         <v>8888</v>
       </c>
       <c r="D14" t="n">
-        <v>408.25</v>
+        <v>1307.13</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -711,17 +711,17 @@
         <v>46218</v>
       </c>
       <c r="B15" t="n">
-        <v>1808</v>
+        <v>2651</v>
       </c>
       <c r="C15" t="n">
         <v>8888</v>
       </c>
       <c r="D15" t="n">
-        <v>695.3200000000001</v>
+        <v>660.95</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -730,17 +730,17 @@
         <v>46218</v>
       </c>
       <c r="B16" t="n">
-        <v>949</v>
+        <v>2118</v>
       </c>
       <c r="C16" t="n">
-        <v>1134</v>
+        <v>8888</v>
       </c>
       <c r="D16" t="n">
-        <v>30.46</v>
+        <v>5535.71</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -749,13 +749,13 @@
         <v>46218</v>
       </c>
       <c r="B17" t="n">
-        <v>2499</v>
+        <v>2197</v>
       </c>
       <c r="C17" t="n">
         <v>8888</v>
       </c>
       <c r="D17" t="n">
-        <v>261.63</v>
+        <v>892.66</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -768,17 +768,17 @@
         <v>46218</v>
       </c>
       <c r="B18" t="n">
-        <v>58</v>
+        <v>1869</v>
       </c>
       <c r="C18" t="n">
         <v>8888</v>
       </c>
       <c r="D18" t="n">
-        <v>499.11</v>
+        <v>1263.2</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -787,17 +787,17 @@
         <v>46218</v>
       </c>
       <c r="B19" t="n">
-        <v>2245</v>
+        <v>2133</v>
       </c>
       <c r="C19" t="n">
-        <v>8888</v>
+        <v>691</v>
       </c>
       <c r="D19" t="n">
-        <v>2740.06</v>
+        <v>2058.93</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -806,17 +806,17 @@
         <v>46218</v>
       </c>
       <c r="B20" t="n">
-        <v>2383</v>
+        <v>452</v>
       </c>
       <c r="C20" t="n">
         <v>8888</v>
       </c>
       <c r="D20" t="n">
-        <v>7926.02</v>
+        <v>1832.74</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -825,17 +825,17 @@
         <v>46218</v>
       </c>
       <c r="B21" t="n">
-        <v>1117</v>
+        <v>2250</v>
       </c>
       <c r="C21" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D21" t="n">
-        <v>916.72</v>
+        <v>1686.37</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -844,17 +844,17 @@
         <v>46218</v>
       </c>
       <c r="B22" t="n">
-        <v>2279</v>
+        <v>931</v>
       </c>
       <c r="C22" t="n">
-        <v>8888</v>
+        <v>423</v>
       </c>
       <c r="D22" t="n">
-        <v>712.66</v>
+        <v>492.34</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -863,13 +863,13 @@
         <v>46218</v>
       </c>
       <c r="B23" t="n">
-        <v>535</v>
+        <v>951</v>
       </c>
       <c r="C23" t="n">
         <v>8888</v>
       </c>
       <c r="D23" t="n">
-        <v>3228.46</v>
+        <v>2171.08</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -882,13 +882,13 @@
         <v>46218</v>
       </c>
       <c r="B24" t="n">
-        <v>535</v>
+        <v>2695</v>
       </c>
       <c r="C24" t="n">
         <v>8888</v>
       </c>
       <c r="D24" t="n">
-        <v>1352.51</v>
+        <v>411.42</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -901,17 +901,17 @@
         <v>46218</v>
       </c>
       <c r="B25" t="n">
-        <v>2678</v>
+        <v>525</v>
       </c>
       <c r="C25" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D25" t="n">
-        <v>364.96</v>
+        <v>408.25</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
         <v>46218</v>
       </c>
       <c r="B26" t="n">
-        <v>438</v>
+        <v>1808</v>
       </c>
       <c r="C26" t="n">
         <v>8888</v>
       </c>
       <c r="D26" t="n">
-        <v>220.06</v>
+        <v>695.3200000000001</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -939,17 +939,17 @@
         <v>46218</v>
       </c>
       <c r="B27" t="n">
-        <v>1293</v>
+        <v>949</v>
       </c>
       <c r="C27" t="n">
-        <v>8888</v>
+        <v>1134</v>
       </c>
       <c r="D27" t="n">
-        <v>1388.12</v>
+        <v>30.46</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -958,17 +958,17 @@
         <v>46218</v>
       </c>
       <c r="B28" t="n">
-        <v>2279</v>
+        <v>2499</v>
       </c>
       <c r="C28" t="n">
         <v>8888</v>
       </c>
       <c r="D28" t="n">
-        <v>2753.96</v>
+        <v>261.63</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -977,13 +977,13 @@
         <v>46218</v>
       </c>
       <c r="B29" t="n">
-        <v>1137</v>
+        <v>58</v>
       </c>
       <c r="C29" t="n">
         <v>8888</v>
       </c>
       <c r="D29" t="n">
-        <v>952.95</v>
+        <v>499.11</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -996,17 +996,17 @@
         <v>46218</v>
       </c>
       <c r="B30" t="n">
-        <v>325</v>
+        <v>2245</v>
       </c>
       <c r="C30" t="n">
         <v>8888</v>
       </c>
       <c r="D30" t="n">
-        <v>399.62</v>
+        <v>2740.06</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1015,17 +1015,17 @@
         <v>46218</v>
       </c>
       <c r="B31" t="n">
-        <v>664</v>
+        <v>325</v>
       </c>
       <c r="C31" t="n">
         <v>8888</v>
       </c>
       <c r="D31" t="n">
-        <v>682.3200000000001</v>
+        <v>524.36</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1034,17 +1034,17 @@
         <v>46218</v>
       </c>
       <c r="B32" t="n">
-        <v>945</v>
+        <v>2383</v>
       </c>
       <c r="C32" t="n">
         <v>8888</v>
       </c>
       <c r="D32" t="n">
-        <v>365.11</v>
+        <v>7926.02</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>PEDIDO ELETRÔNICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1053,17 +1053,17 @@
         <v>46218</v>
       </c>
       <c r="B33" t="n">
-        <v>451</v>
+        <v>1117</v>
       </c>
       <c r="C33" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D33" t="n">
-        <v>368.93</v>
+        <v>916.72</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1072,13 +1072,13 @@
         <v>46218</v>
       </c>
       <c r="B34" t="n">
-        <v>1756</v>
+        <v>2279</v>
       </c>
       <c r="C34" t="n">
         <v>8888</v>
       </c>
       <c r="D34" t="n">
-        <v>824.3200000000001</v>
+        <v>712.66</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1091,17 +1091,17 @@
         <v>46218</v>
       </c>
       <c r="B35" t="n">
-        <v>2631</v>
+        <v>535</v>
       </c>
       <c r="C35" t="n">
-        <v>2853</v>
+        <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>509.88</v>
+        <v>4810</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1110,17 @@
         <v>46218</v>
       </c>
       <c r="B36" t="n">
-        <v>2714</v>
+        <v>535</v>
       </c>
       <c r="C36" t="n">
-        <v>519</v>
+        <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>61939.22</v>
+        <v>1352.51</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1129,17 @@
         <v>46218</v>
       </c>
       <c r="B37" t="n">
-        <v>483</v>
+        <v>2678</v>
       </c>
       <c r="C37" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D37" t="n">
-        <v>4920.11</v>
+        <v>364.96</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1148,13 +1148,13 @@
         <v>46218</v>
       </c>
       <c r="B38" t="n">
-        <v>1075</v>
+        <v>2345</v>
       </c>
       <c r="C38" t="n">
         <v>8888</v>
       </c>
       <c r="D38" t="n">
-        <v>11607.79</v>
+        <v>863.16</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1167,17 +1167,17 @@
         <v>46218</v>
       </c>
       <c r="B39" t="n">
-        <v>629</v>
+        <v>438</v>
       </c>
       <c r="C39" t="n">
         <v>8888</v>
       </c>
       <c r="D39" t="n">
-        <v>9233.719999999999</v>
+        <v>220.06</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1186,13 +1186,13 @@
         <v>46218</v>
       </c>
       <c r="B40" t="n">
-        <v>1983</v>
+        <v>353</v>
       </c>
       <c r="C40" t="n">
-        <v>841</v>
+        <v>3179</v>
       </c>
       <c r="D40" t="n">
-        <v>105.6</v>
+        <v>495.84</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1205,13 +1205,13 @@
         <v>46218</v>
       </c>
       <c r="B41" t="n">
-        <v>1137</v>
+        <v>1293</v>
       </c>
       <c r="C41" t="n">
         <v>8888</v>
       </c>
       <c r="D41" t="n">
-        <v>3578.51</v>
+        <v>3129.07</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1224,17 +1224,17 @@
         <v>46218</v>
       </c>
       <c r="B42" t="n">
-        <v>2651</v>
+        <v>2279</v>
       </c>
       <c r="C42" t="n">
         <v>8888</v>
       </c>
       <c r="D42" t="n">
-        <v>1296.58</v>
+        <v>2753.96</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1243,17 +1243,17 @@
         <v>46218</v>
       </c>
       <c r="B43" t="n">
-        <v>2709</v>
+        <v>1137</v>
       </c>
       <c r="C43" t="n">
         <v>8888</v>
       </c>
       <c r="D43" t="n">
-        <v>547.6900000000001</v>
+        <v>1437.44</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1262,13 +1262,13 @@
         <v>46218</v>
       </c>
       <c r="B44" t="n">
-        <v>89</v>
+        <v>2793</v>
       </c>
       <c r="C44" t="n">
-        <v>13148</v>
+        <v>977</v>
       </c>
       <c r="D44" t="n">
-        <v>1883.74</v>
+        <v>695.72</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1281,17 +1281,17 @@
         <v>46218</v>
       </c>
       <c r="B45" t="n">
-        <v>2709</v>
+        <v>945</v>
       </c>
       <c r="C45" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>390.19</v>
+        <v>1934.84</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>PEDIDO ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -1300,17 +1300,17 @@
         <v>46218</v>
       </c>
       <c r="B46" t="n">
-        <v>2345</v>
+        <v>374</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>748.86</v>
+        <v>22.62</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1319,13 +1319,13 @@
         <v>46218</v>
       </c>
       <c r="B47" t="n">
-        <v>1308</v>
+        <v>664</v>
       </c>
       <c r="C47" t="n">
         <v>8888</v>
       </c>
       <c r="D47" t="n">
-        <v>276.16</v>
+        <v>1510.56</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1338,17 +1338,17 @@
         <v>46218</v>
       </c>
       <c r="B48" t="n">
-        <v>2211</v>
+        <v>703</v>
       </c>
       <c r="C48" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D48" t="n">
-        <v>1526.94</v>
+        <v>12155.46</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1357,17 +1357,17 @@
         <v>46218</v>
       </c>
       <c r="B49" t="n">
-        <v>559</v>
+        <v>1937</v>
       </c>
       <c r="C49" t="n">
         <v>8888</v>
       </c>
       <c r="D49" t="n">
-        <v>859.92</v>
+        <v>1032.73</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1376,13 +1376,13 @@
         <v>46218</v>
       </c>
       <c r="B50" t="n">
-        <v>1063</v>
+        <v>451</v>
       </c>
       <c r="C50" t="n">
         <v>8888</v>
       </c>
       <c r="D50" t="n">
-        <v>4487.11</v>
+        <v>368.93</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1395,17 +1395,17 @@
         <v>46218</v>
       </c>
       <c r="B51" t="n">
-        <v>2279</v>
+        <v>1756</v>
       </c>
       <c r="C51" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D51" t="n">
-        <v>652.51</v>
+        <v>996.17</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
         <v>46218</v>
       </c>
       <c r="B52" t="n">
-        <v>1299</v>
+        <v>1956</v>
       </c>
       <c r="C52" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D52" t="n">
-        <v>1435.52</v>
+        <v>4557.34</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1433,17 +1433,17 @@
         <v>46218</v>
       </c>
       <c r="B53" t="n">
-        <v>1478</v>
+        <v>925</v>
       </c>
       <c r="C53" t="n">
-        <v>675</v>
+        <v>8888</v>
       </c>
       <c r="D53" t="n">
-        <v>511.84</v>
+        <v>651.59</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1452,17 +1452,17 @@
         <v>46218</v>
       </c>
       <c r="B54" t="n">
-        <v>285</v>
+        <v>2631</v>
       </c>
       <c r="C54" t="n">
-        <v>8888</v>
+        <v>2853</v>
       </c>
       <c r="D54" t="n">
-        <v>3349.8</v>
+        <v>509.88</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1471,13 +1471,13 @@
         <v>46218</v>
       </c>
       <c r="B55" t="n">
-        <v>1983</v>
+        <v>2648</v>
       </c>
       <c r="C55" t="n">
         <v>8888</v>
       </c>
       <c r="D55" t="n">
-        <v>2451.28</v>
+        <v>1594.42</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1490,13 +1490,13 @@
         <v>46218</v>
       </c>
       <c r="B56" t="n">
-        <v>477</v>
+        <v>2714</v>
       </c>
       <c r="C56" t="n">
-        <v>58</v>
+        <v>519</v>
       </c>
       <c r="D56" t="n">
-        <v>1540.55</v>
+        <v>61939.22</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1509,17 +1509,17 @@
         <v>46218</v>
       </c>
       <c r="B57" t="n">
-        <v>1063</v>
+        <v>483</v>
       </c>
       <c r="C57" t="n">
         <v>8888</v>
       </c>
       <c r="D57" t="n">
-        <v>2549.86</v>
+        <v>6625.87</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1528,13 +1528,13 @@
         <v>46218</v>
       </c>
       <c r="B58" t="n">
-        <v>424</v>
+        <v>1075</v>
       </c>
       <c r="C58" t="n">
         <v>8888</v>
       </c>
       <c r="D58" t="n">
-        <v>1035.17</v>
+        <v>11607.79</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1547,17 +1547,17 @@
         <v>46218</v>
       </c>
       <c r="B59" t="n">
-        <v>675</v>
+        <v>629</v>
       </c>
       <c r="C59" t="n">
         <v>8888</v>
       </c>
       <c r="D59" t="n">
-        <v>616.73</v>
+        <v>9233.719999999999</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1566,17 +1566,17 @@
         <v>46218</v>
       </c>
       <c r="B60" t="n">
-        <v>1993</v>
+        <v>1983</v>
       </c>
       <c r="C60" t="n">
-        <v>8888</v>
+        <v>841</v>
       </c>
       <c r="D60" t="n">
-        <v>362.63</v>
+        <v>243.92</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1585,13 +1585,13 @@
         <v>46218</v>
       </c>
       <c r="B61" t="n">
-        <v>1465</v>
+        <v>1137</v>
       </c>
       <c r="C61" t="n">
         <v>8888</v>
       </c>
       <c r="D61" t="n">
-        <v>3373.83</v>
+        <v>3578.51</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1604,13 +1604,13 @@
         <v>46218</v>
       </c>
       <c r="B62" t="n">
-        <v>89</v>
+        <v>2651</v>
       </c>
       <c r="C62" t="n">
         <v>8888</v>
       </c>
       <c r="D62" t="n">
-        <v>479</v>
+        <v>1296.58</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1623,13 +1623,13 @@
         <v>46218</v>
       </c>
       <c r="B63" t="n">
-        <v>2696</v>
+        <v>1956</v>
       </c>
       <c r="C63" t="n">
-        <v>1954</v>
+        <v>423</v>
       </c>
       <c r="D63" t="n">
-        <v>259.97</v>
+        <v>455.37</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1642,13 +1642,13 @@
         <v>46218</v>
       </c>
       <c r="B64" t="n">
-        <v>360</v>
+        <v>2709</v>
       </c>
       <c r="C64" t="n">
         <v>8888</v>
       </c>
       <c r="D64" t="n">
-        <v>2023.17</v>
+        <v>547.6900000000001</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1661,17 +1661,17 @@
         <v>46218</v>
       </c>
       <c r="B65" t="n">
-        <v>1465</v>
+        <v>2026</v>
       </c>
       <c r="C65" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D65" t="n">
-        <v>777.2</v>
+        <v>2237.62</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1680,17 +1680,17 @@
         <v>46218</v>
       </c>
       <c r="B66" t="n">
-        <v>1937</v>
+        <v>89</v>
       </c>
       <c r="C66" t="n">
-        <v>8888</v>
+        <v>13148</v>
       </c>
       <c r="D66" t="n">
-        <v>833.52</v>
+        <v>1883.74</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1699,17 +1699,17 @@
         <v>46218</v>
       </c>
       <c r="B67" t="n">
-        <v>1293</v>
+        <v>2709</v>
       </c>
       <c r="C67" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D67" t="n">
-        <v>1607.2</v>
+        <v>390.19</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1718,17 +1718,17 @@
         <v>46218</v>
       </c>
       <c r="B68" t="n">
-        <v>630</v>
+        <v>2345</v>
       </c>
       <c r="C68" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D68" t="n">
-        <v>1210.85</v>
+        <v>748.86</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1737,17 +1737,17 @@
         <v>46218</v>
       </c>
       <c r="B69" t="n">
-        <v>2571</v>
+        <v>1308</v>
       </c>
       <c r="C69" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D69" t="n">
-        <v>268.53</v>
+        <v>276.16</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1756,13 +1756,13 @@
         <v>46218</v>
       </c>
       <c r="B70" t="n">
-        <v>1063</v>
+        <v>2308</v>
       </c>
       <c r="C70" t="n">
         <v>8888</v>
       </c>
       <c r="D70" t="n">
-        <v>1113.08</v>
+        <v>488.69</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -1775,17 +1775,17 @@
         <v>46218</v>
       </c>
       <c r="B71" t="n">
-        <v>1756</v>
+        <v>360</v>
       </c>
       <c r="C71" t="n">
-        <v>8888</v>
+        <v>546</v>
       </c>
       <c r="D71" t="n">
-        <v>1357.12</v>
+        <v>709.75</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1794,17 +1794,17 @@
         <v>46218</v>
       </c>
       <c r="B72" t="n">
-        <v>569</v>
+        <v>2211</v>
       </c>
       <c r="C72" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D72" t="n">
-        <v>4504.72</v>
+        <v>1526.94</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1813,17 +1813,17 @@
         <v>46218</v>
       </c>
       <c r="B73" t="n">
-        <v>2089</v>
+        <v>559</v>
       </c>
       <c r="C73" t="n">
-        <v>1533</v>
+        <v>8888</v>
       </c>
       <c r="D73" t="n">
-        <v>442.44</v>
+        <v>859.92</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1832,17 +1832,17 @@
         <v>46218</v>
       </c>
       <c r="B74" t="n">
-        <v>1007</v>
+        <v>569</v>
       </c>
       <c r="C74" t="n">
         <v>8888</v>
       </c>
       <c r="D74" t="n">
-        <v>241.44</v>
+        <v>673.01</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1851,17 +1851,17 @@
         <v>46218</v>
       </c>
       <c r="B75" t="n">
-        <v>1380</v>
+        <v>890</v>
       </c>
       <c r="C75" t="n">
         <v>8888</v>
       </c>
       <c r="D75" t="n">
-        <v>520.2</v>
+        <v>387.2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1870,13 +1870,13 @@
         <v>46218</v>
       </c>
       <c r="B76" t="n">
-        <v>1102</v>
+        <v>1063</v>
       </c>
       <c r="C76" t="n">
         <v>8888</v>
       </c>
       <c r="D76" t="n">
-        <v>1137.04</v>
+        <v>4487.11</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -1889,17 +1889,17 @@
         <v>46218</v>
       </c>
       <c r="B77" t="n">
-        <v>1075</v>
+        <v>2279</v>
       </c>
       <c r="C77" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D77" t="n">
-        <v>2179.03</v>
+        <v>652.51</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1908,17 +1908,17 @@
         <v>46218</v>
       </c>
       <c r="B78" t="n">
-        <v>2245</v>
+        <v>1299</v>
       </c>
       <c r="C78" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D78" t="n">
-        <v>361.58</v>
+        <v>1435.52</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1927,17 +1927,17 @@
         <v>46218</v>
       </c>
       <c r="B79" t="n">
-        <v>2660</v>
+        <v>1478</v>
       </c>
       <c r="C79" t="n">
-        <v>8888</v>
+        <v>675</v>
       </c>
       <c r="D79" t="n">
-        <v>528.4299999999999</v>
+        <v>1600.01</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1946,17 +1946,17 @@
         <v>46218</v>
       </c>
       <c r="B80" t="n">
-        <v>452</v>
+        <v>285</v>
       </c>
       <c r="C80" t="n">
         <v>8888</v>
       </c>
       <c r="D80" t="n">
-        <v>608.78</v>
+        <v>3349.8</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1965,17 +1965,17 @@
         <v>46218</v>
       </c>
       <c r="B81" t="n">
-        <v>1293</v>
+        <v>1983</v>
       </c>
       <c r="C81" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D81" t="n">
-        <v>1780.93</v>
+        <v>2451.28</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1984,17 +1984,17 @@
         <v>46218</v>
       </c>
       <c r="B82" t="n">
-        <v>525</v>
+        <v>477</v>
       </c>
       <c r="C82" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D82" t="n">
-        <v>4599.72</v>
+        <v>1540.55</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2003,13 +2003,13 @@
         <v>46218</v>
       </c>
       <c r="B83" t="n">
-        <v>609</v>
+        <v>1063</v>
       </c>
       <c r="C83" t="n">
         <v>8888</v>
       </c>
       <c r="D83" t="n">
-        <v>886.1</v>
+        <v>2549.86</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2022,17 +2022,17 @@
         <v>46218</v>
       </c>
       <c r="B84" t="n">
-        <v>619</v>
+        <v>424</v>
       </c>
       <c r="C84" t="n">
         <v>8888</v>
       </c>
       <c r="D84" t="n">
-        <v>2330.47</v>
+        <v>1035.17</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2041,17 +2041,17 @@
         <v>46218</v>
       </c>
       <c r="B85" t="n">
-        <v>285</v>
+        <v>675</v>
       </c>
       <c r="C85" t="n">
         <v>8888</v>
       </c>
       <c r="D85" t="n">
-        <v>2090.81</v>
+        <v>616.73</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2060,17 +2060,17 @@
         <v>46218</v>
       </c>
       <c r="B86" t="n">
-        <v>1102</v>
+        <v>2768</v>
       </c>
       <c r="C86" t="n">
         <v>8888</v>
       </c>
       <c r="D86" t="n">
-        <v>1119.32</v>
+        <v>4245.73</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2079,17 +2079,17 @@
         <v>46218</v>
       </c>
       <c r="B87" t="n">
-        <v>626</v>
+        <v>1993</v>
       </c>
       <c r="C87" t="n">
         <v>8888</v>
       </c>
       <c r="D87" t="n">
-        <v>5211.29</v>
+        <v>362.63</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2098,17 +2098,17 @@
         <v>46218</v>
       </c>
       <c r="B88" t="n">
-        <v>1137</v>
+        <v>1465</v>
       </c>
       <c r="C88" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D88" t="n">
-        <v>1370.86</v>
+        <v>3373.83</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2117,17 +2117,17 @@
         <v>46218</v>
       </c>
       <c r="B89" t="n">
-        <v>1756</v>
+        <v>89</v>
       </c>
       <c r="C89" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D89" t="n">
-        <v>5078.1</v>
+        <v>479</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2136,17 +2136,17 @@
         <v>46218</v>
       </c>
       <c r="B90" t="n">
-        <v>2651</v>
+        <v>595</v>
       </c>
       <c r="C90" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D90" t="n">
-        <v>363.7</v>
+        <v>18084.5</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2155,17 +2155,17 @@
         <v>46218</v>
       </c>
       <c r="B91" t="n">
-        <v>360</v>
+        <v>2696</v>
       </c>
       <c r="C91" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D91" t="n">
-        <v>1594.84</v>
+        <v>259.97</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2174,17 +2174,17 @@
         <v>46218</v>
       </c>
       <c r="B92" t="n">
-        <v>2582</v>
+        <v>360</v>
       </c>
       <c r="C92" t="n">
         <v>8888</v>
       </c>
       <c r="D92" t="n">
-        <v>379.33</v>
+        <v>2023.17</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2193,17 +2193,17 @@
         <v>46218</v>
       </c>
       <c r="B93" t="n">
-        <v>1756</v>
+        <v>1465</v>
       </c>
       <c r="C93" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D93" t="n">
-        <v>1715.26</v>
+        <v>777.2</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2212,17 +2212,17 @@
         <v>46218</v>
       </c>
       <c r="B94" t="n">
-        <v>1289</v>
+        <v>947</v>
       </c>
       <c r="C94" t="n">
         <v>8888</v>
       </c>
       <c r="D94" t="n">
-        <v>2396.98</v>
+        <v>2087.97</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>PEDIDO ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -2231,13 +2231,13 @@
         <v>46218</v>
       </c>
       <c r="B95" t="n">
-        <v>2015</v>
+        <v>2178</v>
       </c>
       <c r="C95" t="n">
         <v>8888</v>
       </c>
       <c r="D95" t="n">
-        <v>315.69</v>
+        <v>619.92</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2250,17 +2250,17 @@
         <v>46218</v>
       </c>
       <c r="B96" t="n">
-        <v>1064</v>
+        <v>630</v>
       </c>
       <c r="C96" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D96" t="n">
-        <v>1274.3</v>
+        <v>1801.63</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2269,17 +2269,17 @@
         <v>46218</v>
       </c>
       <c r="B97" t="n">
-        <v>2698</v>
+        <v>1937</v>
       </c>
       <c r="C97" t="n">
         <v>8888</v>
       </c>
       <c r="D97" t="n">
-        <v>552.15</v>
+        <v>2132.95</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2288,13 +2288,13 @@
         <v>46218</v>
       </c>
       <c r="B98" t="n">
-        <v>629</v>
+        <v>2577</v>
       </c>
       <c r="C98" t="n">
         <v>8888</v>
       </c>
       <c r="D98" t="n">
-        <v>721.25</v>
+        <v>1647.08</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2307,17 +2307,17 @@
         <v>46218</v>
       </c>
       <c r="B99" t="n">
-        <v>2686</v>
+        <v>1293</v>
       </c>
       <c r="C99" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D99" t="n">
-        <v>521.79</v>
+        <v>1607.2</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2326,17 +2326,17 @@
         <v>46218</v>
       </c>
       <c r="B100" t="n">
-        <v>2584</v>
+        <v>1317</v>
       </c>
       <c r="C100" t="n">
         <v>8888</v>
       </c>
       <c r="D100" t="n">
-        <v>1852.83</v>
+        <v>907.72</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2345,17 +2345,17 @@
         <v>46218</v>
       </c>
       <c r="B101" t="n">
-        <v>2641</v>
+        <v>2571</v>
       </c>
       <c r="C101" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D101" t="n">
-        <v>820</v>
+        <v>268.53</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2364,13 +2364,13 @@
         <v>46218</v>
       </c>
       <c r="B102" t="n">
-        <v>664</v>
+        <v>1937</v>
       </c>
       <c r="C102" t="n">
         <v>8888</v>
       </c>
       <c r="D102" t="n">
-        <v>1595.68</v>
+        <v>1803.32</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2383,17 +2383,17 @@
         <v>46218</v>
       </c>
       <c r="B103" t="n">
-        <v>816</v>
+        <v>1063</v>
       </c>
       <c r="C103" t="n">
         <v>8888</v>
       </c>
       <c r="D103" t="n">
-        <v>438.24</v>
+        <v>1113.08</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2402,17 +2402,17 @@
         <v>46218</v>
       </c>
       <c r="B104" t="n">
-        <v>285</v>
+        <v>1906</v>
       </c>
       <c r="C104" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D104" t="n">
-        <v>364.99</v>
+        <v>990.22</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2421,13 +2421,13 @@
         <v>46218</v>
       </c>
       <c r="B105" t="n">
-        <v>2114</v>
+        <v>1756</v>
       </c>
       <c r="C105" t="n">
         <v>8888</v>
       </c>
       <c r="D105" t="n">
-        <v>1682.3</v>
+        <v>1357.12</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2440,17 +2440,17 @@
         <v>46218</v>
       </c>
       <c r="B106" t="n">
-        <v>953</v>
+        <v>20</v>
       </c>
       <c r="C106" t="n">
         <v>8888</v>
       </c>
       <c r="D106" t="n">
-        <v>2618.89</v>
+        <v>276.64</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2459,13 +2459,13 @@
         <v>46218</v>
       </c>
       <c r="B107" t="n">
-        <v>1102</v>
+        <v>477</v>
       </c>
       <c r="C107" t="n">
         <v>8888</v>
       </c>
       <c r="D107" t="n">
-        <v>2344.41</v>
+        <v>372.69</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -2478,17 +2478,17 @@
         <v>46218</v>
       </c>
       <c r="B108" t="n">
-        <v>619</v>
+        <v>477</v>
       </c>
       <c r="C108" t="n">
         <v>8888</v>
       </c>
       <c r="D108" t="n">
-        <v>2021.67</v>
+        <v>707.52</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2497,17 +2497,17 @@
         <v>46218</v>
       </c>
       <c r="B109" t="n">
-        <v>1465</v>
+        <v>2660</v>
       </c>
       <c r="C109" t="n">
         <v>8888</v>
       </c>
       <c r="D109" t="n">
-        <v>3504</v>
+        <v>2684.97</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2516,17 +2516,17 @@
         <v>46218</v>
       </c>
       <c r="B110" t="n">
-        <v>2767</v>
+        <v>569</v>
       </c>
       <c r="C110" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D110" t="n">
-        <v>466.12</v>
+        <v>18512.6</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2535,17 +2535,17 @@
         <v>46218</v>
       </c>
       <c r="B111" t="n">
-        <v>2245</v>
+        <v>2089</v>
       </c>
       <c r="C111" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D111" t="n">
-        <v>427.51</v>
+        <v>969.24</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2554,13 +2554,13 @@
         <v>46218</v>
       </c>
       <c r="B112" t="n">
-        <v>2657</v>
+        <v>1007</v>
       </c>
       <c r="C112" t="n">
         <v>8888</v>
       </c>
       <c r="D112" t="n">
-        <v>703.6799999999999</v>
+        <v>241.44</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -2573,17 +2573,17 @@
         <v>46218</v>
       </c>
       <c r="B113" t="n">
-        <v>131</v>
+        <v>1380</v>
       </c>
       <c r="C113" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D113" t="n">
-        <v>299.37</v>
+        <v>520.2</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2592,17 +2592,17 @@
         <v>46218</v>
       </c>
       <c r="B114" t="n">
-        <v>2692</v>
+        <v>1102</v>
       </c>
       <c r="C114" t="n">
         <v>8888</v>
       </c>
       <c r="D114" t="n">
-        <v>731.28</v>
+        <v>1137.04</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2611,17 +2611,17 @@
         <v>46218</v>
       </c>
       <c r="B115" t="n">
-        <v>1317</v>
+        <v>1075</v>
       </c>
       <c r="C115" t="n">
-        <v>3179</v>
+        <v>8888</v>
       </c>
       <c r="D115" t="n">
-        <v>991.6799999999999</v>
+        <v>2179.03</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2630,17 +2630,17 @@
         <v>46218</v>
       </c>
       <c r="B116" t="n">
-        <v>1993</v>
+        <v>2245</v>
       </c>
       <c r="C116" t="n">
         <v>8888</v>
       </c>
       <c r="D116" t="n">
-        <v>2875.39</v>
+        <v>361.58</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2649,13 +2649,13 @@
         <v>46218</v>
       </c>
       <c r="B117" t="n">
-        <v>1632</v>
+        <v>132</v>
       </c>
       <c r="C117" t="n">
         <v>8888</v>
       </c>
       <c r="D117" t="n">
-        <v>564.55</v>
+        <v>6522.92</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -2668,17 +2668,17 @@
         <v>46218</v>
       </c>
       <c r="B118" t="n">
-        <v>1890</v>
+        <v>452</v>
       </c>
       <c r="C118" t="n">
-        <v>3449</v>
+        <v>8888</v>
       </c>
       <c r="D118" t="n">
-        <v>3063.24</v>
+        <v>608.78</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2687,13 +2687,13 @@
         <v>46218</v>
       </c>
       <c r="B119" t="n">
-        <v>451</v>
+        <v>1293</v>
       </c>
       <c r="C119" t="n">
-        <v>3403</v>
+        <v>1281</v>
       </c>
       <c r="D119" t="n">
-        <v>445.58</v>
+        <v>1780.93</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -2706,17 +2706,17 @@
         <v>46218</v>
       </c>
       <c r="B120" t="n">
-        <v>2749</v>
+        <v>525</v>
       </c>
       <c r="C120" t="n">
         <v>8888</v>
       </c>
       <c r="D120" t="n">
-        <v>1860.64</v>
+        <v>5658.57</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2725,17 +2725,17 @@
         <v>46218</v>
       </c>
       <c r="B121" t="n">
-        <v>1117</v>
+        <v>609</v>
       </c>
       <c r="C121" t="n">
         <v>8888</v>
       </c>
       <c r="D121" t="n">
-        <v>342.2</v>
+        <v>886.1</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2744,17 +2744,17 @@
         <v>46218</v>
       </c>
       <c r="B122" t="n">
-        <v>1478</v>
+        <v>619</v>
       </c>
       <c r="C122" t="n">
         <v>8888</v>
       </c>
       <c r="D122" t="n">
-        <v>875.34</v>
+        <v>2330.47</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2763,13 +2763,13 @@
         <v>46218</v>
       </c>
       <c r="B123" t="n">
-        <v>2491</v>
+        <v>58</v>
       </c>
       <c r="C123" t="n">
         <v>8888</v>
       </c>
       <c r="D123" t="n">
-        <v>650.4299999999999</v>
+        <v>1123.87</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -2782,17 +2782,17 @@
         <v>46218</v>
       </c>
       <c r="B124" t="n">
-        <v>2015</v>
+        <v>358</v>
       </c>
       <c r="C124" t="n">
         <v>8888</v>
       </c>
       <c r="D124" t="n">
-        <v>4436.15</v>
+        <v>1675.95</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2801,13 +2801,13 @@
         <v>46218</v>
       </c>
       <c r="B125" t="n">
-        <v>2782</v>
+        <v>2431</v>
       </c>
       <c r="C125" t="n">
         <v>8888</v>
       </c>
       <c r="D125" t="n">
-        <v>1786.32</v>
+        <v>266.89</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -2820,17 +2820,17 @@
         <v>46218</v>
       </c>
       <c r="B126" t="n">
-        <v>483</v>
+        <v>285</v>
       </c>
       <c r="C126" t="n">
-        <v>841</v>
+        <v>8888</v>
       </c>
       <c r="D126" t="n">
-        <v>1393.15</v>
+        <v>2090.81</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2839,17 +2839,17 @@
         <v>46218</v>
       </c>
       <c r="B127" t="n">
-        <v>2648</v>
+        <v>1102</v>
       </c>
       <c r="C127" t="n">
         <v>8888</v>
       </c>
       <c r="D127" t="n">
-        <v>1873.52</v>
+        <v>1119.32</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2858,13 +2858,13 @@
         <v>46218</v>
       </c>
       <c r="B128" t="n">
-        <v>131</v>
+        <v>626</v>
       </c>
       <c r="C128" t="n">
         <v>8888</v>
       </c>
       <c r="D128" t="n">
-        <v>1369.91</v>
+        <v>11337.75</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -2877,17 +2877,17 @@
         <v>46218</v>
       </c>
       <c r="B129" t="n">
-        <v>2109</v>
+        <v>1137</v>
       </c>
       <c r="C129" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D129" t="n">
-        <v>2293.78</v>
+        <v>1370.86</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2896,17 +2896,17 @@
         <v>46218</v>
       </c>
       <c r="B130" t="n">
-        <v>1116</v>
+        <v>1756</v>
       </c>
       <c r="C130" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D130" t="n">
-        <v>2919.53</v>
+        <v>5078.1</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2915,13 +2915,13 @@
         <v>46218</v>
       </c>
       <c r="B131" t="n">
-        <v>2250</v>
+        <v>2651</v>
       </c>
       <c r="C131" t="n">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="D131" t="n">
-        <v>1573.32</v>
+        <v>363.7</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -2934,17 +2934,17 @@
         <v>46218</v>
       </c>
       <c r="B132" t="n">
-        <v>2698</v>
+        <v>360</v>
       </c>
       <c r="C132" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D132" t="n">
-        <v>1230.43</v>
+        <v>1594.84</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2953,13 +2953,13 @@
         <v>46218</v>
       </c>
       <c r="B133" t="n">
-        <v>42</v>
+        <v>2582</v>
       </c>
       <c r="C133" t="n">
         <v>8888</v>
       </c>
       <c r="D133" t="n">
-        <v>79947.14999999999</v>
+        <v>379.33</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -2972,17 +2972,17 @@
         <v>46218</v>
       </c>
       <c r="B134" t="n">
-        <v>2716</v>
+        <v>1756</v>
       </c>
       <c r="C134" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D134" t="n">
-        <v>750.4299999999999</v>
+        <v>1715.26</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2991,17 +2991,17 @@
         <v>46218</v>
       </c>
       <c r="B135" t="n">
-        <v>2716</v>
+        <v>1254</v>
       </c>
       <c r="C135" t="n">
-        <v>977</v>
+        <v>8888</v>
       </c>
       <c r="D135" t="n">
-        <v>729.29</v>
+        <v>855.76</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3010,17 +3010,17 @@
         <v>46218</v>
       </c>
       <c r="B136" t="n">
-        <v>1993</v>
+        <v>1289</v>
       </c>
       <c r="C136" t="n">
         <v>8888</v>
       </c>
       <c r="D136" t="n">
-        <v>456.62</v>
+        <v>2396.98</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3029,15 +3029,1003 @@
         <v>46218</v>
       </c>
       <c r="B137" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C137" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D137" t="n">
+        <v>315.69</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B138" t="n">
+        <v>1064</v>
+      </c>
+      <c r="C138" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D138" t="n">
+        <v>1274.3</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B139" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C139" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D139" t="n">
+        <v>552.15</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B140" t="n">
         <v>629</v>
       </c>
-      <c r="C137" t="n">
+      <c r="C140" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D140" t="n">
+        <v>3035.38</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B141" t="n">
+        <v>664</v>
+      </c>
+      <c r="C141" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D141" t="n">
+        <v>4973.15</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B142" t="n">
+        <v>2686</v>
+      </c>
+      <c r="C142" t="n">
+        <v>1929</v>
+      </c>
+      <c r="D142" t="n">
+        <v>521.79</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B143" t="n">
+        <v>2584</v>
+      </c>
+      <c r="C143" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D143" t="n">
+        <v>1852.83</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B144" t="n">
+        <v>2641</v>
+      </c>
+      <c r="C144" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D144" t="n">
+        <v>820</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B145" t="n">
+        <v>816</v>
+      </c>
+      <c r="C145" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D145" t="n">
+        <v>438.24</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B146" t="n">
+        <v>285</v>
+      </c>
+      <c r="C146" t="n">
+        <v>58</v>
+      </c>
+      <c r="D146" t="n">
+        <v>364.99</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B147" t="n">
+        <v>2114</v>
+      </c>
+      <c r="C147" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D147" t="n">
+        <v>2726.04</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B148" t="n">
+        <v>953</v>
+      </c>
+      <c r="C148" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D148" t="n">
+        <v>2618.89</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B149" t="n">
+        <v>1102</v>
+      </c>
+      <c r="C149" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D149" t="n">
+        <v>2344.41</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B150" t="n">
+        <v>619</v>
+      </c>
+      <c r="C150" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D150" t="n">
+        <v>2021.67</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B151" t="n">
+        <v>1465</v>
+      </c>
+      <c r="C151" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D151" t="n">
+        <v>3504</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B152" t="n">
+        <v>2767</v>
+      </c>
+      <c r="C152" t="n">
+        <v>1898</v>
+      </c>
+      <c r="D152" t="n">
+        <v>1135.64</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B153" t="n">
+        <v>2245</v>
+      </c>
+      <c r="C153" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D153" t="n">
+        <v>427.51</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B154" t="n">
+        <v>2197</v>
+      </c>
+      <c r="C154" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D154" t="n">
+        <v>1085.45</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B155" t="n">
+        <v>2657</v>
+      </c>
+      <c r="C155" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D155" t="n">
+        <v>1187.68</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B156" t="n">
+        <v>1277</v>
+      </c>
+      <c r="C156" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D156" t="n">
+        <v>1949</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B157" t="n">
+        <v>131</v>
+      </c>
+      <c r="C157" t="n">
+        <v>27</v>
+      </c>
+      <c r="D157" t="n">
+        <v>1268.57</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B158" t="n">
+        <v>2692</v>
+      </c>
+      <c r="C158" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D158" t="n">
+        <v>731.28</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B159" t="n">
+        <v>1317</v>
+      </c>
+      <c r="C159" t="n">
+        <v>3179</v>
+      </c>
+      <c r="D159" t="n">
+        <v>991.6799999999999</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B160" t="n">
+        <v>1993</v>
+      </c>
+      <c r="C160" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D160" t="n">
+        <v>2875.39</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B161" t="n">
+        <v>1632</v>
+      </c>
+      <c r="C161" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D161" t="n">
+        <v>564.55</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B162" t="n">
+        <v>1890</v>
+      </c>
+      <c r="C162" t="n">
+        <v>3449</v>
+      </c>
+      <c r="D162" t="n">
+        <v>3590.04</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B163" t="n">
+        <v>451</v>
+      </c>
+      <c r="C163" t="n">
+        <v>3403</v>
+      </c>
+      <c r="D163" t="n">
+        <v>445.58</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B164" t="n">
+        <v>2749</v>
+      </c>
+      <c r="C164" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D164" t="n">
+        <v>1860.64</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B165" t="n">
+        <v>1117</v>
+      </c>
+      <c r="C165" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D165" t="n">
+        <v>342.2</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B166" t="n">
+        <v>1478</v>
+      </c>
+      <c r="C166" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D166" t="n">
+        <v>875.34</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B167" t="n">
+        <v>2491</v>
+      </c>
+      <c r="C167" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D167" t="n">
+        <v>650.4299999999999</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B168" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C168" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D168" t="n">
+        <v>4436.15</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B169" t="n">
+        <v>1890</v>
+      </c>
+      <c r="C169" t="n">
+        <v>1953</v>
+      </c>
+      <c r="D169" t="n">
+        <v>500.92</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B170" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C170" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D170" t="n">
+        <v>1786.32</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B171" t="n">
+        <v>483</v>
+      </c>
+      <c r="C171" t="n">
+        <v>841</v>
+      </c>
+      <c r="D171" t="n">
+        <v>1393.15</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B172" t="n">
+        <v>2133</v>
+      </c>
+      <c r="C172" t="n">
+        <v>213</v>
+      </c>
+      <c r="D172" t="n">
+        <v>526.8</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B173" t="n">
+        <v>351</v>
+      </c>
+      <c r="C173" t="n">
+        <v>3009</v>
+      </c>
+      <c r="D173" t="n">
+        <v>416.36</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B174" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C174" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D174" t="n">
+        <v>709.46</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B175" t="n">
+        <v>2648</v>
+      </c>
+      <c r="C175" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D175" t="n">
+        <v>1873.52</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B176" t="n">
+        <v>131</v>
+      </c>
+      <c r="C176" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D176" t="n">
+        <v>1369.91</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B177" t="n">
+        <v>2639</v>
+      </c>
+      <c r="C177" t="n">
+        <v>1953</v>
+      </c>
+      <c r="D177" t="n">
+        <v>504.09</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B178" t="n">
+        <v>2109</v>
+      </c>
+      <c r="C178" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D178" t="n">
+        <v>2293.78</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B179" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C179" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D179" t="n">
+        <v>2919.53</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B180" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C180" t="n">
+        <v>27</v>
+      </c>
+      <c r="D180" t="n">
+        <v>1803.76</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B181" t="n">
+        <v>353</v>
+      </c>
+      <c r="C181" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D181" t="n">
+        <v>108.6</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B182" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C182" t="n">
+        <v>874</v>
+      </c>
+      <c r="D182" t="n">
+        <v>1230.43</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B183" t="n">
+        <v>42</v>
+      </c>
+      <c r="C183" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D183" t="n">
+        <v>79947.14999999999</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B184" t="n">
+        <v>772</v>
+      </c>
+      <c r="C184" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D184" t="n">
+        <v>400.25</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B185" t="n">
+        <v>2728</v>
+      </c>
+      <c r="C185" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D185" t="n">
+        <v>1397.07</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B186" t="n">
+        <v>2716</v>
+      </c>
+      <c r="C186" t="n">
+        <v>1929</v>
+      </c>
+      <c r="D186" t="n">
+        <v>750.4299999999999</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B187" t="n">
+        <v>2716</v>
+      </c>
+      <c r="C187" t="n">
+        <v>977</v>
+      </c>
+      <c r="D187" t="n">
+        <v>729.29</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B188" t="n">
+        <v>1993</v>
+      </c>
+      <c r="C188" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D188" t="n">
+        <v>456.62</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B189" t="n">
+        <v>629</v>
+      </c>
+      <c r="C189" t="n">
         <v>675</v>
       </c>
-      <c r="D137" t="n">
+      <c r="D189" t="n">
         <v>1054.76</v>
       </c>
-      <c r="E137" t="inlineStr">
+      <c r="E189" t="inlineStr">
         <is>
           <t>TELEMARKETING</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 15:30:14
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E189"/>
+  <dimension ref="A1:E205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,7 +470,7 @@
         <v>8888</v>
       </c>
       <c r="D2" t="n">
-        <v>312.98</v>
+        <v>406.97</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -578,17 +578,17 @@
         <v>46218</v>
       </c>
       <c r="B8" t="n">
-        <v>2015</v>
+        <v>1632</v>
       </c>
       <c r="C8" t="n">
-        <v>2571</v>
+        <v>8888</v>
       </c>
       <c r="D8" t="n">
-        <v>714.53</v>
+        <v>768.84</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -597,13 +597,13 @@
         <v>46218</v>
       </c>
       <c r="B9" t="n">
-        <v>1289</v>
+        <v>2015</v>
       </c>
       <c r="C9" t="n">
-        <v>1929</v>
+        <v>2571</v>
       </c>
       <c r="D9" t="n">
-        <v>727.05</v>
+        <v>3147.53</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -616,13 +616,13 @@
         <v>46218</v>
       </c>
       <c r="B10" t="n">
-        <v>609</v>
+        <v>1289</v>
       </c>
       <c r="C10" t="n">
-        <v>3179</v>
+        <v>1929</v>
       </c>
       <c r="D10" t="n">
-        <v>2603.16</v>
+        <v>727.05</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -635,17 +635,17 @@
         <v>46218</v>
       </c>
       <c r="B11" t="n">
-        <v>2211</v>
+        <v>609</v>
       </c>
       <c r="C11" t="n">
-        <v>8888</v>
+        <v>3179</v>
       </c>
       <c r="D11" t="n">
-        <v>2190.93</v>
+        <v>2603.16</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -654,13 +654,13 @@
         <v>46218</v>
       </c>
       <c r="B12" t="n">
-        <v>2660</v>
+        <v>2211</v>
       </c>
       <c r="C12" t="n">
         <v>8888</v>
       </c>
       <c r="D12" t="n">
-        <v>875.61</v>
+        <v>2190.93</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -673,13 +673,13 @@
         <v>46218</v>
       </c>
       <c r="B13" t="n">
-        <v>890</v>
+        <v>2660</v>
       </c>
       <c r="C13" t="n">
         <v>8888</v>
       </c>
       <c r="D13" t="n">
-        <v>1051.23</v>
+        <v>875.61</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -692,13 +692,13 @@
         <v>46218</v>
       </c>
       <c r="B14" t="n">
-        <v>2190</v>
+        <v>890</v>
       </c>
       <c r="C14" t="n">
         <v>8888</v>
       </c>
       <c r="D14" t="n">
-        <v>1307.13</v>
+        <v>1051.23</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -711,17 +711,17 @@
         <v>46218</v>
       </c>
       <c r="B15" t="n">
-        <v>2651</v>
+        <v>2190</v>
       </c>
       <c r="C15" t="n">
         <v>8888</v>
       </c>
       <c r="D15" t="n">
-        <v>660.95</v>
+        <v>1307.13</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -730,17 +730,17 @@
         <v>46218</v>
       </c>
       <c r="B16" t="n">
-        <v>2118</v>
+        <v>2651</v>
       </c>
       <c r="C16" t="n">
         <v>8888</v>
       </c>
       <c r="D16" t="n">
-        <v>5535.71</v>
+        <v>660.95</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -749,17 +749,17 @@
         <v>46218</v>
       </c>
       <c r="B17" t="n">
-        <v>2197</v>
+        <v>2118</v>
       </c>
       <c r="C17" t="n">
         <v>8888</v>
       </c>
       <c r="D17" t="n">
-        <v>892.66</v>
+        <v>5535.71</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -768,13 +768,13 @@
         <v>46218</v>
       </c>
       <c r="B18" t="n">
-        <v>1869</v>
+        <v>2507</v>
       </c>
       <c r="C18" t="n">
         <v>8888</v>
       </c>
       <c r="D18" t="n">
-        <v>1263.2</v>
+        <v>1174.1</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -787,17 +787,17 @@
         <v>46218</v>
       </c>
       <c r="B19" t="n">
-        <v>2133</v>
+        <v>2197</v>
       </c>
       <c r="C19" t="n">
-        <v>691</v>
+        <v>8888</v>
       </c>
       <c r="D19" t="n">
-        <v>2058.93</v>
+        <v>892.66</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -806,17 +806,17 @@
         <v>46218</v>
       </c>
       <c r="B20" t="n">
-        <v>452</v>
+        <v>363</v>
       </c>
       <c r="C20" t="n">
         <v>8888</v>
       </c>
       <c r="D20" t="n">
-        <v>1832.74</v>
+        <v>836.9400000000001</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -825,13 +825,13 @@
         <v>46218</v>
       </c>
       <c r="B21" t="n">
-        <v>2250</v>
+        <v>1869</v>
       </c>
       <c r="C21" t="n">
         <v>8888</v>
       </c>
       <c r="D21" t="n">
-        <v>1686.37</v>
+        <v>1263.2</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -844,13 +844,13 @@
         <v>46218</v>
       </c>
       <c r="B22" t="n">
-        <v>931</v>
+        <v>2133</v>
       </c>
       <c r="C22" t="n">
-        <v>423</v>
+        <v>691</v>
       </c>
       <c r="D22" t="n">
-        <v>492.34</v>
+        <v>2058.93</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -863,17 +863,17 @@
         <v>46218</v>
       </c>
       <c r="B23" t="n">
-        <v>951</v>
+        <v>452</v>
       </c>
       <c r="C23" t="n">
         <v>8888</v>
       </c>
       <c r="D23" t="n">
-        <v>2171.08</v>
+        <v>1832.74</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -882,17 +882,17 @@
         <v>46218</v>
       </c>
       <c r="B24" t="n">
-        <v>2695</v>
+        <v>2250</v>
       </c>
       <c r="C24" t="n">
         <v>8888</v>
       </c>
       <c r="D24" t="n">
-        <v>411.42</v>
+        <v>1686.37</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -901,17 +901,17 @@
         <v>46218</v>
       </c>
       <c r="B25" t="n">
-        <v>525</v>
+        <v>931</v>
       </c>
       <c r="C25" t="n">
-        <v>8888</v>
+        <v>423</v>
       </c>
       <c r="D25" t="n">
-        <v>408.25</v>
+        <v>492.34</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
         <v>46218</v>
       </c>
       <c r="B26" t="n">
-        <v>1808</v>
+        <v>951</v>
       </c>
       <c r="C26" t="n">
         <v>8888</v>
       </c>
       <c r="D26" t="n">
-        <v>695.3200000000001</v>
+        <v>2171.08</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -939,17 +939,17 @@
         <v>46218</v>
       </c>
       <c r="B27" t="n">
-        <v>949</v>
+        <v>2695</v>
       </c>
       <c r="C27" t="n">
-        <v>1134</v>
+        <v>8888</v>
       </c>
       <c r="D27" t="n">
-        <v>30.46</v>
+        <v>411.42</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -958,17 +958,17 @@
         <v>46218</v>
       </c>
       <c r="B28" t="n">
-        <v>2499</v>
+        <v>525</v>
       </c>
       <c r="C28" t="n">
         <v>8888</v>
       </c>
       <c r="D28" t="n">
-        <v>261.63</v>
+        <v>408.25</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -977,17 +977,17 @@
         <v>46218</v>
       </c>
       <c r="B29" t="n">
-        <v>58</v>
+        <v>1808</v>
       </c>
       <c r="C29" t="n">
         <v>8888</v>
       </c>
       <c r="D29" t="n">
-        <v>499.11</v>
+        <v>695.3200000000001</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -996,17 +996,17 @@
         <v>46218</v>
       </c>
       <c r="B30" t="n">
-        <v>2245</v>
+        <v>1632</v>
       </c>
       <c r="C30" t="n">
-        <v>8888</v>
+        <v>423</v>
       </c>
       <c r="D30" t="n">
-        <v>2740.06</v>
+        <v>1266.17</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1015,17 +1015,17 @@
         <v>46218</v>
       </c>
       <c r="B31" t="n">
-        <v>325</v>
+        <v>949</v>
       </c>
       <c r="C31" t="n">
-        <v>8888</v>
+        <v>1134</v>
       </c>
       <c r="D31" t="n">
-        <v>524.36</v>
+        <v>30.46</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1034,17 +1034,17 @@
         <v>46218</v>
       </c>
       <c r="B32" t="n">
-        <v>2383</v>
+        <v>2499</v>
       </c>
       <c r="C32" t="n">
         <v>8888</v>
       </c>
       <c r="D32" t="n">
-        <v>7926.02</v>
+        <v>261.63</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1053,17 +1053,17 @@
         <v>46218</v>
       </c>
       <c r="B33" t="n">
-        <v>1117</v>
+        <v>58</v>
       </c>
       <c r="C33" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D33" t="n">
-        <v>916.72</v>
+        <v>499.11</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1072,13 +1072,13 @@
         <v>46218</v>
       </c>
       <c r="B34" t="n">
-        <v>2279</v>
+        <v>2245</v>
       </c>
       <c r="C34" t="n">
         <v>8888</v>
       </c>
       <c r="D34" t="n">
-        <v>712.66</v>
+        <v>2740.06</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1091,17 +1091,17 @@
         <v>46218</v>
       </c>
       <c r="B35" t="n">
-        <v>535</v>
+        <v>325</v>
       </c>
       <c r="C35" t="n">
         <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>4810</v>
+        <v>524.36</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1110,17 @@
         <v>46218</v>
       </c>
       <c r="B36" t="n">
-        <v>535</v>
+        <v>2383</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>1352.51</v>
+        <v>7926.02</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1129,13 +1129,13 @@
         <v>46218</v>
       </c>
       <c r="B37" t="n">
-        <v>2678</v>
+        <v>1117</v>
       </c>
       <c r="C37" t="n">
-        <v>1312</v>
+        <v>1139</v>
       </c>
       <c r="D37" t="n">
-        <v>364.96</v>
+        <v>916.72</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1148,13 +1148,13 @@
         <v>46218</v>
       </c>
       <c r="B38" t="n">
-        <v>2345</v>
+        <v>2279</v>
       </c>
       <c r="C38" t="n">
         <v>8888</v>
       </c>
       <c r="D38" t="n">
-        <v>863.16</v>
+        <v>712.66</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1167,13 +1167,13 @@
         <v>46218</v>
       </c>
       <c r="B39" t="n">
-        <v>438</v>
+        <v>535</v>
       </c>
       <c r="C39" t="n">
         <v>8888</v>
       </c>
       <c r="D39" t="n">
-        <v>220.06</v>
+        <v>4810</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1186,17 +1186,17 @@
         <v>46218</v>
       </c>
       <c r="B40" t="n">
-        <v>353</v>
+        <v>535</v>
       </c>
       <c r="C40" t="n">
-        <v>3179</v>
+        <v>8888</v>
       </c>
       <c r="D40" t="n">
-        <v>495.84</v>
+        <v>1352.51</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1205,17 +1205,17 @@
         <v>46218</v>
       </c>
       <c r="B41" t="n">
-        <v>1293</v>
+        <v>2678</v>
       </c>
       <c r="C41" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D41" t="n">
-        <v>3129.07</v>
+        <v>364.96</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1224,17 +1224,17 @@
         <v>46218</v>
       </c>
       <c r="B42" t="n">
-        <v>2279</v>
+        <v>2345</v>
       </c>
       <c r="C42" t="n">
         <v>8888</v>
       </c>
       <c r="D42" t="n">
-        <v>2753.96</v>
+        <v>863.16</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1243,17 +1243,17 @@
         <v>46218</v>
       </c>
       <c r="B43" t="n">
-        <v>1137</v>
+        <v>945</v>
       </c>
       <c r="C43" t="n">
         <v>8888</v>
       </c>
       <c r="D43" t="n">
-        <v>1437.44</v>
+        <v>21973.45</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>PEDIDO ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -1262,17 +1262,17 @@
         <v>46218</v>
       </c>
       <c r="B44" t="n">
-        <v>2793</v>
+        <v>438</v>
       </c>
       <c r="C44" t="n">
-        <v>977</v>
+        <v>8888</v>
       </c>
       <c r="D44" t="n">
-        <v>695.72</v>
+        <v>220.06</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1281,17 +1281,17 @@
         <v>46218</v>
       </c>
       <c r="B45" t="n">
-        <v>945</v>
+        <v>353</v>
       </c>
       <c r="C45" t="n">
-        <v>8888</v>
+        <v>3179</v>
       </c>
       <c r="D45" t="n">
-        <v>1934.84</v>
+        <v>495.84</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>PEDIDO ELETRÔNICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1300,17 +1300,17 @@
         <v>46218</v>
       </c>
       <c r="B46" t="n">
-        <v>374</v>
+        <v>1293</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>22.62</v>
+        <v>3129.07</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1319,13 +1319,13 @@
         <v>46218</v>
       </c>
       <c r="B47" t="n">
-        <v>664</v>
+        <v>2279</v>
       </c>
       <c r="C47" t="n">
         <v>8888</v>
       </c>
       <c r="D47" t="n">
-        <v>1510.56</v>
+        <v>2753.96</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1338,17 +1338,17 @@
         <v>46218</v>
       </c>
       <c r="B48" t="n">
-        <v>703</v>
+        <v>1137</v>
       </c>
       <c r="C48" t="n">
         <v>8888</v>
       </c>
       <c r="D48" t="n">
-        <v>12155.46</v>
+        <v>1947.93</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1357,17 +1357,17 @@
         <v>46218</v>
       </c>
       <c r="B49" t="n">
-        <v>1937</v>
+        <v>374</v>
       </c>
       <c r="C49" t="n">
         <v>8888</v>
       </c>
       <c r="D49" t="n">
-        <v>1032.73</v>
+        <v>712.71</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1376,17 +1376,17 @@
         <v>46218</v>
       </c>
       <c r="B50" t="n">
-        <v>451</v>
+        <v>2686</v>
       </c>
       <c r="C50" t="n">
         <v>8888</v>
       </c>
       <c r="D50" t="n">
-        <v>368.93</v>
+        <v>332.6</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1395,17 +1395,17 @@
         <v>46218</v>
       </c>
       <c r="B51" t="n">
-        <v>1756</v>
+        <v>2793</v>
       </c>
       <c r="C51" t="n">
-        <v>8888</v>
+        <v>977</v>
       </c>
       <c r="D51" t="n">
-        <v>996.17</v>
+        <v>695.72</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
         <v>46218</v>
       </c>
       <c r="B52" t="n">
-        <v>1956</v>
+        <v>374</v>
       </c>
       <c r="C52" t="n">
         <v>8888</v>
       </c>
       <c r="D52" t="n">
-        <v>4557.34</v>
+        <v>22.62</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1433,13 +1433,13 @@
         <v>46218</v>
       </c>
       <c r="B53" t="n">
-        <v>925</v>
+        <v>664</v>
       </c>
       <c r="C53" t="n">
         <v>8888</v>
       </c>
       <c r="D53" t="n">
-        <v>651.59</v>
+        <v>1510.56</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1452,17 +1452,17 @@
         <v>46218</v>
       </c>
       <c r="B54" t="n">
-        <v>2631</v>
+        <v>703</v>
       </c>
       <c r="C54" t="n">
-        <v>2853</v>
+        <v>8888</v>
       </c>
       <c r="D54" t="n">
-        <v>509.88</v>
+        <v>12155.46</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1471,17 +1471,17 @@
         <v>46218</v>
       </c>
       <c r="B55" t="n">
-        <v>2648</v>
+        <v>1937</v>
       </c>
       <c r="C55" t="n">
         <v>8888</v>
       </c>
       <c r="D55" t="n">
-        <v>1594.42</v>
+        <v>1032.73</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1490,17 +1490,17 @@
         <v>46218</v>
       </c>
       <c r="B56" t="n">
-        <v>2714</v>
+        <v>451</v>
       </c>
       <c r="C56" t="n">
-        <v>519</v>
+        <v>8888</v>
       </c>
       <c r="D56" t="n">
-        <v>61939.22</v>
+        <v>368.93</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1509,17 +1509,17 @@
         <v>46218</v>
       </c>
       <c r="B57" t="n">
-        <v>483</v>
+        <v>1756</v>
       </c>
       <c r="C57" t="n">
         <v>8888</v>
       </c>
       <c r="D57" t="n">
-        <v>6625.87</v>
+        <v>996.17</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1528,13 +1528,13 @@
         <v>46218</v>
       </c>
       <c r="B58" t="n">
-        <v>1075</v>
+        <v>1956</v>
       </c>
       <c r="C58" t="n">
         <v>8888</v>
       </c>
       <c r="D58" t="n">
-        <v>11607.79</v>
+        <v>4557.34</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1547,17 +1547,17 @@
         <v>46218</v>
       </c>
       <c r="B59" t="n">
-        <v>629</v>
+        <v>925</v>
       </c>
       <c r="C59" t="n">
         <v>8888</v>
       </c>
       <c r="D59" t="n">
-        <v>9233.719999999999</v>
+        <v>651.59</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1566,13 +1566,13 @@
         <v>46218</v>
       </c>
       <c r="B60" t="n">
-        <v>1983</v>
+        <v>2631</v>
       </c>
       <c r="C60" t="n">
-        <v>841</v>
+        <v>2853</v>
       </c>
       <c r="D60" t="n">
-        <v>243.92</v>
+        <v>509.88</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1585,17 +1585,17 @@
         <v>46218</v>
       </c>
       <c r="B61" t="n">
-        <v>1137</v>
+        <v>2648</v>
       </c>
       <c r="C61" t="n">
         <v>8888</v>
       </c>
       <c r="D61" t="n">
-        <v>3578.51</v>
+        <v>1594.42</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1604,17 +1604,17 @@
         <v>46218</v>
       </c>
       <c r="B62" t="n">
-        <v>2651</v>
+        <v>2714</v>
       </c>
       <c r="C62" t="n">
-        <v>8888</v>
+        <v>519</v>
       </c>
       <c r="D62" t="n">
-        <v>1296.58</v>
+        <v>61939.22</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1623,17 +1623,17 @@
         <v>46218</v>
       </c>
       <c r="B63" t="n">
-        <v>1956</v>
+        <v>483</v>
       </c>
       <c r="C63" t="n">
-        <v>423</v>
+        <v>8888</v>
       </c>
       <c r="D63" t="n">
-        <v>455.37</v>
+        <v>6625.87</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1642,17 +1642,17 @@
         <v>46218</v>
       </c>
       <c r="B64" t="n">
-        <v>2709</v>
+        <v>1075</v>
       </c>
       <c r="C64" t="n">
         <v>8888</v>
       </c>
       <c r="D64" t="n">
-        <v>547.6900000000001</v>
+        <v>11607.79</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1661,13 +1661,13 @@
         <v>46218</v>
       </c>
       <c r="B65" t="n">
-        <v>2026</v>
+        <v>629</v>
       </c>
       <c r="C65" t="n">
         <v>8888</v>
       </c>
       <c r="D65" t="n">
-        <v>2237.62</v>
+        <v>9233.719999999999</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1680,13 +1680,13 @@
         <v>46218</v>
       </c>
       <c r="B66" t="n">
-        <v>89</v>
+        <v>1983</v>
       </c>
       <c r="C66" t="n">
-        <v>13148</v>
+        <v>841</v>
       </c>
       <c r="D66" t="n">
-        <v>1883.74</v>
+        <v>243.92</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1699,17 +1699,17 @@
         <v>46218</v>
       </c>
       <c r="B67" t="n">
-        <v>2709</v>
+        <v>1137</v>
       </c>
       <c r="C67" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D67" t="n">
-        <v>390.19</v>
+        <v>3578.51</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1718,17 +1718,17 @@
         <v>46218</v>
       </c>
       <c r="B68" t="n">
-        <v>2345</v>
+        <v>2651</v>
       </c>
       <c r="C68" t="n">
         <v>8888</v>
       </c>
       <c r="D68" t="n">
-        <v>748.86</v>
+        <v>1296.58</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1737,17 +1737,17 @@
         <v>46218</v>
       </c>
       <c r="B69" t="n">
-        <v>1308</v>
+        <v>1956</v>
       </c>
       <c r="C69" t="n">
-        <v>8888</v>
+        <v>423</v>
       </c>
       <c r="D69" t="n">
-        <v>276.16</v>
+        <v>455.37</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1756,17 +1756,17 @@
         <v>46218</v>
       </c>
       <c r="B70" t="n">
-        <v>2308</v>
+        <v>2709</v>
       </c>
       <c r="C70" t="n">
         <v>8888</v>
       </c>
       <c r="D70" t="n">
-        <v>488.69</v>
+        <v>547.6900000000001</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1775,17 @@
         <v>46218</v>
       </c>
       <c r="B71" t="n">
-        <v>360</v>
+        <v>2026</v>
       </c>
       <c r="C71" t="n">
-        <v>546</v>
+        <v>8888</v>
       </c>
       <c r="D71" t="n">
-        <v>709.75</v>
+        <v>2237.62</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1794,17 +1794,17 @@
         <v>46218</v>
       </c>
       <c r="B72" t="n">
-        <v>2211</v>
+        <v>2789</v>
       </c>
       <c r="C72" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D72" t="n">
-        <v>1526.94</v>
+        <v>747.77</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1813,17 +1813,17 @@
         <v>46218</v>
       </c>
       <c r="B73" t="n">
-        <v>559</v>
+        <v>89</v>
       </c>
       <c r="C73" t="n">
-        <v>8888</v>
+        <v>13148</v>
       </c>
       <c r="D73" t="n">
-        <v>859.92</v>
+        <v>1883.74</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1832,17 +1832,17 @@
         <v>46218</v>
       </c>
       <c r="B74" t="n">
-        <v>569</v>
+        <v>2709</v>
       </c>
       <c r="C74" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D74" t="n">
-        <v>673.01</v>
+        <v>390.19</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1851,17 +1851,17 @@
         <v>46218</v>
       </c>
       <c r="B75" t="n">
-        <v>890</v>
+        <v>2345</v>
       </c>
       <c r="C75" t="n">
         <v>8888</v>
       </c>
       <c r="D75" t="n">
-        <v>387.2</v>
+        <v>748.86</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1870,13 +1870,13 @@
         <v>46218</v>
       </c>
       <c r="B76" t="n">
-        <v>1063</v>
+        <v>1308</v>
       </c>
       <c r="C76" t="n">
         <v>8888</v>
       </c>
       <c r="D76" t="n">
-        <v>4487.11</v>
+        <v>276.16</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -1889,13 +1889,13 @@
         <v>46218</v>
       </c>
       <c r="B77" t="n">
-        <v>2279</v>
+        <v>360</v>
       </c>
       <c r="C77" t="n">
-        <v>1139</v>
+        <v>546</v>
       </c>
       <c r="D77" t="n">
-        <v>652.51</v>
+        <v>1609.68</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -1908,17 +1908,17 @@
         <v>46218</v>
       </c>
       <c r="B78" t="n">
-        <v>1299</v>
+        <v>2308</v>
       </c>
       <c r="C78" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D78" t="n">
-        <v>1435.52</v>
+        <v>488.69</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1927,13 +1927,13 @@
         <v>46218</v>
       </c>
       <c r="B79" t="n">
-        <v>1478</v>
+        <v>2211</v>
       </c>
       <c r="C79" t="n">
-        <v>675</v>
+        <v>874</v>
       </c>
       <c r="D79" t="n">
-        <v>1600.01</v>
+        <v>1526.94</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -1946,17 +1946,17 @@
         <v>46218</v>
       </c>
       <c r="B80" t="n">
-        <v>285</v>
+        <v>559</v>
       </c>
       <c r="C80" t="n">
         <v>8888</v>
       </c>
       <c r="D80" t="n">
-        <v>3349.8</v>
+        <v>859.92</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1965,13 +1965,13 @@
         <v>46218</v>
       </c>
       <c r="B81" t="n">
-        <v>1983</v>
+        <v>569</v>
       </c>
       <c r="C81" t="n">
         <v>8888</v>
       </c>
       <c r="D81" t="n">
-        <v>2451.28</v>
+        <v>673.01</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -1984,17 +1984,17 @@
         <v>46218</v>
       </c>
       <c r="B82" t="n">
-        <v>477</v>
+        <v>890</v>
       </c>
       <c r="C82" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D82" t="n">
-        <v>1540.55</v>
+        <v>387.2</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2009,11 +2009,11 @@
         <v>8888</v>
       </c>
       <c r="D83" t="n">
-        <v>2549.86</v>
+        <v>4487.11</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2022,17 +2022,17 @@
         <v>46218</v>
       </c>
       <c r="B84" t="n">
-        <v>424</v>
+        <v>2279</v>
       </c>
       <c r="C84" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D84" t="n">
-        <v>1035.17</v>
+        <v>652.51</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2041,17 +2041,17 @@
         <v>46218</v>
       </c>
       <c r="B85" t="n">
-        <v>675</v>
+        <v>1299</v>
       </c>
       <c r="C85" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D85" t="n">
-        <v>616.73</v>
+        <v>1435.52</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2060,17 +2060,17 @@
         <v>46218</v>
       </c>
       <c r="B86" t="n">
-        <v>2768</v>
+        <v>1478</v>
       </c>
       <c r="C86" t="n">
-        <v>8888</v>
+        <v>675</v>
       </c>
       <c r="D86" t="n">
-        <v>4245.73</v>
+        <v>1600.01</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2079,17 +2079,17 @@
         <v>46218</v>
       </c>
       <c r="B87" t="n">
-        <v>1993</v>
+        <v>285</v>
       </c>
       <c r="C87" t="n">
         <v>8888</v>
       </c>
       <c r="D87" t="n">
-        <v>362.63</v>
+        <v>3349.8</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2098,17 +2098,17 @@
         <v>46218</v>
       </c>
       <c r="B88" t="n">
-        <v>1465</v>
+        <v>1983</v>
       </c>
       <c r="C88" t="n">
         <v>8888</v>
       </c>
       <c r="D88" t="n">
-        <v>3373.83</v>
+        <v>2451.28</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2117,17 +2117,17 @@
         <v>46218</v>
       </c>
       <c r="B89" t="n">
-        <v>89</v>
+        <v>477</v>
       </c>
       <c r="C89" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D89" t="n">
-        <v>479</v>
+        <v>1540.55</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2136,17 +2136,17 @@
         <v>46218</v>
       </c>
       <c r="B90" t="n">
-        <v>595</v>
+        <v>1063</v>
       </c>
       <c r="C90" t="n">
         <v>8888</v>
       </c>
       <c r="D90" t="n">
-        <v>18084.5</v>
+        <v>2549.86</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2155,17 +2155,17 @@
         <v>46218</v>
       </c>
       <c r="B91" t="n">
-        <v>2696</v>
+        <v>424</v>
       </c>
       <c r="C91" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D91" t="n">
-        <v>259.97</v>
+        <v>1035.17</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2174,13 +2174,13 @@
         <v>46218</v>
       </c>
       <c r="B92" t="n">
-        <v>360</v>
+        <v>675</v>
       </c>
       <c r="C92" t="n">
         <v>8888</v>
       </c>
       <c r="D92" t="n">
-        <v>2023.17</v>
+        <v>616.73</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2193,17 +2193,17 @@
         <v>46218</v>
       </c>
       <c r="B93" t="n">
-        <v>1465</v>
+        <v>2768</v>
       </c>
       <c r="C93" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D93" t="n">
-        <v>777.2</v>
+        <v>5607.14</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2212,17 +2212,17 @@
         <v>46218</v>
       </c>
       <c r="B94" t="n">
-        <v>947</v>
+        <v>1993</v>
       </c>
       <c r="C94" t="n">
         <v>8888</v>
       </c>
       <c r="D94" t="n">
-        <v>2087.97</v>
+        <v>362.63</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>PEDIDO ELETRÔNICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2231,17 +2231,17 @@
         <v>46218</v>
       </c>
       <c r="B95" t="n">
-        <v>2178</v>
+        <v>1465</v>
       </c>
       <c r="C95" t="n">
         <v>8888</v>
       </c>
       <c r="D95" t="n">
-        <v>619.92</v>
+        <v>3373.83</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2250,17 +2250,17 @@
         <v>46218</v>
       </c>
       <c r="B96" t="n">
-        <v>630</v>
+        <v>89</v>
       </c>
       <c r="C96" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D96" t="n">
-        <v>1801.63</v>
+        <v>479</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2269,17 +2269,17 @@
         <v>46218</v>
       </c>
       <c r="B97" t="n">
-        <v>1937</v>
+        <v>595</v>
       </c>
       <c r="C97" t="n">
         <v>8888</v>
       </c>
       <c r="D97" t="n">
-        <v>2132.95</v>
+        <v>18084.5</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2288,17 +2288,17 @@
         <v>46218</v>
       </c>
       <c r="B98" t="n">
-        <v>2577</v>
+        <v>2696</v>
       </c>
       <c r="C98" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D98" t="n">
-        <v>1647.08</v>
+        <v>1597.76</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2307,17 +2307,17 @@
         <v>46218</v>
       </c>
       <c r="B99" t="n">
-        <v>1293</v>
+        <v>360</v>
       </c>
       <c r="C99" t="n">
         <v>8888</v>
       </c>
       <c r="D99" t="n">
-        <v>1607.2</v>
+        <v>4596.89</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2326,17 +2326,17 @@
         <v>46218</v>
       </c>
       <c r="B100" t="n">
-        <v>1317</v>
+        <v>1465</v>
       </c>
       <c r="C100" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D100" t="n">
-        <v>907.72</v>
+        <v>777.2</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2345,17 +2345,17 @@
         <v>46218</v>
       </c>
       <c r="B101" t="n">
-        <v>2571</v>
+        <v>947</v>
       </c>
       <c r="C101" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D101" t="n">
-        <v>268.53</v>
+        <v>2087.97</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>PEDIDO ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -2364,17 +2364,17 @@
         <v>46218</v>
       </c>
       <c r="B102" t="n">
-        <v>1937</v>
+        <v>2178</v>
       </c>
       <c r="C102" t="n">
         <v>8888</v>
       </c>
       <c r="D102" t="n">
-        <v>1803.32</v>
+        <v>619.92</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2383,17 +2383,17 @@
         <v>46218</v>
       </c>
       <c r="B103" t="n">
-        <v>1063</v>
+        <v>630</v>
       </c>
       <c r="C103" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D103" t="n">
-        <v>1113.08</v>
+        <v>1801.63</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2402,17 +2402,17 @@
         <v>46218</v>
       </c>
       <c r="B104" t="n">
-        <v>1906</v>
+        <v>1937</v>
       </c>
       <c r="C104" t="n">
         <v>8888</v>
       </c>
       <c r="D104" t="n">
-        <v>990.22</v>
+        <v>2132.95</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2421,13 +2421,13 @@
         <v>46218</v>
       </c>
       <c r="B105" t="n">
-        <v>1756</v>
+        <v>2577</v>
       </c>
       <c r="C105" t="n">
         <v>8888</v>
       </c>
       <c r="D105" t="n">
-        <v>1357.12</v>
+        <v>1647.08</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2440,17 +2440,17 @@
         <v>46218</v>
       </c>
       <c r="B106" t="n">
-        <v>20</v>
+        <v>1293</v>
       </c>
       <c r="C106" t="n">
         <v>8888</v>
       </c>
       <c r="D106" t="n">
-        <v>276.64</v>
+        <v>2135.89</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2459,17 +2459,17 @@
         <v>46218</v>
       </c>
       <c r="B107" t="n">
-        <v>477</v>
+        <v>2026</v>
       </c>
       <c r="C107" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D107" t="n">
-        <v>372.69</v>
+        <v>1680.89</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2478,17 +2478,17 @@
         <v>46218</v>
       </c>
       <c r="B108" t="n">
-        <v>477</v>
+        <v>2607</v>
       </c>
       <c r="C108" t="n">
         <v>8888</v>
       </c>
       <c r="D108" t="n">
-        <v>707.52</v>
+        <v>490.31</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2497,13 +2497,13 @@
         <v>46218</v>
       </c>
       <c r="B109" t="n">
-        <v>2660</v>
+        <v>1317</v>
       </c>
       <c r="C109" t="n">
         <v>8888</v>
       </c>
       <c r="D109" t="n">
-        <v>2684.97</v>
+        <v>907.72</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -2516,17 +2516,17 @@
         <v>46218</v>
       </c>
       <c r="B110" t="n">
-        <v>569</v>
+        <v>2571</v>
       </c>
       <c r="C110" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D110" t="n">
-        <v>18512.6</v>
+        <v>268.53</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2535,17 +2535,17 @@
         <v>46218</v>
       </c>
       <c r="B111" t="n">
-        <v>2089</v>
+        <v>1937</v>
       </c>
       <c r="C111" t="n">
-        <v>1533</v>
+        <v>8888</v>
       </c>
       <c r="D111" t="n">
-        <v>969.24</v>
+        <v>1803.32</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2554,17 +2554,17 @@
         <v>46218</v>
       </c>
       <c r="B112" t="n">
-        <v>1007</v>
+        <v>1063</v>
       </c>
       <c r="C112" t="n">
         <v>8888</v>
       </c>
       <c r="D112" t="n">
-        <v>241.44</v>
+        <v>1113.08</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2573,17 +2573,17 @@
         <v>46218</v>
       </c>
       <c r="B113" t="n">
-        <v>1380</v>
+        <v>2631</v>
       </c>
       <c r="C113" t="n">
         <v>8888</v>
       </c>
       <c r="D113" t="n">
-        <v>520.2</v>
+        <v>1447.86</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2592,13 +2592,13 @@
         <v>46218</v>
       </c>
       <c r="B114" t="n">
-        <v>1102</v>
+        <v>1906</v>
       </c>
       <c r="C114" t="n">
         <v>8888</v>
       </c>
       <c r="D114" t="n">
-        <v>1137.04</v>
+        <v>2774.84</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -2611,13 +2611,13 @@
         <v>46218</v>
       </c>
       <c r="B115" t="n">
-        <v>1075</v>
+        <v>1756</v>
       </c>
       <c r="C115" t="n">
         <v>8888</v>
       </c>
       <c r="D115" t="n">
-        <v>2179.03</v>
+        <v>1357.12</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -2630,17 +2630,17 @@
         <v>46218</v>
       </c>
       <c r="B116" t="n">
-        <v>2245</v>
+        <v>20</v>
       </c>
       <c r="C116" t="n">
         <v>8888</v>
       </c>
       <c r="D116" t="n">
-        <v>361.58</v>
+        <v>276.64</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2649,17 +2649,17 @@
         <v>46218</v>
       </c>
       <c r="B117" t="n">
-        <v>132</v>
+        <v>477</v>
       </c>
       <c r="C117" t="n">
         <v>8888</v>
       </c>
       <c r="D117" t="n">
-        <v>6522.92</v>
+        <v>372.69</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2668,17 +2668,17 @@
         <v>46218</v>
       </c>
       <c r="B118" t="n">
-        <v>452</v>
+        <v>477</v>
       </c>
       <c r="C118" t="n">
         <v>8888</v>
       </c>
       <c r="D118" t="n">
-        <v>608.78</v>
+        <v>707.52</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2687,17 +2687,17 @@
         <v>46218</v>
       </c>
       <c r="B119" t="n">
-        <v>1293</v>
+        <v>2660</v>
       </c>
       <c r="C119" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D119" t="n">
-        <v>1780.93</v>
+        <v>2684.97</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2706,17 +2706,17 @@
         <v>46218</v>
       </c>
       <c r="B120" t="n">
-        <v>525</v>
+        <v>569</v>
       </c>
       <c r="C120" t="n">
         <v>8888</v>
       </c>
       <c r="D120" t="n">
-        <v>5658.57</v>
+        <v>19352.11</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2725,17 +2725,17 @@
         <v>46218</v>
       </c>
       <c r="B121" t="n">
-        <v>609</v>
+        <v>2089</v>
       </c>
       <c r="C121" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D121" t="n">
-        <v>886.1</v>
+        <v>969.24</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2744,17 +2744,17 @@
         <v>46218</v>
       </c>
       <c r="B122" t="n">
-        <v>619</v>
+        <v>1007</v>
       </c>
       <c r="C122" t="n">
         <v>8888</v>
       </c>
       <c r="D122" t="n">
-        <v>2330.47</v>
+        <v>241.44</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2763,13 +2763,13 @@
         <v>46218</v>
       </c>
       <c r="B123" t="n">
-        <v>58</v>
+        <v>1380</v>
       </c>
       <c r="C123" t="n">
         <v>8888</v>
       </c>
       <c r="D123" t="n">
-        <v>1123.87</v>
+        <v>520.2</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -2782,17 +2782,17 @@
         <v>46218</v>
       </c>
       <c r="B124" t="n">
-        <v>358</v>
+        <v>1102</v>
       </c>
       <c r="C124" t="n">
         <v>8888</v>
       </c>
       <c r="D124" t="n">
-        <v>1675.95</v>
+        <v>1137.04</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2801,13 +2801,13 @@
         <v>46218</v>
       </c>
       <c r="B125" t="n">
-        <v>2431</v>
+        <v>1075</v>
       </c>
       <c r="C125" t="n">
         <v>8888</v>
       </c>
       <c r="D125" t="n">
-        <v>266.89</v>
+        <v>2179.03</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -2820,13 +2820,13 @@
         <v>46218</v>
       </c>
       <c r="B126" t="n">
-        <v>285</v>
+        <v>2245</v>
       </c>
       <c r="C126" t="n">
         <v>8888</v>
       </c>
       <c r="D126" t="n">
-        <v>2090.81</v>
+        <v>361.58</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -2839,17 +2839,17 @@
         <v>46218</v>
       </c>
       <c r="B127" t="n">
-        <v>1102</v>
+        <v>132</v>
       </c>
       <c r="C127" t="n">
         <v>8888</v>
       </c>
       <c r="D127" t="n">
-        <v>1119.32</v>
+        <v>6522.92</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2858,17 +2858,17 @@
         <v>46218</v>
       </c>
       <c r="B128" t="n">
-        <v>626</v>
+        <v>452</v>
       </c>
       <c r="C128" t="n">
         <v>8888</v>
       </c>
       <c r="D128" t="n">
-        <v>11337.75</v>
+        <v>608.78</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2877,13 +2877,13 @@
         <v>46218</v>
       </c>
       <c r="B129" t="n">
-        <v>1137</v>
+        <v>1293</v>
       </c>
       <c r="C129" t="n">
-        <v>2220</v>
+        <v>1281</v>
       </c>
       <c r="D129" t="n">
-        <v>1370.86</v>
+        <v>1780.93</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -2896,17 +2896,17 @@
         <v>46218</v>
       </c>
       <c r="B130" t="n">
-        <v>1756</v>
+        <v>525</v>
       </c>
       <c r="C130" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D130" t="n">
-        <v>5078.1</v>
+        <v>5658.57</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2915,17 +2915,17 @@
         <v>46218</v>
       </c>
       <c r="B131" t="n">
-        <v>2651</v>
+        <v>2641</v>
       </c>
       <c r="C131" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D131" t="n">
-        <v>363.7</v>
+        <v>1720.99</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2934,17 +2934,17 @@
         <v>46218</v>
       </c>
       <c r="B132" t="n">
-        <v>360</v>
+        <v>609</v>
       </c>
       <c r="C132" t="n">
         <v>8888</v>
       </c>
       <c r="D132" t="n">
-        <v>1594.84</v>
+        <v>886.1</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2953,17 +2953,17 @@
         <v>46218</v>
       </c>
       <c r="B133" t="n">
-        <v>2582</v>
+        <v>619</v>
       </c>
       <c r="C133" t="n">
         <v>8888</v>
       </c>
       <c r="D133" t="n">
-        <v>379.33</v>
+        <v>2330.47</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2972,17 +2972,17 @@
         <v>46218</v>
       </c>
       <c r="B134" t="n">
-        <v>1756</v>
+        <v>2697</v>
       </c>
       <c r="C134" t="n">
         <v>8888</v>
       </c>
       <c r="D134" t="n">
-        <v>1715.26</v>
+        <v>418.65</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2991,13 +2991,13 @@
         <v>46218</v>
       </c>
       <c r="B135" t="n">
-        <v>1254</v>
+        <v>58</v>
       </c>
       <c r="C135" t="n">
         <v>8888</v>
       </c>
       <c r="D135" t="n">
-        <v>855.76</v>
+        <v>1123.87</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3010,17 +3010,17 @@
         <v>46218</v>
       </c>
       <c r="B136" t="n">
-        <v>1289</v>
+        <v>358</v>
       </c>
       <c r="C136" t="n">
         <v>8888</v>
       </c>
       <c r="D136" t="n">
-        <v>2396.98</v>
+        <v>1675.95</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3029,17 +3029,17 @@
         <v>46218</v>
       </c>
       <c r="B137" t="n">
-        <v>2015</v>
+        <v>2431</v>
       </c>
       <c r="C137" t="n">
         <v>8888</v>
       </c>
       <c r="D137" t="n">
-        <v>315.69</v>
+        <v>266.89</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3048,17 +3048,17 @@
         <v>46218</v>
       </c>
       <c r="B138" t="n">
-        <v>1064</v>
+        <v>285</v>
       </c>
       <c r="C138" t="n">
         <v>8888</v>
       </c>
       <c r="D138" t="n">
-        <v>1274.3</v>
+        <v>2090.81</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3067,17 +3067,17 @@
         <v>46218</v>
       </c>
       <c r="B139" t="n">
-        <v>2698</v>
+        <v>1102</v>
       </c>
       <c r="C139" t="n">
         <v>8888</v>
       </c>
       <c r="D139" t="n">
-        <v>552.15</v>
+        <v>1119.32</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3086,17 +3086,17 @@
         <v>46218</v>
       </c>
       <c r="B140" t="n">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="C140" t="n">
         <v>8888</v>
       </c>
       <c r="D140" t="n">
-        <v>3035.38</v>
+        <v>11881.87</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3105,17 +3105,17 @@
         <v>46218</v>
       </c>
       <c r="B141" t="n">
-        <v>664</v>
+        <v>1137</v>
       </c>
       <c r="C141" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D141" t="n">
-        <v>4973.15</v>
+        <v>1370.86</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3130,7 @@
         <v>1929</v>
       </c>
       <c r="D142" t="n">
-        <v>521.79</v>
+        <v>2066.36</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3143,17 +3143,17 @@
         <v>46218</v>
       </c>
       <c r="B143" t="n">
-        <v>2584</v>
+        <v>1756</v>
       </c>
       <c r="C143" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D143" t="n">
-        <v>1852.83</v>
+        <v>5078.1</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3162,17 +3162,17 @@
         <v>46218</v>
       </c>
       <c r="B144" t="n">
-        <v>2641</v>
+        <v>2651</v>
       </c>
       <c r="C144" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D144" t="n">
-        <v>820</v>
+        <v>363.7</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3181,17 +3181,17 @@
         <v>46218</v>
       </c>
       <c r="B145" t="n">
-        <v>816</v>
+        <v>360</v>
       </c>
       <c r="C145" t="n">
         <v>8888</v>
       </c>
       <c r="D145" t="n">
-        <v>438.24</v>
+        <v>1594.84</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3200,17 +3200,17 @@
         <v>46218</v>
       </c>
       <c r="B146" t="n">
-        <v>285</v>
+        <v>2582</v>
       </c>
       <c r="C146" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D146" t="n">
-        <v>364.99</v>
+        <v>379.33</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3219,17 +3219,17 @@
         <v>46218</v>
       </c>
       <c r="B147" t="n">
-        <v>2114</v>
+        <v>1756</v>
       </c>
       <c r="C147" t="n">
         <v>8888</v>
       </c>
       <c r="D147" t="n">
-        <v>2726.04</v>
+        <v>1715.26</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3238,17 +3238,17 @@
         <v>46218</v>
       </c>
       <c r="B148" t="n">
-        <v>953</v>
+        <v>1254</v>
       </c>
       <c r="C148" t="n">
         <v>8888</v>
       </c>
       <c r="D148" t="n">
-        <v>2618.89</v>
+        <v>855.76</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3257,17 +3257,17 @@
         <v>46218</v>
       </c>
       <c r="B149" t="n">
-        <v>1102</v>
+        <v>1289</v>
       </c>
       <c r="C149" t="n">
         <v>8888</v>
       </c>
       <c r="D149" t="n">
-        <v>2344.41</v>
+        <v>2396.98</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3276,13 +3276,13 @@
         <v>46218</v>
       </c>
       <c r="B150" t="n">
-        <v>619</v>
+        <v>2015</v>
       </c>
       <c r="C150" t="n">
         <v>8888</v>
       </c>
       <c r="D150" t="n">
-        <v>2021.67</v>
+        <v>315.69</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -3295,17 +3295,17 @@
         <v>46218</v>
       </c>
       <c r="B151" t="n">
-        <v>1465</v>
+        <v>1064</v>
       </c>
       <c r="C151" t="n">
         <v>8888</v>
       </c>
       <c r="D151" t="n">
-        <v>3504</v>
+        <v>1274.3</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3314,17 +3314,17 @@
         <v>46218</v>
       </c>
       <c r="B152" t="n">
-        <v>2767</v>
+        <v>2698</v>
       </c>
       <c r="C152" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D152" t="n">
-        <v>1135.64</v>
+        <v>552.15</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3333,13 +3333,13 @@
         <v>46218</v>
       </c>
       <c r="B153" t="n">
-        <v>2245</v>
+        <v>629</v>
       </c>
       <c r="C153" t="n">
         <v>8888</v>
       </c>
       <c r="D153" t="n">
-        <v>427.51</v>
+        <v>3035.38</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -3352,13 +3352,13 @@
         <v>46218</v>
       </c>
       <c r="B154" t="n">
-        <v>2197</v>
+        <v>664</v>
       </c>
       <c r="C154" t="n">
         <v>8888</v>
       </c>
       <c r="D154" t="n">
-        <v>1085.45</v>
+        <v>4973.15</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -3371,17 +3371,17 @@
         <v>46218</v>
       </c>
       <c r="B155" t="n">
-        <v>2657</v>
+        <v>2584</v>
       </c>
       <c r="C155" t="n">
         <v>8888</v>
       </c>
       <c r="D155" t="n">
-        <v>1187.68</v>
+        <v>1852.83</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3390,17 +3390,17 @@
         <v>46218</v>
       </c>
       <c r="B156" t="n">
-        <v>1277</v>
+        <v>2641</v>
       </c>
       <c r="C156" t="n">
         <v>8888</v>
       </c>
       <c r="D156" t="n">
-        <v>1949</v>
+        <v>820</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3409,17 +3409,17 @@
         <v>46218</v>
       </c>
       <c r="B157" t="n">
-        <v>131</v>
+        <v>429</v>
       </c>
       <c r="C157" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D157" t="n">
-        <v>1268.57</v>
+        <v>2593.49</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3428,17 +3428,17 @@
         <v>46218</v>
       </c>
       <c r="B158" t="n">
-        <v>2692</v>
+        <v>816</v>
       </c>
       <c r="C158" t="n">
         <v>8888</v>
       </c>
       <c r="D158" t="n">
-        <v>731.28</v>
+        <v>438.24</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3447,17 +3447,17 @@
         <v>46218</v>
       </c>
       <c r="B159" t="n">
-        <v>1317</v>
+        <v>2359</v>
       </c>
       <c r="C159" t="n">
-        <v>3179</v>
+        <v>8888</v>
       </c>
       <c r="D159" t="n">
-        <v>991.6799999999999</v>
+        <v>381.95</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3466,17 +3466,17 @@
         <v>46218</v>
       </c>
       <c r="B160" t="n">
-        <v>1993</v>
+        <v>285</v>
       </c>
       <c r="C160" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D160" t="n">
-        <v>2875.39</v>
+        <v>364.99</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3485,13 +3485,13 @@
         <v>46218</v>
       </c>
       <c r="B161" t="n">
-        <v>1632</v>
+        <v>2114</v>
       </c>
       <c r="C161" t="n">
         <v>8888</v>
       </c>
       <c r="D161" t="n">
-        <v>564.55</v>
+        <v>2726.04</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -3504,17 +3504,17 @@
         <v>46218</v>
       </c>
       <c r="B162" t="n">
-        <v>1890</v>
+        <v>953</v>
       </c>
       <c r="C162" t="n">
-        <v>3449</v>
+        <v>8888</v>
       </c>
       <c r="D162" t="n">
-        <v>3590.04</v>
+        <v>2618.89</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3523,17 +3523,17 @@
         <v>46218</v>
       </c>
       <c r="B163" t="n">
-        <v>451</v>
+        <v>1102</v>
       </c>
       <c r="C163" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D163" t="n">
-        <v>445.58</v>
+        <v>2344.41</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3542,13 +3542,13 @@
         <v>46218</v>
       </c>
       <c r="B164" t="n">
-        <v>2749</v>
+        <v>619</v>
       </c>
       <c r="C164" t="n">
         <v>8888</v>
       </c>
       <c r="D164" t="n">
-        <v>1860.64</v>
+        <v>2021.67</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -3561,17 +3561,17 @@
         <v>46218</v>
       </c>
       <c r="B165" t="n">
-        <v>1117</v>
+        <v>1465</v>
       </c>
       <c r="C165" t="n">
         <v>8888</v>
       </c>
       <c r="D165" t="n">
-        <v>342.2</v>
+        <v>3504</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3580,17 +3580,17 @@
         <v>46218</v>
       </c>
       <c r="B166" t="n">
-        <v>1478</v>
+        <v>2767</v>
       </c>
       <c r="C166" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D166" t="n">
-        <v>875.34</v>
+        <v>1135.64</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3599,13 +3599,13 @@
         <v>46218</v>
       </c>
       <c r="B167" t="n">
-        <v>2491</v>
+        <v>2245</v>
       </c>
       <c r="C167" t="n">
         <v>8888</v>
       </c>
       <c r="D167" t="n">
-        <v>650.4299999999999</v>
+        <v>427.51</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -3618,17 +3618,17 @@
         <v>46218</v>
       </c>
       <c r="B168" t="n">
-        <v>2015</v>
+        <v>2197</v>
       </c>
       <c r="C168" t="n">
         <v>8888</v>
       </c>
       <c r="D168" t="n">
-        <v>4436.15</v>
+        <v>1085.45</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3637,17 +3637,17 @@
         <v>46218</v>
       </c>
       <c r="B169" t="n">
-        <v>1890</v>
+        <v>2657</v>
       </c>
       <c r="C169" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D169" t="n">
-        <v>500.92</v>
+        <v>2683.06</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3656,13 +3656,13 @@
         <v>46218</v>
       </c>
       <c r="B170" t="n">
-        <v>2782</v>
+        <v>1277</v>
       </c>
       <c r="C170" t="n">
         <v>8888</v>
       </c>
       <c r="D170" t="n">
-        <v>1786.32</v>
+        <v>1949</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -3675,13 +3675,13 @@
         <v>46218</v>
       </c>
       <c r="B171" t="n">
-        <v>483</v>
+        <v>131</v>
       </c>
       <c r="C171" t="n">
-        <v>841</v>
+        <v>27</v>
       </c>
       <c r="D171" t="n">
-        <v>1393.15</v>
+        <v>1268.57</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -3694,17 +3694,17 @@
         <v>46218</v>
       </c>
       <c r="B172" t="n">
-        <v>2133</v>
+        <v>2692</v>
       </c>
       <c r="C172" t="n">
-        <v>213</v>
+        <v>8888</v>
       </c>
       <c r="D172" t="n">
-        <v>526.8</v>
+        <v>731.28</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3713,13 +3713,13 @@
         <v>46218</v>
       </c>
       <c r="B173" t="n">
-        <v>351</v>
+        <v>1317</v>
       </c>
       <c r="C173" t="n">
-        <v>3009</v>
+        <v>3179</v>
       </c>
       <c r="D173" t="n">
-        <v>416.36</v>
+        <v>991.6799999999999</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -3732,17 +3732,17 @@
         <v>46218</v>
       </c>
       <c r="B174" t="n">
-        <v>2250</v>
+        <v>1993</v>
       </c>
       <c r="C174" t="n">
         <v>8888</v>
       </c>
       <c r="D174" t="n">
-        <v>709.46</v>
+        <v>2875.39</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3751,13 +3751,13 @@
         <v>46218</v>
       </c>
       <c r="B175" t="n">
-        <v>2648</v>
+        <v>1632</v>
       </c>
       <c r="C175" t="n">
         <v>8888</v>
       </c>
       <c r="D175" t="n">
-        <v>1873.52</v>
+        <v>564.55</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -3770,17 +3770,17 @@
         <v>46218</v>
       </c>
       <c r="B176" t="n">
-        <v>131</v>
+        <v>1890</v>
       </c>
       <c r="C176" t="n">
-        <v>8888</v>
+        <v>3449</v>
       </c>
       <c r="D176" t="n">
-        <v>1369.91</v>
+        <v>3590.04</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3789,13 +3789,13 @@
         <v>46218</v>
       </c>
       <c r="B177" t="n">
-        <v>2639</v>
+        <v>451</v>
       </c>
       <c r="C177" t="n">
-        <v>1953</v>
+        <v>3403</v>
       </c>
       <c r="D177" t="n">
-        <v>504.09</v>
+        <v>445.58</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -3808,17 +3808,17 @@
         <v>46218</v>
       </c>
       <c r="B178" t="n">
-        <v>2109</v>
+        <v>2749</v>
       </c>
       <c r="C178" t="n">
         <v>8888</v>
       </c>
       <c r="D178" t="n">
-        <v>2293.78</v>
+        <v>1860.64</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3827,17 +3827,17 @@
         <v>46218</v>
       </c>
       <c r="B179" t="n">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="C179" t="n">
         <v>8888</v>
       </c>
       <c r="D179" t="n">
-        <v>2919.53</v>
+        <v>342.2</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3846,17 +3846,17 @@
         <v>46218</v>
       </c>
       <c r="B180" t="n">
-        <v>2250</v>
+        <v>1478</v>
       </c>
       <c r="C180" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D180" t="n">
-        <v>1803.76</v>
+        <v>875.34</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3865,13 +3865,13 @@
         <v>46218</v>
       </c>
       <c r="B181" t="n">
-        <v>353</v>
+        <v>2491</v>
       </c>
       <c r="C181" t="n">
         <v>8888</v>
       </c>
       <c r="D181" t="n">
-        <v>108.6</v>
+        <v>650.4299999999999</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -3884,17 +3884,17 @@
         <v>46218</v>
       </c>
       <c r="B182" t="n">
-        <v>2698</v>
+        <v>2015</v>
       </c>
       <c r="C182" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D182" t="n">
-        <v>1230.43</v>
+        <v>4436.15</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3903,17 +3903,17 @@
         <v>46218</v>
       </c>
       <c r="B183" t="n">
-        <v>42</v>
+        <v>1890</v>
       </c>
       <c r="C183" t="n">
-        <v>8888</v>
+        <v>1953</v>
       </c>
       <c r="D183" t="n">
-        <v>79947.14999999999</v>
+        <v>1674.57</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3922,13 +3922,13 @@
         <v>46218</v>
       </c>
       <c r="B184" t="n">
-        <v>772</v>
+        <v>2782</v>
       </c>
       <c r="C184" t="n">
         <v>8888</v>
       </c>
       <c r="D184" t="n">
-        <v>400.25</v>
+        <v>1786.32</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -3941,17 +3941,17 @@
         <v>46218</v>
       </c>
       <c r="B185" t="n">
-        <v>2728</v>
+        <v>483</v>
       </c>
       <c r="C185" t="n">
-        <v>8888</v>
+        <v>841</v>
       </c>
       <c r="D185" t="n">
-        <v>1397.07</v>
+        <v>1393.15</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3960,13 +3960,13 @@
         <v>46218</v>
       </c>
       <c r="B186" t="n">
-        <v>2716</v>
+        <v>2133</v>
       </c>
       <c r="C186" t="n">
-        <v>1929</v>
+        <v>213</v>
       </c>
       <c r="D186" t="n">
-        <v>750.4299999999999</v>
+        <v>526.8</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -3979,13 +3979,13 @@
         <v>46218</v>
       </c>
       <c r="B187" t="n">
-        <v>2716</v>
+        <v>351</v>
       </c>
       <c r="C187" t="n">
-        <v>977</v>
+        <v>3009</v>
       </c>
       <c r="D187" t="n">
-        <v>729.29</v>
+        <v>416.36</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -3998,13 +3998,13 @@
         <v>46218</v>
       </c>
       <c r="B188" t="n">
-        <v>1993</v>
+        <v>2250</v>
       </c>
       <c r="C188" t="n">
         <v>8888</v>
       </c>
       <c r="D188" t="n">
-        <v>456.62</v>
+        <v>709.46</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -4017,15 +4017,319 @@
         <v>46218</v>
       </c>
       <c r="B189" t="n">
+        <v>2648</v>
+      </c>
+      <c r="C189" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D189" t="n">
+        <v>1873.52</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B190" t="n">
+        <v>131</v>
+      </c>
+      <c r="C190" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D190" t="n">
+        <v>1369.91</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B191" t="n">
+        <v>2790</v>
+      </c>
+      <c r="C191" t="n">
+        <v>1953</v>
+      </c>
+      <c r="D191" t="n">
+        <v>371.88</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B192" t="n">
+        <v>2639</v>
+      </c>
+      <c r="C192" t="n">
+        <v>1953</v>
+      </c>
+      <c r="D192" t="n">
+        <v>504.09</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B193" t="n">
+        <v>2109</v>
+      </c>
+      <c r="C193" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D193" t="n">
+        <v>2293.78</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B194" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C194" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D194" t="n">
+        <v>2919.53</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B195" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C195" t="n">
+        <v>27</v>
+      </c>
+      <c r="D195" t="n">
+        <v>1803.76</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B196" t="n">
+        <v>353</v>
+      </c>
+      <c r="C196" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D196" t="n">
+        <v>108.6</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B197" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C197" t="n">
+        <v>874</v>
+      </c>
+      <c r="D197" t="n">
+        <v>1230.43</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B198" t="n">
+        <v>42</v>
+      </c>
+      <c r="C198" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D198" t="n">
+        <v>79947.14999999999</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B199" t="n">
+        <v>772</v>
+      </c>
+      <c r="C199" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D199" t="n">
+        <v>400.25</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B200" t="n">
+        <v>2728</v>
+      </c>
+      <c r="C200" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D200" t="n">
+        <v>1397.07</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B201" t="n">
+        <v>2197</v>
+      </c>
+      <c r="C201" t="n">
+        <v>423</v>
+      </c>
+      <c r="D201" t="n">
+        <v>2267.61</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B202" t="n">
+        <v>2716</v>
+      </c>
+      <c r="C202" t="n">
+        <v>1929</v>
+      </c>
+      <c r="D202" t="n">
+        <v>750.4299999999999</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B203" t="n">
+        <v>2716</v>
+      </c>
+      <c r="C203" t="n">
+        <v>977</v>
+      </c>
+      <c r="D203" t="n">
+        <v>729.29</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B204" t="n">
+        <v>1993</v>
+      </c>
+      <c r="C204" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D204" t="n">
+        <v>456.62</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B205" t="n">
         <v>629</v>
       </c>
-      <c r="C189" t="n">
+      <c r="C205" t="n">
         <v>675</v>
       </c>
-      <c r="D189" t="n">
+      <c r="D205" t="n">
         <v>1054.76</v>
       </c>
-      <c r="E189" t="inlineStr">
+      <c r="E205" t="inlineStr">
         <is>
           <t>TELEMARKETING</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 16:30:03
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E213"/>
+  <dimension ref="A1:E234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,7 +489,7 @@
         <v>8888</v>
       </c>
       <c r="D3" t="n">
-        <v>406.97</v>
+        <v>544.78</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -768,17 +768,17 @@
         <v>46218</v>
       </c>
       <c r="B18" t="n">
-        <v>2118</v>
+        <v>890</v>
       </c>
       <c r="C18" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D18" t="n">
-        <v>5535.71</v>
+        <v>898.83</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -787,17 +787,17 @@
         <v>46218</v>
       </c>
       <c r="B19" t="n">
-        <v>2197</v>
+        <v>40</v>
       </c>
       <c r="C19" t="n">
         <v>8888</v>
       </c>
       <c r="D19" t="n">
-        <v>1441.76</v>
+        <v>768.78</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -806,17 +806,17 @@
         <v>46218</v>
       </c>
       <c r="B20" t="n">
-        <v>363</v>
+        <v>2118</v>
       </c>
       <c r="C20" t="n">
         <v>8888</v>
       </c>
       <c r="D20" t="n">
-        <v>836.9400000000001</v>
+        <v>5535.71</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -825,17 +825,17 @@
         <v>46218</v>
       </c>
       <c r="B21" t="n">
-        <v>1869</v>
+        <v>2197</v>
       </c>
       <c r="C21" t="n">
         <v>8888</v>
       </c>
       <c r="D21" t="n">
-        <v>1263.2</v>
+        <v>2855.48</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -844,17 +844,17 @@
         <v>46218</v>
       </c>
       <c r="B22" t="n">
-        <v>1137</v>
+        <v>325</v>
       </c>
       <c r="C22" t="n">
-        <v>8888</v>
+        <v>14</v>
       </c>
       <c r="D22" t="n">
-        <v>359.06</v>
+        <v>301.57</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -863,17 +863,17 @@
         <v>46218</v>
       </c>
       <c r="B23" t="n">
-        <v>2133</v>
+        <v>363</v>
       </c>
       <c r="C23" t="n">
-        <v>691</v>
+        <v>8888</v>
       </c>
       <c r="D23" t="n">
-        <v>2058.93</v>
+        <v>836.9400000000001</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -882,17 +882,17 @@
         <v>46218</v>
       </c>
       <c r="B24" t="n">
-        <v>452</v>
+        <v>1869</v>
       </c>
       <c r="C24" t="n">
         <v>8888</v>
       </c>
       <c r="D24" t="n">
-        <v>1832.74</v>
+        <v>1263.2</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -901,17 +901,17 @@
         <v>46218</v>
       </c>
       <c r="B25" t="n">
-        <v>1632</v>
+        <v>1137</v>
       </c>
       <c r="C25" t="n">
-        <v>423</v>
+        <v>8888</v>
       </c>
       <c r="D25" t="n">
-        <v>2811.9</v>
+        <v>359.06</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -920,17 +920,17 @@
         <v>46218</v>
       </c>
       <c r="B26" t="n">
-        <v>2250</v>
+        <v>2133</v>
       </c>
       <c r="C26" t="n">
-        <v>8888</v>
+        <v>691</v>
       </c>
       <c r="D26" t="n">
-        <v>1686.37</v>
+        <v>2058.93</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -939,17 +939,17 @@
         <v>46218</v>
       </c>
       <c r="B27" t="n">
-        <v>931</v>
+        <v>452</v>
       </c>
       <c r="C27" t="n">
-        <v>423</v>
+        <v>8888</v>
       </c>
       <c r="D27" t="n">
-        <v>492.34</v>
+        <v>1832.74</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -958,17 +958,17 @@
         <v>46218</v>
       </c>
       <c r="B28" t="n">
-        <v>951</v>
+        <v>1632</v>
       </c>
       <c r="C28" t="n">
-        <v>8888</v>
+        <v>423</v>
       </c>
       <c r="D28" t="n">
-        <v>2171.08</v>
+        <v>2811.9</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -977,17 +977,17 @@
         <v>46218</v>
       </c>
       <c r="B29" t="n">
-        <v>2695</v>
+        <v>2250</v>
       </c>
       <c r="C29" t="n">
         <v>8888</v>
       </c>
       <c r="D29" t="n">
-        <v>411.42</v>
+        <v>1686.37</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -996,17 +996,17 @@
         <v>46218</v>
       </c>
       <c r="B30" t="n">
-        <v>525</v>
+        <v>931</v>
       </c>
       <c r="C30" t="n">
-        <v>8888</v>
+        <v>423</v>
       </c>
       <c r="D30" t="n">
-        <v>408.25</v>
+        <v>492.34</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1015,17 +1015,17 @@
         <v>46218</v>
       </c>
       <c r="B31" t="n">
-        <v>1808</v>
+        <v>951</v>
       </c>
       <c r="C31" t="n">
         <v>8888</v>
       </c>
       <c r="D31" t="n">
-        <v>695.3200000000001</v>
+        <v>2171.08</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1034,17 +1034,17 @@
         <v>46218</v>
       </c>
       <c r="B32" t="n">
-        <v>609</v>
+        <v>2695</v>
       </c>
       <c r="C32" t="n">
         <v>8888</v>
       </c>
       <c r="D32" t="n">
-        <v>1909.37</v>
+        <v>411.42</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1053,17 +1053,17 @@
         <v>46218</v>
       </c>
       <c r="B33" t="n">
-        <v>949</v>
+        <v>525</v>
       </c>
       <c r="C33" t="n">
-        <v>1134</v>
+        <v>8888</v>
       </c>
       <c r="D33" t="n">
-        <v>30.46</v>
+        <v>408.25</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1072,17 +1072,17 @@
         <v>46218</v>
       </c>
       <c r="B34" t="n">
-        <v>2499</v>
+        <v>1808</v>
       </c>
       <c r="C34" t="n">
         <v>8888</v>
       </c>
       <c r="D34" t="n">
-        <v>261.63</v>
+        <v>695.3200000000001</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1091,17 +1091,17 @@
         <v>46218</v>
       </c>
       <c r="B35" t="n">
-        <v>58</v>
+        <v>609</v>
       </c>
       <c r="C35" t="n">
         <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>499.11</v>
+        <v>1909.37</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1110,17 @@
         <v>46218</v>
       </c>
       <c r="B36" t="n">
-        <v>2245</v>
+        <v>949</v>
       </c>
       <c r="C36" t="n">
-        <v>8888</v>
+        <v>1134</v>
       </c>
       <c r="D36" t="n">
-        <v>2740.06</v>
+        <v>30.46</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1129,17 @@
         <v>46218</v>
       </c>
       <c r="B37" t="n">
-        <v>325</v>
+        <v>42</v>
       </c>
       <c r="C37" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D37" t="n">
-        <v>871.14</v>
+        <v>358.97</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1148,17 +1148,17 @@
         <v>46218</v>
       </c>
       <c r="B38" t="n">
-        <v>2383</v>
+        <v>2499</v>
       </c>
       <c r="C38" t="n">
         <v>8888</v>
       </c>
       <c r="D38" t="n">
-        <v>7926.02</v>
+        <v>1049.3</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1167,17 +1167,17 @@
         <v>46218</v>
       </c>
       <c r="B39" t="n">
-        <v>1117</v>
+        <v>58</v>
       </c>
       <c r="C39" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D39" t="n">
-        <v>916.72</v>
+        <v>499.11</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1186,13 +1186,13 @@
         <v>46218</v>
       </c>
       <c r="B40" t="n">
-        <v>2279</v>
+        <v>2245</v>
       </c>
       <c r="C40" t="n">
         <v>8888</v>
       </c>
       <c r="D40" t="n">
-        <v>712.66</v>
+        <v>2740.06</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1205,17 +1205,17 @@
         <v>46218</v>
       </c>
       <c r="B41" t="n">
-        <v>535</v>
+        <v>325</v>
       </c>
       <c r="C41" t="n">
         <v>8888</v>
       </c>
       <c r="D41" t="n">
-        <v>5836.12</v>
+        <v>952.75</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1224,17 +1224,17 @@
         <v>46218</v>
       </c>
       <c r="B42" t="n">
-        <v>535</v>
+        <v>2383</v>
       </c>
       <c r="C42" t="n">
         <v>8888</v>
       </c>
       <c r="D42" t="n">
-        <v>1352.51</v>
+        <v>7926.02</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1243,13 +1243,13 @@
         <v>46218</v>
       </c>
       <c r="B43" t="n">
-        <v>2678</v>
+        <v>1117</v>
       </c>
       <c r="C43" t="n">
-        <v>1312</v>
+        <v>1139</v>
       </c>
       <c r="D43" t="n">
-        <v>364.96</v>
+        <v>916.72</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1262,13 +1262,13 @@
         <v>46218</v>
       </c>
       <c r="B44" t="n">
-        <v>2345</v>
+        <v>2279</v>
       </c>
       <c r="C44" t="n">
         <v>8888</v>
       </c>
       <c r="D44" t="n">
-        <v>863.16</v>
+        <v>712.66</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1281,17 +1281,17 @@
         <v>46218</v>
       </c>
       <c r="B45" t="n">
-        <v>945</v>
+        <v>535</v>
       </c>
       <c r="C45" t="n">
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>27337.21</v>
+        <v>5836.12</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>PEDIDO ELETRÔNICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1300,17 +1300,17 @@
         <v>46218</v>
       </c>
       <c r="B46" t="n">
-        <v>2686</v>
+        <v>535</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>684.2</v>
+        <v>1352.51</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1319,17 +1319,17 @@
         <v>46218</v>
       </c>
       <c r="B47" t="n">
-        <v>438</v>
+        <v>2678</v>
       </c>
       <c r="C47" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D47" t="n">
-        <v>220.06</v>
+        <v>364.96</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1338,17 +1338,17 @@
         <v>46218</v>
       </c>
       <c r="B48" t="n">
-        <v>353</v>
+        <v>2345</v>
       </c>
       <c r="C48" t="n">
-        <v>3179</v>
+        <v>8888</v>
       </c>
       <c r="D48" t="n">
-        <v>495.84</v>
+        <v>863.16</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1357,17 +1357,17 @@
         <v>46218</v>
       </c>
       <c r="B49" t="n">
-        <v>1293</v>
+        <v>945</v>
       </c>
       <c r="C49" t="n">
         <v>8888</v>
       </c>
       <c r="D49" t="n">
-        <v>3129.07</v>
+        <v>27337.21</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>PEDIDO ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -1376,17 +1376,17 @@
         <v>46218</v>
       </c>
       <c r="B50" t="n">
-        <v>2279</v>
+        <v>2686</v>
       </c>
       <c r="C50" t="n">
         <v>8888</v>
       </c>
       <c r="D50" t="n">
-        <v>2753.96</v>
+        <v>684.2</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1395,17 +1395,17 @@
         <v>46218</v>
       </c>
       <c r="B51" t="n">
-        <v>1137</v>
+        <v>438</v>
       </c>
       <c r="C51" t="n">
         <v>8888</v>
       </c>
       <c r="D51" t="n">
-        <v>1947.93</v>
+        <v>220.06</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
         <v>46218</v>
       </c>
       <c r="B52" t="n">
-        <v>374</v>
+        <v>664</v>
       </c>
       <c r="C52" t="n">
         <v>8888</v>
       </c>
       <c r="D52" t="n">
-        <v>1390.6</v>
+        <v>2598.01</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1433,13 +1433,13 @@
         <v>46218</v>
       </c>
       <c r="B53" t="n">
-        <v>2793</v>
+        <v>353</v>
       </c>
       <c r="C53" t="n">
-        <v>977</v>
+        <v>3179</v>
       </c>
       <c r="D53" t="n">
-        <v>695.72</v>
+        <v>495.84</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1452,13 +1452,13 @@
         <v>46218</v>
       </c>
       <c r="B54" t="n">
-        <v>2802</v>
+        <v>1293</v>
       </c>
       <c r="C54" t="n">
         <v>8888</v>
       </c>
       <c r="D54" t="n">
-        <v>1264.57</v>
+        <v>3129.07</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1471,17 +1471,17 @@
         <v>46218</v>
       </c>
       <c r="B55" t="n">
-        <v>374</v>
+        <v>2279</v>
       </c>
       <c r="C55" t="n">
         <v>8888</v>
       </c>
       <c r="D55" t="n">
-        <v>44.6</v>
+        <v>2753.96</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1490,13 +1490,13 @@
         <v>46218</v>
       </c>
       <c r="B56" t="n">
-        <v>664</v>
+        <v>1937</v>
       </c>
       <c r="C56" t="n">
         <v>8888</v>
       </c>
       <c r="D56" t="n">
-        <v>1510.56</v>
+        <v>1685.72</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1509,17 +1509,17 @@
         <v>46218</v>
       </c>
       <c r="B57" t="n">
-        <v>703</v>
+        <v>941</v>
       </c>
       <c r="C57" t="n">
         <v>8888</v>
       </c>
       <c r="D57" t="n">
-        <v>12155.46</v>
+        <v>864.14</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1528,17 +1528,17 @@
         <v>46218</v>
       </c>
       <c r="B58" t="n">
-        <v>1937</v>
+        <v>1137</v>
       </c>
       <c r="C58" t="n">
         <v>8888</v>
       </c>
       <c r="D58" t="n">
-        <v>1032.73</v>
+        <v>1947.93</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1547,17 +1547,17 @@
         <v>46218</v>
       </c>
       <c r="B59" t="n">
-        <v>451</v>
+        <v>2631</v>
       </c>
       <c r="C59" t="n">
-        <v>8888</v>
+        <v>2853</v>
       </c>
       <c r="D59" t="n">
-        <v>368.93</v>
+        <v>1272.12</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1566,17 +1566,17 @@
         <v>46218</v>
       </c>
       <c r="B60" t="n">
-        <v>1756</v>
+        <v>2793</v>
       </c>
       <c r="C60" t="n">
-        <v>8888</v>
+        <v>977</v>
       </c>
       <c r="D60" t="n">
-        <v>996.17</v>
+        <v>1188.59</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1585,13 +1585,13 @@
         <v>46218</v>
       </c>
       <c r="B61" t="n">
-        <v>1956</v>
+        <v>374</v>
       </c>
       <c r="C61" t="n">
         <v>8888</v>
       </c>
       <c r="D61" t="n">
-        <v>4557.34</v>
+        <v>2103.29</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1604,13 +1604,13 @@
         <v>46218</v>
       </c>
       <c r="B62" t="n">
-        <v>925</v>
+        <v>2802</v>
       </c>
       <c r="C62" t="n">
         <v>8888</v>
       </c>
       <c r="D62" t="n">
-        <v>651.59</v>
+        <v>1264.57</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1623,17 +1623,17 @@
         <v>46218</v>
       </c>
       <c r="B63" t="n">
-        <v>2631</v>
+        <v>451</v>
       </c>
       <c r="C63" t="n">
-        <v>2853</v>
+        <v>8888</v>
       </c>
       <c r="D63" t="n">
-        <v>509.88</v>
+        <v>757.5700000000001</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1642,13 +1642,13 @@
         <v>46218</v>
       </c>
       <c r="B64" t="n">
-        <v>2648</v>
+        <v>374</v>
       </c>
       <c r="C64" t="n">
         <v>8888</v>
       </c>
       <c r="D64" t="n">
-        <v>1594.42</v>
+        <v>44.6</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1661,17 +1661,17 @@
         <v>46218</v>
       </c>
       <c r="B65" t="n">
-        <v>2714</v>
+        <v>703</v>
       </c>
       <c r="C65" t="n">
-        <v>519</v>
+        <v>8888</v>
       </c>
       <c r="D65" t="n">
-        <v>61939.22</v>
+        <v>12155.46</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1680,17 +1680,17 @@
         <v>46218</v>
       </c>
       <c r="B66" t="n">
-        <v>483</v>
+        <v>1756</v>
       </c>
       <c r="C66" t="n">
         <v>8888</v>
       </c>
       <c r="D66" t="n">
-        <v>6625.87</v>
+        <v>996.17</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1699,13 +1699,13 @@
         <v>46218</v>
       </c>
       <c r="B67" t="n">
-        <v>1075</v>
+        <v>1956</v>
       </c>
       <c r="C67" t="n">
         <v>8888</v>
       </c>
       <c r="D67" t="n">
-        <v>11607.79</v>
+        <v>4557.34</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1718,17 +1718,17 @@
         <v>46218</v>
       </c>
       <c r="B68" t="n">
-        <v>629</v>
+        <v>925</v>
       </c>
       <c r="C68" t="n">
         <v>8888</v>
       </c>
       <c r="D68" t="n">
-        <v>9233.719999999999</v>
+        <v>651.59</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1737,17 +1737,17 @@
         <v>46218</v>
       </c>
       <c r="B69" t="n">
-        <v>1983</v>
+        <v>2648</v>
       </c>
       <c r="C69" t="n">
-        <v>841</v>
+        <v>8888</v>
       </c>
       <c r="D69" t="n">
-        <v>243.92</v>
+        <v>1594.42</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1756,17 +1756,17 @@
         <v>46218</v>
       </c>
       <c r="B70" t="n">
-        <v>1137</v>
+        <v>2714</v>
       </c>
       <c r="C70" t="n">
-        <v>8888</v>
+        <v>519</v>
       </c>
       <c r="D70" t="n">
-        <v>3578.51</v>
+        <v>61939.22</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1775,17 @@
         <v>46218</v>
       </c>
       <c r="B71" t="n">
-        <v>2651</v>
+        <v>483</v>
       </c>
       <c r="C71" t="n">
         <v>8888</v>
       </c>
       <c r="D71" t="n">
-        <v>1296.58</v>
+        <v>8624.57</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1794,17 +1794,17 @@
         <v>46218</v>
       </c>
       <c r="B72" t="n">
-        <v>1956</v>
+        <v>1075</v>
       </c>
       <c r="C72" t="n">
-        <v>423</v>
+        <v>8888</v>
       </c>
       <c r="D72" t="n">
-        <v>1416.35</v>
+        <v>11607.79</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1813,17 +1813,17 @@
         <v>46218</v>
       </c>
       <c r="B73" t="n">
-        <v>2709</v>
+        <v>629</v>
       </c>
       <c r="C73" t="n">
         <v>8888</v>
       </c>
       <c r="D73" t="n">
-        <v>547.6900000000001</v>
+        <v>9233.719999999999</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1832,17 +1832,17 @@
         <v>46218</v>
       </c>
       <c r="B74" t="n">
-        <v>1308</v>
+        <v>1983</v>
       </c>
       <c r="C74" t="n">
-        <v>8888</v>
+        <v>841</v>
       </c>
       <c r="D74" t="n">
-        <v>1460.53</v>
+        <v>243.92</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1851,17 +1851,17 @@
         <v>46218</v>
       </c>
       <c r="B75" t="n">
-        <v>2026</v>
+        <v>1137</v>
       </c>
       <c r="C75" t="n">
         <v>8888</v>
       </c>
       <c r="D75" t="n">
-        <v>2237.62</v>
+        <v>3578.51</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1870,17 +1870,17 @@
         <v>46218</v>
       </c>
       <c r="B76" t="n">
-        <v>2789</v>
+        <v>2651</v>
       </c>
       <c r="C76" t="n">
         <v>8888</v>
       </c>
       <c r="D76" t="n">
-        <v>747.77</v>
+        <v>1296.58</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1889,17 +1889,17 @@
         <v>46218</v>
       </c>
       <c r="B77" t="n">
-        <v>89</v>
+        <v>663</v>
       </c>
       <c r="C77" t="n">
-        <v>13148</v>
+        <v>8888</v>
       </c>
       <c r="D77" t="n">
-        <v>1883.74</v>
+        <v>5851.1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1908,13 +1908,13 @@
         <v>46218</v>
       </c>
       <c r="B78" t="n">
-        <v>2709</v>
+        <v>1956</v>
       </c>
       <c r="C78" t="n">
-        <v>2220</v>
+        <v>423</v>
       </c>
       <c r="D78" t="n">
-        <v>390.19</v>
+        <v>1416.35</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -1927,13 +1927,13 @@
         <v>46218</v>
       </c>
       <c r="B79" t="n">
-        <v>2345</v>
+        <v>2709</v>
       </c>
       <c r="C79" t="n">
         <v>8888</v>
       </c>
       <c r="D79" t="n">
-        <v>748.86</v>
+        <v>547.6900000000001</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -1946,17 +1946,17 @@
         <v>46218</v>
       </c>
       <c r="B80" t="n">
-        <v>569</v>
+        <v>1308</v>
       </c>
       <c r="C80" t="n">
         <v>8888</v>
       </c>
       <c r="D80" t="n">
-        <v>995.33</v>
+        <v>1460.53</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1965,17 +1965,17 @@
         <v>46218</v>
       </c>
       <c r="B81" t="n">
-        <v>360</v>
+        <v>2026</v>
       </c>
       <c r="C81" t="n">
-        <v>546</v>
+        <v>8888</v>
       </c>
       <c r="D81" t="n">
-        <v>1609.68</v>
+        <v>2237.62</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1984,17 +1984,17 @@
         <v>46218</v>
       </c>
       <c r="B82" t="n">
-        <v>2308</v>
+        <v>2789</v>
       </c>
       <c r="C82" t="n">
         <v>8888</v>
       </c>
       <c r="D82" t="n">
-        <v>488.69</v>
+        <v>747.77</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2003,13 +2003,13 @@
         <v>46218</v>
       </c>
       <c r="B83" t="n">
-        <v>2211</v>
+        <v>89</v>
       </c>
       <c r="C83" t="n">
-        <v>874</v>
+        <v>13148</v>
       </c>
       <c r="D83" t="n">
-        <v>1526.94</v>
+        <v>1883.74</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2022,17 +2022,17 @@
         <v>46218</v>
       </c>
       <c r="B84" t="n">
-        <v>559</v>
+        <v>2709</v>
       </c>
       <c r="C84" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D84" t="n">
-        <v>859.92</v>
+        <v>390.19</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2041,17 +2041,17 @@
         <v>46218</v>
       </c>
       <c r="B85" t="n">
-        <v>890</v>
+        <v>2789</v>
       </c>
       <c r="C85" t="n">
         <v>8888</v>
       </c>
       <c r="D85" t="n">
-        <v>387.2</v>
+        <v>691.37</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2060,13 +2060,13 @@
         <v>46218</v>
       </c>
       <c r="B86" t="n">
-        <v>2768</v>
+        <v>2345</v>
       </c>
       <c r="C86" t="n">
         <v>8888</v>
       </c>
       <c r="D86" t="n">
-        <v>6523.26</v>
+        <v>748.86</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2079,17 +2079,17 @@
         <v>46218</v>
       </c>
       <c r="B87" t="n">
-        <v>1063</v>
+        <v>2765</v>
       </c>
       <c r="C87" t="n">
-        <v>8888</v>
+        <v>1883</v>
       </c>
       <c r="D87" t="n">
-        <v>4487.11</v>
+        <v>3638.6</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2098,17 +2098,17 @@
         <v>46218</v>
       </c>
       <c r="B88" t="n">
-        <v>2279</v>
+        <v>569</v>
       </c>
       <c r="C88" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D88" t="n">
-        <v>652.51</v>
+        <v>995.33</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2117,13 +2117,13 @@
         <v>46218</v>
       </c>
       <c r="B89" t="n">
-        <v>1299</v>
+        <v>360</v>
       </c>
       <c r="C89" t="n">
-        <v>27</v>
+        <v>546</v>
       </c>
       <c r="D89" t="n">
-        <v>1435.52</v>
+        <v>1609.68</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2136,17 +2136,17 @@
         <v>46218</v>
       </c>
       <c r="B90" t="n">
-        <v>1478</v>
+        <v>2308</v>
       </c>
       <c r="C90" t="n">
-        <v>675</v>
+        <v>8888</v>
       </c>
       <c r="D90" t="n">
-        <v>1600.01</v>
+        <v>488.69</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2155,17 +2155,17 @@
         <v>46218</v>
       </c>
       <c r="B91" t="n">
-        <v>285</v>
+        <v>2211</v>
       </c>
       <c r="C91" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D91" t="n">
-        <v>3349.8</v>
+        <v>1526.94</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2174,13 +2174,13 @@
         <v>46218</v>
       </c>
       <c r="B92" t="n">
-        <v>1983</v>
+        <v>559</v>
       </c>
       <c r="C92" t="n">
         <v>8888</v>
       </c>
       <c r="D92" t="n">
-        <v>2451.28</v>
+        <v>859.92</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2193,17 +2193,17 @@
         <v>46218</v>
       </c>
       <c r="B93" t="n">
-        <v>477</v>
+        <v>890</v>
       </c>
       <c r="C93" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D93" t="n">
-        <v>1540.55</v>
+        <v>387.2</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2212,17 +2212,17 @@
         <v>46218</v>
       </c>
       <c r="B94" t="n">
-        <v>1063</v>
+        <v>2768</v>
       </c>
       <c r="C94" t="n">
         <v>8888</v>
       </c>
       <c r="D94" t="n">
-        <v>2549.86</v>
+        <v>6523.26</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2231,17 +2231,17 @@
         <v>46218</v>
       </c>
       <c r="B95" t="n">
-        <v>424</v>
+        <v>1063</v>
       </c>
       <c r="C95" t="n">
         <v>8888</v>
       </c>
       <c r="D95" t="n">
-        <v>1035.17</v>
+        <v>4487.11</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2250,17 +2250,17 @@
         <v>46218</v>
       </c>
       <c r="B96" t="n">
-        <v>675</v>
+        <v>2279</v>
       </c>
       <c r="C96" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D96" t="n">
-        <v>616.73</v>
+        <v>652.51</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2269,17 +2269,17 @@
         <v>46218</v>
       </c>
       <c r="B97" t="n">
-        <v>1993</v>
+        <v>1299</v>
       </c>
       <c r="C97" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D97" t="n">
-        <v>362.63</v>
+        <v>1435.52</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2288,17 +2288,17 @@
         <v>46218</v>
       </c>
       <c r="B98" t="n">
-        <v>1465</v>
+        <v>1478</v>
       </c>
       <c r="C98" t="n">
-        <v>8888</v>
+        <v>675</v>
       </c>
       <c r="D98" t="n">
-        <v>3373.83</v>
+        <v>1600.01</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2307,17 +2307,17 @@
         <v>46218</v>
       </c>
       <c r="B99" t="n">
-        <v>89</v>
+        <v>285</v>
       </c>
       <c r="C99" t="n">
         <v>8888</v>
       </c>
       <c r="D99" t="n">
-        <v>479</v>
+        <v>3349.8</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2326,17 +2326,17 @@
         <v>46218</v>
       </c>
       <c r="B100" t="n">
-        <v>595</v>
+        <v>477</v>
       </c>
       <c r="C100" t="n">
         <v>8888</v>
       </c>
       <c r="D100" t="n">
-        <v>18084.5</v>
+        <v>917.33</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2345,17 +2345,17 @@
         <v>46218</v>
       </c>
       <c r="B101" t="n">
-        <v>2696</v>
+        <v>1983</v>
       </c>
       <c r="C101" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D101" t="n">
-        <v>1597.76</v>
+        <v>5115.01</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2364,17 +2364,17 @@
         <v>46218</v>
       </c>
       <c r="B102" t="n">
-        <v>360</v>
+        <v>477</v>
       </c>
       <c r="C102" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D102" t="n">
-        <v>4596.89</v>
+        <v>1540.55</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2383,17 +2383,17 @@
         <v>46218</v>
       </c>
       <c r="B103" t="n">
-        <v>1465</v>
+        <v>1063</v>
       </c>
       <c r="C103" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D103" t="n">
-        <v>777.2</v>
+        <v>2549.86</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2402,17 +2402,17 @@
         <v>46218</v>
       </c>
       <c r="B104" t="n">
-        <v>947</v>
+        <v>424</v>
       </c>
       <c r="C104" t="n">
         <v>8888</v>
       </c>
       <c r="D104" t="n">
-        <v>2087.97</v>
+        <v>1362.42</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>PEDIDO ELETRÔNICO</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2421,17 +2421,17 @@
         <v>46218</v>
       </c>
       <c r="B105" t="n">
-        <v>2178</v>
+        <v>675</v>
       </c>
       <c r="C105" t="n">
         <v>8888</v>
       </c>
       <c r="D105" t="n">
-        <v>619.92</v>
+        <v>616.73</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2440,17 +2440,17 @@
         <v>46218</v>
       </c>
       <c r="B106" t="n">
-        <v>630</v>
+        <v>663</v>
       </c>
       <c r="C106" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D106" t="n">
-        <v>1801.63</v>
+        <v>255.13</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2459,17 +2459,17 @@
         <v>46218</v>
       </c>
       <c r="B107" t="n">
-        <v>1937</v>
+        <v>1993</v>
       </c>
       <c r="C107" t="n">
         <v>8888</v>
       </c>
       <c r="D107" t="n">
-        <v>2132.95</v>
+        <v>362.63</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2478,13 +2478,13 @@
         <v>46218</v>
       </c>
       <c r="B108" t="n">
-        <v>2577</v>
+        <v>1465</v>
       </c>
       <c r="C108" t="n">
         <v>8888</v>
       </c>
       <c r="D108" t="n">
-        <v>1647.08</v>
+        <v>3373.83</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -2497,17 +2497,17 @@
         <v>46218</v>
       </c>
       <c r="B109" t="n">
-        <v>1293</v>
+        <v>89</v>
       </c>
       <c r="C109" t="n">
         <v>8888</v>
       </c>
       <c r="D109" t="n">
-        <v>2135.89</v>
+        <v>479</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2516,17 +2516,17 @@
         <v>46218</v>
       </c>
       <c r="B110" t="n">
-        <v>2026</v>
+        <v>595</v>
       </c>
       <c r="C110" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D110" t="n">
-        <v>1680.89</v>
+        <v>18084.5</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2535,17 +2535,17 @@
         <v>46218</v>
       </c>
       <c r="B111" t="n">
-        <v>2607</v>
+        <v>2696</v>
       </c>
       <c r="C111" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D111" t="n">
-        <v>490.31</v>
+        <v>1597.76</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2554,17 +2554,17 @@
         <v>46218</v>
       </c>
       <c r="B112" t="n">
-        <v>1317</v>
+        <v>360</v>
       </c>
       <c r="C112" t="n">
         <v>8888</v>
       </c>
       <c r="D112" t="n">
-        <v>907.72</v>
+        <v>4596.89</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2573,17 +2573,17 @@
         <v>46218</v>
       </c>
       <c r="B113" t="n">
-        <v>767</v>
+        <v>1465</v>
       </c>
       <c r="C113" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D113" t="n">
-        <v>637.23</v>
+        <v>777.2</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2592,17 +2592,17 @@
         <v>46218</v>
       </c>
       <c r="B114" t="n">
-        <v>2571</v>
+        <v>947</v>
       </c>
       <c r="C114" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D114" t="n">
-        <v>268.53</v>
+        <v>5115.36</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>PEDIDO ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -2611,17 +2611,17 @@
         <v>46218</v>
       </c>
       <c r="B115" t="n">
-        <v>1937</v>
+        <v>2178</v>
       </c>
       <c r="C115" t="n">
         <v>8888</v>
       </c>
       <c r="D115" t="n">
-        <v>1803.32</v>
+        <v>619.92</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2630,17 +2630,17 @@
         <v>46218</v>
       </c>
       <c r="B116" t="n">
-        <v>1063</v>
+        <v>2026</v>
       </c>
       <c r="C116" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D116" t="n">
-        <v>1113.08</v>
+        <v>3418.07</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2649,17 +2649,17 @@
         <v>46218</v>
       </c>
       <c r="B117" t="n">
-        <v>2631</v>
+        <v>630</v>
       </c>
       <c r="C117" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D117" t="n">
-        <v>1447.86</v>
+        <v>1801.63</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2668,17 +2668,17 @@
         <v>46218</v>
       </c>
       <c r="B118" t="n">
-        <v>1906</v>
+        <v>1937</v>
       </c>
       <c r="C118" t="n">
         <v>8888</v>
       </c>
       <c r="D118" t="n">
-        <v>2774.84</v>
+        <v>2132.95</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2687,13 +2687,13 @@
         <v>46218</v>
       </c>
       <c r="B119" t="n">
-        <v>1756</v>
+        <v>2577</v>
       </c>
       <c r="C119" t="n">
         <v>8888</v>
       </c>
       <c r="D119" t="n">
-        <v>1357.12</v>
+        <v>1647.08</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -2706,17 +2706,17 @@
         <v>46218</v>
       </c>
       <c r="B120" t="n">
-        <v>20</v>
+        <v>1293</v>
       </c>
       <c r="C120" t="n">
         <v>8888</v>
       </c>
       <c r="D120" t="n">
-        <v>276.64</v>
+        <v>2135.89</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2725,17 +2725,17 @@
         <v>46218</v>
       </c>
       <c r="B121" t="n">
-        <v>477</v>
+        <v>2607</v>
       </c>
       <c r="C121" t="n">
         <v>8888</v>
       </c>
       <c r="D121" t="n">
-        <v>372.69</v>
+        <v>490.31</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2744,13 +2744,13 @@
         <v>46218</v>
       </c>
       <c r="B122" t="n">
-        <v>477</v>
+        <v>1317</v>
       </c>
       <c r="C122" t="n">
         <v>8888</v>
       </c>
       <c r="D122" t="n">
-        <v>707.52</v>
+        <v>907.72</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -2763,13 +2763,13 @@
         <v>46218</v>
       </c>
       <c r="B123" t="n">
-        <v>2660</v>
+        <v>767</v>
       </c>
       <c r="C123" t="n">
         <v>8888</v>
       </c>
       <c r="D123" t="n">
-        <v>2684.97</v>
+        <v>637.23</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -2782,17 +2782,17 @@
         <v>46218</v>
       </c>
       <c r="B124" t="n">
-        <v>569</v>
+        <v>2571</v>
       </c>
       <c r="C124" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D124" t="n">
-        <v>23608.83</v>
+        <v>268.53</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2801,17 +2801,17 @@
         <v>46218</v>
       </c>
       <c r="B125" t="n">
-        <v>2089</v>
+        <v>1937</v>
       </c>
       <c r="C125" t="n">
-        <v>1533</v>
+        <v>8888</v>
       </c>
       <c r="D125" t="n">
-        <v>969.24</v>
+        <v>1803.32</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2820,13 +2820,13 @@
         <v>46218</v>
       </c>
       <c r="B126" t="n">
-        <v>1007</v>
+        <v>20</v>
       </c>
       <c r="C126" t="n">
         <v>8888</v>
       </c>
       <c r="D126" t="n">
-        <v>241.44</v>
+        <v>745.55</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -2839,17 +2839,17 @@
         <v>46218</v>
       </c>
       <c r="B127" t="n">
-        <v>1380</v>
+        <v>1063</v>
       </c>
       <c r="C127" t="n">
         <v>8888</v>
       </c>
       <c r="D127" t="n">
-        <v>520.2</v>
+        <v>1113.08</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2858,17 +2858,17 @@
         <v>46218</v>
       </c>
       <c r="B128" t="n">
-        <v>1102</v>
+        <v>2631</v>
       </c>
       <c r="C128" t="n">
         <v>8888</v>
       </c>
       <c r="D128" t="n">
-        <v>1137.04</v>
+        <v>1447.86</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2877,13 +2877,13 @@
         <v>46218</v>
       </c>
       <c r="B129" t="n">
-        <v>1075</v>
+        <v>1906</v>
       </c>
       <c r="C129" t="n">
         <v>8888</v>
       </c>
       <c r="D129" t="n">
-        <v>2179.03</v>
+        <v>2774.84</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -2896,17 +2896,17 @@
         <v>46218</v>
       </c>
       <c r="B130" t="n">
-        <v>2681</v>
+        <v>1756</v>
       </c>
       <c r="C130" t="n">
         <v>8888</v>
       </c>
       <c r="D130" t="n">
-        <v>729.25</v>
+        <v>2275.21</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2915,13 +2915,13 @@
         <v>46218</v>
       </c>
       <c r="B131" t="n">
-        <v>2245</v>
+        <v>477</v>
       </c>
       <c r="C131" t="n">
         <v>8888</v>
       </c>
       <c r="D131" t="n">
-        <v>361.58</v>
+        <v>707.52</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -2934,17 +2934,17 @@
         <v>46218</v>
       </c>
       <c r="B132" t="n">
-        <v>132</v>
+        <v>2660</v>
       </c>
       <c r="C132" t="n">
         <v>8888</v>
       </c>
       <c r="D132" t="n">
-        <v>6522.92</v>
+        <v>2684.97</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2953,17 +2953,17 @@
         <v>46218</v>
       </c>
       <c r="B133" t="n">
-        <v>452</v>
+        <v>569</v>
       </c>
       <c r="C133" t="n">
         <v>8888</v>
       </c>
       <c r="D133" t="n">
-        <v>608.78</v>
+        <v>33214.39</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2972,17 +2972,17 @@
         <v>46218</v>
       </c>
       <c r="B134" t="n">
-        <v>1293</v>
+        <v>483</v>
       </c>
       <c r="C134" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D134" t="n">
-        <v>1780.93</v>
+        <v>2401.99</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2991,17 +2991,17 @@
         <v>46218</v>
       </c>
       <c r="B135" t="n">
-        <v>525</v>
+        <v>483</v>
       </c>
       <c r="C135" t="n">
         <v>8888</v>
       </c>
       <c r="D135" t="n">
-        <v>5658.57</v>
+        <v>1124.96</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3010,17 +3010,17 @@
         <v>46218</v>
       </c>
       <c r="B136" t="n">
-        <v>2641</v>
+        <v>2089</v>
       </c>
       <c r="C136" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D136" t="n">
-        <v>1720.99</v>
+        <v>1309.01</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3029,17 +3029,17 @@
         <v>46218</v>
       </c>
       <c r="B137" t="n">
-        <v>609</v>
+        <v>1007</v>
       </c>
       <c r="C137" t="n">
         <v>8888</v>
       </c>
       <c r="D137" t="n">
-        <v>886.1</v>
+        <v>241.44</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3048,17 +3048,17 @@
         <v>46218</v>
       </c>
       <c r="B138" t="n">
-        <v>619</v>
+        <v>1380</v>
       </c>
       <c r="C138" t="n">
         <v>8888</v>
       </c>
       <c r="D138" t="n">
-        <v>2330.47</v>
+        <v>520.2</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3067,13 +3067,13 @@
         <v>46218</v>
       </c>
       <c r="B139" t="n">
-        <v>2697</v>
+        <v>1102</v>
       </c>
       <c r="C139" t="n">
         <v>8888</v>
       </c>
       <c r="D139" t="n">
-        <v>418.65</v>
+        <v>1137.04</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3086,13 +3086,13 @@
         <v>46218</v>
       </c>
       <c r="B140" t="n">
-        <v>58</v>
+        <v>1075</v>
       </c>
       <c r="C140" t="n">
         <v>8888</v>
       </c>
       <c r="D140" t="n">
-        <v>1123.87</v>
+        <v>4194.79</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3105,13 +3105,13 @@
         <v>46218</v>
       </c>
       <c r="B141" t="n">
-        <v>358</v>
+        <v>2681</v>
       </c>
       <c r="C141" t="n">
         <v>8888</v>
       </c>
       <c r="D141" t="n">
-        <v>1675.95</v>
+        <v>729.25</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3124,17 +3124,17 @@
         <v>46218</v>
       </c>
       <c r="B142" t="n">
-        <v>2431</v>
+        <v>2245</v>
       </c>
       <c r="C142" t="n">
         <v>8888</v>
       </c>
       <c r="D142" t="n">
-        <v>266.89</v>
+        <v>361.58</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3143,13 +3143,13 @@
         <v>46218</v>
       </c>
       <c r="B143" t="n">
-        <v>285</v>
+        <v>33</v>
       </c>
       <c r="C143" t="n">
         <v>8888</v>
       </c>
       <c r="D143" t="n">
-        <v>2090.81</v>
+        <v>926.97</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3162,17 +3162,17 @@
         <v>46218</v>
       </c>
       <c r="B144" t="n">
-        <v>1102</v>
+        <v>132</v>
       </c>
       <c r="C144" t="n">
         <v>8888</v>
       </c>
       <c r="D144" t="n">
-        <v>1119.32</v>
+        <v>6522.92</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3181,17 +3181,17 @@
         <v>46218</v>
       </c>
       <c r="B145" t="n">
-        <v>626</v>
+        <v>619</v>
       </c>
       <c r="C145" t="n">
         <v>8888</v>
       </c>
       <c r="D145" t="n">
-        <v>12556.19</v>
+        <v>2912.89</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3200,17 +3200,17 @@
         <v>46218</v>
       </c>
       <c r="B146" t="n">
-        <v>1137</v>
+        <v>452</v>
       </c>
       <c r="C146" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D146" t="n">
-        <v>1370.86</v>
+        <v>608.78</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3219,17 +3219,17 @@
         <v>46218</v>
       </c>
       <c r="B147" t="n">
-        <v>2686</v>
+        <v>2463</v>
       </c>
       <c r="C147" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D147" t="n">
-        <v>2066.36</v>
+        <v>363.69</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3238,13 +3238,13 @@
         <v>46218</v>
       </c>
       <c r="B148" t="n">
-        <v>1756</v>
+        <v>1293</v>
       </c>
       <c r="C148" t="n">
-        <v>27</v>
+        <v>1281</v>
       </c>
       <c r="D148" t="n">
-        <v>5078.1</v>
+        <v>1780.93</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -3257,17 +3257,17 @@
         <v>46218</v>
       </c>
       <c r="B149" t="n">
-        <v>2651</v>
+        <v>525</v>
       </c>
       <c r="C149" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D149" t="n">
-        <v>363.7</v>
+        <v>5658.57</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3276,13 +3276,13 @@
         <v>46218</v>
       </c>
       <c r="B150" t="n">
-        <v>360</v>
+        <v>2641</v>
       </c>
       <c r="C150" t="n">
         <v>8888</v>
       </c>
       <c r="D150" t="n">
-        <v>1594.84</v>
+        <v>1720.99</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -3295,13 +3295,13 @@
         <v>46218</v>
       </c>
       <c r="B151" t="n">
-        <v>2582</v>
+        <v>609</v>
       </c>
       <c r="C151" t="n">
         <v>8888</v>
       </c>
       <c r="D151" t="n">
-        <v>379.33</v>
+        <v>886.1</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -3314,17 +3314,17 @@
         <v>46218</v>
       </c>
       <c r="B152" t="n">
-        <v>1756</v>
+        <v>2697</v>
       </c>
       <c r="C152" t="n">
         <v>8888</v>
       </c>
       <c r="D152" t="n">
-        <v>1715.26</v>
+        <v>418.65</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3333,13 +3333,13 @@
         <v>46218</v>
       </c>
       <c r="B153" t="n">
-        <v>636</v>
+        <v>58</v>
       </c>
       <c r="C153" t="n">
         <v>8888</v>
       </c>
       <c r="D153" t="n">
-        <v>2447.56</v>
+        <v>1123.87</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -3352,17 +3352,17 @@
         <v>46218</v>
       </c>
       <c r="B154" t="n">
-        <v>1254</v>
+        <v>358</v>
       </c>
       <c r="C154" t="n">
         <v>8888</v>
       </c>
       <c r="D154" t="n">
-        <v>855.76</v>
+        <v>1675.95</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3371,13 +3371,13 @@
         <v>46218</v>
       </c>
       <c r="B155" t="n">
-        <v>1289</v>
+        <v>2431</v>
       </c>
       <c r="C155" t="n">
         <v>8888</v>
       </c>
       <c r="D155" t="n">
-        <v>2396.98</v>
+        <v>266.89</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -3390,17 +3390,17 @@
         <v>46218</v>
       </c>
       <c r="B156" t="n">
-        <v>2015</v>
+        <v>285</v>
       </c>
       <c r="C156" t="n">
         <v>8888</v>
       </c>
       <c r="D156" t="n">
-        <v>315.69</v>
+        <v>5673.85</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3409,17 +3409,17 @@
         <v>46218</v>
       </c>
       <c r="B157" t="n">
-        <v>1064</v>
+        <v>1102</v>
       </c>
       <c r="C157" t="n">
         <v>8888</v>
       </c>
       <c r="D157" t="n">
-        <v>1274.3</v>
+        <v>1119.32</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3428,17 +3428,17 @@
         <v>46218</v>
       </c>
       <c r="B158" t="n">
-        <v>2698</v>
+        <v>626</v>
       </c>
       <c r="C158" t="n">
         <v>8888</v>
       </c>
       <c r="D158" t="n">
-        <v>552.15</v>
+        <v>12556.19</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3447,17 +3447,17 @@
         <v>46218</v>
       </c>
       <c r="B159" t="n">
-        <v>629</v>
+        <v>1137</v>
       </c>
       <c r="C159" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D159" t="n">
-        <v>3035.38</v>
+        <v>1370.86</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3466,17 +3466,17 @@
         <v>46218</v>
       </c>
       <c r="B160" t="n">
-        <v>664</v>
+        <v>2686</v>
       </c>
       <c r="C160" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D160" t="n">
-        <v>4973.15</v>
+        <v>2066.36</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3491,7 @@
         <v>8888</v>
       </c>
       <c r="D161" t="n">
-        <v>1852.83</v>
+        <v>5635.67</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -3504,17 +3504,17 @@
         <v>46218</v>
       </c>
       <c r="B162" t="n">
-        <v>2641</v>
+        <v>1756</v>
       </c>
       <c r="C162" t="n">
         <v>8888</v>
       </c>
       <c r="D162" t="n">
-        <v>820</v>
+        <v>2201.67</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3523,17 +3523,17 @@
         <v>46218</v>
       </c>
       <c r="B163" t="n">
-        <v>429</v>
+        <v>1756</v>
       </c>
       <c r="C163" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D163" t="n">
-        <v>2593.49</v>
+        <v>5078.1</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3542,17 +3542,17 @@
         <v>46218</v>
       </c>
       <c r="B164" t="n">
-        <v>816</v>
+        <v>2651</v>
       </c>
       <c r="C164" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D164" t="n">
-        <v>438.24</v>
+        <v>363.7</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3561,13 +3561,13 @@
         <v>46218</v>
       </c>
       <c r="B165" t="n">
-        <v>2793</v>
+        <v>664</v>
       </c>
       <c r="C165" t="n">
         <v>8888</v>
       </c>
       <c r="D165" t="n">
-        <v>767.58</v>
+        <v>5672.57</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -3580,17 +3580,17 @@
         <v>46218</v>
       </c>
       <c r="B166" t="n">
-        <v>2359</v>
+        <v>360</v>
       </c>
       <c r="C166" t="n">
         <v>8888</v>
       </c>
       <c r="D166" t="n">
-        <v>381.95</v>
+        <v>1594.84</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3599,17 +3599,17 @@
         <v>46218</v>
       </c>
       <c r="B167" t="n">
-        <v>285</v>
+        <v>2582</v>
       </c>
       <c r="C167" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D167" t="n">
-        <v>364.99</v>
+        <v>379.33</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3618,13 +3618,13 @@
         <v>46218</v>
       </c>
       <c r="B168" t="n">
-        <v>2114</v>
+        <v>636</v>
       </c>
       <c r="C168" t="n">
         <v>8888</v>
       </c>
       <c r="D168" t="n">
-        <v>2726.04</v>
+        <v>2447.56</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -3637,17 +3637,17 @@
         <v>46218</v>
       </c>
       <c r="B169" t="n">
-        <v>953</v>
+        <v>1254</v>
       </c>
       <c r="C169" t="n">
         <v>8888</v>
       </c>
       <c r="D169" t="n">
-        <v>2618.89</v>
+        <v>2643.22</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3656,17 +3656,17 @@
         <v>46218</v>
       </c>
       <c r="B170" t="n">
-        <v>1102</v>
+        <v>1289</v>
       </c>
       <c r="C170" t="n">
         <v>8888</v>
       </c>
       <c r="D170" t="n">
-        <v>2344.41</v>
+        <v>2396.98</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3675,17 +3675,17 @@
         <v>46218</v>
       </c>
       <c r="B171" t="n">
-        <v>619</v>
+        <v>2726</v>
       </c>
       <c r="C171" t="n">
-        <v>8888</v>
+        <v>977</v>
       </c>
       <c r="D171" t="n">
-        <v>2021.67</v>
+        <v>586.0599999999999</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3694,13 +3694,13 @@
         <v>46218</v>
       </c>
       <c r="B172" t="n">
-        <v>1465</v>
+        <v>2015</v>
       </c>
       <c r="C172" t="n">
         <v>8888</v>
       </c>
       <c r="D172" t="n">
-        <v>3504</v>
+        <v>315.69</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -3713,17 +3713,17 @@
         <v>46218</v>
       </c>
       <c r="B173" t="n">
-        <v>2767</v>
+        <v>1064</v>
       </c>
       <c r="C173" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D173" t="n">
-        <v>1135.64</v>
+        <v>1274.3</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3732,13 +3732,13 @@
         <v>46218</v>
       </c>
       <c r="B174" t="n">
-        <v>2245</v>
+        <v>2698</v>
       </c>
       <c r="C174" t="n">
         <v>8888</v>
       </c>
       <c r="D174" t="n">
-        <v>427.51</v>
+        <v>552.15</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -3751,17 +3751,17 @@
         <v>46218</v>
       </c>
       <c r="B175" t="n">
-        <v>2197</v>
+        <v>629</v>
       </c>
       <c r="C175" t="n">
         <v>8888</v>
       </c>
       <c r="D175" t="n">
-        <v>1085.45</v>
+        <v>3544.51</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3770,17 +3770,17 @@
         <v>46218</v>
       </c>
       <c r="B176" t="n">
-        <v>2657</v>
+        <v>2641</v>
       </c>
       <c r="C176" t="n">
         <v>8888</v>
       </c>
       <c r="D176" t="n">
-        <v>2683.06</v>
+        <v>820</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3789,13 +3789,13 @@
         <v>46218</v>
       </c>
       <c r="B177" t="n">
-        <v>1277</v>
+        <v>429</v>
       </c>
       <c r="C177" t="n">
         <v>8888</v>
       </c>
       <c r="D177" t="n">
-        <v>1949</v>
+        <v>2593.49</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -3808,17 +3808,17 @@
         <v>46218</v>
       </c>
       <c r="B178" t="n">
-        <v>131</v>
+        <v>816</v>
       </c>
       <c r="C178" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D178" t="n">
-        <v>1268.57</v>
+        <v>438.24</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3827,17 +3827,17 @@
         <v>46218</v>
       </c>
       <c r="B179" t="n">
-        <v>2692</v>
+        <v>2793</v>
       </c>
       <c r="C179" t="n">
         <v>8888</v>
       </c>
       <c r="D179" t="n">
-        <v>731.28</v>
+        <v>767.58</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3846,17 +3846,17 @@
         <v>46218</v>
       </c>
       <c r="B180" t="n">
-        <v>1317</v>
+        <v>2359</v>
       </c>
       <c r="C180" t="n">
-        <v>3179</v>
+        <v>8888</v>
       </c>
       <c r="D180" t="n">
-        <v>991.6799999999999</v>
+        <v>381.95</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3865,17 +3865,17 @@
         <v>46218</v>
       </c>
       <c r="B181" t="n">
-        <v>1993</v>
+        <v>285</v>
       </c>
       <c r="C181" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D181" t="n">
-        <v>2875.39</v>
+        <v>364.99</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3884,13 +3884,13 @@
         <v>46218</v>
       </c>
       <c r="B182" t="n">
-        <v>1632</v>
+        <v>2114</v>
       </c>
       <c r="C182" t="n">
         <v>8888</v>
       </c>
       <c r="D182" t="n">
-        <v>564.55</v>
+        <v>2726.04</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -3903,17 +3903,17 @@
         <v>46218</v>
       </c>
       <c r="B183" t="n">
-        <v>1890</v>
+        <v>953</v>
       </c>
       <c r="C183" t="n">
-        <v>3449</v>
+        <v>8888</v>
       </c>
       <c r="D183" t="n">
-        <v>3590.04</v>
+        <v>2889.63</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3922,17 +3922,17 @@
         <v>46218</v>
       </c>
       <c r="B184" t="n">
-        <v>451</v>
+        <v>1102</v>
       </c>
       <c r="C184" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D184" t="n">
-        <v>445.58</v>
+        <v>3093.73</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3941,13 +3941,13 @@
         <v>46218</v>
       </c>
       <c r="B185" t="n">
-        <v>2749</v>
+        <v>1465</v>
       </c>
       <c r="C185" t="n">
         <v>8888</v>
       </c>
       <c r="D185" t="n">
-        <v>1860.64</v>
+        <v>4281.39</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -3960,17 +3960,17 @@
         <v>46218</v>
       </c>
       <c r="B186" t="n">
-        <v>1117</v>
+        <v>619</v>
       </c>
       <c r="C186" t="n">
         <v>8888</v>
       </c>
       <c r="D186" t="n">
-        <v>342.2</v>
+        <v>2021.67</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
         <v>46218</v>
       </c>
       <c r="B187" t="n">
-        <v>1478</v>
+        <v>2716</v>
       </c>
       <c r="C187" t="n">
         <v>8888</v>
       </c>
       <c r="D187" t="n">
-        <v>875.34</v>
+        <v>601.58</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -3998,17 +3998,17 @@
         <v>46218</v>
       </c>
       <c r="B188" t="n">
-        <v>2491</v>
+        <v>2767</v>
       </c>
       <c r="C188" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D188" t="n">
-        <v>650.4299999999999</v>
+        <v>1135.64</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4017,13 +4017,13 @@
         <v>46218</v>
       </c>
       <c r="B189" t="n">
-        <v>2015</v>
+        <v>2245</v>
       </c>
       <c r="C189" t="n">
         <v>8888</v>
       </c>
       <c r="D189" t="n">
-        <v>4436.15</v>
+        <v>427.51</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -4036,17 +4036,17 @@
         <v>46218</v>
       </c>
       <c r="B190" t="n">
-        <v>1890</v>
+        <v>2197</v>
       </c>
       <c r="C190" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D190" t="n">
-        <v>1674.57</v>
+        <v>1085.45</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4055,13 +4055,13 @@
         <v>46218</v>
       </c>
       <c r="B191" t="n">
-        <v>2782</v>
+        <v>2657</v>
       </c>
       <c r="C191" t="n">
         <v>8888</v>
       </c>
       <c r="D191" t="n">
-        <v>1786.32</v>
+        <v>2683.06</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -4074,13 +4074,13 @@
         <v>46218</v>
       </c>
       <c r="B192" t="n">
-        <v>483</v>
+        <v>451</v>
       </c>
       <c r="C192" t="n">
-        <v>841</v>
+        <v>3403</v>
       </c>
       <c r="D192" t="n">
-        <v>1393.15</v>
+        <v>2091.77</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -4093,13 +4093,13 @@
         <v>46218</v>
       </c>
       <c r="B193" t="n">
-        <v>2133</v>
+        <v>1116</v>
       </c>
       <c r="C193" t="n">
-        <v>213</v>
+        <v>13148</v>
       </c>
       <c r="D193" t="n">
-        <v>526.8</v>
+        <v>207.91</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -4112,17 +4112,17 @@
         <v>46218</v>
       </c>
       <c r="B194" t="n">
-        <v>351</v>
+        <v>1277</v>
       </c>
       <c r="C194" t="n">
-        <v>3009</v>
+        <v>8888</v>
       </c>
       <c r="D194" t="n">
-        <v>416.36</v>
+        <v>1949</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4131,17 +4131,17 @@
         <v>46218</v>
       </c>
       <c r="B195" t="n">
-        <v>2250</v>
+        <v>131</v>
       </c>
       <c r="C195" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D195" t="n">
-        <v>709.46</v>
+        <v>3850.09</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4150,17 +4150,17 @@
         <v>46218</v>
       </c>
       <c r="B196" t="n">
-        <v>2648</v>
+        <v>2692</v>
       </c>
       <c r="C196" t="n">
         <v>8888</v>
       </c>
       <c r="D196" t="n">
-        <v>1873.52</v>
+        <v>731.28</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4169,17 +4169,17 @@
         <v>46218</v>
       </c>
       <c r="B197" t="n">
-        <v>131</v>
+        <v>1632</v>
       </c>
       <c r="C197" t="n">
         <v>8888</v>
       </c>
       <c r="D197" t="n">
-        <v>1369.91</v>
+        <v>7519.7</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4188,13 +4188,13 @@
         <v>46218</v>
       </c>
       <c r="B198" t="n">
-        <v>2790</v>
+        <v>1317</v>
       </c>
       <c r="C198" t="n">
-        <v>1953</v>
+        <v>3179</v>
       </c>
       <c r="D198" t="n">
-        <v>371.88</v>
+        <v>991.6799999999999</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -4207,17 +4207,17 @@
         <v>46218</v>
       </c>
       <c r="B199" t="n">
-        <v>363</v>
+        <v>1993</v>
       </c>
       <c r="C199" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D199" t="n">
-        <v>635.1</v>
+        <v>2875.39</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4226,13 +4226,13 @@
         <v>46218</v>
       </c>
       <c r="B200" t="n">
-        <v>2716</v>
+        <v>1890</v>
       </c>
       <c r="C200" t="n">
-        <v>1929</v>
+        <v>3449</v>
       </c>
       <c r="D200" t="n">
-        <v>1073.33</v>
+        <v>6313.56</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -4245,17 +4245,17 @@
         <v>46218</v>
       </c>
       <c r="B201" t="n">
-        <v>2639</v>
+        <v>2749</v>
       </c>
       <c r="C201" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D201" t="n">
-        <v>504.09</v>
+        <v>1860.64</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4264,17 +4264,17 @@
         <v>46218</v>
       </c>
       <c r="B202" t="n">
-        <v>2109</v>
+        <v>1117</v>
       </c>
       <c r="C202" t="n">
         <v>8888</v>
       </c>
       <c r="D202" t="n">
-        <v>2293.78</v>
+        <v>342.2</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4283,17 +4283,17 @@
         <v>46218</v>
       </c>
       <c r="B203" t="n">
-        <v>1116</v>
+        <v>42</v>
       </c>
       <c r="C203" t="n">
         <v>8888</v>
       </c>
       <c r="D203" t="n">
-        <v>2919.53</v>
+        <v>280.05</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4302,17 +4302,17 @@
         <v>46218</v>
       </c>
       <c r="B204" t="n">
-        <v>2250</v>
+        <v>1478</v>
       </c>
       <c r="C204" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D204" t="n">
-        <v>1803.76</v>
+        <v>875.34</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4321,13 +4321,13 @@
         <v>46218</v>
       </c>
       <c r="B205" t="n">
-        <v>353</v>
+        <v>2491</v>
       </c>
       <c r="C205" t="n">
         <v>8888</v>
       </c>
       <c r="D205" t="n">
-        <v>108.6</v>
+        <v>650.4299999999999</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -4340,17 +4340,17 @@
         <v>46218</v>
       </c>
       <c r="B206" t="n">
-        <v>2698</v>
+        <v>2015</v>
       </c>
       <c r="C206" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D206" t="n">
-        <v>1230.43</v>
+        <v>4436.15</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4359,17 +4359,17 @@
         <v>46218</v>
       </c>
       <c r="B207" t="n">
-        <v>42</v>
+        <v>1890</v>
       </c>
       <c r="C207" t="n">
-        <v>8888</v>
+        <v>1953</v>
       </c>
       <c r="D207" t="n">
-        <v>79947.14999999999</v>
+        <v>1674.57</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4378,17 +4378,17 @@
         <v>46218</v>
       </c>
       <c r="B208" t="n">
-        <v>772</v>
+        <v>1317</v>
       </c>
       <c r="C208" t="n">
         <v>8888</v>
       </c>
       <c r="D208" t="n">
-        <v>400.25</v>
+        <v>1626.02</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4397,17 +4397,17 @@
         <v>46218</v>
       </c>
       <c r="B209" t="n">
-        <v>2728</v>
+        <v>2782</v>
       </c>
       <c r="C209" t="n">
         <v>8888</v>
       </c>
       <c r="D209" t="n">
-        <v>1397.07</v>
+        <v>1786.32</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4416,17 +4416,17 @@
         <v>46218</v>
       </c>
       <c r="B210" t="n">
-        <v>2197</v>
+        <v>953</v>
       </c>
       <c r="C210" t="n">
-        <v>423</v>
+        <v>8888</v>
       </c>
       <c r="D210" t="n">
-        <v>2267.61</v>
+        <v>364.44</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4435,17 +4435,17 @@
         <v>46218</v>
       </c>
       <c r="B211" t="n">
-        <v>2716</v>
+        <v>2251</v>
       </c>
       <c r="C211" t="n">
-        <v>977</v>
+        <v>8888</v>
       </c>
       <c r="D211" t="n">
-        <v>729.29</v>
+        <v>309.22</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4454,17 +4454,17 @@
         <v>46218</v>
       </c>
       <c r="B212" t="n">
-        <v>1993</v>
+        <v>483</v>
       </c>
       <c r="C212" t="n">
-        <v>8888</v>
+        <v>841</v>
       </c>
       <c r="D212" t="n">
-        <v>456.62</v>
+        <v>2085.09</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4473,15 +4473,414 @@
         <v>46218</v>
       </c>
       <c r="B213" t="n">
+        <v>2133</v>
+      </c>
+      <c r="C213" t="n">
+        <v>213</v>
+      </c>
+      <c r="D213" t="n">
+        <v>526.8</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B214" t="n">
+        <v>351</v>
+      </c>
+      <c r="C214" t="n">
+        <v>3009</v>
+      </c>
+      <c r="D214" t="n">
+        <v>416.36</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B215" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C215" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D215" t="n">
+        <v>709.46</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B216" t="n">
+        <v>2648</v>
+      </c>
+      <c r="C216" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D216" t="n">
+        <v>1873.52</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B217" t="n">
+        <v>131</v>
+      </c>
+      <c r="C217" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D217" t="n">
+        <v>1369.91</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B218" t="n">
+        <v>2790</v>
+      </c>
+      <c r="C218" t="n">
+        <v>1953</v>
+      </c>
+      <c r="D218" t="n">
+        <v>371.88</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B219" t="n">
+        <v>363</v>
+      </c>
+      <c r="C219" t="n">
+        <v>1898</v>
+      </c>
+      <c r="D219" t="n">
+        <v>635.1</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B220" t="n">
+        <v>2716</v>
+      </c>
+      <c r="C220" t="n">
+        <v>1929</v>
+      </c>
+      <c r="D220" t="n">
+        <v>1073.33</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B221" t="n">
+        <v>2298</v>
+      </c>
+      <c r="C221" t="n">
+        <v>675</v>
+      </c>
+      <c r="D221" t="n">
+        <v>401.85</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B222" t="n">
+        <v>2639</v>
+      </c>
+      <c r="C222" t="n">
+        <v>1953</v>
+      </c>
+      <c r="D222" t="n">
+        <v>504.09</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B223" t="n">
+        <v>2109</v>
+      </c>
+      <c r="C223" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D223" t="n">
+        <v>2293.78</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B224" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C224" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D224" t="n">
+        <v>2919.53</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B225" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C225" t="n">
+        <v>27</v>
+      </c>
+      <c r="D225" t="n">
+        <v>1803.76</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B226" t="n">
+        <v>353</v>
+      </c>
+      <c r="C226" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D226" t="n">
+        <v>349.33</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B227" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C227" t="n">
+        <v>874</v>
+      </c>
+      <c r="D227" t="n">
+        <v>1230.43</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B228" t="n">
+        <v>42</v>
+      </c>
+      <c r="C228" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D228" t="n">
+        <v>79947.14999999999</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B229" t="n">
+        <v>772</v>
+      </c>
+      <c r="C229" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D229" t="n">
+        <v>400.25</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B230" t="n">
+        <v>2728</v>
+      </c>
+      <c r="C230" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D230" t="n">
+        <v>1397.07</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B231" t="n">
+        <v>2197</v>
+      </c>
+      <c r="C231" t="n">
+        <v>423</v>
+      </c>
+      <c r="D231" t="n">
+        <v>2267.61</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B232" t="n">
+        <v>2716</v>
+      </c>
+      <c r="C232" t="n">
+        <v>977</v>
+      </c>
+      <c r="D232" t="n">
+        <v>729.29</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B233" t="n">
+        <v>1993</v>
+      </c>
+      <c r="C233" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D233" t="n">
+        <v>456.62</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B234" t="n">
         <v>629</v>
       </c>
-      <c r="C213" t="n">
+      <c r="C234" t="n">
         <v>675</v>
       </c>
-      <c r="D213" t="n">
+      <c r="D234" t="n">
         <v>1054.76</v>
       </c>
-      <c r="E213" t="inlineStr">
+      <c r="E234" t="inlineStr">
         <is>
           <t>TELEMARKETING</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 17:00:05
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E234"/>
+  <dimension ref="A1:E248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -660,7 +660,7 @@
         <v>3179</v>
       </c>
       <c r="D12" t="n">
-        <v>2603.16</v>
+        <v>4618.88</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1034,17 +1034,17 @@
         <v>46218</v>
       </c>
       <c r="B32" t="n">
-        <v>2695</v>
+        <v>2641</v>
       </c>
       <c r="C32" t="n">
         <v>8888</v>
       </c>
       <c r="D32" t="n">
-        <v>411.42</v>
+        <v>2527.79</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1053,17 +1053,17 @@
         <v>46218</v>
       </c>
       <c r="B33" t="n">
-        <v>525</v>
+        <v>2695</v>
       </c>
       <c r="C33" t="n">
         <v>8888</v>
       </c>
       <c r="D33" t="n">
-        <v>408.25</v>
+        <v>411.42</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1072,17 +1072,17 @@
         <v>46218</v>
       </c>
       <c r="B34" t="n">
-        <v>1808</v>
+        <v>525</v>
       </c>
       <c r="C34" t="n">
         <v>8888</v>
       </c>
       <c r="D34" t="n">
-        <v>695.3200000000001</v>
+        <v>408.25</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1091,17 +1091,17 @@
         <v>46218</v>
       </c>
       <c r="B35" t="n">
-        <v>609</v>
+        <v>1808</v>
       </c>
       <c r="C35" t="n">
         <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>1909.37</v>
+        <v>695.3200000000001</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1110,17 @@
         <v>46218</v>
       </c>
       <c r="B36" t="n">
-        <v>949</v>
+        <v>609</v>
       </c>
       <c r="C36" t="n">
-        <v>1134</v>
+        <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>30.46</v>
+        <v>1909.37</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1129,13 +1129,13 @@
         <v>46218</v>
       </c>
       <c r="B37" t="n">
-        <v>42</v>
+        <v>949</v>
       </c>
       <c r="C37" t="n">
-        <v>1139</v>
+        <v>1134</v>
       </c>
       <c r="D37" t="n">
-        <v>358.97</v>
+        <v>30.46</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1148,17 +1148,17 @@
         <v>46218</v>
       </c>
       <c r="B38" t="n">
-        <v>2499</v>
+        <v>42</v>
       </c>
       <c r="C38" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D38" t="n">
-        <v>1049.3</v>
+        <v>358.97</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1167,13 +1167,13 @@
         <v>46218</v>
       </c>
       <c r="B39" t="n">
-        <v>58</v>
+        <v>2499</v>
       </c>
       <c r="C39" t="n">
         <v>8888</v>
       </c>
       <c r="D39" t="n">
-        <v>499.11</v>
+        <v>1049.3</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1186,13 +1186,13 @@
         <v>46218</v>
       </c>
       <c r="B40" t="n">
-        <v>2245</v>
+        <v>58</v>
       </c>
       <c r="C40" t="n">
         <v>8888</v>
       </c>
       <c r="D40" t="n">
-        <v>2740.06</v>
+        <v>1643.73</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1205,17 +1205,17 @@
         <v>46218</v>
       </c>
       <c r="B41" t="n">
-        <v>325</v>
+        <v>2245</v>
       </c>
       <c r="C41" t="n">
         <v>8888</v>
       </c>
       <c r="D41" t="n">
-        <v>952.75</v>
+        <v>2740.06</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1224,17 +1224,17 @@
         <v>46218</v>
       </c>
       <c r="B42" t="n">
-        <v>2383</v>
+        <v>325</v>
       </c>
       <c r="C42" t="n">
         <v>8888</v>
       </c>
       <c r="D42" t="n">
-        <v>7926.02</v>
+        <v>952.75</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1243,17 +1243,17 @@
         <v>46218</v>
       </c>
       <c r="B43" t="n">
-        <v>1117</v>
+        <v>2383</v>
       </c>
       <c r="C43" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D43" t="n">
-        <v>916.72</v>
+        <v>7926.02</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1262,17 +1262,17 @@
         <v>46218</v>
       </c>
       <c r="B44" t="n">
-        <v>2279</v>
+        <v>1117</v>
       </c>
       <c r="C44" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D44" t="n">
-        <v>712.66</v>
+        <v>916.72</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1281,17 +1281,17 @@
         <v>46218</v>
       </c>
       <c r="B45" t="n">
-        <v>535</v>
+        <v>374</v>
       </c>
       <c r="C45" t="n">
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>5836.12</v>
+        <v>2810.86</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1300,13 +1300,13 @@
         <v>46218</v>
       </c>
       <c r="B46" t="n">
-        <v>535</v>
+        <v>2279</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>1352.51</v>
+        <v>712.66</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1319,17 +1319,17 @@
         <v>46218</v>
       </c>
       <c r="B47" t="n">
-        <v>2678</v>
+        <v>535</v>
       </c>
       <c r="C47" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D47" t="n">
-        <v>364.96</v>
+        <v>5836.12</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1338,13 +1338,13 @@
         <v>46218</v>
       </c>
       <c r="B48" t="n">
-        <v>2345</v>
+        <v>535</v>
       </c>
       <c r="C48" t="n">
         <v>8888</v>
       </c>
       <c r="D48" t="n">
-        <v>863.16</v>
+        <v>1352.51</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1357,17 +1357,17 @@
         <v>46218</v>
       </c>
       <c r="B49" t="n">
-        <v>945</v>
+        <v>2678</v>
       </c>
       <c r="C49" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D49" t="n">
-        <v>27337.21</v>
+        <v>364.96</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>PEDIDO ELETRÔNICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1376,17 +1376,17 @@
         <v>46218</v>
       </c>
       <c r="B50" t="n">
-        <v>2686</v>
+        <v>2345</v>
       </c>
       <c r="C50" t="n">
         <v>8888</v>
       </c>
       <c r="D50" t="n">
-        <v>684.2</v>
+        <v>863.16</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1395,17 +1395,17 @@
         <v>46218</v>
       </c>
       <c r="B51" t="n">
-        <v>438</v>
+        <v>945</v>
       </c>
       <c r="C51" t="n">
         <v>8888</v>
       </c>
       <c r="D51" t="n">
-        <v>220.06</v>
+        <v>27337.21</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>PEDIDO ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
         <v>46218</v>
       </c>
       <c r="B52" t="n">
-        <v>664</v>
+        <v>2686</v>
       </c>
       <c r="C52" t="n">
         <v>8888</v>
       </c>
       <c r="D52" t="n">
-        <v>2598.01</v>
+        <v>684.2</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1433,17 +1433,17 @@
         <v>46218</v>
       </c>
       <c r="B53" t="n">
-        <v>353</v>
+        <v>438</v>
       </c>
       <c r="C53" t="n">
-        <v>3179</v>
+        <v>8888</v>
       </c>
       <c r="D53" t="n">
-        <v>495.84</v>
+        <v>220.06</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1452,13 +1452,13 @@
         <v>46218</v>
       </c>
       <c r="B54" t="n">
-        <v>1293</v>
+        <v>664</v>
       </c>
       <c r="C54" t="n">
         <v>8888</v>
       </c>
       <c r="D54" t="n">
-        <v>3129.07</v>
+        <v>6275.01</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1471,17 +1471,17 @@
         <v>46218</v>
       </c>
       <c r="B55" t="n">
-        <v>2279</v>
+        <v>353</v>
       </c>
       <c r="C55" t="n">
-        <v>8888</v>
+        <v>3179</v>
       </c>
       <c r="D55" t="n">
-        <v>2753.96</v>
+        <v>495.84</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1490,13 +1490,13 @@
         <v>46218</v>
       </c>
       <c r="B56" t="n">
-        <v>1937</v>
+        <v>1293</v>
       </c>
       <c r="C56" t="n">
         <v>8888</v>
       </c>
       <c r="D56" t="n">
-        <v>1685.72</v>
+        <v>3129.07</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1509,17 +1509,17 @@
         <v>46218</v>
       </c>
       <c r="B57" t="n">
-        <v>941</v>
+        <v>2279</v>
       </c>
       <c r="C57" t="n">
         <v>8888</v>
       </c>
       <c r="D57" t="n">
-        <v>864.14</v>
+        <v>2753.96</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1528,17 +1528,17 @@
         <v>46218</v>
       </c>
       <c r="B58" t="n">
-        <v>1137</v>
+        <v>1937</v>
       </c>
       <c r="C58" t="n">
         <v>8888</v>
       </c>
       <c r="D58" t="n">
-        <v>1947.93</v>
+        <v>1685.72</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1547,17 +1547,17 @@
         <v>46218</v>
       </c>
       <c r="B59" t="n">
-        <v>2631</v>
+        <v>941</v>
       </c>
       <c r="C59" t="n">
-        <v>2853</v>
+        <v>8888</v>
       </c>
       <c r="D59" t="n">
-        <v>1272.12</v>
+        <v>864.14</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1566,17 +1566,17 @@
         <v>46218</v>
       </c>
       <c r="B60" t="n">
-        <v>2793</v>
+        <v>1137</v>
       </c>
       <c r="C60" t="n">
-        <v>977</v>
+        <v>8888</v>
       </c>
       <c r="D60" t="n">
-        <v>1188.59</v>
+        <v>1947.93</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1585,17 +1585,17 @@
         <v>46218</v>
       </c>
       <c r="B61" t="n">
-        <v>374</v>
+        <v>2631</v>
       </c>
       <c r="C61" t="n">
-        <v>8888</v>
+        <v>2853</v>
       </c>
       <c r="D61" t="n">
-        <v>2103.29</v>
+        <v>1272.12</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1604,17 +1604,17 @@
         <v>46218</v>
       </c>
       <c r="B62" t="n">
-        <v>2802</v>
+        <v>2793</v>
       </c>
       <c r="C62" t="n">
-        <v>8888</v>
+        <v>977</v>
       </c>
       <c r="D62" t="n">
-        <v>1264.57</v>
+        <v>1188.59</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1623,13 +1623,13 @@
         <v>46218</v>
       </c>
       <c r="B63" t="n">
-        <v>451</v>
+        <v>2802</v>
       </c>
       <c r="C63" t="n">
         <v>8888</v>
       </c>
       <c r="D63" t="n">
-        <v>757.5700000000001</v>
+        <v>1264.57</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1642,17 +1642,17 @@
         <v>46218</v>
       </c>
       <c r="B64" t="n">
-        <v>374</v>
+        <v>451</v>
       </c>
       <c r="C64" t="n">
         <v>8888</v>
       </c>
       <c r="D64" t="n">
-        <v>44.6</v>
+        <v>757.5700000000001</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1661,17 +1661,17 @@
         <v>46218</v>
       </c>
       <c r="B65" t="n">
-        <v>703</v>
+        <v>374</v>
       </c>
       <c r="C65" t="n">
         <v>8888</v>
       </c>
       <c r="D65" t="n">
-        <v>12155.46</v>
+        <v>44.6</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1680,17 +1680,17 @@
         <v>46218</v>
       </c>
       <c r="B66" t="n">
-        <v>1756</v>
+        <v>703</v>
       </c>
       <c r="C66" t="n">
         <v>8888</v>
       </c>
       <c r="D66" t="n">
-        <v>996.17</v>
+        <v>12155.46</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1699,13 +1699,13 @@
         <v>46218</v>
       </c>
       <c r="B67" t="n">
-        <v>1956</v>
+        <v>1756</v>
       </c>
       <c r="C67" t="n">
         <v>8888</v>
       </c>
       <c r="D67" t="n">
-        <v>4557.34</v>
+        <v>4416.47</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1718,17 +1718,17 @@
         <v>46218</v>
       </c>
       <c r="B68" t="n">
-        <v>925</v>
+        <v>1956</v>
       </c>
       <c r="C68" t="n">
         <v>8888</v>
       </c>
       <c r="D68" t="n">
-        <v>651.59</v>
+        <v>4557.34</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1737,17 +1737,17 @@
         <v>46218</v>
       </c>
       <c r="B69" t="n">
-        <v>2648</v>
+        <v>925</v>
       </c>
       <c r="C69" t="n">
         <v>8888</v>
       </c>
       <c r="D69" t="n">
-        <v>1594.42</v>
+        <v>651.59</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1756,13 +1756,13 @@
         <v>46218</v>
       </c>
       <c r="B70" t="n">
-        <v>2714</v>
+        <v>941</v>
       </c>
       <c r="C70" t="n">
-        <v>519</v>
+        <v>977</v>
       </c>
       <c r="D70" t="n">
-        <v>61939.22</v>
+        <v>359.73</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -1775,17 +1775,17 @@
         <v>46218</v>
       </c>
       <c r="B71" t="n">
-        <v>483</v>
+        <v>2648</v>
       </c>
       <c r="C71" t="n">
         <v>8888</v>
       </c>
       <c r="D71" t="n">
-        <v>8624.57</v>
+        <v>1594.42</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1794,17 +1794,17 @@
         <v>46218</v>
       </c>
       <c r="B72" t="n">
-        <v>1075</v>
+        <v>663</v>
       </c>
       <c r="C72" t="n">
         <v>8888</v>
       </c>
       <c r="D72" t="n">
-        <v>11607.79</v>
+        <v>6645.33</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1813,17 +1813,17 @@
         <v>46218</v>
       </c>
       <c r="B73" t="n">
-        <v>629</v>
+        <v>2714</v>
       </c>
       <c r="C73" t="n">
-        <v>8888</v>
+        <v>519</v>
       </c>
       <c r="D73" t="n">
-        <v>9233.719999999999</v>
+        <v>61939.22</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1832,17 +1832,17 @@
         <v>46218</v>
       </c>
       <c r="B74" t="n">
-        <v>1983</v>
+        <v>483</v>
       </c>
       <c r="C74" t="n">
-        <v>841</v>
+        <v>8888</v>
       </c>
       <c r="D74" t="n">
-        <v>243.92</v>
+        <v>11360.2</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1851,17 +1851,17 @@
         <v>46218</v>
       </c>
       <c r="B75" t="n">
-        <v>1137</v>
+        <v>1075</v>
       </c>
       <c r="C75" t="n">
         <v>8888</v>
       </c>
       <c r="D75" t="n">
-        <v>3578.51</v>
+        <v>11607.79</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1870,17 +1870,17 @@
         <v>46218</v>
       </c>
       <c r="B76" t="n">
-        <v>2651</v>
+        <v>629</v>
       </c>
       <c r="C76" t="n">
         <v>8888</v>
       </c>
       <c r="D76" t="n">
-        <v>1296.58</v>
+        <v>9233.719999999999</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1889,17 +1889,17 @@
         <v>46218</v>
       </c>
       <c r="B77" t="n">
-        <v>663</v>
+        <v>1983</v>
       </c>
       <c r="C77" t="n">
-        <v>8888</v>
+        <v>841</v>
       </c>
       <c r="D77" t="n">
-        <v>5851.1</v>
+        <v>243.92</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1908,17 +1908,17 @@
         <v>46218</v>
       </c>
       <c r="B78" t="n">
-        <v>1956</v>
+        <v>1137</v>
       </c>
       <c r="C78" t="n">
-        <v>423</v>
+        <v>8888</v>
       </c>
       <c r="D78" t="n">
-        <v>1416.35</v>
+        <v>3578.51</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1927,17 +1927,17 @@
         <v>46218</v>
       </c>
       <c r="B79" t="n">
-        <v>2709</v>
+        <v>2651</v>
       </c>
       <c r="C79" t="n">
         <v>8888</v>
       </c>
       <c r="D79" t="n">
-        <v>547.6900000000001</v>
+        <v>1296.58</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1946,13 +1946,13 @@
         <v>46218</v>
       </c>
       <c r="B80" t="n">
-        <v>1308</v>
+        <v>2789</v>
       </c>
       <c r="C80" t="n">
         <v>8888</v>
       </c>
       <c r="D80" t="n">
-        <v>1460.53</v>
+        <v>1293.93</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -1965,17 +1965,17 @@
         <v>46218</v>
       </c>
       <c r="B81" t="n">
-        <v>2026</v>
+        <v>1956</v>
       </c>
       <c r="C81" t="n">
-        <v>8888</v>
+        <v>423</v>
       </c>
       <c r="D81" t="n">
-        <v>2237.62</v>
+        <v>1416.35</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1984,17 +1984,17 @@
         <v>46218</v>
       </c>
       <c r="B82" t="n">
-        <v>2789</v>
+        <v>2709</v>
       </c>
       <c r="C82" t="n">
         <v>8888</v>
       </c>
       <c r="D82" t="n">
-        <v>747.77</v>
+        <v>547.6900000000001</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2003,17 +2003,17 @@
         <v>46218</v>
       </c>
       <c r="B83" t="n">
-        <v>89</v>
+        <v>1308</v>
       </c>
       <c r="C83" t="n">
-        <v>13148</v>
+        <v>8888</v>
       </c>
       <c r="D83" t="n">
-        <v>1883.74</v>
+        <v>1460.53</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2022,17 +2022,17 @@
         <v>46218</v>
       </c>
       <c r="B84" t="n">
-        <v>2709</v>
+        <v>2026</v>
       </c>
       <c r="C84" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D84" t="n">
-        <v>390.19</v>
+        <v>2237.62</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2047,11 +2047,11 @@
         <v>8888</v>
       </c>
       <c r="D85" t="n">
-        <v>691.37</v>
+        <v>747.77</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2060,17 +2060,17 @@
         <v>46218</v>
       </c>
       <c r="B86" t="n">
-        <v>2345</v>
+        <v>89</v>
       </c>
       <c r="C86" t="n">
-        <v>8888</v>
+        <v>13148</v>
       </c>
       <c r="D86" t="n">
-        <v>748.86</v>
+        <v>1883.74</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2079,13 +2079,13 @@
         <v>46218</v>
       </c>
       <c r="B87" t="n">
-        <v>2765</v>
+        <v>2709</v>
       </c>
       <c r="C87" t="n">
-        <v>1883</v>
+        <v>2220</v>
       </c>
       <c r="D87" t="n">
-        <v>3638.6</v>
+        <v>390.19</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2098,17 +2098,17 @@
         <v>46218</v>
       </c>
       <c r="B88" t="n">
-        <v>569</v>
+        <v>2345</v>
       </c>
       <c r="C88" t="n">
         <v>8888</v>
       </c>
       <c r="D88" t="n">
-        <v>995.33</v>
+        <v>748.86</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2117,17 +2117,17 @@
         <v>46218</v>
       </c>
       <c r="B89" t="n">
-        <v>360</v>
+        <v>1983</v>
       </c>
       <c r="C89" t="n">
-        <v>546</v>
+        <v>8888</v>
       </c>
       <c r="D89" t="n">
-        <v>1609.68</v>
+        <v>851.7</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2136,17 +2136,17 @@
         <v>46218</v>
       </c>
       <c r="B90" t="n">
-        <v>2308</v>
+        <v>2765</v>
       </c>
       <c r="C90" t="n">
-        <v>8888</v>
+        <v>1883</v>
       </c>
       <c r="D90" t="n">
-        <v>488.69</v>
+        <v>3638.6</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2155,17 +2155,17 @@
         <v>46218</v>
       </c>
       <c r="B91" t="n">
-        <v>2211</v>
+        <v>569</v>
       </c>
       <c r="C91" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D91" t="n">
-        <v>1526.94</v>
+        <v>995.33</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2174,17 +2174,17 @@
         <v>46218</v>
       </c>
       <c r="B92" t="n">
-        <v>559</v>
+        <v>360</v>
       </c>
       <c r="C92" t="n">
-        <v>8888</v>
+        <v>546</v>
       </c>
       <c r="D92" t="n">
-        <v>859.92</v>
+        <v>1609.68</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2193,17 +2193,17 @@
         <v>46218</v>
       </c>
       <c r="B93" t="n">
-        <v>890</v>
+        <v>2711</v>
       </c>
       <c r="C93" t="n">
-        <v>8888</v>
+        <v>1953</v>
       </c>
       <c r="D93" t="n">
-        <v>387.2</v>
+        <v>150.27</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2212,17 +2212,17 @@
         <v>46218</v>
       </c>
       <c r="B94" t="n">
-        <v>2768</v>
+        <v>2308</v>
       </c>
       <c r="C94" t="n">
         <v>8888</v>
       </c>
       <c r="D94" t="n">
-        <v>6523.26</v>
+        <v>488.69</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2231,17 +2231,17 @@
         <v>46218</v>
       </c>
       <c r="B95" t="n">
-        <v>1063</v>
+        <v>2211</v>
       </c>
       <c r="C95" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D95" t="n">
-        <v>4487.11</v>
+        <v>1526.94</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2250,17 +2250,17 @@
         <v>46218</v>
       </c>
       <c r="B96" t="n">
-        <v>2279</v>
+        <v>559</v>
       </c>
       <c r="C96" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D96" t="n">
-        <v>652.51</v>
+        <v>859.92</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2269,17 +2269,17 @@
         <v>46218</v>
       </c>
       <c r="B97" t="n">
-        <v>1299</v>
+        <v>890</v>
       </c>
       <c r="C97" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D97" t="n">
-        <v>1435.52</v>
+        <v>387.2</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2288,17 +2288,17 @@
         <v>46218</v>
       </c>
       <c r="B98" t="n">
-        <v>1478</v>
+        <v>2768</v>
       </c>
       <c r="C98" t="n">
-        <v>675</v>
+        <v>8888</v>
       </c>
       <c r="D98" t="n">
-        <v>1600.01</v>
+        <v>6523.26</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2307,17 +2307,17 @@
         <v>46218</v>
       </c>
       <c r="B99" t="n">
-        <v>285</v>
+        <v>1063</v>
       </c>
       <c r="C99" t="n">
         <v>8888</v>
       </c>
       <c r="D99" t="n">
-        <v>3349.8</v>
+        <v>4487.11</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2326,17 +2326,17 @@
         <v>46218</v>
       </c>
       <c r="B100" t="n">
-        <v>477</v>
+        <v>2279</v>
       </c>
       <c r="C100" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D100" t="n">
-        <v>917.33</v>
+        <v>652.51</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2345,17 +2345,17 @@
         <v>46218</v>
       </c>
       <c r="B101" t="n">
-        <v>1983</v>
+        <v>1299</v>
       </c>
       <c r="C101" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D101" t="n">
-        <v>5115.01</v>
+        <v>1435.52</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2364,13 +2364,13 @@
         <v>46218</v>
       </c>
       <c r="B102" t="n">
-        <v>477</v>
+        <v>1478</v>
       </c>
       <c r="C102" t="n">
-        <v>58</v>
+        <v>675</v>
       </c>
       <c r="D102" t="n">
-        <v>1540.55</v>
+        <v>1967.85</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2383,17 +2383,17 @@
         <v>46218</v>
       </c>
       <c r="B103" t="n">
-        <v>1063</v>
+        <v>767</v>
       </c>
       <c r="C103" t="n">
         <v>8888</v>
       </c>
       <c r="D103" t="n">
-        <v>2549.86</v>
+        <v>3292.44</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2402,13 +2402,13 @@
         <v>46218</v>
       </c>
       <c r="B104" t="n">
-        <v>424</v>
+        <v>285</v>
       </c>
       <c r="C104" t="n">
         <v>8888</v>
       </c>
       <c r="D104" t="n">
-        <v>1362.42</v>
+        <v>3349.8</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2421,17 +2421,17 @@
         <v>46218</v>
       </c>
       <c r="B105" t="n">
-        <v>675</v>
+        <v>477</v>
       </c>
       <c r="C105" t="n">
         <v>8888</v>
       </c>
       <c r="D105" t="n">
-        <v>616.73</v>
+        <v>917.33</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2440,17 +2440,17 @@
         <v>46218</v>
       </c>
       <c r="B106" t="n">
-        <v>663</v>
+        <v>1983</v>
       </c>
       <c r="C106" t="n">
         <v>8888</v>
       </c>
       <c r="D106" t="n">
-        <v>255.13</v>
+        <v>5115.01</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2459,17 +2459,17 @@
         <v>46218</v>
       </c>
       <c r="B107" t="n">
-        <v>1993</v>
+        <v>477</v>
       </c>
       <c r="C107" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D107" t="n">
-        <v>362.63</v>
+        <v>1540.55</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2478,17 +2478,17 @@
         <v>46218</v>
       </c>
       <c r="B108" t="n">
-        <v>1465</v>
+        <v>1937</v>
       </c>
       <c r="C108" t="n">
         <v>8888</v>
       </c>
       <c r="D108" t="n">
-        <v>3373.83</v>
+        <v>2600.61</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2497,17 +2497,17 @@
         <v>46218</v>
       </c>
       <c r="B109" t="n">
-        <v>89</v>
+        <v>1063</v>
       </c>
       <c r="C109" t="n">
         <v>8888</v>
       </c>
       <c r="D109" t="n">
-        <v>479</v>
+        <v>2549.86</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2516,17 +2516,17 @@
         <v>46218</v>
       </c>
       <c r="B110" t="n">
-        <v>595</v>
+        <v>2584</v>
       </c>
       <c r="C110" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D110" t="n">
-        <v>18084.5</v>
+        <v>756.16</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2535,17 +2535,17 @@
         <v>46218</v>
       </c>
       <c r="B111" t="n">
-        <v>2696</v>
+        <v>58</v>
       </c>
       <c r="C111" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D111" t="n">
-        <v>1597.76</v>
+        <v>558.03</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2554,17 +2554,17 @@
         <v>46218</v>
       </c>
       <c r="B112" t="n">
-        <v>360</v>
+        <v>424</v>
       </c>
       <c r="C112" t="n">
         <v>8888</v>
       </c>
       <c r="D112" t="n">
-        <v>4596.89</v>
+        <v>1362.42</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2573,17 +2573,17 @@
         <v>46218</v>
       </c>
       <c r="B113" t="n">
-        <v>1465</v>
+        <v>675</v>
       </c>
       <c r="C113" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D113" t="n">
-        <v>777.2</v>
+        <v>616.73</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2592,17 +2592,17 @@
         <v>46218</v>
       </c>
       <c r="B114" t="n">
-        <v>947</v>
+        <v>663</v>
       </c>
       <c r="C114" t="n">
         <v>8888</v>
       </c>
       <c r="D114" t="n">
-        <v>5115.36</v>
+        <v>255.13</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>PEDIDO ELETRÔNICO</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2611,17 +2611,17 @@
         <v>46218</v>
       </c>
       <c r="B115" t="n">
-        <v>2178</v>
+        <v>1993</v>
       </c>
       <c r="C115" t="n">
         <v>8888</v>
       </c>
       <c r="D115" t="n">
-        <v>619.92</v>
+        <v>362.63</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2630,17 +2630,17 @@
         <v>46218</v>
       </c>
       <c r="B116" t="n">
-        <v>2026</v>
+        <v>1465</v>
       </c>
       <c r="C116" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D116" t="n">
-        <v>3418.07</v>
+        <v>3373.83</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2649,17 +2649,17 @@
         <v>46218</v>
       </c>
       <c r="B117" t="n">
-        <v>630</v>
+        <v>89</v>
       </c>
       <c r="C117" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D117" t="n">
-        <v>1801.63</v>
+        <v>479</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2668,17 +2668,17 @@
         <v>46218</v>
       </c>
       <c r="B118" t="n">
-        <v>1937</v>
+        <v>595</v>
       </c>
       <c r="C118" t="n">
         <v>8888</v>
       </c>
       <c r="D118" t="n">
-        <v>2132.95</v>
+        <v>18084.5</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2687,17 +2687,17 @@
         <v>46218</v>
       </c>
       <c r="B119" t="n">
-        <v>2577</v>
+        <v>2696</v>
       </c>
       <c r="C119" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D119" t="n">
-        <v>1647.08</v>
+        <v>1597.76</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2706,17 +2706,17 @@
         <v>46218</v>
       </c>
       <c r="B120" t="n">
-        <v>1293</v>
+        <v>360</v>
       </c>
       <c r="C120" t="n">
         <v>8888</v>
       </c>
       <c r="D120" t="n">
-        <v>2135.89</v>
+        <v>4596.89</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2725,17 +2725,17 @@
         <v>46218</v>
       </c>
       <c r="B121" t="n">
-        <v>2607</v>
+        <v>1465</v>
       </c>
       <c r="C121" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D121" t="n">
-        <v>490.31</v>
+        <v>777.2</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2744,17 +2744,17 @@
         <v>46218</v>
       </c>
       <c r="B122" t="n">
-        <v>1317</v>
+        <v>947</v>
       </c>
       <c r="C122" t="n">
         <v>8888</v>
       </c>
       <c r="D122" t="n">
-        <v>907.72</v>
+        <v>5115.36</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>PEDIDO ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -2763,17 +2763,17 @@
         <v>46218</v>
       </c>
       <c r="B123" t="n">
-        <v>767</v>
+        <v>2178</v>
       </c>
       <c r="C123" t="n">
         <v>8888</v>
       </c>
       <c r="D123" t="n">
-        <v>637.23</v>
+        <v>619.92</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2782,13 +2782,13 @@
         <v>46218</v>
       </c>
       <c r="B124" t="n">
-        <v>2571</v>
+        <v>2026</v>
       </c>
       <c r="C124" t="n">
-        <v>1312</v>
+        <v>1929</v>
       </c>
       <c r="D124" t="n">
-        <v>268.53</v>
+        <v>5293.13</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -2801,17 +2801,17 @@
         <v>46218</v>
       </c>
       <c r="B125" t="n">
-        <v>1937</v>
+        <v>630</v>
       </c>
       <c r="C125" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D125" t="n">
-        <v>1803.32</v>
+        <v>1801.63</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2820,17 +2820,17 @@
         <v>46218</v>
       </c>
       <c r="B126" t="n">
-        <v>20</v>
+        <v>1937</v>
       </c>
       <c r="C126" t="n">
         <v>8888</v>
       </c>
       <c r="D126" t="n">
-        <v>745.55</v>
+        <v>2132.95</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2839,17 +2839,17 @@
         <v>46218</v>
       </c>
       <c r="B127" t="n">
-        <v>1063</v>
+        <v>2577</v>
       </c>
       <c r="C127" t="n">
         <v>8888</v>
       </c>
       <c r="D127" t="n">
-        <v>1113.08</v>
+        <v>1647.08</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2858,17 +2858,17 @@
         <v>46218</v>
       </c>
       <c r="B128" t="n">
-        <v>2631</v>
+        <v>1293</v>
       </c>
       <c r="C128" t="n">
         <v>8888</v>
       </c>
       <c r="D128" t="n">
-        <v>1447.86</v>
+        <v>2135.89</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2877,13 +2877,13 @@
         <v>46218</v>
       </c>
       <c r="B129" t="n">
-        <v>1906</v>
+        <v>2607</v>
       </c>
       <c r="C129" t="n">
         <v>8888</v>
       </c>
       <c r="D129" t="n">
-        <v>2774.84</v>
+        <v>490.31</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -2896,17 +2896,17 @@
         <v>46218</v>
       </c>
       <c r="B130" t="n">
-        <v>1756</v>
+        <v>1317</v>
       </c>
       <c r="C130" t="n">
         <v>8888</v>
       </c>
       <c r="D130" t="n">
-        <v>2275.21</v>
+        <v>907.72</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2915,17 +2915,17 @@
         <v>46218</v>
       </c>
       <c r="B131" t="n">
-        <v>477</v>
+        <v>619</v>
       </c>
       <c r="C131" t="n">
         <v>8888</v>
       </c>
       <c r="D131" t="n">
-        <v>707.52</v>
+        <v>1081.74</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2934,17 +2934,17 @@
         <v>46218</v>
       </c>
       <c r="B132" t="n">
-        <v>2660</v>
+        <v>2571</v>
       </c>
       <c r="C132" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D132" t="n">
-        <v>2684.97</v>
+        <v>268.53</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2953,17 +2953,17 @@
         <v>46218</v>
       </c>
       <c r="B133" t="n">
-        <v>569</v>
+        <v>20</v>
       </c>
       <c r="C133" t="n">
         <v>8888</v>
       </c>
       <c r="D133" t="n">
-        <v>33214.39</v>
+        <v>745.55</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2972,13 +2972,13 @@
         <v>46218</v>
       </c>
       <c r="B134" t="n">
-        <v>483</v>
+        <v>1063</v>
       </c>
       <c r="C134" t="n">
         <v>8888</v>
       </c>
       <c r="D134" t="n">
-        <v>2401.99</v>
+        <v>1113.08</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -2991,17 +2991,17 @@
         <v>46218</v>
       </c>
       <c r="B135" t="n">
-        <v>483</v>
+        <v>2631</v>
       </c>
       <c r="C135" t="n">
         <v>8888</v>
       </c>
       <c r="D135" t="n">
-        <v>1124.96</v>
+        <v>1447.86</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3010,17 +3010,17 @@
         <v>46218</v>
       </c>
       <c r="B136" t="n">
-        <v>2089</v>
+        <v>1906</v>
       </c>
       <c r="C136" t="n">
-        <v>1533</v>
+        <v>8888</v>
       </c>
       <c r="D136" t="n">
-        <v>1309.01</v>
+        <v>2774.84</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3029,13 +3029,13 @@
         <v>46218</v>
       </c>
       <c r="B137" t="n">
-        <v>1007</v>
+        <v>1756</v>
       </c>
       <c r="C137" t="n">
         <v>8888</v>
       </c>
       <c r="D137" t="n">
-        <v>241.44</v>
+        <v>2275.21</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3048,17 +3048,17 @@
         <v>46218</v>
       </c>
       <c r="B138" t="n">
-        <v>1380</v>
+        <v>477</v>
       </c>
       <c r="C138" t="n">
         <v>8888</v>
       </c>
       <c r="D138" t="n">
-        <v>520.2</v>
+        <v>707.52</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3067,17 +3067,17 @@
         <v>46218</v>
       </c>
       <c r="B139" t="n">
-        <v>1102</v>
+        <v>2660</v>
       </c>
       <c r="C139" t="n">
         <v>8888</v>
       </c>
       <c r="D139" t="n">
-        <v>1137.04</v>
+        <v>2684.97</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3086,17 +3086,17 @@
         <v>46218</v>
       </c>
       <c r="B140" t="n">
-        <v>1075</v>
+        <v>569</v>
       </c>
       <c r="C140" t="n">
         <v>8888</v>
       </c>
       <c r="D140" t="n">
-        <v>4194.79</v>
+        <v>36782.12</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3105,17 +3105,17 @@
         <v>46218</v>
       </c>
       <c r="B141" t="n">
-        <v>2681</v>
+        <v>483</v>
       </c>
       <c r="C141" t="n">
         <v>8888</v>
       </c>
       <c r="D141" t="n">
-        <v>729.25</v>
+        <v>3102.48</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3124,17 +3124,17 @@
         <v>46218</v>
       </c>
       <c r="B142" t="n">
-        <v>2245</v>
+        <v>609</v>
       </c>
       <c r="C142" t="n">
         <v>8888</v>
       </c>
       <c r="D142" t="n">
-        <v>361.58</v>
+        <v>1633.68</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3143,17 +3143,17 @@
         <v>46218</v>
       </c>
       <c r="B143" t="n">
-        <v>33</v>
+        <v>483</v>
       </c>
       <c r="C143" t="n">
         <v>8888</v>
       </c>
       <c r="D143" t="n">
-        <v>926.97</v>
+        <v>1578.32</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3162,17 +3162,17 @@
         <v>46218</v>
       </c>
       <c r="B144" t="n">
-        <v>132</v>
+        <v>2089</v>
       </c>
       <c r="C144" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D144" t="n">
-        <v>6522.92</v>
+        <v>1309.01</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3181,17 +3181,17 @@
         <v>46218</v>
       </c>
       <c r="B145" t="n">
-        <v>619</v>
+        <v>1007</v>
       </c>
       <c r="C145" t="n">
         <v>8888</v>
       </c>
       <c r="D145" t="n">
-        <v>2912.89</v>
+        <v>241.44</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3200,13 +3200,13 @@
         <v>46218</v>
       </c>
       <c r="B146" t="n">
-        <v>452</v>
+        <v>1380</v>
       </c>
       <c r="C146" t="n">
         <v>8888</v>
       </c>
       <c r="D146" t="n">
-        <v>608.78</v>
+        <v>520.2</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3219,17 +3219,17 @@
         <v>46218</v>
       </c>
       <c r="B147" t="n">
-        <v>2463</v>
+        <v>1102</v>
       </c>
       <c r="C147" t="n">
         <v>8888</v>
       </c>
       <c r="D147" t="n">
-        <v>363.69</v>
+        <v>1137.04</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3238,17 +3238,17 @@
         <v>46218</v>
       </c>
       <c r="B148" t="n">
-        <v>1293</v>
+        <v>1075</v>
       </c>
       <c r="C148" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D148" t="n">
-        <v>1780.93</v>
+        <v>5710.94</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3257,17 +3257,17 @@
         <v>46218</v>
       </c>
       <c r="B149" t="n">
-        <v>525</v>
+        <v>2681</v>
       </c>
       <c r="C149" t="n">
         <v>8888</v>
       </c>
       <c r="D149" t="n">
-        <v>5658.57</v>
+        <v>729.25</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3276,13 +3276,13 @@
         <v>46218</v>
       </c>
       <c r="B150" t="n">
-        <v>2641</v>
+        <v>2245</v>
       </c>
       <c r="C150" t="n">
         <v>8888</v>
       </c>
       <c r="D150" t="n">
-        <v>1720.99</v>
+        <v>700.2</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -3295,17 +3295,17 @@
         <v>46218</v>
       </c>
       <c r="B151" t="n">
-        <v>609</v>
+        <v>33</v>
       </c>
       <c r="C151" t="n">
         <v>8888</v>
       </c>
       <c r="D151" t="n">
-        <v>886.1</v>
+        <v>926.97</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3314,13 +3314,13 @@
         <v>46218</v>
       </c>
       <c r="B152" t="n">
-        <v>2697</v>
+        <v>132</v>
       </c>
       <c r="C152" t="n">
         <v>8888</v>
       </c>
       <c r="D152" t="n">
-        <v>418.65</v>
+        <v>6522.92</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -3333,17 +3333,17 @@
         <v>46218</v>
       </c>
       <c r="B153" t="n">
-        <v>58</v>
+        <v>619</v>
       </c>
       <c r="C153" t="n">
         <v>8888</v>
       </c>
       <c r="D153" t="n">
-        <v>1123.87</v>
+        <v>2912.89</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3352,17 +3352,17 @@
         <v>46218</v>
       </c>
       <c r="B154" t="n">
-        <v>358</v>
+        <v>452</v>
       </c>
       <c r="C154" t="n">
         <v>8888</v>
       </c>
       <c r="D154" t="n">
-        <v>1675.95</v>
+        <v>608.78</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3371,17 +3371,17 @@
         <v>46218</v>
       </c>
       <c r="B155" t="n">
-        <v>2431</v>
+        <v>2463</v>
       </c>
       <c r="C155" t="n">
         <v>8888</v>
       </c>
       <c r="D155" t="n">
-        <v>266.89</v>
+        <v>363.69</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3390,17 +3390,17 @@
         <v>46218</v>
       </c>
       <c r="B156" t="n">
-        <v>285</v>
+        <v>1293</v>
       </c>
       <c r="C156" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D156" t="n">
-        <v>5673.85</v>
+        <v>1780.93</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3409,13 +3409,13 @@
         <v>46218</v>
       </c>
       <c r="B157" t="n">
-        <v>1102</v>
+        <v>525</v>
       </c>
       <c r="C157" t="n">
         <v>8888</v>
       </c>
       <c r="D157" t="n">
-        <v>1119.32</v>
+        <v>5658.57</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -3428,17 +3428,17 @@
         <v>46218</v>
       </c>
       <c r="B158" t="n">
-        <v>626</v>
+        <v>2641</v>
       </c>
       <c r="C158" t="n">
         <v>8888</v>
       </c>
       <c r="D158" t="n">
-        <v>12556.19</v>
+        <v>1720.99</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3447,17 +3447,17 @@
         <v>46218</v>
       </c>
       <c r="B159" t="n">
-        <v>1137</v>
+        <v>2697</v>
       </c>
       <c r="C159" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D159" t="n">
-        <v>1370.86</v>
+        <v>418.65</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3466,13 +3466,13 @@
         <v>46218</v>
       </c>
       <c r="B160" t="n">
-        <v>2686</v>
+        <v>2472</v>
       </c>
       <c r="C160" t="n">
-        <v>1929</v>
+        <v>2853</v>
       </c>
       <c r="D160" t="n">
-        <v>2066.36</v>
+        <v>1402.64</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -3485,17 +3485,17 @@
         <v>46218</v>
       </c>
       <c r="B161" t="n">
-        <v>2584</v>
+        <v>58</v>
       </c>
       <c r="C161" t="n">
         <v>8888</v>
       </c>
       <c r="D161" t="n">
-        <v>5635.67</v>
+        <v>1123.87</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3504,17 +3504,17 @@
         <v>46218</v>
       </c>
       <c r="B162" t="n">
-        <v>1756</v>
+        <v>358</v>
       </c>
       <c r="C162" t="n">
         <v>8888</v>
       </c>
       <c r="D162" t="n">
-        <v>2201.67</v>
+        <v>1675.95</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3523,17 +3523,17 @@
         <v>46218</v>
       </c>
       <c r="B163" t="n">
-        <v>1756</v>
+        <v>2431</v>
       </c>
       <c r="C163" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D163" t="n">
-        <v>5078.1</v>
+        <v>266.89</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3542,17 +3542,17 @@
         <v>46218</v>
       </c>
       <c r="B164" t="n">
-        <v>2651</v>
+        <v>285</v>
       </c>
       <c r="C164" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D164" t="n">
-        <v>363.7</v>
+        <v>5673.85</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3561,13 +3561,13 @@
         <v>46218</v>
       </c>
       <c r="B165" t="n">
-        <v>664</v>
+        <v>1102</v>
       </c>
       <c r="C165" t="n">
         <v>8888</v>
       </c>
       <c r="D165" t="n">
-        <v>5672.57</v>
+        <v>1119.32</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -3580,13 +3580,13 @@
         <v>46218</v>
       </c>
       <c r="B166" t="n">
-        <v>360</v>
+        <v>2793</v>
       </c>
       <c r="C166" t="n">
         <v>8888</v>
       </c>
       <c r="D166" t="n">
-        <v>1594.84</v>
+        <v>1238.11</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -3599,13 +3599,13 @@
         <v>46218</v>
       </c>
       <c r="B167" t="n">
-        <v>2582</v>
+        <v>626</v>
       </c>
       <c r="C167" t="n">
         <v>8888</v>
       </c>
       <c r="D167" t="n">
-        <v>379.33</v>
+        <v>12556.19</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -3618,17 +3618,17 @@
         <v>46218</v>
       </c>
       <c r="B168" t="n">
-        <v>636</v>
+        <v>1137</v>
       </c>
       <c r="C168" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D168" t="n">
-        <v>2447.56</v>
+        <v>1370.86</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3637,13 +3637,13 @@
         <v>46218</v>
       </c>
       <c r="B169" t="n">
-        <v>1254</v>
+        <v>1289</v>
       </c>
       <c r="C169" t="n">
         <v>8888</v>
       </c>
       <c r="D169" t="n">
-        <v>2643.22</v>
+        <v>5565.44</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -3656,17 +3656,17 @@
         <v>46218</v>
       </c>
       <c r="B170" t="n">
-        <v>1289</v>
+        <v>2686</v>
       </c>
       <c r="C170" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D170" t="n">
-        <v>2396.98</v>
+        <v>2066.36</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3675,17 +3675,17 @@
         <v>46218</v>
       </c>
       <c r="B171" t="n">
-        <v>2726</v>
+        <v>629</v>
       </c>
       <c r="C171" t="n">
-        <v>977</v>
+        <v>8888</v>
       </c>
       <c r="D171" t="n">
-        <v>586.0599999999999</v>
+        <v>5212.76</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3694,13 +3694,13 @@
         <v>46218</v>
       </c>
       <c r="B172" t="n">
-        <v>2015</v>
+        <v>2584</v>
       </c>
       <c r="C172" t="n">
         <v>8888</v>
       </c>
       <c r="D172" t="n">
-        <v>315.69</v>
+        <v>5635.67</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -3713,17 +3713,17 @@
         <v>46218</v>
       </c>
       <c r="B173" t="n">
-        <v>1064</v>
+        <v>1756</v>
       </c>
       <c r="C173" t="n">
         <v>8888</v>
       </c>
       <c r="D173" t="n">
-        <v>1274.3</v>
+        <v>2201.67</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3732,17 +3732,17 @@
         <v>46218</v>
       </c>
       <c r="B174" t="n">
-        <v>2698</v>
+        <v>1756</v>
       </c>
       <c r="C174" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D174" t="n">
-        <v>552.15</v>
+        <v>5078.1</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3751,17 +3751,17 @@
         <v>46218</v>
       </c>
       <c r="B175" t="n">
-        <v>629</v>
+        <v>2651</v>
       </c>
       <c r="C175" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D175" t="n">
-        <v>3544.51</v>
+        <v>363.7</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3770,17 +3770,17 @@
         <v>46218</v>
       </c>
       <c r="B176" t="n">
-        <v>2641</v>
+        <v>664</v>
       </c>
       <c r="C176" t="n">
         <v>8888</v>
       </c>
       <c r="D176" t="n">
-        <v>820</v>
+        <v>5672.57</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3789,17 +3789,17 @@
         <v>46218</v>
       </c>
       <c r="B177" t="n">
-        <v>429</v>
+        <v>360</v>
       </c>
       <c r="C177" t="n">
         <v>8888</v>
       </c>
       <c r="D177" t="n">
-        <v>2593.49</v>
+        <v>1594.84</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3808,17 +3808,17 @@
         <v>46218</v>
       </c>
       <c r="B178" t="n">
-        <v>816</v>
+        <v>2582</v>
       </c>
       <c r="C178" t="n">
         <v>8888</v>
       </c>
       <c r="D178" t="n">
-        <v>438.24</v>
+        <v>379.33</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3827,17 +3827,17 @@
         <v>46218</v>
       </c>
       <c r="B179" t="n">
-        <v>2793</v>
+        <v>636</v>
       </c>
       <c r="C179" t="n">
         <v>8888</v>
       </c>
       <c r="D179" t="n">
-        <v>767.58</v>
+        <v>2447.56</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3846,13 +3846,13 @@
         <v>46218</v>
       </c>
       <c r="B180" t="n">
-        <v>2359</v>
+        <v>1254</v>
       </c>
       <c r="C180" t="n">
         <v>8888</v>
       </c>
       <c r="D180" t="n">
-        <v>381.95</v>
+        <v>2643.22</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -3865,13 +3865,13 @@
         <v>46218</v>
       </c>
       <c r="B181" t="n">
-        <v>285</v>
+        <v>2726</v>
       </c>
       <c r="C181" t="n">
-        <v>58</v>
+        <v>977</v>
       </c>
       <c r="D181" t="n">
-        <v>364.99</v>
+        <v>586.0599999999999</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -3884,17 +3884,17 @@
         <v>46218</v>
       </c>
       <c r="B182" t="n">
-        <v>2114</v>
+        <v>2015</v>
       </c>
       <c r="C182" t="n">
         <v>8888</v>
       </c>
       <c r="D182" t="n">
-        <v>2726.04</v>
+        <v>315.69</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3903,17 +3903,17 @@
         <v>46218</v>
       </c>
       <c r="B183" t="n">
-        <v>953</v>
+        <v>1064</v>
       </c>
       <c r="C183" t="n">
         <v>8888</v>
       </c>
       <c r="D183" t="n">
-        <v>2889.63</v>
+        <v>1274.3</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3922,17 +3922,17 @@
         <v>46218</v>
       </c>
       <c r="B184" t="n">
-        <v>1102</v>
+        <v>2698</v>
       </c>
       <c r="C184" t="n">
         <v>8888</v>
       </c>
       <c r="D184" t="n">
-        <v>3093.73</v>
+        <v>552.15</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3941,13 +3941,13 @@
         <v>46218</v>
       </c>
       <c r="B185" t="n">
-        <v>1465</v>
+        <v>2641</v>
       </c>
       <c r="C185" t="n">
         <v>8888</v>
       </c>
       <c r="D185" t="n">
-        <v>4281.39</v>
+        <v>820</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -3960,17 +3960,17 @@
         <v>46218</v>
       </c>
       <c r="B186" t="n">
-        <v>619</v>
+        <v>429</v>
       </c>
       <c r="C186" t="n">
         <v>8888</v>
       </c>
       <c r="D186" t="n">
-        <v>2021.67</v>
+        <v>2593.49</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3979,17 +3979,17 @@
         <v>46218</v>
       </c>
       <c r="B187" t="n">
-        <v>2716</v>
+        <v>1301</v>
       </c>
       <c r="C187" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D187" t="n">
-        <v>601.58</v>
+        <v>750.66</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3998,17 +3998,17 @@
         <v>46218</v>
       </c>
       <c r="B188" t="n">
-        <v>2767</v>
+        <v>816</v>
       </c>
       <c r="C188" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D188" t="n">
-        <v>1135.64</v>
+        <v>438.24</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4017,13 +4017,13 @@
         <v>46218</v>
       </c>
       <c r="B189" t="n">
-        <v>2245</v>
+        <v>2359</v>
       </c>
       <c r="C189" t="n">
         <v>8888</v>
       </c>
       <c r="D189" t="n">
-        <v>427.51</v>
+        <v>381.95</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -4036,17 +4036,17 @@
         <v>46218</v>
       </c>
       <c r="B190" t="n">
-        <v>2197</v>
+        <v>2251</v>
       </c>
       <c r="C190" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D190" t="n">
-        <v>1085.45</v>
+        <v>802.08</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4055,17 +4055,17 @@
         <v>46218</v>
       </c>
       <c r="B191" t="n">
-        <v>2657</v>
+        <v>285</v>
       </c>
       <c r="C191" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D191" t="n">
-        <v>2683.06</v>
+        <v>364.99</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4074,17 +4074,17 @@
         <v>46218</v>
       </c>
       <c r="B192" t="n">
-        <v>451</v>
+        <v>2114</v>
       </c>
       <c r="C192" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D192" t="n">
-        <v>2091.77</v>
+        <v>2726.04</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4093,17 +4093,17 @@
         <v>46218</v>
       </c>
       <c r="B193" t="n">
-        <v>1116</v>
+        <v>953</v>
       </c>
       <c r="C193" t="n">
-        <v>13148</v>
+        <v>8888</v>
       </c>
       <c r="D193" t="n">
-        <v>207.91</v>
+        <v>2889.63</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4112,17 +4112,17 @@
         <v>46218</v>
       </c>
       <c r="B194" t="n">
-        <v>1277</v>
+        <v>1102</v>
       </c>
       <c r="C194" t="n">
         <v>8888</v>
       </c>
       <c r="D194" t="n">
-        <v>1949</v>
+        <v>4637.07</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4131,17 +4131,17 @@
         <v>46218</v>
       </c>
       <c r="B195" t="n">
-        <v>131</v>
+        <v>1465</v>
       </c>
       <c r="C195" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D195" t="n">
-        <v>3850.09</v>
+        <v>4281.39</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4150,13 +4150,13 @@
         <v>46218</v>
       </c>
       <c r="B196" t="n">
-        <v>2692</v>
+        <v>619</v>
       </c>
       <c r="C196" t="n">
         <v>8888</v>
       </c>
       <c r="D196" t="n">
-        <v>731.28</v>
+        <v>2021.67</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -4169,17 +4169,17 @@
         <v>46218</v>
       </c>
       <c r="B197" t="n">
-        <v>1632</v>
+        <v>2716</v>
       </c>
       <c r="C197" t="n">
         <v>8888</v>
       </c>
       <c r="D197" t="n">
-        <v>7519.7</v>
+        <v>1063.42</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4188,13 +4188,13 @@
         <v>46218</v>
       </c>
       <c r="B198" t="n">
-        <v>1317</v>
+        <v>2767</v>
       </c>
       <c r="C198" t="n">
-        <v>3179</v>
+        <v>1898</v>
       </c>
       <c r="D198" t="n">
-        <v>991.6799999999999</v>
+        <v>1135.64</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -4207,13 +4207,13 @@
         <v>46218</v>
       </c>
       <c r="B199" t="n">
-        <v>1993</v>
+        <v>2245</v>
       </c>
       <c r="C199" t="n">
         <v>8888</v>
       </c>
       <c r="D199" t="n">
-        <v>2875.39</v>
+        <v>764.66</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -4226,17 +4226,17 @@
         <v>46218</v>
       </c>
       <c r="B200" t="n">
-        <v>1890</v>
+        <v>2197</v>
       </c>
       <c r="C200" t="n">
-        <v>3449</v>
+        <v>8888</v>
       </c>
       <c r="D200" t="n">
-        <v>6313.56</v>
+        <v>1085.45</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4245,17 +4245,17 @@
         <v>46218</v>
       </c>
       <c r="B201" t="n">
-        <v>2749</v>
+        <v>1064</v>
       </c>
       <c r="C201" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D201" t="n">
-        <v>1860.64</v>
+        <v>574.7</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4264,17 +4264,17 @@
         <v>46218</v>
       </c>
       <c r="B202" t="n">
-        <v>1117</v>
+        <v>2657</v>
       </c>
       <c r="C202" t="n">
         <v>8888</v>
       </c>
       <c r="D202" t="n">
-        <v>342.2</v>
+        <v>2683.06</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4283,17 +4283,17 @@
         <v>46218</v>
       </c>
       <c r="B203" t="n">
-        <v>42</v>
+        <v>451</v>
       </c>
       <c r="C203" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D203" t="n">
-        <v>280.05</v>
+        <v>2091.77</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4302,17 +4302,17 @@
         <v>46218</v>
       </c>
       <c r="B204" t="n">
-        <v>1478</v>
+        <v>1116</v>
       </c>
       <c r="C204" t="n">
-        <v>8888</v>
+        <v>13148</v>
       </c>
       <c r="D204" t="n">
-        <v>875.34</v>
+        <v>207.91</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4321,13 +4321,13 @@
         <v>46218</v>
       </c>
       <c r="B205" t="n">
-        <v>2491</v>
+        <v>1277</v>
       </c>
       <c r="C205" t="n">
         <v>8888</v>
       </c>
       <c r="D205" t="n">
-        <v>650.4299999999999</v>
+        <v>1949</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -4340,17 +4340,17 @@
         <v>46218</v>
       </c>
       <c r="B206" t="n">
-        <v>2015</v>
+        <v>131</v>
       </c>
       <c r="C206" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D206" t="n">
-        <v>4436.15</v>
+        <v>3850.09</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4359,17 +4359,17 @@
         <v>46218</v>
       </c>
       <c r="B207" t="n">
-        <v>1890</v>
+        <v>2692</v>
       </c>
       <c r="C207" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D207" t="n">
-        <v>1674.57</v>
+        <v>731.28</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4378,17 +4378,17 @@
         <v>46218</v>
       </c>
       <c r="B208" t="n">
-        <v>1317</v>
+        <v>1632</v>
       </c>
       <c r="C208" t="n">
         <v>8888</v>
       </c>
       <c r="D208" t="n">
-        <v>1626.02</v>
+        <v>7519.7</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4397,17 +4397,17 @@
         <v>46218</v>
       </c>
       <c r="B209" t="n">
-        <v>2782</v>
+        <v>1317</v>
       </c>
       <c r="C209" t="n">
-        <v>8888</v>
+        <v>3179</v>
       </c>
       <c r="D209" t="n">
-        <v>1786.32</v>
+        <v>991.6799999999999</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4416,13 +4416,13 @@
         <v>46218</v>
       </c>
       <c r="B210" t="n">
-        <v>953</v>
+        <v>1993</v>
       </c>
       <c r="C210" t="n">
         <v>8888</v>
       </c>
       <c r="D210" t="n">
-        <v>364.44</v>
+        <v>2875.39</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -4435,17 +4435,17 @@
         <v>46218</v>
       </c>
       <c r="B211" t="n">
-        <v>2251</v>
+        <v>1890</v>
       </c>
       <c r="C211" t="n">
-        <v>8888</v>
+        <v>3449</v>
       </c>
       <c r="D211" t="n">
-        <v>309.22</v>
+        <v>6313.56</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4454,17 +4454,17 @@
         <v>46218</v>
       </c>
       <c r="B212" t="n">
-        <v>483</v>
+        <v>1800</v>
       </c>
       <c r="C212" t="n">
-        <v>841</v>
+        <v>8888</v>
       </c>
       <c r="D212" t="n">
-        <v>2085.09</v>
+        <v>430.37</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4473,17 +4473,17 @@
         <v>46218</v>
       </c>
       <c r="B213" t="n">
-        <v>2133</v>
+        <v>1117</v>
       </c>
       <c r="C213" t="n">
-        <v>213</v>
+        <v>8888</v>
       </c>
       <c r="D213" t="n">
-        <v>526.8</v>
+        <v>672.47</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4492,17 +4492,17 @@
         <v>46218</v>
       </c>
       <c r="B214" t="n">
-        <v>351</v>
+        <v>2749</v>
       </c>
       <c r="C214" t="n">
-        <v>3009</v>
+        <v>8888</v>
       </c>
       <c r="D214" t="n">
-        <v>416.36</v>
+        <v>1860.64</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4511,17 +4511,17 @@
         <v>46218</v>
       </c>
       <c r="B215" t="n">
-        <v>2250</v>
+        <v>42</v>
       </c>
       <c r="C215" t="n">
         <v>8888</v>
       </c>
       <c r="D215" t="n">
-        <v>709.46</v>
+        <v>280.05</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4530,17 +4530,17 @@
         <v>46218</v>
       </c>
       <c r="B216" t="n">
-        <v>2648</v>
+        <v>1478</v>
       </c>
       <c r="C216" t="n">
         <v>8888</v>
       </c>
       <c r="D216" t="n">
-        <v>1873.52</v>
+        <v>875.34</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4549,17 +4549,17 @@
         <v>46218</v>
       </c>
       <c r="B217" t="n">
-        <v>131</v>
+        <v>2491</v>
       </c>
       <c r="C217" t="n">
         <v>8888</v>
       </c>
       <c r="D217" t="n">
-        <v>1369.91</v>
+        <v>650.4299999999999</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4568,17 +4568,17 @@
         <v>46218</v>
       </c>
       <c r="B218" t="n">
-        <v>2790</v>
+        <v>353</v>
       </c>
       <c r="C218" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D218" t="n">
-        <v>371.88</v>
+        <v>653.13</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4587,17 +4587,17 @@
         <v>46218</v>
       </c>
       <c r="B219" t="n">
-        <v>363</v>
+        <v>2015</v>
       </c>
       <c r="C219" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D219" t="n">
-        <v>635.1</v>
+        <v>4436.15</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4606,17 +4606,17 @@
         <v>46218</v>
       </c>
       <c r="B220" t="n">
-        <v>2716</v>
+        <v>559</v>
       </c>
       <c r="C220" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D220" t="n">
-        <v>1073.33</v>
+        <v>1453.53</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4625,13 +4625,13 @@
         <v>46218</v>
       </c>
       <c r="B221" t="n">
-        <v>2298</v>
+        <v>1890</v>
       </c>
       <c r="C221" t="n">
-        <v>675</v>
+        <v>1953</v>
       </c>
       <c r="D221" t="n">
-        <v>401.85</v>
+        <v>1674.57</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -4644,17 +4644,17 @@
         <v>46218</v>
       </c>
       <c r="B222" t="n">
-        <v>2639</v>
+        <v>1317</v>
       </c>
       <c r="C222" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D222" t="n">
-        <v>504.09</v>
+        <v>1626.02</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4663,13 +4663,13 @@
         <v>46218</v>
       </c>
       <c r="B223" t="n">
-        <v>2109</v>
+        <v>2782</v>
       </c>
       <c r="C223" t="n">
         <v>8888</v>
       </c>
       <c r="D223" t="n">
-        <v>2293.78</v>
+        <v>1786.32</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -4682,17 +4682,17 @@
         <v>46218</v>
       </c>
       <c r="B224" t="n">
-        <v>1116</v>
+        <v>953</v>
       </c>
       <c r="C224" t="n">
         <v>8888</v>
       </c>
       <c r="D224" t="n">
-        <v>2919.53</v>
+        <v>364.44</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4701,17 +4701,17 @@
         <v>46218</v>
       </c>
       <c r="B225" t="n">
-        <v>2250</v>
+        <v>2251</v>
       </c>
       <c r="C225" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D225" t="n">
-        <v>1803.76</v>
+        <v>989.26</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4720,17 +4720,17 @@
         <v>46218</v>
       </c>
       <c r="B226" t="n">
-        <v>353</v>
+        <v>483</v>
       </c>
       <c r="C226" t="n">
-        <v>8888</v>
+        <v>841</v>
       </c>
       <c r="D226" t="n">
-        <v>349.33</v>
+        <v>2085.09</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4739,13 +4739,13 @@
         <v>46218</v>
       </c>
       <c r="B227" t="n">
-        <v>2698</v>
+        <v>2133</v>
       </c>
       <c r="C227" t="n">
-        <v>874</v>
+        <v>213</v>
       </c>
       <c r="D227" t="n">
-        <v>1230.43</v>
+        <v>526.8</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -4758,17 +4758,17 @@
         <v>46218</v>
       </c>
       <c r="B228" t="n">
-        <v>42</v>
+        <v>351</v>
       </c>
       <c r="C228" t="n">
-        <v>8888</v>
+        <v>3009</v>
       </c>
       <c r="D228" t="n">
-        <v>79947.14999999999</v>
+        <v>416.36</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4777,17 +4777,17 @@
         <v>46218</v>
       </c>
       <c r="B229" t="n">
-        <v>772</v>
+        <v>2250</v>
       </c>
       <c r="C229" t="n">
         <v>8888</v>
       </c>
       <c r="D229" t="n">
-        <v>400.25</v>
+        <v>709.46</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4796,17 +4796,17 @@
         <v>46218</v>
       </c>
       <c r="B230" t="n">
-        <v>2728</v>
+        <v>2648</v>
       </c>
       <c r="C230" t="n">
         <v>8888</v>
       </c>
       <c r="D230" t="n">
-        <v>1397.07</v>
+        <v>1873.52</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4815,17 +4815,17 @@
         <v>46218</v>
       </c>
       <c r="B231" t="n">
-        <v>2197</v>
+        <v>131</v>
       </c>
       <c r="C231" t="n">
-        <v>423</v>
+        <v>8888</v>
       </c>
       <c r="D231" t="n">
-        <v>2267.61</v>
+        <v>1369.91</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4834,13 +4834,13 @@
         <v>46218</v>
       </c>
       <c r="B232" t="n">
-        <v>2716</v>
+        <v>2790</v>
       </c>
       <c r="C232" t="n">
-        <v>977</v>
+        <v>1953</v>
       </c>
       <c r="D232" t="n">
-        <v>729.29</v>
+        <v>371.88</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -4853,17 +4853,17 @@
         <v>46218</v>
       </c>
       <c r="B233" t="n">
-        <v>1993</v>
+        <v>363</v>
       </c>
       <c r="C233" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D233" t="n">
-        <v>456.62</v>
+        <v>635.1</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4872,15 +4872,281 @@
         <v>46218</v>
       </c>
       <c r="B234" t="n">
+        <v>2716</v>
+      </c>
+      <c r="C234" t="n">
+        <v>1929</v>
+      </c>
+      <c r="D234" t="n">
+        <v>1073.33</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B235" t="n">
+        <v>2298</v>
+      </c>
+      <c r="C235" t="n">
+        <v>675</v>
+      </c>
+      <c r="D235" t="n">
+        <v>401.85</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B236" t="n">
+        <v>2639</v>
+      </c>
+      <c r="C236" t="n">
+        <v>1953</v>
+      </c>
+      <c r="D236" t="n">
+        <v>504.09</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B237" t="n">
+        <v>619</v>
+      </c>
+      <c r="C237" t="n">
+        <v>1139</v>
+      </c>
+      <c r="D237" t="n">
+        <v>1341.64</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B238" t="n">
+        <v>2109</v>
+      </c>
+      <c r="C238" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D238" t="n">
+        <v>2293.78</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B239" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C239" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D239" t="n">
+        <v>2919.53</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B240" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C240" t="n">
+        <v>27</v>
+      </c>
+      <c r="D240" t="n">
+        <v>1803.76</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B241" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C241" t="n">
+        <v>874</v>
+      </c>
+      <c r="D241" t="n">
+        <v>1230.43</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B242" t="n">
+        <v>42</v>
+      </c>
+      <c r="C242" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D242" t="n">
+        <v>79947.14999999999</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B243" t="n">
+        <v>772</v>
+      </c>
+      <c r="C243" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D243" t="n">
+        <v>400.25</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B244" t="n">
+        <v>2728</v>
+      </c>
+      <c r="C244" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D244" t="n">
+        <v>1397.07</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B245" t="n">
+        <v>2197</v>
+      </c>
+      <c r="C245" t="n">
+        <v>423</v>
+      </c>
+      <c r="D245" t="n">
+        <v>2267.61</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B246" t="n">
+        <v>2716</v>
+      </c>
+      <c r="C246" t="n">
+        <v>977</v>
+      </c>
+      <c r="D246" t="n">
+        <v>729.29</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B247" t="n">
+        <v>1993</v>
+      </c>
+      <c r="C247" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D247" t="n">
+        <v>456.62</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B248" t="n">
         <v>629</v>
       </c>
-      <c r="C234" t="n">
+      <c r="C248" t="n">
         <v>675</v>
       </c>
-      <c r="D234" t="n">
+      <c r="D248" t="n">
         <v>1054.76</v>
       </c>
-      <c r="E234" t="inlineStr">
+      <c r="E248" t="inlineStr">
         <is>
           <t>TELEMARKETING</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 17:30:03
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E248"/>
+  <dimension ref="A1:E257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,7 +489,7 @@
         <v>8888</v>
       </c>
       <c r="D3" t="n">
-        <v>544.78</v>
+        <v>651.77</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -546,7 +546,7 @@
         <v>3403</v>
       </c>
       <c r="D6" t="n">
-        <v>1300.54</v>
+        <v>1559.04</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -996,17 +996,17 @@
         <v>46218</v>
       </c>
       <c r="B30" t="n">
-        <v>931</v>
+        <v>2695</v>
       </c>
       <c r="C30" t="n">
-        <v>423</v>
+        <v>8888</v>
       </c>
       <c r="D30" t="n">
-        <v>492.34</v>
+        <v>677.6799999999999</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1015,17 +1015,17 @@
         <v>46218</v>
       </c>
       <c r="B31" t="n">
-        <v>951</v>
+        <v>931</v>
       </c>
       <c r="C31" t="n">
-        <v>8888</v>
+        <v>423</v>
       </c>
       <c r="D31" t="n">
-        <v>2171.08</v>
+        <v>492.34</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1034,13 +1034,13 @@
         <v>46218</v>
       </c>
       <c r="B32" t="n">
-        <v>2641</v>
+        <v>1117</v>
       </c>
       <c r="C32" t="n">
         <v>8888</v>
       </c>
       <c r="D32" t="n">
-        <v>2527.79</v>
+        <v>540.15</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1053,17 +1053,17 @@
         <v>46218</v>
       </c>
       <c r="B33" t="n">
-        <v>2695</v>
+        <v>2641</v>
       </c>
       <c r="C33" t="n">
         <v>8888</v>
       </c>
       <c r="D33" t="n">
-        <v>411.42</v>
+        <v>2527.79</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1072,17 +1072,17 @@
         <v>46218</v>
       </c>
       <c r="B34" t="n">
-        <v>525</v>
+        <v>2251</v>
       </c>
       <c r="C34" t="n">
         <v>8888</v>
       </c>
       <c r="D34" t="n">
-        <v>408.25</v>
+        <v>1010.74</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1091,17 +1091,17 @@
         <v>46218</v>
       </c>
       <c r="B35" t="n">
-        <v>1808</v>
+        <v>951</v>
       </c>
       <c r="C35" t="n">
         <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>695.3200000000001</v>
+        <v>2171.08</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1110,13 +1110,13 @@
         <v>46218</v>
       </c>
       <c r="B36" t="n">
-        <v>609</v>
+        <v>525</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>1909.37</v>
+        <v>408.25</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1129,17 +1129,17 @@
         <v>46218</v>
       </c>
       <c r="B37" t="n">
-        <v>949</v>
+        <v>1808</v>
       </c>
       <c r="C37" t="n">
-        <v>1134</v>
+        <v>8888</v>
       </c>
       <c r="D37" t="n">
-        <v>30.46</v>
+        <v>695.3200000000001</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1148,17 +1148,17 @@
         <v>46218</v>
       </c>
       <c r="B38" t="n">
-        <v>42</v>
+        <v>609</v>
       </c>
       <c r="C38" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D38" t="n">
-        <v>358.97</v>
+        <v>1909.37</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1167,17 +1167,17 @@
         <v>46218</v>
       </c>
       <c r="B39" t="n">
-        <v>2499</v>
+        <v>949</v>
       </c>
       <c r="C39" t="n">
-        <v>8888</v>
+        <v>1134</v>
       </c>
       <c r="D39" t="n">
-        <v>1049.3</v>
+        <v>30.46</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1186,17 +1186,17 @@
         <v>46218</v>
       </c>
       <c r="B40" t="n">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="C40" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D40" t="n">
-        <v>1643.73</v>
+        <v>358.97</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
         <v>46218</v>
       </c>
       <c r="B41" t="n">
-        <v>2245</v>
+        <v>2499</v>
       </c>
       <c r="C41" t="n">
         <v>8888</v>
       </c>
       <c r="D41" t="n">
-        <v>2740.06</v>
+        <v>1049.3</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1224,17 +1224,17 @@
         <v>46218</v>
       </c>
       <c r="B42" t="n">
-        <v>325</v>
+        <v>58</v>
       </c>
       <c r="C42" t="n">
         <v>8888</v>
       </c>
       <c r="D42" t="n">
-        <v>952.75</v>
+        <v>2194.12</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1243,17 +1243,17 @@
         <v>46218</v>
       </c>
       <c r="B43" t="n">
-        <v>2383</v>
+        <v>2245</v>
       </c>
       <c r="C43" t="n">
         <v>8888</v>
       </c>
       <c r="D43" t="n">
-        <v>7926.02</v>
+        <v>3382.78</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1262,17 +1262,17 @@
         <v>46218</v>
       </c>
       <c r="B44" t="n">
-        <v>1117</v>
+        <v>325</v>
       </c>
       <c r="C44" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D44" t="n">
-        <v>916.72</v>
+        <v>1079.66</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1281,17 +1281,17 @@
         <v>46218</v>
       </c>
       <c r="B45" t="n">
-        <v>374</v>
+        <v>2383</v>
       </c>
       <c r="C45" t="n">
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>2810.86</v>
+        <v>7926.02</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1300,17 +1300,17 @@
         <v>46218</v>
       </c>
       <c r="B46" t="n">
-        <v>2279</v>
+        <v>1117</v>
       </c>
       <c r="C46" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D46" t="n">
-        <v>712.66</v>
+        <v>916.72</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1319,17 +1319,17 @@
         <v>46218</v>
       </c>
       <c r="B47" t="n">
-        <v>535</v>
+        <v>374</v>
       </c>
       <c r="C47" t="n">
         <v>8888</v>
       </c>
       <c r="D47" t="n">
-        <v>5836.12</v>
+        <v>2810.86</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1338,13 +1338,13 @@
         <v>46218</v>
       </c>
       <c r="B48" t="n">
-        <v>535</v>
+        <v>2279</v>
       </c>
       <c r="C48" t="n">
         <v>8888</v>
       </c>
       <c r="D48" t="n">
-        <v>1352.51</v>
+        <v>712.66</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1357,17 +1357,17 @@
         <v>46218</v>
       </c>
       <c r="B49" t="n">
-        <v>2678</v>
+        <v>535</v>
       </c>
       <c r="C49" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D49" t="n">
-        <v>364.96</v>
+        <v>5836.12</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1376,13 +1376,13 @@
         <v>46218</v>
       </c>
       <c r="B50" t="n">
-        <v>2345</v>
+        <v>535</v>
       </c>
       <c r="C50" t="n">
         <v>8888</v>
       </c>
       <c r="D50" t="n">
-        <v>863.16</v>
+        <v>1352.51</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1395,17 +1395,17 @@
         <v>46218</v>
       </c>
       <c r="B51" t="n">
-        <v>945</v>
+        <v>2678</v>
       </c>
       <c r="C51" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D51" t="n">
-        <v>27337.21</v>
+        <v>364.96</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>PEDIDO ELETRÔNICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
         <v>46218</v>
       </c>
       <c r="B52" t="n">
-        <v>2686</v>
+        <v>2345</v>
       </c>
       <c r="C52" t="n">
         <v>8888</v>
       </c>
       <c r="D52" t="n">
-        <v>684.2</v>
+        <v>863.16</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1433,17 +1433,17 @@
         <v>46218</v>
       </c>
       <c r="B53" t="n">
-        <v>438</v>
+        <v>945</v>
       </c>
       <c r="C53" t="n">
         <v>8888</v>
       </c>
       <c r="D53" t="n">
-        <v>220.06</v>
+        <v>27337.21</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>PEDIDO ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -1452,17 +1452,17 @@
         <v>46218</v>
       </c>
       <c r="B54" t="n">
-        <v>664</v>
+        <v>2686</v>
       </c>
       <c r="C54" t="n">
         <v>8888</v>
       </c>
       <c r="D54" t="n">
-        <v>6275.01</v>
+        <v>684.2</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1471,17 +1471,17 @@
         <v>46218</v>
       </c>
       <c r="B55" t="n">
-        <v>353</v>
+        <v>438</v>
       </c>
       <c r="C55" t="n">
-        <v>3179</v>
+        <v>8888</v>
       </c>
       <c r="D55" t="n">
-        <v>495.84</v>
+        <v>220.06</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1490,17 +1490,17 @@
         <v>46218</v>
       </c>
       <c r="B56" t="n">
-        <v>1293</v>
+        <v>1956</v>
       </c>
       <c r="C56" t="n">
         <v>8888</v>
       </c>
       <c r="D56" t="n">
-        <v>3129.07</v>
+        <v>5311.01</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1509,13 +1509,13 @@
         <v>46218</v>
       </c>
       <c r="B57" t="n">
-        <v>2279</v>
+        <v>664</v>
       </c>
       <c r="C57" t="n">
         <v>8888</v>
       </c>
       <c r="D57" t="n">
-        <v>2753.96</v>
+        <v>6275.01</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1528,17 +1528,17 @@
         <v>46218</v>
       </c>
       <c r="B58" t="n">
-        <v>1937</v>
+        <v>353</v>
       </c>
       <c r="C58" t="n">
-        <v>8888</v>
+        <v>3179</v>
       </c>
       <c r="D58" t="n">
-        <v>1685.72</v>
+        <v>495.84</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1547,17 +1547,17 @@
         <v>46218</v>
       </c>
       <c r="B59" t="n">
-        <v>941</v>
+        <v>1293</v>
       </c>
       <c r="C59" t="n">
         <v>8888</v>
       </c>
       <c r="D59" t="n">
-        <v>864.14</v>
+        <v>3129.07</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1566,17 +1566,17 @@
         <v>46218</v>
       </c>
       <c r="B60" t="n">
-        <v>1137</v>
+        <v>2279</v>
       </c>
       <c r="C60" t="n">
         <v>8888</v>
       </c>
       <c r="D60" t="n">
-        <v>1947.93</v>
+        <v>3900.07</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1585,17 +1585,17 @@
         <v>46218</v>
       </c>
       <c r="B61" t="n">
-        <v>2631</v>
+        <v>1937</v>
       </c>
       <c r="C61" t="n">
-        <v>2853</v>
+        <v>8888</v>
       </c>
       <c r="D61" t="n">
-        <v>1272.12</v>
+        <v>1685.72</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1604,17 +1604,17 @@
         <v>46218</v>
       </c>
       <c r="B62" t="n">
-        <v>2793</v>
+        <v>941</v>
       </c>
       <c r="C62" t="n">
-        <v>977</v>
+        <v>8888</v>
       </c>
       <c r="D62" t="n">
-        <v>1188.59</v>
+        <v>864.14</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1623,17 +1623,17 @@
         <v>46218</v>
       </c>
       <c r="B63" t="n">
-        <v>2802</v>
+        <v>1137</v>
       </c>
       <c r="C63" t="n">
         <v>8888</v>
       </c>
       <c r="D63" t="n">
-        <v>1264.57</v>
+        <v>1947.93</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1642,17 +1642,17 @@
         <v>46218</v>
       </c>
       <c r="B64" t="n">
-        <v>451</v>
+        <v>2631</v>
       </c>
       <c r="C64" t="n">
-        <v>8888</v>
+        <v>2853</v>
       </c>
       <c r="D64" t="n">
-        <v>757.5700000000001</v>
+        <v>2418.28</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1661,17 +1661,17 @@
         <v>46218</v>
       </c>
       <c r="B65" t="n">
-        <v>374</v>
+        <v>2793</v>
       </c>
       <c r="C65" t="n">
-        <v>8888</v>
+        <v>977</v>
       </c>
       <c r="D65" t="n">
-        <v>44.6</v>
+        <v>1188.59</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1680,13 +1680,13 @@
         <v>46218</v>
       </c>
       <c r="B66" t="n">
-        <v>703</v>
+        <v>2802</v>
       </c>
       <c r="C66" t="n">
         <v>8888</v>
       </c>
       <c r="D66" t="n">
-        <v>12155.46</v>
+        <v>1264.57</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1699,17 +1699,17 @@
         <v>46218</v>
       </c>
       <c r="B67" t="n">
-        <v>1756</v>
+        <v>451</v>
       </c>
       <c r="C67" t="n">
         <v>8888</v>
       </c>
       <c r="D67" t="n">
-        <v>4416.47</v>
+        <v>757.5700000000001</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1718,17 +1718,17 @@
         <v>46218</v>
       </c>
       <c r="B68" t="n">
-        <v>1956</v>
+        <v>374</v>
       </c>
       <c r="C68" t="n">
         <v>8888</v>
       </c>
       <c r="D68" t="n">
-        <v>4557.34</v>
+        <v>44.6</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1737,13 +1737,13 @@
         <v>46218</v>
       </c>
       <c r="B69" t="n">
-        <v>925</v>
+        <v>703</v>
       </c>
       <c r="C69" t="n">
         <v>8888</v>
       </c>
       <c r="D69" t="n">
-        <v>651.59</v>
+        <v>12155.46</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1756,17 +1756,17 @@
         <v>46218</v>
       </c>
       <c r="B70" t="n">
-        <v>941</v>
+        <v>1756</v>
       </c>
       <c r="C70" t="n">
-        <v>977</v>
+        <v>8888</v>
       </c>
       <c r="D70" t="n">
-        <v>359.73</v>
+        <v>4416.47</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1775,17 @@
         <v>46218</v>
       </c>
       <c r="B71" t="n">
-        <v>2648</v>
+        <v>925</v>
       </c>
       <c r="C71" t="n">
         <v>8888</v>
       </c>
       <c r="D71" t="n">
-        <v>1594.42</v>
+        <v>651.59</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1794,17 +1794,17 @@
         <v>46218</v>
       </c>
       <c r="B72" t="n">
-        <v>663</v>
+        <v>941</v>
       </c>
       <c r="C72" t="n">
-        <v>8888</v>
+        <v>977</v>
       </c>
       <c r="D72" t="n">
-        <v>6645.33</v>
+        <v>359.73</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1813,17 +1813,17 @@
         <v>46218</v>
       </c>
       <c r="B73" t="n">
-        <v>2714</v>
+        <v>2648</v>
       </c>
       <c r="C73" t="n">
-        <v>519</v>
+        <v>8888</v>
       </c>
       <c r="D73" t="n">
-        <v>61939.22</v>
+        <v>1594.42</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1832,17 +1832,17 @@
         <v>46218</v>
       </c>
       <c r="B74" t="n">
-        <v>483</v>
+        <v>663</v>
       </c>
       <c r="C74" t="n">
         <v>8888</v>
       </c>
       <c r="D74" t="n">
-        <v>11360.2</v>
+        <v>6645.33</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1851,17 +1851,17 @@
         <v>46218</v>
       </c>
       <c r="B75" t="n">
-        <v>1075</v>
+        <v>2714</v>
       </c>
       <c r="C75" t="n">
-        <v>8888</v>
+        <v>519</v>
       </c>
       <c r="D75" t="n">
-        <v>11607.79</v>
+        <v>61939.22</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1870,17 +1870,17 @@
         <v>46218</v>
       </c>
       <c r="B76" t="n">
-        <v>629</v>
+        <v>483</v>
       </c>
       <c r="C76" t="n">
         <v>8888</v>
       </c>
       <c r="D76" t="n">
-        <v>9233.719999999999</v>
+        <v>12405.46</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1889,17 +1889,17 @@
         <v>46218</v>
       </c>
       <c r="B77" t="n">
-        <v>1983</v>
+        <v>1075</v>
       </c>
       <c r="C77" t="n">
-        <v>841</v>
+        <v>8888</v>
       </c>
       <c r="D77" t="n">
-        <v>243.92</v>
+        <v>11607.79</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1908,17 +1908,17 @@
         <v>46218</v>
       </c>
       <c r="B78" t="n">
-        <v>1137</v>
+        <v>629</v>
       </c>
       <c r="C78" t="n">
         <v>8888</v>
       </c>
       <c r="D78" t="n">
-        <v>3578.51</v>
+        <v>9233.719999999999</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1927,17 +1927,17 @@
         <v>46218</v>
       </c>
       <c r="B79" t="n">
-        <v>2651</v>
+        <v>1983</v>
       </c>
       <c r="C79" t="n">
-        <v>8888</v>
+        <v>841</v>
       </c>
       <c r="D79" t="n">
-        <v>1296.58</v>
+        <v>633.79</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1946,13 +1946,13 @@
         <v>46218</v>
       </c>
       <c r="B80" t="n">
-        <v>2789</v>
+        <v>1137</v>
       </c>
       <c r="C80" t="n">
         <v>8888</v>
       </c>
       <c r="D80" t="n">
-        <v>1293.93</v>
+        <v>3578.51</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -1965,17 +1965,17 @@
         <v>46218</v>
       </c>
       <c r="B81" t="n">
-        <v>1956</v>
+        <v>2651</v>
       </c>
       <c r="C81" t="n">
-        <v>423</v>
+        <v>8888</v>
       </c>
       <c r="D81" t="n">
-        <v>1416.35</v>
+        <v>1296.58</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1984,13 +1984,13 @@
         <v>46218</v>
       </c>
       <c r="B82" t="n">
-        <v>2709</v>
+        <v>2789</v>
       </c>
       <c r="C82" t="n">
         <v>8888</v>
       </c>
       <c r="D82" t="n">
-        <v>547.6900000000001</v>
+        <v>1293.93</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2003,17 +2003,17 @@
         <v>46218</v>
       </c>
       <c r="B83" t="n">
-        <v>1308</v>
+        <v>1956</v>
       </c>
       <c r="C83" t="n">
-        <v>8888</v>
+        <v>423</v>
       </c>
       <c r="D83" t="n">
-        <v>1460.53</v>
+        <v>1416.35</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2022,17 +2022,17 @@
         <v>46218</v>
       </c>
       <c r="B84" t="n">
-        <v>2026</v>
+        <v>2709</v>
       </c>
       <c r="C84" t="n">
         <v>8888</v>
       </c>
       <c r="D84" t="n">
-        <v>2237.62</v>
+        <v>547.6900000000001</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2041,17 +2041,17 @@
         <v>46218</v>
       </c>
       <c r="B85" t="n">
-        <v>2789</v>
+        <v>1308</v>
       </c>
       <c r="C85" t="n">
         <v>8888</v>
       </c>
       <c r="D85" t="n">
-        <v>747.77</v>
+        <v>1460.53</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2060,17 +2060,17 @@
         <v>46218</v>
       </c>
       <c r="B86" t="n">
-        <v>89</v>
+        <v>2026</v>
       </c>
       <c r="C86" t="n">
-        <v>13148</v>
+        <v>8888</v>
       </c>
       <c r="D86" t="n">
-        <v>1883.74</v>
+        <v>2237.62</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2079,17 +2079,17 @@
         <v>46218</v>
       </c>
       <c r="B87" t="n">
-        <v>2709</v>
+        <v>2789</v>
       </c>
       <c r="C87" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D87" t="n">
-        <v>390.19</v>
+        <v>747.77</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2098,17 +2098,17 @@
         <v>46218</v>
       </c>
       <c r="B88" t="n">
-        <v>2345</v>
+        <v>89</v>
       </c>
       <c r="C88" t="n">
-        <v>8888</v>
+        <v>13148</v>
       </c>
       <c r="D88" t="n">
-        <v>748.86</v>
+        <v>2842.03</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2117,17 +2117,17 @@
         <v>46218</v>
       </c>
       <c r="B89" t="n">
-        <v>1983</v>
+        <v>1075</v>
       </c>
       <c r="C89" t="n">
         <v>8888</v>
       </c>
       <c r="D89" t="n">
-        <v>851.7</v>
+        <v>698.63</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2136,13 +2136,13 @@
         <v>46218</v>
       </c>
       <c r="B90" t="n">
-        <v>2765</v>
+        <v>2709</v>
       </c>
       <c r="C90" t="n">
-        <v>1883</v>
+        <v>2220</v>
       </c>
       <c r="D90" t="n">
-        <v>3638.6</v>
+        <v>390.19</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2155,17 +2155,17 @@
         <v>46218</v>
       </c>
       <c r="B91" t="n">
-        <v>569</v>
+        <v>2345</v>
       </c>
       <c r="C91" t="n">
         <v>8888</v>
       </c>
       <c r="D91" t="n">
-        <v>995.33</v>
+        <v>748.86</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2174,17 +2174,17 @@
         <v>46218</v>
       </c>
       <c r="B92" t="n">
-        <v>360</v>
+        <v>1983</v>
       </c>
       <c r="C92" t="n">
-        <v>546</v>
+        <v>8888</v>
       </c>
       <c r="D92" t="n">
-        <v>1609.68</v>
+        <v>2806.44</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2193,13 +2193,13 @@
         <v>46218</v>
       </c>
       <c r="B93" t="n">
-        <v>2711</v>
+        <v>2765</v>
       </c>
       <c r="C93" t="n">
-        <v>1953</v>
+        <v>1883</v>
       </c>
       <c r="D93" t="n">
-        <v>150.27</v>
+        <v>3638.6</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2212,13 +2212,13 @@
         <v>46218</v>
       </c>
       <c r="B94" t="n">
-        <v>2308</v>
+        <v>569</v>
       </c>
       <c r="C94" t="n">
         <v>8888</v>
       </c>
       <c r="D94" t="n">
-        <v>488.69</v>
+        <v>995.33</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2231,13 +2231,13 @@
         <v>46218</v>
       </c>
       <c r="B95" t="n">
-        <v>2211</v>
+        <v>360</v>
       </c>
       <c r="C95" t="n">
-        <v>874</v>
+        <v>546</v>
       </c>
       <c r="D95" t="n">
-        <v>1526.94</v>
+        <v>1609.68</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2250,17 +2250,17 @@
         <v>46218</v>
       </c>
       <c r="B96" t="n">
-        <v>559</v>
+        <v>2711</v>
       </c>
       <c r="C96" t="n">
-        <v>8888</v>
+        <v>1953</v>
       </c>
       <c r="D96" t="n">
-        <v>859.92</v>
+        <v>150.27</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2269,13 +2269,13 @@
         <v>46218</v>
       </c>
       <c r="B97" t="n">
-        <v>890</v>
+        <v>2279</v>
       </c>
       <c r="C97" t="n">
         <v>8888</v>
       </c>
       <c r="D97" t="n">
-        <v>387.2</v>
+        <v>447.5</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2288,17 +2288,17 @@
         <v>46218</v>
       </c>
       <c r="B98" t="n">
-        <v>2768</v>
+        <v>2308</v>
       </c>
       <c r="C98" t="n">
         <v>8888</v>
       </c>
       <c r="D98" t="n">
-        <v>6523.26</v>
+        <v>488.69</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2307,17 +2307,17 @@
         <v>46218</v>
       </c>
       <c r="B99" t="n">
-        <v>1063</v>
+        <v>2211</v>
       </c>
       <c r="C99" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D99" t="n">
-        <v>4487.11</v>
+        <v>1526.94</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2326,17 +2326,17 @@
         <v>46218</v>
       </c>
       <c r="B100" t="n">
-        <v>2279</v>
+        <v>559</v>
       </c>
       <c r="C100" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D100" t="n">
-        <v>652.51</v>
+        <v>859.92</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2345,17 +2345,17 @@
         <v>46218</v>
       </c>
       <c r="B101" t="n">
-        <v>1299</v>
+        <v>890</v>
       </c>
       <c r="C101" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D101" t="n">
-        <v>1435.52</v>
+        <v>387.2</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2364,17 +2364,17 @@
         <v>46218</v>
       </c>
       <c r="B102" t="n">
-        <v>1478</v>
+        <v>2768</v>
       </c>
       <c r="C102" t="n">
-        <v>675</v>
+        <v>8888</v>
       </c>
       <c r="D102" t="n">
-        <v>1967.85</v>
+        <v>6523.26</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2383,17 +2383,17 @@
         <v>46218</v>
       </c>
       <c r="B103" t="n">
-        <v>767</v>
+        <v>1063</v>
       </c>
       <c r="C103" t="n">
         <v>8888</v>
       </c>
       <c r="D103" t="n">
-        <v>3292.44</v>
+        <v>4487.11</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2402,17 +2402,17 @@
         <v>46218</v>
       </c>
       <c r="B104" t="n">
-        <v>285</v>
+        <v>947</v>
       </c>
       <c r="C104" t="n">
         <v>8888</v>
       </c>
       <c r="D104" t="n">
-        <v>3349.8</v>
+        <v>5667.85</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>PEDIDO ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -2421,17 +2421,17 @@
         <v>46218</v>
       </c>
       <c r="B105" t="n">
-        <v>477</v>
+        <v>2279</v>
       </c>
       <c r="C105" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D105" t="n">
-        <v>917.33</v>
+        <v>1031.06</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2440,17 +2440,17 @@
         <v>46218</v>
       </c>
       <c r="B106" t="n">
-        <v>1983</v>
+        <v>1299</v>
       </c>
       <c r="C106" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D106" t="n">
-        <v>5115.01</v>
+        <v>1435.52</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2459,13 +2459,13 @@
         <v>46218</v>
       </c>
       <c r="B107" t="n">
-        <v>477</v>
+        <v>1478</v>
       </c>
       <c r="C107" t="n">
-        <v>58</v>
+        <v>675</v>
       </c>
       <c r="D107" t="n">
-        <v>1540.55</v>
+        <v>1967.85</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -2478,13 +2478,13 @@
         <v>46218</v>
       </c>
       <c r="B108" t="n">
-        <v>1937</v>
+        <v>767</v>
       </c>
       <c r="C108" t="n">
         <v>8888</v>
       </c>
       <c r="D108" t="n">
-        <v>2600.61</v>
+        <v>3292.44</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -2497,13 +2497,13 @@
         <v>46218</v>
       </c>
       <c r="B109" t="n">
-        <v>1063</v>
+        <v>285</v>
       </c>
       <c r="C109" t="n">
         <v>8888</v>
       </c>
       <c r="D109" t="n">
-        <v>2549.86</v>
+        <v>3349.8</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -2516,17 +2516,17 @@
         <v>46218</v>
       </c>
       <c r="B110" t="n">
-        <v>2584</v>
+        <v>477</v>
       </c>
       <c r="C110" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D110" t="n">
-        <v>756.16</v>
+        <v>917.33</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2535,13 +2535,13 @@
         <v>46218</v>
       </c>
       <c r="B111" t="n">
-        <v>58</v>
+        <v>1983</v>
       </c>
       <c r="C111" t="n">
         <v>8888</v>
       </c>
       <c r="D111" t="n">
-        <v>558.03</v>
+        <v>5115.01</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -2554,17 +2554,17 @@
         <v>46218</v>
       </c>
       <c r="B112" t="n">
-        <v>424</v>
+        <v>477</v>
       </c>
       <c r="C112" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D112" t="n">
-        <v>1362.42</v>
+        <v>3946.44</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2573,17 +2573,17 @@
         <v>46218</v>
       </c>
       <c r="B113" t="n">
-        <v>675</v>
+        <v>1937</v>
       </c>
       <c r="C113" t="n">
         <v>8888</v>
       </c>
       <c r="D113" t="n">
-        <v>616.73</v>
+        <v>2600.61</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2592,13 +2592,13 @@
         <v>46218</v>
       </c>
       <c r="B114" t="n">
-        <v>663</v>
+        <v>1063</v>
       </c>
       <c r="C114" t="n">
         <v>8888</v>
       </c>
       <c r="D114" t="n">
-        <v>255.13</v>
+        <v>2549.86</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -2611,17 +2611,17 @@
         <v>46218</v>
       </c>
       <c r="B115" t="n">
-        <v>1993</v>
+        <v>2584</v>
       </c>
       <c r="C115" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D115" t="n">
-        <v>362.63</v>
+        <v>756.16</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2630,17 +2630,17 @@
         <v>46218</v>
       </c>
       <c r="B116" t="n">
-        <v>1465</v>
+        <v>58</v>
       </c>
       <c r="C116" t="n">
         <v>8888</v>
       </c>
       <c r="D116" t="n">
-        <v>3373.83</v>
+        <v>558.03</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2649,17 +2649,17 @@
         <v>46218</v>
       </c>
       <c r="B117" t="n">
-        <v>89</v>
+        <v>424</v>
       </c>
       <c r="C117" t="n">
         <v>8888</v>
       </c>
       <c r="D117" t="n">
-        <v>479</v>
+        <v>1362.42</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2668,13 +2668,13 @@
         <v>46218</v>
       </c>
       <c r="B118" t="n">
-        <v>595</v>
+        <v>675</v>
       </c>
       <c r="C118" t="n">
         <v>8888</v>
       </c>
       <c r="D118" t="n">
-        <v>18084.5</v>
+        <v>616.73</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -2687,17 +2687,17 @@
         <v>46218</v>
       </c>
       <c r="B119" t="n">
-        <v>2696</v>
+        <v>663</v>
       </c>
       <c r="C119" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D119" t="n">
-        <v>1597.76</v>
+        <v>255.13</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2706,17 +2706,17 @@
         <v>46218</v>
       </c>
       <c r="B120" t="n">
-        <v>360</v>
+        <v>1993</v>
       </c>
       <c r="C120" t="n">
         <v>8888</v>
       </c>
       <c r="D120" t="n">
-        <v>4596.89</v>
+        <v>724.14</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2728,14 +2728,14 @@
         <v>1465</v>
       </c>
       <c r="C121" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D121" t="n">
-        <v>777.2</v>
+        <v>7362.56</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2744,17 +2744,17 @@
         <v>46218</v>
       </c>
       <c r="B122" t="n">
-        <v>947</v>
+        <v>89</v>
       </c>
       <c r="C122" t="n">
         <v>8888</v>
       </c>
       <c r="D122" t="n">
-        <v>5115.36</v>
+        <v>479</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>PEDIDO ELETRÔNICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2763,17 +2763,17 @@
         <v>46218</v>
       </c>
       <c r="B123" t="n">
-        <v>2178</v>
+        <v>595</v>
       </c>
       <c r="C123" t="n">
         <v>8888</v>
       </c>
       <c r="D123" t="n">
-        <v>619.92</v>
+        <v>18084.5</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2782,13 +2782,13 @@
         <v>46218</v>
       </c>
       <c r="B124" t="n">
-        <v>2026</v>
+        <v>2696</v>
       </c>
       <c r="C124" t="n">
-        <v>1929</v>
+        <v>1954</v>
       </c>
       <c r="D124" t="n">
-        <v>5293.13</v>
+        <v>1597.76</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -2801,17 +2801,17 @@
         <v>46218</v>
       </c>
       <c r="B125" t="n">
-        <v>630</v>
+        <v>360</v>
       </c>
       <c r="C125" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D125" t="n">
-        <v>1801.63</v>
+        <v>4596.89</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2820,17 +2820,17 @@
         <v>46218</v>
       </c>
       <c r="B126" t="n">
-        <v>1937</v>
+        <v>1465</v>
       </c>
       <c r="C126" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D126" t="n">
-        <v>2132.95</v>
+        <v>777.2</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2839,17 +2839,17 @@
         <v>46218</v>
       </c>
       <c r="B127" t="n">
-        <v>2577</v>
+        <v>2178</v>
       </c>
       <c r="C127" t="n">
         <v>8888</v>
       </c>
       <c r="D127" t="n">
-        <v>1647.08</v>
+        <v>619.92</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2858,17 +2858,17 @@
         <v>46218</v>
       </c>
       <c r="B128" t="n">
-        <v>1293</v>
+        <v>2026</v>
       </c>
       <c r="C128" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D128" t="n">
-        <v>2135.89</v>
+        <v>6021.92</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2877,17 +2877,17 @@
         <v>46218</v>
       </c>
       <c r="B129" t="n">
-        <v>2607</v>
+        <v>630</v>
       </c>
       <c r="C129" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D129" t="n">
-        <v>490.31</v>
+        <v>1801.63</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2896,17 +2896,17 @@
         <v>46218</v>
       </c>
       <c r="B130" t="n">
-        <v>1317</v>
+        <v>1937</v>
       </c>
       <c r="C130" t="n">
         <v>8888</v>
       </c>
       <c r="D130" t="n">
-        <v>907.72</v>
+        <v>2132.95</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2915,13 +2915,13 @@
         <v>46218</v>
       </c>
       <c r="B131" t="n">
-        <v>619</v>
+        <v>2577</v>
       </c>
       <c r="C131" t="n">
         <v>8888</v>
       </c>
       <c r="D131" t="n">
-        <v>1081.74</v>
+        <v>1647.08</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -2934,17 +2934,17 @@
         <v>46218</v>
       </c>
       <c r="B132" t="n">
-        <v>2571</v>
+        <v>1293</v>
       </c>
       <c r="C132" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D132" t="n">
-        <v>268.53</v>
+        <v>2135.89</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2953,13 +2953,13 @@
         <v>46218</v>
       </c>
       <c r="B133" t="n">
-        <v>20</v>
+        <v>2607</v>
       </c>
       <c r="C133" t="n">
         <v>8888</v>
       </c>
       <c r="D133" t="n">
-        <v>745.55</v>
+        <v>490.31</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -2972,13 +2972,13 @@
         <v>46218</v>
       </c>
       <c r="B134" t="n">
-        <v>1063</v>
+        <v>1317</v>
       </c>
       <c r="C134" t="n">
         <v>8888</v>
       </c>
       <c r="D134" t="n">
-        <v>1113.08</v>
+        <v>907.72</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -2991,17 +2991,17 @@
         <v>46218</v>
       </c>
       <c r="B135" t="n">
-        <v>2631</v>
+        <v>619</v>
       </c>
       <c r="C135" t="n">
         <v>8888</v>
       </c>
       <c r="D135" t="n">
-        <v>1447.86</v>
+        <v>1081.74</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3010,17 +3010,17 @@
         <v>46218</v>
       </c>
       <c r="B136" t="n">
-        <v>1906</v>
+        <v>2571</v>
       </c>
       <c r="C136" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D136" t="n">
-        <v>2774.84</v>
+        <v>268.53</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3029,13 +3029,13 @@
         <v>46218</v>
       </c>
       <c r="B137" t="n">
-        <v>1756</v>
+        <v>20</v>
       </c>
       <c r="C137" t="n">
         <v>8888</v>
       </c>
       <c r="D137" t="n">
-        <v>2275.21</v>
+        <v>745.55</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3048,13 +3048,13 @@
         <v>46218</v>
       </c>
       <c r="B138" t="n">
-        <v>477</v>
+        <v>1063</v>
       </c>
       <c r="C138" t="n">
         <v>8888</v>
       </c>
       <c r="D138" t="n">
-        <v>707.52</v>
+        <v>1113.08</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3067,13 +3067,13 @@
         <v>46218</v>
       </c>
       <c r="B139" t="n">
-        <v>2660</v>
+        <v>2631</v>
       </c>
       <c r="C139" t="n">
         <v>8888</v>
       </c>
       <c r="D139" t="n">
-        <v>2684.97</v>
+        <v>1447.86</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3086,17 +3086,17 @@
         <v>46218</v>
       </c>
       <c r="B140" t="n">
-        <v>569</v>
+        <v>1906</v>
       </c>
       <c r="C140" t="n">
         <v>8888</v>
       </c>
       <c r="D140" t="n">
-        <v>36782.12</v>
+        <v>2774.84</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3105,17 +3105,17 @@
         <v>46218</v>
       </c>
       <c r="B141" t="n">
-        <v>483</v>
+        <v>1756</v>
       </c>
       <c r="C141" t="n">
         <v>8888</v>
       </c>
       <c r="D141" t="n">
-        <v>3102.48</v>
+        <v>2275.21</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3124,17 +3124,17 @@
         <v>46218</v>
       </c>
       <c r="B142" t="n">
-        <v>609</v>
+        <v>477</v>
       </c>
       <c r="C142" t="n">
         <v>8888</v>
       </c>
       <c r="D142" t="n">
-        <v>1633.68</v>
+        <v>707.52</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3143,17 +3143,17 @@
         <v>46218</v>
       </c>
       <c r="B143" t="n">
-        <v>483</v>
+        <v>2660</v>
       </c>
       <c r="C143" t="n">
         <v>8888</v>
       </c>
       <c r="D143" t="n">
-        <v>1578.32</v>
+        <v>2684.97</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3162,17 +3162,17 @@
         <v>46218</v>
       </c>
       <c r="B144" t="n">
-        <v>2089</v>
+        <v>569</v>
       </c>
       <c r="C144" t="n">
-        <v>1533</v>
+        <v>8888</v>
       </c>
       <c r="D144" t="n">
-        <v>1309.01</v>
+        <v>43745.83</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3181,17 +3181,17 @@
         <v>46218</v>
       </c>
       <c r="B145" t="n">
-        <v>1007</v>
+        <v>483</v>
       </c>
       <c r="C145" t="n">
         <v>8888</v>
       </c>
       <c r="D145" t="n">
-        <v>241.44</v>
+        <v>3102.48</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3200,17 +3200,17 @@
         <v>46218</v>
       </c>
       <c r="B146" t="n">
-        <v>1380</v>
+        <v>609</v>
       </c>
       <c r="C146" t="n">
         <v>8888</v>
       </c>
       <c r="D146" t="n">
-        <v>520.2</v>
+        <v>1633.68</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3219,17 +3219,17 @@
         <v>46218</v>
       </c>
       <c r="B147" t="n">
-        <v>1102</v>
+        <v>483</v>
       </c>
       <c r="C147" t="n">
         <v>8888</v>
       </c>
       <c r="D147" t="n">
-        <v>1137.04</v>
+        <v>2011.13</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3238,17 +3238,17 @@
         <v>46218</v>
       </c>
       <c r="B148" t="n">
-        <v>1075</v>
+        <v>2089</v>
       </c>
       <c r="C148" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D148" t="n">
-        <v>5710.94</v>
+        <v>1309.01</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3257,17 +3257,17 @@
         <v>46218</v>
       </c>
       <c r="B149" t="n">
-        <v>2681</v>
+        <v>1007</v>
       </c>
       <c r="C149" t="n">
         <v>8888</v>
       </c>
       <c r="D149" t="n">
-        <v>729.25</v>
+        <v>241.44</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3276,17 +3276,17 @@
         <v>46218</v>
       </c>
       <c r="B150" t="n">
-        <v>2245</v>
+        <v>1380</v>
       </c>
       <c r="C150" t="n">
         <v>8888</v>
       </c>
       <c r="D150" t="n">
-        <v>700.2</v>
+        <v>520.2</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3295,17 +3295,17 @@
         <v>46218</v>
       </c>
       <c r="B151" t="n">
-        <v>33</v>
+        <v>1102</v>
       </c>
       <c r="C151" t="n">
         <v>8888</v>
       </c>
       <c r="D151" t="n">
-        <v>926.97</v>
+        <v>1137.04</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3314,13 +3314,13 @@
         <v>46218</v>
       </c>
       <c r="B152" t="n">
-        <v>132</v>
+        <v>1075</v>
       </c>
       <c r="C152" t="n">
         <v>8888</v>
       </c>
       <c r="D152" t="n">
-        <v>6522.92</v>
+        <v>5710.94</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -3333,17 +3333,17 @@
         <v>46218</v>
       </c>
       <c r="B153" t="n">
-        <v>619</v>
+        <v>2681</v>
       </c>
       <c r="C153" t="n">
         <v>8888</v>
       </c>
       <c r="D153" t="n">
-        <v>2912.89</v>
+        <v>729.25</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3352,17 +3352,17 @@
         <v>46218</v>
       </c>
       <c r="B154" t="n">
-        <v>452</v>
+        <v>2245</v>
       </c>
       <c r="C154" t="n">
         <v>8888</v>
       </c>
       <c r="D154" t="n">
-        <v>608.78</v>
+        <v>700.2</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3371,17 +3371,17 @@
         <v>46218</v>
       </c>
       <c r="B155" t="n">
-        <v>2463</v>
+        <v>40</v>
       </c>
       <c r="C155" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D155" t="n">
-        <v>363.69</v>
+        <v>678.21</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3390,17 +3390,17 @@
         <v>46218</v>
       </c>
       <c r="B156" t="n">
-        <v>1293</v>
+        <v>33</v>
       </c>
       <c r="C156" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D156" t="n">
-        <v>1780.93</v>
+        <v>926.97</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3409,17 +3409,17 @@
         <v>46218</v>
       </c>
       <c r="B157" t="n">
-        <v>525</v>
+        <v>132</v>
       </c>
       <c r="C157" t="n">
         <v>8888</v>
       </c>
       <c r="D157" t="n">
-        <v>5658.57</v>
+        <v>6522.92</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3428,13 +3428,13 @@
         <v>46218</v>
       </c>
       <c r="B158" t="n">
-        <v>2641</v>
+        <v>619</v>
       </c>
       <c r="C158" t="n">
         <v>8888</v>
       </c>
       <c r="D158" t="n">
-        <v>1720.99</v>
+        <v>2912.89</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -3447,17 +3447,17 @@
         <v>46218</v>
       </c>
       <c r="B159" t="n">
-        <v>2697</v>
+        <v>2769</v>
       </c>
       <c r="C159" t="n">
-        <v>8888</v>
+        <v>977</v>
       </c>
       <c r="D159" t="n">
-        <v>418.65</v>
+        <v>1116.56</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3466,17 +3466,17 @@
         <v>46218</v>
       </c>
       <c r="B160" t="n">
-        <v>2472</v>
+        <v>452</v>
       </c>
       <c r="C160" t="n">
-        <v>2853</v>
+        <v>8888</v>
       </c>
       <c r="D160" t="n">
-        <v>1402.64</v>
+        <v>608.78</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3485,17 +3485,17 @@
         <v>46218</v>
       </c>
       <c r="B161" t="n">
-        <v>58</v>
+        <v>2463</v>
       </c>
       <c r="C161" t="n">
         <v>8888</v>
       </c>
       <c r="D161" t="n">
-        <v>1123.87</v>
+        <v>363.69</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3504,17 +3504,17 @@
         <v>46218</v>
       </c>
       <c r="B162" t="n">
-        <v>358</v>
+        <v>1293</v>
       </c>
       <c r="C162" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D162" t="n">
-        <v>1675.95</v>
+        <v>1780.93</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3523,17 +3523,17 @@
         <v>46218</v>
       </c>
       <c r="B163" t="n">
-        <v>2431</v>
+        <v>525</v>
       </c>
       <c r="C163" t="n">
         <v>8888</v>
       </c>
       <c r="D163" t="n">
-        <v>266.89</v>
+        <v>5658.57</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3542,13 +3542,13 @@
         <v>46218</v>
       </c>
       <c r="B164" t="n">
-        <v>285</v>
+        <v>2641</v>
       </c>
       <c r="C164" t="n">
         <v>8888</v>
       </c>
       <c r="D164" t="n">
-        <v>5673.85</v>
+        <v>1720.99</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -3561,17 +3561,17 @@
         <v>46218</v>
       </c>
       <c r="B165" t="n">
-        <v>1102</v>
+        <v>58</v>
       </c>
       <c r="C165" t="n">
         <v>8888</v>
       </c>
       <c r="D165" t="n">
-        <v>1119.32</v>
+        <v>4929.8</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3580,17 +3580,17 @@
         <v>46218</v>
       </c>
       <c r="B166" t="n">
-        <v>2793</v>
+        <v>325</v>
       </c>
       <c r="C166" t="n">
-        <v>8888</v>
+        <v>1098</v>
       </c>
       <c r="D166" t="n">
-        <v>1238.11</v>
+        <v>50.06</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3599,17 +3599,17 @@
         <v>46218</v>
       </c>
       <c r="B167" t="n">
-        <v>626</v>
+        <v>2697</v>
       </c>
       <c r="C167" t="n">
         <v>8888</v>
       </c>
       <c r="D167" t="n">
-        <v>12556.19</v>
+        <v>418.65</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3618,13 +3618,13 @@
         <v>46218</v>
       </c>
       <c r="B168" t="n">
-        <v>1137</v>
+        <v>2472</v>
       </c>
       <c r="C168" t="n">
-        <v>2220</v>
+        <v>2853</v>
       </c>
       <c r="D168" t="n">
-        <v>1370.86</v>
+        <v>1402.64</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -3637,17 +3637,17 @@
         <v>46218</v>
       </c>
       <c r="B169" t="n">
-        <v>1289</v>
+        <v>358</v>
       </c>
       <c r="C169" t="n">
         <v>8888</v>
       </c>
       <c r="D169" t="n">
-        <v>5565.44</v>
+        <v>1675.95</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3656,17 +3656,17 @@
         <v>46218</v>
       </c>
       <c r="B170" t="n">
-        <v>2686</v>
+        <v>2431</v>
       </c>
       <c r="C170" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D170" t="n">
-        <v>2066.36</v>
+        <v>266.89</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3675,17 +3675,17 @@
         <v>46218</v>
       </c>
       <c r="B171" t="n">
-        <v>629</v>
+        <v>285</v>
       </c>
       <c r="C171" t="n">
         <v>8888</v>
       </c>
       <c r="D171" t="n">
-        <v>5212.76</v>
+        <v>5673.85</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3694,17 +3694,17 @@
         <v>46218</v>
       </c>
       <c r="B172" t="n">
-        <v>2584</v>
+        <v>1102</v>
       </c>
       <c r="C172" t="n">
         <v>8888</v>
       </c>
       <c r="D172" t="n">
-        <v>5635.67</v>
+        <v>2301.43</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3713,13 +3713,13 @@
         <v>46218</v>
       </c>
       <c r="B173" t="n">
-        <v>1756</v>
+        <v>2793</v>
       </c>
       <c r="C173" t="n">
         <v>8888</v>
       </c>
       <c r="D173" t="n">
-        <v>2201.67</v>
+        <v>1238.11</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -3732,17 +3732,17 @@
         <v>46218</v>
       </c>
       <c r="B174" t="n">
-        <v>1756</v>
+        <v>626</v>
       </c>
       <c r="C174" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D174" t="n">
-        <v>5078.1</v>
+        <v>12556.19</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3751,17 +3751,17 @@
         <v>46218</v>
       </c>
       <c r="B175" t="n">
-        <v>2651</v>
+        <v>424</v>
       </c>
       <c r="C175" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D175" t="n">
-        <v>363.7</v>
+        <v>1124.8</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3770,17 +3770,17 @@
         <v>46218</v>
       </c>
       <c r="B176" t="n">
-        <v>664</v>
+        <v>1137</v>
       </c>
       <c r="C176" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D176" t="n">
-        <v>5672.57</v>
+        <v>1370.86</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3789,17 +3789,17 @@
         <v>46218</v>
       </c>
       <c r="B177" t="n">
-        <v>360</v>
+        <v>1299</v>
       </c>
       <c r="C177" t="n">
-        <v>8888</v>
+        <v>2522</v>
       </c>
       <c r="D177" t="n">
-        <v>1594.84</v>
+        <v>8881.309999999999</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3808,17 +3808,17 @@
         <v>46218</v>
       </c>
       <c r="B178" t="n">
-        <v>2582</v>
+        <v>1289</v>
       </c>
       <c r="C178" t="n">
         <v>8888</v>
       </c>
       <c r="D178" t="n">
-        <v>379.33</v>
+        <v>5565.44</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3827,17 +3827,17 @@
         <v>46218</v>
       </c>
       <c r="B179" t="n">
-        <v>636</v>
+        <v>2686</v>
       </c>
       <c r="C179" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D179" t="n">
-        <v>2447.56</v>
+        <v>2066.36</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3846,13 +3846,13 @@
         <v>46218</v>
       </c>
       <c r="B180" t="n">
-        <v>1254</v>
+        <v>629</v>
       </c>
       <c r="C180" t="n">
         <v>8888</v>
       </c>
       <c r="D180" t="n">
-        <v>2643.22</v>
+        <v>5212.76</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -3865,17 +3865,17 @@
         <v>46218</v>
       </c>
       <c r="B181" t="n">
-        <v>2726</v>
+        <v>2584</v>
       </c>
       <c r="C181" t="n">
-        <v>977</v>
+        <v>8888</v>
       </c>
       <c r="D181" t="n">
-        <v>586.0599999999999</v>
+        <v>5635.67</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3884,17 +3884,17 @@
         <v>46218</v>
       </c>
       <c r="B182" t="n">
-        <v>2015</v>
+        <v>1756</v>
       </c>
       <c r="C182" t="n">
         <v>8888</v>
       </c>
       <c r="D182" t="n">
-        <v>315.69</v>
+        <v>3242.54</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3903,17 +3903,17 @@
         <v>46218</v>
       </c>
       <c r="B183" t="n">
-        <v>1064</v>
+        <v>1756</v>
       </c>
       <c r="C183" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D183" t="n">
-        <v>1274.3</v>
+        <v>5078.1</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3922,17 +3922,17 @@
         <v>46218</v>
       </c>
       <c r="B184" t="n">
-        <v>2698</v>
+        <v>2651</v>
       </c>
       <c r="C184" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D184" t="n">
-        <v>552.15</v>
+        <v>363.7</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3941,17 +3941,17 @@
         <v>46218</v>
       </c>
       <c r="B185" t="n">
-        <v>2641</v>
+        <v>664</v>
       </c>
       <c r="C185" t="n">
         <v>8888</v>
       </c>
       <c r="D185" t="n">
-        <v>820</v>
+        <v>6478.17</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3960,17 +3960,17 @@
         <v>46218</v>
       </c>
       <c r="B186" t="n">
-        <v>429</v>
+        <v>360</v>
       </c>
       <c r="C186" t="n">
         <v>8888</v>
       </c>
       <c r="D186" t="n">
-        <v>2593.49</v>
+        <v>1594.84</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3979,17 +3979,17 @@
         <v>46218</v>
       </c>
       <c r="B187" t="n">
-        <v>1301</v>
+        <v>2582</v>
       </c>
       <c r="C187" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D187" t="n">
-        <v>750.66</v>
+        <v>379.33</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3998,13 +3998,13 @@
         <v>46218</v>
       </c>
       <c r="B188" t="n">
-        <v>816</v>
+        <v>636</v>
       </c>
       <c r="C188" t="n">
         <v>8888</v>
       </c>
       <c r="D188" t="n">
-        <v>438.24</v>
+        <v>2447.56</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -4017,13 +4017,13 @@
         <v>46218</v>
       </c>
       <c r="B189" t="n">
-        <v>2359</v>
+        <v>1254</v>
       </c>
       <c r="C189" t="n">
         <v>8888</v>
       </c>
       <c r="D189" t="n">
-        <v>381.95</v>
+        <v>2643.22</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -4036,13 +4036,13 @@
         <v>46218</v>
       </c>
       <c r="B190" t="n">
-        <v>2251</v>
+        <v>2726</v>
       </c>
       <c r="C190" t="n">
-        <v>3403</v>
+        <v>977</v>
       </c>
       <c r="D190" t="n">
-        <v>802.08</v>
+        <v>586.0599999999999</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -4055,17 +4055,17 @@
         <v>46218</v>
       </c>
       <c r="B191" t="n">
-        <v>285</v>
+        <v>2015</v>
       </c>
       <c r="C191" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D191" t="n">
-        <v>364.99</v>
+        <v>315.69</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4074,13 +4074,13 @@
         <v>46218</v>
       </c>
       <c r="B192" t="n">
-        <v>2114</v>
+        <v>1064</v>
       </c>
       <c r="C192" t="n">
         <v>8888</v>
       </c>
       <c r="D192" t="n">
-        <v>2726.04</v>
+        <v>1274.3</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -4093,17 +4093,17 @@
         <v>46218</v>
       </c>
       <c r="B193" t="n">
-        <v>953</v>
+        <v>2698</v>
       </c>
       <c r="C193" t="n">
         <v>8888</v>
       </c>
       <c r="D193" t="n">
-        <v>2889.63</v>
+        <v>552.15</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4112,13 +4112,13 @@
         <v>46218</v>
       </c>
       <c r="B194" t="n">
-        <v>1102</v>
+        <v>2641</v>
       </c>
       <c r="C194" t="n">
         <v>8888</v>
       </c>
       <c r="D194" t="n">
-        <v>4637.07</v>
+        <v>820</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -4131,17 +4131,17 @@
         <v>46218</v>
       </c>
       <c r="B195" t="n">
-        <v>1465</v>
+        <v>429</v>
       </c>
       <c r="C195" t="n">
         <v>8888</v>
       </c>
       <c r="D195" t="n">
-        <v>4281.39</v>
+        <v>2593.49</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4150,17 +4150,17 @@
         <v>46218</v>
       </c>
       <c r="B196" t="n">
-        <v>619</v>
+        <v>1301</v>
       </c>
       <c r="C196" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D196" t="n">
-        <v>2021.67</v>
+        <v>750.66</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4169,17 +4169,17 @@
         <v>46218</v>
       </c>
       <c r="B197" t="n">
-        <v>2716</v>
+        <v>816</v>
       </c>
       <c r="C197" t="n">
         <v>8888</v>
       </c>
       <c r="D197" t="n">
-        <v>1063.42</v>
+        <v>438.24</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4188,17 +4188,17 @@
         <v>46218</v>
       </c>
       <c r="B198" t="n">
-        <v>2767</v>
+        <v>2359</v>
       </c>
       <c r="C198" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D198" t="n">
-        <v>1135.64</v>
+        <v>381.95</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4207,17 +4207,17 @@
         <v>46218</v>
       </c>
       <c r="B199" t="n">
-        <v>2245</v>
+        <v>2251</v>
       </c>
       <c r="C199" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D199" t="n">
-        <v>764.66</v>
+        <v>802.08</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4226,17 +4226,17 @@
         <v>46218</v>
       </c>
       <c r="B200" t="n">
-        <v>2197</v>
+        <v>285</v>
       </c>
       <c r="C200" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D200" t="n">
-        <v>1085.45</v>
+        <v>1797.95</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4245,17 +4245,17 @@
         <v>46218</v>
       </c>
       <c r="B201" t="n">
-        <v>1064</v>
+        <v>2114</v>
       </c>
       <c r="C201" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D201" t="n">
-        <v>574.7</v>
+        <v>2726.04</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4264,17 +4264,17 @@
         <v>46218</v>
       </c>
       <c r="B202" t="n">
-        <v>2657</v>
+        <v>953</v>
       </c>
       <c r="C202" t="n">
         <v>8888</v>
       </c>
       <c r="D202" t="n">
-        <v>2683.06</v>
+        <v>2889.63</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4283,17 +4283,17 @@
         <v>46218</v>
       </c>
       <c r="B203" t="n">
-        <v>451</v>
+        <v>1102</v>
       </c>
       <c r="C203" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D203" t="n">
-        <v>2091.77</v>
+        <v>6347.79</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4302,17 +4302,17 @@
         <v>46218</v>
       </c>
       <c r="B204" t="n">
-        <v>1116</v>
+        <v>1465</v>
       </c>
       <c r="C204" t="n">
-        <v>13148</v>
+        <v>8888</v>
       </c>
       <c r="D204" t="n">
-        <v>207.91</v>
+        <v>4281.39</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4321,17 +4321,17 @@
         <v>46218</v>
       </c>
       <c r="B205" t="n">
-        <v>1277</v>
+        <v>619</v>
       </c>
       <c r="C205" t="n">
         <v>8888</v>
       </c>
       <c r="D205" t="n">
-        <v>1949</v>
+        <v>2021.67</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4340,17 +4340,17 @@
         <v>46218</v>
       </c>
       <c r="B206" t="n">
-        <v>131</v>
+        <v>2716</v>
       </c>
       <c r="C206" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D206" t="n">
-        <v>3850.09</v>
+        <v>1063.42</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4359,17 +4359,17 @@
         <v>46218</v>
       </c>
       <c r="B207" t="n">
-        <v>2692</v>
+        <v>2767</v>
       </c>
       <c r="C207" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D207" t="n">
-        <v>731.28</v>
+        <v>1135.64</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4378,13 +4378,13 @@
         <v>46218</v>
       </c>
       <c r="B208" t="n">
-        <v>1632</v>
+        <v>2657</v>
       </c>
       <c r="C208" t="n">
         <v>8888</v>
       </c>
       <c r="D208" t="n">
-        <v>7519.7</v>
+        <v>3149.7</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -4397,17 +4397,17 @@
         <v>46218</v>
       </c>
       <c r="B209" t="n">
-        <v>1317</v>
+        <v>2245</v>
       </c>
       <c r="C209" t="n">
-        <v>3179</v>
+        <v>8888</v>
       </c>
       <c r="D209" t="n">
-        <v>991.6799999999999</v>
+        <v>764.66</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4416,17 +4416,17 @@
         <v>46218</v>
       </c>
       <c r="B210" t="n">
-        <v>1993</v>
+        <v>2197</v>
       </c>
       <c r="C210" t="n">
         <v>8888</v>
       </c>
       <c r="D210" t="n">
-        <v>2875.39</v>
+        <v>1085.45</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4435,13 +4435,13 @@
         <v>46218</v>
       </c>
       <c r="B211" t="n">
-        <v>1890</v>
+        <v>1064</v>
       </c>
       <c r="C211" t="n">
-        <v>3449</v>
+        <v>27</v>
       </c>
       <c r="D211" t="n">
-        <v>6313.56</v>
+        <v>574.7</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -4454,17 +4454,17 @@
         <v>46218</v>
       </c>
       <c r="B212" t="n">
-        <v>1800</v>
+        <v>451</v>
       </c>
       <c r="C212" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D212" t="n">
-        <v>430.37</v>
+        <v>2091.77</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4473,17 +4473,17 @@
         <v>46218</v>
       </c>
       <c r="B213" t="n">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="C213" t="n">
-        <v>8888</v>
+        <v>13148</v>
       </c>
       <c r="D213" t="n">
-        <v>672.47</v>
+        <v>1455.21</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4492,17 +4492,17 @@
         <v>46218</v>
       </c>
       <c r="B214" t="n">
-        <v>2749</v>
+        <v>1277</v>
       </c>
       <c r="C214" t="n">
         <v>8888</v>
       </c>
       <c r="D214" t="n">
-        <v>1860.64</v>
+        <v>1949</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4511,17 +4511,17 @@
         <v>46218</v>
       </c>
       <c r="B215" t="n">
-        <v>42</v>
+        <v>131</v>
       </c>
       <c r="C215" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D215" t="n">
-        <v>280.05</v>
+        <v>3850.09</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4530,13 +4530,13 @@
         <v>46218</v>
       </c>
       <c r="B216" t="n">
-        <v>1478</v>
+        <v>2692</v>
       </c>
       <c r="C216" t="n">
         <v>8888</v>
       </c>
       <c r="D216" t="n">
-        <v>875.34</v>
+        <v>731.28</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -4549,13 +4549,13 @@
         <v>46218</v>
       </c>
       <c r="B217" t="n">
-        <v>2491</v>
+        <v>1632</v>
       </c>
       <c r="C217" t="n">
         <v>8888</v>
       </c>
       <c r="D217" t="n">
-        <v>650.4299999999999</v>
+        <v>7519.7</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -4568,17 +4568,17 @@
         <v>46218</v>
       </c>
       <c r="B218" t="n">
-        <v>353</v>
+        <v>1317</v>
       </c>
       <c r="C218" t="n">
-        <v>8888</v>
+        <v>3179</v>
       </c>
       <c r="D218" t="n">
-        <v>653.13</v>
+        <v>991.6799999999999</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4587,13 +4587,13 @@
         <v>46218</v>
       </c>
       <c r="B219" t="n">
-        <v>2015</v>
+        <v>1993</v>
       </c>
       <c r="C219" t="n">
         <v>8888</v>
       </c>
       <c r="D219" t="n">
-        <v>4436.15</v>
+        <v>3508.59</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -4606,17 +4606,17 @@
         <v>46218</v>
       </c>
       <c r="B220" t="n">
-        <v>559</v>
+        <v>1890</v>
       </c>
       <c r="C220" t="n">
-        <v>8888</v>
+        <v>3449</v>
       </c>
       <c r="D220" t="n">
-        <v>1453.53</v>
+        <v>6313.56</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4625,17 +4625,17 @@
         <v>46218</v>
       </c>
       <c r="B221" t="n">
-        <v>1890</v>
+        <v>1800</v>
       </c>
       <c r="C221" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D221" t="n">
-        <v>1674.57</v>
+        <v>430.37</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4644,17 +4644,17 @@
         <v>46218</v>
       </c>
       <c r="B222" t="n">
-        <v>1317</v>
+        <v>1117</v>
       </c>
       <c r="C222" t="n">
         <v>8888</v>
       </c>
       <c r="D222" t="n">
-        <v>1626.02</v>
+        <v>672.47</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4663,17 +4663,17 @@
         <v>46218</v>
       </c>
       <c r="B223" t="n">
-        <v>2782</v>
+        <v>2749</v>
       </c>
       <c r="C223" t="n">
         <v>8888</v>
       </c>
       <c r="D223" t="n">
-        <v>1786.32</v>
+        <v>1860.64</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4682,13 +4682,13 @@
         <v>46218</v>
       </c>
       <c r="B224" t="n">
-        <v>953</v>
+        <v>42</v>
       </c>
       <c r="C224" t="n">
         <v>8888</v>
       </c>
       <c r="D224" t="n">
-        <v>364.44</v>
+        <v>280.05</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -4701,17 +4701,17 @@
         <v>46218</v>
       </c>
       <c r="B225" t="n">
-        <v>2251</v>
+        <v>1478</v>
       </c>
       <c r="C225" t="n">
         <v>8888</v>
       </c>
       <c r="D225" t="n">
-        <v>989.26</v>
+        <v>875.34</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4720,17 +4720,17 @@
         <v>46218</v>
       </c>
       <c r="B226" t="n">
-        <v>483</v>
+        <v>2491</v>
       </c>
       <c r="C226" t="n">
-        <v>841</v>
+        <v>8888</v>
       </c>
       <c r="D226" t="n">
-        <v>2085.09</v>
+        <v>650.4299999999999</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4739,17 +4739,17 @@
         <v>46218</v>
       </c>
       <c r="B227" t="n">
-        <v>2133</v>
+        <v>353</v>
       </c>
       <c r="C227" t="n">
-        <v>213</v>
+        <v>8888</v>
       </c>
       <c r="D227" t="n">
-        <v>526.8</v>
+        <v>653.13</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4758,17 +4758,17 @@
         <v>46218</v>
       </c>
       <c r="B228" t="n">
-        <v>351</v>
+        <v>2015</v>
       </c>
       <c r="C228" t="n">
-        <v>3009</v>
+        <v>8888</v>
       </c>
       <c r="D228" t="n">
-        <v>416.36</v>
+        <v>4436.15</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4777,17 +4777,17 @@
         <v>46218</v>
       </c>
       <c r="B229" t="n">
-        <v>2250</v>
+        <v>559</v>
       </c>
       <c r="C229" t="n">
         <v>8888</v>
       </c>
       <c r="D229" t="n">
-        <v>709.46</v>
+        <v>3838.57</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4796,17 +4796,17 @@
         <v>46218</v>
       </c>
       <c r="B230" t="n">
-        <v>2648</v>
+        <v>1890</v>
       </c>
       <c r="C230" t="n">
-        <v>8888</v>
+        <v>1953</v>
       </c>
       <c r="D230" t="n">
-        <v>1873.52</v>
+        <v>1674.57</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4815,13 +4815,13 @@
         <v>46218</v>
       </c>
       <c r="B231" t="n">
-        <v>131</v>
+        <v>1317</v>
       </c>
       <c r="C231" t="n">
         <v>8888</v>
       </c>
       <c r="D231" t="n">
-        <v>1369.91</v>
+        <v>1626.02</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -4834,17 +4834,17 @@
         <v>46218</v>
       </c>
       <c r="B232" t="n">
-        <v>2790</v>
+        <v>2782</v>
       </c>
       <c r="C232" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D232" t="n">
-        <v>371.88</v>
+        <v>1786.32</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4853,17 +4853,17 @@
         <v>46218</v>
       </c>
       <c r="B233" t="n">
-        <v>363</v>
+        <v>953</v>
       </c>
       <c r="C233" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D233" t="n">
-        <v>635.1</v>
+        <v>364.44</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4872,17 +4872,17 @@
         <v>46218</v>
       </c>
       <c r="B234" t="n">
-        <v>2716</v>
+        <v>2251</v>
       </c>
       <c r="C234" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D234" t="n">
-        <v>1073.33</v>
+        <v>989.26</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4891,13 +4891,13 @@
         <v>46218</v>
       </c>
       <c r="B235" t="n">
-        <v>2298</v>
+        <v>483</v>
       </c>
       <c r="C235" t="n">
-        <v>675</v>
+        <v>841</v>
       </c>
       <c r="D235" t="n">
-        <v>401.85</v>
+        <v>2564.59</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -4910,13 +4910,13 @@
         <v>46218</v>
       </c>
       <c r="B236" t="n">
-        <v>2639</v>
+        <v>2133</v>
       </c>
       <c r="C236" t="n">
-        <v>1953</v>
+        <v>213</v>
       </c>
       <c r="D236" t="n">
-        <v>504.09</v>
+        <v>526.8</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -4929,13 +4929,13 @@
         <v>46218</v>
       </c>
       <c r="B237" t="n">
-        <v>619</v>
+        <v>351</v>
       </c>
       <c r="C237" t="n">
-        <v>1139</v>
+        <v>3009</v>
       </c>
       <c r="D237" t="n">
-        <v>1341.64</v>
+        <v>416.36</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -4948,17 +4948,17 @@
         <v>46218</v>
       </c>
       <c r="B238" t="n">
-        <v>2109</v>
+        <v>2250</v>
       </c>
       <c r="C238" t="n">
         <v>8888</v>
       </c>
       <c r="D238" t="n">
-        <v>2293.78</v>
+        <v>709.46</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4967,17 +4967,17 @@
         <v>46218</v>
       </c>
       <c r="B239" t="n">
-        <v>1116</v>
+        <v>2648</v>
       </c>
       <c r="C239" t="n">
         <v>8888</v>
       </c>
       <c r="D239" t="n">
-        <v>2919.53</v>
+        <v>1873.52</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4986,17 +4986,17 @@
         <v>46218</v>
       </c>
       <c r="B240" t="n">
-        <v>2250</v>
+        <v>131</v>
       </c>
       <c r="C240" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D240" t="n">
-        <v>1803.76</v>
+        <v>1369.91</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -5005,13 +5005,13 @@
         <v>46218</v>
       </c>
       <c r="B241" t="n">
-        <v>2698</v>
+        <v>2298</v>
       </c>
       <c r="C241" t="n">
-        <v>874</v>
+        <v>675</v>
       </c>
       <c r="D241" t="n">
-        <v>1230.43</v>
+        <v>2301.31</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -5024,17 +5024,17 @@
         <v>46218</v>
       </c>
       <c r="B242" t="n">
-        <v>42</v>
+        <v>2790</v>
       </c>
       <c r="C242" t="n">
-        <v>8888</v>
+        <v>1953</v>
       </c>
       <c r="D242" t="n">
-        <v>79947.14999999999</v>
+        <v>371.88</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -5043,17 +5043,17 @@
         <v>46218</v>
       </c>
       <c r="B243" t="n">
-        <v>772</v>
+        <v>363</v>
       </c>
       <c r="C243" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D243" t="n">
-        <v>400.25</v>
+        <v>635.1</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -5062,17 +5062,17 @@
         <v>46218</v>
       </c>
       <c r="B244" t="n">
-        <v>2728</v>
+        <v>2716</v>
       </c>
       <c r="C244" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D244" t="n">
-        <v>1397.07</v>
+        <v>1073.33</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -5081,13 +5081,13 @@
         <v>46218</v>
       </c>
       <c r="B245" t="n">
-        <v>2197</v>
+        <v>2639</v>
       </c>
       <c r="C245" t="n">
-        <v>423</v>
+        <v>1953</v>
       </c>
       <c r="D245" t="n">
-        <v>2267.61</v>
+        <v>504.09</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -5100,13 +5100,13 @@
         <v>46218</v>
       </c>
       <c r="B246" t="n">
-        <v>2716</v>
+        <v>629</v>
       </c>
       <c r="C246" t="n">
-        <v>977</v>
+        <v>675</v>
       </c>
       <c r="D246" t="n">
-        <v>729.29</v>
+        <v>2419.73</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -5119,17 +5119,17 @@
         <v>46218</v>
       </c>
       <c r="B247" t="n">
-        <v>1993</v>
+        <v>619</v>
       </c>
       <c r="C247" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D247" t="n">
-        <v>456.62</v>
+        <v>1341.64</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -5138,17 +5138,188 @@
         <v>46218</v>
       </c>
       <c r="B248" t="n">
-        <v>629</v>
+        <v>2109</v>
       </c>
       <c r="C248" t="n">
-        <v>675</v>
+        <v>8888</v>
       </c>
       <c r="D248" t="n">
-        <v>1054.76</v>
+        <v>2293.78</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B249" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C249" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D249" t="n">
+        <v>2919.53</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B250" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C250" t="n">
+        <v>27</v>
+      </c>
+      <c r="D250" t="n">
+        <v>1803.76</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B251" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C251" t="n">
+        <v>874</v>
+      </c>
+      <c r="D251" t="n">
+        <v>1230.43</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B252" t="n">
+        <v>42</v>
+      </c>
+      <c r="C252" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D252" t="n">
+        <v>79947.14999999999</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B253" t="n">
+        <v>772</v>
+      </c>
+      <c r="C253" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D253" t="n">
+        <v>400.25</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B254" t="n">
+        <v>2728</v>
+      </c>
+      <c r="C254" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D254" t="n">
+        <v>1397.07</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B255" t="n">
+        <v>2197</v>
+      </c>
+      <c r="C255" t="n">
+        <v>423</v>
+      </c>
+      <c r="D255" t="n">
+        <v>2267.61</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B256" t="n">
+        <v>2716</v>
+      </c>
+      <c r="C256" t="n">
+        <v>977</v>
+      </c>
+      <c r="D256" t="n">
+        <v>729.29</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B257" t="n">
+        <v>1993</v>
+      </c>
+      <c r="C257" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D257" t="n">
+        <v>456.62</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 18:00:04
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E257"/>
+  <dimension ref="A1:E267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,7 +489,7 @@
         <v>8888</v>
       </c>
       <c r="D3" t="n">
-        <v>651.77</v>
+        <v>769.05</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -673,13 +673,13 @@
         <v>46218</v>
       </c>
       <c r="B13" t="n">
-        <v>2211</v>
+        <v>2118</v>
       </c>
       <c r="C13" t="n">
         <v>8888</v>
       </c>
       <c r="D13" t="n">
-        <v>2706.2</v>
+        <v>5847.19</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -692,13 +692,13 @@
         <v>46218</v>
       </c>
       <c r="B14" t="n">
-        <v>2660</v>
+        <v>2211</v>
       </c>
       <c r="C14" t="n">
         <v>8888</v>
       </c>
       <c r="D14" t="n">
-        <v>875.61</v>
+        <v>2706.2</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -711,13 +711,13 @@
         <v>46218</v>
       </c>
       <c r="B15" t="n">
-        <v>890</v>
+        <v>2660</v>
       </c>
       <c r="C15" t="n">
         <v>8888</v>
       </c>
       <c r="D15" t="n">
-        <v>1051.23</v>
+        <v>875.61</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -730,13 +730,13 @@
         <v>46218</v>
       </c>
       <c r="B16" t="n">
-        <v>2190</v>
+        <v>890</v>
       </c>
       <c r="C16" t="n">
         <v>8888</v>
       </c>
       <c r="D16" t="n">
-        <v>1307.13</v>
+        <v>1051.23</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -749,17 +749,17 @@
         <v>46218</v>
       </c>
       <c r="B17" t="n">
-        <v>2651</v>
+        <v>2190</v>
       </c>
       <c r="C17" t="n">
         <v>8888</v>
       </c>
       <c r="D17" t="n">
-        <v>660.95</v>
+        <v>1307.13</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -768,17 +768,17 @@
         <v>46218</v>
       </c>
       <c r="B18" t="n">
-        <v>890</v>
+        <v>2651</v>
       </c>
       <c r="C18" t="n">
-        <v>1533</v>
+        <v>8888</v>
       </c>
       <c r="D18" t="n">
-        <v>898.83</v>
+        <v>660.95</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -787,17 +787,17 @@
         <v>46218</v>
       </c>
       <c r="B19" t="n">
-        <v>40</v>
+        <v>890</v>
       </c>
       <c r="C19" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D19" t="n">
-        <v>768.78</v>
+        <v>898.83</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -806,17 +806,17 @@
         <v>46218</v>
       </c>
       <c r="B20" t="n">
-        <v>2118</v>
+        <v>40</v>
       </c>
       <c r="C20" t="n">
         <v>8888</v>
       </c>
       <c r="D20" t="n">
-        <v>5535.71</v>
+        <v>768.78</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -977,13 +977,13 @@
         <v>46218</v>
       </c>
       <c r="B29" t="n">
-        <v>2250</v>
+        <v>2767</v>
       </c>
       <c r="C29" t="n">
         <v>8888</v>
       </c>
       <c r="D29" t="n">
-        <v>1686.37</v>
+        <v>1866.38</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -996,17 +996,17 @@
         <v>46218</v>
       </c>
       <c r="B30" t="n">
-        <v>2695</v>
+        <v>2250</v>
       </c>
       <c r="C30" t="n">
         <v>8888</v>
       </c>
       <c r="D30" t="n">
-        <v>677.6799999999999</v>
+        <v>1686.37</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1015,17 +1015,17 @@
         <v>46218</v>
       </c>
       <c r="B31" t="n">
-        <v>931</v>
+        <v>2695</v>
       </c>
       <c r="C31" t="n">
-        <v>423</v>
+        <v>8888</v>
       </c>
       <c r="D31" t="n">
-        <v>492.34</v>
+        <v>677.6799999999999</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1034,17 +1034,17 @@
         <v>46218</v>
       </c>
       <c r="B32" t="n">
-        <v>1117</v>
+        <v>931</v>
       </c>
       <c r="C32" t="n">
-        <v>8888</v>
+        <v>423</v>
       </c>
       <c r="D32" t="n">
-        <v>540.15</v>
+        <v>492.34</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1053,13 +1053,13 @@
         <v>46218</v>
       </c>
       <c r="B33" t="n">
-        <v>2641</v>
+        <v>1117</v>
       </c>
       <c r="C33" t="n">
         <v>8888</v>
       </c>
       <c r="D33" t="n">
-        <v>2527.79</v>
+        <v>540.15</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1110,13 +1110,13 @@
         <v>46218</v>
       </c>
       <c r="B36" t="n">
-        <v>525</v>
+        <v>2641</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>408.25</v>
+        <v>2527.79</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1129,17 +1129,17 @@
         <v>46218</v>
       </c>
       <c r="B37" t="n">
-        <v>1808</v>
+        <v>525</v>
       </c>
       <c r="C37" t="n">
         <v>8888</v>
       </c>
       <c r="D37" t="n">
-        <v>695.3200000000001</v>
+        <v>408.25</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1148,17 +1148,17 @@
         <v>46218</v>
       </c>
       <c r="B38" t="n">
-        <v>609</v>
+        <v>1808</v>
       </c>
       <c r="C38" t="n">
         <v>8888</v>
       </c>
       <c r="D38" t="n">
-        <v>1909.37</v>
+        <v>695.3200000000001</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1167,17 +1167,17 @@
         <v>46218</v>
       </c>
       <c r="B39" t="n">
-        <v>949</v>
+        <v>609</v>
       </c>
       <c r="C39" t="n">
-        <v>1134</v>
+        <v>8888</v>
       </c>
       <c r="D39" t="n">
-        <v>30.46</v>
+        <v>1909.37</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1186,13 +1186,13 @@
         <v>46218</v>
       </c>
       <c r="B40" t="n">
-        <v>42</v>
+        <v>949</v>
       </c>
       <c r="C40" t="n">
-        <v>1139</v>
+        <v>1134</v>
       </c>
       <c r="D40" t="n">
-        <v>358.97</v>
+        <v>30.46</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1205,17 +1205,17 @@
         <v>46218</v>
       </c>
       <c r="B41" t="n">
-        <v>2499</v>
+        <v>42</v>
       </c>
       <c r="C41" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D41" t="n">
-        <v>1049.3</v>
+        <v>358.97</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1224,13 +1224,13 @@
         <v>46218</v>
       </c>
       <c r="B42" t="n">
-        <v>58</v>
+        <v>2499</v>
       </c>
       <c r="C42" t="n">
         <v>8888</v>
       </c>
       <c r="D42" t="n">
-        <v>2194.12</v>
+        <v>1049.3</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1243,13 +1243,13 @@
         <v>46218</v>
       </c>
       <c r="B43" t="n">
-        <v>2245</v>
+        <v>58</v>
       </c>
       <c r="C43" t="n">
         <v>8888</v>
       </c>
       <c r="D43" t="n">
-        <v>3382.78</v>
+        <v>2194.12</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1262,17 +1262,17 @@
         <v>46218</v>
       </c>
       <c r="B44" t="n">
-        <v>325</v>
+        <v>2245</v>
       </c>
       <c r="C44" t="n">
         <v>8888</v>
       </c>
       <c r="D44" t="n">
-        <v>1079.66</v>
+        <v>3382.78</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1281,17 +1281,17 @@
         <v>46218</v>
       </c>
       <c r="B45" t="n">
-        <v>2383</v>
+        <v>325</v>
       </c>
       <c r="C45" t="n">
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>7926.02</v>
+        <v>1279.15</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1300,17 +1300,17 @@
         <v>46218</v>
       </c>
       <c r="B46" t="n">
-        <v>1117</v>
+        <v>2383</v>
       </c>
       <c r="C46" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>916.72</v>
+        <v>9004.809999999999</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1319,17 +1319,17 @@
         <v>46218</v>
       </c>
       <c r="B47" t="n">
-        <v>374</v>
+        <v>1117</v>
       </c>
       <c r="C47" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D47" t="n">
-        <v>2810.86</v>
+        <v>916.72</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1338,13 +1338,13 @@
         <v>46218</v>
       </c>
       <c r="B48" t="n">
-        <v>2279</v>
+        <v>374</v>
       </c>
       <c r="C48" t="n">
         <v>8888</v>
       </c>
       <c r="D48" t="n">
-        <v>712.66</v>
+        <v>2810.86</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1357,17 +1357,17 @@
         <v>46218</v>
       </c>
       <c r="B49" t="n">
-        <v>535</v>
+        <v>2279</v>
       </c>
       <c r="C49" t="n">
         <v>8888</v>
       </c>
       <c r="D49" t="n">
-        <v>5836.12</v>
+        <v>712.66</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1382,11 +1382,11 @@
         <v>8888</v>
       </c>
       <c r="D50" t="n">
-        <v>1352.51</v>
+        <v>9291.4</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1395,17 +1395,17 @@
         <v>46218</v>
       </c>
       <c r="B51" t="n">
-        <v>2678</v>
+        <v>535</v>
       </c>
       <c r="C51" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D51" t="n">
-        <v>364.96</v>
+        <v>1352.51</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
         <v>46218</v>
       </c>
       <c r="B52" t="n">
-        <v>2345</v>
+        <v>2678</v>
       </c>
       <c r="C52" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D52" t="n">
-        <v>863.16</v>
+        <v>364.96</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1433,17 +1433,17 @@
         <v>46218</v>
       </c>
       <c r="B53" t="n">
-        <v>945</v>
+        <v>2345</v>
       </c>
       <c r="C53" t="n">
         <v>8888</v>
       </c>
       <c r="D53" t="n">
-        <v>27337.21</v>
+        <v>863.16</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>PEDIDO ELETRÔNICO</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1452,17 +1452,17 @@
         <v>46218</v>
       </c>
       <c r="B54" t="n">
-        <v>2686</v>
+        <v>945</v>
       </c>
       <c r="C54" t="n">
         <v>8888</v>
       </c>
       <c r="D54" t="n">
-        <v>684.2</v>
+        <v>30706.36</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>PEDIDO ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -1471,17 +1471,17 @@
         <v>46218</v>
       </c>
       <c r="B55" t="n">
-        <v>438</v>
+        <v>2686</v>
       </c>
       <c r="C55" t="n">
         <v>8888</v>
       </c>
       <c r="D55" t="n">
-        <v>220.06</v>
+        <v>684.2</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1490,17 +1490,17 @@
         <v>46218</v>
       </c>
       <c r="B56" t="n">
-        <v>1956</v>
+        <v>438</v>
       </c>
       <c r="C56" t="n">
         <v>8888</v>
       </c>
       <c r="D56" t="n">
-        <v>5311.01</v>
+        <v>220.06</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1509,17 +1509,17 @@
         <v>46218</v>
       </c>
       <c r="B57" t="n">
-        <v>664</v>
+        <v>1956</v>
       </c>
       <c r="C57" t="n">
         <v>8888</v>
       </c>
       <c r="D57" t="n">
-        <v>6275.01</v>
+        <v>5311.01</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1528,17 +1528,17 @@
         <v>46218</v>
       </c>
       <c r="B58" t="n">
-        <v>353</v>
+        <v>664</v>
       </c>
       <c r="C58" t="n">
-        <v>3179</v>
+        <v>8888</v>
       </c>
       <c r="D58" t="n">
-        <v>495.84</v>
+        <v>6275.01</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1547,17 +1547,17 @@
         <v>46218</v>
       </c>
       <c r="B59" t="n">
-        <v>1293</v>
+        <v>353</v>
       </c>
       <c r="C59" t="n">
-        <v>8888</v>
+        <v>3179</v>
       </c>
       <c r="D59" t="n">
-        <v>3129.07</v>
+        <v>495.84</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1566,13 +1566,13 @@
         <v>46218</v>
       </c>
       <c r="B60" t="n">
-        <v>2279</v>
+        <v>1293</v>
       </c>
       <c r="C60" t="n">
         <v>8888</v>
       </c>
       <c r="D60" t="n">
-        <v>3900.07</v>
+        <v>3129.07</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1585,13 +1585,13 @@
         <v>46218</v>
       </c>
       <c r="B61" t="n">
-        <v>1937</v>
+        <v>2279</v>
       </c>
       <c r="C61" t="n">
         <v>8888</v>
       </c>
       <c r="D61" t="n">
-        <v>1685.72</v>
+        <v>3900.07</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1604,17 +1604,17 @@
         <v>46218</v>
       </c>
       <c r="B62" t="n">
-        <v>941</v>
+        <v>1937</v>
       </c>
       <c r="C62" t="n">
         <v>8888</v>
       </c>
       <c r="D62" t="n">
-        <v>864.14</v>
+        <v>1685.72</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1623,17 +1623,17 @@
         <v>46218</v>
       </c>
       <c r="B63" t="n">
-        <v>1137</v>
+        <v>941</v>
       </c>
       <c r="C63" t="n">
         <v>8888</v>
       </c>
       <c r="D63" t="n">
-        <v>1947.93</v>
+        <v>864.14</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1642,17 +1642,17 @@
         <v>46218</v>
       </c>
       <c r="B64" t="n">
-        <v>2631</v>
+        <v>1137</v>
       </c>
       <c r="C64" t="n">
-        <v>2853</v>
+        <v>8888</v>
       </c>
       <c r="D64" t="n">
-        <v>2418.28</v>
+        <v>3168.9</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1661,13 +1661,13 @@
         <v>46218</v>
       </c>
       <c r="B65" t="n">
-        <v>2793</v>
+        <v>2631</v>
       </c>
       <c r="C65" t="n">
-        <v>977</v>
+        <v>2853</v>
       </c>
       <c r="D65" t="n">
-        <v>1188.59</v>
+        <v>2418.28</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1680,17 +1680,17 @@
         <v>46218</v>
       </c>
       <c r="B66" t="n">
-        <v>2802</v>
+        <v>2793</v>
       </c>
       <c r="C66" t="n">
-        <v>8888</v>
+        <v>977</v>
       </c>
       <c r="D66" t="n">
-        <v>1264.57</v>
+        <v>1188.59</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1699,13 +1699,13 @@
         <v>46218</v>
       </c>
       <c r="B67" t="n">
-        <v>451</v>
+        <v>2802</v>
       </c>
       <c r="C67" t="n">
         <v>8888</v>
       </c>
       <c r="D67" t="n">
-        <v>757.5700000000001</v>
+        <v>1264.57</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1718,17 +1718,17 @@
         <v>46218</v>
       </c>
       <c r="B68" t="n">
-        <v>374</v>
+        <v>451</v>
       </c>
       <c r="C68" t="n">
         <v>8888</v>
       </c>
       <c r="D68" t="n">
-        <v>44.6</v>
+        <v>757.5700000000001</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1737,17 +1737,17 @@
         <v>46218</v>
       </c>
       <c r="B69" t="n">
-        <v>703</v>
+        <v>374</v>
       </c>
       <c r="C69" t="n">
         <v>8888</v>
       </c>
       <c r="D69" t="n">
-        <v>12155.46</v>
+        <v>44.6</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1756,17 +1756,17 @@
         <v>46218</v>
       </c>
       <c r="B70" t="n">
-        <v>1756</v>
+        <v>703</v>
       </c>
       <c r="C70" t="n">
         <v>8888</v>
       </c>
       <c r="D70" t="n">
-        <v>4416.47</v>
+        <v>12155.46</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1775,17 @@
         <v>46218</v>
       </c>
       <c r="B71" t="n">
-        <v>925</v>
+        <v>1756</v>
       </c>
       <c r="C71" t="n">
         <v>8888</v>
       </c>
       <c r="D71" t="n">
-        <v>651.59</v>
+        <v>4416.47</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1794,17 +1794,17 @@
         <v>46218</v>
       </c>
       <c r="B72" t="n">
-        <v>941</v>
+        <v>925</v>
       </c>
       <c r="C72" t="n">
-        <v>977</v>
+        <v>8888</v>
       </c>
       <c r="D72" t="n">
-        <v>359.73</v>
+        <v>651.59</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1813,17 +1813,17 @@
         <v>46218</v>
       </c>
       <c r="B73" t="n">
-        <v>2648</v>
+        <v>941</v>
       </c>
       <c r="C73" t="n">
-        <v>8888</v>
+        <v>977</v>
       </c>
       <c r="D73" t="n">
-        <v>1594.42</v>
+        <v>359.73</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1832,13 +1832,13 @@
         <v>46218</v>
       </c>
       <c r="B74" t="n">
-        <v>663</v>
+        <v>2648</v>
       </c>
       <c r="C74" t="n">
         <v>8888</v>
       </c>
       <c r="D74" t="n">
-        <v>6645.33</v>
+        <v>1594.42</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -1851,17 +1851,17 @@
         <v>46218</v>
       </c>
       <c r="B75" t="n">
-        <v>2714</v>
+        <v>663</v>
       </c>
       <c r="C75" t="n">
-        <v>519</v>
+        <v>8888</v>
       </c>
       <c r="D75" t="n">
-        <v>61939.22</v>
+        <v>6645.33</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1870,17 +1870,17 @@
         <v>46218</v>
       </c>
       <c r="B76" t="n">
-        <v>483</v>
+        <v>2714</v>
       </c>
       <c r="C76" t="n">
-        <v>8888</v>
+        <v>519</v>
       </c>
       <c r="D76" t="n">
-        <v>12405.46</v>
+        <v>61939.22</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1889,17 +1889,17 @@
         <v>46218</v>
       </c>
       <c r="B77" t="n">
-        <v>1075</v>
+        <v>483</v>
       </c>
       <c r="C77" t="n">
         <v>8888</v>
       </c>
       <c r="D77" t="n">
-        <v>11607.79</v>
+        <v>12405.46</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1908,13 +1908,13 @@
         <v>46218</v>
       </c>
       <c r="B78" t="n">
-        <v>629</v>
+        <v>1075</v>
       </c>
       <c r="C78" t="n">
         <v>8888</v>
       </c>
       <c r="D78" t="n">
-        <v>9233.719999999999</v>
+        <v>11607.79</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -1927,17 +1927,17 @@
         <v>46218</v>
       </c>
       <c r="B79" t="n">
-        <v>1983</v>
+        <v>629</v>
       </c>
       <c r="C79" t="n">
-        <v>841</v>
+        <v>8888</v>
       </c>
       <c r="D79" t="n">
-        <v>633.79</v>
+        <v>9233.719999999999</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1946,17 +1946,17 @@
         <v>46218</v>
       </c>
       <c r="B80" t="n">
-        <v>1137</v>
+        <v>1983</v>
       </c>
       <c r="C80" t="n">
-        <v>8888</v>
+        <v>841</v>
       </c>
       <c r="D80" t="n">
-        <v>3578.51</v>
+        <v>633.79</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1965,17 +1965,17 @@
         <v>46218</v>
       </c>
       <c r="B81" t="n">
-        <v>2651</v>
+        <v>1137</v>
       </c>
       <c r="C81" t="n">
         <v>8888</v>
       </c>
       <c r="D81" t="n">
-        <v>1296.58</v>
+        <v>4842.54</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1984,17 +1984,17 @@
         <v>46218</v>
       </c>
       <c r="B82" t="n">
-        <v>2789</v>
+        <v>2651</v>
       </c>
       <c r="C82" t="n">
         <v>8888</v>
       </c>
       <c r="D82" t="n">
-        <v>1293.93</v>
+        <v>1296.58</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2003,17 +2003,17 @@
         <v>46218</v>
       </c>
       <c r="B83" t="n">
-        <v>1956</v>
+        <v>2789</v>
       </c>
       <c r="C83" t="n">
-        <v>423</v>
+        <v>8888</v>
       </c>
       <c r="D83" t="n">
-        <v>1416.35</v>
+        <v>1293.93</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2022,17 +2022,17 @@
         <v>46218</v>
       </c>
       <c r="B84" t="n">
-        <v>2709</v>
+        <v>1956</v>
       </c>
       <c r="C84" t="n">
-        <v>8888</v>
+        <v>423</v>
       </c>
       <c r="D84" t="n">
-        <v>547.6900000000001</v>
+        <v>1416.35</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2041,13 +2041,13 @@
         <v>46218</v>
       </c>
       <c r="B85" t="n">
-        <v>1308</v>
+        <v>2709</v>
       </c>
       <c r="C85" t="n">
         <v>8888</v>
       </c>
       <c r="D85" t="n">
-        <v>1460.53</v>
+        <v>547.6900000000001</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2060,17 +2060,17 @@
         <v>46218</v>
       </c>
       <c r="B86" t="n">
-        <v>2026</v>
+        <v>1308</v>
       </c>
       <c r="C86" t="n">
         <v>8888</v>
       </c>
       <c r="D86" t="n">
-        <v>2237.62</v>
+        <v>2264.86</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2079,13 +2079,13 @@
         <v>46218</v>
       </c>
       <c r="B87" t="n">
-        <v>2789</v>
+        <v>2026</v>
       </c>
       <c r="C87" t="n">
         <v>8888</v>
       </c>
       <c r="D87" t="n">
-        <v>747.77</v>
+        <v>2237.62</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2098,17 +2098,17 @@
         <v>46218</v>
       </c>
       <c r="B88" t="n">
-        <v>89</v>
+        <v>2789</v>
       </c>
       <c r="C88" t="n">
-        <v>13148</v>
+        <v>8888</v>
       </c>
       <c r="D88" t="n">
-        <v>2842.03</v>
+        <v>747.77</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2117,17 +2117,17 @@
         <v>46218</v>
       </c>
       <c r="B89" t="n">
-        <v>1075</v>
+        <v>89</v>
       </c>
       <c r="C89" t="n">
-        <v>8888</v>
+        <v>13148</v>
       </c>
       <c r="D89" t="n">
-        <v>698.63</v>
+        <v>2842.03</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2136,17 +2136,17 @@
         <v>46218</v>
       </c>
       <c r="B90" t="n">
-        <v>2709</v>
+        <v>1075</v>
       </c>
       <c r="C90" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D90" t="n">
-        <v>390.19</v>
+        <v>698.63</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2155,17 +2155,17 @@
         <v>46218</v>
       </c>
       <c r="B91" t="n">
-        <v>2345</v>
+        <v>2709</v>
       </c>
       <c r="C91" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D91" t="n">
-        <v>748.86</v>
+        <v>390.19</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2174,17 +2174,17 @@
         <v>46218</v>
       </c>
       <c r="B92" t="n">
-        <v>1983</v>
+        <v>2211</v>
       </c>
       <c r="C92" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D92" t="n">
-        <v>2806.44</v>
+        <v>2268.78</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2193,17 +2193,17 @@
         <v>46218</v>
       </c>
       <c r="B93" t="n">
-        <v>2765</v>
+        <v>2345</v>
       </c>
       <c r="C93" t="n">
-        <v>1883</v>
+        <v>8888</v>
       </c>
       <c r="D93" t="n">
-        <v>3638.6</v>
+        <v>748.86</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2212,17 +2212,17 @@
         <v>46218</v>
       </c>
       <c r="B94" t="n">
-        <v>569</v>
+        <v>1983</v>
       </c>
       <c r="C94" t="n">
         <v>8888</v>
       </c>
       <c r="D94" t="n">
-        <v>995.33</v>
+        <v>2806.44</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2231,13 +2231,13 @@
         <v>46218</v>
       </c>
       <c r="B95" t="n">
-        <v>360</v>
+        <v>2765</v>
       </c>
       <c r="C95" t="n">
-        <v>546</v>
+        <v>1883</v>
       </c>
       <c r="D95" t="n">
-        <v>1609.68</v>
+        <v>3638.6</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2250,17 +2250,17 @@
         <v>46218</v>
       </c>
       <c r="B96" t="n">
-        <v>2711</v>
+        <v>569</v>
       </c>
       <c r="C96" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D96" t="n">
-        <v>150.27</v>
+        <v>995.33</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2269,17 +2269,17 @@
         <v>46218</v>
       </c>
       <c r="B97" t="n">
-        <v>2279</v>
+        <v>360</v>
       </c>
       <c r="C97" t="n">
-        <v>8888</v>
+        <v>546</v>
       </c>
       <c r="D97" t="n">
-        <v>447.5</v>
+        <v>1609.68</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2288,17 +2288,17 @@
         <v>46218</v>
       </c>
       <c r="B98" t="n">
-        <v>2308</v>
+        <v>2711</v>
       </c>
       <c r="C98" t="n">
-        <v>8888</v>
+        <v>1953</v>
       </c>
       <c r="D98" t="n">
-        <v>488.69</v>
+        <v>150.27</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2307,17 +2307,17 @@
         <v>46218</v>
       </c>
       <c r="B99" t="n">
-        <v>2211</v>
+        <v>2279</v>
       </c>
       <c r="C99" t="n">
-        <v>874</v>
+        <v>8888</v>
       </c>
       <c r="D99" t="n">
-        <v>1526.94</v>
+        <v>447.5</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2326,13 +2326,13 @@
         <v>46218</v>
       </c>
       <c r="B100" t="n">
-        <v>559</v>
+        <v>2308</v>
       </c>
       <c r="C100" t="n">
         <v>8888</v>
       </c>
       <c r="D100" t="n">
-        <v>859.92</v>
+        <v>488.69</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2345,13 +2345,13 @@
         <v>46218</v>
       </c>
       <c r="B101" t="n">
-        <v>890</v>
+        <v>559</v>
       </c>
       <c r="C101" t="n">
         <v>8888</v>
       </c>
       <c r="D101" t="n">
-        <v>387.2</v>
+        <v>859.92</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2364,17 +2364,17 @@
         <v>46218</v>
       </c>
       <c r="B102" t="n">
-        <v>2768</v>
+        <v>890</v>
       </c>
       <c r="C102" t="n">
         <v>8888</v>
       </c>
       <c r="D102" t="n">
-        <v>6523.26</v>
+        <v>387.2</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2383,13 +2383,13 @@
         <v>46218</v>
       </c>
       <c r="B103" t="n">
-        <v>1063</v>
+        <v>2768</v>
       </c>
       <c r="C103" t="n">
         <v>8888</v>
       </c>
       <c r="D103" t="n">
-        <v>4487.11</v>
+        <v>7812.09</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2402,17 +2402,17 @@
         <v>46218</v>
       </c>
       <c r="B104" t="n">
-        <v>947</v>
+        <v>1063</v>
       </c>
       <c r="C104" t="n">
         <v>8888</v>
       </c>
       <c r="D104" t="n">
-        <v>5667.85</v>
+        <v>4487.11</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>PEDIDO ELETRÔNICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2421,17 +2421,17 @@
         <v>46218</v>
       </c>
       <c r="B105" t="n">
-        <v>2279</v>
+        <v>947</v>
       </c>
       <c r="C105" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D105" t="n">
-        <v>1031.06</v>
+        <v>5667.85</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>PEDIDO ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -2440,13 +2440,13 @@
         <v>46218</v>
       </c>
       <c r="B106" t="n">
-        <v>1299</v>
+        <v>2279</v>
       </c>
       <c r="C106" t="n">
-        <v>27</v>
+        <v>1139</v>
       </c>
       <c r="D106" t="n">
-        <v>1435.52</v>
+        <v>1031.06</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2459,13 +2459,13 @@
         <v>46218</v>
       </c>
       <c r="B107" t="n">
-        <v>1478</v>
+        <v>1299</v>
       </c>
       <c r="C107" t="n">
-        <v>675</v>
+        <v>27</v>
       </c>
       <c r="D107" t="n">
-        <v>1967.85</v>
+        <v>1435.52</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -2478,17 +2478,17 @@
         <v>46218</v>
       </c>
       <c r="B108" t="n">
-        <v>767</v>
+        <v>1478</v>
       </c>
       <c r="C108" t="n">
-        <v>8888</v>
+        <v>675</v>
       </c>
       <c r="D108" t="n">
-        <v>3292.44</v>
+        <v>1967.85</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2497,17 +2497,17 @@
         <v>46218</v>
       </c>
       <c r="B109" t="n">
-        <v>285</v>
+        <v>675</v>
       </c>
       <c r="C109" t="n">
         <v>8888</v>
       </c>
       <c r="D109" t="n">
-        <v>3349.8</v>
+        <v>2685.73</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2516,17 +2516,17 @@
         <v>46218</v>
       </c>
       <c r="B110" t="n">
-        <v>477</v>
+        <v>767</v>
       </c>
       <c r="C110" t="n">
         <v>8888</v>
       </c>
       <c r="D110" t="n">
-        <v>917.33</v>
+        <v>3292.44</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2535,17 +2535,17 @@
         <v>46218</v>
       </c>
       <c r="B111" t="n">
-        <v>1983</v>
+        <v>285</v>
       </c>
       <c r="C111" t="n">
         <v>8888</v>
       </c>
       <c r="D111" t="n">
-        <v>5115.01</v>
+        <v>3349.8</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2557,14 +2557,14 @@
         <v>477</v>
       </c>
       <c r="C112" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D112" t="n">
-        <v>3946.44</v>
+        <v>917.33</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2573,13 +2573,13 @@
         <v>46218</v>
       </c>
       <c r="B113" t="n">
-        <v>1937</v>
+        <v>1983</v>
       </c>
       <c r="C113" t="n">
         <v>8888</v>
       </c>
       <c r="D113" t="n">
-        <v>2600.61</v>
+        <v>5115.01</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -2592,17 +2592,17 @@
         <v>46218</v>
       </c>
       <c r="B114" t="n">
-        <v>1063</v>
+        <v>477</v>
       </c>
       <c r="C114" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D114" t="n">
-        <v>2549.86</v>
+        <v>3946.44</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2611,17 +2611,17 @@
         <v>46218</v>
       </c>
       <c r="B115" t="n">
-        <v>2584</v>
+        <v>1937</v>
       </c>
       <c r="C115" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D115" t="n">
-        <v>756.16</v>
+        <v>2600.61</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2630,17 +2630,17 @@
         <v>46218</v>
       </c>
       <c r="B116" t="n">
-        <v>58</v>
+        <v>363</v>
       </c>
       <c r="C116" t="n">
         <v>8888</v>
       </c>
       <c r="D116" t="n">
-        <v>558.03</v>
+        <v>780.35</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2649,13 +2649,13 @@
         <v>46218</v>
       </c>
       <c r="B117" t="n">
-        <v>424</v>
+        <v>1063</v>
       </c>
       <c r="C117" t="n">
         <v>8888</v>
       </c>
       <c r="D117" t="n">
-        <v>1362.42</v>
+        <v>2549.86</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -2668,13 +2668,13 @@
         <v>46218</v>
       </c>
       <c r="B118" t="n">
-        <v>675</v>
+        <v>360</v>
       </c>
       <c r="C118" t="n">
         <v>8888</v>
       </c>
       <c r="D118" t="n">
-        <v>616.73</v>
+        <v>5917.55</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -2687,17 +2687,17 @@
         <v>46218</v>
       </c>
       <c r="B119" t="n">
-        <v>663</v>
+        <v>2584</v>
       </c>
       <c r="C119" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D119" t="n">
-        <v>255.13</v>
+        <v>756.16</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2706,13 +2706,13 @@
         <v>46218</v>
       </c>
       <c r="B120" t="n">
-        <v>1993</v>
+        <v>58</v>
       </c>
       <c r="C120" t="n">
         <v>8888</v>
       </c>
       <c r="D120" t="n">
-        <v>724.14</v>
+        <v>558.03</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -2725,17 +2725,17 @@
         <v>46218</v>
       </c>
       <c r="B121" t="n">
-        <v>1465</v>
+        <v>424</v>
       </c>
       <c r="C121" t="n">
         <v>8888</v>
       </c>
       <c r="D121" t="n">
-        <v>7362.56</v>
+        <v>1362.42</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2744,17 +2744,17 @@
         <v>46218</v>
       </c>
       <c r="B122" t="n">
-        <v>89</v>
+        <v>663</v>
       </c>
       <c r="C122" t="n">
         <v>8888</v>
       </c>
       <c r="D122" t="n">
-        <v>479</v>
+        <v>255.13</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2763,17 +2763,17 @@
         <v>46218</v>
       </c>
       <c r="B123" t="n">
-        <v>595</v>
+        <v>1993</v>
       </c>
       <c r="C123" t="n">
         <v>8888</v>
       </c>
       <c r="D123" t="n">
-        <v>18084.5</v>
+        <v>724.14</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2782,17 +2782,17 @@
         <v>46218</v>
       </c>
       <c r="B124" t="n">
-        <v>2696</v>
+        <v>1465</v>
       </c>
       <c r="C124" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D124" t="n">
-        <v>1597.76</v>
+        <v>7362.56</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2801,17 +2801,17 @@
         <v>46218</v>
       </c>
       <c r="B125" t="n">
-        <v>360</v>
+        <v>89</v>
       </c>
       <c r="C125" t="n">
         <v>8888</v>
       </c>
       <c r="D125" t="n">
-        <v>4596.89</v>
+        <v>479</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2820,17 +2820,17 @@
         <v>46218</v>
       </c>
       <c r="B126" t="n">
-        <v>1465</v>
+        <v>595</v>
       </c>
       <c r="C126" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D126" t="n">
-        <v>777.2</v>
+        <v>18084.5</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2839,17 +2839,17 @@
         <v>46218</v>
       </c>
       <c r="B127" t="n">
-        <v>2178</v>
+        <v>2696</v>
       </c>
       <c r="C127" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D127" t="n">
-        <v>619.92</v>
+        <v>1597.76</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2858,13 +2858,13 @@
         <v>46218</v>
       </c>
       <c r="B128" t="n">
-        <v>2026</v>
+        <v>1465</v>
       </c>
       <c r="C128" t="n">
-        <v>1929</v>
+        <v>3403</v>
       </c>
       <c r="D128" t="n">
-        <v>6021.92</v>
+        <v>777.2</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -2877,17 +2877,17 @@
         <v>46218</v>
       </c>
       <c r="B129" t="n">
-        <v>630</v>
+        <v>2178</v>
       </c>
       <c r="C129" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D129" t="n">
-        <v>1801.63</v>
+        <v>619.92</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2896,17 +2896,17 @@
         <v>46218</v>
       </c>
       <c r="B130" t="n">
-        <v>1937</v>
+        <v>2026</v>
       </c>
       <c r="C130" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D130" t="n">
-        <v>2132.95</v>
+        <v>6021.92</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2915,17 +2915,17 @@
         <v>46218</v>
       </c>
       <c r="B131" t="n">
-        <v>2577</v>
+        <v>630</v>
       </c>
       <c r="C131" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D131" t="n">
-        <v>1647.08</v>
+        <v>1801.63</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2934,13 +2934,13 @@
         <v>46218</v>
       </c>
       <c r="B132" t="n">
-        <v>1293</v>
+        <v>1937</v>
       </c>
       <c r="C132" t="n">
         <v>8888</v>
       </c>
       <c r="D132" t="n">
-        <v>2135.89</v>
+        <v>2132.95</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -2953,13 +2953,13 @@
         <v>46218</v>
       </c>
       <c r="B133" t="n">
-        <v>2607</v>
+        <v>2577</v>
       </c>
       <c r="C133" t="n">
         <v>8888</v>
       </c>
       <c r="D133" t="n">
-        <v>490.31</v>
+        <v>1647.08</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -2972,17 +2972,17 @@
         <v>46218</v>
       </c>
       <c r="B134" t="n">
-        <v>1317</v>
+        <v>1293</v>
       </c>
       <c r="C134" t="n">
         <v>8888</v>
       </c>
       <c r="D134" t="n">
-        <v>907.72</v>
+        <v>2135.89</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2991,13 +2991,13 @@
         <v>46218</v>
       </c>
       <c r="B135" t="n">
-        <v>619</v>
+        <v>2607</v>
       </c>
       <c r="C135" t="n">
         <v>8888</v>
       </c>
       <c r="D135" t="n">
-        <v>1081.74</v>
+        <v>490.31</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3010,17 +3010,17 @@
         <v>46218</v>
       </c>
       <c r="B136" t="n">
-        <v>2571</v>
+        <v>1317</v>
       </c>
       <c r="C136" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D136" t="n">
-        <v>268.53</v>
+        <v>907.72</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3029,17 +3029,17 @@
         <v>46218</v>
       </c>
       <c r="B137" t="n">
-        <v>20</v>
+        <v>535</v>
       </c>
       <c r="C137" t="n">
-        <v>8888</v>
+        <v>2571</v>
       </c>
       <c r="D137" t="n">
-        <v>745.55</v>
+        <v>1124.46</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3048,13 +3048,13 @@
         <v>46218</v>
       </c>
       <c r="B138" t="n">
-        <v>1063</v>
+        <v>675</v>
       </c>
       <c r="C138" t="n">
         <v>8888</v>
       </c>
       <c r="D138" t="n">
-        <v>1113.08</v>
+        <v>337.89</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3067,17 +3067,17 @@
         <v>46218</v>
       </c>
       <c r="B139" t="n">
-        <v>2631</v>
+        <v>2571</v>
       </c>
       <c r="C139" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D139" t="n">
-        <v>1447.86</v>
+        <v>743.01</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3086,13 +3086,13 @@
         <v>46218</v>
       </c>
       <c r="B140" t="n">
-        <v>1906</v>
+        <v>619</v>
       </c>
       <c r="C140" t="n">
         <v>8888</v>
       </c>
       <c r="D140" t="n">
-        <v>2774.84</v>
+        <v>1081.74</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3105,13 +3105,13 @@
         <v>46218</v>
       </c>
       <c r="B141" t="n">
-        <v>1756</v>
+        <v>20</v>
       </c>
       <c r="C141" t="n">
         <v>8888</v>
       </c>
       <c r="D141" t="n">
-        <v>2275.21</v>
+        <v>745.55</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3124,13 +3124,13 @@
         <v>46218</v>
       </c>
       <c r="B142" t="n">
-        <v>477</v>
+        <v>1063</v>
       </c>
       <c r="C142" t="n">
         <v>8888</v>
       </c>
       <c r="D142" t="n">
-        <v>707.52</v>
+        <v>1113.08</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3143,13 +3143,13 @@
         <v>46218</v>
       </c>
       <c r="B143" t="n">
-        <v>2660</v>
+        <v>2631</v>
       </c>
       <c r="C143" t="n">
         <v>8888</v>
       </c>
       <c r="D143" t="n">
-        <v>2684.97</v>
+        <v>1447.86</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3162,17 +3162,17 @@
         <v>46218</v>
       </c>
       <c r="B144" t="n">
-        <v>569</v>
+        <v>1906</v>
       </c>
       <c r="C144" t="n">
         <v>8888</v>
       </c>
       <c r="D144" t="n">
-        <v>43745.83</v>
+        <v>2774.84</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3181,17 +3181,17 @@
         <v>46218</v>
       </c>
       <c r="B145" t="n">
-        <v>483</v>
+        <v>1756</v>
       </c>
       <c r="C145" t="n">
         <v>8888</v>
       </c>
       <c r="D145" t="n">
-        <v>3102.48</v>
+        <v>2275.21</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3200,17 +3200,17 @@
         <v>46218</v>
       </c>
       <c r="B146" t="n">
-        <v>609</v>
+        <v>477</v>
       </c>
       <c r="C146" t="n">
         <v>8888</v>
       </c>
       <c r="D146" t="n">
-        <v>1633.68</v>
+        <v>707.52</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3219,17 +3219,17 @@
         <v>46218</v>
       </c>
       <c r="B147" t="n">
-        <v>483</v>
+        <v>2660</v>
       </c>
       <c r="C147" t="n">
         <v>8888</v>
       </c>
       <c r="D147" t="n">
-        <v>2011.13</v>
+        <v>2684.97</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3238,17 +3238,17 @@
         <v>46218</v>
       </c>
       <c r="B148" t="n">
-        <v>2089</v>
+        <v>569</v>
       </c>
       <c r="C148" t="n">
-        <v>1533</v>
+        <v>8888</v>
       </c>
       <c r="D148" t="n">
-        <v>1309.01</v>
+        <v>43745.83</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3257,17 +3257,17 @@
         <v>46218</v>
       </c>
       <c r="B149" t="n">
-        <v>1007</v>
+        <v>483</v>
       </c>
       <c r="C149" t="n">
         <v>8888</v>
       </c>
       <c r="D149" t="n">
-        <v>241.44</v>
+        <v>3102.48</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3276,17 +3276,17 @@
         <v>46218</v>
       </c>
       <c r="B150" t="n">
-        <v>1380</v>
+        <v>609</v>
       </c>
       <c r="C150" t="n">
         <v>8888</v>
       </c>
       <c r="D150" t="n">
-        <v>520.2</v>
+        <v>1633.68</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3295,17 +3295,17 @@
         <v>46218</v>
       </c>
       <c r="B151" t="n">
-        <v>1102</v>
+        <v>483</v>
       </c>
       <c r="C151" t="n">
         <v>8888</v>
       </c>
       <c r="D151" t="n">
-        <v>1137.04</v>
+        <v>2011.13</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3314,17 +3314,17 @@
         <v>46218</v>
       </c>
       <c r="B152" t="n">
-        <v>1075</v>
+        <v>2089</v>
       </c>
       <c r="C152" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D152" t="n">
-        <v>5710.94</v>
+        <v>1309.01</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3333,17 +3333,17 @@
         <v>46218</v>
       </c>
       <c r="B153" t="n">
-        <v>2681</v>
+        <v>1007</v>
       </c>
       <c r="C153" t="n">
         <v>8888</v>
       </c>
       <c r="D153" t="n">
-        <v>729.25</v>
+        <v>241.44</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3352,17 +3352,17 @@
         <v>46218</v>
       </c>
       <c r="B154" t="n">
-        <v>2245</v>
+        <v>1380</v>
       </c>
       <c r="C154" t="n">
         <v>8888</v>
       </c>
       <c r="D154" t="n">
-        <v>700.2</v>
+        <v>520.2</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3371,17 +3371,17 @@
         <v>46218</v>
       </c>
       <c r="B155" t="n">
-        <v>40</v>
+        <v>1102</v>
       </c>
       <c r="C155" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D155" t="n">
-        <v>678.21</v>
+        <v>1137.04</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3390,17 +3390,17 @@
         <v>46218</v>
       </c>
       <c r="B156" t="n">
-        <v>33</v>
+        <v>358</v>
       </c>
       <c r="C156" t="n">
         <v>8888</v>
       </c>
       <c r="D156" t="n">
-        <v>926.97</v>
+        <v>3380.3</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3409,13 +3409,13 @@
         <v>46218</v>
       </c>
       <c r="B157" t="n">
-        <v>132</v>
+        <v>1075</v>
       </c>
       <c r="C157" t="n">
         <v>8888</v>
       </c>
       <c r="D157" t="n">
-        <v>6522.92</v>
+        <v>5710.94</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -3428,17 +3428,17 @@
         <v>46218</v>
       </c>
       <c r="B158" t="n">
-        <v>619</v>
+        <v>2681</v>
       </c>
       <c r="C158" t="n">
         <v>8888</v>
       </c>
       <c r="D158" t="n">
-        <v>2912.89</v>
+        <v>729.25</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3447,17 +3447,17 @@
         <v>46218</v>
       </c>
       <c r="B159" t="n">
-        <v>2769</v>
+        <v>2245</v>
       </c>
       <c r="C159" t="n">
-        <v>977</v>
+        <v>8888</v>
       </c>
       <c r="D159" t="n">
-        <v>1116.56</v>
+        <v>700.2</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3466,17 +3466,17 @@
         <v>46218</v>
       </c>
       <c r="B160" t="n">
-        <v>452</v>
+        <v>40</v>
       </c>
       <c r="C160" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D160" t="n">
-        <v>608.78</v>
+        <v>678.21</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3485,17 +3485,17 @@
         <v>46218</v>
       </c>
       <c r="B161" t="n">
-        <v>2463</v>
+        <v>33</v>
       </c>
       <c r="C161" t="n">
         <v>8888</v>
       </c>
       <c r="D161" t="n">
-        <v>363.69</v>
+        <v>926.97</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3504,17 +3504,17 @@
         <v>46218</v>
       </c>
       <c r="B162" t="n">
-        <v>1293</v>
+        <v>132</v>
       </c>
       <c r="C162" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D162" t="n">
-        <v>1780.93</v>
+        <v>6522.92</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3523,13 +3523,13 @@
         <v>46218</v>
       </c>
       <c r="B163" t="n">
-        <v>525</v>
+        <v>619</v>
       </c>
       <c r="C163" t="n">
         <v>8888</v>
       </c>
       <c r="D163" t="n">
-        <v>5658.57</v>
+        <v>2912.89</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -3542,17 +3542,17 @@
         <v>46218</v>
       </c>
       <c r="B164" t="n">
-        <v>2641</v>
+        <v>2769</v>
       </c>
       <c r="C164" t="n">
-        <v>8888</v>
+        <v>977</v>
       </c>
       <c r="D164" t="n">
-        <v>1720.99</v>
+        <v>1116.56</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3561,13 +3561,13 @@
         <v>46218</v>
       </c>
       <c r="B165" t="n">
-        <v>58</v>
+        <v>452</v>
       </c>
       <c r="C165" t="n">
         <v>8888</v>
       </c>
       <c r="D165" t="n">
-        <v>4929.8</v>
+        <v>608.78</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -3580,17 +3580,17 @@
         <v>46218</v>
       </c>
       <c r="B166" t="n">
-        <v>325</v>
+        <v>2463</v>
       </c>
       <c r="C166" t="n">
-        <v>1098</v>
+        <v>8888</v>
       </c>
       <c r="D166" t="n">
-        <v>50.06</v>
+        <v>363.69</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3599,17 +3599,17 @@
         <v>46218</v>
       </c>
       <c r="B167" t="n">
-        <v>2697</v>
+        <v>1293</v>
       </c>
       <c r="C167" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D167" t="n">
-        <v>418.65</v>
+        <v>1780.93</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3618,17 +3618,17 @@
         <v>46218</v>
       </c>
       <c r="B168" t="n">
-        <v>2472</v>
+        <v>525</v>
       </c>
       <c r="C168" t="n">
-        <v>2853</v>
+        <v>8888</v>
       </c>
       <c r="D168" t="n">
-        <v>1402.64</v>
+        <v>5658.57</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3637,17 +3637,17 @@
         <v>46218</v>
       </c>
       <c r="B169" t="n">
-        <v>358</v>
+        <v>2641</v>
       </c>
       <c r="C169" t="n">
         <v>8888</v>
       </c>
       <c r="D169" t="n">
-        <v>1675.95</v>
+        <v>1720.99</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3656,17 +3656,17 @@
         <v>46218</v>
       </c>
       <c r="B170" t="n">
-        <v>2431</v>
+        <v>675</v>
       </c>
       <c r="C170" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D170" t="n">
-        <v>266.89</v>
+        <v>504.07</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3675,17 +3675,17 @@
         <v>46218</v>
       </c>
       <c r="B171" t="n">
-        <v>285</v>
+        <v>58</v>
       </c>
       <c r="C171" t="n">
         <v>8888</v>
       </c>
       <c r="D171" t="n">
-        <v>5673.85</v>
+        <v>4929.8</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3694,17 +3694,17 @@
         <v>46218</v>
       </c>
       <c r="B172" t="n">
-        <v>1102</v>
+        <v>358</v>
       </c>
       <c r="C172" t="n">
-        <v>8888</v>
+        <v>546</v>
       </c>
       <c r="D172" t="n">
-        <v>2301.43</v>
+        <v>862.4400000000001</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3713,17 +3713,17 @@
         <v>46218</v>
       </c>
       <c r="B173" t="n">
-        <v>2793</v>
+        <v>325</v>
       </c>
       <c r="C173" t="n">
-        <v>8888</v>
+        <v>1098</v>
       </c>
       <c r="D173" t="n">
-        <v>1238.11</v>
+        <v>50.06</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3732,17 +3732,17 @@
         <v>46218</v>
       </c>
       <c r="B174" t="n">
-        <v>626</v>
+        <v>2697</v>
       </c>
       <c r="C174" t="n">
         <v>8888</v>
       </c>
       <c r="D174" t="n">
-        <v>12556.19</v>
+        <v>833.38</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3751,17 +3751,17 @@
         <v>46218</v>
       </c>
       <c r="B175" t="n">
-        <v>424</v>
+        <v>2472</v>
       </c>
       <c r="C175" t="n">
-        <v>8888</v>
+        <v>2853</v>
       </c>
       <c r="D175" t="n">
-        <v>1124.8</v>
+        <v>1402.64</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3770,17 +3770,17 @@
         <v>46218</v>
       </c>
       <c r="B176" t="n">
-        <v>1137</v>
+        <v>2431</v>
       </c>
       <c r="C176" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D176" t="n">
-        <v>1370.86</v>
+        <v>266.89</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3789,17 +3789,17 @@
         <v>46218</v>
       </c>
       <c r="B177" t="n">
-        <v>1299</v>
+        <v>285</v>
       </c>
       <c r="C177" t="n">
-        <v>2522</v>
+        <v>8888</v>
       </c>
       <c r="D177" t="n">
-        <v>8881.309999999999</v>
+        <v>5673.85</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3808,17 +3808,17 @@
         <v>46218</v>
       </c>
       <c r="B178" t="n">
-        <v>1289</v>
+        <v>1102</v>
       </c>
       <c r="C178" t="n">
         <v>8888</v>
       </c>
       <c r="D178" t="n">
-        <v>5565.44</v>
+        <v>2301.43</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3827,17 +3827,17 @@
         <v>46218</v>
       </c>
       <c r="B179" t="n">
-        <v>2686</v>
+        <v>2793</v>
       </c>
       <c r="C179" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D179" t="n">
-        <v>2066.36</v>
+        <v>1238.11</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3846,17 +3846,17 @@
         <v>46218</v>
       </c>
       <c r="B180" t="n">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="C180" t="n">
         <v>8888</v>
       </c>
       <c r="D180" t="n">
-        <v>5212.76</v>
+        <v>23157.24</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3865,17 +3865,17 @@
         <v>46218</v>
       </c>
       <c r="B181" t="n">
-        <v>2584</v>
+        <v>424</v>
       </c>
       <c r="C181" t="n">
         <v>8888</v>
       </c>
       <c r="D181" t="n">
-        <v>5635.67</v>
+        <v>1124.8</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3884,17 +3884,17 @@
         <v>46218</v>
       </c>
       <c r="B182" t="n">
-        <v>1756</v>
+        <v>1137</v>
       </c>
       <c r="C182" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D182" t="n">
-        <v>3242.54</v>
+        <v>3285.55</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3903,13 +3903,13 @@
         <v>46218</v>
       </c>
       <c r="B183" t="n">
-        <v>1756</v>
+        <v>1299</v>
       </c>
       <c r="C183" t="n">
-        <v>27</v>
+        <v>2522</v>
       </c>
       <c r="D183" t="n">
-        <v>5078.1</v>
+        <v>8881.309999999999</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -3922,17 +3922,17 @@
         <v>46218</v>
       </c>
       <c r="B184" t="n">
-        <v>2651</v>
+        <v>1289</v>
       </c>
       <c r="C184" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D184" t="n">
-        <v>363.7</v>
+        <v>5565.44</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3941,17 +3941,17 @@
         <v>46218</v>
       </c>
       <c r="B185" t="n">
-        <v>664</v>
+        <v>2686</v>
       </c>
       <c r="C185" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D185" t="n">
-        <v>6478.17</v>
+        <v>2066.36</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3960,17 +3960,17 @@
         <v>46218</v>
       </c>
       <c r="B186" t="n">
-        <v>360</v>
+        <v>629</v>
       </c>
       <c r="C186" t="n">
         <v>8888</v>
       </c>
       <c r="D186" t="n">
-        <v>1594.84</v>
+        <v>5212.76</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3979,17 +3979,17 @@
         <v>46218</v>
       </c>
       <c r="B187" t="n">
-        <v>2582</v>
+        <v>636</v>
       </c>
       <c r="C187" t="n">
         <v>8888</v>
       </c>
       <c r="D187" t="n">
-        <v>379.33</v>
+        <v>5742.49</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3998,17 +3998,17 @@
         <v>46218</v>
       </c>
       <c r="B188" t="n">
-        <v>636</v>
+        <v>2584</v>
       </c>
       <c r="C188" t="n">
         <v>8888</v>
       </c>
       <c r="D188" t="n">
-        <v>2447.56</v>
+        <v>5635.67</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4017,17 +4017,17 @@
         <v>46218</v>
       </c>
       <c r="B189" t="n">
-        <v>1254</v>
+        <v>1756</v>
       </c>
       <c r="C189" t="n">
         <v>8888</v>
       </c>
       <c r="D189" t="n">
-        <v>2643.22</v>
+        <v>3242.54</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4036,17 +4036,17 @@
         <v>46218</v>
       </c>
       <c r="B190" t="n">
-        <v>2726</v>
+        <v>2698</v>
       </c>
       <c r="C190" t="n">
-        <v>977</v>
+        <v>8888</v>
       </c>
       <c r="D190" t="n">
-        <v>586.0599999999999</v>
+        <v>859.49</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4055,17 +4055,17 @@
         <v>46218</v>
       </c>
       <c r="B191" t="n">
-        <v>2015</v>
+        <v>1756</v>
       </c>
       <c r="C191" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D191" t="n">
-        <v>315.69</v>
+        <v>5078.1</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4074,17 +4074,17 @@
         <v>46218</v>
       </c>
       <c r="B192" t="n">
-        <v>1064</v>
+        <v>2651</v>
       </c>
       <c r="C192" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D192" t="n">
-        <v>1274.3</v>
+        <v>363.7</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4093,17 +4093,17 @@
         <v>46218</v>
       </c>
       <c r="B193" t="n">
-        <v>2698</v>
+        <v>664</v>
       </c>
       <c r="C193" t="n">
         <v>8888</v>
       </c>
       <c r="D193" t="n">
-        <v>552.15</v>
+        <v>6478.17</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4112,17 +4112,17 @@
         <v>46218</v>
       </c>
       <c r="B194" t="n">
-        <v>2641</v>
+        <v>360</v>
       </c>
       <c r="C194" t="n">
         <v>8888</v>
       </c>
       <c r="D194" t="n">
-        <v>820</v>
+        <v>1594.84</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4131,17 +4131,17 @@
         <v>46218</v>
       </c>
       <c r="B195" t="n">
-        <v>429</v>
+        <v>2582</v>
       </c>
       <c r="C195" t="n">
         <v>8888</v>
       </c>
       <c r="D195" t="n">
-        <v>2593.49</v>
+        <v>379.33</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4150,17 +4150,17 @@
         <v>46218</v>
       </c>
       <c r="B196" t="n">
-        <v>1301</v>
+        <v>1254</v>
       </c>
       <c r="C196" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D196" t="n">
-        <v>750.66</v>
+        <v>2643.22</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4169,17 +4169,17 @@
         <v>46218</v>
       </c>
       <c r="B197" t="n">
-        <v>816</v>
+        <v>2726</v>
       </c>
       <c r="C197" t="n">
-        <v>8888</v>
+        <v>977</v>
       </c>
       <c r="D197" t="n">
-        <v>438.24</v>
+        <v>586.0599999999999</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4188,17 +4188,17 @@
         <v>46218</v>
       </c>
       <c r="B198" t="n">
-        <v>2359</v>
+        <v>2015</v>
       </c>
       <c r="C198" t="n">
         <v>8888</v>
       </c>
       <c r="D198" t="n">
-        <v>381.95</v>
+        <v>315.69</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4207,17 +4207,17 @@
         <v>46218</v>
       </c>
       <c r="B199" t="n">
-        <v>2251</v>
+        <v>1064</v>
       </c>
       <c r="C199" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D199" t="n">
-        <v>802.08</v>
+        <v>1274.3</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4226,17 +4226,17 @@
         <v>46218</v>
       </c>
       <c r="B200" t="n">
-        <v>285</v>
+        <v>358</v>
       </c>
       <c r="C200" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D200" t="n">
-        <v>1797.95</v>
+        <v>2619.4</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4245,17 +4245,17 @@
         <v>46218</v>
       </c>
       <c r="B201" t="n">
-        <v>2114</v>
+        <v>2641</v>
       </c>
       <c r="C201" t="n">
         <v>8888</v>
       </c>
       <c r="D201" t="n">
-        <v>2726.04</v>
+        <v>820</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4264,17 +4264,17 @@
         <v>46218</v>
       </c>
       <c r="B202" t="n">
-        <v>953</v>
+        <v>429</v>
       </c>
       <c r="C202" t="n">
         <v>8888</v>
       </c>
       <c r="D202" t="n">
-        <v>2889.63</v>
+        <v>2593.49</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4283,17 +4283,17 @@
         <v>46218</v>
       </c>
       <c r="B203" t="n">
-        <v>1102</v>
+        <v>1301</v>
       </c>
       <c r="C203" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D203" t="n">
-        <v>6347.79</v>
+        <v>750.66</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4302,17 +4302,17 @@
         <v>46218</v>
       </c>
       <c r="B204" t="n">
-        <v>1465</v>
+        <v>816</v>
       </c>
       <c r="C204" t="n">
         <v>8888</v>
       </c>
       <c r="D204" t="n">
-        <v>4281.39</v>
+        <v>438.24</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4321,17 +4321,17 @@
         <v>46218</v>
       </c>
       <c r="B205" t="n">
-        <v>619</v>
+        <v>2359</v>
       </c>
       <c r="C205" t="n">
         <v>8888</v>
       </c>
       <c r="D205" t="n">
-        <v>2021.67</v>
+        <v>381.95</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4340,17 +4340,17 @@
         <v>46218</v>
       </c>
       <c r="B206" t="n">
-        <v>2716</v>
+        <v>2251</v>
       </c>
       <c r="C206" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D206" t="n">
-        <v>1063.42</v>
+        <v>802.08</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4359,13 +4359,13 @@
         <v>46218</v>
       </c>
       <c r="B207" t="n">
-        <v>2767</v>
+        <v>285</v>
       </c>
       <c r="C207" t="n">
-        <v>1898</v>
+        <v>58</v>
       </c>
       <c r="D207" t="n">
-        <v>1135.64</v>
+        <v>1797.95</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -4378,13 +4378,13 @@
         <v>46218</v>
       </c>
       <c r="B208" t="n">
-        <v>2657</v>
+        <v>2114</v>
       </c>
       <c r="C208" t="n">
         <v>8888</v>
       </c>
       <c r="D208" t="n">
-        <v>3149.7</v>
+        <v>2726.04</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -4397,17 +4397,17 @@
         <v>46218</v>
       </c>
       <c r="B209" t="n">
-        <v>2245</v>
+        <v>953</v>
       </c>
       <c r="C209" t="n">
         <v>8888</v>
       </c>
       <c r="D209" t="n">
-        <v>764.66</v>
+        <v>2889.63</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4416,17 +4416,17 @@
         <v>46218</v>
       </c>
       <c r="B210" t="n">
-        <v>2197</v>
+        <v>1102</v>
       </c>
       <c r="C210" t="n">
         <v>8888</v>
       </c>
       <c r="D210" t="n">
-        <v>1085.45</v>
+        <v>6347.79</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4435,17 +4435,17 @@
         <v>46218</v>
       </c>
       <c r="B211" t="n">
-        <v>1064</v>
+        <v>1465</v>
       </c>
       <c r="C211" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D211" t="n">
-        <v>574.7</v>
+        <v>4281.39</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4454,17 +4454,17 @@
         <v>46218</v>
       </c>
       <c r="B212" t="n">
-        <v>451</v>
+        <v>619</v>
       </c>
       <c r="C212" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D212" t="n">
-        <v>2091.77</v>
+        <v>2021.67</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4473,17 +4473,17 @@
         <v>46218</v>
       </c>
       <c r="B213" t="n">
-        <v>1116</v>
+        <v>2716</v>
       </c>
       <c r="C213" t="n">
-        <v>13148</v>
+        <v>8888</v>
       </c>
       <c r="D213" t="n">
-        <v>1455.21</v>
+        <v>1063.42</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4492,17 +4492,17 @@
         <v>46218</v>
       </c>
       <c r="B214" t="n">
-        <v>1277</v>
+        <v>2767</v>
       </c>
       <c r="C214" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D214" t="n">
-        <v>1949</v>
+        <v>1135.64</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4511,17 +4511,17 @@
         <v>46218</v>
       </c>
       <c r="B215" t="n">
-        <v>131</v>
+        <v>2657</v>
       </c>
       <c r="C215" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D215" t="n">
-        <v>3850.09</v>
+        <v>3149.7</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4530,17 +4530,17 @@
         <v>46218</v>
       </c>
       <c r="B216" t="n">
-        <v>2692</v>
+        <v>2245</v>
       </c>
       <c r="C216" t="n">
         <v>8888</v>
       </c>
       <c r="D216" t="n">
-        <v>731.28</v>
+        <v>764.66</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4549,17 +4549,17 @@
         <v>46218</v>
       </c>
       <c r="B217" t="n">
-        <v>1632</v>
+        <v>2197</v>
       </c>
       <c r="C217" t="n">
         <v>8888</v>
       </c>
       <c r="D217" t="n">
-        <v>7519.7</v>
+        <v>1085.45</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4568,13 +4568,13 @@
         <v>46218</v>
       </c>
       <c r="B218" t="n">
-        <v>1317</v>
+        <v>1064</v>
       </c>
       <c r="C218" t="n">
-        <v>3179</v>
+        <v>27</v>
       </c>
       <c r="D218" t="n">
-        <v>991.6799999999999</v>
+        <v>574.7</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -4587,17 +4587,17 @@
         <v>46218</v>
       </c>
       <c r="B219" t="n">
-        <v>1993</v>
+        <v>451</v>
       </c>
       <c r="C219" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D219" t="n">
-        <v>3508.59</v>
+        <v>2091.77</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4606,13 +4606,13 @@
         <v>46218</v>
       </c>
       <c r="B220" t="n">
-        <v>1890</v>
+        <v>1116</v>
       </c>
       <c r="C220" t="n">
-        <v>3449</v>
+        <v>13148</v>
       </c>
       <c r="D220" t="n">
-        <v>6313.56</v>
+        <v>1455.21</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -4625,17 +4625,17 @@
         <v>46218</v>
       </c>
       <c r="B221" t="n">
-        <v>1800</v>
+        <v>1277</v>
       </c>
       <c r="C221" t="n">
         <v>8888</v>
       </c>
       <c r="D221" t="n">
-        <v>430.37</v>
+        <v>1949</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4644,17 +4644,17 @@
         <v>46218</v>
       </c>
       <c r="B222" t="n">
-        <v>1117</v>
+        <v>131</v>
       </c>
       <c r="C222" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D222" t="n">
-        <v>672.47</v>
+        <v>3850.09</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4663,13 +4663,13 @@
         <v>46218</v>
       </c>
       <c r="B223" t="n">
-        <v>2749</v>
+        <v>2692</v>
       </c>
       <c r="C223" t="n">
         <v>8888</v>
       </c>
       <c r="D223" t="n">
-        <v>1860.64</v>
+        <v>731.28</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -4682,13 +4682,13 @@
         <v>46218</v>
       </c>
       <c r="B224" t="n">
-        <v>42</v>
+        <v>1632</v>
       </c>
       <c r="C224" t="n">
         <v>8888</v>
       </c>
       <c r="D224" t="n">
-        <v>280.05</v>
+        <v>7519.7</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -4701,17 +4701,17 @@
         <v>46218</v>
       </c>
       <c r="B225" t="n">
-        <v>1478</v>
+        <v>1317</v>
       </c>
       <c r="C225" t="n">
-        <v>8888</v>
+        <v>3179</v>
       </c>
       <c r="D225" t="n">
-        <v>875.34</v>
+        <v>991.6799999999999</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4720,13 +4720,13 @@
         <v>46218</v>
       </c>
       <c r="B226" t="n">
-        <v>2491</v>
+        <v>1993</v>
       </c>
       <c r="C226" t="n">
         <v>8888</v>
       </c>
       <c r="D226" t="n">
-        <v>650.4299999999999</v>
+        <v>3508.59</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -4739,17 +4739,17 @@
         <v>46218</v>
       </c>
       <c r="B227" t="n">
-        <v>353</v>
+        <v>1890</v>
       </c>
       <c r="C227" t="n">
-        <v>8888</v>
+        <v>3449</v>
       </c>
       <c r="D227" t="n">
-        <v>653.13</v>
+        <v>6313.56</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4758,17 +4758,17 @@
         <v>46218</v>
       </c>
       <c r="B228" t="n">
-        <v>2015</v>
+        <v>1800</v>
       </c>
       <c r="C228" t="n">
         <v>8888</v>
       </c>
       <c r="D228" t="n">
-        <v>4436.15</v>
+        <v>430.37</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4777,17 +4777,17 @@
         <v>46218</v>
       </c>
       <c r="B229" t="n">
-        <v>559</v>
+        <v>1117</v>
       </c>
       <c r="C229" t="n">
         <v>8888</v>
       </c>
       <c r="D229" t="n">
-        <v>3838.57</v>
+        <v>672.47</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4796,17 +4796,17 @@
         <v>46218</v>
       </c>
       <c r="B230" t="n">
-        <v>1890</v>
+        <v>2749</v>
       </c>
       <c r="C230" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D230" t="n">
-        <v>1674.57</v>
+        <v>1860.64</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4815,17 +4815,17 @@
         <v>46218</v>
       </c>
       <c r="B231" t="n">
-        <v>1317</v>
+        <v>716</v>
       </c>
       <c r="C231" t="n">
-        <v>8888</v>
+        <v>15</v>
       </c>
       <c r="D231" t="n">
-        <v>1626.02</v>
+        <v>30000</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4834,13 +4834,13 @@
         <v>46218</v>
       </c>
       <c r="B232" t="n">
-        <v>2782</v>
+        <v>42</v>
       </c>
       <c r="C232" t="n">
         <v>8888</v>
       </c>
       <c r="D232" t="n">
-        <v>1786.32</v>
+        <v>280.05</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -4853,17 +4853,17 @@
         <v>46218</v>
       </c>
       <c r="B233" t="n">
-        <v>953</v>
+        <v>1478</v>
       </c>
       <c r="C233" t="n">
         <v>8888</v>
       </c>
       <c r="D233" t="n">
-        <v>364.44</v>
+        <v>875.34</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4872,13 +4872,13 @@
         <v>46218</v>
       </c>
       <c r="B234" t="n">
-        <v>2251</v>
+        <v>2491</v>
       </c>
       <c r="C234" t="n">
         <v>8888</v>
       </c>
       <c r="D234" t="n">
-        <v>989.26</v>
+        <v>650.4299999999999</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -4891,17 +4891,17 @@
         <v>46218</v>
       </c>
       <c r="B235" t="n">
-        <v>483</v>
+        <v>353</v>
       </c>
       <c r="C235" t="n">
-        <v>841</v>
+        <v>8888</v>
       </c>
       <c r="D235" t="n">
-        <v>2564.59</v>
+        <v>653.13</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4910,17 +4910,17 @@
         <v>46218</v>
       </c>
       <c r="B236" t="n">
-        <v>2133</v>
+        <v>2015</v>
       </c>
       <c r="C236" t="n">
-        <v>213</v>
+        <v>8888</v>
       </c>
       <c r="D236" t="n">
-        <v>526.8</v>
+        <v>4436.15</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4929,17 +4929,17 @@
         <v>46218</v>
       </c>
       <c r="B237" t="n">
-        <v>351</v>
+        <v>559</v>
       </c>
       <c r="C237" t="n">
-        <v>3009</v>
+        <v>8888</v>
       </c>
       <c r="D237" t="n">
-        <v>416.36</v>
+        <v>3838.57</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4948,17 +4948,17 @@
         <v>46218</v>
       </c>
       <c r="B238" t="n">
-        <v>2250</v>
+        <v>1890</v>
       </c>
       <c r="C238" t="n">
-        <v>8888</v>
+        <v>1953</v>
       </c>
       <c r="D238" t="n">
-        <v>709.46</v>
+        <v>2998.69</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4967,17 +4967,17 @@
         <v>46218</v>
       </c>
       <c r="B239" t="n">
-        <v>2648</v>
+        <v>1317</v>
       </c>
       <c r="C239" t="n">
         <v>8888</v>
       </c>
       <c r="D239" t="n">
-        <v>1873.52</v>
+        <v>1626.02</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4986,17 +4986,17 @@
         <v>46218</v>
       </c>
       <c r="B240" t="n">
-        <v>131</v>
+        <v>429</v>
       </c>
       <c r="C240" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D240" t="n">
-        <v>1369.91</v>
+        <v>1000.44</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -5005,17 +5005,17 @@
         <v>46218</v>
       </c>
       <c r="B241" t="n">
-        <v>2298</v>
+        <v>2782</v>
       </c>
       <c r="C241" t="n">
-        <v>675</v>
+        <v>8888</v>
       </c>
       <c r="D241" t="n">
-        <v>2301.31</v>
+        <v>1786.32</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5024,17 +5024,17 @@
         <v>46218</v>
       </c>
       <c r="B242" t="n">
-        <v>2790</v>
+        <v>953</v>
       </c>
       <c r="C242" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D242" t="n">
-        <v>371.88</v>
+        <v>364.44</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5043,17 +5043,17 @@
         <v>46218</v>
       </c>
       <c r="B243" t="n">
-        <v>363</v>
+        <v>2251</v>
       </c>
       <c r="C243" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D243" t="n">
-        <v>635.1</v>
+        <v>989.26</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5062,13 +5062,13 @@
         <v>46218</v>
       </c>
       <c r="B244" t="n">
-        <v>2716</v>
+        <v>483</v>
       </c>
       <c r="C244" t="n">
-        <v>1929</v>
+        <v>841</v>
       </c>
       <c r="D244" t="n">
-        <v>1073.33</v>
+        <v>2564.59</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -5081,13 +5081,13 @@
         <v>46218</v>
       </c>
       <c r="B245" t="n">
-        <v>2639</v>
+        <v>2133</v>
       </c>
       <c r="C245" t="n">
-        <v>1953</v>
+        <v>213</v>
       </c>
       <c r="D245" t="n">
-        <v>504.09</v>
+        <v>526.8</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -5100,13 +5100,13 @@
         <v>46218</v>
       </c>
       <c r="B246" t="n">
-        <v>629</v>
+        <v>351</v>
       </c>
       <c r="C246" t="n">
-        <v>675</v>
+        <v>3009</v>
       </c>
       <c r="D246" t="n">
-        <v>2419.73</v>
+        <v>416.36</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -5119,17 +5119,17 @@
         <v>46218</v>
       </c>
       <c r="B247" t="n">
-        <v>619</v>
+        <v>2250</v>
       </c>
       <c r="C247" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D247" t="n">
-        <v>1341.64</v>
+        <v>709.46</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -5138,13 +5138,13 @@
         <v>46218</v>
       </c>
       <c r="B248" t="n">
-        <v>2109</v>
+        <v>2648</v>
       </c>
       <c r="C248" t="n">
         <v>8888</v>
       </c>
       <c r="D248" t="n">
-        <v>2293.78</v>
+        <v>1873.52</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -5157,13 +5157,13 @@
         <v>46218</v>
       </c>
       <c r="B249" t="n">
-        <v>1116</v>
+        <v>131</v>
       </c>
       <c r="C249" t="n">
         <v>8888</v>
       </c>
       <c r="D249" t="n">
-        <v>2919.53</v>
+        <v>1369.91</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -5176,13 +5176,13 @@
         <v>46218</v>
       </c>
       <c r="B250" t="n">
-        <v>2250</v>
+        <v>2298</v>
       </c>
       <c r="C250" t="n">
-        <v>27</v>
+        <v>675</v>
       </c>
       <c r="D250" t="n">
-        <v>1803.76</v>
+        <v>2301.31</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -5195,13 +5195,13 @@
         <v>46218</v>
       </c>
       <c r="B251" t="n">
-        <v>2698</v>
+        <v>2790</v>
       </c>
       <c r="C251" t="n">
-        <v>874</v>
+        <v>1953</v>
       </c>
       <c r="D251" t="n">
-        <v>1230.43</v>
+        <v>371.88</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -5214,17 +5214,17 @@
         <v>46218</v>
       </c>
       <c r="B252" t="n">
-        <v>42</v>
+        <v>363</v>
       </c>
       <c r="C252" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D252" t="n">
-        <v>79947.14999999999</v>
+        <v>635.1</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -5233,17 +5233,17 @@
         <v>46218</v>
       </c>
       <c r="B253" t="n">
-        <v>772</v>
+        <v>2716</v>
       </c>
       <c r="C253" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D253" t="n">
-        <v>400.25</v>
+        <v>1073.33</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -5252,17 +5252,17 @@
         <v>46218</v>
       </c>
       <c r="B254" t="n">
-        <v>2728</v>
+        <v>2639</v>
       </c>
       <c r="C254" t="n">
-        <v>8888</v>
+        <v>1953</v>
       </c>
       <c r="D254" t="n">
-        <v>1397.07</v>
+        <v>504.09</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -5271,13 +5271,13 @@
         <v>46218</v>
       </c>
       <c r="B255" t="n">
-        <v>2197</v>
+        <v>629</v>
       </c>
       <c r="C255" t="n">
-        <v>423</v>
+        <v>675</v>
       </c>
       <c r="D255" t="n">
-        <v>2267.61</v>
+        <v>2419.73</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -5290,13 +5290,13 @@
         <v>46218</v>
       </c>
       <c r="B256" t="n">
-        <v>2716</v>
+        <v>619</v>
       </c>
       <c r="C256" t="n">
-        <v>977</v>
+        <v>1139</v>
       </c>
       <c r="D256" t="n">
-        <v>729.29</v>
+        <v>1341.64</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -5309,15 +5309,205 @@
         <v>46218</v>
       </c>
       <c r="B257" t="n">
+        <v>2109</v>
+      </c>
+      <c r="C257" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D257" t="n">
+        <v>2293.78</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B258" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C258" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D258" t="n">
+        <v>2919.53</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B259" t="n">
+        <v>1293</v>
+      </c>
+      <c r="C259" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D259" t="n">
+        <v>696.77</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B260" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C260" t="n">
+        <v>27</v>
+      </c>
+      <c r="D260" t="n">
+        <v>1803.76</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B261" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C261" t="n">
+        <v>874</v>
+      </c>
+      <c r="D261" t="n">
+        <v>1556.09</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B262" t="n">
+        <v>42</v>
+      </c>
+      <c r="C262" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D262" t="n">
+        <v>79947.14999999999</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B263" t="n">
+        <v>772</v>
+      </c>
+      <c r="C263" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D263" t="n">
+        <v>400.25</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B264" t="n">
+        <v>2728</v>
+      </c>
+      <c r="C264" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D264" t="n">
+        <v>1397.07</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B265" t="n">
+        <v>2197</v>
+      </c>
+      <c r="C265" t="n">
+        <v>423</v>
+      </c>
+      <c r="D265" t="n">
+        <v>2267.61</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B266" t="n">
+        <v>2716</v>
+      </c>
+      <c r="C266" t="n">
+        <v>977</v>
+      </c>
+      <c r="D266" t="n">
+        <v>729.29</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B267" t="n">
         <v>1993</v>
       </c>
-      <c r="C257" t="n">
-        <v>8888</v>
-      </c>
-      <c r="D257" t="n">
+      <c r="C267" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D267" t="n">
         <v>456.62</v>
       </c>
-      <c r="E257" t="inlineStr">
+      <c r="E267" t="inlineStr">
         <is>
           <t>OPERADOR LOGÍSTICO</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 18:30:04
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E267"/>
+  <dimension ref="A1:E279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,7 +489,7 @@
         <v>8888</v>
       </c>
       <c r="D3" t="n">
-        <v>769.05</v>
+        <v>814.6900000000001</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1072,17 +1072,17 @@
         <v>46218</v>
       </c>
       <c r="B34" t="n">
-        <v>2251</v>
+        <v>951</v>
       </c>
       <c r="C34" t="n">
         <v>8888</v>
       </c>
       <c r="D34" t="n">
-        <v>1010.74</v>
+        <v>2171.08</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1091,13 +1091,13 @@
         <v>46218</v>
       </c>
       <c r="B35" t="n">
-        <v>951</v>
+        <v>2641</v>
       </c>
       <c r="C35" t="n">
         <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>2171.08</v>
+        <v>2527.79</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1110,17 +1110,17 @@
         <v>46218</v>
       </c>
       <c r="B36" t="n">
-        <v>2641</v>
+        <v>2251</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>2527.79</v>
+        <v>1010.74</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1287,7 @@
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>1279.15</v>
+        <v>1404.58</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1458,7 +1458,7 @@
         <v>8888</v>
       </c>
       <c r="D54" t="n">
-        <v>30706.36</v>
+        <v>35695.37</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1528,17 +1528,17 @@
         <v>46218</v>
       </c>
       <c r="B58" t="n">
-        <v>664</v>
+        <v>2631</v>
       </c>
       <c r="C58" t="n">
-        <v>8888</v>
+        <v>2853</v>
       </c>
       <c r="D58" t="n">
-        <v>6275.01</v>
+        <v>3633.39</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1547,17 +1547,17 @@
         <v>46218</v>
       </c>
       <c r="B59" t="n">
-        <v>353</v>
+        <v>664</v>
       </c>
       <c r="C59" t="n">
-        <v>3179</v>
+        <v>8888</v>
       </c>
       <c r="D59" t="n">
-        <v>495.84</v>
+        <v>6275.01</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1566,17 +1566,17 @@
         <v>46218</v>
       </c>
       <c r="B60" t="n">
-        <v>1293</v>
+        <v>353</v>
       </c>
       <c r="C60" t="n">
-        <v>8888</v>
+        <v>3179</v>
       </c>
       <c r="D60" t="n">
-        <v>3129.07</v>
+        <v>495.84</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1585,13 +1585,13 @@
         <v>46218</v>
       </c>
       <c r="B61" t="n">
-        <v>2279</v>
+        <v>1293</v>
       </c>
       <c r="C61" t="n">
         <v>8888</v>
       </c>
       <c r="D61" t="n">
-        <v>3900.07</v>
+        <v>3129.07</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1604,13 +1604,13 @@
         <v>46218</v>
       </c>
       <c r="B62" t="n">
-        <v>1937</v>
+        <v>2279</v>
       </c>
       <c r="C62" t="n">
         <v>8888</v>
       </c>
       <c r="D62" t="n">
-        <v>1685.72</v>
+        <v>3900.07</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1623,17 +1623,17 @@
         <v>46218</v>
       </c>
       <c r="B63" t="n">
-        <v>941</v>
+        <v>1937</v>
       </c>
       <c r="C63" t="n">
         <v>8888</v>
       </c>
       <c r="D63" t="n">
-        <v>864.14</v>
+        <v>1685.72</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1642,17 +1642,17 @@
         <v>46218</v>
       </c>
       <c r="B64" t="n">
-        <v>1137</v>
+        <v>941</v>
       </c>
       <c r="C64" t="n">
         <v>8888</v>
       </c>
       <c r="D64" t="n">
-        <v>3168.9</v>
+        <v>864.14</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1661,17 +1661,17 @@
         <v>46218</v>
       </c>
       <c r="B65" t="n">
-        <v>2631</v>
+        <v>1137</v>
       </c>
       <c r="C65" t="n">
-        <v>2853</v>
+        <v>8888</v>
       </c>
       <c r="D65" t="n">
-        <v>2418.28</v>
+        <v>3168.9</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
         <v>8888</v>
       </c>
       <c r="D71" t="n">
-        <v>4416.47</v>
+        <v>4644.88</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -1889,13 +1889,13 @@
         <v>46218</v>
       </c>
       <c r="B77" t="n">
-        <v>483</v>
+        <v>1308</v>
       </c>
       <c r="C77" t="n">
         <v>8888</v>
       </c>
       <c r="D77" t="n">
-        <v>12405.46</v>
+        <v>2702.14</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -1908,17 +1908,17 @@
         <v>46218</v>
       </c>
       <c r="B78" t="n">
-        <v>1075</v>
+        <v>483</v>
       </c>
       <c r="C78" t="n">
         <v>8888</v>
       </c>
       <c r="D78" t="n">
-        <v>11607.79</v>
+        <v>12405.46</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1927,13 +1927,13 @@
         <v>46218</v>
       </c>
       <c r="B79" t="n">
-        <v>629</v>
+        <v>1075</v>
       </c>
       <c r="C79" t="n">
         <v>8888</v>
       </c>
       <c r="D79" t="n">
-        <v>9233.719999999999</v>
+        <v>11607.79</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -1946,17 +1946,17 @@
         <v>46218</v>
       </c>
       <c r="B80" t="n">
-        <v>1983</v>
+        <v>629</v>
       </c>
       <c r="C80" t="n">
-        <v>841</v>
+        <v>8888</v>
       </c>
       <c r="D80" t="n">
-        <v>633.79</v>
+        <v>13218.63</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -1965,17 +1965,17 @@
         <v>46218</v>
       </c>
       <c r="B81" t="n">
-        <v>1137</v>
+        <v>1983</v>
       </c>
       <c r="C81" t="n">
-        <v>8888</v>
+        <v>841</v>
       </c>
       <c r="D81" t="n">
-        <v>4842.54</v>
+        <v>633.79</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1984,17 +1984,17 @@
         <v>46218</v>
       </c>
       <c r="B82" t="n">
-        <v>2651</v>
+        <v>1137</v>
       </c>
       <c r="C82" t="n">
         <v>8888</v>
       </c>
       <c r="D82" t="n">
-        <v>1296.58</v>
+        <v>4842.54</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2003,17 +2003,17 @@
         <v>46218</v>
       </c>
       <c r="B83" t="n">
-        <v>2789</v>
+        <v>2651</v>
       </c>
       <c r="C83" t="n">
         <v>8888</v>
       </c>
       <c r="D83" t="n">
-        <v>1293.93</v>
+        <v>1296.58</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2022,17 +2022,17 @@
         <v>46218</v>
       </c>
       <c r="B84" t="n">
-        <v>1956</v>
+        <v>2789</v>
       </c>
       <c r="C84" t="n">
-        <v>423</v>
+        <v>8888</v>
       </c>
       <c r="D84" t="n">
-        <v>1416.35</v>
+        <v>1293.93</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2041,17 +2041,17 @@
         <v>46218</v>
       </c>
       <c r="B85" t="n">
-        <v>2709</v>
+        <v>1956</v>
       </c>
       <c r="C85" t="n">
-        <v>8888</v>
+        <v>423</v>
       </c>
       <c r="D85" t="n">
-        <v>547.6900000000001</v>
+        <v>1416.35</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2060,13 +2060,13 @@
         <v>46218</v>
       </c>
       <c r="B86" t="n">
-        <v>1308</v>
+        <v>2709</v>
       </c>
       <c r="C86" t="n">
         <v>8888</v>
       </c>
       <c r="D86" t="n">
-        <v>2264.86</v>
+        <v>547.6900000000001</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2383,13 +2383,13 @@
         <v>46218</v>
       </c>
       <c r="B103" t="n">
-        <v>2768</v>
+        <v>2402</v>
       </c>
       <c r="C103" t="n">
         <v>8888</v>
       </c>
       <c r="D103" t="n">
-        <v>7812.09</v>
+        <v>1998.28</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2402,13 +2402,13 @@
         <v>46218</v>
       </c>
       <c r="B104" t="n">
-        <v>1063</v>
+        <v>1906</v>
       </c>
       <c r="C104" t="n">
         <v>8888</v>
       </c>
       <c r="D104" t="n">
-        <v>4487.11</v>
+        <v>3504.37</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2421,17 +2421,17 @@
         <v>46218</v>
       </c>
       <c r="B105" t="n">
-        <v>947</v>
+        <v>2768</v>
       </c>
       <c r="C105" t="n">
         <v>8888</v>
       </c>
       <c r="D105" t="n">
-        <v>5667.85</v>
+        <v>7812.09</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>PEDIDO ELETRÔNICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2440,17 +2440,17 @@
         <v>46218</v>
       </c>
       <c r="B106" t="n">
-        <v>2279</v>
+        <v>1063</v>
       </c>
       <c r="C106" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D106" t="n">
-        <v>1031.06</v>
+        <v>4487.11</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2459,17 +2459,17 @@
         <v>46218</v>
       </c>
       <c r="B107" t="n">
-        <v>1299</v>
+        <v>947</v>
       </c>
       <c r="C107" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D107" t="n">
-        <v>1435.52</v>
+        <v>7409.08</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>PEDIDO ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -2478,13 +2478,13 @@
         <v>46218</v>
       </c>
       <c r="B108" t="n">
-        <v>1478</v>
+        <v>2279</v>
       </c>
       <c r="C108" t="n">
-        <v>675</v>
+        <v>1139</v>
       </c>
       <c r="D108" t="n">
-        <v>1967.85</v>
+        <v>1031.06</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -2497,17 +2497,17 @@
         <v>46218</v>
       </c>
       <c r="B109" t="n">
-        <v>675</v>
+        <v>1299</v>
       </c>
       <c r="C109" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D109" t="n">
-        <v>2685.73</v>
+        <v>1435.52</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2516,17 +2516,17 @@
         <v>46218</v>
       </c>
       <c r="B110" t="n">
-        <v>767</v>
+        <v>1478</v>
       </c>
       <c r="C110" t="n">
-        <v>8888</v>
+        <v>675</v>
       </c>
       <c r="D110" t="n">
-        <v>3292.44</v>
+        <v>1967.85</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2535,17 +2535,17 @@
         <v>46218</v>
       </c>
       <c r="B111" t="n">
-        <v>285</v>
+        <v>675</v>
       </c>
       <c r="C111" t="n">
         <v>8888</v>
       </c>
       <c r="D111" t="n">
-        <v>3349.8</v>
+        <v>2685.73</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2554,17 +2554,17 @@
         <v>46218</v>
       </c>
       <c r="B112" t="n">
-        <v>477</v>
+        <v>767</v>
       </c>
       <c r="C112" t="n">
         <v>8888</v>
       </c>
       <c r="D112" t="n">
-        <v>917.33</v>
+        <v>3292.44</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2573,17 +2573,17 @@
         <v>46218</v>
       </c>
       <c r="B113" t="n">
-        <v>1983</v>
+        <v>285</v>
       </c>
       <c r="C113" t="n">
         <v>8888</v>
       </c>
       <c r="D113" t="n">
-        <v>5115.01</v>
+        <v>3349.8</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2595,14 +2595,14 @@
         <v>477</v>
       </c>
       <c r="C114" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D114" t="n">
-        <v>3946.44</v>
+        <v>917.33</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2611,13 +2611,13 @@
         <v>46218</v>
       </c>
       <c r="B115" t="n">
-        <v>1937</v>
+        <v>1983</v>
       </c>
       <c r="C115" t="n">
         <v>8888</v>
       </c>
       <c r="D115" t="n">
-        <v>2600.61</v>
+        <v>5115.01</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -2630,17 +2630,17 @@
         <v>46218</v>
       </c>
       <c r="B116" t="n">
-        <v>363</v>
+        <v>477</v>
       </c>
       <c r="C116" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D116" t="n">
-        <v>780.35</v>
+        <v>3946.44</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2649,17 +2649,17 @@
         <v>46218</v>
       </c>
       <c r="B117" t="n">
-        <v>1063</v>
+        <v>1937</v>
       </c>
       <c r="C117" t="n">
         <v>8888</v>
       </c>
       <c r="D117" t="n">
-        <v>2549.86</v>
+        <v>2600.61</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2668,13 +2668,13 @@
         <v>46218</v>
       </c>
       <c r="B118" t="n">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="C118" t="n">
         <v>8888</v>
       </c>
       <c r="D118" t="n">
-        <v>5917.55</v>
+        <v>780.35</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -2687,17 +2687,17 @@
         <v>46218</v>
       </c>
       <c r="B119" t="n">
-        <v>2584</v>
+        <v>1063</v>
       </c>
       <c r="C119" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D119" t="n">
-        <v>756.16</v>
+        <v>4359.02</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2706,17 +2706,17 @@
         <v>46218</v>
       </c>
       <c r="B120" t="n">
-        <v>58</v>
+        <v>360</v>
       </c>
       <c r="C120" t="n">
         <v>8888</v>
       </c>
       <c r="D120" t="n">
-        <v>558.03</v>
+        <v>5917.55</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2725,17 +2725,17 @@
         <v>46218</v>
       </c>
       <c r="B121" t="n">
-        <v>424</v>
+        <v>2584</v>
       </c>
       <c r="C121" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D121" t="n">
-        <v>1362.42</v>
+        <v>756.16</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2744,17 +2744,17 @@
         <v>46218</v>
       </c>
       <c r="B122" t="n">
-        <v>663</v>
+        <v>58</v>
       </c>
       <c r="C122" t="n">
         <v>8888</v>
       </c>
       <c r="D122" t="n">
-        <v>255.13</v>
+        <v>558.03</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2763,17 +2763,17 @@
         <v>46218</v>
       </c>
       <c r="B123" t="n">
-        <v>1993</v>
+        <v>424</v>
       </c>
       <c r="C123" t="n">
         <v>8888</v>
       </c>
       <c r="D123" t="n">
-        <v>724.14</v>
+        <v>1362.42</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2782,17 +2782,17 @@
         <v>46218</v>
       </c>
       <c r="B124" t="n">
-        <v>1465</v>
+        <v>663</v>
       </c>
       <c r="C124" t="n">
         <v>8888</v>
       </c>
       <c r="D124" t="n">
-        <v>7362.56</v>
+        <v>255.13</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2801,13 +2801,13 @@
         <v>46218</v>
       </c>
       <c r="B125" t="n">
-        <v>89</v>
+        <v>1993</v>
       </c>
       <c r="C125" t="n">
         <v>8888</v>
       </c>
       <c r="D125" t="n">
-        <v>479</v>
+        <v>724.14</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -2820,13 +2820,13 @@
         <v>46218</v>
       </c>
       <c r="B126" t="n">
-        <v>595</v>
+        <v>1465</v>
       </c>
       <c r="C126" t="n">
         <v>8888</v>
       </c>
       <c r="D126" t="n">
-        <v>18084.5</v>
+        <v>7362.56</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -2839,17 +2839,17 @@
         <v>46218</v>
       </c>
       <c r="B127" t="n">
-        <v>2696</v>
+        <v>89</v>
       </c>
       <c r="C127" t="n">
-        <v>1954</v>
+        <v>8888</v>
       </c>
       <c r="D127" t="n">
-        <v>1597.76</v>
+        <v>479</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2858,17 +2858,17 @@
         <v>46218</v>
       </c>
       <c r="B128" t="n">
-        <v>1465</v>
+        <v>595</v>
       </c>
       <c r="C128" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D128" t="n">
-        <v>777.2</v>
+        <v>18084.5</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2877,17 +2877,17 @@
         <v>46218</v>
       </c>
       <c r="B129" t="n">
-        <v>2178</v>
+        <v>2696</v>
       </c>
       <c r="C129" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D129" t="n">
-        <v>619.92</v>
+        <v>1597.76</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2896,13 +2896,13 @@
         <v>46218</v>
       </c>
       <c r="B130" t="n">
-        <v>2026</v>
+        <v>1465</v>
       </c>
       <c r="C130" t="n">
-        <v>1929</v>
+        <v>3403</v>
       </c>
       <c r="D130" t="n">
-        <v>6021.92</v>
+        <v>777.2</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -2915,17 +2915,17 @@
         <v>46218</v>
       </c>
       <c r="B131" t="n">
-        <v>630</v>
+        <v>2178</v>
       </c>
       <c r="C131" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D131" t="n">
-        <v>1801.63</v>
+        <v>619.92</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -2934,17 +2934,17 @@
         <v>46218</v>
       </c>
       <c r="B132" t="n">
-        <v>1937</v>
+        <v>2026</v>
       </c>
       <c r="C132" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D132" t="n">
-        <v>2132.95</v>
+        <v>6021.92</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2953,17 +2953,17 @@
         <v>46218</v>
       </c>
       <c r="B133" t="n">
-        <v>2577</v>
+        <v>630</v>
       </c>
       <c r="C133" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D133" t="n">
-        <v>1647.08</v>
+        <v>1801.63</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2972,13 +2972,13 @@
         <v>46218</v>
       </c>
       <c r="B134" t="n">
-        <v>1293</v>
+        <v>1937</v>
       </c>
       <c r="C134" t="n">
         <v>8888</v>
       </c>
       <c r="D134" t="n">
-        <v>2135.89</v>
+        <v>2132.95</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -2991,13 +2991,13 @@
         <v>46218</v>
       </c>
       <c r="B135" t="n">
-        <v>2607</v>
+        <v>2577</v>
       </c>
       <c r="C135" t="n">
         <v>8888</v>
       </c>
       <c r="D135" t="n">
-        <v>490.31</v>
+        <v>1647.08</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3010,17 +3010,17 @@
         <v>46218</v>
       </c>
       <c r="B136" t="n">
-        <v>1317</v>
+        <v>1293</v>
       </c>
       <c r="C136" t="n">
         <v>8888</v>
       </c>
       <c r="D136" t="n">
-        <v>907.72</v>
+        <v>2135.89</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3029,13 +3029,13 @@
         <v>46218</v>
       </c>
       <c r="B137" t="n">
-        <v>535</v>
+        <v>2571</v>
       </c>
       <c r="C137" t="n">
-        <v>2571</v>
+        <v>1312</v>
       </c>
       <c r="D137" t="n">
-        <v>1124.46</v>
+        <v>1523.15</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3048,17 +3048,17 @@
         <v>46218</v>
       </c>
       <c r="B138" t="n">
-        <v>675</v>
+        <v>2607</v>
       </c>
       <c r="C138" t="n">
         <v>8888</v>
       </c>
       <c r="D138" t="n">
-        <v>337.89</v>
+        <v>490.31</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3067,17 +3067,17 @@
         <v>46218</v>
       </c>
       <c r="B139" t="n">
-        <v>2571</v>
+        <v>1317</v>
       </c>
       <c r="C139" t="n">
-        <v>1312</v>
+        <v>8888</v>
       </c>
       <c r="D139" t="n">
-        <v>743.01</v>
+        <v>907.72</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3086,17 +3086,17 @@
         <v>46218</v>
       </c>
       <c r="B140" t="n">
-        <v>619</v>
+        <v>535</v>
       </c>
       <c r="C140" t="n">
-        <v>8888</v>
+        <v>2571</v>
       </c>
       <c r="D140" t="n">
-        <v>1081.74</v>
+        <v>1124.46</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3105,13 +3105,13 @@
         <v>46218</v>
       </c>
       <c r="B141" t="n">
-        <v>20</v>
+        <v>2510</v>
       </c>
       <c r="C141" t="n">
         <v>8888</v>
       </c>
       <c r="D141" t="n">
-        <v>745.55</v>
+        <v>8587.950000000001</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3124,13 +3124,13 @@
         <v>46218</v>
       </c>
       <c r="B142" t="n">
-        <v>1063</v>
+        <v>675</v>
       </c>
       <c r="C142" t="n">
         <v>8888</v>
       </c>
       <c r="D142" t="n">
-        <v>1113.08</v>
+        <v>337.89</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3143,17 +3143,17 @@
         <v>46218</v>
       </c>
       <c r="B143" t="n">
-        <v>2631</v>
+        <v>619</v>
       </c>
       <c r="C143" t="n">
         <v>8888</v>
       </c>
       <c r="D143" t="n">
-        <v>1447.86</v>
+        <v>1081.74</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3162,13 +3162,13 @@
         <v>46218</v>
       </c>
       <c r="B144" t="n">
-        <v>1906</v>
+        <v>20</v>
       </c>
       <c r="C144" t="n">
         <v>8888</v>
       </c>
       <c r="D144" t="n">
-        <v>2774.84</v>
+        <v>745.55</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3181,17 +3181,17 @@
         <v>46218</v>
       </c>
       <c r="B145" t="n">
-        <v>1756</v>
+        <v>2118</v>
       </c>
       <c r="C145" t="n">
-        <v>8888</v>
+        <v>1954</v>
       </c>
       <c r="D145" t="n">
-        <v>2275.21</v>
+        <v>804.16</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3200,13 +3200,13 @@
         <v>46218</v>
       </c>
       <c r="B146" t="n">
-        <v>477</v>
+        <v>1063</v>
       </c>
       <c r="C146" t="n">
         <v>8888</v>
       </c>
       <c r="D146" t="n">
-        <v>707.52</v>
+        <v>1113.08</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3219,13 +3219,13 @@
         <v>46218</v>
       </c>
       <c r="B147" t="n">
-        <v>2660</v>
+        <v>2631</v>
       </c>
       <c r="C147" t="n">
         <v>8888</v>
       </c>
       <c r="D147" t="n">
-        <v>2684.97</v>
+        <v>1447.86</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -3238,17 +3238,17 @@
         <v>46218</v>
       </c>
       <c r="B148" t="n">
-        <v>569</v>
+        <v>1756</v>
       </c>
       <c r="C148" t="n">
         <v>8888</v>
       </c>
       <c r="D148" t="n">
-        <v>43745.83</v>
+        <v>2275.21</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3257,13 +3257,13 @@
         <v>46218</v>
       </c>
       <c r="B149" t="n">
-        <v>483</v>
+        <v>477</v>
       </c>
       <c r="C149" t="n">
         <v>8888</v>
       </c>
       <c r="D149" t="n">
-        <v>3102.48</v>
+        <v>707.52</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -3276,17 +3276,17 @@
         <v>46218</v>
       </c>
       <c r="B150" t="n">
-        <v>609</v>
+        <v>2660</v>
       </c>
       <c r="C150" t="n">
         <v>8888</v>
       </c>
       <c r="D150" t="n">
-        <v>1633.68</v>
+        <v>2684.97</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3295,13 +3295,13 @@
         <v>46218</v>
       </c>
       <c r="B151" t="n">
-        <v>483</v>
+        <v>569</v>
       </c>
       <c r="C151" t="n">
         <v>8888</v>
       </c>
       <c r="D151" t="n">
-        <v>2011.13</v>
+        <v>43745.83</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -3314,17 +3314,17 @@
         <v>46218</v>
       </c>
       <c r="B152" t="n">
-        <v>2089</v>
+        <v>483</v>
       </c>
       <c r="C152" t="n">
-        <v>1533</v>
+        <v>8888</v>
       </c>
       <c r="D152" t="n">
-        <v>1309.01</v>
+        <v>3102.48</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3333,17 +3333,17 @@
         <v>46218</v>
       </c>
       <c r="B153" t="n">
-        <v>1007</v>
+        <v>609</v>
       </c>
       <c r="C153" t="n">
         <v>8888</v>
       </c>
       <c r="D153" t="n">
-        <v>241.44</v>
+        <v>1633.68</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3352,17 +3352,17 @@
         <v>46218</v>
       </c>
       <c r="B154" t="n">
-        <v>1380</v>
+        <v>483</v>
       </c>
       <c r="C154" t="n">
         <v>8888</v>
       </c>
       <c r="D154" t="n">
-        <v>520.2</v>
+        <v>2011.13</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3371,17 +3371,17 @@
         <v>46218</v>
       </c>
       <c r="B155" t="n">
-        <v>1102</v>
+        <v>2089</v>
       </c>
       <c r="C155" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D155" t="n">
-        <v>1137.04</v>
+        <v>1309.01</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3390,17 +3390,17 @@
         <v>46218</v>
       </c>
       <c r="B156" t="n">
-        <v>358</v>
+        <v>1007</v>
       </c>
       <c r="C156" t="n">
         <v>8888</v>
       </c>
       <c r="D156" t="n">
-        <v>3380.3</v>
+        <v>241.44</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3409,13 +3409,13 @@
         <v>46218</v>
       </c>
       <c r="B157" t="n">
-        <v>1075</v>
+        <v>1380</v>
       </c>
       <c r="C157" t="n">
         <v>8888</v>
       </c>
       <c r="D157" t="n">
-        <v>5710.94</v>
+        <v>520.2</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -3428,17 +3428,17 @@
         <v>46218</v>
       </c>
       <c r="B158" t="n">
-        <v>2681</v>
+        <v>1102</v>
       </c>
       <c r="C158" t="n">
         <v>8888</v>
       </c>
       <c r="D158" t="n">
-        <v>729.25</v>
+        <v>1137.04</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3447,17 +3447,17 @@
         <v>46218</v>
       </c>
       <c r="B159" t="n">
-        <v>2245</v>
+        <v>358</v>
       </c>
       <c r="C159" t="n">
         <v>8888</v>
       </c>
       <c r="D159" t="n">
-        <v>700.2</v>
+        <v>3380.3</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3466,17 +3466,17 @@
         <v>46218</v>
       </c>
       <c r="B160" t="n">
-        <v>40</v>
+        <v>1075</v>
       </c>
       <c r="C160" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D160" t="n">
-        <v>678.21</v>
+        <v>5710.94</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3485,17 +3485,17 @@
         <v>46218</v>
       </c>
       <c r="B161" t="n">
-        <v>33</v>
+        <v>2681</v>
       </c>
       <c r="C161" t="n">
         <v>8888</v>
       </c>
       <c r="D161" t="n">
-        <v>926.97</v>
+        <v>729.25</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3504,17 +3504,17 @@
         <v>46218</v>
       </c>
       <c r="B162" t="n">
-        <v>132</v>
+        <v>2245</v>
       </c>
       <c r="C162" t="n">
         <v>8888</v>
       </c>
       <c r="D162" t="n">
-        <v>6522.92</v>
+        <v>700.2</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3523,17 +3523,17 @@
         <v>46218</v>
       </c>
       <c r="B163" t="n">
-        <v>619</v>
+        <v>40</v>
       </c>
       <c r="C163" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D163" t="n">
-        <v>2912.89</v>
+        <v>678.21</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3542,17 +3542,17 @@
         <v>46218</v>
       </c>
       <c r="B164" t="n">
-        <v>2769</v>
+        <v>33</v>
       </c>
       <c r="C164" t="n">
-        <v>977</v>
+        <v>8888</v>
       </c>
       <c r="D164" t="n">
-        <v>1116.56</v>
+        <v>926.97</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3561,17 +3561,17 @@
         <v>46218</v>
       </c>
       <c r="B165" t="n">
-        <v>452</v>
+        <v>2463</v>
       </c>
       <c r="C165" t="n">
         <v>8888</v>
       </c>
       <c r="D165" t="n">
-        <v>608.78</v>
+        <v>887.74</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3580,17 +3580,17 @@
         <v>46218</v>
       </c>
       <c r="B166" t="n">
-        <v>2463</v>
+        <v>132</v>
       </c>
       <c r="C166" t="n">
         <v>8888</v>
       </c>
       <c r="D166" t="n">
-        <v>363.69</v>
+        <v>6522.92</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3599,17 +3599,17 @@
         <v>46218</v>
       </c>
       <c r="B167" t="n">
-        <v>1293</v>
+        <v>619</v>
       </c>
       <c r="C167" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D167" t="n">
-        <v>1780.93</v>
+        <v>2912.89</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3618,17 +3618,17 @@
         <v>46218</v>
       </c>
       <c r="B168" t="n">
-        <v>525</v>
+        <v>2769</v>
       </c>
       <c r="C168" t="n">
-        <v>8888</v>
+        <v>977</v>
       </c>
       <c r="D168" t="n">
-        <v>5658.57</v>
+        <v>1116.56</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3637,17 +3637,17 @@
         <v>46218</v>
       </c>
       <c r="B169" t="n">
-        <v>2641</v>
+        <v>452</v>
       </c>
       <c r="C169" t="n">
         <v>8888</v>
       </c>
       <c r="D169" t="n">
-        <v>1720.99</v>
+        <v>608.78</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3656,13 +3656,13 @@
         <v>46218</v>
       </c>
       <c r="B170" t="n">
-        <v>675</v>
+        <v>1293</v>
       </c>
       <c r="C170" t="n">
-        <v>1898</v>
+        <v>1281</v>
       </c>
       <c r="D170" t="n">
-        <v>504.07</v>
+        <v>2292.86</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -3675,17 +3675,17 @@
         <v>46218</v>
       </c>
       <c r="B171" t="n">
-        <v>58</v>
+        <v>525</v>
       </c>
       <c r="C171" t="n">
         <v>8888</v>
       </c>
       <c r="D171" t="n">
-        <v>4929.8</v>
+        <v>5658.57</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3694,17 +3694,17 @@
         <v>46218</v>
       </c>
       <c r="B172" t="n">
-        <v>358</v>
+        <v>2641</v>
       </c>
       <c r="C172" t="n">
-        <v>546</v>
+        <v>8888</v>
       </c>
       <c r="D172" t="n">
-        <v>862.4400000000001</v>
+        <v>1720.99</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3713,13 +3713,13 @@
         <v>46218</v>
       </c>
       <c r="B173" t="n">
-        <v>325</v>
+        <v>675</v>
       </c>
       <c r="C173" t="n">
-        <v>1098</v>
+        <v>1898</v>
       </c>
       <c r="D173" t="n">
-        <v>50.06</v>
+        <v>504.07</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -3732,13 +3732,13 @@
         <v>46218</v>
       </c>
       <c r="B174" t="n">
-        <v>2697</v>
+        <v>58</v>
       </c>
       <c r="C174" t="n">
         <v>8888</v>
       </c>
       <c r="D174" t="n">
-        <v>833.38</v>
+        <v>4929.8</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -3751,13 +3751,13 @@
         <v>46218</v>
       </c>
       <c r="B175" t="n">
-        <v>2472</v>
+        <v>358</v>
       </c>
       <c r="C175" t="n">
-        <v>2853</v>
+        <v>546</v>
       </c>
       <c r="D175" t="n">
-        <v>1402.64</v>
+        <v>862.4400000000001</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -3770,13 +3770,13 @@
         <v>46218</v>
       </c>
       <c r="B176" t="n">
-        <v>2431</v>
+        <v>2606</v>
       </c>
       <c r="C176" t="n">
         <v>8888</v>
       </c>
       <c r="D176" t="n">
-        <v>266.89</v>
+        <v>2939.17</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -3789,17 +3789,17 @@
         <v>46218</v>
       </c>
       <c r="B177" t="n">
-        <v>285</v>
+        <v>325</v>
       </c>
       <c r="C177" t="n">
-        <v>8888</v>
+        <v>1098</v>
       </c>
       <c r="D177" t="n">
-        <v>5673.85</v>
+        <v>50.06</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3808,17 +3808,17 @@
         <v>46218</v>
       </c>
       <c r="B178" t="n">
-        <v>1102</v>
+        <v>2697</v>
       </c>
       <c r="C178" t="n">
         <v>8888</v>
       </c>
       <c r="D178" t="n">
-        <v>2301.43</v>
+        <v>833.38</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3827,17 +3827,17 @@
         <v>46218</v>
       </c>
       <c r="B179" t="n">
-        <v>2793</v>
+        <v>2472</v>
       </c>
       <c r="C179" t="n">
-        <v>8888</v>
+        <v>2853</v>
       </c>
       <c r="D179" t="n">
-        <v>1238.11</v>
+        <v>1402.64</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3846,17 +3846,17 @@
         <v>46218</v>
       </c>
       <c r="B180" t="n">
-        <v>626</v>
+        <v>2431</v>
       </c>
       <c r="C180" t="n">
         <v>8888</v>
       </c>
       <c r="D180" t="n">
-        <v>23157.24</v>
+        <v>266.89</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3865,13 +3865,13 @@
         <v>46218</v>
       </c>
       <c r="B181" t="n">
-        <v>424</v>
+        <v>285</v>
       </c>
       <c r="C181" t="n">
         <v>8888</v>
       </c>
       <c r="D181" t="n">
-        <v>1124.8</v>
+        <v>5673.85</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -3884,17 +3884,17 @@
         <v>46218</v>
       </c>
       <c r="B182" t="n">
-        <v>1137</v>
+        <v>1102</v>
       </c>
       <c r="C182" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D182" t="n">
-        <v>3285.55</v>
+        <v>2301.43</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3903,17 +3903,17 @@
         <v>46218</v>
       </c>
       <c r="B183" t="n">
-        <v>1299</v>
+        <v>2793</v>
       </c>
       <c r="C183" t="n">
-        <v>2522</v>
+        <v>8888</v>
       </c>
       <c r="D183" t="n">
-        <v>8881.309999999999</v>
+        <v>1238.11</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3922,17 +3922,17 @@
         <v>46218</v>
       </c>
       <c r="B184" t="n">
-        <v>1289</v>
+        <v>626</v>
       </c>
       <c r="C184" t="n">
         <v>8888</v>
       </c>
       <c r="D184" t="n">
-        <v>5565.44</v>
+        <v>23157.24</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -3941,17 +3941,17 @@
         <v>46218</v>
       </c>
       <c r="B185" t="n">
-        <v>2686</v>
+        <v>424</v>
       </c>
       <c r="C185" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D185" t="n">
-        <v>2066.36</v>
+        <v>1124.8</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3960,17 +3960,17 @@
         <v>46218</v>
       </c>
       <c r="B186" t="n">
-        <v>629</v>
+        <v>1137</v>
       </c>
       <c r="C186" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D186" t="n">
-        <v>5212.76</v>
+        <v>3285.55</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3979,17 +3979,17 @@
         <v>46218</v>
       </c>
       <c r="B187" t="n">
-        <v>636</v>
+        <v>1299</v>
       </c>
       <c r="C187" t="n">
-        <v>8888</v>
+        <v>2522</v>
       </c>
       <c r="D187" t="n">
-        <v>5742.49</v>
+        <v>8881.309999999999</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3998,17 +3998,17 @@
         <v>46218</v>
       </c>
       <c r="B188" t="n">
-        <v>2584</v>
+        <v>1289</v>
       </c>
       <c r="C188" t="n">
         <v>8888</v>
       </c>
       <c r="D188" t="n">
-        <v>5635.67</v>
+        <v>5565.44</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4017,17 +4017,17 @@
         <v>46218</v>
       </c>
       <c r="B189" t="n">
-        <v>1756</v>
+        <v>2686</v>
       </c>
       <c r="C189" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D189" t="n">
-        <v>3242.54</v>
+        <v>2066.36</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4036,13 +4036,13 @@
         <v>46218</v>
       </c>
       <c r="B190" t="n">
-        <v>2698</v>
+        <v>629</v>
       </c>
       <c r="C190" t="n">
         <v>8888</v>
       </c>
       <c r="D190" t="n">
-        <v>859.49</v>
+        <v>5212.76</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -4055,17 +4055,17 @@
         <v>46218</v>
       </c>
       <c r="B191" t="n">
-        <v>1756</v>
+        <v>636</v>
       </c>
       <c r="C191" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D191" t="n">
-        <v>5078.1</v>
+        <v>5742.49</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4074,17 +4074,17 @@
         <v>46218</v>
       </c>
       <c r="B192" t="n">
-        <v>2651</v>
+        <v>2584</v>
       </c>
       <c r="C192" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D192" t="n">
-        <v>363.7</v>
+        <v>5635.67</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4093,13 +4093,13 @@
         <v>46218</v>
       </c>
       <c r="B193" t="n">
-        <v>664</v>
+        <v>1756</v>
       </c>
       <c r="C193" t="n">
         <v>8888</v>
       </c>
       <c r="D193" t="n">
-        <v>6478.17</v>
+        <v>3242.54</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -4112,17 +4112,17 @@
         <v>46218</v>
       </c>
       <c r="B194" t="n">
-        <v>360</v>
+        <v>2698</v>
       </c>
       <c r="C194" t="n">
         <v>8888</v>
       </c>
       <c r="D194" t="n">
-        <v>1594.84</v>
+        <v>859.49</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4131,17 +4131,17 @@
         <v>46218</v>
       </c>
       <c r="B195" t="n">
-        <v>2582</v>
+        <v>1756</v>
       </c>
       <c r="C195" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D195" t="n">
-        <v>379.33</v>
+        <v>5078.1</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4150,17 +4150,17 @@
         <v>46218</v>
       </c>
       <c r="B196" t="n">
-        <v>1254</v>
+        <v>2651</v>
       </c>
       <c r="C196" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D196" t="n">
-        <v>2643.22</v>
+        <v>363.7</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4169,17 +4169,17 @@
         <v>46218</v>
       </c>
       <c r="B197" t="n">
-        <v>2726</v>
+        <v>664</v>
       </c>
       <c r="C197" t="n">
-        <v>977</v>
+        <v>8888</v>
       </c>
       <c r="D197" t="n">
-        <v>586.0599999999999</v>
+        <v>6478.17</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4188,17 +4188,17 @@
         <v>46218</v>
       </c>
       <c r="B198" t="n">
-        <v>2015</v>
+        <v>360</v>
       </c>
       <c r="C198" t="n">
         <v>8888</v>
       </c>
       <c r="D198" t="n">
-        <v>315.69</v>
+        <v>1594.84</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4207,17 +4207,17 @@
         <v>46218</v>
       </c>
       <c r="B199" t="n">
-        <v>1064</v>
+        <v>2582</v>
       </c>
       <c r="C199" t="n">
         <v>8888</v>
       </c>
       <c r="D199" t="n">
-        <v>1274.3</v>
+        <v>379.33</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4226,17 +4226,17 @@
         <v>46218</v>
       </c>
       <c r="B200" t="n">
-        <v>358</v>
+        <v>2698</v>
       </c>
       <c r="C200" t="n">
-        <v>8888</v>
+        <v>1312</v>
       </c>
       <c r="D200" t="n">
-        <v>2619.4</v>
+        <v>440.3</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4245,17 +4245,17 @@
         <v>46218</v>
       </c>
       <c r="B201" t="n">
-        <v>2641</v>
+        <v>1254</v>
       </c>
       <c r="C201" t="n">
         <v>8888</v>
       </c>
       <c r="D201" t="n">
-        <v>820</v>
+        <v>2643.22</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4264,17 +4264,17 @@
         <v>46218</v>
       </c>
       <c r="B202" t="n">
-        <v>429</v>
+        <v>2726</v>
       </c>
       <c r="C202" t="n">
-        <v>8888</v>
+        <v>977</v>
       </c>
       <c r="D202" t="n">
-        <v>2593.49</v>
+        <v>586.0599999999999</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4283,17 +4283,17 @@
         <v>46218</v>
       </c>
       <c r="B203" t="n">
-        <v>1301</v>
+        <v>2015</v>
       </c>
       <c r="C203" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D203" t="n">
-        <v>750.66</v>
+        <v>315.69</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4302,13 +4302,13 @@
         <v>46218</v>
       </c>
       <c r="B204" t="n">
-        <v>816</v>
+        <v>1064</v>
       </c>
       <c r="C204" t="n">
         <v>8888</v>
       </c>
       <c r="D204" t="n">
-        <v>438.24</v>
+        <v>1274.3</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -4321,13 +4321,13 @@
         <v>46218</v>
       </c>
       <c r="B205" t="n">
-        <v>2359</v>
+        <v>358</v>
       </c>
       <c r="C205" t="n">
         <v>8888</v>
       </c>
       <c r="D205" t="n">
-        <v>381.95</v>
+        <v>4129.47</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -4340,17 +4340,17 @@
         <v>46218</v>
       </c>
       <c r="B206" t="n">
-        <v>2251</v>
+        <v>2641</v>
       </c>
       <c r="C206" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D206" t="n">
-        <v>802.08</v>
+        <v>820</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4359,17 +4359,17 @@
         <v>46218</v>
       </c>
       <c r="B207" t="n">
-        <v>285</v>
+        <v>429</v>
       </c>
       <c r="C207" t="n">
-        <v>58</v>
+        <v>8888</v>
       </c>
       <c r="D207" t="n">
-        <v>1797.95</v>
+        <v>2593.49</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4378,17 +4378,17 @@
         <v>46218</v>
       </c>
       <c r="B208" t="n">
-        <v>2114</v>
+        <v>1301</v>
       </c>
       <c r="C208" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D208" t="n">
-        <v>2726.04</v>
+        <v>750.66</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4397,17 +4397,17 @@
         <v>46218</v>
       </c>
       <c r="B209" t="n">
-        <v>953</v>
+        <v>816</v>
       </c>
       <c r="C209" t="n">
         <v>8888</v>
       </c>
       <c r="D209" t="n">
-        <v>2889.63</v>
+        <v>438.24</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4416,17 +4416,17 @@
         <v>46218</v>
       </c>
       <c r="B210" t="n">
-        <v>1102</v>
+        <v>2249</v>
       </c>
       <c r="C210" t="n">
         <v>8888</v>
       </c>
       <c r="D210" t="n">
-        <v>6347.79</v>
+        <v>3047.57</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4435,17 +4435,17 @@
         <v>46218</v>
       </c>
       <c r="B211" t="n">
-        <v>1465</v>
+        <v>2359</v>
       </c>
       <c r="C211" t="n">
         <v>8888</v>
       </c>
       <c r="D211" t="n">
-        <v>4281.39</v>
+        <v>381.95</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4454,17 +4454,17 @@
         <v>46218</v>
       </c>
       <c r="B212" t="n">
-        <v>619</v>
+        <v>2251</v>
       </c>
       <c r="C212" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D212" t="n">
-        <v>2021.67</v>
+        <v>802.08</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4473,17 +4473,17 @@
         <v>46218</v>
       </c>
       <c r="B213" t="n">
-        <v>2716</v>
+        <v>285</v>
       </c>
       <c r="C213" t="n">
-        <v>8888</v>
+        <v>58</v>
       </c>
       <c r="D213" t="n">
-        <v>1063.42</v>
+        <v>1797.95</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4492,17 +4492,17 @@
         <v>46218</v>
       </c>
       <c r="B214" t="n">
-        <v>2767</v>
+        <v>2114</v>
       </c>
       <c r="C214" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D214" t="n">
-        <v>1135.64</v>
+        <v>2726.04</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4511,17 +4511,17 @@
         <v>46218</v>
       </c>
       <c r="B215" t="n">
-        <v>2657</v>
+        <v>1137</v>
       </c>
       <c r="C215" t="n">
-        <v>8888</v>
+        <v>874</v>
       </c>
       <c r="D215" t="n">
-        <v>3149.7</v>
+        <v>444.86</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4530,17 +4530,17 @@
         <v>46218</v>
       </c>
       <c r="B216" t="n">
-        <v>2245</v>
+        <v>953</v>
       </c>
       <c r="C216" t="n">
         <v>8888</v>
       </c>
       <c r="D216" t="n">
-        <v>764.66</v>
+        <v>2889.63</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4549,17 +4549,17 @@
         <v>46218</v>
       </c>
       <c r="B217" t="n">
-        <v>2197</v>
+        <v>1102</v>
       </c>
       <c r="C217" t="n">
         <v>8888</v>
       </c>
       <c r="D217" t="n">
-        <v>1085.45</v>
+        <v>6347.79</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4568,17 +4568,17 @@
         <v>46218</v>
       </c>
       <c r="B218" t="n">
-        <v>1064</v>
+        <v>1465</v>
       </c>
       <c r="C218" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D218" t="n">
-        <v>574.7</v>
+        <v>4281.39</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4587,17 +4587,17 @@
         <v>46218</v>
       </c>
       <c r="B219" t="n">
-        <v>451</v>
+        <v>619</v>
       </c>
       <c r="C219" t="n">
-        <v>3403</v>
+        <v>8888</v>
       </c>
       <c r="D219" t="n">
-        <v>2091.77</v>
+        <v>2021.67</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4606,17 +4606,17 @@
         <v>46218</v>
       </c>
       <c r="B220" t="n">
-        <v>1116</v>
+        <v>2716</v>
       </c>
       <c r="C220" t="n">
-        <v>13148</v>
+        <v>8888</v>
       </c>
       <c r="D220" t="n">
-        <v>1455.21</v>
+        <v>1063.42</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4625,17 +4625,17 @@
         <v>46218</v>
       </c>
       <c r="B221" t="n">
-        <v>1277</v>
+        <v>2767</v>
       </c>
       <c r="C221" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D221" t="n">
-        <v>1949</v>
+        <v>1135.64</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4644,17 +4644,17 @@
         <v>46218</v>
       </c>
       <c r="B222" t="n">
-        <v>131</v>
+        <v>2657</v>
       </c>
       <c r="C222" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D222" t="n">
-        <v>3850.09</v>
+        <v>3149.7</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4663,17 +4663,17 @@
         <v>46218</v>
       </c>
       <c r="B223" t="n">
-        <v>2692</v>
+        <v>2245</v>
       </c>
       <c r="C223" t="n">
         <v>8888</v>
       </c>
       <c r="D223" t="n">
-        <v>731.28</v>
+        <v>764.66</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4682,17 +4682,17 @@
         <v>46218</v>
       </c>
       <c r="B224" t="n">
-        <v>1632</v>
+        <v>2197</v>
       </c>
       <c r="C224" t="n">
         <v>8888</v>
       </c>
       <c r="D224" t="n">
-        <v>7519.7</v>
+        <v>1085.45</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4701,13 +4701,13 @@
         <v>46218</v>
       </c>
       <c r="B225" t="n">
-        <v>1317</v>
+        <v>1064</v>
       </c>
       <c r="C225" t="n">
-        <v>3179</v>
+        <v>27</v>
       </c>
       <c r="D225" t="n">
-        <v>991.6799999999999</v>
+        <v>574.7</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -4720,17 +4720,17 @@
         <v>46218</v>
       </c>
       <c r="B226" t="n">
-        <v>1993</v>
+        <v>451</v>
       </c>
       <c r="C226" t="n">
-        <v>8888</v>
+        <v>3403</v>
       </c>
       <c r="D226" t="n">
-        <v>3508.59</v>
+        <v>2443.16</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4739,13 +4739,13 @@
         <v>46218</v>
       </c>
       <c r="B227" t="n">
-        <v>1890</v>
+        <v>1116</v>
       </c>
       <c r="C227" t="n">
-        <v>3449</v>
+        <v>13148</v>
       </c>
       <c r="D227" t="n">
-        <v>6313.56</v>
+        <v>1455.21</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -4758,17 +4758,17 @@
         <v>46218</v>
       </c>
       <c r="B228" t="n">
-        <v>1800</v>
+        <v>1277</v>
       </c>
       <c r="C228" t="n">
         <v>8888</v>
       </c>
       <c r="D228" t="n">
-        <v>430.37</v>
+        <v>1949</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4777,17 +4777,17 @@
         <v>46218</v>
       </c>
       <c r="B229" t="n">
-        <v>1117</v>
+        <v>131</v>
       </c>
       <c r="C229" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D229" t="n">
-        <v>672.47</v>
+        <v>3850.09</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4796,13 +4796,13 @@
         <v>46218</v>
       </c>
       <c r="B230" t="n">
-        <v>2749</v>
+        <v>2692</v>
       </c>
       <c r="C230" t="n">
         <v>8888</v>
       </c>
       <c r="D230" t="n">
-        <v>1860.64</v>
+        <v>731.28</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -4815,17 +4815,17 @@
         <v>46218</v>
       </c>
       <c r="B231" t="n">
-        <v>716</v>
+        <v>1632</v>
       </c>
       <c r="C231" t="n">
-        <v>15</v>
+        <v>8888</v>
       </c>
       <c r="D231" t="n">
-        <v>30000</v>
+        <v>7519.7</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4834,17 +4834,17 @@
         <v>46218</v>
       </c>
       <c r="B232" t="n">
-        <v>42</v>
+        <v>2015</v>
       </c>
       <c r="C232" t="n">
         <v>8888</v>
       </c>
       <c r="D232" t="n">
-        <v>280.05</v>
+        <v>377.84</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4853,17 +4853,17 @@
         <v>46218</v>
       </c>
       <c r="B233" t="n">
-        <v>1478</v>
+        <v>42</v>
       </c>
       <c r="C233" t="n">
         <v>8888</v>
       </c>
       <c r="D233" t="n">
-        <v>875.34</v>
+        <v>371.51</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4872,17 +4872,17 @@
         <v>46218</v>
       </c>
       <c r="B234" t="n">
-        <v>2491</v>
+        <v>1317</v>
       </c>
       <c r="C234" t="n">
-        <v>8888</v>
+        <v>3179</v>
       </c>
       <c r="D234" t="n">
-        <v>650.4299999999999</v>
+        <v>991.6799999999999</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4891,13 +4891,13 @@
         <v>46218</v>
       </c>
       <c r="B235" t="n">
-        <v>353</v>
+        <v>1993</v>
       </c>
       <c r="C235" t="n">
         <v>8888</v>
       </c>
       <c r="D235" t="n">
-        <v>653.13</v>
+        <v>3508.59</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -4910,17 +4910,17 @@
         <v>46218</v>
       </c>
       <c r="B236" t="n">
-        <v>2015</v>
+        <v>2606</v>
       </c>
       <c r="C236" t="n">
-        <v>8888</v>
+        <v>2727</v>
       </c>
       <c r="D236" t="n">
-        <v>4436.15</v>
+        <v>1282.92</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4929,17 +4929,17 @@
         <v>46218</v>
       </c>
       <c r="B237" t="n">
-        <v>559</v>
+        <v>1890</v>
       </c>
       <c r="C237" t="n">
-        <v>8888</v>
+        <v>3449</v>
       </c>
       <c r="D237" t="n">
-        <v>3838.57</v>
+        <v>6313.56</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4948,17 +4948,17 @@
         <v>46218</v>
       </c>
       <c r="B238" t="n">
-        <v>1890</v>
+        <v>1800</v>
       </c>
       <c r="C238" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D238" t="n">
-        <v>2998.69</v>
+        <v>430.37</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -4967,17 +4967,17 @@
         <v>46218</v>
       </c>
       <c r="B239" t="n">
-        <v>1317</v>
+        <v>1117</v>
       </c>
       <c r="C239" t="n">
         <v>8888</v>
       </c>
       <c r="D239" t="n">
-        <v>1626.02</v>
+        <v>672.47</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4986,17 +4986,17 @@
         <v>46218</v>
       </c>
       <c r="B240" t="n">
-        <v>429</v>
+        <v>2749</v>
       </c>
       <c r="C240" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D240" t="n">
-        <v>1000.44</v>
+        <v>1860.64</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -5005,17 +5005,17 @@
         <v>46218</v>
       </c>
       <c r="B241" t="n">
-        <v>2782</v>
+        <v>716</v>
       </c>
       <c r="C241" t="n">
-        <v>8888</v>
+        <v>15</v>
       </c>
       <c r="D241" t="n">
-        <v>1786.32</v>
+        <v>30000</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -5024,13 +5024,13 @@
         <v>46218</v>
       </c>
       <c r="B242" t="n">
-        <v>953</v>
+        <v>42</v>
       </c>
       <c r="C242" t="n">
         <v>8888</v>
       </c>
       <c r="D242" t="n">
-        <v>364.44</v>
+        <v>280.05</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -5043,17 +5043,17 @@
         <v>46218</v>
       </c>
       <c r="B243" t="n">
-        <v>2251</v>
+        <v>1478</v>
       </c>
       <c r="C243" t="n">
         <v>8888</v>
       </c>
       <c r="D243" t="n">
-        <v>989.26</v>
+        <v>875.34</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -5062,17 +5062,17 @@
         <v>46218</v>
       </c>
       <c r="B244" t="n">
-        <v>483</v>
+        <v>2491</v>
       </c>
       <c r="C244" t="n">
-        <v>841</v>
+        <v>8888</v>
       </c>
       <c r="D244" t="n">
-        <v>2564.59</v>
+        <v>1690.31</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5081,17 +5081,17 @@
         <v>46218</v>
       </c>
       <c r="B245" t="n">
-        <v>2133</v>
+        <v>353</v>
       </c>
       <c r="C245" t="n">
-        <v>213</v>
+        <v>8888</v>
       </c>
       <c r="D245" t="n">
-        <v>526.8</v>
+        <v>653.13</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5100,17 +5100,17 @@
         <v>46218</v>
       </c>
       <c r="B246" t="n">
-        <v>351</v>
+        <v>2015</v>
       </c>
       <c r="C246" t="n">
-        <v>3009</v>
+        <v>8888</v>
       </c>
       <c r="D246" t="n">
-        <v>416.36</v>
+        <v>4436.15</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5119,17 +5119,17 @@
         <v>46218</v>
       </c>
       <c r="B247" t="n">
-        <v>2250</v>
+        <v>559</v>
       </c>
       <c r="C247" t="n">
         <v>8888</v>
       </c>
       <c r="D247" t="n">
-        <v>709.46</v>
+        <v>3838.57</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5138,17 +5138,17 @@
         <v>46218</v>
       </c>
       <c r="B248" t="n">
-        <v>2648</v>
+        <v>1890</v>
       </c>
       <c r="C248" t="n">
-        <v>8888</v>
+        <v>1953</v>
       </c>
       <c r="D248" t="n">
-        <v>1873.52</v>
+        <v>2998.69</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -5157,13 +5157,13 @@
         <v>46218</v>
       </c>
       <c r="B249" t="n">
-        <v>131</v>
+        <v>1317</v>
       </c>
       <c r="C249" t="n">
         <v>8888</v>
       </c>
       <c r="D249" t="n">
-        <v>1369.91</v>
+        <v>1626.02</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -5176,13 +5176,13 @@
         <v>46218</v>
       </c>
       <c r="B250" t="n">
-        <v>2298</v>
+        <v>429</v>
       </c>
       <c r="C250" t="n">
-        <v>675</v>
+        <v>1281</v>
       </c>
       <c r="D250" t="n">
-        <v>2301.31</v>
+        <v>1000.44</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -5195,17 +5195,17 @@
         <v>46218</v>
       </c>
       <c r="B251" t="n">
-        <v>2790</v>
+        <v>2782</v>
       </c>
       <c r="C251" t="n">
-        <v>1953</v>
+        <v>8888</v>
       </c>
       <c r="D251" t="n">
-        <v>371.88</v>
+        <v>1786.32</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5214,17 +5214,17 @@
         <v>46218</v>
       </c>
       <c r="B252" t="n">
-        <v>363</v>
+        <v>953</v>
       </c>
       <c r="C252" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D252" t="n">
-        <v>635.1</v>
+        <v>364.44</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5233,17 +5233,17 @@
         <v>46218</v>
       </c>
       <c r="B253" t="n">
-        <v>2716</v>
+        <v>2251</v>
       </c>
       <c r="C253" t="n">
-        <v>1929</v>
+        <v>8888</v>
       </c>
       <c r="D253" t="n">
-        <v>1073.33</v>
+        <v>989.26</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5252,13 +5252,13 @@
         <v>46218</v>
       </c>
       <c r="B254" t="n">
-        <v>2639</v>
+        <v>483</v>
       </c>
       <c r="C254" t="n">
-        <v>1953</v>
+        <v>841</v>
       </c>
       <c r="D254" t="n">
-        <v>504.09</v>
+        <v>2564.59</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -5271,13 +5271,13 @@
         <v>46218</v>
       </c>
       <c r="B255" t="n">
-        <v>629</v>
+        <v>2133</v>
       </c>
       <c r="C255" t="n">
-        <v>675</v>
+        <v>213</v>
       </c>
       <c r="D255" t="n">
-        <v>2419.73</v>
+        <v>526.8</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -5290,13 +5290,13 @@
         <v>46218</v>
       </c>
       <c r="B256" t="n">
-        <v>619</v>
+        <v>351</v>
       </c>
       <c r="C256" t="n">
-        <v>1139</v>
+        <v>3009</v>
       </c>
       <c r="D256" t="n">
-        <v>1341.64</v>
+        <v>416.36</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -5309,17 +5309,17 @@
         <v>46218</v>
       </c>
       <c r="B257" t="n">
-        <v>2109</v>
+        <v>2250</v>
       </c>
       <c r="C257" t="n">
         <v>8888</v>
       </c>
       <c r="D257" t="n">
-        <v>2293.78</v>
+        <v>709.46</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -5328,17 +5328,17 @@
         <v>46218</v>
       </c>
       <c r="B258" t="n">
-        <v>1116</v>
+        <v>2141</v>
       </c>
       <c r="C258" t="n">
         <v>8888</v>
       </c>
       <c r="D258" t="n">
-        <v>2919.53</v>
+        <v>1453.86</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5347,17 +5347,17 @@
         <v>46218</v>
       </c>
       <c r="B259" t="n">
-        <v>1293</v>
+        <v>2648</v>
       </c>
       <c r="C259" t="n">
         <v>8888</v>
       </c>
       <c r="D259" t="n">
-        <v>696.77</v>
+        <v>1873.52</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5366,17 +5366,17 @@
         <v>46218</v>
       </c>
       <c r="B260" t="n">
-        <v>2250</v>
+        <v>131</v>
       </c>
       <c r="C260" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D260" t="n">
-        <v>1803.76</v>
+        <v>1369.91</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>OPERADOR LOGÍSTICO</t>
         </is>
       </c>
     </row>
@@ -5385,13 +5385,13 @@
         <v>46218</v>
       </c>
       <c r="B261" t="n">
-        <v>2698</v>
+        <v>2298</v>
       </c>
       <c r="C261" t="n">
-        <v>874</v>
+        <v>675</v>
       </c>
       <c r="D261" t="n">
-        <v>1556.09</v>
+        <v>2301.31</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -5404,17 +5404,17 @@
         <v>46218</v>
       </c>
       <c r="B262" t="n">
-        <v>42</v>
+        <v>2790</v>
       </c>
       <c r="C262" t="n">
-        <v>8888</v>
+        <v>1953</v>
       </c>
       <c r="D262" t="n">
-        <v>79947.14999999999</v>
+        <v>371.88</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>OPERADOR LOGÍSTICO</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -5423,17 +5423,17 @@
         <v>46218</v>
       </c>
       <c r="B263" t="n">
-        <v>772</v>
+        <v>363</v>
       </c>
       <c r="C263" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D263" t="n">
-        <v>400.25</v>
+        <v>635.1</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -5442,17 +5442,17 @@
         <v>46218</v>
       </c>
       <c r="B264" t="n">
-        <v>2728</v>
+        <v>2716</v>
       </c>
       <c r="C264" t="n">
-        <v>8888</v>
+        <v>1929</v>
       </c>
       <c r="D264" t="n">
-        <v>1397.07</v>
+        <v>1073.33</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -5461,13 +5461,13 @@
         <v>46218</v>
       </c>
       <c r="B265" t="n">
-        <v>2197</v>
+        <v>2639</v>
       </c>
       <c r="C265" t="n">
-        <v>423</v>
+        <v>1953</v>
       </c>
       <c r="D265" t="n">
-        <v>2267.61</v>
+        <v>504.09</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -5480,13 +5480,13 @@
         <v>46218</v>
       </c>
       <c r="B266" t="n">
-        <v>2716</v>
+        <v>629</v>
       </c>
       <c r="C266" t="n">
-        <v>977</v>
+        <v>675</v>
       </c>
       <c r="D266" t="n">
-        <v>729.29</v>
+        <v>2419.73</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -5499,17 +5499,245 @@
         <v>46218</v>
       </c>
       <c r="B267" t="n">
+        <v>619</v>
+      </c>
+      <c r="C267" t="n">
+        <v>1139</v>
+      </c>
+      <c r="D267" t="n">
+        <v>1341.64</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B268" t="n">
+        <v>2109</v>
+      </c>
+      <c r="C268" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D268" t="n">
+        <v>2293.78</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B269" t="n">
+        <v>1116</v>
+      </c>
+      <c r="C269" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D269" t="n">
+        <v>2919.53</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B270" t="n">
+        <v>1293</v>
+      </c>
+      <c r="C270" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D270" t="n">
+        <v>696.77</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B271" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C271" t="n">
+        <v>27</v>
+      </c>
+      <c r="D271" t="n">
+        <v>1803.76</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B272" t="n">
+        <v>2698</v>
+      </c>
+      <c r="C272" t="n">
+        <v>874</v>
+      </c>
+      <c r="D272" t="n">
+        <v>1556.09</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B273" t="n">
+        <v>42</v>
+      </c>
+      <c r="C273" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D273" t="n">
+        <v>79947.14999999999</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B274" t="n">
+        <v>772</v>
+      </c>
+      <c r="C274" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D274" t="n">
+        <v>400.25</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B275" t="n">
+        <v>2728</v>
+      </c>
+      <c r="C275" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D275" t="n">
+        <v>1397.07</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>E-COMMERCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B276" t="n">
+        <v>2197</v>
+      </c>
+      <c r="C276" t="n">
+        <v>423</v>
+      </c>
+      <c r="D276" t="n">
+        <v>2267.61</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B277" t="n">
+        <v>2716</v>
+      </c>
+      <c r="C277" t="n">
+        <v>977</v>
+      </c>
+      <c r="D277" t="n">
+        <v>729.29</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B278" t="n">
         <v>1993</v>
       </c>
-      <c r="C267" t="n">
-        <v>8888</v>
-      </c>
-      <c r="D267" t="n">
+      <c r="C278" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D278" t="n">
         <v>456.62</v>
       </c>
-      <c r="E267" t="inlineStr">
+      <c r="E278" t="inlineStr">
         <is>
           <t>OPERADOR LOGÍSTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B279" t="n">
+        <v>2767</v>
+      </c>
+      <c r="C279" t="n">
+        <v>2220</v>
+      </c>
+      <c r="D279" t="n">
+        <v>339.66</v>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 08:45:03
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F248"/>
+  <dimension ref="A1:F257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -729,13 +729,13 @@
         <v>46219</v>
       </c>
       <c r="B15" t="n">
-        <v>2362</v>
+        <v>2660</v>
       </c>
       <c r="C15" t="n">
         <v>8888</v>
       </c>
       <c r="D15" t="n">
-        <v>2827.89</v>
+        <v>832.51</v>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
@@ -749,13 +749,13 @@
         <v>46219</v>
       </c>
       <c r="B16" t="n">
-        <v>629</v>
+        <v>2362</v>
       </c>
       <c r="C16" t="n">
         <v>8888</v>
       </c>
       <c r="D16" t="n">
-        <v>1693.36</v>
+        <v>2827.89</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
@@ -769,13 +769,13 @@
         <v>46219</v>
       </c>
       <c r="B17" t="n">
-        <v>131</v>
+        <v>629</v>
       </c>
       <c r="C17" t="n">
         <v>8888</v>
       </c>
       <c r="D17" t="n">
-        <v>623.52</v>
+        <v>1693.36</v>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
@@ -789,13 +789,13 @@
         <v>46219</v>
       </c>
       <c r="B18" t="n">
-        <v>609</v>
+        <v>131</v>
       </c>
       <c r="C18" t="n">
         <v>8888</v>
       </c>
       <c r="D18" t="n">
-        <v>556.35</v>
+        <v>623.52</v>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
@@ -809,13 +809,13 @@
         <v>46219</v>
       </c>
       <c r="B19" t="n">
-        <v>131</v>
+        <v>609</v>
       </c>
       <c r="C19" t="n">
         <v>8888</v>
       </c>
       <c r="D19" t="n">
-        <v>623.52</v>
+        <v>556.35</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
@@ -829,13 +829,13 @@
         <v>46219</v>
       </c>
       <c r="B20" t="n">
-        <v>559</v>
+        <v>131</v>
       </c>
       <c r="C20" t="n">
         <v>8888</v>
       </c>
       <c r="D20" t="n">
-        <v>9596.75</v>
+        <v>623.52</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
@@ -849,13 +849,13 @@
         <v>46219</v>
       </c>
       <c r="B21" t="n">
-        <v>2107</v>
+        <v>559</v>
       </c>
       <c r="C21" t="n">
         <v>8888</v>
       </c>
       <c r="D21" t="n">
-        <v>6978.14</v>
+        <v>9596.75</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
@@ -869,13 +869,13 @@
         <v>46219</v>
       </c>
       <c r="B22" t="n">
-        <v>131</v>
+        <v>2107</v>
       </c>
       <c r="C22" t="n">
         <v>8888</v>
       </c>
       <c r="D22" t="n">
-        <v>934.3200000000001</v>
+        <v>6978.14</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
@@ -889,13 +889,13 @@
         <v>46219</v>
       </c>
       <c r="B23" t="n">
-        <v>360</v>
+        <v>131</v>
       </c>
       <c r="C23" t="n">
         <v>8888</v>
       </c>
       <c r="D23" t="n">
-        <v>1990.42</v>
+        <v>934.3200000000001</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
@@ -909,13 +909,13 @@
         <v>46219</v>
       </c>
       <c r="B24" t="n">
-        <v>768</v>
+        <v>360</v>
       </c>
       <c r="C24" t="n">
         <v>8888</v>
       </c>
       <c r="D24" t="n">
-        <v>3646.68</v>
+        <v>1990.42</v>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
@@ -929,13 +929,13 @@
         <v>46219</v>
       </c>
       <c r="B25" t="n">
-        <v>483</v>
+        <v>768</v>
       </c>
       <c r="C25" t="n">
         <v>8888</v>
       </c>
       <c r="D25" t="n">
-        <v>150.08</v>
+        <v>3646.68</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
@@ -949,13 +949,13 @@
         <v>46219</v>
       </c>
       <c r="B26" t="n">
-        <v>131</v>
+        <v>483</v>
       </c>
       <c r="C26" t="n">
         <v>8888</v>
       </c>
       <c r="D26" t="n">
-        <v>1742.9</v>
+        <v>150.08</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
@@ -969,13 +969,13 @@
         <v>46219</v>
       </c>
       <c r="B27" t="n">
-        <v>1478</v>
+        <v>131</v>
       </c>
       <c r="C27" t="n">
         <v>8888</v>
       </c>
       <c r="D27" t="n">
-        <v>4313.2</v>
+        <v>1742.9</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
@@ -989,18 +989,18 @@
         <v>46219</v>
       </c>
       <c r="B28" t="n">
-        <v>1756</v>
+        <v>1478</v>
       </c>
       <c r="C28" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D28" t="n">
-        <v>1217.45</v>
+        <v>4313.2</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1009,18 +1009,18 @@
         <v>46219</v>
       </c>
       <c r="B29" t="n">
-        <v>609</v>
+        <v>1756</v>
       </c>
       <c r="C29" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D29" t="n">
-        <v>741.79</v>
+        <v>1217.45</v>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1029,13 +1029,13 @@
         <v>46219</v>
       </c>
       <c r="B30" t="n">
-        <v>2015</v>
+        <v>609</v>
       </c>
       <c r="C30" t="n">
         <v>8888</v>
       </c>
       <c r="D30" t="n">
-        <v>1011.48</v>
+        <v>741.79</v>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
@@ -1049,13 +1049,13 @@
         <v>46219</v>
       </c>
       <c r="B31" t="n">
-        <v>629</v>
+        <v>2015</v>
       </c>
       <c r="C31" t="n">
         <v>8888</v>
       </c>
       <c r="D31" t="n">
-        <v>1338.55</v>
+        <v>1011.48</v>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
@@ -1069,18 +1069,18 @@
         <v>46219</v>
       </c>
       <c r="B32" t="n">
-        <v>2250</v>
+        <v>629</v>
       </c>
       <c r="C32" t="n">
         <v>8888</v>
       </c>
       <c r="D32" t="n">
-        <v>1134</v>
+        <v>1338.55</v>
       </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1089,13 +1089,13 @@
         <v>46219</v>
       </c>
       <c r="B33" t="n">
-        <v>1259</v>
+        <v>2250</v>
       </c>
       <c r="C33" t="n">
         <v>8888</v>
       </c>
       <c r="D33" t="n">
-        <v>213.64</v>
+        <v>1134</v>
       </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
@@ -1109,13 +1109,13 @@
         <v>46219</v>
       </c>
       <c r="B34" t="n">
-        <v>1756</v>
+        <v>1478</v>
       </c>
       <c r="C34" t="n">
         <v>8888</v>
       </c>
       <c r="D34" t="n">
-        <v>3007.36</v>
+        <v>1224</v>
       </c>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
@@ -1129,18 +1129,18 @@
         <v>46219</v>
       </c>
       <c r="B35" t="n">
-        <v>1064</v>
+        <v>1259</v>
       </c>
       <c r="C35" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D35" t="n">
-        <v>954.13</v>
+        <v>213.64</v>
       </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1149,13 +1149,13 @@
         <v>46219</v>
       </c>
       <c r="B36" t="n">
-        <v>629</v>
+        <v>1756</v>
       </c>
       <c r="C36" t="n">
         <v>8888</v>
       </c>
       <c r="D36" t="n">
-        <v>1997.38</v>
+        <v>3007.36</v>
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
@@ -1169,18 +1169,18 @@
         <v>46219</v>
       </c>
       <c r="B37" t="n">
-        <v>1756</v>
+        <v>131</v>
       </c>
       <c r="C37" t="n">
         <v>8888</v>
       </c>
       <c r="D37" t="n">
-        <v>1399.6</v>
+        <v>425.61</v>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1189,18 +1189,18 @@
         <v>46219</v>
       </c>
       <c r="B38" t="n">
-        <v>1756</v>
+        <v>1064</v>
       </c>
       <c r="C38" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D38" t="n">
-        <v>1383.55</v>
+        <v>954.13</v>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1209,13 +1209,13 @@
         <v>46219</v>
       </c>
       <c r="B39" t="n">
-        <v>2114</v>
+        <v>629</v>
       </c>
       <c r="C39" t="n">
         <v>8888</v>
       </c>
       <c r="D39" t="n">
-        <v>23987.35</v>
+        <v>1997.38</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
@@ -1229,13 +1229,13 @@
         <v>46219</v>
       </c>
       <c r="B40" t="n">
-        <v>131</v>
+        <v>1756</v>
       </c>
       <c r="C40" t="n">
         <v>8888</v>
       </c>
       <c r="D40" t="n">
-        <v>527.52</v>
+        <v>1399.6</v>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
@@ -1249,13 +1249,13 @@
         <v>46219</v>
       </c>
       <c r="B41" t="n">
-        <v>816</v>
+        <v>1756</v>
       </c>
       <c r="C41" t="n">
         <v>8888</v>
       </c>
       <c r="D41" t="n">
-        <v>2983.2</v>
+        <v>1383.55</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
@@ -1269,13 +1269,13 @@
         <v>46219</v>
       </c>
       <c r="B42" t="n">
-        <v>767</v>
+        <v>2114</v>
       </c>
       <c r="C42" t="n">
         <v>8888</v>
       </c>
       <c r="D42" t="n">
-        <v>428.17</v>
+        <v>23987.35</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
@@ -1289,13 +1289,13 @@
         <v>46219</v>
       </c>
       <c r="B43" t="n">
-        <v>14</v>
+        <v>2190</v>
       </c>
       <c r="C43" t="n">
         <v>8888</v>
       </c>
       <c r="D43" t="n">
-        <v>1155.74</v>
+        <v>1917.4</v>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
@@ -1309,13 +1309,13 @@
         <v>46219</v>
       </c>
       <c r="B44" t="n">
-        <v>20</v>
+        <v>131</v>
       </c>
       <c r="C44" t="n">
         <v>8888</v>
       </c>
       <c r="D44" t="n">
-        <v>10866.88</v>
+        <v>527.52</v>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
@@ -1329,13 +1329,13 @@
         <v>46219</v>
       </c>
       <c r="B45" t="n">
-        <v>629</v>
+        <v>816</v>
       </c>
       <c r="C45" t="n">
         <v>8888</v>
       </c>
       <c r="D45" t="n">
-        <v>14273.2</v>
+        <v>2983.2</v>
       </c>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
@@ -1349,13 +1349,13 @@
         <v>46219</v>
       </c>
       <c r="B46" t="n">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="C46" t="n">
         <v>8888</v>
       </c>
       <c r="D46" t="n">
-        <v>14378.8</v>
+        <v>428.17</v>
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
@@ -1369,18 +1369,18 @@
         <v>46219</v>
       </c>
       <c r="B47" t="n">
-        <v>1756</v>
+        <v>14</v>
       </c>
       <c r="C47" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D47" t="n">
-        <v>926.13</v>
+        <v>1155.74</v>
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1389,13 +1389,13 @@
         <v>46219</v>
       </c>
       <c r="B48" t="n">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="C48" t="n">
         <v>8888</v>
       </c>
       <c r="D48" t="n">
-        <v>1904.76</v>
+        <v>10866.88</v>
       </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
@@ -1409,13 +1409,13 @@
         <v>46219</v>
       </c>
       <c r="B49" t="n">
-        <v>131</v>
+        <v>629</v>
       </c>
       <c r="C49" t="n">
         <v>8888</v>
       </c>
       <c r="D49" t="n">
-        <v>594.8099999999999</v>
+        <v>14273.2</v>
       </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
@@ -1429,13 +1429,13 @@
         <v>46219</v>
       </c>
       <c r="B50" t="n">
-        <v>2452</v>
+        <v>768</v>
       </c>
       <c r="C50" t="n">
         <v>8888</v>
       </c>
       <c r="D50" t="n">
-        <v>3086.66</v>
+        <v>14378.8</v>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
@@ -1449,18 +1449,18 @@
         <v>46219</v>
       </c>
       <c r="B51" t="n">
-        <v>953</v>
+        <v>1756</v>
       </c>
       <c r="C51" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D51" t="n">
-        <v>604.53</v>
+        <v>926.13</v>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1469,13 +1469,13 @@
         <v>46219</v>
       </c>
       <c r="B52" t="n">
-        <v>768</v>
+        <v>58</v>
       </c>
       <c r="C52" t="n">
         <v>8888</v>
       </c>
       <c r="D52" t="n">
-        <v>1655.28</v>
+        <v>1904.76</v>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
@@ -1489,13 +1489,13 @@
         <v>46219</v>
       </c>
       <c r="B53" t="n">
-        <v>768</v>
+        <v>131</v>
       </c>
       <c r="C53" t="n">
         <v>8888</v>
       </c>
       <c r="D53" t="n">
-        <v>536.16</v>
+        <v>594.8099999999999</v>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
@@ -1509,13 +1509,13 @@
         <v>46219</v>
       </c>
       <c r="B54" t="n">
-        <v>629</v>
+        <v>2452</v>
       </c>
       <c r="C54" t="n">
         <v>8888</v>
       </c>
       <c r="D54" t="n">
-        <v>1276.58</v>
+        <v>3086.66</v>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
@@ -1529,13 +1529,13 @@
         <v>46219</v>
       </c>
       <c r="B55" t="n">
-        <v>1277</v>
+        <v>953</v>
       </c>
       <c r="C55" t="n">
         <v>8888</v>
       </c>
       <c r="D55" t="n">
-        <v>1591.9</v>
+        <v>604.53</v>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
@@ -1549,13 +1549,13 @@
         <v>46219</v>
       </c>
       <c r="B56" t="n">
-        <v>2163</v>
+        <v>768</v>
       </c>
       <c r="C56" t="n">
         <v>8888</v>
       </c>
       <c r="D56" t="n">
-        <v>406.1</v>
+        <v>1655.28</v>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
@@ -1569,13 +1569,13 @@
         <v>46219</v>
       </c>
       <c r="B57" t="n">
-        <v>14</v>
+        <v>768</v>
       </c>
       <c r="C57" t="n">
         <v>8888</v>
       </c>
       <c r="D57" t="n">
-        <v>343.54</v>
+        <v>536.16</v>
       </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
@@ -1589,13 +1589,13 @@
         <v>46219</v>
       </c>
       <c r="B58" t="n">
-        <v>438</v>
+        <v>629</v>
       </c>
       <c r="C58" t="n">
         <v>8888</v>
       </c>
       <c r="D58" t="n">
-        <v>1952.31</v>
+        <v>1276.58</v>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
@@ -1609,18 +1609,18 @@
         <v>46219</v>
       </c>
       <c r="B59" t="n">
-        <v>768</v>
+        <v>1277</v>
       </c>
       <c r="C59" t="n">
         <v>8888</v>
       </c>
       <c r="D59" t="n">
-        <v>7813.68</v>
+        <v>1591.9</v>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1629,13 +1629,13 @@
         <v>46219</v>
       </c>
       <c r="B60" t="n">
-        <v>768</v>
+        <v>2163</v>
       </c>
       <c r="C60" t="n">
         <v>8888</v>
       </c>
       <c r="D60" t="n">
-        <v>1291.96</v>
+        <v>406.1</v>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
@@ -1649,18 +1649,18 @@
         <v>46219</v>
       </c>
       <c r="B61" t="n">
-        <v>1518</v>
+        <v>14</v>
       </c>
       <c r="C61" t="n">
-        <v>1533</v>
+        <v>8888</v>
       </c>
       <c r="D61" t="n">
-        <v>5163.32</v>
+        <v>343.54</v>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1669,13 +1669,13 @@
         <v>46219</v>
       </c>
       <c r="B62" t="n">
-        <v>2190</v>
+        <v>438</v>
       </c>
       <c r="C62" t="n">
         <v>8888</v>
       </c>
       <c r="D62" t="n">
-        <v>870.03</v>
+        <v>1952.31</v>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
@@ -1689,18 +1689,18 @@
         <v>46219</v>
       </c>
       <c r="B63" t="n">
-        <v>1518</v>
+        <v>768</v>
       </c>
       <c r="C63" t="n">
-        <v>1533</v>
+        <v>8888</v>
       </c>
       <c r="D63" t="n">
-        <v>4494.7</v>
+        <v>7813.68</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
         <v>46219</v>
       </c>
       <c r="B64" t="n">
-        <v>2452</v>
+        <v>768</v>
       </c>
       <c r="C64" t="n">
         <v>8888</v>
       </c>
       <c r="D64" t="n">
-        <v>1253.5</v>
+        <v>1291.96</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
@@ -1729,13 +1729,13 @@
         <v>46219</v>
       </c>
       <c r="B65" t="n">
-        <v>1756</v>
+        <v>1518</v>
       </c>
       <c r="C65" t="n">
-        <v>27</v>
+        <v>1533</v>
       </c>
       <c r="D65" t="n">
-        <v>1575.17</v>
+        <v>5163.32</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
@@ -1749,13 +1749,13 @@
         <v>46219</v>
       </c>
       <c r="B66" t="n">
-        <v>768</v>
+        <v>2190</v>
       </c>
       <c r="C66" t="n">
         <v>8888</v>
       </c>
       <c r="D66" t="n">
-        <v>3118.72</v>
+        <v>870.03</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
@@ -1769,18 +1769,18 @@
         <v>46219</v>
       </c>
       <c r="B67" t="n">
-        <v>438</v>
+        <v>1518</v>
       </c>
       <c r="C67" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D67" t="n">
-        <v>338.69</v>
+        <v>4494.7</v>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1789,18 +1789,18 @@
         <v>46219</v>
       </c>
       <c r="B68" t="n">
-        <v>429</v>
+        <v>2452</v>
       </c>
       <c r="C68" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D68" t="n">
-        <v>1867.66</v>
+        <v>1253.5</v>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1809,18 +1809,18 @@
         <v>46219</v>
       </c>
       <c r="B69" t="n">
-        <v>1075</v>
+        <v>1756</v>
       </c>
       <c r="C69" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D69" t="n">
-        <v>1282.67</v>
+        <v>1575.17</v>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1829,13 +1829,13 @@
         <v>46219</v>
       </c>
       <c r="B70" t="n">
-        <v>1064</v>
+        <v>768</v>
       </c>
       <c r="C70" t="n">
         <v>8888</v>
       </c>
       <c r="D70" t="n">
-        <v>2550.8</v>
+        <v>3118.72</v>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
@@ -1849,13 +1849,13 @@
         <v>46219</v>
       </c>
       <c r="B71" t="n">
-        <v>2131</v>
+        <v>438</v>
       </c>
       <c r="C71" t="n">
         <v>8888</v>
       </c>
       <c r="D71" t="n">
-        <v>1153.68</v>
+        <v>338.69</v>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
@@ -1869,18 +1869,18 @@
         <v>46219</v>
       </c>
       <c r="B72" t="n">
-        <v>609</v>
+        <v>429</v>
       </c>
       <c r="C72" t="n">
-        <v>8888</v>
+        <v>1281</v>
       </c>
       <c r="D72" t="n">
-        <v>1854.48</v>
+        <v>1867.66</v>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -1889,18 +1889,18 @@
         <v>46219</v>
       </c>
       <c r="B73" t="n">
-        <v>438</v>
+        <v>1075</v>
       </c>
       <c r="C73" t="n">
         <v>8888</v>
       </c>
       <c r="D73" t="n">
-        <v>712</v>
+        <v>1282.67</v>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -1909,18 +1909,18 @@
         <v>46219</v>
       </c>
       <c r="B74" t="n">
-        <v>1658</v>
+        <v>1064</v>
       </c>
       <c r="C74" t="n">
         <v>8888</v>
       </c>
       <c r="D74" t="n">
-        <v>311.88</v>
+        <v>2550.8</v>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -1929,13 +1929,13 @@
         <v>46219</v>
       </c>
       <c r="B75" t="n">
-        <v>1293</v>
+        <v>2131</v>
       </c>
       <c r="C75" t="n">
         <v>8888</v>
       </c>
       <c r="D75" t="n">
-        <v>1354.46</v>
+        <v>1153.68</v>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
@@ -1949,13 +1949,13 @@
         <v>46219</v>
       </c>
       <c r="B76" t="n">
-        <v>816</v>
+        <v>609</v>
       </c>
       <c r="C76" t="n">
         <v>8888</v>
       </c>
       <c r="D76" t="n">
-        <v>3118.8</v>
+        <v>1854.48</v>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
@@ -1969,13 +1969,13 @@
         <v>46219</v>
       </c>
       <c r="B77" t="n">
-        <v>451</v>
+        <v>438</v>
       </c>
       <c r="C77" t="n">
         <v>8888</v>
       </c>
       <c r="D77" t="n">
-        <v>2231.47</v>
+        <v>712</v>
       </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
@@ -1989,18 +1989,18 @@
         <v>46219</v>
       </c>
       <c r="B78" t="n">
-        <v>629</v>
+        <v>1658</v>
       </c>
       <c r="C78" t="n">
         <v>8888</v>
       </c>
       <c r="D78" t="n">
-        <v>1178.64</v>
+        <v>311.88</v>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2009,13 +2009,13 @@
         <v>46219</v>
       </c>
       <c r="B79" t="n">
-        <v>703</v>
+        <v>1293</v>
       </c>
       <c r="C79" t="n">
         <v>8888</v>
       </c>
       <c r="D79" t="n">
-        <v>1431.24</v>
+        <v>1354.46</v>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
@@ -2029,13 +2029,13 @@
         <v>46219</v>
       </c>
       <c r="B80" t="n">
-        <v>629</v>
+        <v>816</v>
       </c>
       <c r="C80" t="n">
         <v>8888</v>
       </c>
       <c r="D80" t="n">
-        <v>761.87</v>
+        <v>3118.8</v>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
@@ -2049,13 +2049,13 @@
         <v>46219</v>
       </c>
       <c r="B81" t="n">
-        <v>609</v>
+        <v>451</v>
       </c>
       <c r="C81" t="n">
         <v>8888</v>
       </c>
       <c r="D81" t="n">
-        <v>2107.32</v>
+        <v>2231.47</v>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
@@ -2069,13 +2069,13 @@
         <v>46219</v>
       </c>
       <c r="B82" t="n">
-        <v>1293</v>
+        <v>629</v>
       </c>
       <c r="C82" t="n">
         <v>8888</v>
       </c>
       <c r="D82" t="n">
-        <v>5342.64</v>
+        <v>1178.64</v>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
@@ -2089,13 +2089,13 @@
         <v>46219</v>
       </c>
       <c r="B83" t="n">
-        <v>609</v>
+        <v>703</v>
       </c>
       <c r="C83" t="n">
         <v>8888</v>
       </c>
       <c r="D83" t="n">
-        <v>1919.68</v>
+        <v>1431.24</v>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
@@ -2109,18 +2109,18 @@
         <v>46219</v>
       </c>
       <c r="B84" t="n">
-        <v>1324</v>
+        <v>629</v>
       </c>
       <c r="C84" t="n">
-        <v>3009</v>
+        <v>8888</v>
       </c>
       <c r="D84" t="n">
-        <v>4396.24</v>
+        <v>761.87</v>
       </c>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2129,13 +2129,13 @@
         <v>46219</v>
       </c>
       <c r="B85" t="n">
-        <v>400</v>
+        <v>609</v>
       </c>
       <c r="C85" t="n">
         <v>8888</v>
       </c>
       <c r="D85" t="n">
-        <v>1953.42</v>
+        <v>2107.32</v>
       </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
@@ -2149,13 +2149,13 @@
         <v>46219</v>
       </c>
       <c r="B86" t="n">
-        <v>14</v>
+        <v>1293</v>
       </c>
       <c r="C86" t="n">
         <v>8888</v>
       </c>
       <c r="D86" t="n">
-        <v>1006.88</v>
+        <v>5342.64</v>
       </c>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
@@ -2169,13 +2169,13 @@
         <v>46219</v>
       </c>
       <c r="B87" t="n">
-        <v>2362</v>
+        <v>609</v>
       </c>
       <c r="C87" t="n">
         <v>8888</v>
       </c>
       <c r="D87" t="n">
-        <v>3074.16</v>
+        <v>1919.68</v>
       </c>
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
@@ -2189,13 +2189,13 @@
         <v>46219</v>
       </c>
       <c r="B88" t="n">
-        <v>2279</v>
+        <v>1324</v>
       </c>
       <c r="C88" t="n">
-        <v>1139</v>
+        <v>3009</v>
       </c>
       <c r="D88" t="n">
-        <v>348.16</v>
+        <v>4396.24</v>
       </c>
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
@@ -2209,13 +2209,13 @@
         <v>46219</v>
       </c>
       <c r="B89" t="n">
-        <v>351</v>
+        <v>400</v>
       </c>
       <c r="C89" t="n">
         <v>8888</v>
       </c>
       <c r="D89" t="n">
-        <v>6142.76</v>
+        <v>1953.42</v>
       </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
@@ -2229,18 +2229,18 @@
         <v>46219</v>
       </c>
       <c r="B90" t="n">
-        <v>1299</v>
+        <v>14</v>
       </c>
       <c r="C90" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D90" t="n">
-        <v>1276.32</v>
+        <v>1006.88</v>
       </c>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
         <v>8888</v>
       </c>
       <c r="D91" t="n">
-        <v>2291.35</v>
+        <v>3074.16</v>
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
@@ -2269,18 +2269,18 @@
         <v>46219</v>
       </c>
       <c r="B92" t="n">
-        <v>131</v>
+        <v>2279</v>
       </c>
       <c r="C92" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D92" t="n">
-        <v>857.34</v>
+        <v>348.16</v>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2289,13 +2289,13 @@
         <v>46219</v>
       </c>
       <c r="B93" t="n">
-        <v>14</v>
+        <v>351</v>
       </c>
       <c r="C93" t="n">
         <v>8888</v>
       </c>
       <c r="D93" t="n">
-        <v>311.88</v>
+        <v>6142.76</v>
       </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
@@ -2309,18 +2309,18 @@
         <v>46219</v>
       </c>
       <c r="B94" t="n">
-        <v>1372</v>
+        <v>1299</v>
       </c>
       <c r="C94" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D94" t="n">
-        <v>10235.04</v>
+        <v>1276.32</v>
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2329,13 +2329,13 @@
         <v>46219</v>
       </c>
       <c r="B95" t="n">
-        <v>20</v>
+        <v>2362</v>
       </c>
       <c r="C95" t="n">
         <v>8888</v>
       </c>
       <c r="D95" t="n">
-        <v>4660.07</v>
+        <v>2291.35</v>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
@@ -2349,18 +2349,18 @@
         <v>46219</v>
       </c>
       <c r="B96" t="n">
-        <v>609</v>
+        <v>131</v>
       </c>
       <c r="C96" t="n">
-        <v>3179</v>
+        <v>8888</v>
       </c>
       <c r="D96" t="n">
-        <v>891.63</v>
+        <v>857.34</v>
       </c>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2369,18 +2369,18 @@
         <v>46219</v>
       </c>
       <c r="B97" t="n">
-        <v>2250</v>
+        <v>14</v>
       </c>
       <c r="C97" t="n">
         <v>8888</v>
       </c>
       <c r="D97" t="n">
-        <v>3311.6</v>
+        <v>311.88</v>
       </c>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2389,13 +2389,13 @@
         <v>46219</v>
       </c>
       <c r="B98" t="n">
-        <v>1324</v>
+        <v>1372</v>
       </c>
       <c r="C98" t="n">
         <v>8888</v>
       </c>
       <c r="D98" t="n">
-        <v>8134.2</v>
+        <v>10235.04</v>
       </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
@@ -2409,13 +2409,13 @@
         <v>46219</v>
       </c>
       <c r="B99" t="n">
-        <v>2211</v>
+        <v>20</v>
       </c>
       <c r="C99" t="n">
         <v>8888</v>
       </c>
       <c r="D99" t="n">
-        <v>2125.44</v>
+        <v>4660.07</v>
       </c>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
@@ -2429,18 +2429,18 @@
         <v>46219</v>
       </c>
       <c r="B100" t="n">
-        <v>483</v>
+        <v>609</v>
       </c>
       <c r="C100" t="n">
-        <v>8888</v>
+        <v>3179</v>
       </c>
       <c r="D100" t="n">
-        <v>4217.99</v>
+        <v>891.63</v>
       </c>
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2449,13 +2449,13 @@
         <v>46219</v>
       </c>
       <c r="B101" t="n">
-        <v>1937</v>
+        <v>2250</v>
       </c>
       <c r="C101" t="n">
         <v>8888</v>
       </c>
       <c r="D101" t="n">
-        <v>2231.47</v>
+        <v>3311.6</v>
       </c>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
@@ -2469,13 +2469,13 @@
         <v>46219</v>
       </c>
       <c r="B102" t="n">
-        <v>40</v>
+        <v>1324</v>
       </c>
       <c r="C102" t="n">
         <v>8888</v>
       </c>
       <c r="D102" t="n">
-        <v>613.16</v>
+        <v>8134.2</v>
       </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
@@ -2489,13 +2489,13 @@
         <v>46219</v>
       </c>
       <c r="B103" t="n">
-        <v>1064</v>
+        <v>2211</v>
       </c>
       <c r="C103" t="n">
         <v>8888</v>
       </c>
       <c r="D103" t="n">
-        <v>720.52</v>
+        <v>2125.44</v>
       </c>
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
@@ -2509,13 +2509,13 @@
         <v>46219</v>
       </c>
       <c r="B104" t="n">
-        <v>1873</v>
+        <v>483</v>
       </c>
       <c r="C104" t="n">
         <v>8888</v>
       </c>
       <c r="D104" t="n">
-        <v>138.39</v>
+        <v>4217.99</v>
       </c>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
@@ -2529,18 +2529,18 @@
         <v>46219</v>
       </c>
       <c r="B105" t="n">
-        <v>2250</v>
+        <v>1937</v>
       </c>
       <c r="C105" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D105" t="n">
-        <v>1646.82</v>
+        <v>2231.47</v>
       </c>
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2555,12 +2555,12 @@
         <v>8888</v>
       </c>
       <c r="D106" t="n">
-        <v>956.01</v>
+        <v>613.16</v>
       </c>
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2569,13 +2569,13 @@
         <v>46219</v>
       </c>
       <c r="B107" t="n">
-        <v>629</v>
+        <v>1064</v>
       </c>
       <c r="C107" t="n">
         <v>8888</v>
       </c>
       <c r="D107" t="n">
-        <v>18471.2</v>
+        <v>720.52</v>
       </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
@@ -2589,13 +2589,13 @@
         <v>46219</v>
       </c>
       <c r="B108" t="n">
-        <v>703</v>
+        <v>1873</v>
       </c>
       <c r="C108" t="n">
         <v>8888</v>
       </c>
       <c r="D108" t="n">
-        <v>2946.27</v>
+        <v>138.39</v>
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
@@ -2609,18 +2609,18 @@
         <v>46219</v>
       </c>
       <c r="B109" t="n">
-        <v>629</v>
+        <v>2250</v>
       </c>
       <c r="C109" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D109" t="n">
-        <v>1002.21</v>
+        <v>1646.82</v>
       </c>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2629,13 +2629,13 @@
         <v>46219</v>
       </c>
       <c r="B110" t="n">
-        <v>1876</v>
+        <v>40</v>
       </c>
       <c r="C110" t="n">
         <v>8888</v>
       </c>
       <c r="D110" t="n">
-        <v>660.5599999999999</v>
+        <v>956.01</v>
       </c>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
@@ -2649,18 +2649,18 @@
         <v>46219</v>
       </c>
       <c r="B111" t="n">
-        <v>1075</v>
+        <v>629</v>
       </c>
       <c r="C111" t="n">
         <v>8888</v>
       </c>
       <c r="D111" t="n">
-        <v>325.49</v>
+        <v>18471.2</v>
       </c>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2669,13 +2669,13 @@
         <v>46219</v>
       </c>
       <c r="B112" t="n">
-        <v>451</v>
+        <v>703</v>
       </c>
       <c r="C112" t="n">
         <v>8888</v>
       </c>
       <c r="D112" t="n">
-        <v>1264.4</v>
+        <v>2946.27</v>
       </c>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
@@ -2689,18 +2689,18 @@
         <v>46219</v>
       </c>
       <c r="B113" t="n">
-        <v>619</v>
+        <v>629</v>
       </c>
       <c r="C113" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D113" t="n">
-        <v>1169.16</v>
+        <v>1002.21</v>
       </c>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -2709,13 +2709,13 @@
         <v>46219</v>
       </c>
       <c r="B114" t="n">
-        <v>703</v>
+        <v>20</v>
       </c>
       <c r="C114" t="n">
         <v>8888</v>
       </c>
       <c r="D114" t="n">
-        <v>599.88</v>
+        <v>7233.04</v>
       </c>
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
@@ -2729,18 +2729,18 @@
         <v>46219</v>
       </c>
       <c r="B115" t="n">
-        <v>1064</v>
+        <v>1876</v>
       </c>
       <c r="C115" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D115" t="n">
-        <v>954.13</v>
+        <v>660.5599999999999</v>
       </c>
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2749,18 +2749,18 @@
         <v>46219</v>
       </c>
       <c r="B116" t="n">
-        <v>571</v>
+        <v>1075</v>
       </c>
       <c r="C116" t="n">
         <v>8888</v>
       </c>
       <c r="D116" t="n">
-        <v>25609.34</v>
+        <v>325.49</v>
       </c>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -2769,13 +2769,13 @@
         <v>46219</v>
       </c>
       <c r="B117" t="n">
-        <v>131</v>
+        <v>451</v>
       </c>
       <c r="C117" t="n">
         <v>8888</v>
       </c>
       <c r="D117" t="n">
-        <v>934.3200000000001</v>
+        <v>1264.4</v>
       </c>
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
@@ -2789,18 +2789,18 @@
         <v>46219</v>
       </c>
       <c r="B118" t="n">
-        <v>2660</v>
+        <v>619</v>
       </c>
       <c r="C118" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D118" t="n">
-        <v>3419.84</v>
+        <v>1169.16</v>
       </c>
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2809,13 +2809,13 @@
         <v>46219</v>
       </c>
       <c r="B119" t="n">
-        <v>400</v>
+        <v>703</v>
       </c>
       <c r="C119" t="n">
         <v>8888</v>
       </c>
       <c r="D119" t="n">
-        <v>346.8</v>
+        <v>599.88</v>
       </c>
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
@@ -2829,18 +2829,18 @@
         <v>46219</v>
       </c>
       <c r="B120" t="n">
-        <v>2362</v>
+        <v>1064</v>
       </c>
       <c r="C120" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D120" t="n">
-        <v>1457.7</v>
+        <v>954.13</v>
       </c>
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -2849,13 +2849,13 @@
         <v>46219</v>
       </c>
       <c r="B121" t="n">
-        <v>816</v>
+        <v>571</v>
       </c>
       <c r="C121" t="n">
         <v>8888</v>
       </c>
       <c r="D121" t="n">
-        <v>311.95</v>
+        <v>25609.34</v>
       </c>
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr">
@@ -2869,13 +2869,13 @@
         <v>46219</v>
       </c>
       <c r="B122" t="n">
-        <v>20</v>
+        <v>1277</v>
       </c>
       <c r="C122" t="n">
         <v>8888</v>
       </c>
       <c r="D122" t="n">
-        <v>2247.2</v>
+        <v>2666.71</v>
       </c>
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
@@ -2889,13 +2889,13 @@
         <v>46219</v>
       </c>
       <c r="B123" t="n">
-        <v>890</v>
+        <v>131</v>
       </c>
       <c r="C123" t="n">
         <v>8888</v>
       </c>
       <c r="D123" t="n">
-        <v>310.39</v>
+        <v>934.3200000000001</v>
       </c>
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
@@ -2909,13 +2909,13 @@
         <v>46219</v>
       </c>
       <c r="B124" t="n">
-        <v>1293</v>
+        <v>2660</v>
       </c>
       <c r="C124" t="n">
         <v>8888</v>
       </c>
       <c r="D124" t="n">
-        <v>3237.41</v>
+        <v>3419.84</v>
       </c>
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
@@ -2929,13 +2929,13 @@
         <v>46219</v>
       </c>
       <c r="B125" t="n">
-        <v>2452</v>
+        <v>400</v>
       </c>
       <c r="C125" t="n">
         <v>8888</v>
       </c>
       <c r="D125" t="n">
-        <v>1632.81</v>
+        <v>346.8</v>
       </c>
       <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr">
@@ -2949,13 +2949,13 @@
         <v>46219</v>
       </c>
       <c r="B126" t="n">
-        <v>483</v>
+        <v>2362</v>
       </c>
       <c r="C126" t="n">
         <v>8888</v>
       </c>
       <c r="D126" t="n">
-        <v>2953.24</v>
+        <v>1457.7</v>
       </c>
       <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr">
@@ -2969,13 +2969,13 @@
         <v>46219</v>
       </c>
       <c r="B127" t="n">
-        <v>131</v>
+        <v>816</v>
       </c>
       <c r="C127" t="n">
         <v>8888</v>
       </c>
       <c r="D127" t="n">
-        <v>1384.39</v>
+        <v>311.95</v>
       </c>
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
@@ -2989,13 +2989,13 @@
         <v>46219</v>
       </c>
       <c r="B128" t="n">
-        <v>2652</v>
+        <v>20</v>
       </c>
       <c r="C128" t="n">
         <v>8888</v>
       </c>
       <c r="D128" t="n">
-        <v>3419.64</v>
+        <v>2247.2</v>
       </c>
       <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr">
@@ -3009,18 +3009,18 @@
         <v>46219</v>
       </c>
       <c r="B129" t="n">
-        <v>1117</v>
+        <v>890</v>
       </c>
       <c r="C129" t="n">
-        <v>1139</v>
+        <v>8888</v>
       </c>
       <c r="D129" t="n">
-        <v>238.55</v>
+        <v>310.39</v>
       </c>
       <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3029,13 +3029,13 @@
         <v>46219</v>
       </c>
       <c r="B130" t="n">
-        <v>2107</v>
+        <v>1293</v>
       </c>
       <c r="C130" t="n">
         <v>8888</v>
       </c>
       <c r="D130" t="n">
-        <v>1958.34</v>
+        <v>3237.41</v>
       </c>
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
@@ -3049,13 +3049,13 @@
         <v>46219</v>
       </c>
       <c r="B131" t="n">
-        <v>131</v>
+        <v>2452</v>
       </c>
       <c r="C131" t="n">
         <v>8888</v>
       </c>
       <c r="D131" t="n">
-        <v>767.04</v>
+        <v>1632.81</v>
       </c>
       <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
@@ -3069,18 +3069,18 @@
         <v>46219</v>
       </c>
       <c r="B132" t="n">
-        <v>1756</v>
+        <v>483</v>
       </c>
       <c r="C132" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D132" t="n">
-        <v>1939.32</v>
+        <v>2953.24</v>
       </c>
       <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3089,13 +3089,13 @@
         <v>46219</v>
       </c>
       <c r="B133" t="n">
-        <v>1372</v>
+        <v>131</v>
       </c>
       <c r="C133" t="n">
         <v>8888</v>
       </c>
       <c r="D133" t="n">
-        <v>879.6</v>
+        <v>1384.39</v>
       </c>
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr">
@@ -3109,13 +3109,13 @@
         <v>46219</v>
       </c>
       <c r="B134" t="n">
-        <v>360</v>
+        <v>2652</v>
       </c>
       <c r="C134" t="n">
         <v>8888</v>
       </c>
       <c r="D134" t="n">
-        <v>1906.67</v>
+        <v>3419.64</v>
       </c>
       <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
@@ -3129,18 +3129,18 @@
         <v>46219</v>
       </c>
       <c r="B135" t="n">
-        <v>131</v>
+        <v>1117</v>
       </c>
       <c r="C135" t="n">
-        <v>8888</v>
+        <v>1139</v>
       </c>
       <c r="D135" t="n">
-        <v>2281.48</v>
+        <v>238.55</v>
       </c>
       <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3149,13 +3149,13 @@
         <v>46219</v>
       </c>
       <c r="B136" t="n">
-        <v>1372</v>
+        <v>2107</v>
       </c>
       <c r="C136" t="n">
         <v>8888</v>
       </c>
       <c r="D136" t="n">
-        <v>839.58</v>
+        <v>1958.34</v>
       </c>
       <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
@@ -3169,18 +3169,18 @@
         <v>46219</v>
       </c>
       <c r="B137" t="n">
-        <v>1996</v>
+        <v>131</v>
       </c>
       <c r="C137" t="n">
-        <v>691</v>
+        <v>8888</v>
       </c>
       <c r="D137" t="n">
-        <v>2078.56</v>
+        <v>767.04</v>
       </c>
       <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3189,13 +3189,13 @@
         <v>46219</v>
       </c>
       <c r="B138" t="n">
-        <v>1064</v>
+        <v>1756</v>
       </c>
       <c r="C138" t="n">
         <v>27</v>
       </c>
       <c r="D138" t="n">
-        <v>954.13</v>
+        <v>1939.32</v>
       </c>
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr">
@@ -3209,13 +3209,13 @@
         <v>46219</v>
       </c>
       <c r="B139" t="n">
-        <v>559</v>
+        <v>1372</v>
       </c>
       <c r="C139" t="n">
         <v>8888</v>
       </c>
       <c r="D139" t="n">
-        <v>1245.19</v>
+        <v>879.6</v>
       </c>
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
@@ -3229,13 +3229,13 @@
         <v>46219</v>
       </c>
       <c r="B140" t="n">
-        <v>580</v>
+        <v>360</v>
       </c>
       <c r="C140" t="n">
         <v>8888</v>
       </c>
       <c r="D140" t="n">
-        <v>3020.55</v>
+        <v>1906.67</v>
       </c>
       <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
@@ -3249,13 +3249,13 @@
         <v>46219</v>
       </c>
       <c r="B141" t="n">
-        <v>1064</v>
+        <v>131</v>
       </c>
       <c r="C141" t="n">
         <v>8888</v>
       </c>
       <c r="D141" t="n">
-        <v>1001.61</v>
+        <v>2281.48</v>
       </c>
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr">
@@ -3269,18 +3269,18 @@
         <v>46219</v>
       </c>
       <c r="B142" t="n">
-        <v>325</v>
+        <v>1372</v>
       </c>
       <c r="C142" t="n">
         <v>8888</v>
       </c>
       <c r="D142" t="n">
-        <v>100.62</v>
+        <v>839.58</v>
       </c>
       <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3289,18 +3289,18 @@
         <v>46219</v>
       </c>
       <c r="B143" t="n">
-        <v>1293</v>
+        <v>1996</v>
       </c>
       <c r="C143" t="n">
-        <v>8888</v>
+        <v>691</v>
       </c>
       <c r="D143" t="n">
-        <v>1354.46</v>
+        <v>2078.56</v>
       </c>
       <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3309,18 +3309,18 @@
         <v>46219</v>
       </c>
       <c r="B144" t="n">
-        <v>629</v>
+        <v>1064</v>
       </c>
       <c r="C144" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D144" t="n">
-        <v>1804.42</v>
+        <v>954.13</v>
       </c>
       <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3329,13 +3329,13 @@
         <v>46219</v>
       </c>
       <c r="B145" t="n">
-        <v>2245</v>
+        <v>559</v>
       </c>
       <c r="C145" t="n">
         <v>8888</v>
       </c>
       <c r="D145" t="n">
-        <v>983.59</v>
+        <v>1245.19</v>
       </c>
       <c r="E145" t="inlineStr"/>
       <c r="F145" t="inlineStr">
@@ -3349,13 +3349,13 @@
         <v>46219</v>
       </c>
       <c r="B146" t="n">
-        <v>131</v>
+        <v>580</v>
       </c>
       <c r="C146" t="n">
         <v>8888</v>
       </c>
       <c r="D146" t="n">
-        <v>989.47</v>
+        <v>3020.55</v>
       </c>
       <c r="E146" t="inlineStr"/>
       <c r="F146" t="inlineStr">
@@ -3369,13 +3369,13 @@
         <v>46219</v>
       </c>
       <c r="B147" t="n">
-        <v>131</v>
+        <v>1064</v>
       </c>
       <c r="C147" t="n">
         <v>8888</v>
       </c>
       <c r="D147" t="n">
-        <v>934.3200000000001</v>
+        <v>1001.61</v>
       </c>
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr">
@@ -3389,18 +3389,18 @@
         <v>46219</v>
       </c>
       <c r="B148" t="n">
-        <v>2362</v>
+        <v>325</v>
       </c>
       <c r="C148" t="n">
         <v>8888</v>
       </c>
       <c r="D148" t="n">
-        <v>327.61</v>
+        <v>100.62</v>
       </c>
       <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3409,18 +3409,18 @@
         <v>46219</v>
       </c>
       <c r="B149" t="n">
-        <v>325</v>
+        <v>1293</v>
       </c>
       <c r="C149" t="n">
         <v>8888</v>
       </c>
       <c r="D149" t="n">
-        <v>25.9</v>
+        <v>1354.46</v>
       </c>
       <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3429,13 +3429,13 @@
         <v>46219</v>
       </c>
       <c r="B150" t="n">
-        <v>1756</v>
+        <v>629</v>
       </c>
       <c r="C150" t="n">
         <v>8888</v>
       </c>
       <c r="D150" t="n">
-        <v>5236.57</v>
+        <v>1804.42</v>
       </c>
       <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr">
@@ -3449,13 +3449,13 @@
         <v>46219</v>
       </c>
       <c r="B151" t="n">
-        <v>20</v>
+        <v>2245</v>
       </c>
       <c r="C151" t="n">
         <v>8888</v>
       </c>
       <c r="D151" t="n">
-        <v>5859.38</v>
+        <v>983.59</v>
       </c>
       <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr">
@@ -3469,13 +3469,13 @@
         <v>46219</v>
       </c>
       <c r="B152" t="n">
-        <v>629</v>
+        <v>131</v>
       </c>
       <c r="C152" t="n">
         <v>8888</v>
       </c>
       <c r="D152" t="n">
-        <v>1292.86</v>
+        <v>989.47</v>
       </c>
       <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr">
@@ -3489,13 +3489,13 @@
         <v>46219</v>
       </c>
       <c r="B153" t="n">
-        <v>2383</v>
+        <v>131</v>
       </c>
       <c r="C153" t="n">
         <v>8888</v>
       </c>
       <c r="D153" t="n">
-        <v>5887.04</v>
+        <v>934.3200000000001</v>
       </c>
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr">
@@ -3509,13 +3509,13 @@
         <v>46219</v>
       </c>
       <c r="B154" t="n">
-        <v>131</v>
+        <v>2362</v>
       </c>
       <c r="C154" t="n">
         <v>8888</v>
       </c>
       <c r="D154" t="n">
-        <v>2983.2</v>
+        <v>327.61</v>
       </c>
       <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr">
@@ -3529,18 +3529,18 @@
         <v>46219</v>
       </c>
       <c r="B155" t="n">
-        <v>1007</v>
+        <v>325</v>
       </c>
       <c r="C155" t="n">
         <v>8888</v>
       </c>
       <c r="D155" t="n">
-        <v>1664.69</v>
+        <v>25.9</v>
       </c>
       <c r="E155" t="inlineStr"/>
       <c r="F155" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3549,18 +3549,18 @@
         <v>46219</v>
       </c>
       <c r="B156" t="n">
-        <v>890</v>
+        <v>1756</v>
       </c>
       <c r="C156" t="n">
-        <v>1533</v>
+        <v>8888</v>
       </c>
       <c r="D156" t="n">
-        <v>670.6799999999999</v>
+        <v>5236.57</v>
       </c>
       <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3569,18 +3569,18 @@
         <v>46219</v>
       </c>
       <c r="B157" t="n">
-        <v>325</v>
+        <v>20</v>
       </c>
       <c r="C157" t="n">
         <v>8888</v>
       </c>
       <c r="D157" t="n">
-        <v>44.59</v>
+        <v>5859.38</v>
       </c>
       <c r="E157" t="inlineStr"/>
       <c r="F157" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3589,13 +3589,13 @@
         <v>46219</v>
       </c>
       <c r="B158" t="n">
-        <v>2362</v>
+        <v>629</v>
       </c>
       <c r="C158" t="n">
         <v>8888</v>
       </c>
       <c r="D158" t="n">
-        <v>383.76</v>
+        <v>1292.86</v>
       </c>
       <c r="E158" t="inlineStr"/>
       <c r="F158" t="inlineStr">
@@ -3609,13 +3609,13 @@
         <v>46219</v>
       </c>
       <c r="B159" t="n">
-        <v>1465</v>
+        <v>2383</v>
       </c>
       <c r="C159" t="n">
         <v>8888</v>
       </c>
       <c r="D159" t="n">
-        <v>2350.22</v>
+        <v>5887.04</v>
       </c>
       <c r="E159" t="inlineStr"/>
       <c r="F159" t="inlineStr">
@@ -3629,13 +3629,13 @@
         <v>46219</v>
       </c>
       <c r="B160" t="n">
-        <v>483</v>
+        <v>131</v>
       </c>
       <c r="C160" t="n">
         <v>8888</v>
       </c>
       <c r="D160" t="n">
-        <v>689.02</v>
+        <v>2983.2</v>
       </c>
       <c r="E160" t="inlineStr"/>
       <c r="F160" t="inlineStr">
@@ -3649,13 +3649,13 @@
         <v>46219</v>
       </c>
       <c r="B161" t="n">
-        <v>2452</v>
+        <v>1007</v>
       </c>
       <c r="C161" t="n">
         <v>8888</v>
       </c>
       <c r="D161" t="n">
-        <v>4530.7</v>
+        <v>1664.69</v>
       </c>
       <c r="E161" t="inlineStr"/>
       <c r="F161" t="inlineStr">
@@ -3669,18 +3669,18 @@
         <v>46219</v>
       </c>
       <c r="B162" t="n">
-        <v>400</v>
+        <v>890</v>
       </c>
       <c r="C162" t="n">
-        <v>8888</v>
+        <v>1533</v>
       </c>
       <c r="D162" t="n">
-        <v>1292.32</v>
+        <v>670.6799999999999</v>
       </c>
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -3689,18 +3689,18 @@
         <v>46219</v>
       </c>
       <c r="B163" t="n">
-        <v>2362</v>
+        <v>325</v>
       </c>
       <c r="C163" t="n">
         <v>8888</v>
       </c>
       <c r="D163" t="n">
-        <v>744.4</v>
+        <v>44.59</v>
       </c>
       <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3709,13 +3709,13 @@
         <v>46219</v>
       </c>
       <c r="B164" t="n">
-        <v>1756</v>
+        <v>2362</v>
       </c>
       <c r="C164" t="n">
         <v>8888</v>
       </c>
       <c r="D164" t="n">
-        <v>462.4</v>
+        <v>383.76</v>
       </c>
       <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr">
@@ -3729,13 +3729,13 @@
         <v>46219</v>
       </c>
       <c r="B165" t="n">
-        <v>571</v>
+        <v>1465</v>
       </c>
       <c r="C165" t="n">
         <v>8888</v>
       </c>
       <c r="D165" t="n">
-        <v>1125.6</v>
+        <v>2350.22</v>
       </c>
       <c r="E165" t="inlineStr"/>
       <c r="F165" t="inlineStr">
@@ -3749,13 +3749,13 @@
         <v>46219</v>
       </c>
       <c r="B166" t="n">
-        <v>571</v>
+        <v>483</v>
       </c>
       <c r="C166" t="n">
         <v>8888</v>
       </c>
       <c r="D166" t="n">
-        <v>5997.18</v>
+        <v>689.02</v>
       </c>
       <c r="E166" t="inlineStr"/>
       <c r="F166" t="inlineStr">
@@ -3769,13 +3769,13 @@
         <v>46219</v>
       </c>
       <c r="B167" t="n">
-        <v>2421</v>
+        <v>2452</v>
       </c>
       <c r="C167" t="n">
         <v>8888</v>
       </c>
       <c r="D167" t="n">
-        <v>2786.14</v>
+        <v>4530.7</v>
       </c>
       <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr">
@@ -3789,13 +3789,13 @@
         <v>46219</v>
       </c>
       <c r="B168" t="n">
-        <v>953</v>
+        <v>400</v>
       </c>
       <c r="C168" t="n">
         <v>8888</v>
       </c>
       <c r="D168" t="n">
-        <v>6995.34</v>
+        <v>1292.32</v>
       </c>
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr">
@@ -3809,18 +3809,18 @@
         <v>46219</v>
       </c>
       <c r="B169" t="n">
-        <v>2769</v>
+        <v>2362</v>
       </c>
       <c r="C169" t="n">
         <v>8888</v>
       </c>
       <c r="D169" t="n">
-        <v>620.37</v>
+        <v>744.4</v>
       </c>
       <c r="E169" t="inlineStr"/>
       <c r="F169" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3829,13 +3829,13 @@
         <v>46219</v>
       </c>
       <c r="B170" t="n">
-        <v>2362</v>
+        <v>1478</v>
       </c>
       <c r="C170" t="n">
         <v>8888</v>
       </c>
       <c r="D170" t="n">
-        <v>8080.76</v>
+        <v>1123.2</v>
       </c>
       <c r="E170" t="inlineStr"/>
       <c r="F170" t="inlineStr">
@@ -3849,13 +3849,13 @@
         <v>46219</v>
       </c>
       <c r="B171" t="n">
-        <v>629</v>
+        <v>1756</v>
       </c>
       <c r="C171" t="n">
         <v>8888</v>
       </c>
       <c r="D171" t="n">
-        <v>10075.2</v>
+        <v>462.4</v>
       </c>
       <c r="E171" t="inlineStr"/>
       <c r="F171" t="inlineStr">
@@ -3869,13 +3869,13 @@
         <v>46219</v>
       </c>
       <c r="B172" t="n">
-        <v>360</v>
+        <v>571</v>
       </c>
       <c r="C172" t="n">
         <v>8888</v>
       </c>
       <c r="D172" t="n">
-        <v>4617.15</v>
+        <v>1125.6</v>
       </c>
       <c r="E172" t="inlineStr"/>
       <c r="F172" t="inlineStr">
@@ -3889,13 +3889,13 @@
         <v>46219</v>
       </c>
       <c r="B173" t="n">
-        <v>609</v>
+        <v>571</v>
       </c>
       <c r="C173" t="n">
         <v>8888</v>
       </c>
       <c r="D173" t="n">
-        <v>1112.69</v>
+        <v>5997.18</v>
       </c>
       <c r="E173" t="inlineStr"/>
       <c r="F173" t="inlineStr">
@@ -3909,18 +3909,18 @@
         <v>46219</v>
       </c>
       <c r="B174" t="n">
-        <v>2250</v>
+        <v>2421</v>
       </c>
       <c r="C174" t="n">
         <v>8888</v>
       </c>
       <c r="D174" t="n">
-        <v>2681.88</v>
+        <v>2786.14</v>
       </c>
       <c r="E174" t="inlineStr"/>
       <c r="F174" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3929,13 +3929,13 @@
         <v>46219</v>
       </c>
       <c r="B175" t="n">
-        <v>535</v>
+        <v>953</v>
       </c>
       <c r="C175" t="n">
         <v>8888</v>
       </c>
       <c r="D175" t="n">
-        <v>616.54</v>
+        <v>6995.34</v>
       </c>
       <c r="E175" t="inlineStr"/>
       <c r="F175" t="inlineStr">
@@ -3949,18 +3949,18 @@
         <v>46219</v>
       </c>
       <c r="B176" t="n">
-        <v>629</v>
+        <v>2769</v>
       </c>
       <c r="C176" t="n">
         <v>8888</v>
       </c>
       <c r="D176" t="n">
-        <v>801.97</v>
+        <v>620.37</v>
       </c>
       <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -3969,18 +3969,18 @@
         <v>46219</v>
       </c>
       <c r="B177" t="n">
-        <v>363</v>
+        <v>2362</v>
       </c>
       <c r="C177" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D177" t="n">
-        <v>1618.96</v>
+        <v>8080.76</v>
       </c>
       <c r="E177" t="inlineStr"/>
       <c r="F177" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -3989,18 +3989,18 @@
         <v>46219</v>
       </c>
       <c r="B178" t="n">
-        <v>1064</v>
+        <v>629</v>
       </c>
       <c r="C178" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D178" t="n">
-        <v>2667.18</v>
+        <v>10075.2</v>
       </c>
       <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4009,13 +4009,13 @@
         <v>46219</v>
       </c>
       <c r="B179" t="n">
-        <v>609</v>
+        <v>360</v>
       </c>
       <c r="C179" t="n">
         <v>8888</v>
       </c>
       <c r="D179" t="n">
-        <v>1141.32</v>
+        <v>4617.15</v>
       </c>
       <c r="E179" t="inlineStr"/>
       <c r="F179" t="inlineStr">
@@ -4029,18 +4029,18 @@
         <v>46219</v>
       </c>
       <c r="B180" t="n">
-        <v>2250</v>
+        <v>609</v>
       </c>
       <c r="C180" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D180" t="n">
-        <v>551.76</v>
+        <v>1112.69</v>
       </c>
       <c r="E180" t="inlineStr"/>
       <c r="F180" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4049,18 +4049,18 @@
         <v>46219</v>
       </c>
       <c r="B181" t="n">
-        <v>953</v>
+        <v>2250</v>
       </c>
       <c r="C181" t="n">
         <v>8888</v>
       </c>
       <c r="D181" t="n">
-        <v>4366.21</v>
+        <v>2681.88</v>
       </c>
       <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4069,13 +4069,13 @@
         <v>46219</v>
       </c>
       <c r="B182" t="n">
-        <v>629</v>
+        <v>535</v>
       </c>
       <c r="C182" t="n">
         <v>8888</v>
       </c>
       <c r="D182" t="n">
-        <v>1844.39</v>
+        <v>616.54</v>
       </c>
       <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr">
@@ -4089,13 +4089,13 @@
         <v>46219</v>
       </c>
       <c r="B183" t="n">
-        <v>1465</v>
+        <v>629</v>
       </c>
       <c r="C183" t="n">
         <v>8888</v>
       </c>
       <c r="D183" t="n">
-        <v>1220.4</v>
+        <v>801.97</v>
       </c>
       <c r="E183" t="inlineStr"/>
       <c r="F183" t="inlineStr">
@@ -4109,18 +4109,18 @@
         <v>46219</v>
       </c>
       <c r="B184" t="n">
-        <v>1869</v>
+        <v>363</v>
       </c>
       <c r="C184" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D184" t="n">
-        <v>1103.52</v>
+        <v>1618.96</v>
       </c>
       <c r="E184" t="inlineStr"/>
       <c r="F184" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4129,18 +4129,18 @@
         <v>46219</v>
       </c>
       <c r="B185" t="n">
-        <v>2362</v>
+        <v>1064</v>
       </c>
       <c r="C185" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D185" t="n">
-        <v>3256.49</v>
+        <v>2667.18</v>
       </c>
       <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4149,13 +4149,13 @@
         <v>46219</v>
       </c>
       <c r="B186" t="n">
-        <v>2362</v>
+        <v>609</v>
       </c>
       <c r="C186" t="n">
         <v>8888</v>
       </c>
       <c r="D186" t="n">
-        <v>702.5700000000001</v>
+        <v>1141.32</v>
       </c>
       <c r="E186" t="inlineStr"/>
       <c r="F186" t="inlineStr">
@@ -4169,18 +4169,18 @@
         <v>46219</v>
       </c>
       <c r="B187" t="n">
-        <v>2652</v>
+        <v>2250</v>
       </c>
       <c r="C187" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D187" t="n">
-        <v>260.03</v>
+        <v>551.76</v>
       </c>
       <c r="E187" t="inlineStr"/>
       <c r="F187" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4189,13 +4189,13 @@
         <v>46219</v>
       </c>
       <c r="B188" t="n">
-        <v>1465</v>
+        <v>953</v>
       </c>
       <c r="C188" t="n">
         <v>8888</v>
       </c>
       <c r="D188" t="n">
-        <v>3283.11</v>
+        <v>4366.21</v>
       </c>
       <c r="E188" t="inlineStr"/>
       <c r="F188" t="inlineStr">
@@ -4209,13 +4209,13 @@
         <v>46219</v>
       </c>
       <c r="B189" t="n">
-        <v>131</v>
+        <v>629</v>
       </c>
       <c r="C189" t="n">
         <v>8888</v>
       </c>
       <c r="D189" t="n">
-        <v>233.82</v>
+        <v>1844.39</v>
       </c>
       <c r="E189" t="inlineStr"/>
       <c r="F189" t="inlineStr">
@@ -4229,13 +4229,13 @@
         <v>46219</v>
       </c>
       <c r="B190" t="n">
-        <v>890</v>
+        <v>1465</v>
       </c>
       <c r="C190" t="n">
         <v>8888</v>
       </c>
       <c r="D190" t="n">
-        <v>950.1799999999999</v>
+        <v>1220.4</v>
       </c>
       <c r="E190" t="inlineStr"/>
       <c r="F190" t="inlineStr">
@@ -4249,13 +4249,13 @@
         <v>46219</v>
       </c>
       <c r="B191" t="n">
-        <v>2250</v>
+        <v>1869</v>
       </c>
       <c r="C191" t="n">
         <v>8888</v>
       </c>
       <c r="D191" t="n">
-        <v>1596</v>
+        <v>1103.52</v>
       </c>
       <c r="E191" t="inlineStr"/>
       <c r="F191" t="inlineStr">
@@ -4269,18 +4269,18 @@
         <v>46219</v>
       </c>
       <c r="B192" t="n">
-        <v>2250</v>
+        <v>2362</v>
       </c>
       <c r="C192" t="n">
-        <v>27</v>
+        <v>8888</v>
       </c>
       <c r="D192" t="n">
-        <v>2207.04</v>
+        <v>3256.49</v>
       </c>
       <c r="E192" t="inlineStr"/>
       <c r="F192" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4289,13 +4289,13 @@
         <v>46219</v>
       </c>
       <c r="B193" t="n">
-        <v>559</v>
+        <v>2362</v>
       </c>
       <c r="C193" t="n">
         <v>8888</v>
       </c>
       <c r="D193" t="n">
-        <v>3594</v>
+        <v>702.5700000000001</v>
       </c>
       <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr">
@@ -4309,13 +4309,13 @@
         <v>46219</v>
       </c>
       <c r="B194" t="n">
-        <v>629</v>
+        <v>2652</v>
       </c>
       <c r="C194" t="n">
         <v>8888</v>
       </c>
       <c r="D194" t="n">
-        <v>801.97</v>
+        <v>260.03</v>
       </c>
       <c r="E194" t="inlineStr"/>
       <c r="F194" t="inlineStr">
@@ -4329,13 +4329,13 @@
         <v>46219</v>
       </c>
       <c r="B195" t="n">
-        <v>58</v>
+        <v>1465</v>
       </c>
       <c r="C195" t="n">
         <v>8888</v>
       </c>
       <c r="D195" t="n">
-        <v>697.33</v>
+        <v>3283.11</v>
       </c>
       <c r="E195" t="inlineStr"/>
       <c r="F195" t="inlineStr">
@@ -4349,18 +4349,18 @@
         <v>46219</v>
       </c>
       <c r="B196" t="n">
-        <v>1108</v>
+        <v>131</v>
       </c>
       <c r="C196" t="n">
         <v>8888</v>
       </c>
       <c r="D196" t="n">
-        <v>341.38</v>
+        <v>233.82</v>
       </c>
       <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4369,13 +4369,13 @@
         <v>46219</v>
       </c>
       <c r="B197" t="n">
-        <v>2363</v>
+        <v>890</v>
       </c>
       <c r="C197" t="n">
         <v>8888</v>
       </c>
       <c r="D197" t="n">
-        <v>1884.86</v>
+        <v>950.1799999999999</v>
       </c>
       <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr">
@@ -4389,13 +4389,13 @@
         <v>46219</v>
       </c>
       <c r="B198" t="n">
-        <v>1007</v>
+        <v>2250</v>
       </c>
       <c r="C198" t="n">
         <v>8888</v>
       </c>
       <c r="D198" t="n">
-        <v>1054.68</v>
+        <v>1596</v>
       </c>
       <c r="E198" t="inlineStr"/>
       <c r="F198" t="inlineStr">
@@ -4409,18 +4409,18 @@
         <v>46219</v>
       </c>
       <c r="B199" t="n">
-        <v>1869</v>
+        <v>2250</v>
       </c>
       <c r="C199" t="n">
-        <v>8888</v>
+        <v>27</v>
       </c>
       <c r="D199" t="n">
-        <v>1698.3</v>
+        <v>2207.04</v>
       </c>
       <c r="E199" t="inlineStr"/>
       <c r="F199" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4429,18 +4429,18 @@
         <v>46219</v>
       </c>
       <c r="B200" t="n">
-        <v>1996</v>
+        <v>559</v>
       </c>
       <c r="C200" t="n">
-        <v>691</v>
+        <v>8888</v>
       </c>
       <c r="D200" t="n">
-        <v>2302.2</v>
+        <v>3594</v>
       </c>
       <c r="E200" t="inlineStr"/>
       <c r="F200" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4449,18 +4449,18 @@
         <v>46219</v>
       </c>
       <c r="B201" t="n">
-        <v>2709</v>
+        <v>629</v>
       </c>
       <c r="C201" t="n">
-        <v>2220</v>
+        <v>8888</v>
       </c>
       <c r="D201" t="n">
-        <v>586.1900000000001</v>
+        <v>801.97</v>
       </c>
       <c r="E201" t="inlineStr"/>
       <c r="F201" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4469,13 +4469,13 @@
         <v>46219</v>
       </c>
       <c r="B202" t="n">
-        <v>1064</v>
+        <v>58</v>
       </c>
       <c r="C202" t="n">
         <v>8888</v>
       </c>
       <c r="D202" t="n">
-        <v>372.95</v>
+        <v>697.33</v>
       </c>
       <c r="E202" t="inlineStr"/>
       <c r="F202" t="inlineStr">
@@ -4489,18 +4489,18 @@
         <v>46219</v>
       </c>
       <c r="B203" t="n">
-        <v>40</v>
+        <v>1108</v>
       </c>
       <c r="C203" t="n">
         <v>8888</v>
       </c>
       <c r="D203" t="n">
-        <v>306.58</v>
+        <v>341.38</v>
       </c>
       <c r="E203" t="inlineStr"/>
       <c r="F203" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4509,18 +4509,18 @@
         <v>46219</v>
       </c>
       <c r="B204" t="n">
-        <v>1996</v>
+        <v>2363</v>
       </c>
       <c r="C204" t="n">
         <v>8888</v>
       </c>
       <c r="D204" t="n">
-        <v>514.91</v>
+        <v>1884.86</v>
       </c>
       <c r="E204" t="inlineStr"/>
       <c r="F204" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4529,13 +4529,13 @@
         <v>46219</v>
       </c>
       <c r="B205" t="n">
-        <v>20</v>
+        <v>1007</v>
       </c>
       <c r="C205" t="n">
         <v>8888</v>
       </c>
       <c r="D205" t="n">
-        <v>680.4</v>
+        <v>1054.68</v>
       </c>
       <c r="E205" t="inlineStr"/>
       <c r="F205" t="inlineStr">
@@ -4549,13 +4549,13 @@
         <v>46219</v>
       </c>
       <c r="B206" t="n">
-        <v>2190</v>
+        <v>1869</v>
       </c>
       <c r="C206" t="n">
         <v>8888</v>
       </c>
       <c r="D206" t="n">
-        <v>1035.41</v>
+        <v>1698.3</v>
       </c>
       <c r="E206" t="inlineStr"/>
       <c r="F206" t="inlineStr">
@@ -4569,18 +4569,18 @@
         <v>46219</v>
       </c>
       <c r="B207" t="n">
-        <v>781</v>
+        <v>1996</v>
       </c>
       <c r="C207" t="n">
-        <v>8888</v>
+        <v>691</v>
       </c>
       <c r="D207" t="n">
-        <v>1169.2</v>
+        <v>2302.2</v>
       </c>
       <c r="E207" t="inlineStr"/>
       <c r="F207" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4589,18 +4589,18 @@
         <v>46219</v>
       </c>
       <c r="B208" t="n">
-        <v>351</v>
+        <v>2709</v>
       </c>
       <c r="C208" t="n">
-        <v>8888</v>
+        <v>2220</v>
       </c>
       <c r="D208" t="n">
-        <v>2207.04</v>
+        <v>586.1900000000001</v>
       </c>
       <c r="E208" t="inlineStr"/>
       <c r="F208" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -4615,7 +4615,7 @@
         <v>8888</v>
       </c>
       <c r="D209" t="n">
-        <v>2348.64</v>
+        <v>372.95</v>
       </c>
       <c r="E209" t="inlineStr"/>
       <c r="F209" t="inlineStr">
@@ -4629,13 +4629,13 @@
         <v>46219</v>
       </c>
       <c r="B210" t="n">
-        <v>571</v>
+        <v>40</v>
       </c>
       <c r="C210" t="n">
         <v>8888</v>
       </c>
       <c r="D210" t="n">
-        <v>17843.18</v>
+        <v>306.58</v>
       </c>
       <c r="E210" t="inlineStr"/>
       <c r="F210" t="inlineStr">
@@ -4649,18 +4649,18 @@
         <v>46219</v>
       </c>
       <c r="B211" t="n">
-        <v>629</v>
+        <v>1996</v>
       </c>
       <c r="C211" t="n">
         <v>8888</v>
       </c>
       <c r="D211" t="n">
-        <v>1292.86</v>
+        <v>514.91</v>
       </c>
       <c r="E211" t="inlineStr"/>
       <c r="F211" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4669,13 +4669,13 @@
         <v>46219</v>
       </c>
       <c r="B212" t="n">
-        <v>535</v>
+        <v>20</v>
       </c>
       <c r="C212" t="n">
         <v>8888</v>
       </c>
       <c r="D212" t="n">
-        <v>1395.11</v>
+        <v>680.4</v>
       </c>
       <c r="E212" t="inlineStr"/>
       <c r="F212" t="inlineStr">
@@ -4689,13 +4689,13 @@
         <v>46219</v>
       </c>
       <c r="B213" t="n">
-        <v>609</v>
+        <v>2190</v>
       </c>
       <c r="C213" t="n">
         <v>8888</v>
       </c>
       <c r="D213" t="n">
-        <v>1487.52</v>
+        <v>1035.41</v>
       </c>
       <c r="E213" t="inlineStr"/>
       <c r="F213" t="inlineStr">
@@ -4709,13 +4709,13 @@
         <v>46219</v>
       </c>
       <c r="B214" t="n">
-        <v>609</v>
+        <v>781</v>
       </c>
       <c r="C214" t="n">
         <v>8888</v>
       </c>
       <c r="D214" t="n">
-        <v>1854.48</v>
+        <v>1169.2</v>
       </c>
       <c r="E214" t="inlineStr"/>
       <c r="F214" t="inlineStr">
@@ -4729,13 +4729,13 @@
         <v>46219</v>
       </c>
       <c r="B215" t="n">
-        <v>2660</v>
+        <v>351</v>
       </c>
       <c r="C215" t="n">
         <v>8888</v>
       </c>
       <c r="D215" t="n">
-        <v>1481.24</v>
+        <v>2207.04</v>
       </c>
       <c r="E215" t="inlineStr"/>
       <c r="F215" t="inlineStr">
@@ -4749,13 +4749,13 @@
         <v>46219</v>
       </c>
       <c r="B216" t="n">
-        <v>1293</v>
+        <v>1064</v>
       </c>
       <c r="C216" t="n">
         <v>8888</v>
       </c>
       <c r="D216" t="n">
-        <v>1354.46</v>
+        <v>2348.64</v>
       </c>
       <c r="E216" t="inlineStr"/>
       <c r="F216" t="inlineStr">
@@ -4769,13 +4769,13 @@
         <v>46219</v>
       </c>
       <c r="B217" t="n">
-        <v>2768</v>
+        <v>571</v>
       </c>
       <c r="C217" t="n">
         <v>8888</v>
       </c>
       <c r="D217" t="n">
-        <v>2979.54</v>
+        <v>17843.18</v>
       </c>
       <c r="E217" t="inlineStr"/>
       <c r="F217" t="inlineStr">
@@ -4789,13 +4789,13 @@
         <v>46219</v>
       </c>
       <c r="B218" t="n">
-        <v>1327</v>
+        <v>629</v>
       </c>
       <c r="C218" t="n">
         <v>8888</v>
       </c>
       <c r="D218" t="n">
-        <v>4134.3</v>
+        <v>1292.86</v>
       </c>
       <c r="E218" t="inlineStr"/>
       <c r="F218" t="inlineStr">
@@ -4809,18 +4809,18 @@
         <v>46219</v>
       </c>
       <c r="B219" t="n">
-        <v>2628</v>
+        <v>535</v>
       </c>
       <c r="C219" t="n">
         <v>8888</v>
       </c>
       <c r="D219" t="n">
-        <v>271.2</v>
+        <v>1395.11</v>
       </c>
       <c r="E219" t="inlineStr"/>
       <c r="F219" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -4829,13 +4829,13 @@
         <v>46219</v>
       </c>
       <c r="B220" t="n">
-        <v>2452</v>
+        <v>609</v>
       </c>
       <c r="C220" t="n">
         <v>8888</v>
       </c>
       <c r="D220" t="n">
-        <v>1208.26</v>
+        <v>1487.52</v>
       </c>
       <c r="E220" t="inlineStr"/>
       <c r="F220" t="inlineStr">
@@ -4849,13 +4849,13 @@
         <v>46219</v>
       </c>
       <c r="B221" t="n">
-        <v>131</v>
+        <v>609</v>
       </c>
       <c r="C221" t="n">
         <v>8888</v>
       </c>
       <c r="D221" t="n">
-        <v>848.54</v>
+        <v>1854.48</v>
       </c>
       <c r="E221" t="inlineStr"/>
       <c r="F221" t="inlineStr">
@@ -4869,13 +4869,13 @@
         <v>46219</v>
       </c>
       <c r="B222" t="n">
-        <v>816</v>
+        <v>2660</v>
       </c>
       <c r="C222" t="n">
         <v>8888</v>
       </c>
       <c r="D222" t="n">
-        <v>4017.6</v>
+        <v>1481.24</v>
       </c>
       <c r="E222" t="inlineStr"/>
       <c r="F222" t="inlineStr">
@@ -4889,13 +4889,13 @@
         <v>46219</v>
       </c>
       <c r="B223" t="n">
-        <v>1064</v>
+        <v>1293</v>
       </c>
       <c r="C223" t="n">
         <v>8888</v>
       </c>
       <c r="D223" t="n">
-        <v>4291.42</v>
+        <v>1354.46</v>
       </c>
       <c r="E223" t="inlineStr"/>
       <c r="F223" t="inlineStr">
@@ -4909,13 +4909,13 @@
         <v>46219</v>
       </c>
       <c r="B224" t="n">
-        <v>703</v>
+        <v>2768</v>
       </c>
       <c r="C224" t="n">
         <v>8888</v>
       </c>
       <c r="D224" t="n">
-        <v>3936.87</v>
+        <v>2979.54</v>
       </c>
       <c r="E224" t="inlineStr"/>
       <c r="F224" t="inlineStr">
@@ -4929,13 +4929,13 @@
         <v>46219</v>
       </c>
       <c r="B225" t="n">
-        <v>1340</v>
+        <v>1327</v>
       </c>
       <c r="C225" t="n">
         <v>8888</v>
       </c>
       <c r="D225" t="n">
-        <v>2774.78</v>
+        <v>4134.3</v>
       </c>
       <c r="E225" t="inlineStr"/>
       <c r="F225" t="inlineStr">
@@ -4949,18 +4949,18 @@
         <v>46219</v>
       </c>
       <c r="B226" t="n">
-        <v>2107</v>
+        <v>2628</v>
       </c>
       <c r="C226" t="n">
         <v>8888</v>
       </c>
       <c r="D226" t="n">
-        <v>476.47</v>
+        <v>271.2</v>
       </c>
       <c r="E226" t="inlineStr"/>
       <c r="F226" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -4969,13 +4969,13 @@
         <v>46219</v>
       </c>
       <c r="B227" t="n">
-        <v>400</v>
+        <v>2452</v>
       </c>
       <c r="C227" t="n">
         <v>8888</v>
       </c>
       <c r="D227" t="n">
-        <v>2686.56</v>
+        <v>1208.26</v>
       </c>
       <c r="E227" t="inlineStr"/>
       <c r="F227" t="inlineStr">
@@ -4989,13 +4989,13 @@
         <v>46219</v>
       </c>
       <c r="B228" t="n">
-        <v>559</v>
+        <v>131</v>
       </c>
       <c r="C228" t="n">
         <v>8888</v>
       </c>
       <c r="D228" t="n">
-        <v>9867.299999999999</v>
+        <v>848.54</v>
       </c>
       <c r="E228" t="inlineStr"/>
       <c r="F228" t="inlineStr">
@@ -5009,13 +5009,13 @@
         <v>46219</v>
       </c>
       <c r="B229" t="n">
-        <v>951</v>
+        <v>816</v>
       </c>
       <c r="C229" t="n">
         <v>8888</v>
       </c>
       <c r="D229" t="n">
-        <v>6068.2</v>
+        <v>4017.6</v>
       </c>
       <c r="E229" t="inlineStr"/>
       <c r="F229" t="inlineStr">
@@ -5029,13 +5029,13 @@
         <v>46219</v>
       </c>
       <c r="B230" t="n">
-        <v>571</v>
+        <v>1064</v>
       </c>
       <c r="C230" t="n">
         <v>8888</v>
       </c>
       <c r="D230" t="n">
-        <v>4547.53</v>
+        <v>4291.42</v>
       </c>
       <c r="E230" t="inlineStr"/>
       <c r="F230" t="inlineStr">
@@ -5049,18 +5049,18 @@
         <v>46219</v>
       </c>
       <c r="B231" t="n">
-        <v>1450</v>
+        <v>703</v>
       </c>
       <c r="C231" t="n">
         <v>8888</v>
       </c>
       <c r="D231" t="n">
-        <v>692.3200000000001</v>
+        <v>3936.87</v>
       </c>
       <c r="E231" t="inlineStr"/>
       <c r="F231" t="inlineStr">
         <is>
-          <t>E-COMMERCE</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5069,18 +5069,18 @@
         <v>46219</v>
       </c>
       <c r="B232" t="n">
-        <v>2767</v>
+        <v>1340</v>
       </c>
       <c r="C232" t="n">
-        <v>1898</v>
+        <v>8888</v>
       </c>
       <c r="D232" t="n">
-        <v>1706.73</v>
+        <v>2774.78</v>
       </c>
       <c r="E232" t="inlineStr"/>
       <c r="F232" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5089,18 +5089,18 @@
         <v>46219</v>
       </c>
       <c r="B233" t="n">
-        <v>2810</v>
+        <v>2107</v>
       </c>
       <c r="C233" t="n">
-        <v>3179</v>
+        <v>8888</v>
       </c>
       <c r="D233" t="n">
-        <v>3704.73</v>
+        <v>476.47</v>
       </c>
       <c r="E233" t="inlineStr"/>
       <c r="F233" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5109,13 +5109,13 @@
         <v>46219</v>
       </c>
       <c r="B234" t="n">
-        <v>2452</v>
+        <v>400</v>
       </c>
       <c r="C234" t="n">
         <v>8888</v>
       </c>
       <c r="D234" t="n">
-        <v>1093.58</v>
+        <v>2686.56</v>
       </c>
       <c r="E234" t="inlineStr"/>
       <c r="F234" t="inlineStr">
@@ -5129,13 +5129,13 @@
         <v>46219</v>
       </c>
       <c r="B235" t="n">
-        <v>703</v>
+        <v>559</v>
       </c>
       <c r="C235" t="n">
         <v>8888</v>
       </c>
       <c r="D235" t="n">
-        <v>1829.63</v>
+        <v>9867.299999999999</v>
       </c>
       <c r="E235" t="inlineStr"/>
       <c r="F235" t="inlineStr">
@@ -5149,13 +5149,13 @@
         <v>46219</v>
       </c>
       <c r="B236" t="n">
-        <v>609</v>
+        <v>451</v>
       </c>
       <c r="C236" t="n">
         <v>8888</v>
       </c>
       <c r="D236" t="n">
-        <v>1112.69</v>
+        <v>2131.88</v>
       </c>
       <c r="E236" t="inlineStr"/>
       <c r="F236" t="inlineStr">
@@ -5169,13 +5169,13 @@
         <v>46219</v>
       </c>
       <c r="B237" t="n">
-        <v>2245</v>
+        <v>951</v>
       </c>
       <c r="C237" t="n">
         <v>8888</v>
       </c>
       <c r="D237" t="n">
-        <v>459.01</v>
+        <v>6068.2</v>
       </c>
       <c r="E237" t="inlineStr"/>
       <c r="F237" t="inlineStr">
@@ -5189,13 +5189,13 @@
         <v>46219</v>
       </c>
       <c r="B238" t="n">
-        <v>131</v>
+        <v>571</v>
       </c>
       <c r="C238" t="n">
         <v>8888</v>
       </c>
       <c r="D238" t="n">
-        <v>623.52</v>
+        <v>4547.53</v>
       </c>
       <c r="E238" t="inlineStr"/>
       <c r="F238" t="inlineStr">
@@ -5209,18 +5209,18 @@
         <v>46219</v>
       </c>
       <c r="B239" t="n">
-        <v>429</v>
+        <v>619</v>
       </c>
       <c r="C239" t="n">
-        <v>1281</v>
+        <v>8888</v>
       </c>
       <c r="D239" t="n">
-        <v>376.24</v>
+        <v>1872.16</v>
       </c>
       <c r="E239" t="inlineStr"/>
       <c r="F239" t="inlineStr">
         <is>
-          <t>TELEMARKETING</t>
+          <t>FORÇA DE VENDAS</t>
         </is>
       </c>
     </row>
@@ -5229,18 +5229,18 @@
         <v>46219</v>
       </c>
       <c r="B240" t="n">
-        <v>131</v>
+        <v>1450</v>
       </c>
       <c r="C240" t="n">
         <v>8888</v>
       </c>
       <c r="D240" t="n">
-        <v>909.3</v>
+        <v>692.3200000000001</v>
       </c>
       <c r="E240" t="inlineStr"/>
       <c r="F240" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>E-COMMERCE</t>
         </is>
       </c>
     </row>
@@ -5249,18 +5249,18 @@
         <v>46219</v>
       </c>
       <c r="B241" t="n">
-        <v>1465</v>
+        <v>2767</v>
       </c>
       <c r="C241" t="n">
-        <v>8888</v>
+        <v>1898</v>
       </c>
       <c r="D241" t="n">
-        <v>3044.97</v>
+        <v>1706.73</v>
       </c>
       <c r="E241" t="inlineStr"/>
       <c r="F241" t="inlineStr">
         <is>
-          <t>FORÇA DE VENDAS</t>
+          <t>TELEMARKETING</t>
         </is>
       </c>
     </row>
@@ -5269,13 +5269,13 @@
         <v>46219</v>
       </c>
       <c r="B242" t="n">
-        <v>1518</v>
+        <v>2810</v>
       </c>
       <c r="C242" t="n">
-        <v>1533</v>
+        <v>3179</v>
       </c>
       <c r="D242" t="n">
-        <v>3838.97</v>
+        <v>3704.73</v>
       </c>
       <c r="E242" t="inlineStr"/>
       <c r="F242" t="inlineStr">
@@ -5289,13 +5289,13 @@
         <v>46219</v>
       </c>
       <c r="B243" t="n">
-        <v>1756</v>
+        <v>2452</v>
       </c>
       <c r="C243" t="n">
         <v>8888</v>
       </c>
       <c r="D243" t="n">
-        <v>1283.28</v>
+        <v>1093.58</v>
       </c>
       <c r="E243" t="inlineStr"/>
       <c r="F243" t="inlineStr">
@@ -5309,13 +5309,13 @@
         <v>46219</v>
       </c>
       <c r="B244" t="n">
-        <v>131</v>
+        <v>703</v>
       </c>
       <c r="C244" t="n">
         <v>8888</v>
       </c>
       <c r="D244" t="n">
-        <v>1035.73</v>
+        <v>1829.63</v>
       </c>
       <c r="E244" t="inlineStr"/>
       <c r="F244" t="inlineStr">
@@ -5329,13 +5329,13 @@
         <v>46219</v>
       </c>
       <c r="B245" t="n">
-        <v>629</v>
+        <v>609</v>
       </c>
       <c r="C245" t="n">
         <v>8888</v>
       </c>
       <c r="D245" t="n">
-        <v>2645.87</v>
+        <v>1112.69</v>
       </c>
       <c r="E245" t="inlineStr"/>
       <c r="F245" t="inlineStr">
@@ -5349,13 +5349,13 @@
         <v>46219</v>
       </c>
       <c r="B246" t="n">
-        <v>351</v>
+        <v>2245</v>
       </c>
       <c r="C246" t="n">
         <v>8888</v>
       </c>
       <c r="D246" t="n">
-        <v>3018</v>
+        <v>459.01</v>
       </c>
       <c r="E246" t="inlineStr"/>
       <c r="F246" t="inlineStr">
@@ -5369,13 +5369,13 @@
         <v>46219</v>
       </c>
       <c r="B247" t="n">
-        <v>400</v>
+        <v>131</v>
       </c>
       <c r="C247" t="n">
         <v>8888</v>
       </c>
       <c r="D247" t="n">
-        <v>688.64</v>
+        <v>623.52</v>
       </c>
       <c r="E247" t="inlineStr"/>
       <c r="F247" t="inlineStr">
@@ -5389,16 +5389,196 @@
         <v>46219</v>
       </c>
       <c r="B248" t="n">
-        <v>1324</v>
+        <v>429</v>
       </c>
       <c r="C248" t="n">
-        <v>3009</v>
+        <v>1281</v>
       </c>
       <c r="D248" t="n">
-        <v>680.4</v>
+        <v>376.24</v>
       </c>
       <c r="E248" t="inlineStr"/>
       <c r="F248" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B249" t="n">
+        <v>131</v>
+      </c>
+      <c r="C249" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D249" t="n">
+        <v>909.3</v>
+      </c>
+      <c r="E249" t="inlineStr"/>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B250" t="n">
+        <v>1465</v>
+      </c>
+      <c r="C250" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D250" t="n">
+        <v>3044.97</v>
+      </c>
+      <c r="E250" t="inlineStr"/>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B251" t="n">
+        <v>1518</v>
+      </c>
+      <c r="C251" t="n">
+        <v>1533</v>
+      </c>
+      <c r="D251" t="n">
+        <v>3838.97</v>
+      </c>
+      <c r="E251" t="inlineStr"/>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>TELEMARKETING</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B252" t="n">
+        <v>1756</v>
+      </c>
+      <c r="C252" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D252" t="n">
+        <v>1283.28</v>
+      </c>
+      <c r="E252" t="inlineStr"/>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B253" t="n">
+        <v>131</v>
+      </c>
+      <c r="C253" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D253" t="n">
+        <v>1035.73</v>
+      </c>
+      <c r="E253" t="inlineStr"/>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B254" t="n">
+        <v>629</v>
+      </c>
+      <c r="C254" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D254" t="n">
+        <v>2645.87</v>
+      </c>
+      <c r="E254" t="inlineStr"/>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B255" t="n">
+        <v>351</v>
+      </c>
+      <c r="C255" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D255" t="n">
+        <v>3018</v>
+      </c>
+      <c r="E255" t="inlineStr"/>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B256" t="n">
+        <v>400</v>
+      </c>
+      <c r="C256" t="n">
+        <v>8888</v>
+      </c>
+      <c r="D256" t="n">
+        <v>688.64</v>
+      </c>
+      <c r="E256" t="inlineStr"/>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>FORÇA DE VENDAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B257" t="n">
+        <v>1324</v>
+      </c>
+      <c r="C257" t="n">
+        <v>3009</v>
+      </c>
+      <c r="D257" t="n">
+        <v>680.4</v>
+      </c>
+      <c r="E257" t="inlineStr"/>
+      <c r="F257" t="inlineStr">
         <is>
           <t>TELEMARKETING</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 11:00:04
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F197"/>
+  <dimension ref="A1:F202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,7 +506,7 @@
         <v>47252</v>
       </c>
       <c r="E3" t="n">
-        <v>3418.8</v>
+        <v>3734.77</v>
       </c>
       <c r="F3" t="n">
         <v>688.0700000000001</v>
@@ -530,7 +530,7 @@
         <v>30791</v>
       </c>
       <c r="E4" t="n">
-        <v>7297.39</v>
+        <v>7538.9</v>
       </c>
       <c r="F4" t="n">
         <v>3111.54</v>
@@ -578,7 +578,7 @@
         <v>31267</v>
       </c>
       <c r="E6" t="n">
-        <v>6708.35</v>
+        <v>7318.24</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -629,7 +629,7 @@
         <v>724.89</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>47.94</v>
       </c>
     </row>
     <row r="9">
@@ -794,7 +794,7 @@
         <v>794671</v>
       </c>
       <c r="E15" t="n">
-        <v>88.31999999999999</v>
+        <v>1092.65</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -842,7 +842,7 @@
         <v>30307</v>
       </c>
       <c r="E17" t="n">
-        <v>34077.35</v>
+        <v>34619.75</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -914,7 +914,7 @@
         <v>31267</v>
       </c>
       <c r="E20" t="n">
-        <v>36921.85</v>
+        <v>47896.88</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -1163,22 +1163,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D31" t="n">
-        <v>789228</v>
+        <v>792121</v>
       </c>
       <c r="E31" t="n">
-        <v>17.46</v>
+        <v>394.84</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
@@ -1187,22 +1187,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D32" t="n">
-        <v>30083</v>
+        <v>789228</v>
       </c>
       <c r="E32" t="n">
-        <v>148.02</v>
+        <v>17.46</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -1211,22 +1211,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D33" t="n">
-        <v>30307</v>
+        <v>30083</v>
       </c>
       <c r="E33" t="n">
-        <v>257.12</v>
+        <v>148.02</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
@@ -1235,22 +1235,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D34" t="n">
-        <v>789603</v>
+        <v>30307</v>
       </c>
       <c r="E34" t="n">
-        <v>7602.96</v>
+        <v>257.12</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
@@ -1264,17 +1264,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D35" t="n">
-        <v>139553</v>
+        <v>789603</v>
       </c>
       <c r="E35" t="n">
-        <v>3801.14</v>
+        <v>7602.96</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
@@ -1283,25 +1283,25 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D36" t="n">
-        <v>33286</v>
+        <v>139553</v>
       </c>
       <c r="E36" t="n">
-        <v>122.36</v>
+        <v>3801.14</v>
       </c>
       <c r="F36" t="n">
-        <v>91.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -1312,65 +1312,65 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D37" t="n">
-        <v>31267</v>
+        <v>33286</v>
       </c>
       <c r="E37" t="n">
-        <v>255.1</v>
+        <v>122.36</v>
       </c>
       <c r="F37" t="n">
-        <v>165.42</v>
+        <v>91.13</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D38" t="n">
-        <v>47252</v>
+        <v>31267</v>
       </c>
       <c r="E38" t="n">
-        <v>6990.3</v>
+        <v>255.1</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>165.42</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D39" t="n">
-        <v>30307</v>
+        <v>47252</v>
       </c>
       <c r="E39" t="n">
-        <v>6955.69</v>
+        <v>6990.3</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
@@ -1379,22 +1379,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D40" t="n">
-        <v>30791</v>
+        <v>30307</v>
       </c>
       <c r="E40" t="n">
-        <v>4724.47</v>
+        <v>6955.69</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
@@ -1403,94 +1403,94 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D41" t="n">
-        <v>789525</v>
+        <v>30791</v>
       </c>
       <c r="E41" t="n">
-        <v>572.4400000000001</v>
+        <v>4724.47</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>37.57</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D42" t="n">
-        <v>33057</v>
+        <v>789525</v>
       </c>
       <c r="E42" t="n">
-        <v>389.42</v>
+        <v>572.4400000000001</v>
       </c>
       <c r="F42" t="n">
-        <v>97.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>LUIS REGINALDO ALMEIDA GOMES</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D43" t="n">
-        <v>30307</v>
+        <v>33057</v>
       </c>
       <c r="E43" t="n">
-        <v>2807.48</v>
+        <v>389.42</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>97.77</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>LUIS REGINALDO ALMEIDA GOMES</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D44" t="n">
-        <v>789228</v>
+        <v>30307</v>
       </c>
       <c r="E44" t="n">
-        <v>66.72</v>
+        <v>2807.48</v>
       </c>
       <c r="F44" t="n">
         <v>0</v>
@@ -1499,22 +1499,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D45" t="n">
-        <v>789603</v>
+        <v>789228</v>
       </c>
       <c r="E45" t="n">
-        <v>3037.29</v>
+        <v>66.72</v>
       </c>
       <c r="F45" t="n">
         <v>0</v>
@@ -1523,22 +1523,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D46" t="n">
-        <v>32816</v>
+        <v>33928</v>
       </c>
       <c r="E46" t="n">
-        <v>906.71</v>
+        <v>1204.64</v>
       </c>
       <c r="F46" t="n">
         <v>0</v>
@@ -1547,22 +1547,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D47" t="n">
-        <v>33286</v>
+        <v>789603</v>
       </c>
       <c r="E47" t="n">
-        <v>660.86</v>
+        <v>3037.29</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
@@ -1571,22 +1571,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D48" t="n">
-        <v>792141</v>
+        <v>32816</v>
       </c>
       <c r="E48" t="n">
-        <v>65.7</v>
+        <v>906.71</v>
       </c>
       <c r="F48" t="n">
         <v>0</v>
@@ -1595,22 +1595,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D49" t="n">
-        <v>33928</v>
+        <v>33286</v>
       </c>
       <c r="E49" t="n">
-        <v>1028.36</v>
+        <v>888.9400000000001</v>
       </c>
       <c r="F49" t="n">
         <v>0</v>
@@ -1619,22 +1619,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D50" t="n">
-        <v>30307</v>
+        <v>792141</v>
       </c>
       <c r="E50" t="n">
-        <v>326.87</v>
+        <v>65.7</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -1658,7 +1658,7 @@
         <v>30307</v>
       </c>
       <c r="E51" t="n">
-        <v>2484.88</v>
+        <v>326.87</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
@@ -1667,22 +1667,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D52" t="n">
-        <v>795345</v>
+        <v>30307</v>
       </c>
       <c r="E52" t="n">
-        <v>27.29</v>
+        <v>2484.88</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
@@ -1691,22 +1691,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D53" t="n">
-        <v>793718</v>
+        <v>795345</v>
       </c>
       <c r="E53" t="n">
-        <v>48.07</v>
+        <v>27.29</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
@@ -1715,22 +1715,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D54" t="n">
-        <v>795345</v>
+        <v>793718</v>
       </c>
       <c r="E54" t="n">
-        <v>81.95</v>
+        <v>48.07</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
@@ -1751,10 +1751,10 @@
         <v>46247</v>
       </c>
       <c r="D55" t="n">
-        <v>792121</v>
+        <v>795345</v>
       </c>
       <c r="E55" t="n">
-        <v>60.08</v>
+        <v>81.95</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
@@ -1763,22 +1763,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D56" t="n">
-        <v>789603</v>
+        <v>792121</v>
       </c>
       <c r="E56" t="n">
-        <v>368.27</v>
+        <v>60.08</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
@@ -1787,25 +1787,25 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D57" t="n">
-        <v>33286</v>
+        <v>789603</v>
       </c>
       <c r="E57" t="n">
-        <v>480.45</v>
+        <v>368.27</v>
       </c>
       <c r="F57" t="n">
-        <v>230.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -1816,44 +1816,44 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D58" t="n">
-        <v>30791</v>
+        <v>33286</v>
       </c>
       <c r="E58" t="n">
-        <v>5193.38</v>
+        <v>522.75</v>
       </c>
       <c r="F58" t="n">
-        <v>404.46</v>
+        <v>230.41</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D59" t="n">
-        <v>793718</v>
+        <v>30791</v>
       </c>
       <c r="E59" t="n">
-        <v>497.54</v>
+        <v>5266.68</v>
       </c>
       <c r="F59" t="n">
-        <v>0</v>
+        <v>404.46</v>
       </c>
     </row>
     <row r="60">
@@ -1871,10 +1871,10 @@
         <v>46247</v>
       </c>
       <c r="D60" t="n">
-        <v>31267</v>
+        <v>793718</v>
       </c>
       <c r="E60" t="n">
-        <v>65.95</v>
+        <v>497.54</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
@@ -1883,22 +1883,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D61" t="n">
-        <v>33928</v>
+        <v>31267</v>
       </c>
       <c r="E61" t="n">
-        <v>563.1900000000001</v>
+        <v>65.95</v>
       </c>
       <c r="F61" t="n">
         <v>0</v>
@@ -1907,70 +1907,70 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D62" t="n">
-        <v>793718</v>
+        <v>33928</v>
       </c>
       <c r="E62" t="n">
-        <v>523.04</v>
+        <v>563.1900000000001</v>
       </c>
       <c r="F62" t="n">
-        <v>238.95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D63" t="n">
-        <v>139553</v>
+        <v>793718</v>
       </c>
       <c r="E63" t="n">
-        <v>806.96</v>
+        <v>523.04</v>
       </c>
       <c r="F63" t="n">
-        <v>0</v>
+        <v>238.95</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D64" t="n">
-        <v>33057</v>
+        <v>139553</v>
       </c>
       <c r="E64" t="n">
-        <v>39.4</v>
+        <v>806.96</v>
       </c>
       <c r="F64" t="n">
         <v>0</v>
@@ -1979,22 +1979,22 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D65" t="n">
-        <v>33286</v>
+        <v>33057</v>
       </c>
       <c r="E65" t="n">
-        <v>1418.04</v>
+        <v>39.4</v>
       </c>
       <c r="F65" t="n">
         <v>0</v>
@@ -2015,10 +2015,10 @@
         <v>46247</v>
       </c>
       <c r="D66" t="n">
-        <v>33057</v>
+        <v>33286</v>
       </c>
       <c r="E66" t="n">
-        <v>141.95</v>
+        <v>1418.04</v>
       </c>
       <c r="F66" t="n">
         <v>0</v>
@@ -2027,22 +2027,22 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D67" t="n">
-        <v>139553</v>
+        <v>33057</v>
       </c>
       <c r="E67" t="n">
-        <v>8735.299999999999</v>
+        <v>141.95</v>
       </c>
       <c r="F67" t="n">
         <v>0</v>
@@ -2051,22 +2051,22 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D68" t="n">
-        <v>33057</v>
+        <v>139553</v>
       </c>
       <c r="E68" t="n">
-        <v>200.35</v>
+        <v>8735.299999999999</v>
       </c>
       <c r="F68" t="n">
         <v>0</v>
@@ -2090,7 +2090,7 @@
         <v>33286</v>
       </c>
       <c r="E69" t="n">
-        <v>801.75</v>
+        <v>972.64</v>
       </c>
       <c r="F69" t="n">
         <v>0</v>
@@ -2099,22 +2099,22 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D70" t="n">
-        <v>47252</v>
+        <v>33057</v>
       </c>
       <c r="E70" t="n">
-        <v>2729.12</v>
+        <v>200.35</v>
       </c>
       <c r="F70" t="n">
         <v>0</v>
@@ -2123,22 +2123,22 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D71" t="n">
-        <v>792141</v>
+        <v>47252</v>
       </c>
       <c r="E71" t="n">
-        <v>207.9</v>
+        <v>2729.12</v>
       </c>
       <c r="F71" t="n">
         <v>0</v>
@@ -2147,22 +2147,22 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D72" t="n">
-        <v>47252</v>
+        <v>792141</v>
       </c>
       <c r="E72" t="n">
-        <v>952.34</v>
+        <v>207.9</v>
       </c>
       <c r="F72" t="n">
         <v>0</v>
@@ -2171,22 +2171,22 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D73" t="n">
-        <v>794671</v>
+        <v>47252</v>
       </c>
       <c r="E73" t="n">
-        <v>2070.23</v>
+        <v>952.34</v>
       </c>
       <c r="F73" t="n">
         <v>0</v>
@@ -2207,10 +2207,10 @@
         <v>46247</v>
       </c>
       <c r="D74" t="n">
-        <v>792246</v>
+        <v>794671</v>
       </c>
       <c r="E74" t="n">
-        <v>1308.82</v>
+        <v>2431.37</v>
       </c>
       <c r="F74" t="n">
         <v>0</v>
@@ -2224,17 +2224,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D75" t="n">
-        <v>793718</v>
+        <v>792246</v>
       </c>
       <c r="E75" t="n">
-        <v>48.08</v>
+        <v>1308.82</v>
       </c>
       <c r="F75" t="n">
         <v>0</v>
@@ -2243,22 +2243,22 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D76" t="n">
-        <v>32816</v>
+        <v>793718</v>
       </c>
       <c r="E76" t="n">
-        <v>11.9</v>
+        <v>48.08</v>
       </c>
       <c r="F76" t="n">
         <v>0</v>
@@ -2279,10 +2279,10 @@
         <v>46247</v>
       </c>
       <c r="D77" t="n">
-        <v>796582</v>
+        <v>32816</v>
       </c>
       <c r="E77" t="n">
-        <v>2267.86</v>
+        <v>11.9</v>
       </c>
       <c r="F77" t="n">
         <v>0</v>
@@ -2291,22 +2291,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D78" t="n">
-        <v>30307</v>
+        <v>796582</v>
       </c>
       <c r="E78" t="n">
-        <v>20610.6</v>
+        <v>2267.86</v>
       </c>
       <c r="F78" t="n">
         <v>0</v>
@@ -2315,70 +2315,70 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D79" t="n">
-        <v>789525</v>
+        <v>30307</v>
       </c>
       <c r="E79" t="n">
-        <v>1297.24</v>
+        <v>20610.6</v>
       </c>
       <c r="F79" t="n">
-        <v>288.23</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D80" t="n">
-        <v>792121</v>
+        <v>789525</v>
       </c>
       <c r="E80" t="n">
-        <v>4585.49</v>
+        <v>1369.87</v>
       </c>
       <c r="F80" t="n">
-        <v>0</v>
+        <v>288.23</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D81" t="n">
-        <v>33928</v>
+        <v>792121</v>
       </c>
       <c r="E81" t="n">
-        <v>8388.15</v>
+        <v>4585.49</v>
       </c>
       <c r="F81" t="n">
         <v>0</v>
@@ -2387,22 +2387,22 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D82" t="n">
-        <v>33286</v>
+        <v>33928</v>
       </c>
       <c r="E82" t="n">
-        <v>2195.77</v>
+        <v>8388.15</v>
       </c>
       <c r="F82" t="n">
         <v>0</v>
@@ -2411,22 +2411,22 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D83" t="n">
-        <v>795345</v>
+        <v>33286</v>
       </c>
       <c r="E83" t="n">
-        <v>1400.33</v>
+        <v>2548.83</v>
       </c>
       <c r="F83" t="n">
         <v>0</v>
@@ -2440,17 +2440,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D84" t="n">
-        <v>30083</v>
+        <v>795345</v>
       </c>
       <c r="E84" t="n">
-        <v>242.05</v>
+        <v>1400.33</v>
       </c>
       <c r="F84" t="n">
         <v>0</v>
@@ -2459,22 +2459,22 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D85" t="n">
-        <v>33286</v>
+        <v>30083</v>
       </c>
       <c r="E85" t="n">
-        <v>11.82</v>
+        <v>1061.78</v>
       </c>
       <c r="F85" t="n">
         <v>0</v>
@@ -2483,22 +2483,22 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D86" t="n">
-        <v>30307</v>
+        <v>33286</v>
       </c>
       <c r="E86" t="n">
-        <v>41660.27</v>
+        <v>11.82</v>
       </c>
       <c r="F86" t="n">
         <v>0</v>
@@ -2507,22 +2507,22 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D87" t="n">
-        <v>33286</v>
+        <v>30307</v>
       </c>
       <c r="E87" t="n">
-        <v>180.3</v>
+        <v>41660.27</v>
       </c>
       <c r="F87" t="n">
         <v>0</v>
@@ -2531,22 +2531,22 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D88" t="n">
-        <v>794029</v>
+        <v>33928</v>
       </c>
       <c r="E88" t="n">
-        <v>502.13</v>
+        <v>388.73</v>
       </c>
       <c r="F88" t="n">
         <v>0</v>
@@ -2560,17 +2560,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D89" t="n">
-        <v>792246</v>
+        <v>33286</v>
       </c>
       <c r="E89" t="n">
-        <v>1040.43</v>
+        <v>180.3</v>
       </c>
       <c r="F89" t="n">
         <v>0</v>
@@ -2579,22 +2579,22 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D90" t="n">
-        <v>789603</v>
+        <v>794029</v>
       </c>
       <c r="E90" t="n">
-        <v>1114.03</v>
+        <v>502.13</v>
       </c>
       <c r="F90" t="n">
         <v>0</v>
@@ -2603,22 +2603,22 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D91" t="n">
-        <v>33928</v>
+        <v>792246</v>
       </c>
       <c r="E91" t="n">
-        <v>348.04</v>
+        <v>1040.43</v>
       </c>
       <c r="F91" t="n">
         <v>0</v>
@@ -2627,22 +2627,22 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D92" t="n">
-        <v>31267</v>
+        <v>789603</v>
       </c>
       <c r="E92" t="n">
-        <v>611.5700000000001</v>
+        <v>1114.03</v>
       </c>
       <c r="F92" t="n">
         <v>0</v>
@@ -2651,22 +2651,22 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D93" t="n">
-        <v>30307</v>
+        <v>31267</v>
       </c>
       <c r="E93" t="n">
-        <v>359.76</v>
+        <v>611.5700000000001</v>
       </c>
       <c r="F93" t="n">
         <v>0</v>
@@ -2675,22 +2675,22 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D94" t="n">
-        <v>794671</v>
+        <v>30307</v>
       </c>
       <c r="E94" t="n">
-        <v>206.61</v>
+        <v>359.76</v>
       </c>
       <c r="F94" t="n">
         <v>0</v>
@@ -2699,22 +2699,22 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D95" t="n">
-        <v>789228</v>
+        <v>794671</v>
       </c>
       <c r="E95" t="n">
-        <v>150.57</v>
+        <v>206.61</v>
       </c>
       <c r="F95" t="n">
         <v>0</v>
@@ -2723,46 +2723,46 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D96" t="n">
-        <v>33928</v>
+        <v>789228</v>
       </c>
       <c r="E96" t="n">
-        <v>494.7</v>
+        <v>150.57</v>
       </c>
       <c r="F96" t="n">
-        <v>0</v>
+        <v>25.22</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D97" t="n">
-        <v>792121</v>
+        <v>33928</v>
       </c>
       <c r="E97" t="n">
-        <v>963.4</v>
+        <v>494.7</v>
       </c>
       <c r="F97" t="n">
         <v>0</v>
@@ -2783,10 +2783,10 @@
         <v>46247</v>
       </c>
       <c r="D98" t="n">
-        <v>30218</v>
+        <v>792121</v>
       </c>
       <c r="E98" t="n">
-        <v>173.79</v>
+        <v>963.4</v>
       </c>
       <c r="F98" t="n">
         <v>0</v>
@@ -2795,22 +2795,22 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D99" t="n">
-        <v>789603</v>
+        <v>30218</v>
       </c>
       <c r="E99" t="n">
-        <v>13075.12</v>
+        <v>173.79</v>
       </c>
       <c r="F99" t="n">
         <v>0</v>
@@ -2819,22 +2819,22 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D100" t="n">
-        <v>30791</v>
+        <v>789603</v>
       </c>
       <c r="E100" t="n">
-        <v>1582.7</v>
+        <v>13075.12</v>
       </c>
       <c r="F100" t="n">
         <v>0</v>
@@ -2843,25 +2843,25 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D101" t="n">
-        <v>47252</v>
+        <v>30791</v>
       </c>
       <c r="E101" t="n">
-        <v>14014.78</v>
+        <v>1582.7</v>
       </c>
       <c r="F101" t="n">
-        <v>1686.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102">
@@ -2872,7 +2872,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -2882,10 +2882,10 @@
         <v>47252</v>
       </c>
       <c r="E102" t="n">
-        <v>4965.21</v>
+        <v>14205.41</v>
       </c>
       <c r="F102" t="n">
-        <v>0</v>
+        <v>1686.2</v>
       </c>
     </row>
     <row r="103">
@@ -2896,20 +2896,20 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D103" t="n">
-        <v>793718</v>
+        <v>47252</v>
       </c>
       <c r="E103" t="n">
-        <v>39.84</v>
+        <v>4965.21</v>
       </c>
       <c r="F103" t="n">
-        <v>0</v>
+        <v>91.67</v>
       </c>
     </row>
     <row r="104">
@@ -2927,10 +2927,10 @@
         <v>46247</v>
       </c>
       <c r="D104" t="n">
-        <v>30791</v>
+        <v>793718</v>
       </c>
       <c r="E104" t="n">
-        <v>33.08</v>
+        <v>39.84</v>
       </c>
       <c r="F104" t="n">
         <v>0</v>
@@ -2939,22 +2939,22 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D105" t="n">
-        <v>31267</v>
+        <v>30791</v>
       </c>
       <c r="E105" t="n">
-        <v>160.86</v>
+        <v>33.08</v>
       </c>
       <c r="F105" t="n">
         <v>0</v>
@@ -2963,22 +2963,22 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D106" t="n">
-        <v>33286</v>
+        <v>31267</v>
       </c>
       <c r="E106" t="n">
-        <v>1406.39</v>
+        <v>160.86</v>
       </c>
       <c r="F106" t="n">
         <v>0</v>
@@ -2987,22 +2987,22 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D107" t="n">
-        <v>33057</v>
+        <v>33286</v>
       </c>
       <c r="E107" t="n">
-        <v>89.05</v>
+        <v>1819.31</v>
       </c>
       <c r="F107" t="n">
         <v>0</v>
@@ -3011,22 +3011,22 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D108" t="n">
-        <v>790595</v>
+        <v>33057</v>
       </c>
       <c r="E108" t="n">
-        <v>1274.18</v>
+        <v>89.05</v>
       </c>
       <c r="F108" t="n">
         <v>0</v>
@@ -3040,17 +3040,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D109" t="n">
-        <v>794671</v>
+        <v>790595</v>
       </c>
       <c r="E109" t="n">
-        <v>495.9</v>
+        <v>1274.18</v>
       </c>
       <c r="F109" t="n">
         <v>0</v>
@@ -3059,22 +3059,22 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D110" t="n">
-        <v>47252</v>
+        <v>794671</v>
       </c>
       <c r="E110" t="n">
-        <v>279.06</v>
+        <v>495.9</v>
       </c>
       <c r="F110" t="n">
         <v>0</v>
@@ -3083,22 +3083,22 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D111" t="n">
-        <v>794029</v>
+        <v>47252</v>
       </c>
       <c r="E111" t="n">
-        <v>4098.62</v>
+        <v>279.06</v>
       </c>
       <c r="F111" t="n">
         <v>0</v>
@@ -3107,70 +3107,70 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D112" t="n">
-        <v>789661</v>
+        <v>794029</v>
       </c>
       <c r="E112" t="n">
-        <v>0</v>
+        <v>4098.62</v>
       </c>
       <c r="F112" t="n">
-        <v>258.83</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D113" t="n">
-        <v>31267</v>
+        <v>789661</v>
       </c>
       <c r="E113" t="n">
-        <v>44701.31</v>
+        <v>0</v>
       </c>
       <c r="F113" t="n">
-        <v>0</v>
+        <v>258.83</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D114" t="n">
-        <v>794029</v>
+        <v>31267</v>
       </c>
       <c r="E114" t="n">
-        <v>4429.43</v>
+        <v>48720.5</v>
       </c>
       <c r="F114" t="n">
         <v>0</v>
@@ -3184,17 +3184,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D115" t="n">
-        <v>139553</v>
+        <v>794029</v>
       </c>
       <c r="E115" t="n">
-        <v>6392.04</v>
+        <v>5023.86</v>
       </c>
       <c r="F115" t="n">
         <v>0</v>
@@ -3208,17 +3208,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D116" t="n">
-        <v>792121</v>
+        <v>139553</v>
       </c>
       <c r="E116" t="n">
-        <v>1609.39</v>
+        <v>6392.04</v>
       </c>
       <c r="F116" t="n">
         <v>0</v>
@@ -3227,22 +3227,22 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D117" t="n">
-        <v>795345</v>
+        <v>792121</v>
       </c>
       <c r="E117" t="n">
-        <v>204.29</v>
+        <v>1609.39</v>
       </c>
       <c r="F117" t="n">
         <v>0</v>
@@ -3251,46 +3251,46 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D118" t="n">
-        <v>793186</v>
+        <v>139553</v>
       </c>
       <c r="E118" t="n">
-        <v>0</v>
+        <v>717.6</v>
       </c>
       <c r="F118" t="n">
-        <v>97.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D119" t="n">
-        <v>790595</v>
+        <v>795345</v>
       </c>
       <c r="E119" t="n">
-        <v>117.44</v>
+        <v>204.29</v>
       </c>
       <c r="F119" t="n">
         <v>0</v>
@@ -3299,46 +3299,46 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D120" t="n">
-        <v>792121</v>
+        <v>793186</v>
       </c>
       <c r="E120" t="n">
-        <v>475.96</v>
+        <v>0</v>
       </c>
       <c r="F120" t="n">
-        <v>0</v>
+        <v>97.42</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D121" t="n">
-        <v>30083</v>
+        <v>790595</v>
       </c>
       <c r="E121" t="n">
-        <v>628.4</v>
+        <v>117.44</v>
       </c>
       <c r="F121" t="n">
         <v>0</v>
@@ -3359,10 +3359,10 @@
         <v>46247</v>
       </c>
       <c r="D122" t="n">
-        <v>30307</v>
+        <v>792121</v>
       </c>
       <c r="E122" t="n">
-        <v>1019.5</v>
+        <v>475.96</v>
       </c>
       <c r="F122" t="n">
         <v>0</v>
@@ -3371,22 +3371,22 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D123" t="n">
-        <v>794671</v>
+        <v>30083</v>
       </c>
       <c r="E123" t="n">
-        <v>1344.09</v>
+        <v>628.4</v>
       </c>
       <c r="F123" t="n">
         <v>0</v>
@@ -3395,22 +3395,22 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D124" t="n">
-        <v>32816</v>
+        <v>30307</v>
       </c>
       <c r="E124" t="n">
-        <v>771.3</v>
+        <v>1019.5</v>
       </c>
       <c r="F124" t="n">
         <v>0</v>
@@ -3419,25 +3419,25 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D125" t="n">
-        <v>33057</v>
+        <v>794671</v>
       </c>
       <c r="E125" t="n">
-        <v>12.37</v>
+        <v>1344.09</v>
       </c>
       <c r="F125" t="n">
-        <v>12.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126">
@@ -3448,17 +3448,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D126" t="n">
-        <v>47252</v>
+        <v>32816</v>
       </c>
       <c r="E126" t="n">
-        <v>7354.15</v>
+        <v>771.3</v>
       </c>
       <c r="F126" t="n">
         <v>0</v>
@@ -3467,22 +3467,22 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D127" t="n">
-        <v>789603</v>
+        <v>139553</v>
       </c>
       <c r="E127" t="n">
-        <v>3975.08</v>
+        <v>260.72</v>
       </c>
       <c r="F127" t="n">
         <v>0</v>
@@ -3491,12 +3491,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
@@ -3506,31 +3506,31 @@
         <v>33057</v>
       </c>
       <c r="E128" t="n">
-        <v>27.67</v>
+        <v>12.37</v>
       </c>
       <c r="F128" t="n">
-        <v>0</v>
+        <v>12.37</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C129" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D129" t="n">
-        <v>30307</v>
+        <v>47252</v>
       </c>
       <c r="E129" t="n">
-        <v>33083.51</v>
+        <v>7354.15</v>
       </c>
       <c r="F129" t="n">
         <v>0</v>
@@ -3544,17 +3544,17 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D130" t="n">
-        <v>30307</v>
+        <v>789603</v>
       </c>
       <c r="E130" t="n">
-        <v>6516.78</v>
+        <v>3975.08</v>
       </c>
       <c r="F130" t="n">
         <v>0</v>
@@ -3563,22 +3563,22 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D131" t="n">
-        <v>792141</v>
+        <v>33057</v>
       </c>
       <c r="E131" t="n">
-        <v>13.96</v>
+        <v>27.67</v>
       </c>
       <c r="F131" t="n">
         <v>0</v>
@@ -3587,12 +3587,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
@@ -3602,7 +3602,7 @@
         <v>30307</v>
       </c>
       <c r="E132" t="n">
-        <v>22240.16</v>
+        <v>33083.51</v>
       </c>
       <c r="F132" t="n">
         <v>0</v>
@@ -3611,46 +3611,46 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D133" t="n">
-        <v>792141</v>
+        <v>30307</v>
       </c>
       <c r="E133" t="n">
-        <v>0</v>
+        <v>6516.78</v>
       </c>
       <c r="F133" t="n">
-        <v>791.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D134" t="n">
-        <v>47252</v>
+        <v>792141</v>
       </c>
       <c r="E134" t="n">
-        <v>2429.61</v>
+        <v>13.96</v>
       </c>
       <c r="F134" t="n">
         <v>0</v>
@@ -3659,22 +3659,22 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D135" t="n">
-        <v>792141</v>
+        <v>30307</v>
       </c>
       <c r="E135" t="n">
-        <v>11046.58</v>
+        <v>24395.84</v>
       </c>
       <c r="F135" t="n">
         <v>0</v>
@@ -3683,46 +3683,46 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D136" t="n">
-        <v>789228</v>
+        <v>792141</v>
       </c>
       <c r="E136" t="n">
-        <v>992.67</v>
+        <v>0</v>
       </c>
       <c r="F136" t="n">
-        <v>0</v>
+        <v>791.11</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D137" t="n">
-        <v>32816</v>
+        <v>793718</v>
       </c>
       <c r="E137" t="n">
-        <v>33.34</v>
+        <v>308.44</v>
       </c>
       <c r="F137" t="n">
         <v>0</v>
@@ -3731,22 +3731,22 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D138" t="n">
-        <v>793718</v>
+        <v>47252</v>
       </c>
       <c r="E138" t="n">
-        <v>116.46</v>
+        <v>2429.61</v>
       </c>
       <c r="F138" t="n">
         <v>0</v>
@@ -3755,22 +3755,22 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D139" t="n">
-        <v>793718</v>
+        <v>792141</v>
       </c>
       <c r="E139" t="n">
-        <v>141.07</v>
+        <v>11046.58</v>
       </c>
       <c r="F139" t="n">
         <v>0</v>
@@ -3784,17 +3784,17 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D140" t="n">
-        <v>792141</v>
+        <v>789228</v>
       </c>
       <c r="E140" t="n">
-        <v>33.8</v>
+        <v>1024.21</v>
       </c>
       <c r="F140" t="n">
         <v>0</v>
@@ -3808,92 +3808,92 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D141" t="n">
-        <v>789228</v>
+        <v>32816</v>
       </c>
       <c r="E141" t="n">
-        <v>33.62</v>
+        <v>33.34</v>
       </c>
       <c r="F141" t="n">
-        <v>33.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C142" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D142" t="n">
-        <v>789525</v>
+        <v>793718</v>
       </c>
       <c r="E142" t="n">
-        <v>323.25</v>
+        <v>116.46</v>
       </c>
       <c r="F142" t="n">
-        <v>836.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C143" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D143" t="n">
-        <v>793186</v>
+        <v>792141</v>
       </c>
       <c r="E143" t="n">
-        <v>13.91</v>
+        <v>33.8</v>
       </c>
       <c r="F143" t="n">
-        <v>13.91</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C144" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D144" t="n">
-        <v>47252</v>
+        <v>789228</v>
       </c>
       <c r="E144" t="n">
-        <v>5.57</v>
+        <v>33.62</v>
       </c>
       <c r="F144" t="n">
-        <v>5.57</v>
+        <v>33.67</v>
       </c>
     </row>
     <row r="145">
@@ -3904,44 +3904,44 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C145" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D145" t="n">
-        <v>31267</v>
+        <v>789525</v>
       </c>
       <c r="E145" t="n">
-        <v>14.99</v>
+        <v>323.25</v>
       </c>
       <c r="F145" t="n">
-        <v>0</v>
+        <v>836.2</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C146" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D146" t="n">
-        <v>30791</v>
+        <v>793186</v>
       </c>
       <c r="E146" t="n">
-        <v>1045.7</v>
+        <v>13.91</v>
       </c>
       <c r="F146" t="n">
-        <v>0</v>
+        <v>13.91</v>
       </c>
     </row>
     <row r="147">
@@ -3952,41 +3952,41 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C147" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D147" t="n">
-        <v>30791</v>
+        <v>47252</v>
       </c>
       <c r="E147" t="n">
-        <v>12641.6</v>
+        <v>5.57</v>
       </c>
       <c r="F147" t="n">
-        <v>0</v>
+        <v>5.57</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C148" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D148" t="n">
-        <v>789603</v>
+        <v>31267</v>
       </c>
       <c r="E148" t="n">
-        <v>31178.82</v>
+        <v>14.99</v>
       </c>
       <c r="F148" t="n">
         <v>0</v>
@@ -3995,46 +3995,46 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C149" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D149" t="n">
-        <v>31267</v>
+        <v>30791</v>
       </c>
       <c r="E149" t="n">
-        <v>370.51</v>
+        <v>1045.7</v>
       </c>
       <c r="F149" t="n">
-        <v>24.04</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C150" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D150" t="n">
-        <v>794671</v>
+        <v>30791</v>
       </c>
       <c r="E150" t="n">
-        <v>2697.85</v>
+        <v>12688.95</v>
       </c>
       <c r="F150" t="n">
         <v>0</v>
@@ -4043,22 +4043,22 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C151" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D151" t="n">
-        <v>795345</v>
+        <v>789603</v>
       </c>
       <c r="E151" t="n">
-        <v>2510.84</v>
+        <v>31178.82</v>
       </c>
       <c r="F151" t="n">
         <v>0</v>
@@ -4067,46 +4067,46 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C152" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D152" t="n">
-        <v>794029</v>
+        <v>31267</v>
       </c>
       <c r="E152" t="n">
-        <v>31.16</v>
+        <v>370.51</v>
       </c>
       <c r="F152" t="n">
-        <v>0</v>
+        <v>24.04</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C153" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D153" t="n">
-        <v>33928</v>
+        <v>792141</v>
       </c>
       <c r="E153" t="n">
-        <v>40.62</v>
+        <v>2631.15</v>
       </c>
       <c r="F153" t="n">
         <v>0</v>
@@ -4115,22 +4115,22 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C154" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D154" t="n">
-        <v>32816</v>
+        <v>794671</v>
       </c>
       <c r="E154" t="n">
-        <v>456.96</v>
+        <v>2697.85</v>
       </c>
       <c r="F154" t="n">
         <v>0</v>
@@ -4139,22 +4139,22 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C155" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D155" t="n">
-        <v>790595</v>
+        <v>795345</v>
       </c>
       <c r="E155" t="n">
-        <v>267.36</v>
+        <v>2510.84</v>
       </c>
       <c r="F155" t="n">
         <v>0</v>
@@ -4163,22 +4163,22 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C156" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D156" t="n">
-        <v>47252</v>
+        <v>794029</v>
       </c>
       <c r="E156" t="n">
-        <v>8997.92</v>
+        <v>31.16</v>
       </c>
       <c r="F156" t="n">
         <v>0</v>
@@ -4187,22 +4187,22 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C157" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D157" t="n">
-        <v>794671</v>
+        <v>33928</v>
       </c>
       <c r="E157" t="n">
-        <v>276.11</v>
+        <v>40.62</v>
       </c>
       <c r="F157" t="n">
         <v>0</v>
@@ -4211,22 +4211,22 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C158" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D158" t="n">
-        <v>789603</v>
+        <v>32816</v>
       </c>
       <c r="E158" t="n">
-        <v>2592.83</v>
+        <v>456.96</v>
       </c>
       <c r="F158" t="n">
         <v>0</v>
@@ -4235,22 +4235,22 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C159" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D159" t="n">
-        <v>139553</v>
+        <v>790595</v>
       </c>
       <c r="E159" t="n">
-        <v>6009.46</v>
+        <v>267.36</v>
       </c>
       <c r="F159" t="n">
         <v>0</v>
@@ -4259,22 +4259,22 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C160" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D160" t="n">
-        <v>30218</v>
+        <v>47252</v>
       </c>
       <c r="E160" t="n">
-        <v>1633.63</v>
+        <v>9037.610000000001</v>
       </c>
       <c r="F160" t="n">
         <v>0</v>
@@ -4283,22 +4283,22 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C161" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D161" t="n">
-        <v>793186</v>
+        <v>794671</v>
       </c>
       <c r="E161" t="n">
-        <v>2152.16</v>
+        <v>276.11</v>
       </c>
       <c r="F161" t="n">
         <v>0</v>
@@ -4307,22 +4307,22 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C162" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D162" t="n">
-        <v>30083</v>
+        <v>789603</v>
       </c>
       <c r="E162" t="n">
-        <v>627.34</v>
+        <v>2592.83</v>
       </c>
       <c r="F162" t="n">
         <v>0</v>
@@ -4331,22 +4331,22 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C163" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D163" t="n">
-        <v>30307</v>
+        <v>139553</v>
       </c>
       <c r="E163" t="n">
-        <v>71722.69</v>
+        <v>6009.46</v>
       </c>
       <c r="F163" t="n">
         <v>0</v>
@@ -4355,22 +4355,22 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C164" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D164" t="n">
-        <v>30083</v>
+        <v>30218</v>
       </c>
       <c r="E164" t="n">
-        <v>3113.39</v>
+        <v>1633.63</v>
       </c>
       <c r="F164" t="n">
         <v>0</v>
@@ -4379,73 +4379,73 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C165" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D165" t="n">
-        <v>789661</v>
+        <v>793186</v>
       </c>
       <c r="E165" t="n">
-        <v>0</v>
+        <v>2152.16</v>
       </c>
       <c r="F165" t="n">
-        <v>32.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C166" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D166" t="n">
-        <v>793718</v>
+        <v>30083</v>
       </c>
       <c r="E166" t="n">
-        <v>64.17</v>
+        <v>627.34</v>
       </c>
       <c r="F166" t="n">
-        <v>80.59999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C167" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D167" t="n">
-        <v>33286</v>
+        <v>30307</v>
       </c>
       <c r="E167" t="n">
-        <v>3.99</v>
+        <v>73419.89</v>
       </c>
       <c r="F167" t="n">
-        <v>3.99</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168">
@@ -4456,17 +4456,17 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C168" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D168" t="n">
-        <v>139553</v>
+        <v>30083</v>
       </c>
       <c r="E168" t="n">
-        <v>1400.68</v>
+        <v>3113.39</v>
       </c>
       <c r="F168" t="n">
         <v>0</v>
@@ -4475,94 +4475,94 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C169" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D169" t="n">
-        <v>792121</v>
+        <v>789661</v>
       </c>
       <c r="E169" t="n">
-        <v>42.15</v>
+        <v>0</v>
       </c>
       <c r="F169" t="n">
-        <v>0</v>
+        <v>32.2</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C170" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D170" t="n">
-        <v>33928</v>
+        <v>793718</v>
       </c>
       <c r="E170" t="n">
-        <v>1038.51</v>
+        <v>64.17</v>
       </c>
       <c r="F170" t="n">
-        <v>0</v>
+        <v>80.59999999999999</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C171" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D171" t="n">
-        <v>789525</v>
+        <v>33286</v>
       </c>
       <c r="E171" t="n">
-        <v>251.71</v>
+        <v>3.99</v>
       </c>
       <c r="F171" t="n">
-        <v>0</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C172" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D172" t="n">
-        <v>33057</v>
+        <v>139553</v>
       </c>
       <c r="E172" t="n">
-        <v>89.06</v>
+        <v>1400.68</v>
       </c>
       <c r="F172" t="n">
         <v>0</v>
@@ -4571,22 +4571,22 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C173" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D173" t="n">
-        <v>789525</v>
+        <v>792121</v>
       </c>
       <c r="E173" t="n">
-        <v>3222.01</v>
+        <v>42.15</v>
       </c>
       <c r="F173" t="n">
         <v>0</v>
@@ -4595,22 +4595,22 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C174" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D174" t="n">
-        <v>794671</v>
+        <v>33928</v>
       </c>
       <c r="E174" t="n">
-        <v>627.4</v>
+        <v>1038.51</v>
       </c>
       <c r="F174" t="n">
         <v>0</v>
@@ -4624,17 +4624,17 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C175" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D175" t="n">
-        <v>30307</v>
+        <v>789525</v>
       </c>
       <c r="E175" t="n">
-        <v>575.88</v>
+        <v>251.71</v>
       </c>
       <c r="F175" t="n">
         <v>0</v>
@@ -4648,17 +4648,17 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C176" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D176" t="n">
-        <v>30791</v>
+        <v>33057</v>
       </c>
       <c r="E176" t="n">
-        <v>44.88</v>
+        <v>89.06</v>
       </c>
       <c r="F176" t="n">
         <v>0</v>
@@ -4667,22 +4667,22 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C177" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D177" t="n">
-        <v>47252</v>
+        <v>789525</v>
       </c>
       <c r="E177" t="n">
-        <v>3921.52</v>
+        <v>3886.91</v>
       </c>
       <c r="F177" t="n">
         <v>0</v>
@@ -4696,17 +4696,17 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C178" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D178" t="n">
-        <v>795345</v>
+        <v>794671</v>
       </c>
       <c r="E178" t="n">
-        <v>81</v>
+        <v>787.04</v>
       </c>
       <c r="F178" t="n">
         <v>0</v>
@@ -4715,22 +4715,22 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="C179" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D179" t="n">
-        <v>31267</v>
+        <v>30307</v>
       </c>
       <c r="E179" t="n">
-        <v>26.27</v>
+        <v>575.88</v>
       </c>
       <c r="F179" t="n">
         <v>0</v>
@@ -4739,22 +4739,22 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="C180" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D180" t="n">
-        <v>793186</v>
+        <v>30791</v>
       </c>
       <c r="E180" t="n">
-        <v>54.68</v>
+        <v>44.88</v>
       </c>
       <c r="F180" t="n">
         <v>0</v>
@@ -4763,22 +4763,22 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C181" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D181" t="n">
-        <v>33057</v>
+        <v>47252</v>
       </c>
       <c r="E181" t="n">
-        <v>472.88</v>
+        <v>4921.54</v>
       </c>
       <c r="F181" t="n">
         <v>0</v>
@@ -4787,22 +4787,22 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C182" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D182" t="n">
-        <v>30791</v>
+        <v>795345</v>
       </c>
       <c r="E182" t="n">
-        <v>1913.38</v>
+        <v>81</v>
       </c>
       <c r="F182" t="n">
         <v>0</v>
@@ -4811,22 +4811,22 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C183" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D183" t="n">
-        <v>789603</v>
+        <v>31267</v>
       </c>
       <c r="E183" t="n">
-        <v>553.98</v>
+        <v>26.27</v>
       </c>
       <c r="F183" t="n">
         <v>0</v>
@@ -4835,22 +4835,22 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C184" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D184" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="E184" t="n">
-        <v>10503.77</v>
+        <v>54.68</v>
       </c>
       <c r="F184" t="n">
         <v>0</v>
@@ -4859,22 +4859,22 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C185" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D185" t="n">
-        <v>789525</v>
+        <v>33057</v>
       </c>
       <c r="E185" t="n">
-        <v>525.0599999999999</v>
+        <v>552.15</v>
       </c>
       <c r="F185" t="n">
         <v>0</v>
@@ -4895,10 +4895,10 @@
         <v>46247</v>
       </c>
       <c r="D186" t="n">
-        <v>792141</v>
+        <v>47252</v>
       </c>
       <c r="E186" t="n">
-        <v>50.7</v>
+        <v>12742.11</v>
       </c>
       <c r="F186" t="n">
         <v>0</v>
@@ -4907,22 +4907,22 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C187" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D187" t="n">
-        <v>33928</v>
+        <v>30791</v>
       </c>
       <c r="E187" t="n">
-        <v>509.48</v>
+        <v>2127.36</v>
       </c>
       <c r="F187" t="n">
         <v>0</v>
@@ -4931,22 +4931,22 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C188" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D188" t="n">
-        <v>30083</v>
+        <v>792141</v>
       </c>
       <c r="E188" t="n">
-        <v>2086.14</v>
+        <v>122.4</v>
       </c>
       <c r="F188" t="n">
         <v>0</v>
@@ -4955,22 +4955,22 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C189" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D189" t="n">
-        <v>792121</v>
+        <v>794029</v>
       </c>
       <c r="E189" t="n">
-        <v>1408.4</v>
+        <v>913.4299999999999</v>
       </c>
       <c r="F189" t="n">
         <v>0</v>
@@ -4979,22 +4979,22 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C190" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D190" t="n">
-        <v>30307</v>
+        <v>789603</v>
       </c>
       <c r="E190" t="n">
-        <v>3113.59</v>
+        <v>553.98</v>
       </c>
       <c r="F190" t="n">
         <v>0</v>
@@ -5003,22 +5003,22 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C191" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D191" t="n">
-        <v>792121</v>
+        <v>789525</v>
       </c>
       <c r="E191" t="n">
-        <v>501.32</v>
+        <v>525.0599999999999</v>
       </c>
       <c r="F191" t="n">
         <v>0</v>
@@ -5027,22 +5027,22 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C192" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D192" t="n">
-        <v>32816</v>
+        <v>33928</v>
       </c>
       <c r="E192" t="n">
-        <v>74.84999999999999</v>
+        <v>509.48</v>
       </c>
       <c r="F192" t="n">
         <v>0</v>
@@ -5051,22 +5051,22 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C193" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D193" t="n">
-        <v>33057</v>
+        <v>30083</v>
       </c>
       <c r="E193" t="n">
-        <v>199.41</v>
+        <v>2086.14</v>
       </c>
       <c r="F193" t="n">
         <v>0</v>
@@ -5075,22 +5075,22 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C194" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D194" t="n">
-        <v>789603</v>
+        <v>792121</v>
       </c>
       <c r="E194" t="n">
-        <v>31185.75</v>
+        <v>1408.4</v>
       </c>
       <c r="F194" t="n">
         <v>0</v>
@@ -5104,17 +5104,17 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C195" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D195" t="n">
-        <v>139553</v>
+        <v>30307</v>
       </c>
       <c r="E195" t="n">
-        <v>147.55</v>
+        <v>3113.59</v>
       </c>
       <c r="F195" t="n">
         <v>0</v>
@@ -5123,22 +5123,22 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C196" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D196" t="n">
-        <v>33286</v>
+        <v>792121</v>
       </c>
       <c r="E196" t="n">
-        <v>74.83</v>
+        <v>501.32</v>
       </c>
       <c r="F196" t="n">
         <v>0</v>
@@ -5147,24 +5147,144 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D197" t="n">
+        <v>32816</v>
+      </c>
+      <c r="E197" t="n">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F197" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D198" t="n">
+        <v>33057</v>
+      </c>
+      <c r="E198" t="n">
+        <v>199.41</v>
+      </c>
+      <c r="F198" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D199" t="n">
+        <v>789603</v>
+      </c>
+      <c r="E199" t="n">
+        <v>31185.75</v>
+      </c>
+      <c r="F199" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D200" t="n">
+        <v>139553</v>
+      </c>
+      <c r="E200" t="n">
+        <v>147.55</v>
+      </c>
+      <c r="F200" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D201" t="n">
+        <v>33286</v>
+      </c>
+      <c r="E201" t="n">
+        <v>74.83</v>
+      </c>
+      <c r="F201" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="B197" t="inlineStr">
+      <c r="B202" t="inlineStr">
         <is>
           <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
-      <c r="C197" s="2" t="n">
-        <v>46247</v>
-      </c>
-      <c r="D197" t="n">
+      <c r="C202" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D202" t="n">
         <v>790595</v>
       </c>
-      <c r="E197" t="n">
+      <c r="E202" t="n">
         <v>196.4</v>
       </c>
-      <c r="F197" t="n">
+      <c r="F202" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 12:15:04
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F240"/>
+  <dimension ref="A1:F243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,7 +506,7 @@
         <v>47252</v>
       </c>
       <c r="E3" t="n">
-        <v>10905.94</v>
+        <v>10972.73</v>
       </c>
       <c r="F3" t="n">
         <v>1606.14</v>
@@ -530,7 +530,7 @@
         <v>33928</v>
       </c>
       <c r="E4" t="n">
-        <v>30964.31</v>
+        <v>31109.41</v>
       </c>
       <c r="F4" t="n">
         <v>254.53</v>
@@ -578,7 +578,7 @@
         <v>33928</v>
       </c>
       <c r="E6" t="n">
-        <v>7285.03</v>
+        <v>7349.59</v>
       </c>
       <c r="F6" t="n">
         <v>391.48</v>
@@ -602,7 +602,7 @@
         <v>30791</v>
       </c>
       <c r="E7" t="n">
-        <v>10792.31</v>
+        <v>10939.04</v>
       </c>
       <c r="F7" t="n">
         <v>3111.54</v>
@@ -818,7 +818,7 @@
         <v>792121</v>
       </c>
       <c r="E16" t="n">
-        <v>15643.16</v>
+        <v>16299.18</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -914,10 +914,10 @@
         <v>30307</v>
       </c>
       <c r="E20" t="n">
-        <v>37811.13</v>
+        <v>40773.09</v>
       </c>
       <c r="F20" t="n">
-        <v>10473.88</v>
+        <v>19867.16</v>
       </c>
     </row>
     <row r="21">
@@ -971,22 +971,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D23" t="n">
-        <v>789603</v>
+        <v>139553</v>
       </c>
       <c r="E23" t="n">
-        <v>26814.77</v>
+        <v>4559.33</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -995,22 +995,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D24" t="n">
-        <v>30791</v>
+        <v>789603</v>
       </c>
       <c r="E24" t="n">
-        <v>28.51</v>
+        <v>26814.77</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -1019,22 +1019,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D25" t="n">
-        <v>31267</v>
+        <v>30791</v>
       </c>
       <c r="E25" t="n">
-        <v>118550.67</v>
+        <v>28.51</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -1043,22 +1043,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D26" t="n">
-        <v>139553</v>
+        <v>31267</v>
       </c>
       <c r="E26" t="n">
-        <v>971.03</v>
+        <v>132617.84</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -1370,7 +1370,7 @@
         <v>789603</v>
       </c>
       <c r="E39" t="n">
-        <v>7602.96</v>
+        <v>15969.24</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
@@ -1442,7 +1442,7 @@
         <v>30791</v>
       </c>
       <c r="E42" t="n">
-        <v>8011.33</v>
+        <v>6878.17</v>
       </c>
       <c r="F42" t="n">
         <v>579.78</v>
@@ -1490,7 +1490,7 @@
         <v>31267</v>
       </c>
       <c r="E44" t="n">
-        <v>2448.16</v>
+        <v>2646.48</v>
       </c>
       <c r="F44" t="n">
         <v>165.42</v>
@@ -1514,7 +1514,7 @@
         <v>47252</v>
       </c>
       <c r="E45" t="n">
-        <v>10108.85</v>
+        <v>10803.68</v>
       </c>
       <c r="F45" t="n">
         <v>0</v>
@@ -1682,7 +1682,7 @@
         <v>792121</v>
       </c>
       <c r="E52" t="n">
-        <v>738.23</v>
+        <v>976.8099999999999</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
@@ -1706,7 +1706,7 @@
         <v>789603</v>
       </c>
       <c r="E53" t="n">
-        <v>5348.14</v>
+        <v>9832.360000000001</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
@@ -2042,7 +2042,7 @@
         <v>789603</v>
       </c>
       <c r="E67" t="n">
-        <v>394.86</v>
+        <v>514.26</v>
       </c>
       <c r="F67" t="n">
         <v>0</v>
@@ -2066,7 +2066,7 @@
         <v>30791</v>
       </c>
       <c r="E68" t="n">
-        <v>8415.08</v>
+        <v>8512.24</v>
       </c>
       <c r="F68" t="n">
         <v>404.46</v>
@@ -2090,7 +2090,7 @@
         <v>33286</v>
       </c>
       <c r="E69" t="n">
-        <v>922.61</v>
+        <v>1001.27</v>
       </c>
       <c r="F69" t="n">
         <v>230.41</v>
@@ -2138,7 +2138,7 @@
         <v>793718</v>
       </c>
       <c r="E71" t="n">
-        <v>828.6</v>
+        <v>863.25</v>
       </c>
       <c r="F71" t="n">
         <v>0</v>
@@ -2162,7 +2162,7 @@
         <v>33928</v>
       </c>
       <c r="E72" t="n">
-        <v>805.62</v>
+        <v>977.09</v>
       </c>
       <c r="F72" t="n">
         <v>0</v>
@@ -2210,7 +2210,7 @@
         <v>139553</v>
       </c>
       <c r="E74" t="n">
-        <v>1952.16</v>
+        <v>4462.08</v>
       </c>
       <c r="F74" t="n">
         <v>0</v>
@@ -2450,7 +2450,7 @@
         <v>47252</v>
       </c>
       <c r="E84" t="n">
-        <v>9637.99</v>
+        <v>9585.860000000001</v>
       </c>
       <c r="F84" t="n">
         <v>0</v>
@@ -2579,22 +2579,22 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D90" t="n">
-        <v>793718</v>
+        <v>796582</v>
       </c>
       <c r="E90" t="n">
-        <v>48.08</v>
+        <v>2511.38</v>
       </c>
       <c r="F90" t="n">
         <v>0</v>
@@ -2603,22 +2603,22 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D91" t="n">
-        <v>32816</v>
+        <v>793718</v>
       </c>
       <c r="E91" t="n">
-        <v>11.9</v>
+        <v>48.08</v>
       </c>
       <c r="F91" t="n">
         <v>0</v>
@@ -2639,10 +2639,10 @@
         <v>46247</v>
       </c>
       <c r="D92" t="n">
-        <v>796582</v>
+        <v>32816</v>
       </c>
       <c r="E92" t="n">
-        <v>2267.86</v>
+        <v>11.9</v>
       </c>
       <c r="F92" t="n">
         <v>0</v>
@@ -2690,7 +2690,7 @@
         <v>789525</v>
       </c>
       <c r="E94" t="n">
-        <v>2189.37</v>
+        <v>2779.91</v>
       </c>
       <c r="F94" t="n">
         <v>288.23</v>
@@ -2786,7 +2786,7 @@
         <v>33928</v>
       </c>
       <c r="E98" t="n">
-        <v>11287.34</v>
+        <v>11697.84</v>
       </c>
       <c r="F98" t="n">
         <v>0</v>
@@ -2810,7 +2810,7 @@
         <v>33286</v>
       </c>
       <c r="E99" t="n">
-        <v>2588.63</v>
+        <v>3924.08</v>
       </c>
       <c r="F99" t="n">
         <v>0</v>
@@ -2834,7 +2834,7 @@
         <v>30791</v>
       </c>
       <c r="E100" t="n">
-        <v>2006.6</v>
+        <v>2835.5</v>
       </c>
       <c r="F100" t="n">
         <v>0</v>
@@ -2954,7 +2954,7 @@
         <v>789603</v>
       </c>
       <c r="E105" t="n">
-        <v>21390.64</v>
+        <v>21748.84</v>
       </c>
       <c r="F105" t="n">
         <v>0</v>
@@ -3002,7 +3002,7 @@
         <v>30307</v>
       </c>
       <c r="E107" t="n">
-        <v>43914.18</v>
+        <v>44096.13</v>
       </c>
       <c r="F107" t="n">
         <v>0</v>
@@ -3290,7 +3290,7 @@
         <v>33928</v>
       </c>
       <c r="E119" t="n">
-        <v>657.55</v>
+        <v>692.58</v>
       </c>
       <c r="F119" t="n">
         <v>0</v>
@@ -3371,25 +3371,25 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D123" t="n">
-        <v>47252</v>
+        <v>792121</v>
       </c>
       <c r="E123" t="n">
-        <v>16272.51</v>
+        <v>9.49</v>
       </c>
       <c r="F123" t="n">
-        <v>1686.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124">
@@ -3400,7 +3400,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
@@ -3410,10 +3410,10 @@
         <v>47252</v>
       </c>
       <c r="E124" t="n">
-        <v>10382.55</v>
+        <v>16688.33</v>
       </c>
       <c r="F124" t="n">
-        <v>1352.08</v>
+        <v>1686.2</v>
       </c>
     </row>
     <row r="125">
@@ -3424,20 +3424,20 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D125" t="n">
-        <v>793718</v>
+        <v>47252</v>
       </c>
       <c r="E125" t="n">
-        <v>39.84</v>
+        <v>10382.55</v>
       </c>
       <c r="F125" t="n">
-        <v>0</v>
+        <v>1352.08</v>
       </c>
     </row>
     <row r="126">
@@ -3455,10 +3455,10 @@
         <v>46247</v>
       </c>
       <c r="D126" t="n">
-        <v>30791</v>
+        <v>793718</v>
       </c>
       <c r="E126" t="n">
-        <v>33.08</v>
+        <v>39.84</v>
       </c>
       <c r="F126" t="n">
         <v>0</v>
@@ -3467,22 +3467,22 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D127" t="n">
-        <v>31267</v>
+        <v>30791</v>
       </c>
       <c r="E127" t="n">
-        <v>160.86</v>
+        <v>33.08</v>
       </c>
       <c r="F127" t="n">
         <v>0</v>
@@ -3491,22 +3491,22 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D128" t="n">
-        <v>139553</v>
+        <v>31267</v>
       </c>
       <c r="E128" t="n">
-        <v>222.26</v>
+        <v>160.86</v>
       </c>
       <c r="F128" t="n">
         <v>0</v>
@@ -3527,10 +3527,10 @@
         <v>46247</v>
       </c>
       <c r="D129" t="n">
-        <v>33286</v>
+        <v>139553</v>
       </c>
       <c r="E129" t="n">
-        <v>6858.39</v>
+        <v>222.26</v>
       </c>
       <c r="F129" t="n">
         <v>0</v>
@@ -3539,22 +3539,22 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D130" t="n">
-        <v>30307</v>
+        <v>33286</v>
       </c>
       <c r="E130" t="n">
-        <v>507.68</v>
+        <v>6942.56</v>
       </c>
       <c r="F130" t="n">
         <v>0</v>
@@ -3563,22 +3563,22 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D131" t="n">
-        <v>33057</v>
+        <v>30307</v>
       </c>
       <c r="E131" t="n">
-        <v>89.05</v>
+        <v>507.68</v>
       </c>
       <c r="F131" t="n">
         <v>0</v>
@@ -3587,94 +3587,94 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D132" t="n">
-        <v>793186</v>
+        <v>33057</v>
       </c>
       <c r="E132" t="n">
-        <v>442.74</v>
+        <v>89.05</v>
       </c>
       <c r="F132" t="n">
-        <v>97.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D133" t="n">
-        <v>790595</v>
+        <v>789661</v>
       </c>
       <c r="E133" t="n">
-        <v>1274.18</v>
+        <v>37.05</v>
       </c>
       <c r="F133" t="n">
-        <v>0</v>
+        <v>258.83</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D134" t="n">
-        <v>794671</v>
+        <v>793186</v>
       </c>
       <c r="E134" t="n">
-        <v>495.9</v>
+        <v>442.74</v>
       </c>
       <c r="F134" t="n">
-        <v>0</v>
+        <v>97.42</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D135" t="n">
-        <v>47252</v>
+        <v>790595</v>
       </c>
       <c r="E135" t="n">
-        <v>279.06</v>
+        <v>1274.18</v>
       </c>
       <c r="F135" t="n">
         <v>0</v>
@@ -3688,17 +3688,17 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D136" t="n">
-        <v>794029</v>
+        <v>794671</v>
       </c>
       <c r="E136" t="n">
-        <v>6547.47</v>
+        <v>495.9</v>
       </c>
       <c r="F136" t="n">
         <v>0</v>
@@ -3707,46 +3707,46 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D137" t="n">
-        <v>789661</v>
+        <v>47252</v>
       </c>
       <c r="E137" t="n">
-        <v>0</v>
+        <v>291.52</v>
       </c>
       <c r="F137" t="n">
-        <v>258.83</v>
+        <v>0</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D138" t="n">
-        <v>31267</v>
+        <v>794029</v>
       </c>
       <c r="E138" t="n">
-        <v>82625.14999999999</v>
+        <v>6547.47</v>
       </c>
       <c r="F138" t="n">
         <v>0</v>
@@ -3760,17 +3760,17 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D139" t="n">
-        <v>794029</v>
+        <v>792121</v>
       </c>
       <c r="E139" t="n">
-        <v>6369.81</v>
+        <v>3522.67</v>
       </c>
       <c r="F139" t="n">
         <v>0</v>
@@ -3779,22 +3779,22 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D140" t="n">
-        <v>33928</v>
+        <v>31267</v>
       </c>
       <c r="E140" t="n">
-        <v>823.55</v>
+        <v>113278.62</v>
       </c>
       <c r="F140" t="n">
         <v>0</v>
@@ -3808,17 +3808,17 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D141" t="n">
-        <v>139553</v>
+        <v>794029</v>
       </c>
       <c r="E141" t="n">
-        <v>7003.92</v>
+        <v>6672.47</v>
       </c>
       <c r="F141" t="n">
         <v>0</v>
@@ -3827,22 +3827,22 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C142" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D142" t="n">
-        <v>792121</v>
+        <v>33928</v>
       </c>
       <c r="E142" t="n">
-        <v>1609.39</v>
+        <v>823.55</v>
       </c>
       <c r="F142" t="n">
         <v>0</v>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C143" s="2" t="n">
@@ -3866,7 +3866,7 @@
         <v>139553</v>
       </c>
       <c r="E143" t="n">
-        <v>717.6</v>
+        <v>7003.92</v>
       </c>
       <c r="F143" t="n">
         <v>0</v>
@@ -3875,22 +3875,22 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C144" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D144" t="n">
-        <v>796582</v>
+        <v>139553</v>
       </c>
       <c r="E144" t="n">
-        <v>1247.64</v>
+        <v>717.6</v>
       </c>
       <c r="F144" t="n">
         <v>0</v>
@@ -3899,22 +3899,22 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C145" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D145" t="n">
-        <v>30083</v>
+        <v>796582</v>
       </c>
       <c r="E145" t="n">
-        <v>215.07</v>
+        <v>1247.64</v>
       </c>
       <c r="F145" t="n">
         <v>0</v>
@@ -3923,22 +3923,22 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C146" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D146" t="n">
-        <v>795345</v>
+        <v>30083</v>
       </c>
       <c r="E146" t="n">
-        <v>204.29</v>
+        <v>215.07</v>
       </c>
       <c r="F146" t="n">
         <v>0</v>
@@ -3947,22 +3947,22 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C147" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D147" t="n">
-        <v>790595</v>
+        <v>795345</v>
       </c>
       <c r="E147" t="n">
-        <v>117.44</v>
+        <v>204.29</v>
       </c>
       <c r="F147" t="n">
         <v>0</v>
@@ -3971,22 +3971,22 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C148" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D148" t="n">
-        <v>30083</v>
+        <v>790595</v>
       </c>
       <c r="E148" t="n">
-        <v>727.5700000000001</v>
+        <v>117.44</v>
       </c>
       <c r="F148" t="n">
         <v>0</v>
@@ -4007,10 +4007,10 @@
         <v>46247</v>
       </c>
       <c r="D149" t="n">
-        <v>792121</v>
+        <v>30083</v>
       </c>
       <c r="E149" t="n">
-        <v>550.45</v>
+        <v>727.5700000000001</v>
       </c>
       <c r="F149" t="n">
         <v>0</v>
@@ -4031,10 +4031,10 @@
         <v>46247</v>
       </c>
       <c r="D150" t="n">
-        <v>30307</v>
+        <v>792121</v>
       </c>
       <c r="E150" t="n">
-        <v>3088.64</v>
+        <v>1095.64</v>
       </c>
       <c r="F150" t="n">
         <v>0</v>
@@ -4043,22 +4043,22 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C151" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D151" t="n">
-        <v>794671</v>
+        <v>30307</v>
       </c>
       <c r="E151" t="n">
-        <v>1810.54</v>
+        <v>3088.64</v>
       </c>
       <c r="F151" t="n">
         <v>0</v>
@@ -4067,22 +4067,22 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C152" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D152" t="n">
-        <v>32816</v>
+        <v>794671</v>
       </c>
       <c r="E152" t="n">
-        <v>1721.48</v>
+        <v>1810.54</v>
       </c>
       <c r="F152" t="n">
         <v>0</v>
@@ -4091,22 +4091,22 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C153" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D153" t="n">
-        <v>139553</v>
+        <v>32816</v>
       </c>
       <c r="E153" t="n">
-        <v>260.72</v>
+        <v>1721.48</v>
       </c>
       <c r="F153" t="n">
         <v>0</v>
@@ -4115,22 +4115,22 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C154" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D154" t="n">
-        <v>789603</v>
+        <v>139553</v>
       </c>
       <c r="E154" t="n">
-        <v>7108.74</v>
+        <v>260.72</v>
       </c>
       <c r="F154" t="n">
         <v>0</v>
@@ -4139,94 +4139,94 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C155" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D155" t="n">
-        <v>33057</v>
+        <v>789603</v>
       </c>
       <c r="E155" t="n">
-        <v>12.37</v>
+        <v>7108.74</v>
       </c>
       <c r="F155" t="n">
-        <v>12.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C156" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D156" t="n">
-        <v>47252</v>
+        <v>33057</v>
       </c>
       <c r="E156" t="n">
-        <v>8941.950000000001</v>
+        <v>12.37</v>
       </c>
       <c r="F156" t="n">
-        <v>0</v>
+        <v>12.37</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C157" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D157" t="n">
-        <v>792141</v>
+        <v>47252</v>
       </c>
       <c r="E157" t="n">
-        <v>192.8</v>
+        <v>9297.58</v>
       </c>
       <c r="F157" t="n">
-        <v>791.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C158" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D158" t="n">
-        <v>33057</v>
+        <v>793186</v>
       </c>
       <c r="E158" t="n">
-        <v>102.15</v>
+        <v>342.23</v>
       </c>
       <c r="F158" t="n">
         <v>0</v>
@@ -4235,46 +4235,46 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C159" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D159" t="n">
-        <v>789228</v>
+        <v>792141</v>
       </c>
       <c r="E159" t="n">
-        <v>1204.03</v>
+        <v>192.8</v>
       </c>
       <c r="F159" t="n">
-        <v>0</v>
+        <v>791.11</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C160" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D160" t="n">
-        <v>793718</v>
+        <v>33057</v>
       </c>
       <c r="E160" t="n">
-        <v>542.17</v>
+        <v>102.15</v>
       </c>
       <c r="F160" t="n">
         <v>0</v>
@@ -4283,22 +4283,22 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C161" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D161" t="n">
-        <v>795345</v>
+        <v>789228</v>
       </c>
       <c r="E161" t="n">
-        <v>678.78</v>
+        <v>1204.03</v>
       </c>
       <c r="F161" t="n">
         <v>0</v>
@@ -4307,22 +4307,22 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C162" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D162" t="n">
-        <v>30307</v>
+        <v>793718</v>
       </c>
       <c r="E162" t="n">
-        <v>50921.15</v>
+        <v>542.17</v>
       </c>
       <c r="F162" t="n">
         <v>0</v>
@@ -4336,17 +4336,17 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C163" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D163" t="n">
-        <v>30307</v>
+        <v>795345</v>
       </c>
       <c r="E163" t="n">
-        <v>8561.940000000001</v>
+        <v>678.78</v>
       </c>
       <c r="F163" t="n">
         <v>0</v>
@@ -4355,22 +4355,22 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C164" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D164" t="n">
-        <v>789603</v>
+        <v>30307</v>
       </c>
       <c r="E164" t="n">
-        <v>1091.25</v>
+        <v>50921.15</v>
       </c>
       <c r="F164" t="n">
         <v>0</v>
@@ -4379,22 +4379,22 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C165" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D165" t="n">
-        <v>792141</v>
+        <v>30307</v>
       </c>
       <c r="E165" t="n">
-        <v>13.96</v>
+        <v>11510.44</v>
       </c>
       <c r="F165" t="n">
         <v>0</v>
@@ -4403,22 +4403,22 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C166" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D166" t="n">
-        <v>30307</v>
+        <v>789603</v>
       </c>
       <c r="E166" t="n">
-        <v>52729.56</v>
+        <v>1091.25</v>
       </c>
       <c r="F166" t="n">
         <v>0</v>
@@ -4427,22 +4427,22 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C167" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D167" t="n">
-        <v>32816</v>
+        <v>792141</v>
       </c>
       <c r="E167" t="n">
-        <v>46.4</v>
+        <v>13.96</v>
       </c>
       <c r="F167" t="n">
         <v>0</v>
@@ -4451,22 +4451,22 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C168" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D168" t="n">
-        <v>47252</v>
+        <v>30307</v>
       </c>
       <c r="E168" t="n">
-        <v>3157.51</v>
+        <v>57022.56</v>
       </c>
       <c r="F168" t="n">
         <v>0</v>
@@ -4475,22 +4475,22 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C169" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D169" t="n">
-        <v>795345</v>
+        <v>32816</v>
       </c>
       <c r="E169" t="n">
-        <v>361.98</v>
+        <v>46.4</v>
       </c>
       <c r="F169" t="n">
         <v>0</v>
@@ -4504,41 +4504,41 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C170" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D170" t="n">
-        <v>792141</v>
+        <v>47252</v>
       </c>
       <c r="E170" t="n">
-        <v>11160.8</v>
+        <v>3157.51</v>
       </c>
       <c r="F170" t="n">
-        <v>321.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C171" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D171" t="n">
-        <v>793718</v>
+        <v>795345</v>
       </c>
       <c r="E171" t="n">
-        <v>145.46</v>
+        <v>361.98</v>
       </c>
       <c r="F171" t="n">
         <v>0</v>
@@ -4547,46 +4547,46 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C172" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D172" t="n">
-        <v>792121</v>
+        <v>792141</v>
       </c>
       <c r="E172" t="n">
-        <v>301.76</v>
+        <v>11160.8</v>
       </c>
       <c r="F172" t="n">
-        <v>0</v>
+        <v>321.34</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C173" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D173" t="n">
-        <v>792141</v>
+        <v>793718</v>
       </c>
       <c r="E173" t="n">
-        <v>33.8</v>
+        <v>145.46</v>
       </c>
       <c r="F173" t="n">
         <v>0</v>
@@ -4595,121 +4595,121 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C174" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D174" t="n">
-        <v>31267</v>
+        <v>792121</v>
       </c>
       <c r="E174" t="n">
-        <v>5351.33</v>
+        <v>301.76</v>
       </c>
       <c r="F174" t="n">
-        <v>390.95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C175" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D175" t="n">
-        <v>789228</v>
+        <v>792141</v>
       </c>
       <c r="E175" t="n">
-        <v>33.62</v>
+        <v>33.8</v>
       </c>
       <c r="F175" t="n">
-        <v>33.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C176" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D176" t="n">
-        <v>789525</v>
+        <v>794671</v>
       </c>
       <c r="E176" t="n">
-        <v>775.92</v>
+        <v>32.7</v>
       </c>
       <c r="F176" t="n">
-        <v>836.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C177" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D177" t="n">
-        <v>793186</v>
+        <v>31267</v>
       </c>
       <c r="E177" t="n">
-        <v>13.91</v>
+        <v>17213.41</v>
       </c>
       <c r="F177" t="n">
-        <v>13.91</v>
+        <v>390.95</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C178" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D178" t="n">
-        <v>47252</v>
+        <v>789228</v>
       </c>
       <c r="E178" t="n">
-        <v>5.57</v>
+        <v>55.88</v>
       </c>
       <c r="F178" t="n">
-        <v>5.57</v>
+        <v>33.67</v>
       </c>
     </row>
     <row r="179">
@@ -4720,44 +4720,44 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C179" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D179" t="n">
-        <v>31267</v>
+        <v>789525</v>
       </c>
       <c r="E179" t="n">
-        <v>14.99</v>
+        <v>775.92</v>
       </c>
       <c r="F179" t="n">
-        <v>0</v>
+        <v>836.2</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C180" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D180" t="n">
-        <v>30791</v>
+        <v>793186</v>
       </c>
       <c r="E180" t="n">
-        <v>1241.39</v>
+        <v>13.91</v>
       </c>
       <c r="F180" t="n">
-        <v>0</v>
+        <v>13.91</v>
       </c>
     </row>
     <row r="181">
@@ -4768,41 +4768,41 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C181" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D181" t="n">
-        <v>30791</v>
+        <v>47252</v>
       </c>
       <c r="E181" t="n">
-        <v>16284.29</v>
+        <v>5.57</v>
       </c>
       <c r="F181" t="n">
-        <v>0</v>
+        <v>5.57</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C182" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D182" t="n">
-        <v>789603</v>
+        <v>31267</v>
       </c>
       <c r="E182" t="n">
-        <v>31178.82</v>
+        <v>14.99</v>
       </c>
       <c r="F182" t="n">
         <v>0</v>
@@ -4811,22 +4811,22 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C183" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D183" t="n">
-        <v>792141</v>
+        <v>30791</v>
       </c>
       <c r="E183" t="n">
-        <v>16635.41</v>
+        <v>1864.57</v>
       </c>
       <c r="F183" t="n">
         <v>0</v>
@@ -4835,22 +4835,22 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C184" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D184" t="n">
-        <v>794671</v>
+        <v>30791</v>
       </c>
       <c r="E184" t="n">
-        <v>3081.69</v>
+        <v>16401.28</v>
       </c>
       <c r="F184" t="n">
         <v>0</v>
@@ -4859,22 +4859,22 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C185" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D185" t="n">
-        <v>795345</v>
+        <v>789603</v>
       </c>
       <c r="E185" t="n">
-        <v>2816.55</v>
+        <v>31178.82</v>
       </c>
       <c r="F185" t="n">
         <v>0</v>
@@ -4883,22 +4883,22 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C186" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D186" t="n">
-        <v>794029</v>
+        <v>792141</v>
       </c>
       <c r="E186" t="n">
-        <v>31.16</v>
+        <v>16635.41</v>
       </c>
       <c r="F186" t="n">
         <v>0</v>
@@ -4907,22 +4907,22 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C187" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D187" t="n">
-        <v>33928</v>
+        <v>794671</v>
       </c>
       <c r="E187" t="n">
-        <v>40.62</v>
+        <v>3081.69</v>
       </c>
       <c r="F187" t="n">
         <v>0</v>
@@ -4931,22 +4931,22 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C188" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D188" t="n">
-        <v>32816</v>
+        <v>795345</v>
       </c>
       <c r="E188" t="n">
-        <v>456.96</v>
+        <v>3919.83</v>
       </c>
       <c r="F188" t="n">
         <v>0</v>
@@ -4955,22 +4955,22 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C189" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D189" t="n">
-        <v>31267</v>
+        <v>794029</v>
       </c>
       <c r="E189" t="n">
-        <v>914.84</v>
+        <v>31.16</v>
       </c>
       <c r="F189" t="n">
         <v>0</v>
@@ -4979,22 +4979,22 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C190" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D190" t="n">
-        <v>790595</v>
+        <v>33928</v>
       </c>
       <c r="E190" t="n">
-        <v>267.36</v>
+        <v>40.62</v>
       </c>
       <c r="F190" t="n">
         <v>0</v>
@@ -5008,17 +5008,17 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C191" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D191" t="n">
-        <v>30218</v>
+        <v>32816</v>
       </c>
       <c r="E191" t="n">
-        <v>2443.81</v>
+        <v>456.96</v>
       </c>
       <c r="F191" t="n">
         <v>0</v>
@@ -5027,22 +5027,22 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C192" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D192" t="n">
-        <v>47252</v>
+        <v>31267</v>
       </c>
       <c r="E192" t="n">
-        <v>14111.13</v>
+        <v>914.84</v>
       </c>
       <c r="F192" t="n">
         <v>0</v>
@@ -5051,22 +5051,22 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C193" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D193" t="n">
-        <v>794671</v>
+        <v>790595</v>
       </c>
       <c r="E193" t="n">
-        <v>276.11</v>
+        <v>267.36</v>
       </c>
       <c r="F193" t="n">
         <v>0</v>
@@ -5075,22 +5075,22 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C194" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D194" t="n">
-        <v>789603</v>
+        <v>30218</v>
       </c>
       <c r="E194" t="n">
-        <v>8375.620000000001</v>
+        <v>2443.81</v>
       </c>
       <c r="F194" t="n">
         <v>0</v>
@@ -5099,22 +5099,22 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C195" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D195" t="n">
-        <v>793186</v>
+        <v>47252</v>
       </c>
       <c r="E195" t="n">
-        <v>7905.42</v>
+        <v>15153.43</v>
       </c>
       <c r="F195" t="n">
         <v>0</v>
@@ -5123,22 +5123,22 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C196" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D196" t="n">
-        <v>139553</v>
+        <v>794671</v>
       </c>
       <c r="E196" t="n">
-        <v>8304.940000000001</v>
+        <v>276.11</v>
       </c>
       <c r="F196" t="n">
         <v>0</v>
@@ -5159,10 +5159,10 @@
         <v>46247</v>
       </c>
       <c r="D197" t="n">
-        <v>792246</v>
+        <v>789603</v>
       </c>
       <c r="E197" t="n">
-        <v>587.38</v>
+        <v>9857.200000000001</v>
       </c>
       <c r="F197" t="n">
         <v>0</v>
@@ -5171,22 +5171,22 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C198" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D198" t="n">
-        <v>139553</v>
+        <v>793186</v>
       </c>
       <c r="E198" t="n">
-        <v>209.16</v>
+        <v>7955.41</v>
       </c>
       <c r="F198" t="n">
         <v>0</v>
@@ -5195,22 +5195,22 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C199" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D199" t="n">
-        <v>30083</v>
+        <v>139553</v>
       </c>
       <c r="E199" t="n">
-        <v>627.34</v>
+        <v>8304.940000000001</v>
       </c>
       <c r="F199" t="n">
         <v>0</v>
@@ -5219,22 +5219,22 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C200" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D200" t="n">
-        <v>30307</v>
+        <v>792246</v>
       </c>
       <c r="E200" t="n">
-        <v>77065.77</v>
+        <v>587.38</v>
       </c>
       <c r="F200" t="n">
         <v>0</v>
@@ -5248,17 +5248,17 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C201" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D201" t="n">
-        <v>30083</v>
+        <v>139553</v>
       </c>
       <c r="E201" t="n">
-        <v>4360.5</v>
+        <v>209.16</v>
       </c>
       <c r="F201" t="n">
         <v>0</v>
@@ -5267,166 +5267,166 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C202" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D202" t="n">
-        <v>793718</v>
+        <v>30083</v>
       </c>
       <c r="E202" t="n">
-        <v>1203.05</v>
+        <v>627.34</v>
       </c>
       <c r="F202" t="n">
-        <v>80.59999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C203" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D203" t="n">
-        <v>789661</v>
+        <v>30307</v>
       </c>
       <c r="E203" t="n">
-        <v>0</v>
+        <v>88082.95</v>
       </c>
       <c r="F203" t="n">
-        <v>32.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C204" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D204" t="n">
-        <v>33286</v>
+        <v>30083</v>
       </c>
       <c r="E204" t="n">
-        <v>3.99</v>
+        <v>4360.5</v>
       </c>
       <c r="F204" t="n">
-        <v>3.99</v>
+        <v>0</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C205" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D205" t="n">
-        <v>792121</v>
+        <v>793718</v>
       </c>
       <c r="E205" t="n">
-        <v>42.15</v>
+        <v>1203.05</v>
       </c>
       <c r="F205" t="n">
-        <v>0</v>
+        <v>80.59999999999999</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C206" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D206" t="n">
-        <v>139553</v>
+        <v>789661</v>
       </c>
       <c r="E206" t="n">
-        <v>1300.72</v>
+        <v>0</v>
       </c>
       <c r="F206" t="n">
-        <v>0</v>
+        <v>32.2</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C207" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D207" t="n">
-        <v>33928</v>
+        <v>33286</v>
       </c>
       <c r="E207" t="n">
-        <v>1038.51</v>
+        <v>3.99</v>
       </c>
       <c r="F207" t="n">
-        <v>0</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C208" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D208" t="n">
-        <v>789525</v>
+        <v>792121</v>
       </c>
       <c r="E208" t="n">
-        <v>251.71</v>
+        <v>42.15</v>
       </c>
       <c r="F208" t="n">
         <v>0</v>
@@ -5435,22 +5435,22 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C209" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D209" t="n">
-        <v>33057</v>
+        <v>139553</v>
       </c>
       <c r="E209" t="n">
-        <v>89.06</v>
+        <v>1300.72</v>
       </c>
       <c r="F209" t="n">
         <v>0</v>
@@ -5459,22 +5459,22 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C210" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D210" t="n">
-        <v>789525</v>
+        <v>33928</v>
       </c>
       <c r="E210" t="n">
-        <v>4694.22</v>
+        <v>1038.51</v>
       </c>
       <c r="F210" t="n">
         <v>0</v>
@@ -5483,22 +5483,22 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C211" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D211" t="n">
-        <v>33057</v>
+        <v>789525</v>
       </c>
       <c r="E211" t="n">
-        <v>684.27</v>
+        <v>251.71</v>
       </c>
       <c r="F211" t="n">
         <v>0</v>
@@ -5507,22 +5507,22 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C212" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D212" t="n">
-        <v>794671</v>
+        <v>33057</v>
       </c>
       <c r="E212" t="n">
-        <v>3401.34</v>
+        <v>89.06</v>
       </c>
       <c r="F212" t="n">
         <v>0</v>
@@ -5531,22 +5531,22 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C213" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D213" t="n">
-        <v>47252</v>
+        <v>789525</v>
       </c>
       <c r="E213" t="n">
-        <v>16005.83</v>
+        <v>4718.93</v>
       </c>
       <c r="F213" t="n">
         <v>0</v>
@@ -5555,22 +5555,22 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C214" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D214" t="n">
-        <v>789525</v>
+        <v>33057</v>
       </c>
       <c r="E214" t="n">
-        <v>764.99</v>
+        <v>684.27</v>
       </c>
       <c r="F214" t="n">
         <v>0</v>
@@ -5579,22 +5579,22 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C215" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D215" t="n">
-        <v>30307</v>
+        <v>794671</v>
       </c>
       <c r="E215" t="n">
-        <v>575.88</v>
+        <v>3401.34</v>
       </c>
       <c r="F215" t="n">
         <v>0</v>
@@ -5608,17 +5608,17 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C216" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D216" t="n">
-        <v>30791</v>
+        <v>47252</v>
       </c>
       <c r="E216" t="n">
-        <v>44.88</v>
+        <v>16219.54</v>
       </c>
       <c r="F216" t="n">
         <v>0</v>
@@ -5627,22 +5627,22 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C217" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D217" t="n">
-        <v>790595</v>
+        <v>30791</v>
       </c>
       <c r="E217" t="n">
-        <v>1151.94</v>
+        <v>3619.6</v>
       </c>
       <c r="F217" t="n">
         <v>0</v>
@@ -5656,17 +5656,17 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C218" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D218" t="n">
-        <v>47252</v>
+        <v>789525</v>
       </c>
       <c r="E218" t="n">
-        <v>10349.54</v>
+        <v>764.99</v>
       </c>
       <c r="F218" t="n">
         <v>0</v>
@@ -5675,46 +5675,46 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="C219" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D219" t="n">
-        <v>789603</v>
+        <v>30307</v>
       </c>
       <c r="E219" t="n">
-        <v>32546.35</v>
+        <v>575.88</v>
       </c>
       <c r="F219" t="n">
-        <v>3083.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="C220" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D220" t="n">
-        <v>795345</v>
+        <v>30791</v>
       </c>
       <c r="E220" t="n">
-        <v>81</v>
+        <v>44.88</v>
       </c>
       <c r="F220" t="n">
         <v>0</v>
@@ -5723,22 +5723,22 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C221" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D221" t="n">
-        <v>31267</v>
+        <v>790595</v>
       </c>
       <c r="E221" t="n">
-        <v>26.27</v>
+        <v>1151.94</v>
       </c>
       <c r="F221" t="n">
         <v>0</v>
@@ -5747,70 +5747,70 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C222" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D222" t="n">
-        <v>793186</v>
+        <v>47252</v>
       </c>
       <c r="E222" t="n">
-        <v>443.79</v>
+        <v>10923.19</v>
       </c>
       <c r="F222" t="n">
-        <v>54.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C223" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D223" t="n">
-        <v>794671</v>
+        <v>789603</v>
       </c>
       <c r="E223" t="n">
-        <v>679.33</v>
+        <v>48878.27</v>
       </c>
       <c r="F223" t="n">
-        <v>0</v>
+        <v>29466.34</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C224" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D224" t="n">
-        <v>30307</v>
+        <v>795345</v>
       </c>
       <c r="E224" t="n">
-        <v>4573.05</v>
+        <v>81</v>
       </c>
       <c r="F224" t="n">
         <v>0</v>
@@ -5819,22 +5819,22 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C225" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D225" t="n">
-        <v>30791</v>
+        <v>31267</v>
       </c>
       <c r="E225" t="n">
-        <v>2187.54</v>
+        <v>26.27</v>
       </c>
       <c r="F225" t="n">
         <v>0</v>
@@ -5843,46 +5843,46 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C226" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D226" t="n">
-        <v>792141</v>
+        <v>793186</v>
       </c>
       <c r="E226" t="n">
-        <v>122.4</v>
+        <v>443.79</v>
       </c>
       <c r="F226" t="n">
-        <v>0</v>
+        <v>54.71</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C227" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D227" t="n">
-        <v>793186</v>
+        <v>30307</v>
       </c>
       <c r="E227" t="n">
-        <v>146.11</v>
+        <v>6524.57</v>
       </c>
       <c r="F227" t="n">
         <v>0</v>
@@ -5891,22 +5891,22 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C228" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D228" t="n">
-        <v>30083</v>
+        <v>794671</v>
       </c>
       <c r="E228" t="n">
-        <v>3299.7</v>
+        <v>679.33</v>
       </c>
       <c r="F228" t="n">
         <v>0</v>
@@ -5915,22 +5915,22 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C229" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D229" t="n">
-        <v>794029</v>
+        <v>792141</v>
       </c>
       <c r="E229" t="n">
-        <v>913.4299999999999</v>
+        <v>2529.9</v>
       </c>
       <c r="F229" t="n">
         <v>0</v>
@@ -5939,22 +5939,22 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C230" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D230" t="n">
-        <v>789603</v>
+        <v>793186</v>
       </c>
       <c r="E230" t="n">
-        <v>553.98</v>
+        <v>146.11</v>
       </c>
       <c r="F230" t="n">
         <v>0</v>
@@ -5963,22 +5963,22 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C231" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D231" t="n">
-        <v>33928</v>
+        <v>30083</v>
       </c>
       <c r="E231" t="n">
-        <v>1231.23</v>
+        <v>3299.7</v>
       </c>
       <c r="F231" t="n">
         <v>0</v>
@@ -5987,22 +5987,22 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C232" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D232" t="n">
-        <v>792121</v>
+        <v>794029</v>
       </c>
       <c r="E232" t="n">
-        <v>1472.58</v>
+        <v>913.4299999999999</v>
       </c>
       <c r="F232" t="n">
         <v>0</v>
@@ -6016,17 +6016,17 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C233" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D233" t="n">
-        <v>792121</v>
+        <v>789603</v>
       </c>
       <c r="E233" t="n">
-        <v>501.32</v>
+        <v>553.98</v>
       </c>
       <c r="F233" t="n">
         <v>0</v>
@@ -6035,22 +6035,22 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C234" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D234" t="n">
-        <v>32816</v>
+        <v>33928</v>
       </c>
       <c r="E234" t="n">
-        <v>74.84999999999999</v>
+        <v>1231.23</v>
       </c>
       <c r="F234" t="n">
         <v>0</v>
@@ -6059,22 +6059,22 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C235" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D235" t="n">
-        <v>33057</v>
+        <v>792121</v>
       </c>
       <c r="E235" t="n">
-        <v>2773.8</v>
+        <v>1472.58</v>
       </c>
       <c r="F235" t="n">
         <v>0</v>
@@ -6083,22 +6083,22 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C236" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D236" t="n">
-        <v>139553</v>
+        <v>792121</v>
       </c>
       <c r="E236" t="n">
-        <v>846.42</v>
+        <v>501.32</v>
       </c>
       <c r="F236" t="n">
         <v>0</v>
@@ -6107,22 +6107,22 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C237" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D237" t="n">
-        <v>33286</v>
+        <v>32816</v>
       </c>
       <c r="E237" t="n">
-        <v>106.92</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="F237" t="n">
         <v>0</v>
@@ -6131,22 +6131,22 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C238" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D238" t="n">
-        <v>139553</v>
+        <v>33057</v>
       </c>
       <c r="E238" t="n">
-        <v>611.88</v>
+        <v>2773.8</v>
       </c>
       <c r="F238" t="n">
         <v>0</v>
@@ -6155,22 +6155,22 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C239" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D239" t="n">
-        <v>790595</v>
+        <v>139553</v>
       </c>
       <c r="E239" t="n">
-        <v>294.6</v>
+        <v>2570.35</v>
       </c>
       <c r="F239" t="n">
         <v>0</v>
@@ -6179,24 +6179,96 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D240" t="n">
+        <v>33286</v>
+      </c>
+      <c r="E240" t="n">
+        <v>106.92</v>
+      </c>
+      <c r="F240" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D241" t="n">
+        <v>139553</v>
+      </c>
+      <c r="E241" t="n">
+        <v>611.88</v>
+      </c>
+      <c r="F241" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="B240" t="inlineStr">
+      <c r="B242" t="inlineStr">
         <is>
           <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
-      <c r="C240" s="2" t="n">
-        <v>46247</v>
-      </c>
-      <c r="D240" t="n">
+      <c r="C242" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D242" t="n">
+        <v>790595</v>
+      </c>
+      <c r="E242" t="n">
+        <v>294.6</v>
+      </c>
+      <c r="F242" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D243" t="n">
         <v>795345</v>
       </c>
-      <c r="E240" t="n">
+      <c r="E243" t="n">
         <v>169.57</v>
       </c>
-      <c r="F240" t="n">
+      <c r="F243" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 13:00:03
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F250"/>
+  <dimension ref="A1:F253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,10 +506,10 @@
         <v>47252</v>
       </c>
       <c r="E3" t="n">
-        <v>13437.16</v>
+        <v>13437.74</v>
       </c>
       <c r="F3" t="n">
-        <v>1606.14</v>
+        <v>3810.55</v>
       </c>
     </row>
     <row r="4">
@@ -530,10 +530,10 @@
         <v>33928</v>
       </c>
       <c r="E4" t="n">
-        <v>31534.06</v>
+        <v>31534.35</v>
       </c>
       <c r="F4" t="n">
-        <v>254.53</v>
+        <v>6656.24</v>
       </c>
     </row>
     <row r="5">
@@ -602,7 +602,7 @@
         <v>30791</v>
       </c>
       <c r="E7" t="n">
-        <v>11592.39</v>
+        <v>13129.92</v>
       </c>
       <c r="F7" t="n">
         <v>3111.54</v>
@@ -647,13 +647,13 @@
         <v>46247</v>
       </c>
       <c r="D9" t="n">
-        <v>33928</v>
+        <v>31267</v>
       </c>
       <c r="E9" t="n">
-        <v>5961.9</v>
+        <v>10513.58</v>
       </c>
       <c r="F9" t="n">
-        <v>935.13</v>
+        <v>758.7</v>
       </c>
     </row>
     <row r="10">
@@ -671,13 +671,13 @@
         <v>46247</v>
       </c>
       <c r="D10" t="n">
-        <v>789525</v>
+        <v>33928</v>
       </c>
       <c r="E10" t="n">
-        <v>1260.78</v>
+        <v>5961.9</v>
       </c>
       <c r="F10" t="n">
-        <v>98.76000000000001</v>
+        <v>935.13</v>
       </c>
     </row>
     <row r="11">
@@ -695,13 +695,13 @@
         <v>46247</v>
       </c>
       <c r="D11" t="n">
-        <v>31267</v>
+        <v>789525</v>
       </c>
       <c r="E11" t="n">
-        <v>10513.53</v>
+        <v>1260.78</v>
       </c>
       <c r="F11" t="n">
-        <v>650.1799999999999</v>
+        <v>98.76000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -893,7 +893,7 @@
         <v>47906.17</v>
       </c>
       <c r="F19" t="n">
-        <v>19867.16</v>
+        <v>22829.12</v>
       </c>
     </row>
     <row r="20">
@@ -995,22 +995,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D24" t="n">
-        <v>789603</v>
+        <v>30083</v>
       </c>
       <c r="E24" t="n">
-        <v>27376.19</v>
+        <v>1745.8</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -1019,22 +1019,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D25" t="n">
-        <v>30791</v>
+        <v>789603</v>
       </c>
       <c r="E25" t="n">
-        <v>28.51</v>
+        <v>27376.19</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -1043,22 +1043,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D26" t="n">
-        <v>794671</v>
+        <v>30791</v>
       </c>
       <c r="E26" t="n">
-        <v>4160.56</v>
+        <v>28.51</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -1072,17 +1072,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D27" t="n">
-        <v>31267</v>
+        <v>794671</v>
       </c>
       <c r="E27" t="n">
-        <v>139110.09</v>
+        <v>4160.56</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -1091,22 +1091,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D28" t="n">
-        <v>794671</v>
+        <v>31267</v>
       </c>
       <c r="E28" t="n">
-        <v>11789.62</v>
+        <v>139829.94</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -1127,10 +1127,10 @@
         <v>46247</v>
       </c>
       <c r="D29" t="n">
-        <v>792246</v>
+        <v>794671</v>
       </c>
       <c r="E29" t="n">
-        <v>145.36</v>
+        <v>11789.62</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -1139,22 +1139,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D30" t="n">
-        <v>795345</v>
+        <v>792246</v>
       </c>
       <c r="E30" t="n">
-        <v>98.68000000000001</v>
+        <v>145.36</v>
       </c>
       <c r="F30" t="n">
         <v>0</v>
@@ -1163,22 +1163,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D31" t="n">
-        <v>33057</v>
+        <v>795345</v>
       </c>
       <c r="E31" t="n">
-        <v>475.23</v>
+        <v>98.68000000000001</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
@@ -1187,12 +1187,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -1202,7 +1202,7 @@
         <v>33057</v>
       </c>
       <c r="E32" t="n">
-        <v>157.96</v>
+        <v>475.23</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -1211,22 +1211,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D33" t="n">
-        <v>789603</v>
+        <v>33057</v>
       </c>
       <c r="E33" t="n">
-        <v>2087.64</v>
+        <v>157.96</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
@@ -1235,22 +1235,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D34" t="n">
-        <v>795345</v>
+        <v>789603</v>
       </c>
       <c r="E34" t="n">
-        <v>34.41</v>
+        <v>2087.64</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
@@ -1259,22 +1259,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D35" t="n">
-        <v>30083</v>
+        <v>795345</v>
       </c>
       <c r="E35" t="n">
-        <v>1645.4</v>
+        <v>34.41</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
@@ -1442,7 +1442,7 @@
         <v>30791</v>
       </c>
       <c r="E42" t="n">
-        <v>11447.02</v>
+        <v>12136.78</v>
       </c>
       <c r="F42" t="n">
         <v>685.66</v>
@@ -1514,7 +1514,7 @@
         <v>31267</v>
       </c>
       <c r="E45" t="n">
-        <v>4817.78</v>
+        <v>4970.25</v>
       </c>
       <c r="F45" t="n">
         <v>165.42</v>
@@ -1538,7 +1538,7 @@
         <v>47252</v>
       </c>
       <c r="E46" t="n">
-        <v>12150.21</v>
+        <v>12342.97</v>
       </c>
       <c r="F46" t="n">
         <v>0</v>
@@ -1874,7 +1874,7 @@
         <v>33286</v>
       </c>
       <c r="E60" t="n">
-        <v>2219.1</v>
+        <v>2653.4</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
@@ -2090,10 +2090,10 @@
         <v>30791</v>
       </c>
       <c r="E69" t="n">
-        <v>10907.98</v>
+        <v>10908.04</v>
       </c>
       <c r="F69" t="n">
-        <v>1451.24</v>
+        <v>1524.6</v>
       </c>
     </row>
     <row r="70">
@@ -2234,7 +2234,7 @@
         <v>33928</v>
       </c>
       <c r="E75" t="n">
-        <v>977.09</v>
+        <v>1047.68</v>
       </c>
       <c r="F75" t="n">
         <v>0</v>
@@ -2368,17 +2368,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D81" t="n">
-        <v>33286</v>
+        <v>794671</v>
       </c>
       <c r="E81" t="n">
-        <v>1460.34</v>
+        <v>6317.91</v>
       </c>
       <c r="F81" t="n">
         <v>0</v>
@@ -2392,17 +2392,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D82" t="n">
-        <v>139553</v>
+        <v>792246</v>
       </c>
       <c r="E82" t="n">
-        <v>108.72</v>
+        <v>1852.36</v>
       </c>
       <c r="F82" t="n">
         <v>0</v>
@@ -2411,22 +2411,22 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D83" t="n">
-        <v>789228</v>
+        <v>33286</v>
       </c>
       <c r="E83" t="n">
-        <v>199.03</v>
+        <v>1460.34</v>
       </c>
       <c r="F83" t="n">
         <v>0</v>
@@ -2435,22 +2435,22 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D84" t="n">
-        <v>33057</v>
+        <v>139553</v>
       </c>
       <c r="E84" t="n">
-        <v>29.2</v>
+        <v>108.72</v>
       </c>
       <c r="F84" t="n">
         <v>0</v>
@@ -2459,22 +2459,22 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D85" t="n">
-        <v>33057</v>
+        <v>789228</v>
       </c>
       <c r="E85" t="n">
-        <v>541.71</v>
+        <v>199.03</v>
       </c>
       <c r="F85" t="n">
         <v>0</v>
@@ -2483,22 +2483,22 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D86" t="n">
-        <v>47252</v>
+        <v>33057</v>
       </c>
       <c r="E86" t="n">
-        <v>11998.47</v>
+        <v>29.2</v>
       </c>
       <c r="F86" t="n">
         <v>0</v>
@@ -2507,46 +2507,46 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D87" t="n">
-        <v>792141</v>
+        <v>33057</v>
       </c>
       <c r="E87" t="n">
-        <v>0</v>
+        <v>575.42</v>
       </c>
       <c r="F87" t="n">
-        <v>11651.64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D88" t="n">
-        <v>792141</v>
+        <v>47252</v>
       </c>
       <c r="E88" t="n">
-        <v>207.9</v>
+        <v>13045.36</v>
       </c>
       <c r="F88" t="n">
         <v>0</v>
@@ -2555,46 +2555,46 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D89" t="n">
-        <v>47252</v>
+        <v>792141</v>
       </c>
       <c r="E89" t="n">
-        <v>1829.67</v>
+        <v>0</v>
       </c>
       <c r="F89" t="n">
-        <v>0</v>
+        <v>11651.64</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D90" t="n">
-        <v>794671</v>
+        <v>792141</v>
       </c>
       <c r="E90" t="n">
-        <v>5713.08</v>
+        <v>207.9</v>
       </c>
       <c r="F90" t="n">
         <v>0</v>
@@ -2603,22 +2603,22 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D91" t="n">
-        <v>789661</v>
+        <v>47252</v>
       </c>
       <c r="E91" t="n">
-        <v>647.25</v>
+        <v>1927.46</v>
       </c>
       <c r="F91" t="n">
         <v>0</v>
@@ -2627,22 +2627,22 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D92" t="n">
-        <v>792246</v>
+        <v>789661</v>
       </c>
       <c r="E92" t="n">
-        <v>1308.82</v>
+        <v>647.25</v>
       </c>
       <c r="F92" t="n">
         <v>0</v>
@@ -2738,7 +2738,7 @@
         <v>30307</v>
       </c>
       <c r="E96" t="n">
-        <v>29942.62</v>
+        <v>30986.26</v>
       </c>
       <c r="F96" t="n">
         <v>0</v>
@@ -2906,7 +2906,7 @@
         <v>33286</v>
       </c>
       <c r="E103" t="n">
-        <v>3924.08</v>
+        <v>4016.65</v>
       </c>
       <c r="F103" t="n">
         <v>0</v>
@@ -2930,7 +2930,7 @@
         <v>30791</v>
       </c>
       <c r="E104" t="n">
-        <v>2835.5</v>
+        <v>3015.8</v>
       </c>
       <c r="F104" t="n">
         <v>0</v>
@@ -3107,22 +3107,22 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D112" t="n">
-        <v>793718</v>
+        <v>792121</v>
       </c>
       <c r="E112" t="n">
-        <v>225.33</v>
+        <v>1710.2</v>
       </c>
       <c r="F112" t="n">
         <v>0</v>
@@ -3131,22 +3131,22 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D113" t="n">
-        <v>33928</v>
+        <v>793718</v>
       </c>
       <c r="E113" t="n">
-        <v>868.12</v>
+        <v>225.33</v>
       </c>
       <c r="F113" t="n">
         <v>0</v>
@@ -3167,10 +3167,10 @@
         <v>46247</v>
       </c>
       <c r="D114" t="n">
-        <v>793718</v>
+        <v>33928</v>
       </c>
       <c r="E114" t="n">
-        <v>561.64</v>
+        <v>898.0700000000001</v>
       </c>
       <c r="F114" t="n">
         <v>0</v>
@@ -3179,22 +3179,22 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D115" t="n">
-        <v>33286</v>
+        <v>793718</v>
       </c>
       <c r="E115" t="n">
-        <v>1262.09</v>
+        <v>561.64</v>
       </c>
       <c r="F115" t="n">
         <v>0</v>
@@ -3203,22 +3203,22 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D116" t="n">
-        <v>794029</v>
+        <v>33286</v>
       </c>
       <c r="E116" t="n">
-        <v>731.21</v>
+        <v>1376.17</v>
       </c>
       <c r="F116" t="n">
         <v>0</v>
@@ -3227,22 +3227,22 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D117" t="n">
-        <v>792246</v>
+        <v>794029</v>
       </c>
       <c r="E117" t="n">
-        <v>1040.43</v>
+        <v>731.21</v>
       </c>
       <c r="F117" t="n">
         <v>0</v>
@@ -3251,22 +3251,22 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D118" t="n">
-        <v>789603</v>
+        <v>792246</v>
       </c>
       <c r="E118" t="n">
-        <v>3300.52</v>
+        <v>1040.43</v>
       </c>
       <c r="F118" t="n">
         <v>0</v>
@@ -3275,22 +3275,22 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D119" t="n">
-        <v>31267</v>
+        <v>789603</v>
       </c>
       <c r="E119" t="n">
-        <v>1110.13</v>
+        <v>3300.52</v>
       </c>
       <c r="F119" t="n">
         <v>0</v>
@@ -3299,22 +3299,22 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D120" t="n">
-        <v>30307</v>
+        <v>31267</v>
       </c>
       <c r="E120" t="n">
-        <v>1208.36</v>
+        <v>1110.13</v>
       </c>
       <c r="F120" t="n">
         <v>0</v>
@@ -3323,22 +3323,22 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D121" t="n">
-        <v>794671</v>
+        <v>30307</v>
       </c>
       <c r="E121" t="n">
-        <v>718.38</v>
+        <v>1208.36</v>
       </c>
       <c r="F121" t="n">
         <v>0</v>
@@ -3347,70 +3347,70 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D122" t="n">
-        <v>789228</v>
+        <v>794671</v>
       </c>
       <c r="E122" t="n">
-        <v>194.05</v>
+        <v>718.38</v>
       </c>
       <c r="F122" t="n">
-        <v>159.28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D123" t="n">
-        <v>33928</v>
+        <v>789228</v>
       </c>
       <c r="E123" t="n">
-        <v>894.14</v>
+        <v>194.05</v>
       </c>
       <c r="F123" t="n">
-        <v>0</v>
+        <v>159.28</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D124" t="n">
-        <v>792141</v>
+        <v>33928</v>
       </c>
       <c r="E124" t="n">
-        <v>8.970000000000001</v>
+        <v>894.14</v>
       </c>
       <c r="F124" t="n">
         <v>0</v>
@@ -3419,22 +3419,22 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D125" t="n">
-        <v>792121</v>
+        <v>792141</v>
       </c>
       <c r="E125" t="n">
-        <v>963.4</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="F125" t="n">
         <v>0</v>
@@ -3530,10 +3530,10 @@
         <v>47252</v>
       </c>
       <c r="E129" t="n">
-        <v>21760.85</v>
+        <v>21761.48</v>
       </c>
       <c r="F129" t="n">
-        <v>2903.21</v>
+        <v>4460.38</v>
       </c>
     </row>
     <row r="130">
@@ -3698,7 +3698,7 @@
         <v>33057</v>
       </c>
       <c r="E136" t="n">
-        <v>89.05</v>
+        <v>146.56</v>
       </c>
       <c r="F136" t="n">
         <v>0</v>
@@ -3779,22 +3779,22 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D140" t="n">
-        <v>790595</v>
+        <v>31267</v>
       </c>
       <c r="E140" t="n">
-        <v>1274.18</v>
+        <v>63.33</v>
       </c>
       <c r="F140" t="n">
         <v>0</v>
@@ -3808,17 +3808,17 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D141" t="n">
-        <v>792121</v>
+        <v>790595</v>
       </c>
       <c r="E141" t="n">
-        <v>4843.19</v>
+        <v>1274.18</v>
       </c>
       <c r="F141" t="n">
         <v>0</v>
@@ -3832,17 +3832,17 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C142" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D142" t="n">
-        <v>794671</v>
+        <v>792121</v>
       </c>
       <c r="E142" t="n">
-        <v>495.9</v>
+        <v>4843.19</v>
       </c>
       <c r="F142" t="n">
         <v>0</v>
@@ -3851,22 +3851,22 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C143" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D143" t="n">
-        <v>47252</v>
+        <v>794671</v>
       </c>
       <c r="E143" t="n">
-        <v>291.52</v>
+        <v>495.9</v>
       </c>
       <c r="F143" t="n">
         <v>0</v>
@@ -3875,22 +3875,22 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C144" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D144" t="n">
-        <v>31267</v>
+        <v>47252</v>
       </c>
       <c r="E144" t="n">
-        <v>133928.28</v>
+        <v>291.52</v>
       </c>
       <c r="F144" t="n">
         <v>0</v>
@@ -3899,22 +3899,22 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C145" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D145" t="n">
-        <v>794029</v>
+        <v>31267</v>
       </c>
       <c r="E145" t="n">
-        <v>7508.53</v>
+        <v>135907.88</v>
       </c>
       <c r="F145" t="n">
         <v>0</v>
@@ -3923,22 +3923,22 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C146" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D146" t="n">
-        <v>33928</v>
+        <v>794029</v>
       </c>
       <c r="E146" t="n">
-        <v>823.55</v>
+        <v>7508.53</v>
       </c>
       <c r="F146" t="n">
         <v>0</v>
@@ -3947,22 +3947,22 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C147" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D147" t="n">
-        <v>139553</v>
+        <v>33928</v>
       </c>
       <c r="E147" t="n">
-        <v>7003.92</v>
+        <v>823.55</v>
       </c>
       <c r="F147" t="n">
         <v>0</v>
@@ -3976,7 +3976,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C148" s="2" t="n">
@@ -3986,7 +3986,7 @@
         <v>139553</v>
       </c>
       <c r="E148" t="n">
-        <v>717.6</v>
+        <v>7003.92</v>
       </c>
       <c r="F148" t="n">
         <v>0</v>
@@ -3995,22 +3995,22 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C149" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D149" t="n">
-        <v>796582</v>
+        <v>139553</v>
       </c>
       <c r="E149" t="n">
-        <v>1247.64</v>
+        <v>717.6</v>
       </c>
       <c r="F149" t="n">
         <v>0</v>
@@ -4019,22 +4019,22 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C150" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D150" t="n">
-        <v>30083</v>
+        <v>796582</v>
       </c>
       <c r="E150" t="n">
-        <v>215.07</v>
+        <v>1247.64</v>
       </c>
       <c r="F150" t="n">
         <v>0</v>
@@ -4043,22 +4043,22 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C151" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D151" t="n">
-        <v>795345</v>
+        <v>30083</v>
       </c>
       <c r="E151" t="n">
-        <v>204.29</v>
+        <v>215.07</v>
       </c>
       <c r="F151" t="n">
         <v>0</v>
@@ -4067,22 +4067,22 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C152" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D152" t="n">
-        <v>790595</v>
+        <v>795345</v>
       </c>
       <c r="E152" t="n">
-        <v>117.44</v>
+        <v>204.29</v>
       </c>
       <c r="F152" t="n">
         <v>0</v>
@@ -4091,22 +4091,22 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C153" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D153" t="n">
-        <v>30083</v>
+        <v>790595</v>
       </c>
       <c r="E153" t="n">
-        <v>727.5700000000001</v>
+        <v>117.44</v>
       </c>
       <c r="F153" t="n">
         <v>0</v>
@@ -4127,10 +4127,10 @@
         <v>46247</v>
       </c>
       <c r="D154" t="n">
-        <v>792121</v>
+        <v>30083</v>
       </c>
       <c r="E154" t="n">
-        <v>1095.64</v>
+        <v>727.5700000000001</v>
       </c>
       <c r="F154" t="n">
         <v>0</v>
@@ -4151,10 +4151,10 @@
         <v>46247</v>
       </c>
       <c r="D155" t="n">
-        <v>30307</v>
+        <v>792121</v>
       </c>
       <c r="E155" t="n">
-        <v>4626.15</v>
+        <v>1095.64</v>
       </c>
       <c r="F155" t="n">
         <v>0</v>
@@ -4163,22 +4163,22 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C156" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D156" t="n">
-        <v>794671</v>
+        <v>30307</v>
       </c>
       <c r="E156" t="n">
-        <v>1810.54</v>
+        <v>5277.28</v>
       </c>
       <c r="F156" t="n">
         <v>0</v>
@@ -4187,22 +4187,22 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C157" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D157" t="n">
-        <v>32816</v>
+        <v>794671</v>
       </c>
       <c r="E157" t="n">
-        <v>1721.48</v>
+        <v>1810.54</v>
       </c>
       <c r="F157" t="n">
         <v>0</v>
@@ -4211,22 +4211,22 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C158" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D158" t="n">
-        <v>139553</v>
+        <v>32816</v>
       </c>
       <c r="E158" t="n">
-        <v>260.72</v>
+        <v>1721.48</v>
       </c>
       <c r="F158" t="n">
         <v>0</v>
@@ -4235,22 +4235,22 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C159" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D159" t="n">
-        <v>789603</v>
+        <v>139553</v>
       </c>
       <c r="E159" t="n">
-        <v>7108.74</v>
+        <v>260.72</v>
       </c>
       <c r="F159" t="n">
         <v>0</v>
@@ -4259,22 +4259,22 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C160" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D160" t="n">
-        <v>33057</v>
+        <v>789603</v>
       </c>
       <c r="E160" t="n">
-        <v>414.8</v>
+        <v>7108.74</v>
       </c>
       <c r="F160" t="n">
         <v>0</v>
@@ -4283,12 +4283,12 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C161" s="2" t="n">
@@ -4298,55 +4298,55 @@
         <v>33057</v>
       </c>
       <c r="E161" t="n">
-        <v>12.37</v>
+        <v>414.8</v>
       </c>
       <c r="F161" t="n">
-        <v>12.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C162" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D162" t="n">
-        <v>47252</v>
+        <v>33057</v>
       </c>
       <c r="E162" t="n">
-        <v>9297.58</v>
+        <v>12.37</v>
       </c>
       <c r="F162" t="n">
-        <v>0</v>
+        <v>12.37</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C163" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D163" t="n">
-        <v>793186</v>
+        <v>47252</v>
       </c>
       <c r="E163" t="n">
-        <v>403.84</v>
+        <v>9297.58</v>
       </c>
       <c r="F163" t="n">
         <v>0</v>
@@ -4355,49 +4355,49 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C164" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D164" t="n">
-        <v>792141</v>
+        <v>793186</v>
       </c>
       <c r="E164" t="n">
-        <v>192.8</v>
+        <v>403.84</v>
       </c>
       <c r="F164" t="n">
-        <v>791.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C165" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D165" t="n">
-        <v>789228</v>
+        <v>792141</v>
       </c>
       <c r="E165" t="n">
-        <v>1335.26</v>
+        <v>192.8</v>
       </c>
       <c r="F165" t="n">
-        <v>0</v>
+        <v>791.11</v>
       </c>
     </row>
     <row r="166">
@@ -4415,10 +4415,10 @@
         <v>46247</v>
       </c>
       <c r="D166" t="n">
-        <v>793718</v>
+        <v>789228</v>
       </c>
       <c r="E166" t="n">
-        <v>2584.31</v>
+        <v>1335.26</v>
       </c>
       <c r="F166" t="n">
         <v>0</v>
@@ -4427,22 +4427,22 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C167" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D167" t="n">
-        <v>795345</v>
+        <v>793718</v>
       </c>
       <c r="E167" t="n">
-        <v>1829.8</v>
+        <v>2584.31</v>
       </c>
       <c r="F167" t="n">
         <v>0</v>
@@ -4456,17 +4456,17 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C168" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D168" t="n">
-        <v>30307</v>
+        <v>795345</v>
       </c>
       <c r="E168" t="n">
-        <v>56022.81</v>
+        <v>1829.8</v>
       </c>
       <c r="F168" t="n">
         <v>0</v>
@@ -4480,7 +4480,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C169" s="2" t="n">
@@ -4490,7 +4490,7 @@
         <v>30307</v>
       </c>
       <c r="E169" t="n">
-        <v>16391.14</v>
+        <v>56022.81</v>
       </c>
       <c r="F169" t="n">
         <v>0</v>
@@ -4499,22 +4499,22 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C170" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D170" t="n">
-        <v>789603</v>
+        <v>30307</v>
       </c>
       <c r="E170" t="n">
-        <v>1112.78</v>
+        <v>16391.14</v>
       </c>
       <c r="F170" t="n">
         <v>0</v>
@@ -4535,10 +4535,10 @@
         <v>46247</v>
       </c>
       <c r="D171" t="n">
-        <v>792141</v>
+        <v>789603</v>
       </c>
       <c r="E171" t="n">
-        <v>13.96</v>
+        <v>1112.78</v>
       </c>
       <c r="F171" t="n">
         <v>0</v>
@@ -4547,22 +4547,22 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C172" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D172" t="n">
-        <v>30307</v>
+        <v>792141</v>
       </c>
       <c r="E172" t="n">
-        <v>62217.48</v>
+        <v>13.96</v>
       </c>
       <c r="F172" t="n">
         <v>0</v>
@@ -4571,22 +4571,22 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C173" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D173" t="n">
-        <v>32816</v>
+        <v>30307</v>
       </c>
       <c r="E173" t="n">
-        <v>46.4</v>
+        <v>62217.48</v>
       </c>
       <c r="F173" t="n">
         <v>0</v>
@@ -4600,17 +4600,17 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C174" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D174" t="n">
-        <v>47252</v>
+        <v>32816</v>
       </c>
       <c r="E174" t="n">
-        <v>3157.51</v>
+        <v>46.4</v>
       </c>
       <c r="F174" t="n">
         <v>0</v>
@@ -4619,7 +4619,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4631,10 +4631,10 @@
         <v>46247</v>
       </c>
       <c r="D175" t="n">
-        <v>795345</v>
+        <v>47252</v>
       </c>
       <c r="E175" t="n">
-        <v>361.98</v>
+        <v>3157.51</v>
       </c>
       <c r="F175" t="n">
         <v>0</v>
@@ -4643,49 +4643,49 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C176" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D176" t="n">
-        <v>792141</v>
+        <v>795345</v>
       </c>
       <c r="E176" t="n">
-        <v>11160.8</v>
+        <v>361.98</v>
       </c>
       <c r="F176" t="n">
-        <v>321.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C177" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D177" t="n">
-        <v>793718</v>
+        <v>792141</v>
       </c>
       <c r="E177" t="n">
-        <v>145.46</v>
+        <v>11160.8</v>
       </c>
       <c r="F177" t="n">
-        <v>0</v>
+        <v>321.34</v>
       </c>
     </row>
     <row r="178">
@@ -4696,17 +4696,17 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C178" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D178" t="n">
-        <v>792121</v>
+        <v>793718</v>
       </c>
       <c r="E178" t="n">
-        <v>301.76</v>
+        <v>145.46</v>
       </c>
       <c r="F178" t="n">
         <v>0</v>
@@ -4715,22 +4715,22 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C179" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D179" t="n">
-        <v>792141</v>
+        <v>792121</v>
       </c>
       <c r="E179" t="n">
-        <v>169</v>
+        <v>301.76</v>
       </c>
       <c r="F179" t="n">
         <v>0</v>
@@ -4739,22 +4739,22 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C180" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D180" t="n">
-        <v>794671</v>
+        <v>792141</v>
       </c>
       <c r="E180" t="n">
-        <v>32.7</v>
+        <v>169</v>
       </c>
       <c r="F180" t="n">
         <v>0</v>
@@ -4763,25 +4763,25 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C181" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D181" t="n">
-        <v>31267</v>
+        <v>794671</v>
       </c>
       <c r="E181" t="n">
-        <v>17620.09</v>
+        <v>32.7</v>
       </c>
       <c r="F181" t="n">
-        <v>390.95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="182">
@@ -4799,13 +4799,13 @@
         <v>46247</v>
       </c>
       <c r="D182" t="n">
-        <v>789525</v>
+        <v>31267</v>
       </c>
       <c r="E182" t="n">
-        <v>5049.95</v>
+        <v>17620.09</v>
       </c>
       <c r="F182" t="n">
-        <v>836.2</v>
+        <v>390.95</v>
       </c>
     </row>
     <row r="183">
@@ -4823,37 +4823,37 @@
         <v>46247</v>
       </c>
       <c r="D183" t="n">
-        <v>789228</v>
+        <v>789525</v>
       </c>
       <c r="E183" t="n">
-        <v>113.33</v>
+        <v>5049.95</v>
       </c>
       <c r="F183" t="n">
-        <v>33.67</v>
+        <v>836.2</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C184" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D184" t="n">
-        <v>793186</v>
+        <v>789228</v>
       </c>
       <c r="E184" t="n">
-        <v>13.91</v>
+        <v>113.33</v>
       </c>
       <c r="F184" t="n">
-        <v>13.91</v>
+        <v>33.67</v>
       </c>
     </row>
     <row r="185">
@@ -4871,19 +4871,19 @@
         <v>46247</v>
       </c>
       <c r="D185" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="E185" t="n">
-        <v>5.57</v>
+        <v>13.91</v>
       </c>
       <c r="F185" t="n">
-        <v>5.57</v>
+        <v>13.91</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4895,34 +4895,34 @@
         <v>46247</v>
       </c>
       <c r="D186" t="n">
-        <v>31267</v>
+        <v>47252</v>
       </c>
       <c r="E186" t="n">
-        <v>14.99</v>
+        <v>5.57</v>
       </c>
       <c r="F186" t="n">
-        <v>0</v>
+        <v>5.57</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C187" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D187" t="n">
-        <v>30791</v>
+        <v>31267</v>
       </c>
       <c r="E187" t="n">
-        <v>1864.57</v>
+        <v>14.99</v>
       </c>
       <c r="F187" t="n">
         <v>0</v>
@@ -4931,12 +4931,12 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C188" s="2" t="n">
@@ -4946,7 +4946,7 @@
         <v>30791</v>
       </c>
       <c r="E188" t="n">
-        <v>17306.17</v>
+        <v>1864.57</v>
       </c>
       <c r="F188" t="n">
         <v>0</v>
@@ -4967,10 +4967,10 @@
         <v>46247</v>
       </c>
       <c r="D189" t="n">
-        <v>789603</v>
+        <v>30791</v>
       </c>
       <c r="E189" t="n">
-        <v>32311.1</v>
+        <v>18004.4</v>
       </c>
       <c r="F189" t="n">
         <v>0</v>
@@ -4991,10 +4991,10 @@
         <v>46247</v>
       </c>
       <c r="D190" t="n">
-        <v>30307</v>
+        <v>789603</v>
       </c>
       <c r="E190" t="n">
-        <v>343.86</v>
+        <v>32311.1</v>
       </c>
       <c r="F190" t="n">
         <v>0</v>
@@ -5015,10 +5015,10 @@
         <v>46247</v>
       </c>
       <c r="D191" t="n">
-        <v>792141</v>
+        <v>30307</v>
       </c>
       <c r="E191" t="n">
-        <v>16683.38</v>
+        <v>343.86</v>
       </c>
       <c r="F191" t="n">
         <v>0</v>
@@ -5027,22 +5027,22 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C192" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D192" t="n">
-        <v>794671</v>
+        <v>792141</v>
       </c>
       <c r="E192" t="n">
-        <v>4114.68</v>
+        <v>16683.38</v>
       </c>
       <c r="F192" t="n">
         <v>0</v>
@@ -5063,10 +5063,10 @@
         <v>46247</v>
       </c>
       <c r="D193" t="n">
-        <v>795345</v>
+        <v>794671</v>
       </c>
       <c r="E193" t="n">
-        <v>3919.83</v>
+        <v>4114.68</v>
       </c>
       <c r="F193" t="n">
         <v>0</v>
@@ -5080,17 +5080,17 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C194" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D194" t="n">
-        <v>794029</v>
+        <v>795345</v>
       </c>
       <c r="E194" t="n">
-        <v>31.16</v>
+        <v>3919.83</v>
       </c>
       <c r="F194" t="n">
         <v>0</v>
@@ -5099,22 +5099,22 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C195" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D195" t="n">
-        <v>33928</v>
+        <v>794029</v>
       </c>
       <c r="E195" t="n">
-        <v>46.44</v>
+        <v>31.16</v>
       </c>
       <c r="F195" t="n">
         <v>0</v>
@@ -5123,22 +5123,22 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C196" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D196" t="n">
-        <v>32816</v>
+        <v>33928</v>
       </c>
       <c r="E196" t="n">
-        <v>456.96</v>
+        <v>46.44</v>
       </c>
       <c r="F196" t="n">
         <v>0</v>
@@ -5147,22 +5147,22 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C197" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D197" t="n">
-        <v>31267</v>
+        <v>32816</v>
       </c>
       <c r="E197" t="n">
-        <v>914.84</v>
+        <v>456.96</v>
       </c>
       <c r="F197" t="n">
         <v>0</v>
@@ -5171,22 +5171,22 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C198" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D198" t="n">
-        <v>790595</v>
+        <v>31267</v>
       </c>
       <c r="E198" t="n">
-        <v>267.36</v>
+        <v>914.84</v>
       </c>
       <c r="F198" t="n">
         <v>0</v>
@@ -5207,10 +5207,10 @@
         <v>46247</v>
       </c>
       <c r="D199" t="n">
-        <v>30218</v>
+        <v>790595</v>
       </c>
       <c r="E199" t="n">
-        <v>2443.81</v>
+        <v>267.36</v>
       </c>
       <c r="F199" t="n">
         <v>0</v>
@@ -5219,22 +5219,22 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C200" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D200" t="n">
-        <v>47252</v>
+        <v>30218</v>
       </c>
       <c r="E200" t="n">
-        <v>16301.71</v>
+        <v>2443.81</v>
       </c>
       <c r="F200" t="n">
         <v>0</v>
@@ -5255,10 +5255,10 @@
         <v>46247</v>
       </c>
       <c r="D201" t="n">
-        <v>794671</v>
+        <v>47252</v>
       </c>
       <c r="E201" t="n">
-        <v>276.11</v>
+        <v>16383.13</v>
       </c>
       <c r="F201" t="n">
         <v>0</v>
@@ -5267,22 +5267,22 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C202" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D202" t="n">
-        <v>789603</v>
+        <v>794671</v>
       </c>
       <c r="E202" t="n">
-        <v>12294.52</v>
+        <v>276.11</v>
       </c>
       <c r="F202" t="n">
         <v>0</v>
@@ -5296,17 +5296,17 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C203" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D203" t="n">
-        <v>793186</v>
+        <v>789603</v>
       </c>
       <c r="E203" t="n">
-        <v>9305.58</v>
+        <v>12294.52</v>
       </c>
       <c r="F203" t="n">
         <v>0</v>
@@ -5315,22 +5315,22 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C204" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D204" t="n">
-        <v>139553</v>
+        <v>793186</v>
       </c>
       <c r="E204" t="n">
-        <v>8304.940000000001</v>
+        <v>9623.16</v>
       </c>
       <c r="F204" t="n">
         <v>0</v>
@@ -5339,22 +5339,22 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C205" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D205" t="n">
-        <v>792246</v>
+        <v>139553</v>
       </c>
       <c r="E205" t="n">
-        <v>587.38</v>
+        <v>8304.940000000001</v>
       </c>
       <c r="F205" t="n">
         <v>0</v>
@@ -5363,22 +5363,22 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C206" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D206" t="n">
-        <v>139553</v>
+        <v>792246</v>
       </c>
       <c r="E206" t="n">
-        <v>209.16</v>
+        <v>587.38</v>
       </c>
       <c r="F206" t="n">
         <v>0</v>
@@ -5399,10 +5399,10 @@
         <v>46247</v>
       </c>
       <c r="D207" t="n">
-        <v>30083</v>
+        <v>139553</v>
       </c>
       <c r="E207" t="n">
-        <v>627.34</v>
+        <v>209.16</v>
       </c>
       <c r="F207" t="n">
         <v>0</v>
@@ -5416,17 +5416,17 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C208" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D208" t="n">
-        <v>30307</v>
+        <v>30083</v>
       </c>
       <c r="E208" t="n">
-        <v>89210.53</v>
+        <v>627.34</v>
       </c>
       <c r="F208" t="n">
         <v>0</v>
@@ -5440,17 +5440,17 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C209" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D209" t="n">
-        <v>30083</v>
+        <v>795345</v>
       </c>
       <c r="E209" t="n">
-        <v>4660.64</v>
+        <v>329.64</v>
       </c>
       <c r="F209" t="n">
         <v>0</v>
@@ -5459,103 +5459,103 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C210" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D210" t="n">
-        <v>793718</v>
+        <v>30307</v>
       </c>
       <c r="E210" t="n">
-        <v>32373.83</v>
+        <v>89210.53</v>
       </c>
       <c r="F210" t="n">
-        <v>80.59999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C211" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D211" t="n">
-        <v>789661</v>
+        <v>30083</v>
       </c>
       <c r="E211" t="n">
-        <v>0</v>
+        <v>4660.64</v>
       </c>
       <c r="F211" t="n">
-        <v>32.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C212" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D212" t="n">
-        <v>33286</v>
+        <v>793718</v>
       </c>
       <c r="E212" t="n">
-        <v>3.99</v>
+        <v>32373.83</v>
       </c>
       <c r="F212" t="n">
-        <v>3.99</v>
+        <v>80.59999999999999</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C213" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D213" t="n">
-        <v>794671</v>
+        <v>789661</v>
       </c>
       <c r="E213" t="n">
-        <v>759.41</v>
+        <v>0</v>
       </c>
       <c r="F213" t="n">
-        <v>0</v>
+        <v>32.2</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5567,19 +5567,19 @@
         <v>46247</v>
       </c>
       <c r="D214" t="n">
-        <v>792121</v>
+        <v>33286</v>
       </c>
       <c r="E214" t="n">
-        <v>42.15</v>
+        <v>3.99</v>
       </c>
       <c r="F214" t="n">
-        <v>0</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5591,10 +5591,10 @@
         <v>46247</v>
       </c>
       <c r="D215" t="n">
-        <v>139553</v>
+        <v>794671</v>
       </c>
       <c r="E215" t="n">
-        <v>1300.72</v>
+        <v>759.41</v>
       </c>
       <c r="F215" t="n">
         <v>0</v>
@@ -5615,10 +5615,10 @@
         <v>46247</v>
       </c>
       <c r="D216" t="n">
-        <v>794671</v>
+        <v>792121</v>
       </c>
       <c r="E216" t="n">
-        <v>182.88</v>
+        <v>42.15</v>
       </c>
       <c r="F216" t="n">
         <v>0</v>
@@ -5627,22 +5627,22 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C217" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D217" t="n">
-        <v>33928</v>
+        <v>139553</v>
       </c>
       <c r="E217" t="n">
-        <v>1038.51</v>
+        <v>1300.72</v>
       </c>
       <c r="F217" t="n">
         <v>0</v>
@@ -5651,22 +5651,22 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C218" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D218" t="n">
-        <v>789525</v>
+        <v>794671</v>
       </c>
       <c r="E218" t="n">
-        <v>971.33</v>
+        <v>182.88</v>
       </c>
       <c r="F218" t="n">
         <v>0</v>
@@ -5687,10 +5687,10 @@
         <v>46247</v>
       </c>
       <c r="D219" t="n">
-        <v>33057</v>
+        <v>33928</v>
       </c>
       <c r="E219" t="n">
-        <v>89.06</v>
+        <v>1038.51</v>
       </c>
       <c r="F219" t="n">
         <v>0</v>
@@ -5699,12 +5699,12 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C220" s="2" t="n">
@@ -5714,7 +5714,7 @@
         <v>789525</v>
       </c>
       <c r="E220" t="n">
-        <v>6252.76</v>
+        <v>971.33</v>
       </c>
       <c r="F220" t="n">
         <v>0</v>
@@ -5723,12 +5723,12 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C221" s="2" t="n">
@@ -5738,7 +5738,7 @@
         <v>33057</v>
       </c>
       <c r="E221" t="n">
-        <v>4693.52</v>
+        <v>89.06</v>
       </c>
       <c r="F221" t="n">
         <v>0</v>
@@ -5747,22 +5747,22 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C222" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D222" t="n">
-        <v>794671</v>
+        <v>789525</v>
       </c>
       <c r="E222" t="n">
-        <v>3401.34</v>
+        <v>6252.76</v>
       </c>
       <c r="F222" t="n">
         <v>0</v>
@@ -5771,22 +5771,22 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C223" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D223" t="n">
-        <v>47252</v>
+        <v>33057</v>
       </c>
       <c r="E223" t="n">
-        <v>18942.73</v>
+        <v>4693.52</v>
       </c>
       <c r="F223" t="n">
         <v>0</v>
@@ -5795,22 +5795,22 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C224" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D224" t="n">
-        <v>30791</v>
+        <v>794671</v>
       </c>
       <c r="E224" t="n">
-        <v>5968.83</v>
+        <v>3401.34</v>
       </c>
       <c r="F224" t="n">
         <v>0</v>
@@ -5831,10 +5831,10 @@
         <v>46247</v>
       </c>
       <c r="D225" t="n">
-        <v>789525</v>
+        <v>47252</v>
       </c>
       <c r="E225" t="n">
-        <v>1143.67</v>
+        <v>18942.73</v>
       </c>
       <c r="F225" t="n">
         <v>0</v>
@@ -5848,17 +5848,17 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C226" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D226" t="n">
-        <v>30307</v>
+        <v>30791</v>
       </c>
       <c r="E226" t="n">
-        <v>575.88</v>
+        <v>6557.17</v>
       </c>
       <c r="F226" t="n">
         <v>0</v>
@@ -5872,17 +5872,17 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C227" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D227" t="n">
-        <v>30791</v>
+        <v>789525</v>
       </c>
       <c r="E227" t="n">
-        <v>44.88</v>
+        <v>1143.67</v>
       </c>
       <c r="F227" t="n">
         <v>0</v>
@@ -5891,22 +5891,22 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="C228" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D228" t="n">
-        <v>790595</v>
+        <v>30307</v>
       </c>
       <c r="E228" t="n">
-        <v>1151.94</v>
+        <v>575.88</v>
       </c>
       <c r="F228" t="n">
         <v>0</v>
@@ -5920,17 +5920,17 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="C229" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D229" t="n">
-        <v>47252</v>
+        <v>30791</v>
       </c>
       <c r="E229" t="n">
-        <v>26751.03</v>
+        <v>44.88</v>
       </c>
       <c r="F229" t="n">
         <v>0</v>
@@ -5951,10 +5951,10 @@
         <v>46247</v>
       </c>
       <c r="D230" t="n">
-        <v>794029</v>
+        <v>790595</v>
       </c>
       <c r="E230" t="n">
-        <v>4267.52</v>
+        <v>1151.94</v>
       </c>
       <c r="F230" t="n">
         <v>0</v>
@@ -5963,25 +5963,25 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C231" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D231" t="n">
-        <v>789603</v>
+        <v>47252</v>
       </c>
       <c r="E231" t="n">
-        <v>65039.36</v>
+        <v>26829.07</v>
       </c>
       <c r="F231" t="n">
-        <v>29466.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="232">
@@ -5992,17 +5992,17 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C232" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D232" t="n">
-        <v>795345</v>
+        <v>794029</v>
       </c>
       <c r="E232" t="n">
-        <v>561.4400000000001</v>
+        <v>4267.52</v>
       </c>
       <c r="F232" t="n">
         <v>0</v>
@@ -6011,49 +6011,49 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C233" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D233" t="n">
-        <v>31267</v>
+        <v>789603</v>
       </c>
       <c r="E233" t="n">
-        <v>26.27</v>
+        <v>66932.96000000001</v>
       </c>
       <c r="F233" t="n">
-        <v>0</v>
+        <v>41155.22</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C234" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D234" t="n">
-        <v>793186</v>
+        <v>795345</v>
       </c>
       <c r="E234" t="n">
-        <v>443.79</v>
+        <v>561.4400000000001</v>
       </c>
       <c r="F234" t="n">
-        <v>54.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="235">
@@ -6064,17 +6064,17 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C235" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D235" t="n">
-        <v>30307</v>
+        <v>31267</v>
       </c>
       <c r="E235" t="n">
-        <v>8740.709999999999</v>
+        <v>26.27</v>
       </c>
       <c r="F235" t="n">
         <v>0</v>
@@ -6083,46 +6083,46 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C236" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D236" t="n">
-        <v>794671</v>
+        <v>793186</v>
       </c>
       <c r="E236" t="n">
-        <v>1255.4</v>
+        <v>443.79</v>
       </c>
       <c r="F236" t="n">
-        <v>0</v>
+        <v>54.71</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C237" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D237" t="n">
-        <v>792141</v>
+        <v>30307</v>
       </c>
       <c r="E237" t="n">
-        <v>2529.9</v>
+        <v>8940.68</v>
       </c>
       <c r="F237" t="n">
         <v>0</v>
@@ -6131,22 +6131,22 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C238" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D238" t="n">
-        <v>793186</v>
+        <v>794671</v>
       </c>
       <c r="E238" t="n">
-        <v>146.11</v>
+        <v>1255.4</v>
       </c>
       <c r="F238" t="n">
         <v>0</v>
@@ -6155,22 +6155,22 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C239" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D239" t="n">
-        <v>30083</v>
+        <v>790595</v>
       </c>
       <c r="E239" t="n">
-        <v>3299.7</v>
+        <v>1177.54</v>
       </c>
       <c r="F239" t="n">
         <v>0</v>
@@ -6179,22 +6179,22 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C240" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D240" t="n">
-        <v>789603</v>
+        <v>792141</v>
       </c>
       <c r="E240" t="n">
-        <v>2033.79</v>
+        <v>2529.9</v>
       </c>
       <c r="F240" t="n">
         <v>0</v>
@@ -6203,22 +6203,22 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C241" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D241" t="n">
-        <v>33057</v>
+        <v>793186</v>
       </c>
       <c r="E241" t="n">
-        <v>11969.1</v>
+        <v>146.11</v>
       </c>
       <c r="F241" t="n">
         <v>0</v>
@@ -6227,22 +6227,22 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C242" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D242" t="n">
-        <v>33928</v>
+        <v>30083</v>
       </c>
       <c r="E242" t="n">
-        <v>1729.68</v>
+        <v>3299.7</v>
       </c>
       <c r="F242" t="n">
         <v>0</v>
@@ -6251,22 +6251,22 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C243" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D243" t="n">
-        <v>792121</v>
+        <v>789603</v>
       </c>
       <c r="E243" t="n">
-        <v>1472.58</v>
+        <v>2033.79</v>
       </c>
       <c r="F243" t="n">
         <v>0</v>
@@ -6275,22 +6275,22 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C244" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D244" t="n">
-        <v>792121</v>
+        <v>33057</v>
       </c>
       <c r="E244" t="n">
-        <v>501.32</v>
+        <v>11969.1</v>
       </c>
       <c r="F244" t="n">
         <v>0</v>
@@ -6299,22 +6299,22 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C245" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D245" t="n">
-        <v>32816</v>
+        <v>33928</v>
       </c>
       <c r="E245" t="n">
-        <v>74.84999999999999</v>
+        <v>1840.84</v>
       </c>
       <c r="F245" t="n">
         <v>0</v>
@@ -6323,22 +6323,22 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C246" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D246" t="n">
-        <v>139553</v>
+        <v>792121</v>
       </c>
       <c r="E246" t="n">
-        <v>2570.35</v>
+        <v>1472.58</v>
       </c>
       <c r="F246" t="n">
         <v>0</v>
@@ -6347,22 +6347,22 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C247" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D247" t="n">
-        <v>33286</v>
+        <v>792121</v>
       </c>
       <c r="E247" t="n">
-        <v>106.92</v>
+        <v>501.32</v>
       </c>
       <c r="F247" t="n">
         <v>0</v>
@@ -6371,22 +6371,22 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C248" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D248" t="n">
-        <v>139553</v>
+        <v>32816</v>
       </c>
       <c r="E248" t="n">
-        <v>611.88</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="F248" t="n">
         <v>0</v>
@@ -6395,22 +6395,22 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C249" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D249" t="n">
-        <v>790595</v>
+        <v>139553</v>
       </c>
       <c r="E249" t="n">
-        <v>294.6</v>
+        <v>2570.35</v>
       </c>
       <c r="F249" t="n">
         <v>0</v>
@@ -6419,12 +6419,12 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C250" s="2" t="n">
@@ -6434,9 +6434,81 @@
         <v>795345</v>
       </c>
       <c r="E250" t="n">
+        <v>283.88</v>
+      </c>
+      <c r="F250" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D251" t="n">
+        <v>33286</v>
+      </c>
+      <c r="E251" t="n">
+        <v>106.92</v>
+      </c>
+      <c r="F251" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D252" t="n">
+        <v>139553</v>
+      </c>
+      <c r="E252" t="n">
+        <v>611.88</v>
+      </c>
+      <c r="F252" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D253" t="n">
+        <v>795345</v>
+      </c>
+      <c r="E253" t="n">
         <v>169.57</v>
       </c>
-      <c r="F250" t="n">
+      <c r="F253" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 13:45:04
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F257"/>
+  <dimension ref="A1:F258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,7 +506,7 @@
         <v>47252</v>
       </c>
       <c r="E3" t="n">
-        <v>16553.95</v>
+        <v>19481.27</v>
       </c>
       <c r="F3" t="n">
         <v>3810.55</v>
@@ -530,7 +530,7 @@
         <v>33928</v>
       </c>
       <c r="E4" t="n">
-        <v>31977.43</v>
+        <v>31990.52</v>
       </c>
       <c r="F4" t="n">
         <v>9689.16</v>
@@ -578,7 +578,7 @@
         <v>33928</v>
       </c>
       <c r="E6" t="n">
-        <v>7699.08</v>
+        <v>7815.55</v>
       </c>
       <c r="F6" t="n">
         <v>391.48</v>
@@ -602,7 +602,7 @@
         <v>30791</v>
       </c>
       <c r="E7" t="n">
-        <v>13281.09</v>
+        <v>13846.09</v>
       </c>
       <c r="F7" t="n">
         <v>3111.54</v>
@@ -626,7 +626,7 @@
         <v>789228</v>
       </c>
       <c r="E8" t="n">
-        <v>2559.37</v>
+        <v>4007.92</v>
       </c>
       <c r="F8" t="n">
         <v>178.87</v>
@@ -650,7 +650,7 @@
         <v>31267</v>
       </c>
       <c r="E9" t="n">
-        <v>10601.66</v>
+        <v>10693.14</v>
       </c>
       <c r="F9" t="n">
         <v>758.7</v>
@@ -674,7 +674,7 @@
         <v>33928</v>
       </c>
       <c r="E10" t="n">
-        <v>6240.03</v>
+        <v>6432.83</v>
       </c>
       <c r="F10" t="n">
         <v>935.13</v>
@@ -698,7 +698,7 @@
         <v>789525</v>
       </c>
       <c r="E11" t="n">
-        <v>1448.69</v>
+        <v>1707.89</v>
       </c>
       <c r="F11" t="n">
         <v>98.76000000000001</v>
@@ -770,7 +770,7 @@
         <v>793186</v>
       </c>
       <c r="E14" t="n">
-        <v>1957.2</v>
+        <v>2045.06</v>
       </c>
       <c r="F14" t="n">
         <v>113.14</v>
@@ -1154,7 +1154,7 @@
         <v>31267</v>
       </c>
       <c r="E30" t="n">
-        <v>143377.21</v>
+        <v>144456.99</v>
       </c>
       <c r="F30" t="n">
         <v>0</v>
@@ -1456,20 +1456,20 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D43" t="n">
-        <v>30791</v>
+        <v>31267</v>
       </c>
       <c r="E43" t="n">
-        <v>12450.22</v>
+        <v>7125.01</v>
       </c>
       <c r="F43" t="n">
-        <v>685.66</v>
+        <v>165.42</v>
       </c>
     </row>
     <row r="44">
@@ -1487,13 +1487,13 @@
         <v>46247</v>
       </c>
       <c r="D44" t="n">
-        <v>793718</v>
+        <v>30791</v>
       </c>
       <c r="E44" t="n">
-        <v>4707.29</v>
+        <v>13191.17</v>
       </c>
       <c r="F44" t="n">
-        <v>120.72</v>
+        <v>685.66</v>
       </c>
     </row>
     <row r="45">
@@ -1504,20 +1504,20 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D45" t="n">
-        <v>33286</v>
+        <v>793718</v>
       </c>
       <c r="E45" t="n">
-        <v>554.26</v>
+        <v>4718</v>
       </c>
       <c r="F45" t="n">
-        <v>91.13</v>
+        <v>120.72</v>
       </c>
     </row>
     <row r="46">
@@ -1528,20 +1528,20 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D46" t="n">
-        <v>31267</v>
+        <v>33286</v>
       </c>
       <c r="E46" t="n">
-        <v>5042.32</v>
+        <v>697.6900000000001</v>
       </c>
       <c r="F46" t="n">
-        <v>165.42</v>
+        <v>91.13</v>
       </c>
     </row>
     <row r="47">
@@ -1562,7 +1562,7 @@
         <v>47252</v>
       </c>
       <c r="E47" t="n">
-        <v>13562.78</v>
+        <v>18384.3</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
@@ -1571,22 +1571,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D48" t="n">
-        <v>30307</v>
+        <v>789228</v>
       </c>
       <c r="E48" t="n">
-        <v>10724.33</v>
+        <v>2977.83</v>
       </c>
       <c r="F48" t="n">
         <v>0</v>
@@ -1595,22 +1595,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D49" t="n">
-        <v>789228</v>
+        <v>30307</v>
       </c>
       <c r="E49" t="n">
-        <v>2962.04</v>
+        <v>10724.33</v>
       </c>
       <c r="F49" t="n">
         <v>0</v>
@@ -1634,7 +1634,7 @@
         <v>33928</v>
       </c>
       <c r="E50" t="n">
-        <v>2324.75</v>
+        <v>2347.01</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
@@ -1667,22 +1667,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>LUIS REGINALDO ALMEIDA GOMES</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D52" t="n">
-        <v>30307</v>
+        <v>792121</v>
       </c>
       <c r="E52" t="n">
-        <v>2807.48</v>
+        <v>7508.76</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
@@ -1691,22 +1691,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>LUIS REGINALDO ALMEIDA GOMES</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D53" t="n">
-        <v>30083</v>
+        <v>30307</v>
       </c>
       <c r="E53" t="n">
-        <v>184.44</v>
+        <v>2807.48</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
@@ -1715,22 +1715,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D54" t="n">
-        <v>792121</v>
+        <v>30083</v>
       </c>
       <c r="E54" t="n">
-        <v>3087.81</v>
+        <v>184.44</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
@@ -1751,10 +1751,10 @@
         <v>46247</v>
       </c>
       <c r="D55" t="n">
-        <v>789603</v>
+        <v>792121</v>
       </c>
       <c r="E55" t="n">
-        <v>16803.49</v>
+        <v>3087.81</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
@@ -1775,10 +1775,10 @@
         <v>46247</v>
       </c>
       <c r="D56" t="n">
-        <v>795345</v>
+        <v>789603</v>
       </c>
       <c r="E56" t="n">
-        <v>495.23</v>
+        <v>17472.29</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
@@ -1787,22 +1787,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D57" t="n">
-        <v>30307</v>
+        <v>795345</v>
       </c>
       <c r="E57" t="n">
-        <v>17764.94</v>
+        <v>495.23</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
@@ -1811,22 +1811,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D58" t="n">
-        <v>792141</v>
+        <v>30307</v>
       </c>
       <c r="E58" t="n">
-        <v>20.66</v>
+        <v>17764.94</v>
       </c>
       <c r="F58" t="n">
         <v>0</v>
@@ -1835,22 +1835,22 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D59" t="n">
-        <v>792121</v>
+        <v>792141</v>
       </c>
       <c r="E59" t="n">
-        <v>2921.44</v>
+        <v>20.66</v>
       </c>
       <c r="F59" t="n">
         <v>0</v>
@@ -2138,7 +2138,7 @@
         <v>30791</v>
       </c>
       <c r="E71" t="n">
-        <v>12440.05</v>
+        <v>12485.22</v>
       </c>
       <c r="F71" t="n">
         <v>1524.6</v>
@@ -2162,7 +2162,7 @@
         <v>33286</v>
       </c>
       <c r="E72" t="n">
-        <v>1141.11</v>
+        <v>1213.82</v>
       </c>
       <c r="F72" t="n">
         <v>230.41</v>
@@ -2176,20 +2176,20 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D73" t="n">
-        <v>793718</v>
+        <v>33286</v>
       </c>
       <c r="E73" t="n">
-        <v>630.33</v>
+        <v>2314.28</v>
       </c>
       <c r="F73" t="n">
-        <v>238.95</v>
+        <v>327.9</v>
       </c>
     </row>
     <row r="74">
@@ -2200,41 +2200,41 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D74" t="n">
-        <v>47252</v>
+        <v>793718</v>
       </c>
       <c r="E74" t="n">
-        <v>19.77</v>
+        <v>630.33</v>
       </c>
       <c r="F74" t="n">
-        <v>0</v>
+        <v>238.95</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D75" t="n">
-        <v>793718</v>
+        <v>47252</v>
       </c>
       <c r="E75" t="n">
-        <v>1555.69</v>
+        <v>19.77</v>
       </c>
       <c r="F75" t="n">
         <v>0</v>
@@ -2243,22 +2243,22 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D76" t="n">
-        <v>31267</v>
+        <v>793718</v>
       </c>
       <c r="E76" t="n">
-        <v>3618.49</v>
+        <v>1555.69</v>
       </c>
       <c r="F76" t="n">
         <v>0</v>
@@ -2279,10 +2279,10 @@
         <v>46247</v>
       </c>
       <c r="D77" t="n">
-        <v>793718</v>
+        <v>31267</v>
       </c>
       <c r="E77" t="n">
-        <v>7060.3</v>
+        <v>3631.64</v>
       </c>
       <c r="F77" t="n">
         <v>0</v>
@@ -2291,25 +2291,25 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D78" t="n">
-        <v>33286</v>
+        <v>793718</v>
       </c>
       <c r="E78" t="n">
-        <v>2301.21</v>
+        <v>7136.7</v>
       </c>
       <c r="F78" t="n">
-        <v>327.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -2354,7 +2354,7 @@
         <v>33286</v>
       </c>
       <c r="E80" t="n">
-        <v>1887.86</v>
+        <v>2165.03</v>
       </c>
       <c r="F80" t="n">
         <v>0</v>
@@ -2642,7 +2642,7 @@
         <v>47252</v>
       </c>
       <c r="E92" t="n">
-        <v>16210.06</v>
+        <v>16306.51</v>
       </c>
       <c r="F92" t="n">
         <v>0</v>
@@ -2690,7 +2690,7 @@
         <v>792141</v>
       </c>
       <c r="E94" t="n">
-        <v>207.9</v>
+        <v>98.15000000000001</v>
       </c>
       <c r="F94" t="n">
         <v>0</v>
@@ -2867,25 +2867,25 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D102" t="n">
-        <v>795345</v>
+        <v>789228</v>
       </c>
       <c r="E102" t="n">
-        <v>40.89</v>
+        <v>291.29</v>
       </c>
       <c r="F102" t="n">
-        <v>0</v>
+        <v>159.28</v>
       </c>
     </row>
     <row r="103">
@@ -2896,17 +2896,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D103" t="n">
-        <v>792121</v>
+        <v>795345</v>
       </c>
       <c r="E103" t="n">
-        <v>5765.53</v>
+        <v>40.89</v>
       </c>
       <c r="F103" t="n">
         <v>0</v>
@@ -2915,22 +2915,22 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D104" t="n">
-        <v>30083</v>
+        <v>792121</v>
       </c>
       <c r="E104" t="n">
-        <v>137.67</v>
+        <v>5765.53</v>
       </c>
       <c r="F104" t="n">
         <v>0</v>
@@ -2951,10 +2951,10 @@
         <v>46247</v>
       </c>
       <c r="D105" t="n">
-        <v>33928</v>
+        <v>30083</v>
       </c>
       <c r="E105" t="n">
-        <v>12606.83</v>
+        <v>137.67</v>
       </c>
       <c r="F105" t="n">
         <v>0</v>
@@ -2963,49 +2963,49 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D106" t="n">
-        <v>795345</v>
+        <v>33928</v>
       </c>
       <c r="E106" t="n">
-        <v>1928.91</v>
+        <v>12719.52</v>
       </c>
       <c r="F106" t="n">
-        <v>0</v>
+        <v>30.75</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D107" t="n">
-        <v>789228</v>
+        <v>795345</v>
       </c>
       <c r="E107" t="n">
-        <v>219.27</v>
+        <v>1928.91</v>
       </c>
       <c r="F107" t="n">
-        <v>159.28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108">
@@ -3023,10 +3023,10 @@
         <v>46247</v>
       </c>
       <c r="D108" t="n">
-        <v>33286</v>
+        <v>30791</v>
       </c>
       <c r="E108" t="n">
-        <v>4043.68</v>
+        <v>3253.23</v>
       </c>
       <c r="F108" t="n">
         <v>0</v>
@@ -3047,10 +3047,10 @@
         <v>46247</v>
       </c>
       <c r="D109" t="n">
-        <v>30791</v>
+        <v>33286</v>
       </c>
       <c r="E109" t="n">
-        <v>3015.8</v>
+        <v>4043.68</v>
       </c>
       <c r="F109" t="n">
         <v>0</v>
@@ -3194,10 +3194,10 @@
         <v>30307</v>
       </c>
       <c r="E115" t="n">
-        <v>44784.87</v>
+        <v>44785.4</v>
       </c>
       <c r="F115" t="n">
-        <v>1915.76</v>
+        <v>4936.24</v>
       </c>
     </row>
     <row r="116">
@@ -3299,22 +3299,22 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D120" t="n">
-        <v>33286</v>
+        <v>30307</v>
       </c>
       <c r="E120" t="n">
-        <v>1376.17</v>
+        <v>2286.6</v>
       </c>
       <c r="F120" t="n">
         <v>0</v>
@@ -3323,22 +3323,22 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D121" t="n">
-        <v>794029</v>
+        <v>33286</v>
       </c>
       <c r="E121" t="n">
-        <v>731.21</v>
+        <v>1376.17</v>
       </c>
       <c r="F121" t="n">
         <v>0</v>
@@ -3347,22 +3347,22 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D122" t="n">
-        <v>792246</v>
+        <v>794029</v>
       </c>
       <c r="E122" t="n">
-        <v>1255.6</v>
+        <v>731.21</v>
       </c>
       <c r="F122" t="n">
         <v>0</v>
@@ -3371,22 +3371,22 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D123" t="n">
-        <v>789603</v>
+        <v>792246</v>
       </c>
       <c r="E123" t="n">
-        <v>3636.01</v>
+        <v>1255.6</v>
       </c>
       <c r="F123" t="n">
         <v>0</v>
@@ -3395,22 +3395,22 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D124" t="n">
-        <v>31267</v>
+        <v>789603</v>
       </c>
       <c r="E124" t="n">
-        <v>1127.62</v>
+        <v>3636.01</v>
       </c>
       <c r="F124" t="n">
         <v>0</v>
@@ -3419,22 +3419,22 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D125" t="n">
-        <v>30307</v>
+        <v>31267</v>
       </c>
       <c r="E125" t="n">
-        <v>1208.36</v>
+        <v>1127.62</v>
       </c>
       <c r="F125" t="n">
         <v>0</v>
@@ -3578,7 +3578,7 @@
         <v>47252</v>
       </c>
       <c r="E131" t="n">
-        <v>18278.45</v>
+        <v>18862.95</v>
       </c>
       <c r="F131" t="n">
         <v>1686.2</v>
@@ -3602,7 +3602,7 @@
         <v>47252</v>
       </c>
       <c r="E132" t="n">
-        <v>24588.02</v>
+        <v>24920.77</v>
       </c>
       <c r="F132" t="n">
         <v>4460.38</v>
@@ -3647,10 +3647,10 @@
         <v>46247</v>
       </c>
       <c r="D134" t="n">
-        <v>30791</v>
+        <v>33057</v>
       </c>
       <c r="E134" t="n">
-        <v>33.08</v>
+        <v>42.76</v>
       </c>
       <c r="F134" t="n">
         <v>0</v>
@@ -3659,22 +3659,22 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D135" t="n">
-        <v>31267</v>
+        <v>30791</v>
       </c>
       <c r="E135" t="n">
-        <v>160.86</v>
+        <v>33.08</v>
       </c>
       <c r="F135" t="n">
         <v>0</v>
@@ -3683,22 +3683,22 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D136" t="n">
-        <v>139553</v>
+        <v>31267</v>
       </c>
       <c r="E136" t="n">
-        <v>1106.98</v>
+        <v>160.86</v>
       </c>
       <c r="F136" t="n">
         <v>0</v>
@@ -3719,10 +3719,10 @@
         <v>46247</v>
       </c>
       <c r="D137" t="n">
-        <v>33286</v>
+        <v>139553</v>
       </c>
       <c r="E137" t="n">
-        <v>7676.83</v>
+        <v>1106.98</v>
       </c>
       <c r="F137" t="n">
         <v>0</v>
@@ -3731,22 +3731,22 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D138" t="n">
-        <v>30307</v>
+        <v>33286</v>
       </c>
       <c r="E138" t="n">
-        <v>507.68</v>
+        <v>7688.18</v>
       </c>
       <c r="F138" t="n">
         <v>0</v>
@@ -3755,22 +3755,22 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D139" t="n">
-        <v>33057</v>
+        <v>30307</v>
       </c>
       <c r="E139" t="n">
-        <v>146.56</v>
+        <v>507.68</v>
       </c>
       <c r="F139" t="n">
         <v>0</v>
@@ -3779,25 +3779,25 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D140" t="n">
-        <v>789661</v>
+        <v>33057</v>
       </c>
       <c r="E140" t="n">
-        <v>37.05</v>
+        <v>146.56</v>
       </c>
       <c r="F140" t="n">
-        <v>258.83</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141">
@@ -3815,58 +3815,58 @@
         <v>46247</v>
       </c>
       <c r="D141" t="n">
-        <v>793186</v>
+        <v>789661</v>
       </c>
       <c r="E141" t="n">
-        <v>442.74</v>
+        <v>37.05</v>
       </c>
       <c r="F141" t="n">
-        <v>97.42</v>
+        <v>258.83</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C142" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D142" t="n">
-        <v>794029</v>
+        <v>793186</v>
       </c>
       <c r="E142" t="n">
-        <v>8574.25</v>
+        <v>637.28</v>
       </c>
       <c r="F142" t="n">
-        <v>0</v>
+        <v>97.42</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C143" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D143" t="n">
-        <v>31267</v>
+        <v>794671</v>
       </c>
       <c r="E143" t="n">
-        <v>63.33</v>
+        <v>1295.61</v>
       </c>
       <c r="F143" t="n">
         <v>0</v>
@@ -3880,17 +3880,17 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C144" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D144" t="n">
-        <v>790595</v>
+        <v>30083</v>
       </c>
       <c r="E144" t="n">
-        <v>1274.18</v>
+        <v>227.05</v>
       </c>
       <c r="F144" t="n">
         <v>0</v>
@@ -3904,17 +3904,17 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C145" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D145" t="n">
-        <v>792121</v>
+        <v>794029</v>
       </c>
       <c r="E145" t="n">
-        <v>4843.19</v>
+        <v>8574.25</v>
       </c>
       <c r="F145" t="n">
         <v>0</v>
@@ -3923,22 +3923,22 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C146" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D146" t="n">
-        <v>794671</v>
+        <v>31267</v>
       </c>
       <c r="E146" t="n">
-        <v>495.9</v>
+        <v>63.33</v>
       </c>
       <c r="F146" t="n">
         <v>0</v>
@@ -3947,22 +3947,22 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C147" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D147" t="n">
-        <v>47252</v>
+        <v>790595</v>
       </c>
       <c r="E147" t="n">
-        <v>291.52</v>
+        <v>1274.18</v>
       </c>
       <c r="F147" t="n">
         <v>0</v>
@@ -3971,22 +3971,22 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C148" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D148" t="n">
-        <v>31267</v>
+        <v>792121</v>
       </c>
       <c r="E148" t="n">
-        <v>138007.45</v>
+        <v>4843.19</v>
       </c>
       <c r="F148" t="n">
         <v>0</v>
@@ -3995,22 +3995,22 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C149" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D149" t="n">
-        <v>794029</v>
+        <v>47252</v>
       </c>
       <c r="E149" t="n">
-        <v>7508.53</v>
+        <v>291.52</v>
       </c>
       <c r="F149" t="n">
         <v>0</v>
@@ -4019,22 +4019,22 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C150" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D150" t="n">
-        <v>33928</v>
+        <v>31267</v>
       </c>
       <c r="E150" t="n">
-        <v>823.55</v>
+        <v>138007.45</v>
       </c>
       <c r="F150" t="n">
         <v>0</v>
@@ -4048,17 +4048,17 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C151" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D151" t="n">
-        <v>139553</v>
+        <v>794029</v>
       </c>
       <c r="E151" t="n">
-        <v>7003.92</v>
+        <v>7508.53</v>
       </c>
       <c r="F151" t="n">
         <v>0</v>
@@ -4067,22 +4067,22 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C152" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D152" t="n">
-        <v>139553</v>
+        <v>33928</v>
       </c>
       <c r="E152" t="n">
-        <v>717.6</v>
+        <v>823.55</v>
       </c>
       <c r="F152" t="n">
         <v>0</v>
@@ -4091,22 +4091,22 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C153" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D153" t="n">
-        <v>796582</v>
+        <v>139553</v>
       </c>
       <c r="E153" t="n">
-        <v>1247.64</v>
+        <v>7003.92</v>
       </c>
       <c r="F153" t="n">
         <v>0</v>
@@ -4120,17 +4120,17 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C154" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D154" t="n">
-        <v>30083</v>
+        <v>139553</v>
       </c>
       <c r="E154" t="n">
-        <v>215.07</v>
+        <v>717.6</v>
       </c>
       <c r="F154" t="n">
         <v>0</v>
@@ -4139,22 +4139,22 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C155" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D155" t="n">
-        <v>139553</v>
+        <v>796582</v>
       </c>
       <c r="E155" t="n">
-        <v>1621.76</v>
+        <v>2647.34</v>
       </c>
       <c r="F155" t="n">
         <v>0</v>
@@ -4163,22 +4163,22 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C156" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D156" t="n">
-        <v>795345</v>
+        <v>139553</v>
       </c>
       <c r="E156" t="n">
-        <v>204.29</v>
+        <v>1621.76</v>
       </c>
       <c r="F156" t="n">
         <v>0</v>
@@ -4187,22 +4187,22 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C157" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D157" t="n">
-        <v>790595</v>
+        <v>795345</v>
       </c>
       <c r="E157" t="n">
-        <v>117.44</v>
+        <v>204.29</v>
       </c>
       <c r="F157" t="n">
         <v>0</v>
@@ -4211,22 +4211,22 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C158" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D158" t="n">
-        <v>30083</v>
+        <v>790595</v>
       </c>
       <c r="E158" t="n">
-        <v>727.5700000000001</v>
+        <v>117.44</v>
       </c>
       <c r="F158" t="n">
         <v>0</v>
@@ -4247,10 +4247,10 @@
         <v>46247</v>
       </c>
       <c r="D159" t="n">
-        <v>792121</v>
+        <v>30083</v>
       </c>
       <c r="E159" t="n">
-        <v>1095.64</v>
+        <v>727.5700000000001</v>
       </c>
       <c r="F159" t="n">
         <v>0</v>
@@ -4271,10 +4271,10 @@
         <v>46247</v>
       </c>
       <c r="D160" t="n">
-        <v>30307</v>
+        <v>792121</v>
       </c>
       <c r="E160" t="n">
-        <v>6580.35</v>
+        <v>1095.64</v>
       </c>
       <c r="F160" t="n">
         <v>0</v>
@@ -4283,22 +4283,22 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C161" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D161" t="n">
-        <v>794671</v>
+        <v>30307</v>
       </c>
       <c r="E161" t="n">
-        <v>1810.54</v>
+        <v>6580.35</v>
       </c>
       <c r="F161" t="n">
         <v>0</v>
@@ -4307,22 +4307,22 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C162" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D162" t="n">
-        <v>32816</v>
+        <v>794671</v>
       </c>
       <c r="E162" t="n">
-        <v>1721.48</v>
+        <v>1810.54</v>
       </c>
       <c r="F162" t="n">
         <v>0</v>
@@ -4331,22 +4331,22 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C163" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D163" t="n">
-        <v>789603</v>
+        <v>32816</v>
       </c>
       <c r="E163" t="n">
-        <v>7108.74</v>
+        <v>1721.48</v>
       </c>
       <c r="F163" t="n">
         <v>0</v>
@@ -4355,22 +4355,22 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C164" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D164" t="n">
-        <v>33057</v>
+        <v>789603</v>
       </c>
       <c r="E164" t="n">
-        <v>509.7</v>
+        <v>7108.74</v>
       </c>
       <c r="F164" t="n">
         <v>0</v>
@@ -4379,12 +4379,12 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C165" s="2" t="n">
@@ -4394,55 +4394,55 @@
         <v>33057</v>
       </c>
       <c r="E165" t="n">
-        <v>12.37</v>
+        <v>631.5700000000001</v>
       </c>
       <c r="F165" t="n">
-        <v>12.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C166" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D166" t="n">
-        <v>47252</v>
+        <v>33057</v>
       </c>
       <c r="E166" t="n">
-        <v>10857.89</v>
+        <v>12.37</v>
       </c>
       <c r="F166" t="n">
-        <v>0</v>
+        <v>12.37</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C167" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D167" t="n">
-        <v>793186</v>
+        <v>47252</v>
       </c>
       <c r="E167" t="n">
-        <v>403.84</v>
+        <v>12079.28</v>
       </c>
       <c r="F167" t="n">
         <v>0</v>
@@ -4451,49 +4451,49 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C168" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D168" t="n">
-        <v>792141</v>
+        <v>793186</v>
       </c>
       <c r="E168" t="n">
-        <v>274.78</v>
+        <v>403.84</v>
       </c>
       <c r="F168" t="n">
-        <v>791.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C169" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D169" t="n">
-        <v>793718</v>
+        <v>792141</v>
       </c>
       <c r="E169" t="n">
-        <v>3647.94</v>
+        <v>274.78</v>
       </c>
       <c r="F169" t="n">
-        <v>0</v>
+        <v>791.11</v>
       </c>
     </row>
     <row r="170">
@@ -4511,10 +4511,10 @@
         <v>46247</v>
       </c>
       <c r="D170" t="n">
-        <v>789228</v>
+        <v>793718</v>
       </c>
       <c r="E170" t="n">
-        <v>1588.58</v>
+        <v>3647.94</v>
       </c>
       <c r="F170" t="n">
         <v>0</v>
@@ -4523,22 +4523,22 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C171" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D171" t="n">
-        <v>795345</v>
+        <v>789228</v>
       </c>
       <c r="E171" t="n">
-        <v>1829.8</v>
+        <v>1588.58</v>
       </c>
       <c r="F171" t="n">
         <v>0</v>
@@ -4547,22 +4547,22 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C172" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D172" t="n">
-        <v>792141</v>
+        <v>795345</v>
       </c>
       <c r="E172" t="n">
-        <v>276.6</v>
+        <v>1829.8</v>
       </c>
       <c r="F172" t="n">
         <v>0</v>
@@ -4571,22 +4571,22 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C173" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D173" t="n">
-        <v>30307</v>
+        <v>792141</v>
       </c>
       <c r="E173" t="n">
-        <v>56946.39</v>
+        <v>276.6</v>
       </c>
       <c r="F173" t="n">
         <v>0</v>
@@ -4610,7 +4610,7 @@
         <v>30307</v>
       </c>
       <c r="E174" t="n">
-        <v>17578.72</v>
+        <v>25047.44</v>
       </c>
       <c r="F174" t="n">
         <v>0</v>
@@ -4619,22 +4619,22 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C175" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D175" t="n">
-        <v>789603</v>
+        <v>30307</v>
       </c>
       <c r="E175" t="n">
-        <v>1112.78</v>
+        <v>57414.21</v>
       </c>
       <c r="F175" t="n">
         <v>0</v>
@@ -4655,10 +4655,10 @@
         <v>46247</v>
       </c>
       <c r="D176" t="n">
-        <v>792141</v>
+        <v>789603</v>
       </c>
       <c r="E176" t="n">
-        <v>13.96</v>
+        <v>1112.78</v>
       </c>
       <c r="F176" t="n">
         <v>0</v>
@@ -4667,22 +4667,22 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C177" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D177" t="n">
-        <v>30307</v>
+        <v>792141</v>
       </c>
       <c r="E177" t="n">
-        <v>62217.48</v>
+        <v>13.96</v>
       </c>
       <c r="F177" t="n">
         <v>0</v>
@@ -4691,22 +4691,22 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C178" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D178" t="n">
-        <v>32816</v>
+        <v>30307</v>
       </c>
       <c r="E178" t="n">
-        <v>75.75</v>
+        <v>63661.12</v>
       </c>
       <c r="F178" t="n">
         <v>0</v>
@@ -4720,17 +4720,17 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C179" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D179" t="n">
-        <v>47252</v>
+        <v>32816</v>
       </c>
       <c r="E179" t="n">
-        <v>3157.51</v>
+        <v>75.75</v>
       </c>
       <c r="F179" t="n">
         <v>0</v>
@@ -4739,7 +4739,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4751,10 +4751,10 @@
         <v>46247</v>
       </c>
       <c r="D180" t="n">
-        <v>795345</v>
+        <v>47252</v>
       </c>
       <c r="E180" t="n">
-        <v>361.98</v>
+        <v>3157.51</v>
       </c>
       <c r="F180" t="n">
         <v>0</v>
@@ -4763,49 +4763,49 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C181" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D181" t="n">
-        <v>792141</v>
+        <v>795345</v>
       </c>
       <c r="E181" t="n">
-        <v>11095.24</v>
+        <v>439.18</v>
       </c>
       <c r="F181" t="n">
-        <v>321.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C182" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D182" t="n">
-        <v>793718</v>
+        <v>792141</v>
       </c>
       <c r="E182" t="n">
-        <v>145.46</v>
+        <v>11095.24</v>
       </c>
       <c r="F182" t="n">
-        <v>0</v>
+        <v>321.34</v>
       </c>
     </row>
     <row r="183">
@@ -4816,17 +4816,17 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C183" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D183" t="n">
-        <v>792121</v>
+        <v>793718</v>
       </c>
       <c r="E183" t="n">
-        <v>301.76</v>
+        <v>145.46</v>
       </c>
       <c r="F183" t="n">
         <v>0</v>
@@ -4840,17 +4840,17 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C184" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D184" t="n">
-        <v>794671</v>
+        <v>792121</v>
       </c>
       <c r="E184" t="n">
-        <v>32.7</v>
+        <v>301.76</v>
       </c>
       <c r="F184" t="n">
         <v>0</v>
@@ -4859,25 +4859,25 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C185" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D185" t="n">
-        <v>31267</v>
+        <v>794671</v>
       </c>
       <c r="E185" t="n">
-        <v>18051.22</v>
+        <v>32.7</v>
       </c>
       <c r="F185" t="n">
-        <v>390.95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="186">
@@ -4895,13 +4895,13 @@
         <v>46247</v>
       </c>
       <c r="D186" t="n">
-        <v>789525</v>
+        <v>31267</v>
       </c>
       <c r="E186" t="n">
-        <v>5257.43</v>
+        <v>18051.22</v>
       </c>
       <c r="F186" t="n">
-        <v>836.2</v>
+        <v>390.95</v>
       </c>
     </row>
     <row r="187">
@@ -4919,37 +4919,37 @@
         <v>46247</v>
       </c>
       <c r="D187" t="n">
-        <v>789228</v>
+        <v>789525</v>
       </c>
       <c r="E187" t="n">
-        <v>219.66</v>
+        <v>5257.43</v>
       </c>
       <c r="F187" t="n">
-        <v>33.67</v>
+        <v>836.2</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C188" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D188" t="n">
-        <v>793186</v>
+        <v>789228</v>
       </c>
       <c r="E188" t="n">
-        <v>13.91</v>
+        <v>219.66</v>
       </c>
       <c r="F188" t="n">
-        <v>13.91</v>
+        <v>33.67</v>
       </c>
     </row>
     <row r="189">
@@ -4967,19 +4967,19 @@
         <v>46247</v>
       </c>
       <c r="D189" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="E189" t="n">
-        <v>5.57</v>
+        <v>13.91</v>
       </c>
       <c r="F189" t="n">
-        <v>5.57</v>
+        <v>13.91</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -4991,34 +4991,34 @@
         <v>46247</v>
       </c>
       <c r="D190" t="n">
-        <v>31267</v>
+        <v>47252</v>
       </c>
       <c r="E190" t="n">
-        <v>14.99</v>
+        <v>5.57</v>
       </c>
       <c r="F190" t="n">
-        <v>0</v>
+        <v>5.57</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C191" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D191" t="n">
-        <v>30791</v>
+        <v>31267</v>
       </c>
       <c r="E191" t="n">
-        <v>1864.57</v>
+        <v>14.99</v>
       </c>
       <c r="F191" t="n">
         <v>0</v>
@@ -5027,12 +5027,12 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C192" s="2" t="n">
@@ -5042,10 +5042,10 @@
         <v>30791</v>
       </c>
       <c r="E192" t="n">
-        <v>18265.11</v>
+        <v>1864.57</v>
       </c>
       <c r="F192" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
     </row>
     <row r="193">
@@ -5063,13 +5063,13 @@
         <v>46247</v>
       </c>
       <c r="D193" t="n">
-        <v>789603</v>
+        <v>30791</v>
       </c>
       <c r="E193" t="n">
-        <v>32530.41</v>
+        <v>18398.64</v>
       </c>
       <c r="F193" t="n">
-        <v>372.82</v>
+        <v>72.64</v>
       </c>
     </row>
     <row r="194">
@@ -5087,13 +5087,13 @@
         <v>46247</v>
       </c>
       <c r="D194" t="n">
-        <v>30307</v>
+        <v>789603</v>
       </c>
       <c r="E194" t="n">
-        <v>343.86</v>
+        <v>32530.41</v>
       </c>
       <c r="F194" t="n">
-        <v>0</v>
+        <v>400.32</v>
       </c>
     </row>
     <row r="195">
@@ -5111,10 +5111,10 @@
         <v>46247</v>
       </c>
       <c r="D195" t="n">
-        <v>792141</v>
+        <v>30307</v>
       </c>
       <c r="E195" t="n">
-        <v>16683.38</v>
+        <v>343.86</v>
       </c>
       <c r="F195" t="n">
         <v>0</v>
@@ -5123,22 +5123,22 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C196" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D196" t="n">
-        <v>794671</v>
+        <v>792141</v>
       </c>
       <c r="E196" t="n">
-        <v>4114.68</v>
+        <v>16045.21</v>
       </c>
       <c r="F196" t="n">
         <v>0</v>
@@ -5152,17 +5152,17 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C197" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D197" t="n">
-        <v>795345</v>
+        <v>794029</v>
       </c>
       <c r="E197" t="n">
-        <v>4191.73</v>
+        <v>89.33</v>
       </c>
       <c r="F197" t="n">
         <v>0</v>
@@ -5176,17 +5176,17 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C198" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D198" t="n">
-        <v>794029</v>
+        <v>794671</v>
       </c>
       <c r="E198" t="n">
-        <v>31.16</v>
+        <v>4114.68</v>
       </c>
       <c r="F198" t="n">
         <v>0</v>
@@ -5195,22 +5195,22 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C199" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D199" t="n">
-        <v>33928</v>
+        <v>795345</v>
       </c>
       <c r="E199" t="n">
-        <v>46.44</v>
+        <v>4191.73</v>
       </c>
       <c r="F199" t="n">
         <v>0</v>
@@ -5219,22 +5219,22 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C200" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D200" t="n">
-        <v>30083</v>
+        <v>33928</v>
       </c>
       <c r="E200" t="n">
-        <v>16.38</v>
+        <v>46.44</v>
       </c>
       <c r="F200" t="n">
         <v>0</v>
@@ -5243,22 +5243,22 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C201" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D201" t="n">
-        <v>32816</v>
+        <v>30083</v>
       </c>
       <c r="E201" t="n">
-        <v>456.96</v>
+        <v>16.38</v>
       </c>
       <c r="F201" t="n">
         <v>0</v>
@@ -5267,22 +5267,22 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C202" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D202" t="n">
-        <v>31267</v>
+        <v>32816</v>
       </c>
       <c r="E202" t="n">
-        <v>914.84</v>
+        <v>456.96</v>
       </c>
       <c r="F202" t="n">
         <v>0</v>
@@ -5291,22 +5291,22 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C203" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D203" t="n">
-        <v>790595</v>
+        <v>31267</v>
       </c>
       <c r="E203" t="n">
-        <v>267.36</v>
+        <v>914.84</v>
       </c>
       <c r="F203" t="n">
         <v>0</v>
@@ -5327,10 +5327,10 @@
         <v>46247</v>
       </c>
       <c r="D204" t="n">
-        <v>30218</v>
+        <v>790595</v>
       </c>
       <c r="E204" t="n">
-        <v>2443.81</v>
+        <v>267.36</v>
       </c>
       <c r="F204" t="n">
         <v>0</v>
@@ -5339,22 +5339,22 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C205" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D205" t="n">
-        <v>47252</v>
+        <v>30218</v>
       </c>
       <c r="E205" t="n">
-        <v>21308.05</v>
+        <v>2443.81</v>
       </c>
       <c r="F205" t="n">
         <v>0</v>
@@ -5375,10 +5375,10 @@
         <v>46247</v>
       </c>
       <c r="D206" t="n">
-        <v>794671</v>
+        <v>47252</v>
       </c>
       <c r="E206" t="n">
-        <v>276.11</v>
+        <v>21648.96</v>
       </c>
       <c r="F206" t="n">
         <v>0</v>
@@ -5387,22 +5387,22 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C207" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D207" t="n">
-        <v>789603</v>
+        <v>794671</v>
       </c>
       <c r="E207" t="n">
-        <v>12435.93</v>
+        <v>276.11</v>
       </c>
       <c r="F207" t="n">
         <v>0</v>
@@ -5416,17 +5416,17 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C208" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D208" t="n">
-        <v>793186</v>
+        <v>789603</v>
       </c>
       <c r="E208" t="n">
-        <v>9913.65</v>
+        <v>12435.93</v>
       </c>
       <c r="F208" t="n">
         <v>0</v>
@@ -5435,12 +5435,12 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C209" s="2" t="n">
@@ -5450,7 +5450,7 @@
         <v>139553</v>
       </c>
       <c r="E209" t="n">
-        <v>8304.940000000001</v>
+        <v>406.68</v>
       </c>
       <c r="F209" t="n">
         <v>0</v>
@@ -5464,17 +5464,17 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C210" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D210" t="n">
-        <v>792246</v>
+        <v>793186</v>
       </c>
       <c r="E210" t="n">
-        <v>587.38</v>
+        <v>12043.25</v>
       </c>
       <c r="F210" t="n">
         <v>0</v>
@@ -5483,12 +5483,12 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C211" s="2" t="n">
@@ -5498,7 +5498,7 @@
         <v>139553</v>
       </c>
       <c r="E211" t="n">
-        <v>209.16</v>
+        <v>8304.940000000001</v>
       </c>
       <c r="F211" t="n">
         <v>0</v>
@@ -5507,22 +5507,22 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C212" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D212" t="n">
-        <v>30083</v>
+        <v>792246</v>
       </c>
       <c r="E212" t="n">
-        <v>627.34</v>
+        <v>587.38</v>
       </c>
       <c r="F212" t="n">
         <v>0</v>
@@ -5536,17 +5536,17 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C213" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D213" t="n">
-        <v>795345</v>
+        <v>30083</v>
       </c>
       <c r="E213" t="n">
-        <v>329.64</v>
+        <v>627.34</v>
       </c>
       <c r="F213" t="n">
         <v>0</v>
@@ -5560,17 +5560,17 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C214" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D214" t="n">
-        <v>30307</v>
+        <v>795345</v>
       </c>
       <c r="E214" t="n">
-        <v>89366.47</v>
+        <v>329.64</v>
       </c>
       <c r="F214" t="n">
         <v>0</v>
@@ -5591,10 +5591,10 @@
         <v>46247</v>
       </c>
       <c r="D215" t="n">
-        <v>30083</v>
+        <v>30307</v>
       </c>
       <c r="E215" t="n">
-        <v>5520.3</v>
+        <v>92958.47</v>
       </c>
       <c r="F215" t="n">
         <v>0</v>
@@ -5603,25 +5603,25 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C216" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D216" t="n">
-        <v>793718</v>
+        <v>30083</v>
       </c>
       <c r="E216" t="n">
-        <v>32005.64</v>
+        <v>5716.11</v>
       </c>
       <c r="F216" t="n">
-        <v>80.59999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="217">
@@ -5639,43 +5639,43 @@
         <v>46247</v>
       </c>
       <c r="D217" t="n">
-        <v>789661</v>
+        <v>793718</v>
       </c>
       <c r="E217" t="n">
-        <v>12.35</v>
+        <v>32077.16</v>
       </c>
       <c r="F217" t="n">
-        <v>32.2</v>
+        <v>80.59999999999999</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C218" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D218" t="n">
-        <v>33286</v>
+        <v>789661</v>
       </c>
       <c r="E218" t="n">
-        <v>3.99</v>
+        <v>12.35</v>
       </c>
       <c r="F218" t="n">
-        <v>3.99</v>
+        <v>32.2</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5687,19 +5687,19 @@
         <v>46247</v>
       </c>
       <c r="D219" t="n">
-        <v>794671</v>
+        <v>33286</v>
       </c>
       <c r="E219" t="n">
-        <v>759.41</v>
+        <v>3.99</v>
       </c>
       <c r="F219" t="n">
-        <v>0</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5711,10 +5711,10 @@
         <v>46247</v>
       </c>
       <c r="D220" t="n">
-        <v>792121</v>
+        <v>794671</v>
       </c>
       <c r="E220" t="n">
-        <v>47.14</v>
+        <v>759.41</v>
       </c>
       <c r="F220" t="n">
         <v>0</v>
@@ -5735,10 +5735,10 @@
         <v>46247</v>
       </c>
       <c r="D221" t="n">
-        <v>139553</v>
+        <v>792121</v>
       </c>
       <c r="E221" t="n">
-        <v>1300.72</v>
+        <v>47.14</v>
       </c>
       <c r="F221" t="n">
         <v>0</v>
@@ -5759,10 +5759,10 @@
         <v>46247</v>
       </c>
       <c r="D222" t="n">
-        <v>794671</v>
+        <v>139553</v>
       </c>
       <c r="E222" t="n">
-        <v>182.88</v>
+        <v>1300.72</v>
       </c>
       <c r="F222" t="n">
         <v>0</v>
@@ -5771,22 +5771,22 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C223" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D223" t="n">
-        <v>789525</v>
+        <v>794671</v>
       </c>
       <c r="E223" t="n">
-        <v>971.33</v>
+        <v>182.88</v>
       </c>
       <c r="F223" t="n">
         <v>0</v>
@@ -5807,10 +5807,10 @@
         <v>46247</v>
       </c>
       <c r="D224" t="n">
-        <v>33928</v>
+        <v>789525</v>
       </c>
       <c r="E224" t="n">
-        <v>1038.51</v>
+        <v>971.33</v>
       </c>
       <c r="F224" t="n">
         <v>0</v>
@@ -5831,10 +5831,10 @@
         <v>46247</v>
       </c>
       <c r="D225" t="n">
-        <v>33057</v>
+        <v>33928</v>
       </c>
       <c r="E225" t="n">
-        <v>89.06</v>
+        <v>1038.51</v>
       </c>
       <c r="F225" t="n">
         <v>0</v>
@@ -5843,25 +5843,25 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C226" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D226" t="n">
-        <v>789525</v>
+        <v>33057</v>
       </c>
       <c r="E226" t="n">
-        <v>6252.76</v>
+        <v>89.06</v>
       </c>
       <c r="F226" t="n">
-        <v>258.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="227">
@@ -5879,34 +5879,34 @@
         <v>46247</v>
       </c>
       <c r="D227" t="n">
-        <v>33057</v>
+        <v>789525</v>
       </c>
       <c r="E227" t="n">
-        <v>4693.52</v>
+        <v>6287.93</v>
       </c>
       <c r="F227" t="n">
-        <v>0</v>
+        <v>258.75</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C228" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D228" t="n">
-        <v>794671</v>
+        <v>33057</v>
       </c>
       <c r="E228" t="n">
-        <v>3481.16</v>
+        <v>4693.52</v>
       </c>
       <c r="F228" t="n">
         <v>0</v>
@@ -5915,22 +5915,22 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C229" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D229" t="n">
-        <v>30791</v>
+        <v>794671</v>
       </c>
       <c r="E229" t="n">
-        <v>6651.19</v>
+        <v>3481.16</v>
       </c>
       <c r="F229" t="n">
         <v>0</v>
@@ -5951,10 +5951,10 @@
         <v>46247</v>
       </c>
       <c r="D230" t="n">
-        <v>47252</v>
+        <v>30791</v>
       </c>
       <c r="E230" t="n">
-        <v>21741.29</v>
+        <v>6705.18</v>
       </c>
       <c r="F230" t="n">
         <v>0</v>
@@ -5975,10 +5975,10 @@
         <v>46247</v>
       </c>
       <c r="D231" t="n">
-        <v>789525</v>
+        <v>47252</v>
       </c>
       <c r="E231" t="n">
-        <v>1451.86</v>
+        <v>22580.65</v>
       </c>
       <c r="F231" t="n">
         <v>0</v>
@@ -5992,17 +5992,17 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C232" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D232" t="n">
-        <v>30307</v>
+        <v>789525</v>
       </c>
       <c r="E232" t="n">
-        <v>575.88</v>
+        <v>1451.86</v>
       </c>
       <c r="F232" t="n">
         <v>0</v>
@@ -6023,10 +6023,10 @@
         <v>46247</v>
       </c>
       <c r="D233" t="n">
-        <v>30791</v>
+        <v>30307</v>
       </c>
       <c r="E233" t="n">
-        <v>44.88</v>
+        <v>575.88</v>
       </c>
       <c r="F233" t="n">
         <v>0</v>
@@ -6035,22 +6035,22 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="C234" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D234" t="n">
-        <v>790595</v>
+        <v>30791</v>
       </c>
       <c r="E234" t="n">
-        <v>1151.94</v>
+        <v>44.88</v>
       </c>
       <c r="F234" t="n">
         <v>0</v>
@@ -6059,22 +6059,22 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C235" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D235" t="n">
-        <v>47252</v>
+        <v>790595</v>
       </c>
       <c r="E235" t="n">
-        <v>27375.67</v>
+        <v>1151.94</v>
       </c>
       <c r="F235" t="n">
         <v>0</v>
@@ -6083,22 +6083,22 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C236" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D236" t="n">
-        <v>794029</v>
+        <v>47252</v>
       </c>
       <c r="E236" t="n">
-        <v>4267.52</v>
+        <v>27399.78</v>
       </c>
       <c r="F236" t="n">
         <v>0</v>
@@ -6107,25 +6107,25 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C237" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D237" t="n">
-        <v>789603</v>
+        <v>795345</v>
       </c>
       <c r="E237" t="n">
-        <v>66932.96000000001</v>
+        <v>4352.64</v>
       </c>
       <c r="F237" t="n">
-        <v>41155.22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="238">
@@ -6136,17 +6136,17 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C238" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D238" t="n">
-        <v>795345</v>
+        <v>794029</v>
       </c>
       <c r="E238" t="n">
-        <v>1381.74</v>
+        <v>4267.52</v>
       </c>
       <c r="F238" t="n">
         <v>0</v>
@@ -6155,73 +6155,73 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C239" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D239" t="n">
-        <v>31267</v>
+        <v>789603</v>
       </c>
       <c r="E239" t="n">
-        <v>26.27</v>
+        <v>66932.96000000001</v>
       </c>
       <c r="F239" t="n">
-        <v>0</v>
+        <v>41155.22</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C240" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D240" t="n">
-        <v>793186</v>
+        <v>31267</v>
       </c>
       <c r="E240" t="n">
-        <v>443.79</v>
+        <v>26.27</v>
       </c>
       <c r="F240" t="n">
-        <v>54.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C241" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D241" t="n">
-        <v>30307</v>
+        <v>793186</v>
       </c>
       <c r="E241" t="n">
-        <v>9216.58</v>
+        <v>443.79</v>
       </c>
       <c r="F241" t="n">
-        <v>0</v>
+        <v>54.71</v>
       </c>
     </row>
     <row r="242">
@@ -6239,10 +6239,10 @@
         <v>46247</v>
       </c>
       <c r="D242" t="n">
-        <v>794671</v>
+        <v>30307</v>
       </c>
       <c r="E242" t="n">
-        <v>1670.06</v>
+        <v>9372.809999999999</v>
       </c>
       <c r="F242" t="n">
         <v>0</v>
@@ -6251,22 +6251,22 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C243" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D243" t="n">
-        <v>790595</v>
+        <v>794671</v>
       </c>
       <c r="E243" t="n">
-        <v>1177.54</v>
+        <v>1670.06</v>
       </c>
       <c r="F243" t="n">
         <v>0</v>
@@ -6280,17 +6280,17 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C244" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D244" t="n">
-        <v>792141</v>
+        <v>790595</v>
       </c>
       <c r="E244" t="n">
-        <v>2529.9</v>
+        <v>1177.54</v>
       </c>
       <c r="F244" t="n">
         <v>0</v>
@@ -6299,22 +6299,22 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C245" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D245" t="n">
-        <v>793186</v>
+        <v>792141</v>
       </c>
       <c r="E245" t="n">
-        <v>146.11</v>
+        <v>2529.9</v>
       </c>
       <c r="F245" t="n">
         <v>0</v>
@@ -6323,22 +6323,22 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C246" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D246" t="n">
-        <v>30083</v>
+        <v>793186</v>
       </c>
       <c r="E246" t="n">
-        <v>3299.7</v>
+        <v>146.11</v>
       </c>
       <c r="F246" t="n">
         <v>0</v>
@@ -6347,22 +6347,22 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C247" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D247" t="n">
-        <v>789603</v>
+        <v>792121</v>
       </c>
       <c r="E247" t="n">
-        <v>4572.27</v>
+        <v>1936.84</v>
       </c>
       <c r="F247" t="n">
         <v>0</v>
@@ -6371,22 +6371,22 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C248" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D248" t="n">
-        <v>33057</v>
+        <v>30083</v>
       </c>
       <c r="E248" t="n">
-        <v>12277.63</v>
+        <v>3299.7</v>
       </c>
       <c r="F248" t="n">
         <v>0</v>
@@ -6395,22 +6395,22 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C249" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D249" t="n">
-        <v>33928</v>
+        <v>789603</v>
       </c>
       <c r="E249" t="n">
-        <v>1912.82</v>
+        <v>9428.620000000001</v>
       </c>
       <c r="F249" t="n">
         <v>0</v>
@@ -6419,22 +6419,22 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C250" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D250" t="n">
-        <v>792121</v>
+        <v>33057</v>
       </c>
       <c r="E250" t="n">
-        <v>1472.58</v>
+        <v>12085.79</v>
       </c>
       <c r="F250" t="n">
         <v>0</v>
@@ -6443,22 +6443,22 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C251" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D251" t="n">
-        <v>792121</v>
+        <v>33928</v>
       </c>
       <c r="E251" t="n">
-        <v>501.32</v>
+        <v>2009.33</v>
       </c>
       <c r="F251" t="n">
         <v>0</v>
@@ -6467,22 +6467,22 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C252" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D252" t="n">
-        <v>32816</v>
+        <v>792121</v>
       </c>
       <c r="E252" t="n">
-        <v>74.84999999999999</v>
+        <v>501.32</v>
       </c>
       <c r="F252" t="n">
         <v>0</v>
@@ -6491,22 +6491,22 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C253" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D253" t="n">
-        <v>139553</v>
+        <v>32816</v>
       </c>
       <c r="E253" t="n">
-        <v>2570.35</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="F253" t="n">
         <v>0</v>
@@ -6515,22 +6515,22 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C254" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D254" t="n">
-        <v>795345</v>
+        <v>139553</v>
       </c>
       <c r="E254" t="n">
-        <v>283.88</v>
+        <v>2570.35</v>
       </c>
       <c r="F254" t="n">
         <v>0</v>
@@ -6539,22 +6539,22 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C255" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D255" t="n">
-        <v>33286</v>
+        <v>795345</v>
       </c>
       <c r="E255" t="n">
-        <v>106.92</v>
+        <v>283.88</v>
       </c>
       <c r="F255" t="n">
         <v>0</v>
@@ -6568,17 +6568,17 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C256" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D256" t="n">
-        <v>139553</v>
+        <v>33286</v>
       </c>
       <c r="E256" t="n">
-        <v>611.88</v>
+        <v>106.92</v>
       </c>
       <c r="F256" t="n">
         <v>0</v>
@@ -6587,24 +6587,48 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D257" t="n">
+        <v>139553</v>
+      </c>
+      <c r="E257" t="n">
+        <v>611.88</v>
+      </c>
+      <c r="F257" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="B257" t="inlineStr">
+      <c r="B258" t="inlineStr">
         <is>
           <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
-      <c r="C257" s="2" t="n">
-        <v>46247</v>
-      </c>
-      <c r="D257" t="n">
+      <c r="C258" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D258" t="n">
         <v>795345</v>
       </c>
-      <c r="E257" t="n">
+      <c r="E258" t="n">
         <v>169.57</v>
       </c>
-      <c r="F257" t="n">
+      <c r="F258" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 14:15:04
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F263"/>
+  <dimension ref="A1:F265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,10 +506,10 @@
         <v>47252</v>
       </c>
       <c r="E3" t="n">
-        <v>21291.99</v>
+        <v>23141.62</v>
       </c>
       <c r="F3" t="n">
-        <v>3810.55</v>
+        <v>4337.7</v>
       </c>
     </row>
     <row r="4">
@@ -530,10 +530,10 @@
         <v>33928</v>
       </c>
       <c r="E4" t="n">
-        <v>32150.03</v>
+        <v>32195.44</v>
       </c>
       <c r="F4" t="n">
-        <v>18650.11</v>
+        <v>19037.34</v>
       </c>
     </row>
     <row r="5">
@@ -578,7 +578,7 @@
         <v>33928</v>
       </c>
       <c r="E6" t="n">
-        <v>8094.39</v>
+        <v>8221.49</v>
       </c>
       <c r="F6" t="n">
         <v>391.48</v>
@@ -602,7 +602,7 @@
         <v>30791</v>
       </c>
       <c r="E7" t="n">
-        <v>14561.12</v>
+        <v>14785.58</v>
       </c>
       <c r="F7" t="n">
         <v>3111.54</v>
@@ -626,7 +626,7 @@
         <v>789228</v>
       </c>
       <c r="E8" t="n">
-        <v>4007.92</v>
+        <v>4088.58</v>
       </c>
       <c r="F8" t="n">
         <v>178.87</v>
@@ -674,7 +674,7 @@
         <v>33928</v>
       </c>
       <c r="E10" t="n">
-        <v>7127.19</v>
+        <v>7221.15</v>
       </c>
       <c r="F10" t="n">
         <v>935.13</v>
@@ -698,7 +698,7 @@
         <v>789525</v>
       </c>
       <c r="E11" t="n">
-        <v>1686.94</v>
+        <v>1844.76</v>
       </c>
       <c r="F11" t="n">
         <v>98.76000000000001</v>
@@ -779,22 +779,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D15" t="n">
-        <v>31267</v>
+        <v>794671</v>
       </c>
       <c r="E15" t="n">
-        <v>1163.91</v>
+        <v>3661.47</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -808,17 +808,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D16" t="n">
-        <v>789228</v>
+        <v>31267</v>
       </c>
       <c r="E16" t="n">
-        <v>2061.9</v>
+        <v>1163.91</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -827,25 +827,25 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D17" t="n">
-        <v>795345</v>
+        <v>789228</v>
       </c>
       <c r="E17" t="n">
-        <v>1423.86</v>
+        <v>2061.91</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>17.47</v>
       </c>
     </row>
     <row r="18">
@@ -856,17 +856,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D18" t="n">
-        <v>792121</v>
+        <v>795345</v>
       </c>
       <c r="E18" t="n">
-        <v>19254.27</v>
+        <v>1423.86</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -887,10 +887,10 @@
         <v>46247</v>
       </c>
       <c r="D19" t="n">
-        <v>30083</v>
+        <v>792121</v>
       </c>
       <c r="E19" t="n">
-        <v>7301.38</v>
+        <v>19254.27</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -904,17 +904,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D20" t="n">
-        <v>794671</v>
+        <v>30083</v>
       </c>
       <c r="E20" t="n">
-        <v>1617.84</v>
+        <v>7301.38</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -1010,7 +1010,7 @@
         <v>30083</v>
       </c>
       <c r="E24" t="n">
-        <v>1593.58</v>
+        <v>1634.85</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -1106,7 +1106,7 @@
         <v>33057</v>
       </c>
       <c r="E28" t="n">
-        <v>772.0599999999999</v>
+        <v>1046.83</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -1202,7 +1202,7 @@
         <v>794671</v>
       </c>
       <c r="E32" t="n">
-        <v>11789.62</v>
+        <v>12589.57</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -1274,7 +1274,7 @@
         <v>33057</v>
       </c>
       <c r="E35" t="n">
-        <v>364.69</v>
+        <v>614.12</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
@@ -1466,7 +1466,7 @@
         <v>33057</v>
       </c>
       <c r="E43" t="n">
-        <v>2549.69</v>
+        <v>3916.64</v>
       </c>
       <c r="F43" t="n">
         <v>97.77</v>
@@ -1610,7 +1610,7 @@
         <v>47252</v>
       </c>
       <c r="E49" t="n">
-        <v>18384.3</v>
+        <v>20198.37</v>
       </c>
       <c r="F49" t="n">
         <v>0</v>
@@ -1634,7 +1634,7 @@
         <v>789228</v>
       </c>
       <c r="E50" t="n">
-        <v>2977.83</v>
+        <v>3213.46</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
@@ -1658,7 +1658,7 @@
         <v>30307</v>
       </c>
       <c r="E51" t="n">
-        <v>15446.48</v>
+        <v>16466.96</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
@@ -1682,10 +1682,10 @@
         <v>33928</v>
       </c>
       <c r="E52" t="n">
-        <v>2347.01</v>
+        <v>2347.03</v>
       </c>
       <c r="F52" t="n">
-        <v>0</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="53">
@@ -1706,7 +1706,7 @@
         <v>789525</v>
       </c>
       <c r="E53" t="n">
-        <v>760.11</v>
+        <v>1667.82</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
@@ -1730,7 +1730,7 @@
         <v>792121</v>
       </c>
       <c r="E54" t="n">
-        <v>7508.76</v>
+        <v>9108.209999999999</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
@@ -1802,7 +1802,7 @@
         <v>792121</v>
       </c>
       <c r="E57" t="n">
-        <v>3695.94</v>
+        <v>4297.3</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
@@ -1826,7 +1826,7 @@
         <v>789603</v>
       </c>
       <c r="E58" t="n">
-        <v>17706.92</v>
+        <v>17756.24</v>
       </c>
       <c r="F58" t="n">
         <v>0</v>
@@ -1850,7 +1850,7 @@
         <v>795345</v>
       </c>
       <c r="E59" t="n">
-        <v>547.71</v>
+        <v>582.7</v>
       </c>
       <c r="F59" t="n">
         <v>0</v>
@@ -1877,7 +1877,7 @@
         <v>17764.94</v>
       </c>
       <c r="F60" t="n">
-        <v>0</v>
+        <v>2004.16</v>
       </c>
     </row>
     <row r="61">
@@ -2234,7 +2234,7 @@
         <v>33286</v>
       </c>
       <c r="E75" t="n">
-        <v>1213.82</v>
+        <v>1318.89</v>
       </c>
       <c r="F75" t="n">
         <v>230.41</v>
@@ -2258,7 +2258,7 @@
         <v>33286</v>
       </c>
       <c r="E76" t="n">
-        <v>2820.65</v>
+        <v>2864.26</v>
       </c>
       <c r="F76" t="n">
         <v>327.9</v>
@@ -2330,10 +2330,10 @@
         <v>793718</v>
       </c>
       <c r="E79" t="n">
-        <v>1555.69</v>
+        <v>1556.8</v>
       </c>
       <c r="F79" t="n">
-        <v>0</v>
+        <v>1261.34</v>
       </c>
     </row>
     <row r="80">
@@ -2354,7 +2354,7 @@
         <v>31267</v>
       </c>
       <c r="E80" t="n">
-        <v>3631.64</v>
+        <v>4328.83</v>
       </c>
       <c r="F80" t="n">
         <v>0</v>
@@ -2378,7 +2378,7 @@
         <v>793718</v>
       </c>
       <c r="E81" t="n">
-        <v>7136.7</v>
+        <v>7199.96</v>
       </c>
       <c r="F81" t="n">
         <v>0</v>
@@ -2426,7 +2426,7 @@
         <v>33286</v>
       </c>
       <c r="E83" t="n">
-        <v>2165.03</v>
+        <v>2476.67</v>
       </c>
       <c r="F83" t="n">
         <v>0</v>
@@ -2714,7 +2714,7 @@
         <v>47252</v>
       </c>
       <c r="E95" t="n">
-        <v>16508.24</v>
+        <v>16628.12</v>
       </c>
       <c r="F95" t="n">
         <v>0</v>
@@ -2882,7 +2882,7 @@
         <v>30307</v>
       </c>
       <c r="E102" t="n">
-        <v>30986.26</v>
+        <v>33170.29</v>
       </c>
       <c r="F102" t="n">
         <v>0</v>
@@ -2891,55 +2891,55 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D103" t="n">
-        <v>789525</v>
+        <v>30083</v>
       </c>
       <c r="E103" t="n">
-        <v>2993.64</v>
+        <v>1849.8</v>
       </c>
       <c r="F103" t="n">
-        <v>288.23</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D104" t="n">
-        <v>30307</v>
+        <v>789525</v>
       </c>
       <c r="E104" t="n">
-        <v>1491.02</v>
+        <v>3224.54</v>
       </c>
       <c r="F104" t="n">
-        <v>0</v>
+        <v>288.23</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2951,37 +2951,37 @@
         <v>46247</v>
       </c>
       <c r="D105" t="n">
-        <v>789228</v>
+        <v>30307</v>
       </c>
       <c r="E105" t="n">
-        <v>392.15</v>
+        <v>1491.02</v>
       </c>
       <c r="F105" t="n">
-        <v>159.28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D106" t="n">
-        <v>795345</v>
+        <v>789228</v>
       </c>
       <c r="E106" t="n">
-        <v>40.89</v>
+        <v>392.15</v>
       </c>
       <c r="F106" t="n">
-        <v>0</v>
+        <v>159.28</v>
       </c>
     </row>
     <row r="107">
@@ -2992,17 +2992,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D107" t="n">
-        <v>792121</v>
+        <v>795345</v>
       </c>
       <c r="E107" t="n">
-        <v>5765.53</v>
+        <v>40.89</v>
       </c>
       <c r="F107" t="n">
         <v>0</v>
@@ -3011,22 +3011,22 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D108" t="n">
-        <v>30083</v>
+        <v>792121</v>
       </c>
       <c r="E108" t="n">
-        <v>137.67</v>
+        <v>5765.53</v>
       </c>
       <c r="F108" t="n">
         <v>0</v>
@@ -3047,58 +3047,58 @@
         <v>46247</v>
       </c>
       <c r="D109" t="n">
-        <v>33928</v>
+        <v>30083</v>
       </c>
       <c r="E109" t="n">
-        <v>12719.52</v>
+        <v>137.67</v>
       </c>
       <c r="F109" t="n">
-        <v>30.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D110" t="n">
-        <v>795345</v>
+        <v>33928</v>
       </c>
       <c r="E110" t="n">
-        <v>1928.91</v>
+        <v>13543.08</v>
       </c>
       <c r="F110" t="n">
-        <v>0</v>
+        <v>30.75</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D111" t="n">
-        <v>30791</v>
+        <v>795345</v>
       </c>
       <c r="E111" t="n">
-        <v>3482.43</v>
+        <v>1928.91</v>
       </c>
       <c r="F111" t="n">
         <v>0</v>
@@ -3119,34 +3119,34 @@
         <v>46247</v>
       </c>
       <c r="D112" t="n">
-        <v>33286</v>
+        <v>30791</v>
       </c>
       <c r="E112" t="n">
-        <v>4043.68</v>
+        <v>3482.44</v>
       </c>
       <c r="F112" t="n">
-        <v>0</v>
+        <v>33.47</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D113" t="n">
-        <v>30083</v>
+        <v>33286</v>
       </c>
       <c r="E113" t="n">
-        <v>1561.04</v>
+        <v>4043.68</v>
       </c>
       <c r="F113" t="n">
         <v>0</v>
@@ -3218,7 +3218,7 @@
         <v>789603</v>
       </c>
       <c r="E116" t="n">
-        <v>28785.58</v>
+        <v>29335.98</v>
       </c>
       <c r="F116" t="n">
         <v>0</v>
@@ -3266,7 +3266,7 @@
         <v>30307</v>
       </c>
       <c r="E118" t="n">
-        <v>44785.4</v>
+        <v>46374.66</v>
       </c>
       <c r="F118" t="n">
         <v>4936.24</v>
@@ -3410,7 +3410,7 @@
         <v>33286</v>
       </c>
       <c r="E124" t="n">
-        <v>1376.17</v>
+        <v>1405.95</v>
       </c>
       <c r="F124" t="n">
         <v>0</v>
@@ -3554,7 +3554,7 @@
         <v>33928</v>
       </c>
       <c r="E130" t="n">
-        <v>1111.35</v>
+        <v>1129.26</v>
       </c>
       <c r="F130" t="n">
         <v>0</v>
@@ -3659,25 +3659,25 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D135" t="n">
-        <v>47252</v>
+        <v>792121</v>
       </c>
       <c r="E135" t="n">
-        <v>19078.45</v>
+        <v>7510.83</v>
       </c>
       <c r="F135" t="n">
-        <v>1686.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
@@ -3698,10 +3698,10 @@
         <v>47252</v>
       </c>
       <c r="E136" t="n">
-        <v>26618.18</v>
+        <v>22535.35</v>
       </c>
       <c r="F136" t="n">
-        <v>4460.38</v>
+        <v>1686.2</v>
       </c>
     </row>
     <row r="137">
@@ -3712,20 +3712,20 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D137" t="n">
-        <v>795345</v>
+        <v>47252</v>
       </c>
       <c r="E137" t="n">
-        <v>27.25</v>
+        <v>28289.53</v>
       </c>
       <c r="F137" t="n">
-        <v>0</v>
+        <v>4632.36</v>
       </c>
     </row>
     <row r="138">
@@ -3736,17 +3736,17 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D138" t="n">
-        <v>793718</v>
+        <v>795345</v>
       </c>
       <c r="E138" t="n">
-        <v>39.84</v>
+        <v>27.25</v>
       </c>
       <c r="F138" t="n">
         <v>0</v>
@@ -3767,10 +3767,10 @@
         <v>46247</v>
       </c>
       <c r="D139" t="n">
-        <v>33057</v>
+        <v>793718</v>
       </c>
       <c r="E139" t="n">
-        <v>42.76</v>
+        <v>39.84</v>
       </c>
       <c r="F139" t="n">
         <v>0</v>
@@ -3791,10 +3791,10 @@
         <v>46247</v>
       </c>
       <c r="D140" t="n">
-        <v>30791</v>
+        <v>33057</v>
       </c>
       <c r="E140" t="n">
-        <v>33.08</v>
+        <v>42.76</v>
       </c>
       <c r="F140" t="n">
         <v>0</v>
@@ -3803,22 +3803,22 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D141" t="n">
-        <v>31267</v>
+        <v>30791</v>
       </c>
       <c r="E141" t="n">
-        <v>160.86</v>
+        <v>33.08</v>
       </c>
       <c r="F141" t="n">
         <v>0</v>
@@ -3827,25 +3827,25 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C142" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D142" t="n">
-        <v>139553</v>
+        <v>31267</v>
       </c>
       <c r="E142" t="n">
-        <v>1106.98</v>
+        <v>160.86</v>
       </c>
       <c r="F142" t="n">
-        <v>0</v>
+        <v>42.93</v>
       </c>
     </row>
     <row r="143">
@@ -3866,7 +3866,7 @@
         <v>33286</v>
       </c>
       <c r="E143" t="n">
-        <v>7688.18</v>
+        <v>8955.99</v>
       </c>
       <c r="F143" t="n">
         <v>0</v>
@@ -3875,22 +3875,22 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C144" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D144" t="n">
-        <v>30307</v>
+        <v>139553</v>
       </c>
       <c r="E144" t="n">
-        <v>507.68</v>
+        <v>1106.98</v>
       </c>
       <c r="F144" t="n">
         <v>0</v>
@@ -3904,116 +3904,116 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C145" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D145" t="n">
-        <v>33057</v>
+        <v>30791</v>
       </c>
       <c r="E145" t="n">
-        <v>146.56</v>
+        <v>0</v>
       </c>
       <c r="F145" t="n">
-        <v>0</v>
+        <v>646.85</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C146" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D146" t="n">
-        <v>789661</v>
+        <v>30307</v>
       </c>
       <c r="E146" t="n">
-        <v>37.05</v>
+        <v>507.68</v>
       </c>
       <c r="F146" t="n">
-        <v>258.83</v>
+        <v>0</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C147" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D147" t="n">
-        <v>793186</v>
+        <v>33057</v>
       </c>
       <c r="E147" t="n">
-        <v>637.28</v>
+        <v>146.56</v>
       </c>
       <c r="F147" t="n">
-        <v>97.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C148" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D148" t="n">
-        <v>794671</v>
+        <v>789661</v>
       </c>
       <c r="E148" t="n">
-        <v>1295.61</v>
+        <v>37.05</v>
       </c>
       <c r="F148" t="n">
-        <v>0</v>
+        <v>258.83</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C149" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D149" t="n">
-        <v>30083</v>
+        <v>793186</v>
       </c>
       <c r="E149" t="n">
-        <v>227.05</v>
+        <v>637.28</v>
       </c>
       <c r="F149" t="n">
-        <v>0</v>
+        <v>97.42</v>
       </c>
     </row>
     <row r="150">
@@ -4024,17 +4024,17 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C150" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D150" t="n">
-        <v>794029</v>
+        <v>794671</v>
       </c>
       <c r="E150" t="n">
-        <v>8574.25</v>
+        <v>1295.61</v>
       </c>
       <c r="F150" t="n">
         <v>0</v>
@@ -4043,22 +4043,22 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C151" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D151" t="n">
-        <v>31267</v>
+        <v>30083</v>
       </c>
       <c r="E151" t="n">
-        <v>63.33</v>
+        <v>227.05</v>
       </c>
       <c r="F151" t="n">
         <v>0</v>
@@ -4079,10 +4079,10 @@
         <v>46247</v>
       </c>
       <c r="D152" t="n">
-        <v>790595</v>
+        <v>794029</v>
       </c>
       <c r="E152" t="n">
-        <v>1479.08</v>
+        <v>8574.25</v>
       </c>
       <c r="F152" t="n">
         <v>0</v>
@@ -4091,22 +4091,22 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C153" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D153" t="n">
-        <v>792121</v>
+        <v>31267</v>
       </c>
       <c r="E153" t="n">
-        <v>4843.19</v>
+        <v>63.33</v>
       </c>
       <c r="F153" t="n">
         <v>0</v>
@@ -4115,22 +4115,22 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C154" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D154" t="n">
-        <v>47252</v>
+        <v>790595</v>
       </c>
       <c r="E154" t="n">
-        <v>291.52</v>
+        <v>1479.08</v>
       </c>
       <c r="F154" t="n">
         <v>0</v>
@@ -4139,22 +4139,22 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C155" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D155" t="n">
-        <v>31267</v>
+        <v>47252</v>
       </c>
       <c r="E155" t="n">
-        <v>149532.6</v>
+        <v>291.52</v>
       </c>
       <c r="F155" t="n">
         <v>0</v>
@@ -4163,22 +4163,22 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C156" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D156" t="n">
-        <v>794029</v>
+        <v>31267</v>
       </c>
       <c r="E156" t="n">
-        <v>7508.53</v>
+        <v>151452.21</v>
       </c>
       <c r="F156" t="n">
         <v>0</v>
@@ -4187,22 +4187,22 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C157" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D157" t="n">
-        <v>33928</v>
+        <v>794029</v>
       </c>
       <c r="E157" t="n">
-        <v>823.55</v>
+        <v>7623.07</v>
       </c>
       <c r="F157" t="n">
         <v>0</v>
@@ -4211,22 +4211,22 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C158" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D158" t="n">
-        <v>139553</v>
+        <v>33928</v>
       </c>
       <c r="E158" t="n">
-        <v>7003.92</v>
+        <v>823.55</v>
       </c>
       <c r="F158" t="n">
         <v>0</v>
@@ -4240,7 +4240,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C159" s="2" t="n">
@@ -4250,7 +4250,7 @@
         <v>139553</v>
       </c>
       <c r="E159" t="n">
-        <v>717.6</v>
+        <v>7003.92</v>
       </c>
       <c r="F159" t="n">
         <v>0</v>
@@ -4259,22 +4259,22 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C160" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D160" t="n">
-        <v>796582</v>
+        <v>139553</v>
       </c>
       <c r="E160" t="n">
-        <v>2647.34</v>
+        <v>717.6</v>
       </c>
       <c r="F160" t="n">
         <v>0</v>
@@ -4283,22 +4283,22 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C161" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D161" t="n">
-        <v>139553</v>
+        <v>796582</v>
       </c>
       <c r="E161" t="n">
-        <v>1621.76</v>
+        <v>2647.34</v>
       </c>
       <c r="F161" t="n">
         <v>0</v>
@@ -4307,22 +4307,22 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C162" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D162" t="n">
-        <v>795345</v>
+        <v>139553</v>
       </c>
       <c r="E162" t="n">
-        <v>204.29</v>
+        <v>1621.76</v>
       </c>
       <c r="F162" t="n">
         <v>0</v>
@@ -4331,22 +4331,22 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C163" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D163" t="n">
-        <v>790595</v>
+        <v>795345</v>
       </c>
       <c r="E163" t="n">
-        <v>117.44</v>
+        <v>204.29</v>
       </c>
       <c r="F163" t="n">
         <v>0</v>
@@ -4355,22 +4355,22 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C164" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D164" t="n">
-        <v>30083</v>
+        <v>790595</v>
       </c>
       <c r="E164" t="n">
-        <v>727.5700000000001</v>
+        <v>117.44</v>
       </c>
       <c r="F164" t="n">
         <v>0</v>
@@ -4391,10 +4391,10 @@
         <v>46247</v>
       </c>
       <c r="D165" t="n">
-        <v>792121</v>
+        <v>30083</v>
       </c>
       <c r="E165" t="n">
-        <v>1095.64</v>
+        <v>727.5700000000001</v>
       </c>
       <c r="F165" t="n">
         <v>0</v>
@@ -4415,10 +4415,10 @@
         <v>46247</v>
       </c>
       <c r="D166" t="n">
-        <v>30307</v>
+        <v>792121</v>
       </c>
       <c r="E166" t="n">
-        <v>6580.35</v>
+        <v>1095.64</v>
       </c>
       <c r="F166" t="n">
         <v>0</v>
@@ -4427,22 +4427,22 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C167" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D167" t="n">
-        <v>794671</v>
+        <v>30307</v>
       </c>
       <c r="E167" t="n">
-        <v>1810.54</v>
+        <v>6580.35</v>
       </c>
       <c r="F167" t="n">
         <v>0</v>
@@ -4451,22 +4451,22 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C168" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D168" t="n">
-        <v>32816</v>
+        <v>794671</v>
       </c>
       <c r="E168" t="n">
-        <v>1721.48</v>
+        <v>1810.54</v>
       </c>
       <c r="F168" t="n">
         <v>0</v>
@@ -4475,46 +4475,46 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C169" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D169" t="n">
-        <v>789603</v>
+        <v>32816</v>
       </c>
       <c r="E169" t="n">
-        <v>7108.74</v>
+        <v>1721.48</v>
       </c>
       <c r="F169" t="n">
-        <v>0</v>
+        <v>637.4400000000001</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C170" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D170" t="n">
-        <v>33057</v>
+        <v>795345</v>
       </c>
       <c r="E170" t="n">
-        <v>631.5700000000001</v>
+        <v>2169.18</v>
       </c>
       <c r="F170" t="n">
         <v>0</v>
@@ -4523,46 +4523,46 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C171" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D171" t="n">
-        <v>33057</v>
+        <v>789603</v>
       </c>
       <c r="E171" t="n">
-        <v>12.37</v>
+        <v>7108.74</v>
       </c>
       <c r="F171" t="n">
-        <v>12.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C172" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D172" t="n">
-        <v>47252</v>
+        <v>33057</v>
       </c>
       <c r="E172" t="n">
-        <v>12079.28</v>
+        <v>631.5700000000001</v>
       </c>
       <c r="F172" t="n">
         <v>0</v>
@@ -4576,65 +4576,65 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C173" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D173" t="n">
-        <v>793186</v>
+        <v>33057</v>
       </c>
       <c r="E173" t="n">
-        <v>403.84</v>
+        <v>12.37</v>
       </c>
       <c r="F173" t="n">
-        <v>0</v>
+        <v>12.37</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C174" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D174" t="n">
-        <v>792141</v>
+        <v>47252</v>
       </c>
       <c r="E174" t="n">
-        <v>1861.38</v>
+        <v>15920.56</v>
       </c>
       <c r="F174" t="n">
-        <v>791.11</v>
+        <v>236.4</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C175" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D175" t="n">
-        <v>793718</v>
+        <v>793186</v>
       </c>
       <c r="E175" t="n">
-        <v>3647.94</v>
+        <v>403.84</v>
       </c>
       <c r="F175" t="n">
         <v>0</v>
@@ -4643,46 +4643,46 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C176" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D176" t="n">
-        <v>789228</v>
+        <v>792141</v>
       </c>
       <c r="E176" t="n">
-        <v>1746.05</v>
+        <v>1911.44</v>
       </c>
       <c r="F176" t="n">
-        <v>0</v>
+        <v>791.11</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C177" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D177" t="n">
-        <v>795345</v>
+        <v>793718</v>
       </c>
       <c r="E177" t="n">
-        <v>1829.8</v>
+        <v>3647.94</v>
       </c>
       <c r="F177" t="n">
         <v>0</v>
@@ -4696,17 +4696,17 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C178" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D178" t="n">
-        <v>792141</v>
+        <v>789228</v>
       </c>
       <c r="E178" t="n">
-        <v>980.8</v>
+        <v>1746.05</v>
       </c>
       <c r="F178" t="n">
         <v>0</v>
@@ -4715,22 +4715,22 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C179" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D179" t="n">
-        <v>30307</v>
+        <v>792141</v>
       </c>
       <c r="E179" t="n">
-        <v>25047.44</v>
+        <v>980.8</v>
       </c>
       <c r="F179" t="n">
         <v>0</v>
@@ -4744,7 +4744,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C180" s="2" t="n">
@@ -4754,7 +4754,7 @@
         <v>30307</v>
       </c>
       <c r="E180" t="n">
-        <v>57878.05</v>
+        <v>25470.22</v>
       </c>
       <c r="F180" t="n">
         <v>0</v>
@@ -4763,22 +4763,22 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C181" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D181" t="n">
-        <v>789603</v>
+        <v>30307</v>
       </c>
       <c r="E181" t="n">
-        <v>1112.78</v>
+        <v>57878.05</v>
       </c>
       <c r="F181" t="n">
         <v>0</v>
@@ -4799,10 +4799,10 @@
         <v>46247</v>
       </c>
       <c r="D182" t="n">
-        <v>792141</v>
+        <v>789603</v>
       </c>
       <c r="E182" t="n">
-        <v>13.96</v>
+        <v>1112.78</v>
       </c>
       <c r="F182" t="n">
         <v>0</v>
@@ -4811,22 +4811,22 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C183" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D183" t="n">
-        <v>30307</v>
+        <v>792141</v>
       </c>
       <c r="E183" t="n">
-        <v>71014.39999999999</v>
+        <v>13.96</v>
       </c>
       <c r="F183" t="n">
         <v>0</v>
@@ -4835,22 +4835,22 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C184" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D184" t="n">
-        <v>32816</v>
+        <v>30307</v>
       </c>
       <c r="E184" t="n">
-        <v>75.75</v>
+        <v>74741.3</v>
       </c>
       <c r="F184" t="n">
         <v>0</v>
@@ -4864,17 +4864,17 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C185" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D185" t="n">
-        <v>47252</v>
+        <v>32816</v>
       </c>
       <c r="E185" t="n">
-        <v>3157.51</v>
+        <v>75.75</v>
       </c>
       <c r="F185" t="n">
         <v>0</v>
@@ -4883,7 +4883,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4895,61 +4895,61 @@
         <v>46247</v>
       </c>
       <c r="D186" t="n">
-        <v>795345</v>
+        <v>47252</v>
       </c>
       <c r="E186" t="n">
-        <v>439.18</v>
+        <v>3157.51</v>
       </c>
       <c r="F186" t="n">
-        <v>0</v>
+        <v>628.86</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C187" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D187" t="n">
-        <v>792141</v>
+        <v>795345</v>
       </c>
       <c r="E187" t="n">
-        <v>11095.24</v>
+        <v>439.18</v>
       </c>
       <c r="F187" t="n">
-        <v>321.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C188" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D188" t="n">
-        <v>793718</v>
+        <v>792141</v>
       </c>
       <c r="E188" t="n">
-        <v>156.84</v>
+        <v>11095.24</v>
       </c>
       <c r="F188" t="n">
-        <v>0</v>
+        <v>321.34</v>
       </c>
     </row>
     <row r="189">
@@ -4960,17 +4960,17 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C189" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D189" t="n">
-        <v>792121</v>
+        <v>793718</v>
       </c>
       <c r="E189" t="n">
-        <v>301.76</v>
+        <v>156.84</v>
       </c>
       <c r="F189" t="n">
         <v>0</v>
@@ -4984,17 +4984,17 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C190" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D190" t="n">
-        <v>794671</v>
+        <v>792121</v>
       </c>
       <c r="E190" t="n">
-        <v>32.7</v>
+        <v>301.76</v>
       </c>
       <c r="F190" t="n">
         <v>0</v>
@@ -5003,25 +5003,25 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C191" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D191" t="n">
-        <v>31267</v>
+        <v>794671</v>
       </c>
       <c r="E191" t="n">
-        <v>27199.64</v>
+        <v>32.7</v>
       </c>
       <c r="F191" t="n">
-        <v>390.95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="192">
@@ -5039,13 +5039,13 @@
         <v>46247</v>
       </c>
       <c r="D192" t="n">
-        <v>789525</v>
+        <v>31267</v>
       </c>
       <c r="E192" t="n">
-        <v>5257.43</v>
+        <v>27200.06</v>
       </c>
       <c r="F192" t="n">
-        <v>836.2</v>
+        <v>2242.99</v>
       </c>
     </row>
     <row r="193">
@@ -5063,37 +5063,37 @@
         <v>46247</v>
       </c>
       <c r="D193" t="n">
-        <v>789228</v>
+        <v>789525</v>
       </c>
       <c r="E193" t="n">
-        <v>241.92</v>
+        <v>5257.46</v>
       </c>
       <c r="F193" t="n">
-        <v>33.67</v>
+        <v>1019.16</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C194" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D194" t="n">
-        <v>793186</v>
+        <v>789228</v>
       </c>
       <c r="E194" t="n">
-        <v>13.91</v>
+        <v>241.92</v>
       </c>
       <c r="F194" t="n">
-        <v>13.91</v>
+        <v>33.67</v>
       </c>
     </row>
     <row r="195">
@@ -5111,19 +5111,19 @@
         <v>46247</v>
       </c>
       <c r="D195" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="E195" t="n">
-        <v>5.57</v>
+        <v>13.91</v>
       </c>
       <c r="F195" t="n">
-        <v>5.57</v>
+        <v>13.91</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5135,34 +5135,34 @@
         <v>46247</v>
       </c>
       <c r="D196" t="n">
-        <v>31267</v>
+        <v>47252</v>
       </c>
       <c r="E196" t="n">
-        <v>14.99</v>
+        <v>5.57</v>
       </c>
       <c r="F196" t="n">
-        <v>0</v>
+        <v>5.57</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C197" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D197" t="n">
-        <v>30791</v>
+        <v>31267</v>
       </c>
       <c r="E197" t="n">
-        <v>1864.57</v>
+        <v>14.99</v>
       </c>
       <c r="F197" t="n">
         <v>0</v>
@@ -5171,12 +5171,12 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C198" s="2" t="n">
@@ -5186,10 +5186,10 @@
         <v>30791</v>
       </c>
       <c r="E198" t="n">
-        <v>18398.64</v>
+        <v>1864.57</v>
       </c>
       <c r="F198" t="n">
-        <v>72.64</v>
+        <v>174.72</v>
       </c>
     </row>
     <row r="199">
@@ -5207,13 +5207,13 @@
         <v>46247</v>
       </c>
       <c r="D199" t="n">
-        <v>789603</v>
+        <v>30791</v>
       </c>
       <c r="E199" t="n">
-        <v>32530.41</v>
+        <v>18946.94</v>
       </c>
       <c r="F199" t="n">
-        <v>400.32</v>
+        <v>72.64</v>
       </c>
     </row>
     <row r="200">
@@ -5231,13 +5231,13 @@
         <v>46247</v>
       </c>
       <c r="D200" t="n">
-        <v>30307</v>
+        <v>789603</v>
       </c>
       <c r="E200" t="n">
-        <v>343.86</v>
+        <v>37483.89</v>
       </c>
       <c r="F200" t="n">
-        <v>0</v>
+        <v>400.32</v>
       </c>
     </row>
     <row r="201">
@@ -5255,10 +5255,10 @@
         <v>46247</v>
       </c>
       <c r="D201" t="n">
-        <v>792141</v>
+        <v>30307</v>
       </c>
       <c r="E201" t="n">
-        <v>15278.16</v>
+        <v>343.86</v>
       </c>
       <c r="F201" t="n">
         <v>0</v>
@@ -5267,22 +5267,22 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C202" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D202" t="n">
-        <v>794029</v>
+        <v>792141</v>
       </c>
       <c r="E202" t="n">
-        <v>89.33</v>
+        <v>14572.93</v>
       </c>
       <c r="F202" t="n">
         <v>0</v>
@@ -5296,17 +5296,17 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C203" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D203" t="n">
-        <v>794671</v>
+        <v>794029</v>
       </c>
       <c r="E203" t="n">
-        <v>4114.68</v>
+        <v>89.33</v>
       </c>
       <c r="F203" t="n">
         <v>0</v>
@@ -5327,10 +5327,10 @@
         <v>46247</v>
       </c>
       <c r="D204" t="n">
-        <v>795345</v>
+        <v>794671</v>
       </c>
       <c r="E204" t="n">
-        <v>4191.73</v>
+        <v>4114.68</v>
       </c>
       <c r="F204" t="n">
         <v>0</v>
@@ -5339,22 +5339,22 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C205" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D205" t="n">
-        <v>33928</v>
+        <v>795345</v>
       </c>
       <c r="E205" t="n">
-        <v>46.44</v>
+        <v>4191.73</v>
       </c>
       <c r="F205" t="n">
         <v>0</v>
@@ -5363,22 +5363,22 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C206" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D206" t="n">
-        <v>30083</v>
+        <v>33928</v>
       </c>
       <c r="E206" t="n">
-        <v>16.38</v>
+        <v>46.44</v>
       </c>
       <c r="F206" t="n">
         <v>0</v>
@@ -5387,22 +5387,22 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C207" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D207" t="n">
-        <v>32816</v>
+        <v>30083</v>
       </c>
       <c r="E207" t="n">
-        <v>456.96</v>
+        <v>16.38</v>
       </c>
       <c r="F207" t="n">
         <v>0</v>
@@ -5411,22 +5411,22 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C208" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D208" t="n">
-        <v>31267</v>
+        <v>32816</v>
       </c>
       <c r="E208" t="n">
-        <v>914.84</v>
+        <v>456.96</v>
       </c>
       <c r="F208" t="n">
         <v>0</v>
@@ -5435,22 +5435,22 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C209" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D209" t="n">
-        <v>790595</v>
+        <v>31267</v>
       </c>
       <c r="E209" t="n">
-        <v>267.36</v>
+        <v>914.84</v>
       </c>
       <c r="F209" t="n">
         <v>0</v>
@@ -5471,10 +5471,10 @@
         <v>46247</v>
       </c>
       <c r="D210" t="n">
-        <v>30218</v>
+        <v>790595</v>
       </c>
       <c r="E210" t="n">
-        <v>2443.81</v>
+        <v>267.36</v>
       </c>
       <c r="F210" t="n">
         <v>0</v>
@@ -5483,22 +5483,22 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C211" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D211" t="n">
-        <v>47252</v>
+        <v>30218</v>
       </c>
       <c r="E211" t="n">
-        <v>22315.79</v>
+        <v>2443.81</v>
       </c>
       <c r="F211" t="n">
         <v>0</v>
@@ -5519,10 +5519,10 @@
         <v>46247</v>
       </c>
       <c r="D212" t="n">
-        <v>794671</v>
+        <v>47252</v>
       </c>
       <c r="E212" t="n">
-        <v>276.11</v>
+        <v>24264.62</v>
       </c>
       <c r="F212" t="n">
         <v>0</v>
@@ -5531,22 +5531,22 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C213" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D213" t="n">
-        <v>789603</v>
+        <v>794671</v>
       </c>
       <c r="E213" t="n">
-        <v>12435.93</v>
+        <v>276.11</v>
       </c>
       <c r="F213" t="n">
         <v>0</v>
@@ -5555,22 +5555,22 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C214" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D214" t="n">
-        <v>139553</v>
+        <v>789603</v>
       </c>
       <c r="E214" t="n">
-        <v>406.68</v>
+        <v>12435.93</v>
       </c>
       <c r="F214" t="n">
         <v>0</v>
@@ -5579,22 +5579,22 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C215" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D215" t="n">
-        <v>793186</v>
+        <v>139553</v>
       </c>
       <c r="E215" t="n">
-        <v>12043.25</v>
+        <v>406.68</v>
       </c>
       <c r="F215" t="n">
         <v>0</v>
@@ -5603,22 +5603,22 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C216" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D216" t="n">
-        <v>139553</v>
+        <v>793186</v>
       </c>
       <c r="E216" t="n">
-        <v>8304.940000000001</v>
+        <v>15013.93</v>
       </c>
       <c r="F216" t="n">
         <v>0</v>
@@ -5627,46 +5627,46 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C217" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D217" t="n">
-        <v>792246</v>
+        <v>139553</v>
       </c>
       <c r="E217" t="n">
-        <v>587.38</v>
+        <v>8304.940000000001</v>
       </c>
       <c r="F217" t="n">
-        <v>0</v>
+        <v>281.52</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C218" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D218" t="n">
-        <v>30083</v>
+        <v>792246</v>
       </c>
       <c r="E218" t="n">
-        <v>627.34</v>
+        <v>587.38</v>
       </c>
       <c r="F218" t="n">
         <v>0</v>
@@ -5680,17 +5680,17 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C219" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D219" t="n">
-        <v>795345</v>
+        <v>789603</v>
       </c>
       <c r="E219" t="n">
-        <v>329.64</v>
+        <v>4287.44</v>
       </c>
       <c r="F219" t="n">
         <v>0</v>
@@ -5704,17 +5704,17 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C220" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D220" t="n">
-        <v>30307</v>
+        <v>30083</v>
       </c>
       <c r="E220" t="n">
-        <v>92958.47</v>
+        <v>627.34</v>
       </c>
       <c r="F220" t="n">
         <v>0</v>
@@ -5728,17 +5728,17 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C221" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D221" t="n">
-        <v>30083</v>
+        <v>795345</v>
       </c>
       <c r="E221" t="n">
-        <v>5716.11</v>
+        <v>329.64</v>
       </c>
       <c r="F221" t="n">
         <v>0</v>
@@ -5747,127 +5747,127 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C222" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D222" t="n">
-        <v>793718</v>
+        <v>794029</v>
       </c>
       <c r="E222" t="n">
-        <v>31958.48</v>
+        <v>5023.73</v>
       </c>
       <c r="F222" t="n">
-        <v>80.59999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C223" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D223" t="n">
-        <v>789661</v>
+        <v>30307</v>
       </c>
       <c r="E223" t="n">
-        <v>12.35</v>
+        <v>108224.47</v>
       </c>
       <c r="F223" t="n">
-        <v>32.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C224" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D224" t="n">
-        <v>33286</v>
+        <v>30083</v>
       </c>
       <c r="E224" t="n">
-        <v>3.99</v>
+        <v>5716.11</v>
       </c>
       <c r="F224" t="n">
-        <v>3.99</v>
+        <v>0</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C225" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D225" t="n">
-        <v>794671</v>
+        <v>793718</v>
       </c>
       <c r="E225" t="n">
-        <v>759.41</v>
+        <v>31959.13</v>
       </c>
       <c r="F225" t="n">
-        <v>0</v>
+        <v>1167.12</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C226" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D226" t="n">
-        <v>792121</v>
+        <v>789661</v>
       </c>
       <c r="E226" t="n">
-        <v>47.14</v>
+        <v>12.35</v>
       </c>
       <c r="F226" t="n">
-        <v>0</v>
+        <v>32.2</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -5879,19 +5879,19 @@
         <v>46247</v>
       </c>
       <c r="D227" t="n">
-        <v>139553</v>
+        <v>33286</v>
       </c>
       <c r="E227" t="n">
-        <v>1300.72</v>
+        <v>3.99</v>
       </c>
       <c r="F227" t="n">
-        <v>0</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -5906,7 +5906,7 @@
         <v>794671</v>
       </c>
       <c r="E228" t="n">
-        <v>182.88</v>
+        <v>759.41</v>
       </c>
       <c r="F228" t="n">
         <v>0</v>
@@ -5915,22 +5915,22 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C229" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D229" t="n">
-        <v>789525</v>
+        <v>792121</v>
       </c>
       <c r="E229" t="n">
-        <v>971.33</v>
+        <v>47.14</v>
       </c>
       <c r="F229" t="n">
         <v>0</v>
@@ -5939,22 +5939,22 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C230" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D230" t="n">
-        <v>33928</v>
+        <v>139553</v>
       </c>
       <c r="E230" t="n">
-        <v>1038.51</v>
+        <v>1300.72</v>
       </c>
       <c r="F230" t="n">
         <v>0</v>
@@ -5963,22 +5963,22 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C231" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D231" t="n">
-        <v>33057</v>
+        <v>794671</v>
       </c>
       <c r="E231" t="n">
-        <v>89.06</v>
+        <v>1075.68</v>
       </c>
       <c r="F231" t="n">
         <v>0</v>
@@ -5987,70 +5987,70 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C232" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D232" t="n">
-        <v>789525</v>
+        <v>33928</v>
       </c>
       <c r="E232" t="n">
-        <v>6287.93</v>
+        <v>1038.51</v>
       </c>
       <c r="F232" t="n">
-        <v>258.75</v>
+        <v>41.55</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C233" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D233" t="n">
-        <v>33057</v>
+        <v>789525</v>
       </c>
       <c r="E233" t="n">
-        <v>4693.52</v>
+        <v>971.33</v>
       </c>
       <c r="F233" t="n">
-        <v>0</v>
+        <v>773.74</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C234" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D234" t="n">
-        <v>794671</v>
+        <v>33057</v>
       </c>
       <c r="E234" t="n">
-        <v>3481.16</v>
+        <v>89.06</v>
       </c>
       <c r="F234" t="n">
         <v>0</v>
@@ -6059,46 +6059,46 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C235" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D235" t="n">
-        <v>30791</v>
+        <v>789525</v>
       </c>
       <c r="E235" t="n">
-        <v>7474.12</v>
+        <v>6610.45</v>
       </c>
       <c r="F235" t="n">
-        <v>0</v>
+        <v>258.75</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C236" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D236" t="n">
-        <v>47252</v>
+        <v>33057</v>
       </c>
       <c r="E236" t="n">
-        <v>24650.04</v>
+        <v>4738.27</v>
       </c>
       <c r="F236" t="n">
         <v>0</v>
@@ -6107,22 +6107,22 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C237" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D237" t="n">
-        <v>789525</v>
+        <v>794671</v>
       </c>
       <c r="E237" t="n">
-        <v>1451.86</v>
+        <v>3481.16</v>
       </c>
       <c r="F237" t="n">
         <v>0</v>
@@ -6136,17 +6136,17 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C238" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D238" t="n">
-        <v>30307</v>
+        <v>30791</v>
       </c>
       <c r="E238" t="n">
-        <v>575.88</v>
+        <v>8002.71</v>
       </c>
       <c r="F238" t="n">
         <v>0</v>
@@ -6160,44 +6160,44 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C239" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D239" t="n">
-        <v>30791</v>
+        <v>47252</v>
       </c>
       <c r="E239" t="n">
-        <v>44.88</v>
+        <v>24906.33</v>
       </c>
       <c r="F239" t="n">
-        <v>0</v>
+        <v>59.23</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C240" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D240" t="n">
-        <v>790595</v>
+        <v>789525</v>
       </c>
       <c r="E240" t="n">
-        <v>1151.94</v>
+        <v>1452</v>
       </c>
       <c r="F240" t="n">
-        <v>0</v>
+        <v>201.01</v>
       </c>
     </row>
     <row r="241">
@@ -6208,17 +6208,17 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="C241" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D241" t="n">
-        <v>47252</v>
+        <v>30307</v>
       </c>
       <c r="E241" t="n">
-        <v>28417.74</v>
+        <v>575.88</v>
       </c>
       <c r="F241" t="n">
         <v>0</v>
@@ -6227,22 +6227,22 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="C242" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D242" t="n">
-        <v>795345</v>
+        <v>30791</v>
       </c>
       <c r="E242" t="n">
-        <v>4352.64</v>
+        <v>44.88</v>
       </c>
       <c r="F242" t="n">
         <v>0</v>
@@ -6263,10 +6263,10 @@
         <v>46247</v>
       </c>
       <c r="D243" t="n">
-        <v>794029</v>
+        <v>790595</v>
       </c>
       <c r="E243" t="n">
-        <v>4267.52</v>
+        <v>1151.94</v>
       </c>
       <c r="F243" t="n">
         <v>0</v>
@@ -6275,46 +6275,46 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C244" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D244" t="n">
-        <v>789603</v>
+        <v>47252</v>
       </c>
       <c r="E244" t="n">
-        <v>68263.56</v>
+        <v>28417.89</v>
       </c>
       <c r="F244" t="n">
-        <v>41155.22</v>
+        <v>427.24</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C245" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D245" t="n">
-        <v>31267</v>
+        <v>795345</v>
       </c>
       <c r="E245" t="n">
-        <v>26.27</v>
+        <v>5428.94</v>
       </c>
       <c r="F245" t="n">
         <v>0</v>
@@ -6323,25 +6323,25 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C246" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D246" t="n">
-        <v>793186</v>
+        <v>789603</v>
       </c>
       <c r="E246" t="n">
-        <v>443.79</v>
+        <v>69383.48</v>
       </c>
       <c r="F246" t="n">
-        <v>54.71</v>
+        <v>41155.22</v>
       </c>
     </row>
     <row r="247">
@@ -6352,17 +6352,17 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C247" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D247" t="n">
-        <v>30307</v>
+        <v>31267</v>
       </c>
       <c r="E247" t="n">
-        <v>9372.809999999999</v>
+        <v>26.27</v>
       </c>
       <c r="F247" t="n">
         <v>0</v>
@@ -6371,46 +6371,46 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C248" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D248" t="n">
-        <v>794671</v>
+        <v>793186</v>
       </c>
       <c r="E248" t="n">
-        <v>2215.21</v>
+        <v>443.79</v>
       </c>
       <c r="F248" t="n">
-        <v>0</v>
+        <v>54.71</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C249" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D249" t="n">
-        <v>790595</v>
+        <v>30307</v>
       </c>
       <c r="E249" t="n">
-        <v>1266.58</v>
+        <v>9372.809999999999</v>
       </c>
       <c r="F249" t="n">
         <v>0</v>
@@ -6419,22 +6419,22 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C250" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D250" t="n">
-        <v>792141</v>
+        <v>794671</v>
       </c>
       <c r="E250" t="n">
-        <v>3019.8</v>
+        <v>2456.84</v>
       </c>
       <c r="F250" t="n">
         <v>0</v>
@@ -6443,22 +6443,22 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C251" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D251" t="n">
-        <v>793186</v>
+        <v>790595</v>
       </c>
       <c r="E251" t="n">
-        <v>146.11</v>
+        <v>1266.58</v>
       </c>
       <c r="F251" t="n">
         <v>0</v>
@@ -6467,22 +6467,22 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C252" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D252" t="n">
-        <v>792121</v>
+        <v>792141</v>
       </c>
       <c r="E252" t="n">
-        <v>1936.84</v>
+        <v>3019.8</v>
       </c>
       <c r="F252" t="n">
         <v>0</v>
@@ -6491,22 +6491,22 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C253" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D253" t="n">
-        <v>30083</v>
+        <v>793186</v>
       </c>
       <c r="E253" t="n">
-        <v>3299.7</v>
+        <v>146.11</v>
       </c>
       <c r="F253" t="n">
         <v>0</v>
@@ -6515,22 +6515,22 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C254" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D254" t="n">
-        <v>789603</v>
+        <v>792121</v>
       </c>
       <c r="E254" t="n">
-        <v>9428.620000000001</v>
+        <v>3285.89</v>
       </c>
       <c r="F254" t="n">
         <v>0</v>
@@ -6539,22 +6539,22 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C255" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D255" t="n">
-        <v>139553</v>
+        <v>30083</v>
       </c>
       <c r="E255" t="n">
-        <v>6107.48</v>
+        <v>4445.94</v>
       </c>
       <c r="F255" t="n">
         <v>0</v>
@@ -6563,22 +6563,22 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C256" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D256" t="n">
-        <v>33057</v>
+        <v>789603</v>
       </c>
       <c r="E256" t="n">
-        <v>12085.79</v>
+        <v>10399.38</v>
       </c>
       <c r="F256" t="n">
         <v>0</v>
@@ -6587,22 +6587,22 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C257" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D257" t="n">
-        <v>33928</v>
+        <v>139553</v>
       </c>
       <c r="E257" t="n">
-        <v>2009.33</v>
+        <v>6107.48</v>
       </c>
       <c r="F257" t="n">
         <v>0</v>
@@ -6611,22 +6611,22 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C258" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D258" t="n">
-        <v>792121</v>
+        <v>33057</v>
       </c>
       <c r="E258" t="n">
-        <v>501.32</v>
+        <v>12143.3</v>
       </c>
       <c r="F258" t="n">
         <v>0</v>
@@ -6635,22 +6635,22 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C259" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D259" t="n">
-        <v>32816</v>
+        <v>33928</v>
       </c>
       <c r="E259" t="n">
-        <v>74.84999999999999</v>
+        <v>2041.7</v>
       </c>
       <c r="F259" t="n">
         <v>0</v>
@@ -6659,22 +6659,22 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C260" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D260" t="n">
-        <v>139553</v>
+        <v>792121</v>
       </c>
       <c r="E260" t="n">
-        <v>2570.35</v>
+        <v>501.32</v>
       </c>
       <c r="F260" t="n">
         <v>0</v>
@@ -6683,22 +6683,22 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C261" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D261" t="n">
-        <v>795345</v>
+        <v>32816</v>
       </c>
       <c r="E261" t="n">
-        <v>283.88</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="F261" t="n">
         <v>0</v>
@@ -6707,22 +6707,22 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C262" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D262" t="n">
-        <v>33286</v>
+        <v>139553</v>
       </c>
       <c r="E262" t="n">
-        <v>111.21</v>
+        <v>2570.35</v>
       </c>
       <c r="F262" t="n">
         <v>0</v>
@@ -6731,12 +6731,12 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C263" s="2" t="n">
@@ -6746,9 +6746,57 @@
         <v>795345</v>
       </c>
       <c r="E263" t="n">
+        <v>283.88</v>
+      </c>
+      <c r="F263" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D264" t="n">
+        <v>33286</v>
+      </c>
+      <c r="E264" t="n">
+        <v>111.21</v>
+      </c>
+      <c r="F264" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D265" t="n">
+        <v>795345</v>
+      </c>
+      <c r="E265" t="n">
         <v>169.57</v>
       </c>
-      <c r="F263" t="n">
+      <c r="F265" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 14:45:04
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F268"/>
+  <dimension ref="A1:F267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,7 +506,7 @@
         <v>47252</v>
       </c>
       <c r="E3" t="n">
-        <v>23944.81</v>
+        <v>26543.59</v>
       </c>
       <c r="F3" t="n">
         <v>4337.7</v>
@@ -530,7 +530,7 @@
         <v>33928</v>
       </c>
       <c r="E4" t="n">
-        <v>32219.12</v>
+        <v>32246.2</v>
       </c>
       <c r="F4" t="n">
         <v>21693.55</v>
@@ -578,7 +578,7 @@
         <v>33928</v>
       </c>
       <c r="E6" t="n">
-        <v>8280.34</v>
+        <v>8467.49</v>
       </c>
       <c r="F6" t="n">
         <v>391.48</v>
@@ -602,7 +602,7 @@
         <v>30791</v>
       </c>
       <c r="E7" t="n">
-        <v>18956.35</v>
+        <v>19001.51</v>
       </c>
       <c r="F7" t="n">
         <v>3111.54</v>
@@ -698,7 +698,7 @@
         <v>789525</v>
       </c>
       <c r="E11" t="n">
-        <v>1914.23</v>
+        <v>1569.82</v>
       </c>
       <c r="F11" t="n">
         <v>98.76000000000001</v>
@@ -818,7 +818,7 @@
         <v>31267</v>
       </c>
       <c r="E16" t="n">
-        <v>1163.91</v>
+        <v>1403.84</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -866,7 +866,7 @@
         <v>795345</v>
       </c>
       <c r="E18" t="n">
-        <v>1423.86</v>
+        <v>1519.86</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -938,7 +938,7 @@
         <v>30307</v>
       </c>
       <c r="E21" t="n">
-        <v>51515.33</v>
+        <v>52568.93</v>
       </c>
       <c r="F21" t="n">
         <v>22829.12</v>
@@ -962,7 +962,7 @@
         <v>795345</v>
       </c>
       <c r="E22" t="n">
-        <v>2064.91</v>
+        <v>2178.27</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
@@ -1058,7 +1058,7 @@
         <v>139553</v>
       </c>
       <c r="E26" t="n">
-        <v>6757.93</v>
+        <v>7375.71</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -1082,7 +1082,7 @@
         <v>30083</v>
       </c>
       <c r="E27" t="n">
-        <v>3937.97</v>
+        <v>4216.66</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -1130,7 +1130,7 @@
         <v>33057</v>
       </c>
       <c r="E29" t="n">
-        <v>1046.83</v>
+        <v>1090.15</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -1202,7 +1202,7 @@
         <v>31267</v>
       </c>
       <c r="E32" t="n">
-        <v>149376</v>
+        <v>150095.85</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -1226,7 +1226,7 @@
         <v>794671</v>
       </c>
       <c r="E33" t="n">
-        <v>12589.57</v>
+        <v>15176.01</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
@@ -1250,7 +1250,7 @@
         <v>792246</v>
       </c>
       <c r="E34" t="n">
-        <v>518.28</v>
+        <v>888.23</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
@@ -1480,20 +1480,20 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D44" t="n">
-        <v>33057</v>
+        <v>33286</v>
       </c>
       <c r="E44" t="n">
-        <v>3916.64</v>
+        <v>760.92</v>
       </c>
       <c r="F44" t="n">
-        <v>97.77</v>
+        <v>91.13</v>
       </c>
     </row>
     <row r="45">
@@ -1511,13 +1511,13 @@
         <v>46247</v>
       </c>
       <c r="D45" t="n">
-        <v>31267</v>
+        <v>33057</v>
       </c>
       <c r="E45" t="n">
-        <v>7269.61</v>
+        <v>3916.64</v>
       </c>
       <c r="F45" t="n">
-        <v>165.42</v>
+        <v>97.77</v>
       </c>
     </row>
     <row r="46">
@@ -1528,20 +1528,20 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D46" t="n">
-        <v>30791</v>
+        <v>31267</v>
       </c>
       <c r="E46" t="n">
-        <v>17736.76</v>
+        <v>7352.44</v>
       </c>
       <c r="F46" t="n">
-        <v>685.66</v>
+        <v>165.42</v>
       </c>
     </row>
     <row r="47">
@@ -1559,13 +1559,13 @@
         <v>46247</v>
       </c>
       <c r="D47" t="n">
-        <v>793718</v>
+        <v>30791</v>
       </c>
       <c r="E47" t="n">
-        <v>4818.08</v>
+        <v>17736.76</v>
       </c>
       <c r="F47" t="n">
-        <v>120.72</v>
+        <v>685.66</v>
       </c>
     </row>
     <row r="48">
@@ -1576,20 +1576,20 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D48" t="n">
-        <v>33286</v>
+        <v>793718</v>
       </c>
       <c r="E48" t="n">
-        <v>697.6900000000001</v>
+        <v>4818.08</v>
       </c>
       <c r="F48" t="n">
-        <v>91.13</v>
+        <v>120.72</v>
       </c>
     </row>
     <row r="49">
@@ -1634,7 +1634,7 @@
         <v>47252</v>
       </c>
       <c r="E50" t="n">
-        <v>21448.7</v>
+        <v>30992.51</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
@@ -1658,7 +1658,7 @@
         <v>789228</v>
       </c>
       <c r="E51" t="n">
-        <v>3644.72</v>
+        <v>4682.6</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
@@ -1706,7 +1706,7 @@
         <v>33928</v>
       </c>
       <c r="E53" t="n">
-        <v>2301.62</v>
+        <v>2380</v>
       </c>
       <c r="F53" t="n">
         <v>25.2</v>
@@ -1754,7 +1754,7 @@
         <v>792121</v>
       </c>
       <c r="E55" t="n">
-        <v>11111.71</v>
+        <v>12725.13</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
@@ -1826,7 +1826,7 @@
         <v>789603</v>
       </c>
       <c r="E58" t="n">
-        <v>17976.88</v>
+        <v>18244.4</v>
       </c>
       <c r="F58" t="n">
         <v>4547.77</v>
@@ -1850,7 +1850,7 @@
         <v>792121</v>
       </c>
       <c r="E59" t="n">
-        <v>4707.1</v>
+        <v>4898.32</v>
       </c>
       <c r="F59" t="n">
         <v>0</v>
@@ -1898,7 +1898,7 @@
         <v>30307</v>
       </c>
       <c r="E61" t="n">
-        <v>17764.94</v>
+        <v>18511.82</v>
       </c>
       <c r="F61" t="n">
         <v>2004.16</v>
@@ -2234,7 +2234,7 @@
         <v>30791</v>
       </c>
       <c r="E75" t="n">
-        <v>12674.85</v>
+        <v>12757.91</v>
       </c>
       <c r="F75" t="n">
         <v>1524.6</v>
@@ -2255,13 +2255,13 @@
         <v>46247</v>
       </c>
       <c r="D76" t="n">
-        <v>33286</v>
+        <v>793718</v>
       </c>
       <c r="E76" t="n">
-        <v>1345.11</v>
+        <v>676.13</v>
       </c>
       <c r="F76" t="n">
-        <v>230.41</v>
+        <v>238.95</v>
       </c>
     </row>
     <row r="77">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -2282,10 +2282,10 @@
         <v>33286</v>
       </c>
       <c r="E77" t="n">
-        <v>2864.26</v>
+        <v>1403.97</v>
       </c>
       <c r="F77" t="n">
-        <v>327.9</v>
+        <v>230.41</v>
       </c>
     </row>
     <row r="78">
@@ -2296,20 +2296,20 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D78" t="n">
-        <v>793718</v>
+        <v>33286</v>
       </c>
       <c r="E78" t="n">
-        <v>630.33</v>
+        <v>2864.26</v>
       </c>
       <c r="F78" t="n">
-        <v>238.95</v>
+        <v>327.9</v>
       </c>
     </row>
     <row r="79">
@@ -2354,10 +2354,10 @@
         <v>793718</v>
       </c>
       <c r="E80" t="n">
-        <v>1556.8</v>
+        <v>1557.64</v>
       </c>
       <c r="F80" t="n">
-        <v>1261.34</v>
+        <v>1557.63</v>
       </c>
     </row>
     <row r="81">
@@ -2378,7 +2378,7 @@
         <v>31267</v>
       </c>
       <c r="E81" t="n">
-        <v>4328.83</v>
+        <v>5176.78</v>
       </c>
       <c r="F81" t="n">
         <v>0</v>
@@ -2450,7 +2450,7 @@
         <v>33286</v>
       </c>
       <c r="E84" t="n">
-        <v>2476.67</v>
+        <v>2611.19</v>
       </c>
       <c r="F84" t="n">
         <v>0</v>
@@ -2570,7 +2570,7 @@
         <v>139553</v>
       </c>
       <c r="E89" t="n">
-        <v>5468.49</v>
+        <v>3723.95</v>
       </c>
       <c r="F89" t="n">
         <v>0</v>
@@ -2714,7 +2714,7 @@
         <v>33057</v>
       </c>
       <c r="E95" t="n">
-        <v>1995.85</v>
+        <v>3285.71</v>
       </c>
       <c r="F95" t="n">
         <v>0</v>
@@ -2738,7 +2738,7 @@
         <v>47252</v>
       </c>
       <c r="E96" t="n">
-        <v>16628.41</v>
+        <v>16271.9</v>
       </c>
       <c r="F96" t="n">
         <v>4814.96</v>
@@ -2810,7 +2810,7 @@
         <v>47252</v>
       </c>
       <c r="E99" t="n">
-        <v>2836.87</v>
+        <v>4887.9</v>
       </c>
       <c r="F99" t="n">
         <v>0</v>
@@ -2954,7 +2954,7 @@
         <v>789525</v>
       </c>
       <c r="E105" t="n">
-        <v>3318.51</v>
+        <v>3591.73</v>
       </c>
       <c r="F105" t="n">
         <v>288.23</v>
@@ -3071,13 +3071,13 @@
         <v>46247</v>
       </c>
       <c r="D110" t="n">
-        <v>30083</v>
+        <v>33928</v>
       </c>
       <c r="E110" t="n">
-        <v>137.67</v>
+        <v>17926.68</v>
       </c>
       <c r="F110" t="n">
-        <v>0</v>
+        <v>30.75</v>
       </c>
     </row>
     <row r="111">
@@ -3095,13 +3095,13 @@
         <v>46247</v>
       </c>
       <c r="D111" t="n">
-        <v>33928</v>
+        <v>30083</v>
       </c>
       <c r="E111" t="n">
-        <v>14204.55</v>
+        <v>137.67</v>
       </c>
       <c r="F111" t="n">
-        <v>30.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112">
@@ -3290,7 +3290,7 @@
         <v>30307</v>
       </c>
       <c r="E119" t="n">
-        <v>37635.55</v>
+        <v>33538.47</v>
       </c>
       <c r="F119" t="n">
         <v>5110.57</v>
@@ -3314,7 +3314,7 @@
         <v>792121</v>
       </c>
       <c r="E120" t="n">
-        <v>1710.2</v>
+        <v>1748.38</v>
       </c>
       <c r="F120" t="n">
         <v>0</v>
@@ -3386,7 +3386,7 @@
         <v>793718</v>
       </c>
       <c r="E123" t="n">
-        <v>644.3200000000001</v>
+        <v>921.35</v>
       </c>
       <c r="F123" t="n">
         <v>0</v>
@@ -3506,7 +3506,7 @@
         <v>789603</v>
       </c>
       <c r="E128" t="n">
-        <v>3636.01</v>
+        <v>4688.05</v>
       </c>
       <c r="F128" t="n">
         <v>0</v>
@@ -3722,7 +3722,7 @@
         <v>47252</v>
       </c>
       <c r="E137" t="n">
-        <v>22682.14</v>
+        <v>25562.49</v>
       </c>
       <c r="F137" t="n">
         <v>1686.2</v>
@@ -3746,7 +3746,7 @@
         <v>47252</v>
       </c>
       <c r="E138" t="n">
-        <v>26573.59</v>
+        <v>28865.6</v>
       </c>
       <c r="F138" t="n">
         <v>4632.36</v>
@@ -3767,13 +3767,13 @@
         <v>46247</v>
       </c>
       <c r="D139" t="n">
-        <v>795345</v>
+        <v>789661</v>
       </c>
       <c r="E139" t="n">
-        <v>27.25</v>
+        <v>338.42</v>
       </c>
       <c r="F139" t="n">
-        <v>0</v>
+        <v>258.83</v>
       </c>
     </row>
     <row r="140">
@@ -3784,17 +3784,17 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D140" t="n">
-        <v>793718</v>
+        <v>795345</v>
       </c>
       <c r="E140" t="n">
-        <v>39.84</v>
+        <v>27.25</v>
       </c>
       <c r="F140" t="n">
         <v>0</v>
@@ -3803,7 +3803,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -3815,10 +3815,10 @@
         <v>46247</v>
       </c>
       <c r="D141" t="n">
-        <v>789525</v>
+        <v>793718</v>
       </c>
       <c r="E141" t="n">
-        <v>34.37</v>
+        <v>39.84</v>
       </c>
       <c r="F141" t="n">
         <v>0</v>
@@ -3827,7 +3827,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3839,10 +3839,10 @@
         <v>46247</v>
       </c>
       <c r="D142" t="n">
-        <v>33057</v>
+        <v>789525</v>
       </c>
       <c r="E142" t="n">
-        <v>42.76</v>
+        <v>34.37</v>
       </c>
       <c r="F142" t="n">
         <v>0</v>
@@ -3863,10 +3863,10 @@
         <v>46247</v>
       </c>
       <c r="D143" t="n">
-        <v>30791</v>
+        <v>33057</v>
       </c>
       <c r="E143" t="n">
-        <v>33.08</v>
+        <v>42.76</v>
       </c>
       <c r="F143" t="n">
         <v>0</v>
@@ -3875,49 +3875,49 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C144" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D144" t="n">
-        <v>31267</v>
+        <v>30791</v>
       </c>
       <c r="E144" t="n">
-        <v>160.86</v>
+        <v>33.08</v>
       </c>
       <c r="F144" t="n">
-        <v>42.93</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C145" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D145" t="n">
-        <v>33286</v>
+        <v>31267</v>
       </c>
       <c r="E145" t="n">
-        <v>9219.41</v>
+        <v>160.86</v>
       </c>
       <c r="F145" t="n">
-        <v>0</v>
+        <v>42.93</v>
       </c>
     </row>
     <row r="146">
@@ -3935,10 +3935,10 @@
         <v>46247</v>
       </c>
       <c r="D146" t="n">
-        <v>139553</v>
+        <v>33286</v>
       </c>
       <c r="E146" t="n">
-        <v>1106.98</v>
+        <v>9464.99</v>
       </c>
       <c r="F146" t="n">
         <v>0</v>
@@ -3947,70 +3947,70 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C147" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D147" t="n">
-        <v>30791</v>
+        <v>139553</v>
       </c>
       <c r="E147" t="n">
-        <v>0</v>
+        <v>1106.98</v>
       </c>
       <c r="F147" t="n">
-        <v>646.85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C148" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D148" t="n">
-        <v>30307</v>
+        <v>30791</v>
       </c>
       <c r="E148" t="n">
-        <v>507.68</v>
+        <v>0</v>
       </c>
       <c r="F148" t="n">
-        <v>0</v>
+        <v>646.85</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C149" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D149" t="n">
-        <v>33057</v>
+        <v>30307</v>
       </c>
       <c r="E149" t="n">
-        <v>146.56</v>
+        <v>507.68</v>
       </c>
       <c r="F149" t="n">
         <v>0</v>
@@ -4019,25 +4019,25 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C150" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D150" t="n">
-        <v>789661</v>
+        <v>33057</v>
       </c>
       <c r="E150" t="n">
-        <v>37.05</v>
+        <v>146.56</v>
       </c>
       <c r="F150" t="n">
-        <v>258.83</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151">
@@ -4082,7 +4082,7 @@
         <v>794671</v>
       </c>
       <c r="E152" t="n">
-        <v>1295.61</v>
+        <v>3106.15</v>
       </c>
       <c r="F152" t="n">
         <v>0</v>
@@ -4226,7 +4226,7 @@
         <v>31267</v>
       </c>
       <c r="E158" t="n">
-        <v>155868.01</v>
+        <v>156717.26</v>
       </c>
       <c r="F158" t="n">
         <v>0</v>
@@ -4250,7 +4250,7 @@
         <v>794029</v>
       </c>
       <c r="E159" t="n">
-        <v>9162.23</v>
+        <v>10000.21</v>
       </c>
       <c r="F159" t="n">
         <v>0</v>
@@ -4394,7 +4394,7 @@
         <v>139553</v>
       </c>
       <c r="E165" t="n">
-        <v>1621.76</v>
+        <v>1777.7</v>
       </c>
       <c r="F165" t="n">
         <v>0</v>
@@ -4418,7 +4418,7 @@
         <v>795345</v>
       </c>
       <c r="E166" t="n">
-        <v>204.29</v>
+        <v>243.41</v>
       </c>
       <c r="F166" t="n">
         <v>0</v>
@@ -4499,49 +4499,49 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C170" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D170" t="n">
-        <v>794671</v>
+        <v>32816</v>
       </c>
       <c r="E170" t="n">
-        <v>1810.54</v>
+        <v>1721.48</v>
       </c>
       <c r="F170" t="n">
-        <v>0</v>
+        <v>637.4400000000001</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C171" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D171" t="n">
-        <v>32816</v>
+        <v>795345</v>
       </c>
       <c r="E171" t="n">
-        <v>1721.48</v>
+        <v>2169.18</v>
       </c>
       <c r="F171" t="n">
-        <v>637.4400000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="172">
@@ -4552,17 +4552,17 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C172" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D172" t="n">
-        <v>795345</v>
+        <v>789603</v>
       </c>
       <c r="E172" t="n">
-        <v>2169.18</v>
+        <v>7108.74</v>
       </c>
       <c r="F172" t="n">
         <v>0</v>
@@ -4571,22 +4571,22 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C173" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D173" t="n">
-        <v>789603</v>
+        <v>33057</v>
       </c>
       <c r="E173" t="n">
-        <v>7108.74</v>
+        <v>1824.79</v>
       </c>
       <c r="F173" t="n">
         <v>0</v>
@@ -4600,17 +4600,17 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C174" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D174" t="n">
-        <v>33057</v>
+        <v>32816</v>
       </c>
       <c r="E174" t="n">
-        <v>631.5700000000001</v>
+        <v>314.62</v>
       </c>
       <c r="F174" t="n">
         <v>0</v>
@@ -4682,7 +4682,7 @@
         <v>793186</v>
       </c>
       <c r="E177" t="n">
-        <v>403.84</v>
+        <v>1215.54</v>
       </c>
       <c r="F177" t="n">
         <v>0</v>
@@ -4730,7 +4730,7 @@
         <v>793718</v>
       </c>
       <c r="E179" t="n">
-        <v>3381.76</v>
+        <v>3625.12</v>
       </c>
       <c r="F179" t="n">
         <v>0</v>
@@ -4754,7 +4754,7 @@
         <v>789228</v>
       </c>
       <c r="E180" t="n">
-        <v>1746.05</v>
+        <v>1854.71</v>
       </c>
       <c r="F180" t="n">
         <v>0</v>
@@ -4912,26 +4912,26 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C187" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D187" t="n">
-        <v>32816</v>
+        <v>47252</v>
       </c>
       <c r="E187" t="n">
-        <v>75.75</v>
+        <v>3179.29</v>
       </c>
       <c r="F187" t="n">
-        <v>0</v>
+        <v>628.86</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -4943,61 +4943,61 @@
         <v>46247</v>
       </c>
       <c r="D188" t="n">
-        <v>47252</v>
+        <v>795345</v>
       </c>
       <c r="E188" t="n">
-        <v>3179.29</v>
+        <v>439.18</v>
       </c>
       <c r="F188" t="n">
-        <v>628.86</v>
+        <v>0</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C189" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D189" t="n">
-        <v>795345</v>
+        <v>792141</v>
       </c>
       <c r="E189" t="n">
-        <v>439.18</v>
+        <v>11095.24</v>
       </c>
       <c r="F189" t="n">
-        <v>0</v>
+        <v>321.34</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C190" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D190" t="n">
-        <v>792141</v>
+        <v>792121</v>
       </c>
       <c r="E190" t="n">
-        <v>11095.24</v>
+        <v>1025.88</v>
       </c>
       <c r="F190" t="n">
-        <v>321.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="191">
@@ -5008,17 +5008,17 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C191" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D191" t="n">
-        <v>792121</v>
+        <v>793718</v>
       </c>
       <c r="E191" t="n">
-        <v>1025.88</v>
+        <v>269.48</v>
       </c>
       <c r="F191" t="n">
         <v>0</v>
@@ -5032,17 +5032,17 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C192" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D192" t="n">
-        <v>793718</v>
+        <v>794671</v>
       </c>
       <c r="E192" t="n">
-        <v>269.48</v>
+        <v>798.3099999999999</v>
       </c>
       <c r="F192" t="n">
         <v>0</v>
@@ -5051,25 +5051,25 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C193" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D193" t="n">
-        <v>794671</v>
+        <v>31267</v>
       </c>
       <c r="E193" t="n">
-        <v>798.3099999999999</v>
+        <v>27246.56</v>
       </c>
       <c r="F193" t="n">
-        <v>0</v>
+        <v>2242.99</v>
       </c>
     </row>
     <row r="194">
@@ -5087,13 +5087,13 @@
         <v>46247</v>
       </c>
       <c r="D194" t="n">
-        <v>31267</v>
+        <v>789525</v>
       </c>
       <c r="E194" t="n">
-        <v>27246.56</v>
+        <v>5778.32</v>
       </c>
       <c r="F194" t="n">
-        <v>2242.99</v>
+        <v>1019.16</v>
       </c>
     </row>
     <row r="195">
@@ -5111,37 +5111,37 @@
         <v>46247</v>
       </c>
       <c r="D195" t="n">
-        <v>789525</v>
+        <v>789228</v>
       </c>
       <c r="E195" t="n">
-        <v>5327.65</v>
+        <v>241.92</v>
       </c>
       <c r="F195" t="n">
-        <v>1019.16</v>
+        <v>33.67</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C196" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D196" t="n">
-        <v>789228</v>
+        <v>793186</v>
       </c>
       <c r="E196" t="n">
-        <v>241.92</v>
+        <v>13.91</v>
       </c>
       <c r="F196" t="n">
-        <v>33.67</v>
+        <v>13.91</v>
       </c>
     </row>
     <row r="197">
@@ -5159,19 +5159,19 @@
         <v>46247</v>
       </c>
       <c r="D197" t="n">
-        <v>793186</v>
+        <v>47252</v>
       </c>
       <c r="E197" t="n">
-        <v>13.91</v>
+        <v>15.24</v>
       </c>
       <c r="F197" t="n">
-        <v>13.91</v>
+        <v>5.57</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5183,48 +5183,48 @@
         <v>46247</v>
       </c>
       <c r="D198" t="n">
-        <v>47252</v>
+        <v>31267</v>
       </c>
       <c r="E198" t="n">
-        <v>15.24</v>
+        <v>14.99</v>
       </c>
       <c r="F198" t="n">
-        <v>5.57</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C199" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D199" t="n">
-        <v>31267</v>
+        <v>30791</v>
       </c>
       <c r="E199" t="n">
-        <v>14.99</v>
+        <v>6091.31</v>
       </c>
       <c r="F199" t="n">
-        <v>0</v>
+        <v>174.72</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C200" s="2" t="n">
@@ -5234,10 +5234,10 @@
         <v>30791</v>
       </c>
       <c r="E200" t="n">
-        <v>1864.57</v>
+        <v>20763.11</v>
       </c>
       <c r="F200" t="n">
-        <v>174.72</v>
+        <v>461.37</v>
       </c>
     </row>
     <row r="201">
@@ -5255,13 +5255,13 @@
         <v>46247</v>
       </c>
       <c r="D201" t="n">
-        <v>30791</v>
+        <v>789603</v>
       </c>
       <c r="E201" t="n">
-        <v>20564.31</v>
+        <v>37483.89</v>
       </c>
       <c r="F201" t="n">
-        <v>461.37</v>
+        <v>400.32</v>
       </c>
     </row>
     <row r="202">
@@ -5279,13 +5279,13 @@
         <v>46247</v>
       </c>
       <c r="D202" t="n">
-        <v>789603</v>
+        <v>30307</v>
       </c>
       <c r="E202" t="n">
-        <v>37483.89</v>
+        <v>343.86</v>
       </c>
       <c r="F202" t="n">
-        <v>400.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="203">
@@ -5303,10 +5303,10 @@
         <v>46247</v>
       </c>
       <c r="D203" t="n">
-        <v>30307</v>
+        <v>792141</v>
       </c>
       <c r="E203" t="n">
-        <v>343.86</v>
+        <v>20256.59</v>
       </c>
       <c r="F203" t="n">
         <v>0</v>
@@ -5315,22 +5315,22 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C204" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D204" t="n">
-        <v>792141</v>
+        <v>794029</v>
       </c>
       <c r="E204" t="n">
-        <v>16714.21</v>
+        <v>89.33</v>
       </c>
       <c r="F204" t="n">
         <v>0</v>
@@ -5344,17 +5344,17 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C205" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D205" t="n">
-        <v>794029</v>
+        <v>794671</v>
       </c>
       <c r="E205" t="n">
-        <v>89.33</v>
+        <v>4114.68</v>
       </c>
       <c r="F205" t="n">
         <v>0</v>
@@ -5375,10 +5375,10 @@
         <v>46247</v>
       </c>
       <c r="D206" t="n">
-        <v>794671</v>
+        <v>795345</v>
       </c>
       <c r="E206" t="n">
-        <v>4114.68</v>
+        <v>4716.08</v>
       </c>
       <c r="F206" t="n">
         <v>0</v>
@@ -5387,22 +5387,22 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C207" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D207" t="n">
-        <v>795345</v>
+        <v>33928</v>
       </c>
       <c r="E207" t="n">
-        <v>4716.08</v>
+        <v>46.44</v>
       </c>
       <c r="F207" t="n">
         <v>0</v>
@@ -5411,22 +5411,22 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C208" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D208" t="n">
-        <v>33928</v>
+        <v>30083</v>
       </c>
       <c r="E208" t="n">
-        <v>46.44</v>
+        <v>940.67</v>
       </c>
       <c r="F208" t="n">
         <v>0</v>
@@ -5435,22 +5435,22 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C209" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D209" t="n">
-        <v>30083</v>
+        <v>32816</v>
       </c>
       <c r="E209" t="n">
-        <v>940.67</v>
+        <v>456.96</v>
       </c>
       <c r="F209" t="n">
         <v>0</v>
@@ -5459,22 +5459,22 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C210" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D210" t="n">
-        <v>32816</v>
+        <v>31267</v>
       </c>
       <c r="E210" t="n">
-        <v>456.96</v>
+        <v>939.3</v>
       </c>
       <c r="F210" t="n">
         <v>0</v>
@@ -5483,22 +5483,22 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C211" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D211" t="n">
-        <v>31267</v>
+        <v>790595</v>
       </c>
       <c r="E211" t="n">
-        <v>939.3</v>
+        <v>267.36</v>
       </c>
       <c r="F211" t="n">
         <v>0</v>
@@ -5519,10 +5519,10 @@
         <v>46247</v>
       </c>
       <c r="D212" t="n">
-        <v>790595</v>
+        <v>30218</v>
       </c>
       <c r="E212" t="n">
-        <v>267.36</v>
+        <v>3083.55</v>
       </c>
       <c r="F212" t="n">
         <v>0</v>
@@ -5531,22 +5531,22 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C213" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D213" t="n">
-        <v>30218</v>
+        <v>47252</v>
       </c>
       <c r="E213" t="n">
-        <v>2443.81</v>
+        <v>25441.97</v>
       </c>
       <c r="F213" t="n">
         <v>0</v>
@@ -5567,10 +5567,10 @@
         <v>46247</v>
       </c>
       <c r="D214" t="n">
-        <v>47252</v>
+        <v>794671</v>
       </c>
       <c r="E214" t="n">
-        <v>24264.62</v>
+        <v>276.11</v>
       </c>
       <c r="F214" t="n">
         <v>0</v>
@@ -5579,22 +5579,22 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C215" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D215" t="n">
-        <v>794671</v>
+        <v>789603</v>
       </c>
       <c r="E215" t="n">
-        <v>276.11</v>
+        <v>12435.93</v>
       </c>
       <c r="F215" t="n">
         <v>0</v>
@@ -5603,22 +5603,22 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C216" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D216" t="n">
-        <v>789603</v>
+        <v>139553</v>
       </c>
       <c r="E216" t="n">
-        <v>12435.93</v>
+        <v>406.68</v>
       </c>
       <c r="F216" t="n">
         <v>0</v>
@@ -5627,94 +5627,94 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C217" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D217" t="n">
-        <v>139553</v>
+        <v>793186</v>
       </c>
       <c r="E217" t="n">
-        <v>406.68</v>
+        <v>15013.93</v>
       </c>
       <c r="F217" t="n">
-        <v>0</v>
+        <v>702.38</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C218" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D218" t="n">
-        <v>793186</v>
+        <v>139553</v>
       </c>
       <c r="E218" t="n">
-        <v>15013.93</v>
+        <v>8304.940000000001</v>
       </c>
       <c r="F218" t="n">
-        <v>702.38</v>
+        <v>563.04</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C219" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D219" t="n">
-        <v>139553</v>
+        <v>792246</v>
       </c>
       <c r="E219" t="n">
-        <v>8304.940000000001</v>
+        <v>587.38</v>
       </c>
       <c r="F219" t="n">
-        <v>281.52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C220" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D220" t="n">
-        <v>792246</v>
+        <v>789603</v>
       </c>
       <c r="E220" t="n">
-        <v>587.38</v>
+        <v>4287.44</v>
       </c>
       <c r="F220" t="n">
         <v>0</v>
@@ -5728,17 +5728,17 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C221" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D221" t="n">
-        <v>789603</v>
+        <v>30083</v>
       </c>
       <c r="E221" t="n">
-        <v>4287.44</v>
+        <v>627.34</v>
       </c>
       <c r="F221" t="n">
         <v>0</v>
@@ -5752,17 +5752,17 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C222" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D222" t="n">
-        <v>30083</v>
+        <v>795345</v>
       </c>
       <c r="E222" t="n">
-        <v>627.34</v>
+        <v>329.64</v>
       </c>
       <c r="F222" t="n">
         <v>0</v>
@@ -5776,17 +5776,17 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C223" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D223" t="n">
-        <v>795345</v>
+        <v>794029</v>
       </c>
       <c r="E223" t="n">
-        <v>329.64</v>
+        <v>5023.73</v>
       </c>
       <c r="F223" t="n">
         <v>0</v>
@@ -5800,17 +5800,17 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C224" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D224" t="n">
-        <v>794029</v>
+        <v>30307</v>
       </c>
       <c r="E224" t="n">
-        <v>5023.73</v>
+        <v>108224.47</v>
       </c>
       <c r="F224" t="n">
         <v>0</v>
@@ -5831,10 +5831,10 @@
         <v>46247</v>
       </c>
       <c r="D225" t="n">
-        <v>30307</v>
+        <v>30083</v>
       </c>
       <c r="E225" t="n">
-        <v>108224.47</v>
+        <v>5716.11</v>
       </c>
       <c r="F225" t="n">
         <v>0</v>
@@ -5843,25 +5843,25 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C226" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D226" t="n">
-        <v>30083</v>
+        <v>793718</v>
       </c>
       <c r="E226" t="n">
-        <v>5716.11</v>
+        <v>31975.46</v>
       </c>
       <c r="F226" t="n">
-        <v>0</v>
+        <v>1167.12</v>
       </c>
     </row>
     <row r="227">
@@ -5879,43 +5879,43 @@
         <v>46247</v>
       </c>
       <c r="D227" t="n">
-        <v>793718</v>
+        <v>789661</v>
       </c>
       <c r="E227" t="n">
-        <v>31975.46</v>
+        <v>434.06</v>
       </c>
       <c r="F227" t="n">
-        <v>1167.12</v>
+        <v>32.2</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C228" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D228" t="n">
-        <v>789661</v>
+        <v>33286</v>
       </c>
       <c r="E228" t="n">
-        <v>12.35</v>
+        <v>12.44</v>
       </c>
       <c r="F228" t="n">
-        <v>32.2</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -5927,19 +5927,19 @@
         <v>46247</v>
       </c>
       <c r="D229" t="n">
-        <v>33286</v>
+        <v>794671</v>
       </c>
       <c r="E229" t="n">
-        <v>12.44</v>
+        <v>759.41</v>
       </c>
       <c r="F229" t="n">
-        <v>3.99</v>
+        <v>0</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -5951,10 +5951,10 @@
         <v>46247</v>
       </c>
       <c r="D230" t="n">
-        <v>794671</v>
+        <v>30791</v>
       </c>
       <c r="E230" t="n">
-        <v>759.41</v>
+        <v>2.53</v>
       </c>
       <c r="F230" t="n">
         <v>0</v>
@@ -5963,7 +5963,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -5975,10 +5975,10 @@
         <v>46247</v>
       </c>
       <c r="D231" t="n">
-        <v>30791</v>
+        <v>792121</v>
       </c>
       <c r="E231" t="n">
-        <v>2.53</v>
+        <v>47.14</v>
       </c>
       <c r="F231" t="n">
         <v>0</v>
@@ -5999,10 +5999,10 @@
         <v>46247</v>
       </c>
       <c r="D232" t="n">
-        <v>792121</v>
+        <v>139553</v>
       </c>
       <c r="E232" t="n">
-        <v>47.14</v>
+        <v>1300.72</v>
       </c>
       <c r="F232" t="n">
         <v>0</v>
@@ -6023,10 +6023,10 @@
         <v>46247</v>
       </c>
       <c r="D233" t="n">
-        <v>139553</v>
+        <v>794671</v>
       </c>
       <c r="E233" t="n">
-        <v>1300.72</v>
+        <v>1075.68</v>
       </c>
       <c r="F233" t="n">
         <v>0</v>
@@ -6035,25 +6035,25 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C234" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D234" t="n">
-        <v>794671</v>
+        <v>33928</v>
       </c>
       <c r="E234" t="n">
-        <v>1075.68</v>
+        <v>1038.51</v>
       </c>
       <c r="F234" t="n">
-        <v>0</v>
+        <v>41.55</v>
       </c>
     </row>
     <row r="235">
@@ -6071,13 +6071,13 @@
         <v>46247</v>
       </c>
       <c r="D235" t="n">
-        <v>33928</v>
+        <v>789525</v>
       </c>
       <c r="E235" t="n">
-        <v>1038.51</v>
+        <v>971.33</v>
       </c>
       <c r="F235" t="n">
-        <v>41.55</v>
+        <v>773.74</v>
       </c>
     </row>
     <row r="236">
@@ -6095,37 +6095,37 @@
         <v>46247</v>
       </c>
       <c r="D236" t="n">
-        <v>789525</v>
+        <v>33057</v>
       </c>
       <c r="E236" t="n">
-        <v>971.33</v>
+        <v>89.06</v>
       </c>
       <c r="F236" t="n">
-        <v>773.74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C237" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D237" t="n">
-        <v>33057</v>
+        <v>789525</v>
       </c>
       <c r="E237" t="n">
-        <v>89.06</v>
+        <v>7348.77</v>
       </c>
       <c r="F237" t="n">
-        <v>0</v>
+        <v>258.75</v>
       </c>
     </row>
     <row r="238">
@@ -6143,34 +6143,34 @@
         <v>46247</v>
       </c>
       <c r="D238" t="n">
-        <v>789525</v>
+        <v>33057</v>
       </c>
       <c r="E238" t="n">
-        <v>7012.54</v>
+        <v>5515.95</v>
       </c>
       <c r="F238" t="n">
-        <v>258.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C239" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D239" t="n">
-        <v>33057</v>
+        <v>794671</v>
       </c>
       <c r="E239" t="n">
-        <v>4928.66</v>
+        <v>3481.16</v>
       </c>
       <c r="F239" t="n">
         <v>0</v>
@@ -6179,22 +6179,22 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C240" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D240" t="n">
-        <v>794671</v>
+        <v>30791</v>
       </c>
       <c r="E240" t="n">
-        <v>3481.16</v>
+        <v>8002.71</v>
       </c>
       <c r="F240" t="n">
         <v>0</v>
@@ -6215,13 +6215,13 @@
         <v>46247</v>
       </c>
       <c r="D241" t="n">
-        <v>30791</v>
+        <v>47252</v>
       </c>
       <c r="E241" t="n">
-        <v>8002.71</v>
+        <v>25003.88</v>
       </c>
       <c r="F241" t="n">
-        <v>0</v>
+        <v>1336.57</v>
       </c>
     </row>
     <row r="242">
@@ -6239,13 +6239,13 @@
         <v>46247</v>
       </c>
       <c r="D242" t="n">
-        <v>47252</v>
+        <v>789525</v>
       </c>
       <c r="E242" t="n">
-        <v>24906.33</v>
+        <v>1515.92</v>
       </c>
       <c r="F242" t="n">
-        <v>59.23</v>
+        <v>733.89</v>
       </c>
     </row>
     <row r="243">
@@ -6256,20 +6256,20 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="C243" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D243" t="n">
-        <v>789525</v>
+        <v>30307</v>
       </c>
       <c r="E243" t="n">
-        <v>1452</v>
+        <v>575.88</v>
       </c>
       <c r="F243" t="n">
-        <v>201.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="244">
@@ -6287,10 +6287,10 @@
         <v>46247</v>
       </c>
       <c r="D244" t="n">
-        <v>30307</v>
+        <v>30791</v>
       </c>
       <c r="E244" t="n">
-        <v>575.88</v>
+        <v>44.88</v>
       </c>
       <c r="F244" t="n">
         <v>0</v>
@@ -6299,22 +6299,22 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C245" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D245" t="n">
-        <v>30791</v>
+        <v>790595</v>
       </c>
       <c r="E245" t="n">
-        <v>44.88</v>
+        <v>5219.13</v>
       </c>
       <c r="F245" t="n">
         <v>0</v>
@@ -6323,49 +6323,49 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C246" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D246" t="n">
-        <v>790595</v>
+        <v>47252</v>
       </c>
       <c r="E246" t="n">
-        <v>1151.94</v>
+        <v>28417.89</v>
       </c>
       <c r="F246" t="n">
-        <v>0</v>
+        <v>458.35</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C247" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D247" t="n">
-        <v>47252</v>
+        <v>789603</v>
       </c>
       <c r="E247" t="n">
-        <v>28417.89</v>
+        <v>25094.49</v>
       </c>
       <c r="F247" t="n">
-        <v>458.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="248">
@@ -6383,10 +6383,10 @@
         <v>46247</v>
       </c>
       <c r="D248" t="n">
-        <v>789603</v>
+        <v>795345</v>
       </c>
       <c r="E248" t="n">
-        <v>25094.49</v>
+        <v>5994.14</v>
       </c>
       <c r="F248" t="n">
         <v>0</v>
@@ -6395,97 +6395,97 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C249" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D249" t="n">
-        <v>795345</v>
+        <v>789603</v>
       </c>
       <c r="E249" t="n">
-        <v>5994.14</v>
+        <v>70204.08</v>
       </c>
       <c r="F249" t="n">
-        <v>0</v>
+        <v>41155.22</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C250" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D250" t="n">
-        <v>789603</v>
+        <v>31267</v>
       </c>
       <c r="E250" t="n">
-        <v>70204.08</v>
+        <v>26.27</v>
       </c>
       <c r="F250" t="n">
-        <v>41155.22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C251" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D251" t="n">
-        <v>31267</v>
+        <v>793186</v>
       </c>
       <c r="E251" t="n">
-        <v>26.27</v>
+        <v>443.79</v>
       </c>
       <c r="F251" t="n">
-        <v>0</v>
+        <v>54.71</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C252" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D252" t="n">
-        <v>793186</v>
+        <v>30307</v>
       </c>
       <c r="E252" t="n">
-        <v>443.79</v>
+        <v>11243.49</v>
       </c>
       <c r="F252" t="n">
-        <v>54.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="253">
@@ -6503,10 +6503,10 @@
         <v>46247</v>
       </c>
       <c r="D253" t="n">
-        <v>30307</v>
+        <v>794671</v>
       </c>
       <c r="E253" t="n">
-        <v>9712.51</v>
+        <v>2664.9</v>
       </c>
       <c r="F253" t="n">
         <v>0</v>
@@ -6515,22 +6515,22 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C254" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D254" t="n">
-        <v>794671</v>
+        <v>790595</v>
       </c>
       <c r="E254" t="n">
-        <v>2664.9</v>
+        <v>1446.99</v>
       </c>
       <c r="F254" t="n">
         <v>0</v>
@@ -6544,17 +6544,17 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C255" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D255" t="n">
-        <v>790595</v>
+        <v>792141</v>
       </c>
       <c r="E255" t="n">
-        <v>1266.58</v>
+        <v>3019.8</v>
       </c>
       <c r="F255" t="n">
         <v>0</v>
@@ -6563,22 +6563,22 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C256" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D256" t="n">
-        <v>792141</v>
+        <v>793186</v>
       </c>
       <c r="E256" t="n">
-        <v>3019.8</v>
+        <v>146.11</v>
       </c>
       <c r="F256" t="n">
         <v>0</v>
@@ -6587,22 +6587,22 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C257" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D257" t="n">
-        <v>793186</v>
+        <v>792121</v>
       </c>
       <c r="E257" t="n">
-        <v>146.11</v>
+        <v>3708.27</v>
       </c>
       <c r="F257" t="n">
         <v>0</v>
@@ -6623,61 +6623,61 @@
         <v>46247</v>
       </c>
       <c r="D258" t="n">
-        <v>792121</v>
+        <v>30083</v>
       </c>
       <c r="E258" t="n">
-        <v>3285.89</v>
+        <v>4445.97</v>
       </c>
       <c r="F258" t="n">
-        <v>0</v>
+        <v>77.34</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C259" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D259" t="n">
-        <v>30083</v>
+        <v>139553</v>
       </c>
       <c r="E259" t="n">
-        <v>4445.97</v>
+        <v>7671.8</v>
       </c>
       <c r="F259" t="n">
-        <v>77.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C260" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D260" t="n">
-        <v>139553</v>
+        <v>33057</v>
       </c>
       <c r="E260" t="n">
-        <v>7671.8</v>
+        <v>12143.36</v>
       </c>
       <c r="F260" t="n">
-        <v>0</v>
+        <v>261.95</v>
       </c>
     </row>
     <row r="261">
@@ -6695,58 +6695,58 @@
         <v>46247</v>
       </c>
       <c r="D261" t="n">
-        <v>33057</v>
+        <v>33928</v>
       </c>
       <c r="E261" t="n">
-        <v>12143.36</v>
+        <v>2041.75</v>
       </c>
       <c r="F261" t="n">
-        <v>261.95</v>
+        <v>94.43000000000001</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C262" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D262" t="n">
-        <v>33928</v>
+        <v>792121</v>
       </c>
       <c r="E262" t="n">
-        <v>2041.75</v>
+        <v>501.32</v>
       </c>
       <c r="F262" t="n">
-        <v>94.43000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C263" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D263" t="n">
-        <v>792121</v>
+        <v>32816</v>
       </c>
       <c r="E263" t="n">
-        <v>501.32</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="F263" t="n">
         <v>0</v>
@@ -6755,22 +6755,22 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C264" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D264" t="n">
-        <v>32816</v>
+        <v>139553</v>
       </c>
       <c r="E264" t="n">
-        <v>74.84999999999999</v>
+        <v>2570.35</v>
       </c>
       <c r="F264" t="n">
         <v>0</v>
@@ -6779,22 +6779,22 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C265" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D265" t="n">
-        <v>139553</v>
+        <v>795345</v>
       </c>
       <c r="E265" t="n">
-        <v>2570.35</v>
+        <v>272.98</v>
       </c>
       <c r="F265" t="n">
         <v>0</v>
@@ -6803,22 +6803,22 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C266" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D266" t="n">
-        <v>795345</v>
+        <v>33286</v>
       </c>
       <c r="E266" t="n">
-        <v>272.98</v>
+        <v>118.15</v>
       </c>
       <c r="F266" t="n">
         <v>0</v>
@@ -6827,48 +6827,24 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C267" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D267" t="n">
-        <v>33286</v>
+        <v>795345</v>
       </c>
       <c r="E267" t="n">
-        <v>111.21</v>
+        <v>169.57</v>
       </c>
       <c r="F267" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B268" t="inlineStr">
-        <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
-        </is>
-      </c>
-      <c r="C268" s="2" t="n">
-        <v>46247</v>
-      </c>
-      <c r="D268" t="n">
-        <v>795345</v>
-      </c>
-      <c r="E268" t="n">
-        <v>169.57</v>
-      </c>
-      <c r="F268" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 16:15:04
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -482,7 +482,7 @@
         <v>790595</v>
       </c>
       <c r="E2" t="n">
-        <v>606.36</v>
+        <v>640.51</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -509,7 +509,7 @@
         <v>55808.85</v>
       </c>
       <c r="F3" t="n">
-        <v>9700.24</v>
+        <v>10027.07</v>
       </c>
     </row>
     <row r="4">
@@ -533,7 +533,7 @@
         <v>179.4</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>179.4</v>
       </c>
     </row>
     <row r="5">
@@ -554,7 +554,7 @@
         <v>33928</v>
       </c>
       <c r="E5" t="n">
-        <v>34449.64</v>
+        <v>34457.77</v>
       </c>
       <c r="F5" t="n">
         <v>37720.56</v>
@@ -650,7 +650,7 @@
         <v>31267</v>
       </c>
       <c r="E9" t="n">
-        <v>19039.74</v>
+        <v>19344.69</v>
       </c>
       <c r="F9" t="n">
         <v>2577.92</v>
@@ -698,7 +698,7 @@
         <v>33928</v>
       </c>
       <c r="E11" t="n">
-        <v>8505.620000000001</v>
+        <v>8651.73</v>
       </c>
       <c r="F11" t="n">
         <v>3486.49</v>
@@ -842,7 +842,7 @@
         <v>31267</v>
       </c>
       <c r="E17" t="n">
-        <v>1480.8</v>
+        <v>1497.58</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -914,7 +914,7 @@
         <v>792121</v>
       </c>
       <c r="E20" t="n">
-        <v>20614.04</v>
+        <v>22176.39</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -1010,7 +1010,7 @@
         <v>30307</v>
       </c>
       <c r="E24" t="n">
-        <v>57915.37</v>
+        <v>59348.73</v>
       </c>
       <c r="F24" t="n">
         <v>22829.12</v>
@@ -1109,28 +1109,28 @@
         <v>4652.14</v>
       </c>
       <c r="F28" t="n">
-        <v>100.39</v>
+        <v>414.47</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GERUSIA MARIA DA SILVA</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D29" t="n">
-        <v>789603</v>
+        <v>33057</v>
       </c>
       <c r="E29" t="n">
-        <v>15918.88</v>
+        <v>857.54</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -1139,22 +1139,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>GERUSIA MARIA DA SILVA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D30" t="n">
-        <v>33057</v>
+        <v>789603</v>
       </c>
       <c r="E30" t="n">
-        <v>1119.01</v>
+        <v>32819.04</v>
       </c>
       <c r="F30" t="n">
         <v>0</v>
@@ -1163,31 +1163,31 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D31" t="n">
-        <v>30791</v>
+        <v>33057</v>
       </c>
       <c r="E31" t="n">
-        <v>446.32</v>
+        <v>1119.01</v>
       </c>
       <c r="F31" t="n">
-        <v>71.06999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1199,13 +1199,13 @@
         <v>46247</v>
       </c>
       <c r="D32" t="n">
-        <v>792121</v>
+        <v>30791</v>
       </c>
       <c r="E32" t="n">
-        <v>803.5599999999999</v>
+        <v>446.32</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>71.06999999999999</v>
       </c>
     </row>
     <row r="33">
@@ -1223,10 +1223,10 @@
         <v>46247</v>
       </c>
       <c r="D33" t="n">
-        <v>789603</v>
+        <v>792121</v>
       </c>
       <c r="E33" t="n">
-        <v>2551.56</v>
+        <v>803.5599999999999</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
@@ -1235,22 +1235,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D34" t="n">
-        <v>794671</v>
+        <v>789603</v>
       </c>
       <c r="E34" t="n">
-        <v>4550.69</v>
+        <v>2551.56</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
@@ -1264,17 +1264,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D35" t="n">
-        <v>31267</v>
+        <v>794671</v>
       </c>
       <c r="E35" t="n">
-        <v>163874.12</v>
+        <v>4550.69</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
@@ -1283,22 +1283,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D36" t="n">
-        <v>30307</v>
+        <v>31267</v>
       </c>
       <c r="E36" t="n">
-        <v>5678.72</v>
+        <v>164863.92</v>
       </c>
       <c r="F36" t="n">
         <v>0</v>
@@ -1307,25 +1307,25 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D37" t="n">
-        <v>794671</v>
+        <v>30307</v>
       </c>
       <c r="E37" t="n">
-        <v>14872.77</v>
+        <v>5678.72</v>
       </c>
       <c r="F37" t="n">
-        <v>10885.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -1343,58 +1343,58 @@
         <v>46247</v>
       </c>
       <c r="D38" t="n">
-        <v>792246</v>
+        <v>794671</v>
       </c>
       <c r="E38" t="n">
-        <v>944.14</v>
+        <v>14872.77</v>
       </c>
       <c r="F38" t="n">
-        <v>145.36</v>
+        <v>10885.32</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D39" t="n">
-        <v>795345</v>
+        <v>792246</v>
       </c>
       <c r="E39" t="n">
-        <v>98.68000000000001</v>
+        <v>944.14</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>145.36</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D40" t="n">
-        <v>33057</v>
+        <v>795345</v>
       </c>
       <c r="E40" t="n">
-        <v>614.12</v>
+        <v>98.68000000000001</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
@@ -1418,7 +1418,7 @@
         <v>795345</v>
       </c>
       <c r="E41" t="n">
-        <v>34.41</v>
+        <v>67.95</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
@@ -1466,7 +1466,7 @@
         <v>789603</v>
       </c>
       <c r="E43" t="n">
-        <v>17645.28</v>
+        <v>18253.26</v>
       </c>
       <c r="F43" t="n">
         <v>595.26</v>
@@ -1514,7 +1514,7 @@
         <v>33286</v>
       </c>
       <c r="E45" t="n">
-        <v>1225.88</v>
+        <v>1226.18</v>
       </c>
       <c r="F45" t="n">
         <v>398.48</v>
@@ -1562,7 +1562,7 @@
         <v>31267</v>
       </c>
       <c r="E47" t="n">
-        <v>10497.07</v>
+        <v>16596.01</v>
       </c>
       <c r="F47" t="n">
         <v>1375.51</v>
@@ -1586,7 +1586,7 @@
         <v>30791</v>
       </c>
       <c r="E48" t="n">
-        <v>21675.78</v>
+        <v>23414.26</v>
       </c>
       <c r="F48" t="n">
         <v>6061.43</v>
@@ -1610,7 +1610,7 @@
         <v>793718</v>
       </c>
       <c r="E49" t="n">
-        <v>5038.1</v>
+        <v>5102.27</v>
       </c>
       <c r="F49" t="n">
         <v>361.54</v>
@@ -1658,7 +1658,7 @@
         <v>789228</v>
       </c>
       <c r="E51" t="n">
-        <v>4682.6</v>
+        <v>5018.63</v>
       </c>
       <c r="F51" t="n">
         <v>481.75</v>
@@ -1682,7 +1682,7 @@
         <v>47252</v>
       </c>
       <c r="E52" t="n">
-        <v>44810.73</v>
+        <v>46633.18</v>
       </c>
       <c r="F52" t="n">
         <v>2979.35</v>
@@ -1730,7 +1730,7 @@
         <v>33928</v>
       </c>
       <c r="E54" t="n">
-        <v>3210.3</v>
+        <v>3475.39</v>
       </c>
       <c r="F54" t="n">
         <v>25.2</v>
@@ -1970,10 +1970,10 @@
         <v>30307</v>
       </c>
       <c r="E64" t="n">
-        <v>53668.37</v>
+        <v>63289.51</v>
       </c>
       <c r="F64" t="n">
-        <v>6435.58</v>
+        <v>7071.46</v>
       </c>
     </row>
     <row r="65">
@@ -2042,7 +2042,7 @@
         <v>33286</v>
       </c>
       <c r="E67" t="n">
-        <v>3194.35</v>
+        <v>3333.65</v>
       </c>
       <c r="F67" t="n">
         <v>0</v>
@@ -2282,10 +2282,10 @@
         <v>30791</v>
       </c>
       <c r="E77" t="n">
-        <v>28173.35</v>
+        <v>31975.91</v>
       </c>
       <c r="F77" t="n">
-        <v>5742.91</v>
+        <v>5777.74</v>
       </c>
     </row>
     <row r="78">
@@ -2354,7 +2354,7 @@
         <v>33286</v>
       </c>
       <c r="E80" t="n">
-        <v>3012.3</v>
+        <v>3080.19</v>
       </c>
       <c r="F80" t="n">
         <v>1858</v>
@@ -2474,7 +2474,7 @@
         <v>31267</v>
       </c>
       <c r="E85" t="n">
-        <v>6092.44</v>
+        <v>6349.62</v>
       </c>
       <c r="F85" t="n">
         <v>117.01</v>
@@ -2690,7 +2690,7 @@
         <v>33057</v>
       </c>
       <c r="E94" t="n">
-        <v>6208</v>
+        <v>39.4</v>
       </c>
       <c r="F94" t="n">
         <v>0</v>
@@ -2714,7 +2714,7 @@
         <v>139553</v>
       </c>
       <c r="E95" t="n">
-        <v>6005.54</v>
+        <v>7470.64</v>
       </c>
       <c r="F95" t="n">
         <v>2004.68</v>
@@ -2738,10 +2738,10 @@
         <v>794671</v>
       </c>
       <c r="E96" t="n">
-        <v>9305.74</v>
+        <v>11347.59</v>
       </c>
       <c r="F96" t="n">
-        <v>3776.06</v>
+        <v>4308.67</v>
       </c>
     </row>
     <row r="97">
@@ -2765,28 +2765,28 @@
         <v>1852.36</v>
       </c>
       <c r="F97" t="n">
-        <v>0</v>
+        <v>369.52</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D98" t="n">
-        <v>139553</v>
+        <v>47252</v>
       </c>
       <c r="E98" t="n">
-        <v>747.4</v>
+        <v>9432.84</v>
       </c>
       <c r="F98" t="n">
         <v>0</v>
@@ -2795,25 +2795,25 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D99" t="n">
-        <v>789228</v>
+        <v>139553</v>
       </c>
       <c r="E99" t="n">
-        <v>199.03</v>
+        <v>2430.28</v>
       </c>
       <c r="F99" t="n">
-        <v>252.16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -2831,24 +2831,24 @@
         <v>46247</v>
       </c>
       <c r="D100" t="n">
-        <v>33057</v>
+        <v>789228</v>
       </c>
       <c r="E100" t="n">
-        <v>29.2</v>
+        <v>199.03</v>
       </c>
       <c r="F100" t="n">
-        <v>135.41</v>
+        <v>252.16</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -2858,93 +2858,93 @@
         <v>33057</v>
       </c>
       <c r="E101" t="n">
-        <v>3825.89</v>
+        <v>29.2</v>
       </c>
       <c r="F101" t="n">
-        <v>0</v>
+        <v>135.41</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D102" t="n">
-        <v>47252</v>
+        <v>33057</v>
       </c>
       <c r="E102" t="n">
-        <v>22759.98</v>
+        <v>3825.89</v>
       </c>
       <c r="F102" t="n">
-        <v>4814.96</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D103" t="n">
-        <v>139553</v>
+        <v>47252</v>
       </c>
       <c r="E103" t="n">
-        <v>134.76</v>
+        <v>29281.21</v>
       </c>
       <c r="F103" t="n">
-        <v>0</v>
+        <v>4814.96</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D104" t="n">
-        <v>792141</v>
+        <v>139553</v>
       </c>
       <c r="E104" t="n">
-        <v>0</v>
+        <v>134.76</v>
       </c>
       <c r="F104" t="n">
-        <v>11651.64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -2954,34 +2954,34 @@
         <v>792141</v>
       </c>
       <c r="E105" t="n">
-        <v>98.20999999999999</v>
+        <v>0</v>
       </c>
       <c r="F105" t="n">
-        <v>98.2</v>
+        <v>11651.64</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D106" t="n">
-        <v>47252</v>
+        <v>792141</v>
       </c>
       <c r="E106" t="n">
-        <v>9122.09</v>
+        <v>98.20999999999999</v>
       </c>
       <c r="F106" t="n">
-        <v>0</v>
+        <v>98.2</v>
       </c>
     </row>
     <row r="107">
@@ -3098,7 +3098,7 @@
         <v>30307</v>
       </c>
       <c r="E111" t="n">
-        <v>45723.49</v>
+        <v>47301.97</v>
       </c>
       <c r="F111" t="n">
         <v>91.92</v>
@@ -3122,7 +3122,7 @@
         <v>30083</v>
       </c>
       <c r="E112" t="n">
-        <v>3383.86</v>
+        <v>3499.72</v>
       </c>
       <c r="F112" t="n">
         <v>0</v>
@@ -3146,7 +3146,7 @@
         <v>789525</v>
       </c>
       <c r="E113" t="n">
-        <v>5054.8</v>
+        <v>5830.6</v>
       </c>
       <c r="F113" t="n">
         <v>3468.04</v>
@@ -3170,7 +3170,7 @@
         <v>789228</v>
       </c>
       <c r="E114" t="n">
-        <v>481.83</v>
+        <v>507.05</v>
       </c>
       <c r="F114" t="n">
         <v>325.96</v>
@@ -3290,7 +3290,7 @@
         <v>795345</v>
       </c>
       <c r="E119" t="n">
-        <v>1950.71</v>
+        <v>2605.91</v>
       </c>
       <c r="F119" t="n">
         <v>0</v>
@@ -3314,7 +3314,7 @@
         <v>33928</v>
       </c>
       <c r="E120" t="n">
-        <v>38490.97</v>
+        <v>38968.93</v>
       </c>
       <c r="F120" t="n">
         <v>7783.3</v>
@@ -3458,7 +3458,7 @@
         <v>789603</v>
       </c>
       <c r="E126" t="n">
-        <v>38615.94</v>
+        <v>43432.98</v>
       </c>
       <c r="F126" t="n">
         <v>0</v>
@@ -3506,7 +3506,7 @@
         <v>30307</v>
       </c>
       <c r="E128" t="n">
-        <v>37548.6</v>
+        <v>43671.97</v>
       </c>
       <c r="F128" t="n">
         <v>8750.959999999999</v>
@@ -3515,79 +3515,79 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C129" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D129" t="n">
-        <v>792121</v>
+        <v>789603</v>
       </c>
       <c r="E129" t="n">
-        <v>2105.83</v>
+        <v>63275.09</v>
       </c>
       <c r="F129" t="n">
-        <v>856.61</v>
+        <v>2492.32</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D130" t="n">
-        <v>793718</v>
+        <v>792121</v>
       </c>
       <c r="E130" t="n">
-        <v>225.33</v>
+        <v>2105.83</v>
       </c>
       <c r="F130" t="n">
-        <v>97.97</v>
+        <v>856.61</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D131" t="n">
-        <v>33286</v>
+        <v>33928</v>
       </c>
       <c r="E131" t="n">
-        <v>0</v>
+        <v>1686.17</v>
       </c>
       <c r="F131" t="n">
-        <v>123.51</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3599,82 +3599,82 @@
         <v>46247</v>
       </c>
       <c r="D132" t="n">
-        <v>30307</v>
+        <v>793718</v>
       </c>
       <c r="E132" t="n">
-        <v>3934.22</v>
+        <v>225.33</v>
       </c>
       <c r="F132" t="n">
-        <v>311.88</v>
+        <v>97.97</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D133" t="n">
-        <v>33928</v>
+        <v>33286</v>
       </c>
       <c r="E133" t="n">
-        <v>1829.92</v>
+        <v>0</v>
       </c>
       <c r="F133" t="n">
-        <v>0</v>
+        <v>123.51</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D134" t="n">
-        <v>793718</v>
+        <v>30307</v>
       </c>
       <c r="E134" t="n">
-        <v>1231.84</v>
+        <v>3934.22</v>
       </c>
       <c r="F134" t="n">
-        <v>0</v>
+        <v>311.88</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D135" t="n">
-        <v>33286</v>
+        <v>33928</v>
       </c>
       <c r="E135" t="n">
-        <v>2174.73</v>
+        <v>1922.77</v>
       </c>
       <c r="F135" t="n">
         <v>0</v>
@@ -3683,22 +3683,22 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D136" t="n">
-        <v>794029</v>
+        <v>793718</v>
       </c>
       <c r="E136" t="n">
-        <v>731.21</v>
+        <v>1231.84</v>
       </c>
       <c r="F136" t="n">
         <v>0</v>
@@ -3712,17 +3712,17 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D137" t="n">
-        <v>792246</v>
+        <v>33286</v>
       </c>
       <c r="E137" t="n">
-        <v>1255.6</v>
+        <v>2263.98</v>
       </c>
       <c r="F137" t="n">
         <v>0</v>
@@ -3731,49 +3731,49 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D138" t="n">
-        <v>789603</v>
+        <v>31267</v>
       </c>
       <c r="E138" t="n">
-        <v>33938.2</v>
+        <v>2682.29</v>
       </c>
       <c r="F138" t="n">
-        <v>2492.32</v>
+        <v>58.7</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D139" t="n">
-        <v>31267</v>
+        <v>794029</v>
       </c>
       <c r="E139" t="n">
-        <v>1786.62</v>
+        <v>731.21</v>
       </c>
       <c r="F139" t="n">
-        <v>58.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140">
@@ -3784,17 +3784,17 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D140" t="n">
-        <v>794671</v>
+        <v>792246</v>
       </c>
       <c r="E140" t="n">
-        <v>1210.5</v>
+        <v>1255.6</v>
       </c>
       <c r="F140" t="n">
         <v>0</v>
@@ -3803,22 +3803,22 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D141" t="n">
-        <v>33928</v>
+        <v>794671</v>
       </c>
       <c r="E141" t="n">
-        <v>1603.91</v>
+        <v>1210.5</v>
       </c>
       <c r="F141" t="n">
         <v>0</v>
@@ -3917,7 +3917,7 @@
         <v>173.79</v>
       </c>
       <c r="F145" t="n">
-        <v>0</v>
+        <v>173.8</v>
       </c>
     </row>
     <row r="146">
@@ -3986,7 +3986,7 @@
         <v>47252</v>
       </c>
       <c r="E148" t="n">
-        <v>28358.31</v>
+        <v>29625.99</v>
       </c>
       <c r="F148" t="n">
         <v>5590.24</v>
@@ -4010,7 +4010,7 @@
         <v>47252</v>
       </c>
       <c r="E149" t="n">
-        <v>39090.34</v>
+        <v>39322.42</v>
       </c>
       <c r="F149" t="n">
         <v>10035.59</v>
@@ -4226,7 +4226,7 @@
         <v>33286</v>
       </c>
       <c r="E158" t="n">
-        <v>12430.95</v>
+        <v>14129.06</v>
       </c>
       <c r="F158" t="n">
         <v>1286.75</v>
@@ -4418,7 +4418,7 @@
         <v>794029</v>
       </c>
       <c r="E166" t="n">
-        <v>10957.42</v>
+        <v>11301.04</v>
       </c>
       <c r="F166" t="n">
         <v>0</v>
@@ -4466,7 +4466,7 @@
         <v>47252</v>
       </c>
       <c r="E168" t="n">
-        <v>5602.09</v>
+        <v>291.52</v>
       </c>
       <c r="F168" t="n">
         <v>0</v>
@@ -4514,7 +4514,7 @@
         <v>32816</v>
       </c>
       <c r="E170" t="n">
-        <v>2141.54</v>
+        <v>2285.18</v>
       </c>
       <c r="F170" t="n">
         <v>950.1799999999999</v>
@@ -4538,7 +4538,7 @@
         <v>31267</v>
       </c>
       <c r="E171" t="n">
-        <v>168431.98</v>
+        <v>168791.91</v>
       </c>
       <c r="F171" t="n">
         <v>0</v>
@@ -4658,7 +4658,7 @@
         <v>139553</v>
       </c>
       <c r="E176" t="n">
-        <v>4172.52</v>
+        <v>4710.72</v>
       </c>
       <c r="F176" t="n">
         <v>0</v>
@@ -4802,7 +4802,7 @@
         <v>30307</v>
       </c>
       <c r="E182" t="n">
-        <v>7318.22</v>
+        <v>8056.14</v>
       </c>
       <c r="F182" t="n">
         <v>0</v>
@@ -4874,7 +4874,7 @@
         <v>789603</v>
       </c>
       <c r="E185" t="n">
-        <v>10914.92</v>
+        <v>11733.88</v>
       </c>
       <c r="F185" t="n">
         <v>0</v>
@@ -5042,10 +5042,10 @@
         <v>793718</v>
       </c>
       <c r="E192" t="n">
-        <v>3795.63</v>
+        <v>3796.25</v>
       </c>
       <c r="F192" t="n">
-        <v>0</v>
+        <v>509.55</v>
       </c>
     </row>
     <row r="193">
@@ -5066,7 +5066,7 @@
         <v>789228</v>
       </c>
       <c r="E193" t="n">
-        <v>2156.56</v>
+        <v>2591.26</v>
       </c>
       <c r="F193" t="n">
         <v>0</v>
@@ -5234,7 +5234,7 @@
         <v>30307</v>
       </c>
       <c r="E200" t="n">
-        <v>99765.16</v>
+        <v>100524.52</v>
       </c>
       <c r="F200" t="n">
         <v>0</v>
@@ -5429,7 +5429,7 @@
         <v>28115.49</v>
       </c>
       <c r="F208" t="n">
-        <v>5443.93</v>
+        <v>5524.52</v>
       </c>
     </row>
     <row r="209">
@@ -5474,7 +5474,7 @@
         <v>789228</v>
       </c>
       <c r="E210" t="n">
-        <v>5970.16</v>
+        <v>5818.2</v>
       </c>
       <c r="F210" t="n">
         <v>434.79</v>
@@ -5594,7 +5594,7 @@
         <v>30791</v>
       </c>
       <c r="E215" t="n">
-        <v>24773.42</v>
+        <v>25723.97</v>
       </c>
       <c r="F215" t="n">
         <v>3868.53</v>
@@ -5882,10 +5882,10 @@
         <v>139553</v>
       </c>
       <c r="E227" t="n">
-        <v>12006.92</v>
+        <v>14554.92</v>
       </c>
       <c r="F227" t="n">
-        <v>6196.04</v>
+        <v>6735.08</v>
       </c>
     </row>
     <row r="228">
@@ -5978,7 +5978,7 @@
         <v>47252</v>
       </c>
       <c r="E231" t="n">
-        <v>26469.1</v>
+        <v>26558.36</v>
       </c>
       <c r="F231" t="n">
         <v>0</v>
@@ -6074,7 +6074,7 @@
         <v>793186</v>
       </c>
       <c r="E235" t="n">
-        <v>19013.01</v>
+        <v>20047.43</v>
       </c>
       <c r="F235" t="n">
         <v>702.38</v>
@@ -6194,7 +6194,7 @@
         <v>30307</v>
       </c>
       <c r="E240" t="n">
-        <v>150905.83</v>
+        <v>181874.61</v>
       </c>
       <c r="F240" t="n">
         <v>0</v>
@@ -6218,7 +6218,7 @@
         <v>30083</v>
       </c>
       <c r="E241" t="n">
-        <v>5716.11</v>
+        <v>5736.3</v>
       </c>
       <c r="F241" t="n">
         <v>0</v>
@@ -6266,7 +6266,7 @@
         <v>789661</v>
       </c>
       <c r="E243" t="n">
-        <v>434.06</v>
+        <v>3266.69</v>
       </c>
       <c r="F243" t="n">
         <v>32.2</v>
@@ -6482,7 +6482,7 @@
         <v>794671</v>
       </c>
       <c r="E252" t="n">
-        <v>8819.209999999999</v>
+        <v>14412.68</v>
       </c>
       <c r="F252" t="n">
         <v>0</v>
@@ -6578,7 +6578,7 @@
         <v>789525</v>
       </c>
       <c r="E256" t="n">
-        <v>8332.51</v>
+        <v>9252.559999999999</v>
       </c>
       <c r="F256" t="n">
         <v>1560.16</v>
@@ -6602,7 +6602,7 @@
         <v>33057</v>
       </c>
       <c r="E257" t="n">
-        <v>6154.31</v>
+        <v>6696.38</v>
       </c>
       <c r="F257" t="n">
         <v>1294.69</v>
@@ -6626,7 +6626,7 @@
         <v>47252</v>
       </c>
       <c r="E258" t="n">
-        <v>26414.87</v>
+        <v>28598.19</v>
       </c>
       <c r="F258" t="n">
         <v>2156.1</v>
@@ -6650,7 +6650,7 @@
         <v>789525</v>
       </c>
       <c r="E259" t="n">
-        <v>2754.1</v>
+        <v>2842.91</v>
       </c>
       <c r="F259" t="n">
         <v>733.89</v>
@@ -6674,7 +6674,7 @@
         <v>30791</v>
       </c>
       <c r="E260" t="n">
-        <v>8380.6</v>
+        <v>9619.120000000001</v>
       </c>
       <c r="F260" t="n">
         <v>0</v>
@@ -6842,7 +6842,7 @@
         <v>789603</v>
       </c>
       <c r="E267" t="n">
-        <v>81135.2</v>
+        <v>81198.32000000001</v>
       </c>
       <c r="F267" t="n">
         <v>41155.22</v>
@@ -6986,7 +6986,7 @@
         <v>792141</v>
       </c>
       <c r="E273" t="n">
-        <v>4147.46</v>
+        <v>4245.96</v>
       </c>
       <c r="F273" t="n">
         <v>0</v>
@@ -7106,7 +7106,7 @@
         <v>33928</v>
       </c>
       <c r="E278" t="n">
-        <v>3859.85</v>
+        <v>3907.58</v>
       </c>
       <c r="F278" t="n">
         <v>94.43000000000001</v>
@@ -7130,7 +7130,7 @@
         <v>33057</v>
       </c>
       <c r="E279" t="n">
-        <v>15750.39</v>
+        <v>21918.99</v>
       </c>
       <c r="F279" t="n">
         <v>261.95</v>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 16:45:04
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F289"/>
+  <dimension ref="A1:F290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,68 +472,68 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D2" t="n">
-        <v>790595</v>
+        <v>792121</v>
       </c>
       <c r="E2" t="n">
-        <v>640.51</v>
+        <v>22588.18</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>5420.8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D3" t="n">
-        <v>47252</v>
+        <v>789603</v>
       </c>
       <c r="E3" t="n">
-        <v>55808.85</v>
+        <v>50664.26</v>
       </c>
       <c r="F3" t="n">
-        <v>10027.07</v>
+        <v>4817.96</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D4" t="n">
-        <v>139553</v>
+        <v>790595</v>
       </c>
       <c r="E4" t="n">
-        <v>179.4</v>
+        <v>640.51</v>
       </c>
       <c r="F4" t="n">
-        <v>179.4</v>
+        <v>606.36</v>
       </c>
     </row>
     <row r="5">
@@ -551,19 +551,19 @@
         <v>46247</v>
       </c>
       <c r="D5" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="E5" t="n">
-        <v>34457.77</v>
+        <v>62386.96</v>
       </c>
       <c r="F5" t="n">
-        <v>37720.56</v>
+        <v>12850.83</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -575,13 +575,13 @@
         <v>46247</v>
       </c>
       <c r="D6" t="n">
-        <v>795345</v>
+        <v>33928</v>
       </c>
       <c r="E6" t="n">
-        <v>2580.96</v>
+        <v>34608.89</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>38246.94</v>
       </c>
     </row>
     <row r="7">
@@ -592,44 +592,44 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D7" t="n">
-        <v>789228</v>
+        <v>139553</v>
       </c>
       <c r="E7" t="n">
-        <v>4522.32</v>
+        <v>179.4</v>
       </c>
       <c r="F7" t="n">
-        <v>1664.41</v>
+        <v>179.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D8" t="n">
-        <v>33928</v>
+        <v>795345</v>
       </c>
       <c r="E8" t="n">
-        <v>9265.870000000001</v>
+        <v>2780.38</v>
       </c>
       <c r="F8" t="n">
-        <v>3365.06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -647,13 +647,13 @@
         <v>46247</v>
       </c>
       <c r="D9" t="n">
-        <v>30791</v>
+        <v>789228</v>
       </c>
       <c r="E9" t="n">
-        <v>23915.32</v>
+        <v>4522.32</v>
       </c>
       <c r="F9" t="n">
-        <v>10134.07</v>
+        <v>1664.41</v>
       </c>
     </row>
     <row r="10">
@@ -664,20 +664,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D10" t="n">
-        <v>31267</v>
+        <v>30791</v>
       </c>
       <c r="E10" t="n">
-        <v>19344.69</v>
+        <v>24060.05</v>
       </c>
       <c r="F10" t="n">
-        <v>2577.92</v>
+        <v>10134.07</v>
       </c>
     </row>
     <row r="11">
@@ -688,20 +688,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D11" t="n">
-        <v>789525</v>
+        <v>33928</v>
       </c>
       <c r="E11" t="n">
-        <v>2757.85</v>
+        <v>9600.059999999999</v>
       </c>
       <c r="F11" t="n">
-        <v>1242.4</v>
+        <v>3365.06</v>
       </c>
     </row>
     <row r="12">
@@ -719,13 +719,13 @@
         <v>46247</v>
       </c>
       <c r="D12" t="n">
-        <v>33928</v>
+        <v>31267</v>
       </c>
       <c r="E12" t="n">
-        <v>8742.16</v>
+        <v>19344.91</v>
       </c>
       <c r="F12" t="n">
-        <v>3486.49</v>
+        <v>2796.39</v>
       </c>
     </row>
     <row r="13">
@@ -736,20 +736,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D13" t="n">
-        <v>793186</v>
+        <v>33928</v>
       </c>
       <c r="E13" t="n">
-        <v>2521.05</v>
+        <v>8996.83</v>
       </c>
       <c r="F13" t="n">
-        <v>749.47</v>
+        <v>4355.99</v>
       </c>
     </row>
     <row r="14">
@@ -760,65 +760,65 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D14" t="n">
-        <v>792141</v>
+        <v>789525</v>
       </c>
       <c r="E14" t="n">
-        <v>3052.3</v>
+        <v>3361.79</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>1518.62</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D15" t="n">
-        <v>30083</v>
+        <v>793186</v>
       </c>
       <c r="E15" t="n">
-        <v>94.87</v>
+        <v>2521.22</v>
       </c>
       <c r="F15" t="n">
-        <v>94.87</v>
+        <v>837.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D16" t="n">
-        <v>33286</v>
+        <v>792141</v>
       </c>
       <c r="E16" t="n">
-        <v>111.39</v>
+        <v>3052.3</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -832,20 +832,20 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D17" t="n">
-        <v>794671</v>
+        <v>30083</v>
       </c>
       <c r="E17" t="n">
-        <v>9333.74</v>
+        <v>94.87</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>94.87</v>
       </c>
     </row>
     <row r="18">
@@ -856,17 +856,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D18" t="n">
-        <v>31267</v>
+        <v>33286</v>
       </c>
       <c r="E18" t="n">
-        <v>1497.58</v>
+        <v>111.39</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -875,121 +875,121 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D19" t="n">
-        <v>789228</v>
+        <v>794671</v>
       </c>
       <c r="E19" t="n">
-        <v>2898.42</v>
+        <v>9333.74</v>
       </c>
       <c r="F19" t="n">
-        <v>17.47</v>
+        <v>1322.38</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D20" t="n">
-        <v>792121</v>
+        <v>31267</v>
       </c>
       <c r="E20" t="n">
-        <v>22176.39</v>
+        <v>2036.89</v>
       </c>
       <c r="F20" t="n">
-        <v>945.14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D21" t="n">
-        <v>30083</v>
+        <v>33057</v>
       </c>
       <c r="E21" t="n">
-        <v>8854.66</v>
+        <v>1845.44</v>
       </c>
       <c r="F21" t="n">
-        <v>500.64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D22" t="n">
-        <v>789603</v>
+        <v>789228</v>
       </c>
       <c r="E22" t="n">
-        <v>66139.75999999999</v>
+        <v>2909.83</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>17.47</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D23" t="n">
-        <v>795345</v>
+        <v>30083</v>
       </c>
       <c r="E23" t="n">
-        <v>2236.31</v>
+        <v>8854.66</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>3904.57</v>
       </c>
     </row>
     <row r="24">
@@ -1010,7 +1010,7 @@
         <v>30307</v>
       </c>
       <c r="E24" t="n">
-        <v>60429.93</v>
+        <v>63924.65</v>
       </c>
       <c r="F24" t="n">
         <v>22829.12</v>
@@ -1019,22 +1019,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D25" t="n">
-        <v>139553</v>
+        <v>795345</v>
       </c>
       <c r="E25" t="n">
-        <v>203.96</v>
+        <v>2236.31</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -1043,22 +1043,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D26" t="n">
-        <v>30083</v>
+        <v>139553</v>
       </c>
       <c r="E26" t="n">
-        <v>1860.43</v>
+        <v>203.96</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -1079,10 +1079,10 @@
         <v>46247</v>
       </c>
       <c r="D27" t="n">
-        <v>139553</v>
+        <v>30083</v>
       </c>
       <c r="E27" t="n">
-        <v>11466.64</v>
+        <v>1860.43</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -1091,70 +1091,70 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D28" t="n">
-        <v>30083</v>
+        <v>139553</v>
       </c>
       <c r="E28" t="n">
-        <v>4652.14</v>
+        <v>11466.64</v>
       </c>
       <c r="F28" t="n">
-        <v>414.47</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D29" t="n">
-        <v>33057</v>
+        <v>30083</v>
       </c>
       <c r="E29" t="n">
-        <v>857.54</v>
+        <v>4652.14</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>414.47</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>GERUSIA MARIA DA SILVA</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D30" t="n">
-        <v>789603</v>
+        <v>33057</v>
       </c>
       <c r="E30" t="n">
-        <v>32819.04</v>
+        <v>877.29</v>
       </c>
       <c r="F30" t="n">
         <v>0</v>
@@ -1163,22 +1163,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>GERUSIA MARIA DA SILVA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D31" t="n">
-        <v>33057</v>
+        <v>789603</v>
       </c>
       <c r="E31" t="n">
-        <v>1119.01</v>
+        <v>32819.04</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
@@ -1205,7 +1205,7 @@
         <v>446.32</v>
       </c>
       <c r="F32" t="n">
-        <v>71.06999999999999</v>
+        <v>99.58</v>
       </c>
     </row>
     <row r="33">
@@ -1229,7 +1229,7 @@
         <v>803.5599999999999</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>394.84</v>
       </c>
     </row>
     <row r="34">
@@ -1298,7 +1298,7 @@
         <v>31267</v>
       </c>
       <c r="E36" t="n">
-        <v>165223.85</v>
+        <v>168523.19</v>
       </c>
       <c r="F36" t="n">
         <v>0</v>
@@ -1373,7 +1373,7 @@
         <v>944.14</v>
       </c>
       <c r="F39" t="n">
-        <v>145.36</v>
+        <v>518.28</v>
       </c>
     </row>
     <row r="40">
@@ -1469,7 +1469,7 @@
         <v>23801.04</v>
       </c>
       <c r="F43" t="n">
-        <v>595.26</v>
+        <v>2100.06</v>
       </c>
     </row>
     <row r="44">
@@ -1490,10 +1490,10 @@
         <v>139553</v>
       </c>
       <c r="E44" t="n">
-        <v>4614.5</v>
+        <v>8619.139999999999</v>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>2157.18</v>
       </c>
     </row>
     <row r="45">
@@ -1514,10 +1514,10 @@
         <v>33286</v>
       </c>
       <c r="E45" t="n">
-        <v>1226.18</v>
+        <v>1226.56</v>
       </c>
       <c r="F45" t="n">
-        <v>398.48</v>
+        <v>672.15</v>
       </c>
     </row>
     <row r="46">
@@ -1538,7 +1538,7 @@
         <v>792121</v>
       </c>
       <c r="E46" t="n">
-        <v>3394.79</v>
+        <v>3892.44</v>
       </c>
       <c r="F46" t="n">
         <v>0</v>
@@ -1562,10 +1562,10 @@
         <v>33057</v>
       </c>
       <c r="E47" t="n">
-        <v>4421.77</v>
+        <v>4422.36</v>
       </c>
       <c r="F47" t="n">
-        <v>756.33</v>
+        <v>1456.38</v>
       </c>
     </row>
     <row r="48">
@@ -1586,7 +1586,7 @@
         <v>31267</v>
       </c>
       <c r="E48" t="n">
-        <v>16650.52</v>
+        <v>18020.2</v>
       </c>
       <c r="F48" t="n">
         <v>1375.51</v>
@@ -1607,13 +1607,13 @@
         <v>46247</v>
       </c>
       <c r="D49" t="n">
-        <v>30791</v>
+        <v>793718</v>
       </c>
       <c r="E49" t="n">
-        <v>23143</v>
+        <v>5184.61</v>
       </c>
       <c r="F49" t="n">
-        <v>6061.43</v>
+        <v>999.79</v>
       </c>
     </row>
     <row r="50">
@@ -1631,13 +1631,13 @@
         <v>46247</v>
       </c>
       <c r="D50" t="n">
-        <v>793718</v>
+        <v>30791</v>
       </c>
       <c r="E50" t="n">
-        <v>5102.27</v>
+        <v>23196.57</v>
       </c>
       <c r="F50" t="n">
-        <v>361.54</v>
+        <v>7595.98</v>
       </c>
     </row>
     <row r="51">
@@ -1679,13 +1679,13 @@
         <v>46247</v>
       </c>
       <c r="D52" t="n">
-        <v>789228</v>
+        <v>47252</v>
       </c>
       <c r="E52" t="n">
-        <v>5018.72</v>
+        <v>52053.43</v>
       </c>
       <c r="F52" t="n">
-        <v>802.05</v>
+        <v>8243.6</v>
       </c>
     </row>
     <row r="53">
@@ -1703,13 +1703,13 @@
         <v>46247</v>
       </c>
       <c r="D53" t="n">
-        <v>47252</v>
+        <v>789228</v>
       </c>
       <c r="E53" t="n">
-        <v>46983.07</v>
+        <v>5034.99</v>
       </c>
       <c r="F53" t="n">
-        <v>8243.6</v>
+        <v>802.05</v>
       </c>
     </row>
     <row r="54">
@@ -1754,7 +1754,7 @@
         <v>33928</v>
       </c>
       <c r="E55" t="n">
-        <v>5099.24</v>
+        <v>5828.17</v>
       </c>
       <c r="F55" t="n">
         <v>25.2</v>
@@ -1778,7 +1778,7 @@
         <v>789525</v>
       </c>
       <c r="E56" t="n">
-        <v>1843.36</v>
+        <v>1884</v>
       </c>
       <c r="F56" t="n">
         <v>524.09</v>
@@ -1874,7 +1874,7 @@
         <v>30307</v>
       </c>
       <c r="E60" t="n">
-        <v>18943.36</v>
+        <v>15993.25</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
@@ -1919,13 +1919,13 @@
         <v>46247</v>
       </c>
       <c r="D62" t="n">
-        <v>792121</v>
+        <v>789603</v>
       </c>
       <c r="E62" t="n">
-        <v>6517.98</v>
+        <v>28981.91</v>
       </c>
       <c r="F62" t="n">
-        <v>0</v>
+        <v>4547.77</v>
       </c>
     </row>
     <row r="63">
@@ -1943,13 +1943,13 @@
         <v>46247</v>
       </c>
       <c r="D63" t="n">
-        <v>789603</v>
+        <v>792121</v>
       </c>
       <c r="E63" t="n">
-        <v>28510.46</v>
+        <v>6517.98</v>
       </c>
       <c r="F63" t="n">
-        <v>4547.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -1994,10 +1994,10 @@
         <v>30307</v>
       </c>
       <c r="E65" t="n">
-        <v>69319.28999999999</v>
+        <v>76264.75</v>
       </c>
       <c r="F65" t="n">
-        <v>8579.02</v>
+        <v>8672.540000000001</v>
       </c>
     </row>
     <row r="66">
@@ -2042,7 +2042,7 @@
         <v>32816</v>
       </c>
       <c r="E67" t="n">
-        <v>906.71</v>
+        <v>1146.21</v>
       </c>
       <c r="F67" t="n">
         <v>906.72</v>
@@ -2066,7 +2066,7 @@
         <v>33286</v>
       </c>
       <c r="E68" t="n">
-        <v>3380.77</v>
+        <v>3776.2</v>
       </c>
       <c r="F68" t="n">
         <v>0</v>
@@ -2189,7 +2189,7 @@
         <v>83.19</v>
       </c>
       <c r="F73" t="n">
-        <v>0</v>
+        <v>83.19</v>
       </c>
     </row>
     <row r="74">
@@ -2306,10 +2306,10 @@
         <v>30791</v>
       </c>
       <c r="E78" t="n">
-        <v>31975.91</v>
+        <v>32146.03</v>
       </c>
       <c r="F78" t="n">
-        <v>5777.74</v>
+        <v>8718.98</v>
       </c>
     </row>
     <row r="79">
@@ -2330,7 +2330,7 @@
         <v>33286</v>
       </c>
       <c r="E79" t="n">
-        <v>1585.96</v>
+        <v>1676.12</v>
       </c>
       <c r="F79" t="n">
         <v>837.88</v>
@@ -2378,10 +2378,10 @@
         <v>33286</v>
       </c>
       <c r="E81" t="n">
-        <v>3080.19</v>
+        <v>3249.47</v>
       </c>
       <c r="F81" t="n">
-        <v>1858</v>
+        <v>1910.02</v>
       </c>
     </row>
     <row r="82">
@@ -2399,13 +2399,13 @@
         <v>46247</v>
       </c>
       <c r="D82" t="n">
-        <v>793186</v>
+        <v>47252</v>
       </c>
       <c r="E82" t="n">
-        <v>57.99</v>
+        <v>26.36</v>
       </c>
       <c r="F82" t="n">
-        <v>0</v>
+        <v>23.09</v>
       </c>
     </row>
     <row r="83">
@@ -2423,13 +2423,13 @@
         <v>46247</v>
       </c>
       <c r="D83" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="E83" t="n">
-        <v>26.36</v>
+        <v>57.99</v>
       </c>
       <c r="F83" t="n">
-        <v>23.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -2546,10 +2546,10 @@
         <v>33057</v>
       </c>
       <c r="E88" t="n">
-        <v>390.14</v>
+        <v>390.3</v>
       </c>
       <c r="F88" t="n">
-        <v>199.94</v>
+        <v>419.7</v>
       </c>
     </row>
     <row r="89">
@@ -2594,7 +2594,7 @@
         <v>33286</v>
       </c>
       <c r="E90" t="n">
-        <v>3197.62</v>
+        <v>3596.96</v>
       </c>
       <c r="F90" t="n">
         <v>0</v>
@@ -2608,20 +2608,20 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D91" t="n">
-        <v>793718</v>
+        <v>139553</v>
       </c>
       <c r="E91" t="n">
-        <v>375.18</v>
+        <v>3634.34</v>
       </c>
       <c r="F91" t="n">
-        <v>48.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -2639,48 +2639,48 @@
         <v>46247</v>
       </c>
       <c r="D92" t="n">
-        <v>33928</v>
+        <v>793718</v>
       </c>
       <c r="E92" t="n">
-        <v>2416.47</v>
+        <v>407.17</v>
       </c>
       <c r="F92" t="n">
-        <v>244.93</v>
+        <v>48.08</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D93" t="n">
-        <v>139553</v>
+        <v>33928</v>
       </c>
       <c r="E93" t="n">
-        <v>611.88</v>
+        <v>2699.78</v>
       </c>
       <c r="F93" t="n">
-        <v>0</v>
+        <v>244.93</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -2690,82 +2690,82 @@
         <v>139553</v>
       </c>
       <c r="E94" t="n">
-        <v>4462.08</v>
+        <v>611.88</v>
       </c>
       <c r="F94" t="n">
-        <v>4462.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D95" t="n">
-        <v>33057</v>
+        <v>139553</v>
       </c>
       <c r="E95" t="n">
-        <v>39.4</v>
+        <v>5717.04</v>
       </c>
       <c r="F95" t="n">
-        <v>0</v>
+        <v>4462.08</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D96" t="n">
-        <v>139553</v>
+        <v>33057</v>
       </c>
       <c r="E96" t="n">
-        <v>10400.98</v>
+        <v>39.4</v>
       </c>
       <c r="F96" t="n">
-        <v>2440.95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D97" t="n">
-        <v>794671</v>
+        <v>139553</v>
       </c>
       <c r="E97" t="n">
-        <v>11786.46</v>
+        <v>14344.48</v>
       </c>
       <c r="F97" t="n">
-        <v>5772.38</v>
+        <v>2440.95</v>
       </c>
     </row>
     <row r="98">
@@ -2783,58 +2783,58 @@
         <v>46247</v>
       </c>
       <c r="D98" t="n">
-        <v>792246</v>
+        <v>794671</v>
       </c>
       <c r="E98" t="n">
-        <v>1852.36</v>
+        <v>11786.46</v>
       </c>
       <c r="F98" t="n">
-        <v>369.52</v>
+        <v>5772.38</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D99" t="n">
-        <v>47252</v>
+        <v>792246</v>
       </c>
       <c r="E99" t="n">
-        <v>9494.1</v>
+        <v>1852.36</v>
       </c>
       <c r="F99" t="n">
-        <v>0</v>
+        <v>369.52</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D100" t="n">
-        <v>139553</v>
+        <v>47252</v>
       </c>
       <c r="E100" t="n">
-        <v>2430.28</v>
+        <v>9587.780000000001</v>
       </c>
       <c r="F100" t="n">
         <v>0</v>
@@ -2861,7 +2861,7 @@
         <v>199.03</v>
       </c>
       <c r="F101" t="n">
-        <v>252.16</v>
+        <v>451.19</v>
       </c>
     </row>
     <row r="102">
@@ -2930,7 +2930,7 @@
         <v>47252</v>
       </c>
       <c r="E104" t="n">
-        <v>29281.21</v>
+        <v>28125.26</v>
       </c>
       <c r="F104" t="n">
         <v>4814.96</v>
@@ -3125,7 +3125,7 @@
         <v>47301.97</v>
       </c>
       <c r="F112" t="n">
-        <v>91.92</v>
+        <v>8631.360000000001</v>
       </c>
     </row>
     <row r="113">
@@ -3149,18 +3149,18 @@
         <v>3499.72</v>
       </c>
       <c r="F113" t="n">
-        <v>0</v>
+        <v>102.9</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
@@ -3170,10 +3170,10 @@
         <v>795345</v>
       </c>
       <c r="E114" t="n">
-        <v>1702.54</v>
+        <v>2827.01</v>
       </c>
       <c r="F114" t="n">
-        <v>0</v>
+        <v>532.2</v>
       </c>
     </row>
     <row r="115">
@@ -3184,20 +3184,20 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D115" t="n">
-        <v>789525</v>
+        <v>795345</v>
       </c>
       <c r="E115" t="n">
-        <v>5830.6</v>
+        <v>1489.69</v>
       </c>
       <c r="F115" t="n">
-        <v>3468.04</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116">
@@ -3208,20 +3208,20 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D116" t="n">
-        <v>789228</v>
+        <v>789525</v>
       </c>
       <c r="E116" t="n">
-        <v>507.05</v>
+        <v>5954.98</v>
       </c>
       <c r="F116" t="n">
-        <v>325.96</v>
+        <v>3468.04</v>
       </c>
     </row>
     <row r="117">
@@ -3256,26 +3256,26 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D118" t="n">
-        <v>33928</v>
+        <v>789228</v>
       </c>
       <c r="E118" t="n">
-        <v>10.65</v>
+        <v>507.15</v>
       </c>
       <c r="F118" t="n">
-        <v>47.94</v>
+        <v>426.92</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3287,13 +3287,13 @@
         <v>46247</v>
       </c>
       <c r="D119" t="n">
-        <v>795345</v>
+        <v>33928</v>
       </c>
       <c r="E119" t="n">
-        <v>40.89</v>
+        <v>10.65</v>
       </c>
       <c r="F119" t="n">
-        <v>40.89</v>
+        <v>47.94</v>
       </c>
     </row>
     <row r="120">
@@ -3304,20 +3304,20 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D120" t="n">
-        <v>792121</v>
+        <v>795345</v>
       </c>
       <c r="E120" t="n">
-        <v>5833</v>
+        <v>40.89</v>
       </c>
       <c r="F120" t="n">
-        <v>0</v>
+        <v>40.89</v>
       </c>
     </row>
     <row r="121">
@@ -3335,13 +3335,13 @@
         <v>46247</v>
       </c>
       <c r="D121" t="n">
-        <v>795345</v>
+        <v>792121</v>
       </c>
       <c r="E121" t="n">
-        <v>2605.91</v>
+        <v>5833</v>
       </c>
       <c r="F121" t="n">
-        <v>0</v>
+        <v>1213.38</v>
       </c>
     </row>
     <row r="122">
@@ -3362,7 +3362,7 @@
         <v>33928</v>
       </c>
       <c r="E122" t="n">
-        <v>38969.06</v>
+        <v>39079.31</v>
       </c>
       <c r="F122" t="n">
         <v>8258.709999999999</v>
@@ -3407,13 +3407,13 @@
         <v>46247</v>
       </c>
       <c r="D124" t="n">
-        <v>33286</v>
+        <v>30791</v>
       </c>
       <c r="E124" t="n">
-        <v>9942.09</v>
+        <v>22291.88</v>
       </c>
       <c r="F124" t="n">
-        <v>762.3200000000001</v>
+        <v>791.89</v>
       </c>
     </row>
     <row r="125">
@@ -3431,13 +3431,13 @@
         <v>46247</v>
       </c>
       <c r="D125" t="n">
-        <v>30791</v>
+        <v>33286</v>
       </c>
       <c r="E125" t="n">
-        <v>19625.58</v>
+        <v>10639.82</v>
       </c>
       <c r="F125" t="n">
-        <v>791.89</v>
+        <v>762.3200000000001</v>
       </c>
     </row>
     <row r="126">
@@ -3506,7 +3506,7 @@
         <v>789603</v>
       </c>
       <c r="E128" t="n">
-        <v>44480.49</v>
+        <v>46791.91</v>
       </c>
       <c r="F128" t="n">
         <v>0</v>
@@ -3551,13 +3551,13 @@
         <v>46247</v>
       </c>
       <c r="D130" t="n">
-        <v>30307</v>
+        <v>789603</v>
       </c>
       <c r="E130" t="n">
-        <v>52864.95</v>
+        <v>70195.92</v>
       </c>
       <c r="F130" t="n">
-        <v>10642.54</v>
+        <v>3544.72</v>
       </c>
     </row>
     <row r="131">
@@ -3575,13 +3575,13 @@
         <v>46247</v>
       </c>
       <c r="D131" t="n">
-        <v>789603</v>
+        <v>30307</v>
       </c>
       <c r="E131" t="n">
-        <v>67987.97</v>
+        <v>59944.51</v>
       </c>
       <c r="F131" t="n">
-        <v>3544.72</v>
+        <v>10642.54</v>
       </c>
     </row>
     <row r="132">
@@ -3626,7 +3626,7 @@
         <v>33928</v>
       </c>
       <c r="E133" t="n">
-        <v>1686.17</v>
+        <v>1818.28</v>
       </c>
       <c r="F133" t="n">
         <v>0</v>
@@ -3653,7 +3653,7 @@
         <v>225.33</v>
       </c>
       <c r="F134" t="n">
-        <v>97.97</v>
+        <v>323.3</v>
       </c>
     </row>
     <row r="135">
@@ -3722,7 +3722,7 @@
         <v>33928</v>
       </c>
       <c r="E137" t="n">
-        <v>1931.93</v>
+        <v>2163.75</v>
       </c>
       <c r="F137" t="n">
         <v>0</v>
@@ -3794,7 +3794,7 @@
         <v>31267</v>
       </c>
       <c r="E140" t="n">
-        <v>2682.29</v>
+        <v>2697.6</v>
       </c>
       <c r="F140" t="n">
         <v>58.7</v>
@@ -3821,7 +3821,7 @@
         <v>731.21</v>
       </c>
       <c r="F141" t="n">
-        <v>0</v>
+        <v>502.13</v>
       </c>
     </row>
     <row r="142">
@@ -3986,7 +3986,7 @@
         <v>792121</v>
       </c>
       <c r="E148" t="n">
-        <v>313.33</v>
+        <v>10507.33</v>
       </c>
       <c r="F148" t="n">
         <v>0</v>
@@ -4000,92 +4000,92 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C149" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D149" t="n">
-        <v>792121</v>
+        <v>794029</v>
       </c>
       <c r="E149" t="n">
-        <v>8297.24</v>
+        <v>11572.5</v>
       </c>
       <c r="F149" t="n">
-        <v>0</v>
+        <v>2161.12</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C150" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D150" t="n">
-        <v>47252</v>
+        <v>790595</v>
       </c>
       <c r="E150" t="n">
-        <v>29804.86</v>
+        <v>1668.92</v>
       </c>
       <c r="F150" t="n">
-        <v>5590.24</v>
+        <v>1075.97</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C151" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D151" t="n">
-        <v>47252</v>
+        <v>792121</v>
       </c>
       <c r="E151" t="n">
-        <v>39929.19</v>
+        <v>8297.24</v>
       </c>
       <c r="F151" t="n">
-        <v>10035.59</v>
+        <v>459.77</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C152" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D152" t="n">
-        <v>30083</v>
+        <v>47252</v>
       </c>
       <c r="E152" t="n">
-        <v>690.36</v>
+        <v>30952.89</v>
       </c>
       <c r="F152" t="n">
-        <v>237</v>
+        <v>5590.24</v>
       </c>
     </row>
     <row r="153">
@@ -4096,44 +4096,44 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C153" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D153" t="n">
-        <v>789661</v>
+        <v>47252</v>
       </c>
       <c r="E153" t="n">
-        <v>476.23</v>
+        <v>41556.16</v>
       </c>
       <c r="F153" t="n">
-        <v>258.83</v>
+        <v>11918.65</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C154" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D154" t="n">
-        <v>795345</v>
+        <v>30083</v>
       </c>
       <c r="E154" t="n">
-        <v>27.25</v>
+        <v>690.36</v>
       </c>
       <c r="F154" t="n">
-        <v>0</v>
+        <v>237</v>
       </c>
     </row>
     <row r="155">
@@ -4144,41 +4144,41 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C155" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D155" t="n">
-        <v>793718</v>
+        <v>789661</v>
       </c>
       <c r="E155" t="n">
-        <v>39.84</v>
+        <v>476.23</v>
       </c>
       <c r="F155" t="n">
-        <v>0</v>
+        <v>258.83</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C156" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D156" t="n">
-        <v>789525</v>
+        <v>795345</v>
       </c>
       <c r="E156" t="n">
-        <v>34.37</v>
+        <v>27.25</v>
       </c>
       <c r="F156" t="n">
         <v>0</v>
@@ -4199,13 +4199,13 @@
         <v>46247</v>
       </c>
       <c r="D157" t="n">
-        <v>33057</v>
+        <v>793718</v>
       </c>
       <c r="E157" t="n">
-        <v>42.76</v>
+        <v>39.84</v>
       </c>
       <c r="F157" t="n">
-        <v>43.58</v>
+        <v>0</v>
       </c>
     </row>
     <row r="158">
@@ -4235,25 +4235,25 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C159" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D159" t="n">
-        <v>31267</v>
+        <v>33057</v>
       </c>
       <c r="E159" t="n">
-        <v>160.86</v>
+        <v>42.76</v>
       </c>
       <c r="F159" t="n">
-        <v>203.78</v>
+        <v>43.58</v>
       </c>
     </row>
     <row r="160">
@@ -4264,92 +4264,92 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C160" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D160" t="n">
-        <v>33286</v>
+        <v>789525</v>
       </c>
       <c r="E160" t="n">
-        <v>14138.65</v>
+        <v>34.37</v>
       </c>
       <c r="F160" t="n">
-        <v>2131.12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C161" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D161" t="n">
-        <v>139553</v>
+        <v>31267</v>
       </c>
       <c r="E161" t="n">
-        <v>1107.08</v>
+        <v>160.86</v>
       </c>
       <c r="F161" t="n">
-        <v>222.36</v>
+        <v>203.78</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C162" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D162" t="n">
-        <v>30791</v>
+        <v>139553</v>
       </c>
       <c r="E162" t="n">
-        <v>0</v>
+        <v>1107.08</v>
       </c>
       <c r="F162" t="n">
-        <v>646.85</v>
+        <v>222.36</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C163" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D163" t="n">
-        <v>30307</v>
+        <v>33286</v>
       </c>
       <c r="E163" t="n">
-        <v>507.68</v>
+        <v>14138.65</v>
       </c>
       <c r="F163" t="n">
-        <v>0</v>
+        <v>2131.12</v>
       </c>
     </row>
     <row r="164">
@@ -4360,116 +4360,116 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C164" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D164" t="n">
-        <v>33057</v>
+        <v>30791</v>
       </c>
       <c r="E164" t="n">
-        <v>382.84</v>
+        <v>0</v>
       </c>
       <c r="F164" t="n">
-        <v>0</v>
+        <v>646.85</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C165" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D165" t="n">
-        <v>31267</v>
+        <v>30307</v>
       </c>
       <c r="E165" t="n">
-        <v>758.3</v>
+        <v>507.68</v>
       </c>
       <c r="F165" t="n">
-        <v>0</v>
+        <v>507.68</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C166" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D166" t="n">
-        <v>793186</v>
+        <v>33057</v>
       </c>
       <c r="E166" t="n">
-        <v>637.28</v>
+        <v>382.84</v>
       </c>
       <c r="F166" t="n">
-        <v>97.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C167" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D167" t="n">
-        <v>794671</v>
+        <v>31267</v>
       </c>
       <c r="E167" t="n">
-        <v>3174.24</v>
+        <v>856.08</v>
       </c>
       <c r="F167" t="n">
-        <v>7836.18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="C168" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D168" t="n">
-        <v>794029</v>
+        <v>793186</v>
       </c>
       <c r="E168" t="n">
-        <v>11301.04</v>
+        <v>695.27</v>
       </c>
       <c r="F168" t="n">
-        <v>0</v>
+        <v>97.42</v>
       </c>
     </row>
     <row r="169">
@@ -4480,20 +4480,20 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C169" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D169" t="n">
-        <v>790595</v>
+        <v>794671</v>
       </c>
       <c r="E169" t="n">
-        <v>1479.08</v>
+        <v>4114.58</v>
       </c>
       <c r="F169" t="n">
-        <v>162.32</v>
+        <v>7836.18</v>
       </c>
     </row>
     <row r="170">
@@ -4562,10 +4562,10 @@
         <v>32816</v>
       </c>
       <c r="E172" t="n">
-        <v>2285.18</v>
+        <v>3011</v>
       </c>
       <c r="F172" t="n">
-        <v>950.1799999999999</v>
+        <v>1426.28</v>
       </c>
     </row>
     <row r="173">
@@ -4586,7 +4586,7 @@
         <v>31267</v>
       </c>
       <c r="E173" t="n">
-        <v>168971.87</v>
+        <v>169522.13</v>
       </c>
       <c r="F173" t="n">
         <v>0</v>
@@ -4613,7 +4613,7 @@
         <v>13366.54</v>
       </c>
       <c r="F174" t="n">
-        <v>3414.23</v>
+        <v>5864.95</v>
       </c>
     </row>
     <row r="175">
@@ -4637,7 +4637,7 @@
         <v>1001.81</v>
       </c>
       <c r="F175" t="n">
-        <v>341.56</v>
+        <v>904.11</v>
       </c>
     </row>
     <row r="176">
@@ -4685,7 +4685,7 @@
         <v>7003.92</v>
       </c>
       <c r="F177" t="n">
-        <v>0</v>
+        <v>5361.84</v>
       </c>
     </row>
     <row r="178">
@@ -4709,7 +4709,7 @@
         <v>4710.72</v>
       </c>
       <c r="F178" t="n">
-        <v>0</v>
+        <v>717.6</v>
       </c>
     </row>
     <row r="179">
@@ -4847,10 +4847,10 @@
         <v>46247</v>
       </c>
       <c r="D184" t="n">
-        <v>30307</v>
+        <v>30083</v>
       </c>
       <c r="E184" t="n">
-        <v>8056.14</v>
+        <v>862.52</v>
       </c>
       <c r="F184" t="n">
         <v>0</v>
@@ -4871,10 +4871,10 @@
         <v>46247</v>
       </c>
       <c r="D185" t="n">
-        <v>30083</v>
+        <v>30307</v>
       </c>
       <c r="E185" t="n">
-        <v>928.8200000000001</v>
+        <v>8056.14</v>
       </c>
       <c r="F185" t="n">
         <v>0</v>
@@ -4925,7 +4925,7 @@
         <v>11733.88</v>
       </c>
       <c r="F187" t="n">
-        <v>0</v>
+        <v>430.38</v>
       </c>
     </row>
     <row r="188">
@@ -4946,10 +4946,10 @@
         <v>33057</v>
       </c>
       <c r="E188" t="n">
-        <v>1929.99</v>
+        <v>1930.05</v>
       </c>
       <c r="F188" t="n">
-        <v>1144.89</v>
+        <v>1170.9</v>
       </c>
     </row>
     <row r="189">
@@ -4970,7 +4970,7 @@
         <v>790595</v>
       </c>
       <c r="E189" t="n">
-        <v>1664.48</v>
+        <v>1730.23</v>
       </c>
       <c r="F189" t="n">
         <v>0</v>
@@ -5042,7 +5042,7 @@
         <v>47252</v>
       </c>
       <c r="E192" t="n">
-        <v>21893.75</v>
+        <v>22576.61</v>
       </c>
       <c r="F192" t="n">
         <v>8727.5</v>
@@ -5066,7 +5066,7 @@
         <v>793186</v>
       </c>
       <c r="E193" t="n">
-        <v>1867.05</v>
+        <v>2220.33</v>
       </c>
       <c r="F193" t="n">
         <v>266.72</v>
@@ -5114,7 +5114,7 @@
         <v>793718</v>
       </c>
       <c r="E195" t="n">
-        <v>3796.25</v>
+        <v>4255.87</v>
       </c>
       <c r="F195" t="n">
         <v>509.55</v>
@@ -5138,7 +5138,7 @@
         <v>789228</v>
       </c>
       <c r="E196" t="n">
-        <v>2695.7</v>
+        <v>3128.9</v>
       </c>
       <c r="F196" t="n">
         <v>0</v>
@@ -5186,7 +5186,7 @@
         <v>30307</v>
       </c>
       <c r="E198" t="n">
-        <v>41916.4</v>
+        <v>44970.24</v>
       </c>
       <c r="F198" t="n">
         <v>12589.2</v>
@@ -5210,10 +5210,10 @@
         <v>30307</v>
       </c>
       <c r="E199" t="n">
-        <v>66591.42999999999</v>
+        <v>70660.94</v>
       </c>
       <c r="F199" t="n">
-        <v>5387.92</v>
+        <v>24957.15</v>
       </c>
     </row>
     <row r="200">
@@ -5234,7 +5234,7 @@
         <v>789603</v>
       </c>
       <c r="E200" t="n">
-        <v>6461.06</v>
+        <v>6316.89</v>
       </c>
       <c r="F200" t="n">
         <v>21.53</v>
@@ -5258,7 +5258,7 @@
         <v>30083</v>
       </c>
       <c r="E201" t="n">
-        <v>192.1</v>
+        <v>179.24</v>
       </c>
       <c r="F201" t="n">
         <v>0</v>
@@ -5306,7 +5306,7 @@
         <v>30307</v>
       </c>
       <c r="E203" t="n">
-        <v>100704.12</v>
+        <v>102563.64</v>
       </c>
       <c r="F203" t="n">
         <v>0</v>
@@ -5339,7 +5339,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5351,19 +5351,19 @@
         <v>46247</v>
       </c>
       <c r="D205" t="n">
-        <v>795345</v>
+        <v>47252</v>
       </c>
       <c r="E205" t="n">
-        <v>439.18</v>
+        <v>3521</v>
       </c>
       <c r="F205" t="n">
-        <v>0</v>
+        <v>2771.13</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5375,13 +5375,13 @@
         <v>46247</v>
       </c>
       <c r="D206" t="n">
-        <v>47252</v>
+        <v>795345</v>
       </c>
       <c r="E206" t="n">
-        <v>3521</v>
+        <v>439.18</v>
       </c>
       <c r="F206" t="n">
-        <v>2195.62</v>
+        <v>282.48</v>
       </c>
     </row>
     <row r="207">
@@ -5402,7 +5402,7 @@
         <v>792121</v>
       </c>
       <c r="E207" t="n">
-        <v>1025.88</v>
+        <v>1009.9</v>
       </c>
       <c r="F207" t="n">
         <v>0</v>
@@ -5459,25 +5459,25 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C210" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D210" t="n">
-        <v>31267</v>
+        <v>794671</v>
       </c>
       <c r="E210" t="n">
-        <v>28115.49</v>
+        <v>6022.34</v>
       </c>
       <c r="F210" t="n">
-        <v>5524.52</v>
+        <v>2475.65</v>
       </c>
     </row>
     <row r="211">
@@ -5495,13 +5495,13 @@
         <v>46247</v>
       </c>
       <c r="D211" t="n">
-        <v>789525</v>
+        <v>31267</v>
       </c>
       <c r="E211" t="n">
-        <v>9437.219999999999</v>
+        <v>28235.85</v>
       </c>
       <c r="F211" t="n">
-        <v>1578.42</v>
+        <v>5676.84</v>
       </c>
     </row>
     <row r="212">
@@ -5519,13 +5519,13 @@
         <v>46247</v>
       </c>
       <c r="D212" t="n">
-        <v>789228</v>
+        <v>789525</v>
       </c>
       <c r="E212" t="n">
-        <v>5818.2</v>
+        <v>9122.280000000001</v>
       </c>
       <c r="F212" t="n">
-        <v>434.79</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="213">
@@ -5536,20 +5536,20 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C213" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D213" t="n">
-        <v>31267</v>
+        <v>789228</v>
       </c>
       <c r="E213" t="n">
-        <v>42.74</v>
+        <v>5818.28</v>
       </c>
       <c r="F213" t="n">
-        <v>0</v>
+        <v>479.38</v>
       </c>
     </row>
     <row r="214">
@@ -5567,13 +5567,13 @@
         <v>46247</v>
       </c>
       <c r="D214" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="E214" t="n">
-        <v>15.24</v>
+        <v>13.91</v>
       </c>
       <c r="F214" t="n">
-        <v>5.57</v>
+        <v>13.91</v>
       </c>
     </row>
     <row r="215">
@@ -5591,48 +5591,48 @@
         <v>46247</v>
       </c>
       <c r="D215" t="n">
-        <v>793186</v>
+        <v>47252</v>
       </c>
       <c r="E215" t="n">
-        <v>13.91</v>
+        <v>15.24</v>
       </c>
       <c r="F215" t="n">
-        <v>13.91</v>
+        <v>5.57</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C216" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D216" t="n">
-        <v>30791</v>
+        <v>31267</v>
       </c>
       <c r="E216" t="n">
-        <v>7966.86</v>
+        <v>42.74</v>
       </c>
       <c r="F216" t="n">
-        <v>1837.82</v>
+        <v>0</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C217" s="2" t="n">
@@ -5642,10 +5642,10 @@
         <v>30791</v>
       </c>
       <c r="E217" t="n">
-        <v>25725.99</v>
+        <v>7966.86</v>
       </c>
       <c r="F217" t="n">
-        <v>14080.24</v>
+        <v>1837.82</v>
       </c>
     </row>
     <row r="218">
@@ -5675,46 +5675,46 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C219" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D219" t="n">
-        <v>789603</v>
+        <v>30791</v>
       </c>
       <c r="E219" t="n">
-        <v>6690.38</v>
+        <v>26155.82</v>
       </c>
       <c r="F219" t="n">
-        <v>0</v>
+        <v>14080.24</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">MARIA ECILIA ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="C220" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D220" t="n">
-        <v>30307</v>
+        <v>789603</v>
       </c>
       <c r="E220" t="n">
-        <v>343.86</v>
+        <v>6690.38</v>
       </c>
       <c r="F220" t="n">
         <v>0</v>
@@ -5723,22 +5723,22 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C221" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D221" t="n">
-        <v>790595</v>
+        <v>30307</v>
       </c>
       <c r="E221" t="n">
-        <v>775.89</v>
+        <v>343.86</v>
       </c>
       <c r="F221" t="n">
         <v>0</v>
@@ -5747,97 +5747,97 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C222" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D222" t="n">
-        <v>792141</v>
+        <v>790595</v>
       </c>
       <c r="E222" t="n">
-        <v>23276.13</v>
+        <v>775.89</v>
       </c>
       <c r="F222" t="n">
-        <v>3298.38</v>
+        <v>0</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C223" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D223" t="n">
-        <v>794029</v>
+        <v>792141</v>
       </c>
       <c r="E223" t="n">
-        <v>300.39</v>
+        <v>23100.59</v>
       </c>
       <c r="F223" t="n">
-        <v>31.16</v>
+        <v>3298.38</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C224" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D224" t="n">
-        <v>32816</v>
+        <v>794029</v>
       </c>
       <c r="E224" t="n">
-        <v>456.96</v>
+        <v>1328.6</v>
       </c>
       <c r="F224" t="n">
-        <v>30.96</v>
+        <v>31.16</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C225" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D225" t="n">
-        <v>794671</v>
+        <v>32816</v>
       </c>
       <c r="E225" t="n">
-        <v>5871.48</v>
+        <v>456.96</v>
       </c>
       <c r="F225" t="n">
-        <v>249.61</v>
+        <v>30.96</v>
       </c>
     </row>
     <row r="226">
@@ -5861,7 +5861,7 @@
         <v>5217.44</v>
       </c>
       <c r="F226" t="n">
-        <v>158.6</v>
+        <v>2026.28</v>
       </c>
     </row>
     <row r="227">
@@ -5906,7 +5906,7 @@
         <v>33928</v>
       </c>
       <c r="E228" t="n">
-        <v>46.44</v>
+        <v>3868.28</v>
       </c>
       <c r="F228" t="n">
         <v>5.82</v>
@@ -5954,10 +5954,10 @@
         <v>139553</v>
       </c>
       <c r="E230" t="n">
-        <v>16103.62</v>
+        <v>16963.66</v>
       </c>
       <c r="F230" t="n">
-        <v>8082.68</v>
+        <v>8915.299999999999</v>
       </c>
     </row>
     <row r="231">
@@ -5999,13 +5999,13 @@
         <v>46247</v>
       </c>
       <c r="D232" t="n">
-        <v>30218</v>
+        <v>790595</v>
       </c>
       <c r="E232" t="n">
-        <v>3083.55</v>
+        <v>267.36</v>
       </c>
       <c r="F232" t="n">
-        <v>0</v>
+        <v>267.36</v>
       </c>
     </row>
     <row r="233">
@@ -6023,13 +6023,13 @@
         <v>46247</v>
       </c>
       <c r="D233" t="n">
-        <v>790595</v>
+        <v>30218</v>
       </c>
       <c r="E233" t="n">
-        <v>267.36</v>
+        <v>7800.36</v>
       </c>
       <c r="F233" t="n">
-        <v>267.36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="234">
@@ -6050,7 +6050,7 @@
         <v>47252</v>
       </c>
       <c r="E234" t="n">
-        <v>26679.3</v>
+        <v>28425.48</v>
       </c>
       <c r="F234" t="n">
         <v>0</v>
@@ -6098,7 +6098,7 @@
         <v>789603</v>
       </c>
       <c r="E236" t="n">
-        <v>32256.99</v>
+        <v>32736.21</v>
       </c>
       <c r="F236" t="n">
         <v>0</v>
@@ -6146,7 +6146,7 @@
         <v>793186</v>
       </c>
       <c r="E238" t="n">
-        <v>20047.43</v>
+        <v>19711.47</v>
       </c>
       <c r="F238" t="n">
         <v>702.38</v>
@@ -6245,7 +6245,7 @@
         <v>6264.58</v>
       </c>
       <c r="F242" t="n">
-        <v>0</v>
+        <v>1027.97</v>
       </c>
     </row>
     <row r="243">
@@ -6266,10 +6266,10 @@
         <v>30307</v>
       </c>
       <c r="E243" t="n">
-        <v>183946.29</v>
+        <v>184402.05</v>
       </c>
       <c r="F243" t="n">
-        <v>0</v>
+        <v>72128.89</v>
       </c>
     </row>
     <row r="244">
@@ -6293,7 +6293,7 @@
         <v>5736.3</v>
       </c>
       <c r="F244" t="n">
-        <v>0</v>
+        <v>1319.99</v>
       </c>
     </row>
     <row r="245">
@@ -6314,10 +6314,10 @@
         <v>793718</v>
       </c>
       <c r="E245" t="n">
-        <v>44239.56</v>
+        <v>44262.28</v>
       </c>
       <c r="F245" t="n">
-        <v>1369.51</v>
+        <v>1398.31</v>
       </c>
     </row>
     <row r="246">
@@ -6338,7 +6338,7 @@
         <v>30083</v>
       </c>
       <c r="E246" t="n">
-        <v>2164.92</v>
+        <v>3472.61</v>
       </c>
       <c r="F246" t="n">
         <v>0</v>
@@ -6362,7 +6362,7 @@
         <v>789661</v>
       </c>
       <c r="E247" t="n">
-        <v>6362.71</v>
+        <v>5789.8</v>
       </c>
       <c r="F247" t="n">
         <v>32.2</v>
@@ -6371,7 +6371,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -6383,19 +6383,19 @@
         <v>46247</v>
       </c>
       <c r="D248" t="n">
-        <v>794671</v>
+        <v>33286</v>
       </c>
       <c r="E248" t="n">
-        <v>3352.57</v>
+        <v>12.44</v>
       </c>
       <c r="F248" t="n">
-        <v>673.33</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -6407,13 +6407,13 @@
         <v>46247</v>
       </c>
       <c r="D249" t="n">
-        <v>33286</v>
+        <v>792121</v>
       </c>
       <c r="E249" t="n">
-        <v>12.44</v>
+        <v>47.14</v>
       </c>
       <c r="F249" t="n">
-        <v>3.99</v>
+        <v>26.67</v>
       </c>
     </row>
     <row r="250">
@@ -6431,13 +6431,13 @@
         <v>46247</v>
       </c>
       <c r="D250" t="n">
-        <v>792121</v>
+        <v>794671</v>
       </c>
       <c r="E250" t="n">
-        <v>47.14</v>
+        <v>3352.57</v>
       </c>
       <c r="F250" t="n">
-        <v>26.67</v>
+        <v>1576.9</v>
       </c>
     </row>
     <row r="251">
@@ -6491,7 +6491,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6503,10 +6503,10 @@
         <v>46247</v>
       </c>
       <c r="D253" t="n">
-        <v>33286</v>
+        <v>30791</v>
       </c>
       <c r="E253" t="n">
-        <v>8.73</v>
+        <v>2.53</v>
       </c>
       <c r="F253" t="n">
         <v>0</v>
@@ -6539,7 +6539,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6551,10 +6551,10 @@
         <v>46247</v>
       </c>
       <c r="D255" t="n">
-        <v>30791</v>
+        <v>33286</v>
       </c>
       <c r="E255" t="n">
-        <v>2.53</v>
+        <v>8.73</v>
       </c>
       <c r="F255" t="n">
         <v>0</v>
@@ -6581,7 +6581,7 @@
         <v>14181.74</v>
       </c>
       <c r="F256" t="n">
-        <v>0</v>
+        <v>2907.24</v>
       </c>
     </row>
     <row r="257">
@@ -6599,13 +6599,13 @@
         <v>46247</v>
       </c>
       <c r="D257" t="n">
-        <v>789525</v>
+        <v>33928</v>
       </c>
       <c r="E257" t="n">
-        <v>971.33</v>
+        <v>1073.97</v>
       </c>
       <c r="F257" t="n">
-        <v>773.74</v>
+        <v>952.46</v>
       </c>
     </row>
     <row r="258">
@@ -6623,13 +6623,13 @@
         <v>46247</v>
       </c>
       <c r="D258" t="n">
-        <v>33928</v>
+        <v>789525</v>
       </c>
       <c r="E258" t="n">
-        <v>1073.97</v>
+        <v>971.33</v>
       </c>
       <c r="F258" t="n">
-        <v>952.46</v>
+        <v>773.74</v>
       </c>
     </row>
     <row r="259">
@@ -6674,7 +6674,7 @@
         <v>789525</v>
       </c>
       <c r="E260" t="n">
-        <v>9253.02</v>
+        <v>10034.14</v>
       </c>
       <c r="F260" t="n">
         <v>2585.8</v>
@@ -6719,13 +6719,13 @@
         <v>46247</v>
       </c>
       <c r="D262" t="n">
-        <v>47252</v>
+        <v>30791</v>
       </c>
       <c r="E262" t="n">
-        <v>29189.06</v>
+        <v>9999.870000000001</v>
       </c>
       <c r="F262" t="n">
-        <v>2156.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="263">
@@ -6743,13 +6743,13 @@
         <v>46247</v>
       </c>
       <c r="D263" t="n">
-        <v>789525</v>
+        <v>47252</v>
       </c>
       <c r="E263" t="n">
-        <v>3393.84</v>
+        <v>31838.14</v>
       </c>
       <c r="F263" t="n">
-        <v>733.89</v>
+        <v>2156.1</v>
       </c>
     </row>
     <row r="264">
@@ -6767,13 +6767,13 @@
         <v>46247</v>
       </c>
       <c r="D264" t="n">
-        <v>30791</v>
+        <v>789525</v>
       </c>
       <c r="E264" t="n">
-        <v>9619.120000000001</v>
+        <v>3858</v>
       </c>
       <c r="F264" t="n">
-        <v>0</v>
+        <v>733.89</v>
       </c>
     </row>
     <row r="265">
@@ -6845,7 +6845,7 @@
         <v>5370.72</v>
       </c>
       <c r="F267" t="n">
-        <v>0</v>
+        <v>267.06</v>
       </c>
     </row>
     <row r="268">
@@ -6866,7 +6866,7 @@
         <v>795345</v>
       </c>
       <c r="E268" t="n">
-        <v>6178.94</v>
+        <v>6537.42</v>
       </c>
       <c r="F268" t="n">
         <v>283.04</v>
@@ -6890,7 +6890,7 @@
         <v>47252</v>
       </c>
       <c r="E269" t="n">
-        <v>46923.21</v>
+        <v>48823.21</v>
       </c>
       <c r="F269" t="n">
         <v>3164.26</v>
@@ -6914,7 +6914,7 @@
         <v>789603</v>
       </c>
       <c r="E270" t="n">
-        <v>25288.07</v>
+        <v>26308.13</v>
       </c>
       <c r="F270" t="n">
         <v>553.98</v>
@@ -6938,7 +6938,7 @@
         <v>789603</v>
       </c>
       <c r="E271" t="n">
-        <v>82955.17999999999</v>
+        <v>83607.02</v>
       </c>
       <c r="F271" t="n">
         <v>41155.22</v>
@@ -6986,7 +6986,7 @@
         <v>793186</v>
       </c>
       <c r="E273" t="n">
-        <v>619.13</v>
+        <v>652.61</v>
       </c>
       <c r="F273" t="n">
         <v>444.16</v>
@@ -7007,10 +7007,10 @@
         <v>46247</v>
       </c>
       <c r="D274" t="n">
-        <v>794671</v>
+        <v>30307</v>
       </c>
       <c r="E274" t="n">
-        <v>2664.9</v>
+        <v>20060.93</v>
       </c>
       <c r="F274" t="n">
         <v>0</v>
@@ -7031,10 +7031,10 @@
         <v>46247</v>
       </c>
       <c r="D275" t="n">
-        <v>30307</v>
+        <v>794671</v>
       </c>
       <c r="E275" t="n">
-        <v>20060.93</v>
+        <v>2664.9</v>
       </c>
       <c r="F275" t="n">
         <v>0</v>
@@ -7061,7 +7061,7 @@
         <v>1446.99</v>
       </c>
       <c r="F276" t="n">
-        <v>652.84</v>
+        <v>701.9400000000001</v>
       </c>
     </row>
     <row r="277">
@@ -7082,7 +7082,7 @@
         <v>792141</v>
       </c>
       <c r="E277" t="n">
-        <v>4245.96</v>
+        <v>3781.8</v>
       </c>
       <c r="F277" t="n">
         <v>0</v>
@@ -7109,7 +7109,7 @@
         <v>146.11</v>
       </c>
       <c r="F278" t="n">
-        <v>418.78</v>
+        <v>564.89</v>
       </c>
     </row>
     <row r="279">
@@ -7130,7 +7130,7 @@
         <v>792121</v>
       </c>
       <c r="E279" t="n">
-        <v>3925.53</v>
+        <v>5097.93</v>
       </c>
       <c r="F279" t="n">
         <v>388.95</v>
@@ -7154,7 +7154,7 @@
         <v>30083</v>
       </c>
       <c r="E280" t="n">
-        <v>4971.77</v>
+        <v>5754.64</v>
       </c>
       <c r="F280" t="n">
         <v>185.25</v>
@@ -7178,7 +7178,7 @@
         <v>139553</v>
       </c>
       <c r="E281" t="n">
-        <v>9314.6</v>
+        <v>9444.959999999999</v>
       </c>
       <c r="F281" t="n">
         <v>0</v>
@@ -7199,13 +7199,13 @@
         <v>46247</v>
       </c>
       <c r="D282" t="n">
-        <v>33928</v>
+        <v>33057</v>
       </c>
       <c r="E282" t="n">
-        <v>3907.58</v>
+        <v>21955.76</v>
       </c>
       <c r="F282" t="n">
-        <v>94.43000000000001</v>
+        <v>261.95</v>
       </c>
     </row>
     <row r="283">
@@ -7223,13 +7223,13 @@
         <v>46247</v>
       </c>
       <c r="D283" t="n">
-        <v>33057</v>
+        <v>33928</v>
       </c>
       <c r="E283" t="n">
-        <v>21918.99</v>
+        <v>3809.86</v>
       </c>
       <c r="F283" t="n">
-        <v>261.95</v>
+        <v>94.43000000000001</v>
       </c>
     </row>
     <row r="284">
@@ -7346,7 +7346,7 @@
         <v>33286</v>
       </c>
       <c r="E288" t="n">
-        <v>255.99</v>
+        <v>284.32</v>
       </c>
       <c r="F288" t="n">
         <v>0</v>
@@ -7355,24 +7355,48 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D289" t="n">
+        <v>139553</v>
+      </c>
+      <c r="E289" t="n">
+        <v>139.56</v>
+      </c>
+      <c r="F289" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="B289" t="inlineStr">
+      <c r="B290" t="inlineStr">
         <is>
           <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
-      <c r="C289" s="2" t="n">
-        <v>46247</v>
-      </c>
-      <c r="D289" t="n">
+      <c r="C290" s="2" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D290" t="n">
         <v>795345</v>
       </c>
-      <c r="E289" t="n">
+      <c r="E290" t="n">
         <v>169.57</v>
       </c>
-      <c r="F289" t="n">
+      <c r="F290" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 17:53:16
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -575,13 +575,13 @@
         <v>46247</v>
       </c>
       <c r="D6" t="n">
-        <v>139553</v>
+        <v>47252</v>
       </c>
       <c r="E6" t="n">
-        <v>179.4</v>
+        <v>63107.98</v>
       </c>
       <c r="F6" t="n">
-        <v>179.4</v>
+        <v>12850.83</v>
       </c>
     </row>
     <row r="7">
@@ -599,13 +599,13 @@
         <v>46247</v>
       </c>
       <c r="D7" t="n">
-        <v>47252</v>
+        <v>139553</v>
       </c>
       <c r="E7" t="n">
-        <v>63107.98</v>
+        <v>179.4</v>
       </c>
       <c r="F7" t="n">
-        <v>12850.83</v>
+        <v>179.4</v>
       </c>
     </row>
     <row r="8">
@@ -671,13 +671,13 @@
         <v>46247</v>
       </c>
       <c r="D10" t="n">
-        <v>33928</v>
+        <v>789228</v>
       </c>
       <c r="E10" t="n">
-        <v>10156.46</v>
+        <v>4654.59</v>
       </c>
       <c r="F10" t="n">
-        <v>3365.06</v>
+        <v>1664.41</v>
       </c>
     </row>
     <row r="11">
@@ -695,13 +695,13 @@
         <v>46247</v>
       </c>
       <c r="D11" t="n">
-        <v>789228</v>
+        <v>33928</v>
       </c>
       <c r="E11" t="n">
-        <v>4654.59</v>
+        <v>10470.72</v>
       </c>
       <c r="F11" t="n">
-        <v>1664.41</v>
+        <v>3365.06</v>
       </c>
     </row>
     <row r="12">
@@ -938,7 +938,7 @@
         <v>33057</v>
       </c>
       <c r="E21" t="n">
-        <v>1888.76</v>
+        <v>2033.42</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -1034,7 +1034,7 @@
         <v>30307</v>
       </c>
       <c r="E25" t="n">
-        <v>72023.42</v>
+        <v>78186.34</v>
       </c>
       <c r="F25" t="n">
         <v>22829.12</v>
@@ -1274,7 +1274,7 @@
         <v>789603</v>
       </c>
       <c r="E35" t="n">
-        <v>3247.44</v>
+        <v>3827.34</v>
       </c>
       <c r="F35" t="n">
         <v>2087.64</v>
@@ -1394,7 +1394,7 @@
         <v>794671</v>
       </c>
       <c r="E40" t="n">
-        <v>281.7</v>
+        <v>1267.39</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
@@ -1754,10 +1754,10 @@
         <v>789228</v>
       </c>
       <c r="E55" t="n">
-        <v>8641.040000000001</v>
+        <v>8641.049999999999</v>
       </c>
       <c r="F55" t="n">
-        <v>3175.65</v>
+        <v>3191.45</v>
       </c>
     </row>
     <row r="56">
@@ -1778,10 +1778,10 @@
         <v>47252</v>
       </c>
       <c r="E56" t="n">
-        <v>53994.91</v>
+        <v>53995.25</v>
       </c>
       <c r="F56" t="n">
-        <v>9467.51</v>
+        <v>10211.03</v>
       </c>
     </row>
     <row r="57">
@@ -1826,7 +1826,7 @@
         <v>33928</v>
       </c>
       <c r="E58" t="n">
-        <v>6151.76</v>
+        <v>6376.09</v>
       </c>
       <c r="F58" t="n">
         <v>25.2</v>
@@ -2570,10 +2570,10 @@
         <v>31267</v>
       </c>
       <c r="E89" t="n">
-        <v>6830.26</v>
+        <v>6897.71</v>
       </c>
       <c r="F89" t="n">
-        <v>628.91</v>
+        <v>687.99</v>
       </c>
     </row>
     <row r="90">
@@ -2594,10 +2594,10 @@
         <v>793718</v>
       </c>
       <c r="E90" t="n">
-        <v>8887.620000000001</v>
+        <v>8887.719999999999</v>
       </c>
       <c r="F90" t="n">
-        <v>5268.17</v>
+        <v>5501.58</v>
       </c>
     </row>
     <row r="91">
@@ -2690,7 +2690,7 @@
         <v>33286</v>
       </c>
       <c r="E94" t="n">
-        <v>4042.86</v>
+        <v>4225.02</v>
       </c>
       <c r="F94" t="n">
         <v>0</v>
@@ -2837,7 +2837,7 @@
         <v>22170.39</v>
       </c>
       <c r="F100" t="n">
-        <v>2440.95</v>
+        <v>3063.32</v>
       </c>
     </row>
     <row r="101">
@@ -2858,7 +2858,7 @@
         <v>794671</v>
       </c>
       <c r="E101" t="n">
-        <v>21349.69</v>
+        <v>22439.83</v>
       </c>
       <c r="F101" t="n">
         <v>5772.38</v>
@@ -2906,7 +2906,7 @@
         <v>47252</v>
       </c>
       <c r="E103" t="n">
-        <v>10601</v>
+        <v>11034.52</v>
       </c>
       <c r="F103" t="n">
         <v>0</v>
@@ -3002,7 +3002,7 @@
         <v>47252</v>
       </c>
       <c r="E107" t="n">
-        <v>33873.79</v>
+        <v>34233.31</v>
       </c>
       <c r="F107" t="n">
         <v>4814.96</v>
@@ -3434,10 +3434,10 @@
         <v>33928</v>
       </c>
       <c r="E125" t="n">
-        <v>40214.34</v>
+        <v>40397.68</v>
       </c>
       <c r="F125" t="n">
-        <v>10473.43</v>
+        <v>10652.36</v>
       </c>
     </row>
     <row r="126">
@@ -3602,7 +3602,7 @@
         <v>789603</v>
       </c>
       <c r="E132" t="n">
-        <v>56739.69</v>
+        <v>90239.69</v>
       </c>
       <c r="F132" t="n">
         <v>0</v>
@@ -3647,13 +3647,13 @@
         <v>46247</v>
       </c>
       <c r="D134" t="n">
-        <v>30307</v>
+        <v>789603</v>
       </c>
       <c r="E134" t="n">
-        <v>64217.2</v>
+        <v>119793.39</v>
       </c>
       <c r="F134" t="n">
-        <v>12227.89</v>
+        <v>5212.19</v>
       </c>
     </row>
     <row r="135">
@@ -3671,13 +3671,13 @@
         <v>46247</v>
       </c>
       <c r="D135" t="n">
-        <v>789603</v>
+        <v>30307</v>
       </c>
       <c r="E135" t="n">
-        <v>119793.39</v>
+        <v>64217.2</v>
       </c>
       <c r="F135" t="n">
-        <v>5212.19</v>
+        <v>12227.89</v>
       </c>
     </row>
     <row r="136">
@@ -3746,7 +3746,7 @@
         <v>33928</v>
       </c>
       <c r="E138" t="n">
-        <v>2334</v>
+        <v>3123.75</v>
       </c>
       <c r="F138" t="n">
         <v>0</v>
@@ -3770,7 +3770,7 @@
         <v>30307</v>
       </c>
       <c r="E139" t="n">
-        <v>11390.76</v>
+        <v>11905.9</v>
       </c>
       <c r="F139" t="n">
         <v>1601.48</v>
@@ -4130,7 +4130,7 @@
         <v>790595</v>
       </c>
       <c r="E154" t="n">
-        <v>1668.92</v>
+        <v>1967.06</v>
       </c>
       <c r="F154" t="n">
         <v>1075.97</v>
@@ -4178,7 +4178,7 @@
         <v>47252</v>
       </c>
       <c r="E156" t="n">
-        <v>31078.73</v>
+        <v>31485.14</v>
       </c>
       <c r="F156" t="n">
         <v>5590.24</v>
@@ -4418,10 +4418,10 @@
         <v>33286</v>
       </c>
       <c r="E166" t="n">
-        <v>14323.01</v>
+        <v>14406.44</v>
       </c>
       <c r="F166" t="n">
-        <v>2812.24</v>
+        <v>2866.25</v>
       </c>
     </row>
     <row r="167">
@@ -4754,7 +4754,7 @@
         <v>31267</v>
       </c>
       <c r="E180" t="n">
-        <v>181078.74</v>
+        <v>182098.11</v>
       </c>
       <c r="F180" t="n">
         <v>0</v>
@@ -4919,10 +4919,10 @@
         <v>46247</v>
       </c>
       <c r="D187" t="n">
-        <v>792121</v>
+        <v>30307</v>
       </c>
       <c r="E187" t="n">
-        <v>2990.5</v>
+        <v>13892.91</v>
       </c>
       <c r="F187" t="n">
         <v>0</v>
@@ -4943,10 +4943,10 @@
         <v>46247</v>
       </c>
       <c r="D188" t="n">
-        <v>30307</v>
+        <v>792121</v>
       </c>
       <c r="E188" t="n">
-        <v>13509.03</v>
+        <v>2990.5</v>
       </c>
       <c r="F188" t="n">
         <v>0</v>
@@ -5330,7 +5330,7 @@
         <v>789228</v>
       </c>
       <c r="E204" t="n">
-        <v>3549.25</v>
+        <v>3682.88</v>
       </c>
       <c r="F204" t="n">
         <v>0</v>
@@ -5546,7 +5546,7 @@
         <v>795345</v>
       </c>
       <c r="E213" t="n">
-        <v>439.18</v>
+        <v>564.78</v>
       </c>
       <c r="F213" t="n">
         <v>282.48</v>
@@ -5834,10 +5834,10 @@
         <v>30791</v>
       </c>
       <c r="E225" t="n">
-        <v>27846.82</v>
+        <v>27847.37</v>
       </c>
       <c r="F225" t="n">
-        <v>15803.36</v>
+        <v>17636.95</v>
       </c>
     </row>
     <row r="226">
@@ -5858,10 +5858,10 @@
         <v>789603</v>
       </c>
       <c r="E226" t="n">
-        <v>70907.96000000001</v>
+        <v>70908.82000000001</v>
       </c>
       <c r="F226" t="n">
-        <v>5169.86</v>
+        <v>9575.940000000001</v>
       </c>
     </row>
     <row r="227">
@@ -6290,7 +6290,7 @@
         <v>789603</v>
       </c>
       <c r="E244" t="n">
-        <v>38723.14</v>
+        <v>39191.02</v>
       </c>
       <c r="F244" t="n">
         <v>0</v>
@@ -6482,7 +6482,7 @@
         <v>30307</v>
       </c>
       <c r="E252" t="n">
-        <v>191162.33</v>
+        <v>192658.58</v>
       </c>
       <c r="F252" t="n">
         <v>78793.05</v>
@@ -6659,7 +6659,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -6671,19 +6671,19 @@
         <v>46247</v>
       </c>
       <c r="D260" t="n">
-        <v>139553</v>
+        <v>33286</v>
       </c>
       <c r="E260" t="n">
-        <v>1300.72</v>
+        <v>8.73</v>
       </c>
       <c r="F260" t="n">
-        <v>1300.72</v>
+        <v>0</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -6695,10 +6695,10 @@
         <v>46247</v>
       </c>
       <c r="D261" t="n">
-        <v>794671</v>
+        <v>789525</v>
       </c>
       <c r="E261" t="n">
-        <v>759.41</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="F261" t="n">
         <v>0</v>
@@ -6707,7 +6707,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6719,19 +6719,19 @@
         <v>46247</v>
       </c>
       <c r="D262" t="n">
-        <v>33286</v>
+        <v>139553</v>
       </c>
       <c r="E262" t="n">
-        <v>8.73</v>
+        <v>1300.72</v>
       </c>
       <c r="F262" t="n">
-        <v>0</v>
+        <v>1300.72</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -6743,10 +6743,10 @@
         <v>46247</v>
       </c>
       <c r="D263" t="n">
-        <v>789525</v>
+        <v>794671</v>
       </c>
       <c r="E263" t="n">
-        <v>8.949999999999999</v>
+        <v>759.41</v>
       </c>
       <c r="F263" t="n">
         <v>0</v>
@@ -6890,10 +6890,10 @@
         <v>789525</v>
       </c>
       <c r="E269" t="n">
-        <v>12724.23</v>
+        <v>12724.28</v>
       </c>
       <c r="F269" t="n">
-        <v>3499.6</v>
+        <v>3621.64</v>
       </c>
     </row>
     <row r="270">
@@ -6914,10 +6914,10 @@
         <v>33057</v>
       </c>
       <c r="E270" t="n">
-        <v>8332.530000000001</v>
+        <v>8376.639999999999</v>
       </c>
       <c r="F270" t="n">
-        <v>4615.24</v>
+        <v>4714.37</v>
       </c>
     </row>
     <row r="271">
@@ -6938,7 +6938,7 @@
         <v>47252</v>
       </c>
       <c r="E271" t="n">
-        <v>34034.89</v>
+        <v>35445.99</v>
       </c>
       <c r="F271" t="n">
         <v>2156.1</v>
@@ -6962,7 +6962,7 @@
         <v>789525</v>
       </c>
       <c r="E272" t="n">
-        <v>4259.72</v>
+        <v>4346.59</v>
       </c>
       <c r="F272" t="n">
         <v>733.89</v>
@@ -6986,7 +6986,7 @@
         <v>30791</v>
       </c>
       <c r="E273" t="n">
-        <v>10446.27</v>
+        <v>10570.61</v>
       </c>
       <c r="F273" t="n">
         <v>0</v>
@@ -7154,7 +7154,7 @@
         <v>789603</v>
       </c>
       <c r="E280" t="n">
-        <v>129342.5</v>
+        <v>136414.08</v>
       </c>
       <c r="F280" t="n">
         <v>41155.22</v>
@@ -7274,7 +7274,7 @@
         <v>30307</v>
       </c>
       <c r="E285" t="n">
-        <v>23492.6</v>
+        <v>24295.96</v>
       </c>
       <c r="F285" t="n">
         <v>0</v>
@@ -7370,10 +7370,10 @@
         <v>30083</v>
       </c>
       <c r="E289" t="n">
-        <v>6171.14</v>
+        <v>6171.3</v>
       </c>
       <c r="F289" t="n">
-        <v>906.54</v>
+        <v>1901.21</v>
       </c>
     </row>
     <row r="290">
@@ -7439,13 +7439,13 @@
         <v>46247</v>
       </c>
       <c r="D292" t="n">
-        <v>33057</v>
+        <v>33928</v>
       </c>
       <c r="E292" t="n">
-        <v>28347.46</v>
+        <v>6045.77</v>
       </c>
       <c r="F292" t="n">
-        <v>261.95</v>
+        <v>94.43000000000001</v>
       </c>
     </row>
     <row r="293">
@@ -7463,13 +7463,13 @@
         <v>46247</v>
       </c>
       <c r="D293" t="n">
-        <v>33928</v>
+        <v>33057</v>
       </c>
       <c r="E293" t="n">
-        <v>6045.77</v>
+        <v>28347.46</v>
       </c>
       <c r="F293" t="n">
-        <v>94.43000000000001</v>
+        <v>261.95</v>
       </c>
     </row>
     <row r="294">
@@ -7586,7 +7586,7 @@
         <v>33286</v>
       </c>
       <c r="E298" t="n">
-        <v>567.27</v>
+        <v>639.23</v>
       </c>
       <c r="F298" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 13:45:05
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -821,7 +821,7 @@
         <v>20958.15</v>
       </c>
       <c r="F16" t="n">
-        <v>1510.55</v>
+        <v>1559.45</v>
       </c>
     </row>
     <row r="17">
@@ -842,10 +842,10 @@
         <v>47252</v>
       </c>
       <c r="E17" t="n">
-        <v>47431.93</v>
+        <v>47878.22</v>
       </c>
       <c r="F17" t="n">
-        <v>2806.49</v>
+        <v>2898.9</v>
       </c>
     </row>
     <row r="18">
@@ -890,7 +890,7 @@
         <v>793718</v>
       </c>
       <c r="E19" t="n">
-        <v>142.34</v>
+        <v>168.83</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -1370,7 +1370,7 @@
         <v>30307</v>
       </c>
       <c r="E39" t="n">
-        <v>42391.12</v>
+        <v>44505.9</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
@@ -1826,10 +1826,10 @@
         <v>31267</v>
       </c>
       <c r="E58" t="n">
-        <v>826.95</v>
+        <v>827.17</v>
       </c>
       <c r="F58" t="n">
-        <v>0</v>
+        <v>315.17</v>
       </c>
     </row>
     <row r="59">
@@ -1850,7 +1850,7 @@
         <v>30307</v>
       </c>
       <c r="E59" t="n">
-        <v>10558.49</v>
+        <v>10638.41</v>
       </c>
       <c r="F59" t="n">
         <v>0</v>
@@ -2042,10 +2042,10 @@
         <v>789661</v>
       </c>
       <c r="E67" t="n">
-        <v>899.72</v>
+        <v>900.17</v>
       </c>
       <c r="F67" t="n">
-        <v>0</v>
+        <v>812.33</v>
       </c>
     </row>
     <row r="68">
@@ -2282,7 +2282,7 @@
         <v>47252</v>
       </c>
       <c r="E77" t="n">
-        <v>121155.37</v>
+        <v>120316.5</v>
       </c>
       <c r="F77" t="n">
         <v>155.27</v>
@@ -2354,7 +2354,7 @@
         <v>30791</v>
       </c>
       <c r="E80" t="n">
-        <v>3305.86</v>
+        <v>3968.36</v>
       </c>
       <c r="F80" t="n">
         <v>0</v>
@@ -2426,7 +2426,7 @@
         <v>789525</v>
       </c>
       <c r="E83" t="n">
-        <v>3241.61</v>
+        <v>3677.5</v>
       </c>
       <c r="F83" t="n">
         <v>0</v>
@@ -2618,10 +2618,10 @@
         <v>47252</v>
       </c>
       <c r="E91" t="n">
-        <v>62800.03</v>
+        <v>62800.27</v>
       </c>
       <c r="F91" t="n">
-        <v>58270.83</v>
+        <v>59112.84</v>
       </c>
     </row>
     <row r="92">
@@ -2642,10 +2642,10 @@
         <v>789228</v>
       </c>
       <c r="E92" t="n">
-        <v>9531.120000000001</v>
+        <v>9531.17</v>
       </c>
       <c r="F92" t="n">
-        <v>9500.35</v>
+        <v>9676.299999999999</v>
       </c>
     </row>
     <row r="93">
@@ -2714,7 +2714,7 @@
         <v>794671</v>
       </c>
       <c r="E95" t="n">
-        <v>1620.58</v>
+        <v>1756.76</v>
       </c>
       <c r="F95" t="n">
         <v>0</v>
@@ -2762,7 +2762,7 @@
         <v>33286</v>
       </c>
       <c r="E97" t="n">
-        <v>1622.97</v>
+        <v>1652.54</v>
       </c>
       <c r="F97" t="n">
         <v>0</v>
@@ -2882,7 +2882,7 @@
         <v>30083</v>
       </c>
       <c r="E102" t="n">
-        <v>3304.04</v>
+        <v>3548.92</v>
       </c>
       <c r="F102" t="n">
         <v>0</v>
@@ -2930,7 +2930,7 @@
         <v>789603</v>
       </c>
       <c r="E104" t="n">
-        <v>56950.14</v>
+        <v>57071.2</v>
       </c>
       <c r="F104" t="n">
         <v>1811.65</v>
@@ -2978,10 +2978,10 @@
         <v>789603</v>
       </c>
       <c r="E106" t="n">
-        <v>46515.54</v>
+        <v>46516.44</v>
       </c>
       <c r="F106" t="n">
-        <v>42257.24</v>
+        <v>44828.27</v>
       </c>
     </row>
     <row r="107">
@@ -3050,7 +3050,7 @@
         <v>30307</v>
       </c>
       <c r="E109" t="n">
-        <v>38056.69</v>
+        <v>38131.65</v>
       </c>
       <c r="F109" t="n">
         <v>0</v>
@@ -3218,10 +3218,10 @@
         <v>47252</v>
       </c>
       <c r="E116" t="n">
-        <v>21556.35</v>
+        <v>21568.39</v>
       </c>
       <c r="F116" t="n">
-        <v>0</v>
+        <v>13086.36</v>
       </c>
     </row>
     <row r="117">
@@ -3602,7 +3602,7 @@
         <v>795345</v>
       </c>
       <c r="E132" t="n">
-        <v>1887.45</v>
+        <v>2197.5</v>
       </c>
       <c r="F132" t="n">
         <v>0</v>
@@ -3626,7 +3626,7 @@
         <v>139553</v>
       </c>
       <c r="E133" t="n">
-        <v>5517.68</v>
+        <v>7747.28</v>
       </c>
       <c r="F133" t="n">
         <v>0</v>
@@ -4082,10 +4082,10 @@
         <v>30791</v>
       </c>
       <c r="E152" t="n">
-        <v>18310.77</v>
+        <v>18311.77</v>
       </c>
       <c r="F152" t="n">
-        <v>3069.91</v>
+        <v>4798.05</v>
       </c>
     </row>
     <row r="153">
@@ -4250,7 +4250,7 @@
         <v>30791</v>
       </c>
       <c r="E159" t="n">
-        <v>5743.9</v>
+        <v>6015.6</v>
       </c>
       <c r="F159" t="n">
         <v>0</v>
@@ -4418,7 +4418,7 @@
         <v>795345</v>
       </c>
       <c r="E166" t="n">
-        <v>422.09</v>
+        <v>612.89</v>
       </c>
       <c r="F166" t="n">
         <v>0</v>
@@ -5357,7 +5357,7 @@
         <v>1804.46</v>
       </c>
       <c r="F205" t="n">
-        <v>20.25</v>
+        <v>48.55</v>
       </c>
     </row>
     <row r="206">
@@ -5522,10 +5522,10 @@
         <v>33928</v>
       </c>
       <c r="E212" t="n">
-        <v>41656.17</v>
+        <v>41656.19</v>
       </c>
       <c r="F212" t="n">
-        <v>36445.09</v>
+        <v>36512.93</v>
       </c>
     </row>
     <row r="213">
@@ -5642,7 +5642,7 @@
         <v>47252</v>
       </c>
       <c r="E217" t="n">
-        <v>9504.6</v>
+        <v>10068.56</v>
       </c>
       <c r="F217" t="n">
         <v>0</v>
@@ -5738,7 +5738,7 @@
         <v>792121</v>
       </c>
       <c r="E221" t="n">
-        <v>4506.03</v>
+        <v>4741.92</v>
       </c>
       <c r="F221" t="n">
         <v>0</v>
@@ -6002,7 +6002,7 @@
         <v>47252</v>
       </c>
       <c r="E232" t="n">
-        <v>3084</v>
+        <v>3204.11</v>
       </c>
       <c r="F232" t="n">
         <v>0</v>
@@ -6242,7 +6242,7 @@
         <v>794671</v>
       </c>
       <c r="E242" t="n">
-        <v>717.85</v>
+        <v>786.53</v>
       </c>
       <c r="F242" t="n">
         <v>0</v>
@@ -6338,7 +6338,7 @@
         <v>47252</v>
       </c>
       <c r="E246" t="n">
-        <v>2997.97</v>
+        <v>3190.25</v>
       </c>
       <c r="F246" t="n">
         <v>0</v>
@@ -6434,10 +6434,10 @@
         <v>33286</v>
       </c>
       <c r="E250" t="n">
-        <v>395.21</v>
+        <v>416.07</v>
       </c>
       <c r="F250" t="n">
-        <v>0</v>
+        <v>98.14</v>
       </c>
     </row>
     <row r="251">
@@ -6458,7 +6458,7 @@
         <v>139553</v>
       </c>
       <c r="E251" t="n">
-        <v>1567.26</v>
+        <v>1958.34</v>
       </c>
       <c r="F251" t="n">
         <v>0</v>
@@ -6629,7 +6629,7 @@
         <v>12050.63</v>
       </c>
       <c r="F258" t="n">
-        <v>0</v>
+        <v>1019.87</v>
       </c>
     </row>
     <row r="259">
@@ -7130,10 +7130,10 @@
         <v>47252</v>
       </c>
       <c r="E279" t="n">
-        <v>63926.73</v>
+        <v>63927.7</v>
       </c>
       <c r="F279" t="n">
-        <v>32591.8</v>
+        <v>36232.01</v>
       </c>
     </row>
     <row r="280">
@@ -7202,7 +7202,7 @@
         <v>33057</v>
       </c>
       <c r="E282" t="n">
-        <v>444.71</v>
+        <v>1644.05</v>
       </c>
       <c r="F282" t="n">
         <v>0</v>
@@ -7226,7 +7226,7 @@
         <v>33286</v>
       </c>
       <c r="E283" t="n">
-        <v>896.16</v>
+        <v>925.5700000000001</v>
       </c>
       <c r="F283" t="n">
         <v>0</v>
@@ -7250,7 +7250,7 @@
         <v>31267</v>
       </c>
       <c r="E284" t="n">
-        <v>5190.54</v>
+        <v>5283.69</v>
       </c>
       <c r="F284" t="n">
         <v>0</v>
@@ -7706,10 +7706,10 @@
         <v>33286</v>
       </c>
       <c r="E303" t="n">
-        <v>14703.07</v>
+        <v>14703.31</v>
       </c>
       <c r="F303" t="n">
-        <v>9667.18</v>
+        <v>10511.23</v>
       </c>
     </row>
     <row r="304">
@@ -7754,10 +7754,10 @@
         <v>33286</v>
       </c>
       <c r="E305" t="n">
-        <v>2568.65</v>
+        <v>2568.69</v>
       </c>
       <c r="F305" t="n">
-        <v>148.83</v>
+        <v>232.55</v>
       </c>
     </row>
     <row r="306">
@@ -7874,7 +7874,7 @@
         <v>33057</v>
       </c>
       <c r="E310" t="n">
-        <v>497.83</v>
+        <v>604.34</v>
       </c>
       <c r="F310" t="n">
         <v>0</v>
@@ -7898,7 +7898,7 @@
         <v>793718</v>
       </c>
       <c r="E311" t="n">
-        <v>364.78</v>
+        <v>496.15</v>
       </c>
       <c r="F311" t="n">
         <v>0</v>
@@ -8138,7 +8138,7 @@
         <v>790595</v>
       </c>
       <c r="E321" t="n">
-        <v>431.22</v>
+        <v>672.61</v>
       </c>
       <c r="F321" t="n">
         <v>0</v>
@@ -8162,7 +8162,7 @@
         <v>139553</v>
       </c>
       <c r="E322" t="n">
-        <v>407.92</v>
+        <v>1427.72</v>
       </c>
       <c r="F322" t="n">
         <v>0</v>
@@ -8282,10 +8282,10 @@
         <v>792121</v>
       </c>
       <c r="E327" t="n">
-        <v>1963.26</v>
+        <v>2333.62</v>
       </c>
       <c r="F327" t="n">
-        <v>0</v>
+        <v>390.94</v>
       </c>
     </row>
     <row r="328">
@@ -8882,7 +8882,7 @@
         <v>33286</v>
       </c>
       <c r="E352" t="n">
-        <v>656.62</v>
+        <v>704.76</v>
       </c>
       <c r="F352" t="n">
         <v>0</v>
@@ -9173,28 +9173,28 @@
         <v>3580.92</v>
       </c>
       <c r="F364" t="n">
-        <v>46.6</v>
+        <v>93.09</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C365" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="D365" t="n">
-        <v>789603</v>
+        <v>792141</v>
       </c>
       <c r="E365" t="n">
-        <v>100147.54</v>
+        <v>18977.41</v>
       </c>
       <c r="F365" t="n">
         <v>0</v>
@@ -9212,46 +9212,46 @@
         </is>
       </c>
       <c r="C366" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D366" t="n">
-        <v>30307</v>
+        <v>789603</v>
       </c>
       <c r="E366" t="n">
-        <v>84703.44</v>
+        <v>100147.54</v>
       </c>
       <c r="F366" t="n">
-        <v>31024.48</v>
+        <v>0</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t xml:space="preserve">FRANCISCO CHAGAS </t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C367" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D367" t="n">
-        <v>33057</v>
+        <v>30307</v>
       </c>
       <c r="E367" t="n">
-        <v>22.32</v>
+        <v>84703.44</v>
       </c>
       <c r="F367" t="n">
-        <v>22.32</v>
+        <v>31024.48</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
@@ -9263,19 +9263,19 @@
         <v>46247</v>
       </c>
       <c r="D368" t="n">
-        <v>33928</v>
+        <v>33057</v>
       </c>
       <c r="E368" t="n">
-        <v>9.529999999999999</v>
+        <v>22.32</v>
       </c>
       <c r="F368" t="n">
-        <v>9.529999999999999</v>
+        <v>22.32</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
@@ -9284,16 +9284,16 @@
         </is>
       </c>
       <c r="C369" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D369" t="n">
-        <v>789525</v>
+        <v>33928</v>
       </c>
       <c r="E369" t="n">
-        <v>5.89</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="F369" t="n">
-        <v>5.89</v>
+        <v>9.529999999999999</v>
       </c>
     </row>
     <row r="370">
@@ -9311,37 +9311,37 @@
         <v>46248</v>
       </c>
       <c r="D370" t="n">
-        <v>792121</v>
+        <v>789525</v>
       </c>
       <c r="E370" t="n">
-        <v>39.26</v>
+        <v>5.89</v>
       </c>
       <c r="F370" t="n">
-        <v>0</v>
+        <v>5.89</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">FRANCISCO CHAGAS </t>
         </is>
       </c>
       <c r="C371" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D371" t="n">
-        <v>47252</v>
+        <v>792121</v>
       </c>
       <c r="E371" t="n">
-        <v>30676.09</v>
+        <v>39.26</v>
       </c>
       <c r="F371" t="n">
-        <v>25229.07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="372">
@@ -9359,34 +9359,34 @@
         <v>46247</v>
       </c>
       <c r="D372" t="n">
-        <v>792141</v>
+        <v>47252</v>
       </c>
       <c r="E372" t="n">
-        <v>414.3</v>
+        <v>30676.09</v>
       </c>
       <c r="F372" t="n">
-        <v>0</v>
+        <v>25229.07</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="C373" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D373" t="n">
-        <v>793718</v>
+        <v>792141</v>
       </c>
       <c r="E373" t="n">
-        <v>957.1900000000001</v>
+        <v>414.3</v>
       </c>
       <c r="F373" t="n">
         <v>0</v>
@@ -9404,16 +9404,16 @@
         </is>
       </c>
       <c r="C374" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D374" t="n">
-        <v>793186</v>
+        <v>793718</v>
       </c>
       <c r="E374" t="n">
-        <v>2220.5</v>
+        <v>957.1900000000001</v>
       </c>
       <c r="F374" t="n">
-        <v>2220.51</v>
+        <v>0</v>
       </c>
     </row>
     <row r="375">
@@ -9428,40 +9428,40 @@
         </is>
       </c>
       <c r="C375" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D375" t="n">
-        <v>30307</v>
+        <v>793186</v>
       </c>
       <c r="E375" t="n">
-        <v>905.8200000000001</v>
+        <v>2220.5</v>
       </c>
       <c r="F375" t="n">
-        <v>0</v>
+        <v>2220.51</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C376" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D376" t="n">
-        <v>792141</v>
+        <v>30307</v>
       </c>
       <c r="E376" t="n">
-        <v>2231.26</v>
+        <v>905.8200000000001</v>
       </c>
       <c r="F376" t="n">
-        <v>5721.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="377">
@@ -9472,7 +9472,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C377" s="2" t="n">
@@ -9482,34 +9482,34 @@
         <v>792141</v>
       </c>
       <c r="E377" t="n">
-        <v>14441.42</v>
+        <v>2231.26</v>
       </c>
       <c r="F377" t="n">
-        <v>13727.64</v>
+        <v>5721.09</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="C378" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D378" t="n">
-        <v>793718</v>
+        <v>792141</v>
       </c>
       <c r="E378" t="n">
-        <v>4485.27</v>
+        <v>14441.42</v>
       </c>
       <c r="F378" t="n">
-        <v>3053.19</v>
+        <v>13727.64</v>
       </c>
     </row>
     <row r="379">
@@ -9527,13 +9527,13 @@
         <v>46247</v>
       </c>
       <c r="D379" t="n">
-        <v>789228</v>
+        <v>793718</v>
       </c>
       <c r="E379" t="n">
-        <v>4036.35</v>
+        <v>4485.27</v>
       </c>
       <c r="F379" t="n">
-        <v>3098.15</v>
+        <v>3053.19</v>
       </c>
     </row>
     <row r="380">
@@ -9544,68 +9544,68 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="C380" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D380" t="n">
-        <v>792141</v>
+        <v>789228</v>
       </c>
       <c r="E380" t="n">
-        <v>2341.6</v>
+        <v>4036.35</v>
       </c>
       <c r="F380" t="n">
-        <v>2029.2</v>
+        <v>3098.15</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>SALDANHA JUNIOR</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C381" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D381" t="n">
-        <v>795345</v>
+        <v>792141</v>
       </c>
       <c r="E381" t="n">
-        <v>2215.52</v>
+        <v>2341.6</v>
       </c>
       <c r="F381" t="n">
-        <v>0</v>
+        <v>2029.2</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>SALDANHA JUNIOR</t>
         </is>
       </c>
       <c r="C382" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D382" t="n">
-        <v>789603</v>
+        <v>795345</v>
       </c>
       <c r="E382" t="n">
-        <v>42.91</v>
+        <v>2215.52</v>
       </c>
       <c r="F382" t="n">
-        <v>42.91</v>
+        <v>0</v>
       </c>
     </row>
     <row r="383">
@@ -9620,64 +9620,64 @@
         </is>
       </c>
       <c r="C383" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D383" t="n">
-        <v>792121</v>
+        <v>789603</v>
       </c>
       <c r="E383" t="n">
-        <v>70.73</v>
+        <v>42.91</v>
       </c>
       <c r="F383" t="n">
-        <v>0</v>
+        <v>42.91</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C384" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D384" t="n">
-        <v>30307</v>
+        <v>792121</v>
       </c>
       <c r="E384" t="n">
-        <v>113204.88</v>
+        <v>70.73</v>
       </c>
       <c r="F384" t="n">
-        <v>110953.72</v>
+        <v>0</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C385" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D385" t="n">
-        <v>792141</v>
+        <v>30307</v>
       </c>
       <c r="E385" t="n">
-        <v>18006.95</v>
+        <v>113204.88</v>
       </c>
       <c r="F385" t="n">
-        <v>0</v>
+        <v>110953.72</v>
       </c>
     </row>
     <row r="386">
@@ -9869,7 +9869,7 @@
         <v>250.52</v>
       </c>
       <c r="F393" t="n">
-        <v>0</v>
+        <v>150.45</v>
       </c>
     </row>
     <row r="394">
@@ -10154,7 +10154,7 @@
         <v>30083</v>
       </c>
       <c r="E405" t="n">
-        <v>3657.95</v>
+        <v>5076.2</v>
       </c>
       <c r="F405" t="n">
         <v>0</v>
@@ -10250,7 +10250,7 @@
         <v>47252</v>
       </c>
       <c r="E409" t="n">
-        <v>17058.75</v>
+        <v>17428.8</v>
       </c>
       <c r="F409" t="n">
         <v>0</v>
@@ -10637,7 +10637,7 @@
         <v>35134.47</v>
       </c>
       <c r="F425" t="n">
-        <v>31415.07</v>
+        <v>32408.05</v>
       </c>
     </row>
     <row r="426">
@@ -10682,10 +10682,10 @@
         <v>47252</v>
       </c>
       <c r="E427" t="n">
-        <v>35845.05</v>
+        <v>36042.61</v>
       </c>
       <c r="F427" t="n">
-        <v>6031.53</v>
+        <v>7952.38</v>
       </c>
     </row>
     <row r="428">
@@ -10994,7 +10994,7 @@
         <v>139553</v>
       </c>
       <c r="E440" t="n">
-        <v>2526.44</v>
+        <v>4770</v>
       </c>
       <c r="F440" t="n">
         <v>0</v>
@@ -11450,10 +11450,10 @@
         <v>33928</v>
       </c>
       <c r="E459" t="n">
-        <v>1120.01</v>
+        <v>1120.03</v>
       </c>
       <c r="F459" t="n">
-        <v>0</v>
+        <v>50.81</v>
       </c>
     </row>
     <row r="460">
@@ -11570,7 +11570,7 @@
         <v>794671</v>
       </c>
       <c r="E464" t="n">
-        <v>1318.75</v>
+        <v>1656.21</v>
       </c>
       <c r="F464" t="n">
         <v>0</v>
@@ -11594,10 +11594,10 @@
         <v>33057</v>
       </c>
       <c r="E465" t="n">
-        <v>687.21</v>
+        <v>687.36</v>
       </c>
       <c r="F465" t="n">
-        <v>0</v>
+        <v>408.35</v>
       </c>
     </row>
     <row r="466">
@@ -11642,7 +11642,7 @@
         <v>30083</v>
       </c>
       <c r="E467" t="n">
-        <v>828.02</v>
+        <v>1154.13</v>
       </c>
       <c r="F467" t="n">
         <v>0</v>
@@ -11738,7 +11738,7 @@
         <v>792121</v>
       </c>
       <c r="E471" t="n">
-        <v>5877.79</v>
+        <v>5909.96</v>
       </c>
       <c r="F471" t="n">
         <v>0</v>
@@ -11762,7 +11762,7 @@
         <v>30307</v>
       </c>
       <c r="E472" t="n">
-        <v>37235.98</v>
+        <v>39681.38</v>
       </c>
       <c r="F472" t="n">
         <v>0</v>
@@ -11933,7 +11933,7 @@
         <v>1040.49</v>
       </c>
       <c r="F479" t="n">
-        <v>0</v>
+        <v>38.01</v>
       </c>
     </row>
     <row r="480">
@@ -11978,7 +11978,7 @@
         <v>33928</v>
       </c>
       <c r="E481" t="n">
-        <v>667.52</v>
+        <v>1585.92</v>
       </c>
       <c r="F481" t="n">
         <v>0</v>
@@ -12410,10 +12410,10 @@
         <v>789525</v>
       </c>
       <c r="E499" t="n">
-        <v>13140.31</v>
+        <v>13140.46</v>
       </c>
       <c r="F499" t="n">
-        <v>8438.02</v>
+        <v>8939.540000000001</v>
       </c>
     </row>
     <row r="500">
@@ -12458,10 +12458,10 @@
         <v>789525</v>
       </c>
       <c r="E501" t="n">
-        <v>3029.03</v>
+        <v>3029.44</v>
       </c>
       <c r="F501" t="n">
-        <v>135.24</v>
+        <v>622.8200000000001</v>
       </c>
     </row>
     <row r="502">
@@ -12794,7 +12794,7 @@
         <v>789603</v>
       </c>
       <c r="E515" t="n">
-        <v>76780.34</v>
+        <v>80023.06</v>
       </c>
       <c r="F515" t="n">
         <v>0</v>
@@ -12962,7 +12962,7 @@
         <v>789603</v>
       </c>
       <c r="E522" t="n">
-        <v>20371.16</v>
+        <v>21826.73</v>
       </c>
       <c r="F522" t="n">
         <v>0</v>
@@ -13058,7 +13058,7 @@
         <v>31267</v>
       </c>
       <c r="E526" t="n">
-        <v>13212.76</v>
+        <v>16680.41</v>
       </c>
       <c r="F526" t="n">
         <v>0</v>
@@ -13106,7 +13106,7 @@
         <v>33928</v>
       </c>
       <c r="E528" t="n">
-        <v>2601.81</v>
+        <v>3008.54</v>
       </c>
       <c r="F528" t="n">
         <v>0</v>
@@ -13202,10 +13202,10 @@
         <v>30083</v>
       </c>
       <c r="E532" t="n">
-        <v>8259.790000000001</v>
+        <v>8260.059999999999</v>
       </c>
       <c r="F532" t="n">
-        <v>5728.65</v>
+        <v>7464.44</v>
       </c>
     </row>
     <row r="533">
@@ -13250,7 +13250,7 @@
         <v>789228</v>
       </c>
       <c r="E534" t="n">
-        <v>553.21</v>
+        <v>688.49</v>
       </c>
       <c r="F534" t="n">
         <v>0</v>
@@ -13346,10 +13346,10 @@
         <v>33928</v>
       </c>
       <c r="E538" t="n">
-        <v>12439.1</v>
+        <v>12440</v>
       </c>
       <c r="F538" t="n">
-        <v>6698.43</v>
+        <v>8303.040000000001</v>
       </c>
     </row>
     <row r="539">
@@ -13445,7 +13445,7 @@
         <v>446.37</v>
       </c>
       <c r="F542" t="n">
-        <v>281.67</v>
+        <v>446.37</v>
       </c>
     </row>
     <row r="543">

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 14:15:07
</commit_message>
<xml_diff>
--- a/data/fat_total_day.xlsx
+++ b/data/fat_total_day.xlsx
@@ -1709,7 +1709,7 @@
         <v>4828.07</v>
       </c>
       <c r="F53" t="n">
-        <v>1710.15</v>
+        <v>2514.35</v>
       </c>
     </row>
     <row r="54">
@@ -1778,7 +1778,7 @@
         <v>31267</v>
       </c>
       <c r="E56" t="n">
-        <v>16272.52</v>
+        <v>16452.48</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
@@ -1826,7 +1826,7 @@
         <v>31267</v>
       </c>
       <c r="E58" t="n">
-        <v>849.88</v>
+        <v>866.17</v>
       </c>
       <c r="F58" t="n">
         <v>315.17</v>
@@ -1973,7 +1973,7 @@
         <v>18470.52</v>
       </c>
       <c r="F64" t="n">
-        <v>14981.95</v>
+        <v>16447.21</v>
       </c>
     </row>
     <row r="65">
@@ -1994,10 +1994,10 @@
         <v>795345</v>
       </c>
       <c r="E65" t="n">
-        <v>1199.58</v>
+        <v>1380.76</v>
       </c>
       <c r="F65" t="n">
-        <v>0</v>
+        <v>309.8</v>
       </c>
     </row>
     <row r="66">
@@ -2282,7 +2282,7 @@
         <v>47252</v>
       </c>
       <c r="E77" t="n">
-        <v>126198.99</v>
+        <v>173109.03</v>
       </c>
       <c r="F77" t="n">
         <v>155.27</v>
@@ -2402,7 +2402,7 @@
         <v>33057</v>
       </c>
       <c r="E82" t="n">
-        <v>24629.92</v>
+        <v>24098.31</v>
       </c>
       <c r="F82" t="n">
         <v>0</v>
@@ -2762,7 +2762,7 @@
         <v>33286</v>
       </c>
       <c r="E97" t="n">
-        <v>1982.3</v>
+        <v>2060.19</v>
       </c>
       <c r="F97" t="n">
         <v>0</v>
@@ -2795,25 +2795,25 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D99" t="n">
-        <v>789525</v>
+        <v>30083</v>
       </c>
       <c r="E99" t="n">
-        <v>2635</v>
+        <v>4338.1</v>
       </c>
       <c r="F99" t="n">
-        <v>3671.43</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -2831,58 +2831,58 @@
         <v>46247</v>
       </c>
       <c r="D100" t="n">
-        <v>139553</v>
+        <v>789525</v>
       </c>
       <c r="E100" t="n">
-        <v>1295.52</v>
+        <v>2635</v>
       </c>
       <c r="F100" t="n">
-        <v>1295.52</v>
+        <v>3671.43</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>LUIS REGINALDO ALMEIDA GOMES</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D101" t="n">
-        <v>30307</v>
+        <v>139553</v>
       </c>
       <c r="E101" t="n">
-        <v>2807.48</v>
+        <v>1295.52</v>
       </c>
       <c r="F101" t="n">
-        <v>0</v>
+        <v>1295.52</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>JOSE FLAVIO DE SA AZEVEDO</t>
+          <t>LUIS REGINALDO ALMEIDA GOMES</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D102" t="n">
-        <v>790595</v>
+        <v>30307</v>
       </c>
       <c r="E102" t="n">
-        <v>393.85</v>
+        <v>2807.48</v>
       </c>
       <c r="F102" t="n">
         <v>0</v>
@@ -2896,17 +2896,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>JOSE FLAVIO DE SA AZEVEDO</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="D103" t="n">
-        <v>30083</v>
+        <v>790595</v>
       </c>
       <c r="E103" t="n">
-        <v>3548.92</v>
+        <v>378.98</v>
       </c>
       <c r="F103" t="n">
         <v>0</v>
@@ -2954,10 +2954,10 @@
         <v>789603</v>
       </c>
       <c r="E105" t="n">
-        <v>57071.2</v>
+        <v>58816.26</v>
       </c>
       <c r="F105" t="n">
-        <v>1811.65</v>
+        <v>3170.89</v>
       </c>
     </row>
     <row r="106">
@@ -3074,7 +3074,7 @@
         <v>30307</v>
       </c>
       <c r="E110" t="n">
-        <v>38371.41</v>
+        <v>39766.89</v>
       </c>
       <c r="F110" t="n">
         <v>0</v>
@@ -4010,7 +4010,7 @@
         <v>30307</v>
       </c>
       <c r="E149" t="n">
-        <v>35877.32</v>
+        <v>36288.44</v>
       </c>
       <c r="F149" t="n">
         <v>0</v>
@@ -4130,10 +4130,10 @@
         <v>30791</v>
       </c>
       <c r="E154" t="n">
-        <v>18311.77</v>
+        <v>18405.75</v>
       </c>
       <c r="F154" t="n">
-        <v>4495.31</v>
+        <v>5456.92</v>
       </c>
     </row>
     <row r="155">
@@ -4298,7 +4298,7 @@
         <v>30791</v>
       </c>
       <c r="E161" t="n">
-        <v>7369.27</v>
+        <v>9652.25</v>
       </c>
       <c r="F161" t="n">
         <v>0</v>
@@ -4331,25 +4331,25 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C163" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D163" t="n">
-        <v>33928</v>
+        <v>795345</v>
       </c>
       <c r="E163" t="n">
-        <v>3795.93</v>
+        <v>936.95</v>
       </c>
       <c r="F163" t="n">
-        <v>4424.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="164">
@@ -4367,13 +4367,13 @@
         <v>46247</v>
       </c>
       <c r="D164" t="n">
-        <v>793718</v>
+        <v>33928</v>
       </c>
       <c r="E164" t="n">
-        <v>833.39</v>
+        <v>3795.93</v>
       </c>
       <c r="F164" t="n">
-        <v>534.74</v>
+        <v>4424.01</v>
       </c>
     </row>
     <row r="165">
@@ -4388,37 +4388,37 @@
         </is>
       </c>
       <c r="C165" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D165" t="n">
-        <v>33928</v>
+        <v>793718</v>
       </c>
       <c r="E165" t="n">
-        <v>3224.06</v>
+        <v>833.39</v>
       </c>
       <c r="F165" t="n">
-        <v>0</v>
+        <v>534.74</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C166" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="D166" t="n">
-        <v>30083</v>
+        <v>33928</v>
       </c>
       <c r="E166" t="n">
-        <v>128.27</v>
+        <v>3224.06</v>
       </c>
       <c r="F166" t="n">
         <v>0</v>
@@ -4427,49 +4427,49 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="C167" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D167" t="n">
-        <v>139553</v>
+        <v>30083</v>
       </c>
       <c r="E167" t="n">
-        <v>611.88</v>
+        <v>128.27</v>
       </c>
       <c r="F167" t="n">
-        <v>611.88</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C168" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D168" t="n">
-        <v>794671</v>
+        <v>139553</v>
       </c>
       <c r="E168" t="n">
-        <v>2639.83</v>
+        <v>611.88</v>
       </c>
       <c r="F168" t="n">
-        <v>0</v>
+        <v>611.88</v>
       </c>
     </row>
     <row r="169">
@@ -4487,10 +4487,10 @@
         <v>46248</v>
       </c>
       <c r="D169" t="n">
-        <v>795345</v>
+        <v>794671</v>
       </c>
       <c r="E169" t="n">
-        <v>612.89</v>
+        <v>2523.93</v>
       </c>
       <c r="F169" t="n">
         <v>0</v>
@@ -4514,7 +4514,7 @@
         <v>789603</v>
       </c>
       <c r="E170" t="n">
-        <v>36686.97</v>
+        <v>57997.97</v>
       </c>
       <c r="F170" t="n">
         <v>0</v>
@@ -4586,10 +4586,10 @@
         <v>139553</v>
       </c>
       <c r="E173" t="n">
-        <v>22171.46</v>
+        <v>22171.53</v>
       </c>
       <c r="F173" t="n">
-        <v>12304.67</v>
+        <v>13769.84</v>
       </c>
     </row>
     <row r="174">
@@ -5426,7 +5426,7 @@
         <v>33928</v>
       </c>
       <c r="E208" t="n">
-        <v>1804.46</v>
+        <v>4033.51</v>
       </c>
       <c r="F208" t="n">
         <v>48.55</v>
@@ -5666,7 +5666,7 @@
         <v>33057</v>
       </c>
       <c r="E218" t="n">
-        <v>861.27</v>
+        <v>1533.09</v>
       </c>
       <c r="F218" t="n">
         <v>-68.19</v>
@@ -5714,7 +5714,7 @@
         <v>47252</v>
       </c>
       <c r="E220" t="n">
-        <v>11456.61</v>
+        <v>11633.96</v>
       </c>
       <c r="F220" t="n">
         <v>0</v>
@@ -5747,25 +5747,25 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C222" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D222" t="n">
-        <v>33286</v>
+        <v>792121</v>
       </c>
       <c r="E222" t="n">
-        <v>11455.03</v>
+        <v>4760.5</v>
       </c>
       <c r="F222" t="n">
-        <v>11320.79</v>
+        <v>0</v>
       </c>
     </row>
     <row r="223">
@@ -5783,61 +5783,61 @@
         <v>46247</v>
       </c>
       <c r="D223" t="n">
-        <v>30791</v>
+        <v>33286</v>
       </c>
       <c r="E223" t="n">
-        <v>36608.96</v>
+        <v>11455.03</v>
       </c>
       <c r="F223" t="n">
-        <v>22132.9</v>
+        <v>11320.79</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C224" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D224" t="n">
-        <v>30083</v>
+        <v>30791</v>
       </c>
       <c r="E224" t="n">
-        <v>215.6</v>
+        <v>36608.96</v>
       </c>
       <c r="F224" t="n">
-        <v>191.93</v>
+        <v>22132.9</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C225" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D225" t="n">
-        <v>792121</v>
+        <v>30083</v>
       </c>
       <c r="E225" t="n">
-        <v>4741.92</v>
+        <v>215.6</v>
       </c>
       <c r="F225" t="n">
-        <v>0</v>
+        <v>191.93</v>
       </c>
     </row>
     <row r="226">
@@ -5978,10 +5978,10 @@
         <v>30307</v>
       </c>
       <c r="E231" t="n">
-        <v>72515.74000000001</v>
+        <v>72516.32000000001</v>
       </c>
       <c r="F231" t="n">
-        <v>33665.74</v>
+        <v>40477.41</v>
       </c>
     </row>
     <row r="232">
@@ -6458,7 +6458,7 @@
         <v>33928</v>
       </c>
       <c r="E251" t="n">
-        <v>1040.51</v>
+        <v>1794.1</v>
       </c>
       <c r="F251" t="n">
         <v>0</v>
@@ -6554,7 +6554,7 @@
         <v>139553</v>
       </c>
       <c r="E255" t="n">
-        <v>1958.34</v>
+        <v>6649.42</v>
       </c>
       <c r="F255" t="n">
         <v>0</v>
@@ -6683,97 +6683,97 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C261" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="D261" t="n">
-        <v>793186</v>
+        <v>30218</v>
       </c>
       <c r="E261" t="n">
-        <v>12234.6</v>
+        <v>823.65</v>
       </c>
       <c r="F261" t="n">
-        <v>1019.87</v>
+        <v>0</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C262" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="D262" t="n">
-        <v>139553</v>
+        <v>793186</v>
       </c>
       <c r="E262" t="n">
-        <v>2603.06</v>
+        <v>12448.57</v>
       </c>
       <c r="F262" t="n">
-        <v>0</v>
+        <v>1019.87</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C263" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D263" t="n">
-        <v>792141</v>
+        <v>139553</v>
       </c>
       <c r="E263" t="n">
-        <v>140.87</v>
+        <v>2603.06</v>
       </c>
       <c r="F263" t="n">
-        <v>60.43</v>
+        <v>0</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C264" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D264" t="n">
-        <v>30218</v>
+        <v>792141</v>
       </c>
       <c r="E264" t="n">
-        <v>657.62</v>
+        <v>140.87</v>
       </c>
       <c r="F264" t="n">
-        <v>0</v>
+        <v>60.43</v>
       </c>
     </row>
     <row r="265">
@@ -7346,7 +7346,7 @@
         <v>33286</v>
       </c>
       <c r="E288" t="n">
-        <v>969.05</v>
+        <v>1091.75</v>
       </c>
       <c r="F288" t="n">
         <v>0</v>
@@ -7370,7 +7370,7 @@
         <v>31267</v>
       </c>
       <c r="E289" t="n">
-        <v>5283.69</v>
+        <v>5545.92</v>
       </c>
       <c r="F289" t="n">
         <v>0</v>
@@ -7706,7 +7706,7 @@
         <v>795345</v>
       </c>
       <c r="E303" t="n">
-        <v>1114.85</v>
+        <v>1336.45</v>
       </c>
       <c r="F303" t="n">
         <v>0</v>
@@ -8018,7 +8018,7 @@
         <v>793718</v>
       </c>
       <c r="E316" t="n">
-        <v>611.84</v>
+        <v>741.0700000000001</v>
       </c>
       <c r="F316" t="n">
         <v>0</v>
@@ -8114,7 +8114,7 @@
         <v>30083</v>
       </c>
       <c r="E320" t="n">
-        <v>7063.78</v>
+        <v>7587.76</v>
       </c>
       <c r="F320" t="n">
         <v>0</v>
@@ -8402,7 +8402,7 @@
         <v>794671</v>
       </c>
       <c r="E332" t="n">
-        <v>3487.5</v>
+        <v>3876.28</v>
       </c>
       <c r="F332" t="n">
         <v>0</v>
@@ -8426,7 +8426,7 @@
         <v>792121</v>
       </c>
       <c r="E333" t="n">
-        <v>2333.62</v>
+        <v>2593.87</v>
       </c>
       <c r="F333" t="n">
         <v>390.94</v>
@@ -8642,10 +8642,10 @@
         <v>30307</v>
       </c>
       <c r="E342" t="n">
-        <v>14236.12</v>
+        <v>16429.11</v>
       </c>
       <c r="F342" t="n">
-        <v>0</v>
+        <v>566.3200000000001</v>
       </c>
     </row>
     <row r="343">
@@ -8789,7 +8789,7 @@
         <v>11549.62</v>
       </c>
       <c r="F348" t="n">
-        <v>4255.68</v>
+        <v>8251.709999999999</v>
       </c>
     </row>
     <row r="349">
@@ -8834,7 +8834,7 @@
         <v>789525</v>
       </c>
       <c r="E350" t="n">
-        <v>1251.01</v>
+        <v>828.4400000000001</v>
       </c>
       <c r="F350" t="n">
         <v>0</v>
@@ -9530,7 +9530,7 @@
         <v>793718</v>
       </c>
       <c r="E379" t="n">
-        <v>957.1900000000001</v>
+        <v>1122.99</v>
       </c>
       <c r="F379" t="n">
         <v>0</v>
@@ -9698,7 +9698,7 @@
         <v>792121</v>
       </c>
       <c r="E386" t="n">
-        <v>8213.809999999999</v>
+        <v>8330.389999999999</v>
       </c>
       <c r="F386" t="n">
         <v>0</v>
@@ -9995,49 +9995,49 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C399" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="D399" t="n">
-        <v>792141</v>
+        <v>792121</v>
       </c>
       <c r="E399" t="n">
-        <v>250.52</v>
+        <v>354.82</v>
       </c>
       <c r="F399" t="n">
-        <v>150.45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C400" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D400" t="n">
-        <v>793718</v>
+        <v>792141</v>
       </c>
       <c r="E400" t="n">
-        <v>684.14</v>
+        <v>250.52</v>
       </c>
       <c r="F400" t="n">
-        <v>499.76</v>
+        <v>150.45</v>
       </c>
     </row>
     <row r="401">
@@ -10048,41 +10048,41 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C401" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D401" t="n">
         <v>793718</v>
       </c>
       <c r="E401" t="n">
-        <v>65.90000000000001</v>
+        <v>684.14</v>
       </c>
       <c r="F401" t="n">
-        <v>0</v>
+        <v>499.76</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C402" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="D402" t="n">
-        <v>792246</v>
+        <v>793718</v>
       </c>
       <c r="E402" t="n">
-        <v>326.6</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="F402" t="n">
         <v>0</v>
@@ -10103,10 +10103,10 @@
         <v>46248</v>
       </c>
       <c r="D403" t="n">
-        <v>792121</v>
+        <v>792246</v>
       </c>
       <c r="E403" t="n">
-        <v>38.2</v>
+        <v>326.6</v>
       </c>
       <c r="F403" t="n">
         <v>0</v>
@@ -10298,7 +10298,7 @@
         <v>30083</v>
       </c>
       <c r="E411" t="n">
-        <v>5076.2</v>
+        <v>4992.64</v>
       </c>
       <c r="F411" t="n">
         <v>0</v>
@@ -10394,7 +10394,7 @@
         <v>139553</v>
       </c>
       <c r="E415" t="n">
-        <v>323.76</v>
+        <v>16847.04</v>
       </c>
       <c r="F415" t="n">
         <v>0</v>
@@ -10418,7 +10418,7 @@
         <v>47252</v>
       </c>
       <c r="E416" t="n">
-        <v>18116.02</v>
+        <v>19164.57</v>
       </c>
       <c r="F416" t="n">
         <v>0</v>
@@ -10820,16 +10820,16 @@
         </is>
       </c>
       <c r="C433" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D433" t="n">
         <v>789603</v>
       </c>
       <c r="E433" t="n">
-        <v>69105.05</v>
+        <v>33704.21</v>
       </c>
       <c r="F433" t="n">
-        <v>36985.36</v>
+        <v>5435.62</v>
       </c>
     </row>
     <row r="434">
@@ -10844,16 +10844,16 @@
         </is>
       </c>
       <c r="C434" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D434" t="n">
-        <v>47252</v>
+        <v>789603</v>
       </c>
       <c r="E434" t="n">
-        <v>36042.61</v>
+        <v>69105.05</v>
       </c>
       <c r="F434" t="n">
-        <v>7952.38</v>
+        <v>36985.36</v>
       </c>
     </row>
     <row r="435">
@@ -10871,13 +10871,13 @@
         <v>46248</v>
       </c>
       <c r="D435" t="n">
-        <v>789603</v>
+        <v>47252</v>
       </c>
       <c r="E435" t="n">
-        <v>33703.54</v>
+        <v>45105.93</v>
       </c>
       <c r="F435" t="n">
-        <v>0</v>
+        <v>8542.780000000001</v>
       </c>
     </row>
     <row r="436">
@@ -10898,7 +10898,7 @@
         <v>789228</v>
       </c>
       <c r="E436" t="n">
-        <v>2576.69</v>
+        <v>2794.95</v>
       </c>
       <c r="F436" t="n">
         <v>141.24</v>
@@ -11018,7 +11018,7 @@
         <v>790595</v>
       </c>
       <c r="E441" t="n">
-        <v>2802.82</v>
+        <v>2847.43</v>
       </c>
       <c r="F441" t="n">
         <v>0</v>
@@ -11147,22 +11147,22 @@
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>FERNANDA DA SILVA OLIVEIRA</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C447" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="D447" t="n">
-        <v>794029</v>
+        <v>794671</v>
       </c>
       <c r="E447" t="n">
-        <v>2681.11</v>
+        <v>2248.01</v>
       </c>
       <c r="F447" t="n">
         <v>0</v>
@@ -11183,10 +11183,10 @@
         <v>46248</v>
       </c>
       <c r="D448" t="n">
-        <v>139553</v>
+        <v>794029</v>
       </c>
       <c r="E448" t="n">
-        <v>4770</v>
+        <v>2681.11</v>
       </c>
       <c r="F448" t="n">
         <v>0</v>
@@ -11195,97 +11195,97 @@
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>DIRETORIA KA BETA</t>
+          <t>FERNANDA DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="C449" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D449" t="n">
-        <v>33928</v>
+        <v>139553</v>
       </c>
       <c r="E449" t="n">
-        <v>5.82</v>
+        <v>4770</v>
       </c>
       <c r="F449" t="n">
-        <v>5.82</v>
+        <v>0</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+          <t>DIRETORIA KA BETA</t>
         </is>
       </c>
       <c r="C450" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D450" t="n">
-        <v>30083</v>
+        <v>33928</v>
       </c>
       <c r="E450" t="n">
-        <v>940.67</v>
+        <v>5.82</v>
       </c>
       <c r="F450" t="n">
-        <v>940.66</v>
+        <v>5.82</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
         </is>
       </c>
       <c r="C451" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D451" t="n">
-        <v>794671</v>
+        <v>30083</v>
       </c>
       <c r="E451" t="n">
-        <v>266.3</v>
+        <v>940.67</v>
       </c>
       <c r="F451" t="n">
-        <v>0</v>
+        <v>940.66</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C452" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D452" t="n">
-        <v>139553</v>
+        <v>794671</v>
       </c>
       <c r="E452" t="n">
-        <v>17802.62</v>
+        <v>266.3</v>
       </c>
       <c r="F452" t="n">
-        <v>19745.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="453">
@@ -11300,27 +11300,27 @@
         </is>
       </c>
       <c r="C453" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D453" t="n">
-        <v>30218</v>
+        <v>139553</v>
       </c>
       <c r="E453" t="n">
-        <v>326.86</v>
+        <v>17802.62</v>
       </c>
       <c r="F453" t="n">
-        <v>0</v>
+        <v>19745.4</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>RILARY DIENIFER TRAUTMANN LIMA</t>
         </is>
       </c>
       <c r="C454" s="2" t="n">
@@ -11330,58 +11330,58 @@
         <v>30218</v>
       </c>
       <c r="E454" t="n">
-        <v>0</v>
+        <v>326.86</v>
       </c>
       <c r="F454" t="n">
-        <v>334.48</v>
+        <v>0</v>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="C455" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D455" t="n">
-        <v>31267</v>
+        <v>30218</v>
       </c>
       <c r="E455" t="n">
-        <v>1174.65</v>
+        <v>0</v>
       </c>
       <c r="F455" t="n">
-        <v>1411.84</v>
+        <v>334.48</v>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C456" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D456" t="n">
-        <v>790595</v>
+        <v>31267</v>
       </c>
       <c r="E456" t="n">
-        <v>747.4400000000001</v>
+        <v>1174.65</v>
       </c>
       <c r="F456" t="n">
-        <v>316.74</v>
+        <v>1411.84</v>
       </c>
     </row>
     <row r="457">
@@ -11399,109 +11399,109 @@
         <v>46247</v>
       </c>
       <c r="D457" t="n">
-        <v>30218</v>
+        <v>790595</v>
       </c>
       <c r="E457" t="n">
-        <v>10312.13</v>
+        <v>747.4400000000001</v>
       </c>
       <c r="F457" t="n">
-        <v>3247.44</v>
+        <v>316.74</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
         </is>
       </c>
       <c r="C458" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D458" t="n">
-        <v>47252</v>
+        <v>30218</v>
       </c>
       <c r="E458" t="n">
-        <v>37008.87</v>
+        <v>10312.13</v>
       </c>
       <c r="F458" t="n">
-        <v>27679.4</v>
+        <v>3287.8</v>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
         </is>
       </c>
       <c r="C459" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D459" t="n">
-        <v>794671</v>
+        <v>30083</v>
       </c>
       <c r="E459" t="n">
-        <v>276.11</v>
+        <v>1245.03</v>
       </c>
       <c r="F459" t="n">
-        <v>276.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C460" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D460" t="n">
-        <v>789603</v>
+        <v>47252</v>
       </c>
       <c r="E460" t="n">
-        <v>44564.63</v>
+        <v>37008.87</v>
       </c>
       <c r="F460" t="n">
-        <v>51987.12</v>
+        <v>27679.4</v>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>JONATHAS SANTOS ANDRADE - FARMA</t>
         </is>
       </c>
       <c r="C461" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D461" t="n">
-        <v>792246</v>
+        <v>794671</v>
       </c>
       <c r="E461" t="n">
-        <v>725.33</v>
+        <v>276.11</v>
       </c>
       <c r="F461" t="n">
-        <v>1326.33</v>
+        <v>276.11</v>
       </c>
     </row>
     <row r="462">
@@ -11516,16 +11516,16 @@
         </is>
       </c>
       <c r="C462" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D462" t="n">
-        <v>30307</v>
+        <v>789603</v>
       </c>
       <c r="E462" t="n">
-        <v>5133.29</v>
+        <v>44564.63</v>
       </c>
       <c r="F462" t="n">
-        <v>0</v>
+        <v>51987.12</v>
       </c>
     </row>
     <row r="463">
@@ -11540,40 +11540,40 @@
         </is>
       </c>
       <c r="C463" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D463" t="n">
-        <v>789603</v>
+        <v>792246</v>
       </c>
       <c r="E463" t="n">
-        <v>9443.700000000001</v>
+        <v>725.33</v>
       </c>
       <c r="F463" t="n">
-        <v>0</v>
+        <v>1326.33</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C464" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D464" t="n">
-        <v>139553</v>
+        <v>30307</v>
       </c>
       <c r="E464" t="n">
-        <v>406.68</v>
+        <v>5133.29</v>
       </c>
       <c r="F464" t="n">
-        <v>209.16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="465">
@@ -11584,151 +11584,151 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C465" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D465" t="n">
-        <v>793186</v>
+        <v>789603</v>
       </c>
       <c r="E465" t="n">
-        <v>30303.87</v>
+        <v>9443.700000000001</v>
       </c>
       <c r="F465" t="n">
-        <v>28281.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C466" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D466" t="n">
-        <v>33928</v>
+        <v>139553</v>
       </c>
       <c r="E466" t="n">
-        <v>1177.54</v>
+        <v>406.68</v>
       </c>
       <c r="F466" t="n">
-        <v>50.81</v>
+        <v>209.16</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C467" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D467" t="n">
-        <v>47252</v>
+        <v>793186</v>
       </c>
       <c r="E467" t="n">
-        <v>183.4</v>
+        <v>30303.87</v>
       </c>
       <c r="F467" t="n">
-        <v>135.01</v>
+        <v>28281.01</v>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C468" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D468" t="n">
-        <v>32816</v>
+        <v>33928</v>
       </c>
       <c r="E468" t="n">
-        <v>37.02</v>
+        <v>1177.54</v>
       </c>
       <c r="F468" t="n">
-        <v>37.02</v>
+        <v>50.81</v>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>JOSE CAETANO DA SILVA JUNIOR</t>
+          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
         </is>
       </c>
       <c r="C469" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D469" t="n">
-        <v>794671</v>
+        <v>47252</v>
       </c>
       <c r="E469" t="n">
-        <v>1064.7</v>
+        <v>183.4</v>
       </c>
       <c r="F469" t="n">
-        <v>0</v>
+        <v>135.01</v>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="C470" s="2" t="n">
         <v>46247</v>
       </c>
       <c r="D470" t="n">
-        <v>30083</v>
+        <v>32816</v>
       </c>
       <c r="E470" t="n">
-        <v>948.59</v>
+        <v>37.02</v>
       </c>
       <c r="F470" t="n">
-        <v>627.33</v>
+        <v>37.02</v>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+          <t>JOSE CAETANO DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="C471" s="2" t="n">
@@ -11738,7 +11738,7 @@
         <v>794671</v>
       </c>
       <c r="E471" t="n">
-        <v>1656.21</v>
+        <v>1064.7</v>
       </c>
       <c r="F471" t="n">
         <v>0</v>
@@ -11747,70 +11747,70 @@
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>MARIA ELIZIANE MACIEL DE SOUZA</t>
         </is>
       </c>
       <c r="C472" s="2" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="D472" t="n">
-        <v>33057</v>
+        <v>30083</v>
       </c>
       <c r="E472" t="n">
-        <v>698.02</v>
+        <v>948.59</v>
       </c>
       <c r="F472" t="n">
-        <v>408.35</v>
+        <v>627.33</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="C473" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="D473" t="n">
-        <v>33928</v>
+        <v>33057</v>
       </c>
       <c r="E473" t="n">
-        <v>905.38</v>
+        <v>698.02</v>
       </c>
       <c r="F473" t="n">
-        <v>0</v>
+        <v>408.35</v>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+          <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
         </is>
       </c>
       <c r="C474" s="2" t="n">
         <v>46248</v>
       </c>
       <c r="D474" t="n">
-        <v>30083</v>
+        <v>33928</v>
       </c>
       <c r="E474" t="n">
-        <v>1154.13</v>
+        <v>905.38</v>
       </c>
       <c r="F474" t="n">
         <v>0</v>
@@ -12146,7 +12146,7 @@
         <v>33928</v>
       </c>
       <c r="E488" t="n">
-        <v>1647.13</v>
+        <v>1811.54</v>
       </c>
       <c r="F488" t="n">
         <v>0</v>
@@ -12602,10 +12602,10 @@
         <v>33928</v>
       </c>
       <c r="E507" t="n">
-        <v>18594.44</v>
+        <v>20198.11</v>
       </c>
       <c r="F507" t="n">
-        <v>4747.45</v>
+        <v>4810.14</v>
       </c>
     </row>
     <row r="508">
@@ -12626,10 +12626,10 @@
         <v>789525</v>
       </c>
       <c r="E508" t="n">
-        <v>3029.44</v>
+        <v>3029.5</v>
       </c>
       <c r="F508" t="n">
-        <v>358.82</v>
+        <v>518.1799999999999</v>
       </c>
     </row>
     <row r="509">
@@ -12674,7 +12674,7 @@
         <v>789228</v>
       </c>
       <c r="E510" t="n">
-        <v>97.67</v>
+        <v>265.77</v>
       </c>
       <c r="F510" t="n">
         <v>0</v>
@@ -12794,7 +12794,7 @@
         <v>33928</v>
       </c>
       <c r="E515" t="n">
-        <v>4049.81</v>
+        <v>4477.35</v>
       </c>
       <c r="F515" t="n">
         <v>0</v>
@@ -12866,7 +12866,7 @@
         <v>794029</v>
       </c>
       <c r="E518" t="n">
-        <v>3755.53</v>
+        <v>3870.07</v>
       </c>
       <c r="F518" t="n">
         <v>0</v>
@@ -12890,7 +12890,7 @@
         <v>795345</v>
       </c>
       <c r="E519" t="n">
-        <v>4751.99</v>
+        <v>4965.7